<commit_message>
feat: add dev scripts and refine spreadsheet visual styles
- Added Nix shell script helpers for dev, test, lint, fmt, and Go builds
- Updated spreadsheet generator to include borders on all input and formula cells
- Adjusted table styling and UI layout alignment for better readability
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -341,7 +341,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -380,9 +380,110 @@
       <left style="medium">
         <color rgb="FF808080"/>
       </left>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
       <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
       <top style="medium">
         <color rgb="FF808080"/>
       </top>
@@ -397,301 +498,256 @@
       <right style="thin">
         <color rgb="FF808080"/>
       </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
       <top style="medium">
         <color rgb="FF808080"/>
       </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
       <bottom style="thin">
         <color rgb="FF808080"/>
       </bottom>
     </border>
     <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF808080"/>
       </left>
       <right style="medium">
         <color rgb="FF808080"/>
       </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
       <top style="medium">
         <color rgb="FF808080"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF808080"/>
+        <color rgb="FFD3D3D3"/>
       </bottom>
     </border>
     <border>
       <left style="medium">
         <color rgb="FF808080"/>
       </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
       <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="medium">
         <color rgb="FF808080"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF808080"/>
+        <color rgb="FFD3D3D3"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF808080"/>
+        <color rgb="FFD3D3D3"/>
       </left>
       <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="medium">
         <color rgb="FF808080"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF808080"/>
+        <color rgb="FFD3D3D3"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF808080"/>
+        <color rgb="FFD3D3D3"/>
       </left>
       <right style="medium">
         <color rgb="FF808080"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color rgb="FF808080"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-    </border>
-    <border>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD3D3D3"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD3D3D3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD3D3D3"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
+        <color rgb="FFD3D3D3"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
@@ -702,7 +758,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -714,58 +770,46 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="13" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
@@ -786,92 +830,86 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="true" applyAlignment="false">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="true" applyAlignment="false">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="true" applyAlignment="false">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="true" applyAlignment="false">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="28" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -879,14 +917,41 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="33" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="35" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="13" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -898,14 +963,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TblDrittmittel" displayName="TblDrittmittel" ref="K16:M19">
-  <autoFilter ref="K16:M19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TblDrittmittel" displayName="TblDrittmittel" ref="K15:M18">
+  <autoFilter ref="K15:M18"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Name des Gebers"/>
     <tableColumn id="2" name="Betrag (LC)"/>
     <tableColumn id="3" name="Betrag (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -922,7 +987,7 @@
     <tableColumn id="7" name="Jahr 3"/>
     <tableColumn id="8" name="Betrag (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -1205,14 +1270,6 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="34"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="36"/>
       <c r="R1" s="3" t="str">
         <f>=VSTACK({"Projektpartner";"Bank"},IFERROR(FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
       </c>
@@ -1221,7 +1278,7 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="true">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="30" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="1"/>
@@ -1230,34 +1287,34 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="38"/>
-      <c r="K2" s="58" t="s">
+      <c r="I2" s="31"/>
+      <c r="K2" s="50" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="39"/>
-      <c r="I3" s="40"/>
-      <c r="K3" s="59" t="str">
+      <c r="B3" s="32"/>
+      <c r="I3" s="33"/>
+      <c r="K3" s="51" t="str">
         <f>=$P$11</f>
       </c>
     </row>
     <row r="4" ht="24" customHeight="true">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="23" t="s">
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="24" t="str">
+      <c r="H4" s="20" t="str">
         <f>=IFERROR($E$15/$I$15,0)</f>
       </c>
-      <c r="I4" s="42"/>
-      <c r="K4" s="59" t="s">
+      <c r="I4" s="35"/>
+      <c r="K4" s="52" t="s">
         <v>34</v>
       </c>
       <c r="O4" s="3" t="str">
@@ -1268,7 +1325,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="7"/>
@@ -1285,10 +1342,10 @@
       <c r="H5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="21" t="s">
+      <c r="I5" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="59" t="b">
+      <c r="K5" s="53" t="b">
         <v>0</v>
       </c>
       <c r="O5" s="3" t="str">
@@ -1299,17 +1356,17 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="true">
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="44"/>
-      <c r="K6" s="60" t="str">
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="37"/>
+      <c r="K6" s="54" t="str">
         <f>=IF($K$5=TRUE,"FREIGEGEBEN","NICHT FREIGEGEBEN")</f>
       </c>
       <c r="O6" s="3" t="str">
@@ -1320,14 +1377,14 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="true">
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="38" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
-      <c r="I7" s="46"/>
+      <c r="I7" s="14"/>
       <c r="O7" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Projektaktivitaeten")</f>
       </c>
@@ -1336,8 +1393,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="39"/>
-      <c r="I8" s="40"/>
+      <c r="B8" s="32"/>
+      <c r="I8" s="33"/>
+      <c r="K8" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="L8" s="55"/>
+      <c r="M8" s="55"/>
       <c r="O8" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Projektverwaltung")</f>
       </c>
@@ -1346,21 +1408,21 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="true">
-      <c r="B9" s="43" t="s">
+      <c r="B9" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="44"/>
-      <c r="K9" s="61" t="s">
-        <v>35</v>
-      </c>
-      <c r="L9" s="61"/>
-      <c r="M9" s="61"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="37"/>
+      <c r="K9" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="L9" s="56"/>
+      <c r="M9" s="56"/>
       <c r="O9" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Evaluierung")</f>
       </c>
@@ -1369,26 +1431,24 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="true">
-      <c r="B10" s="45" t="s">
+      <c r="B10" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="28" t="str">
+      <c r="E10" s="24" t="str">
         <f>=SUM(TblDrittmittel[Betrag (LC)])</f>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
-      <c r="I10" s="47" t="str">
+      <c r="I10" s="39" t="str">
         <f>=SUM(TblDrittmittel[Betrag (EUR)])</f>
       </c>
-      <c r="K10" s="62" t="s">
-        <v>5</v>
-      </c>
-      <c r="L10" s="62"/>
-      <c r="M10" s="62"/>
+      <c r="K10" s="56"/>
+      <c r="L10" s="56"/>
+      <c r="M10" s="56"/>
       <c r="O10" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Audit")</f>
       </c>
@@ -1397,11 +1457,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="39"/>
-      <c r="I11" s="40"/>
-      <c r="K11" s="62"/>
-      <c r="L11" s="62"/>
-      <c r="M11" s="62"/>
+      <c r="B11" s="32"/>
+      <c r="I11" s="33"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="56"/>
       <c r="O11" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Reserve")</f>
       </c>
@@ -1410,19 +1470,19 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="true">
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="44"/>
-      <c r="K12" s="62"/>
-      <c r="L12" s="62"/>
-      <c r="M12" s="62"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="37"/>
+      <c r="K12" s="56"/>
+      <c r="L12" s="56"/>
+      <c r="M12" s="56"/>
       <c r="O12" s="3" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (LC)])</f>
       </c>
@@ -1431,81 +1491,83 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="true">
-      <c r="B13" s="45" t="s">
+      <c r="B13" s="38" t="s">
         <v>18</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
-      <c r="I13" s="46"/>
-      <c r="K13" s="62"/>
-      <c r="L13" s="62"/>
-      <c r="M13" s="62"/>
+      <c r="I13" s="14"/>
     </row>
     <row r="14">
-      <c r="B14" s="39"/>
-      <c r="I14" s="40"/>
+      <c r="B14" s="32"/>
+      <c r="I14" s="33"/>
+      <c r="K14" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="L14" s="9"/>
+      <c r="M14" s="10"/>
     </row>
     <row r="15" ht="20" customHeight="true">
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32" t="str">
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28" t="str">
         <f>=E7+E10+E13</f>
       </c>
-      <c r="F15" s="32" t="str">
+      <c r="F15" s="28" t="str">
         <f>=F7+F10+F13</f>
       </c>
-      <c r="G15" s="32" t="str">
+      <c r="G15" s="28" t="str">
         <f>=G7+G10+G13</f>
       </c>
-      <c r="H15" s="32" t="str">
+      <c r="H15" s="28" t="str">
         <f>=H7+H10+H13</f>
       </c>
-      <c r="I15" s="49" t="str">
+      <c r="I15" s="41" t="str">
         <f>=I7+I10+I13</f>
       </c>
-      <c r="K15" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="L15" s="18"/>
-      <c r="M15" s="19"/>
+      <c r="K15" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M15" s="12" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
-      <c r="B16" s="39"/>
-      <c r="I16" s="40"/>
-      <c r="K16" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="L16" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M16" s="21" t="s">
-        <v>4</v>
-      </c>
+      <c r="B16" s="32"/>
+      <c r="I16" s="33"/>
+      <c r="K16" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="L16" s="5"/>
+      <c r="M16" s="14"/>
     </row>
     <row r="17" ht="24" customHeight="true">
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="42"/>
-      <c r="K17" s="8" t="s">
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="35"/>
+      <c r="K17" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="L17" s="9"/>
-      <c r="M17" s="10"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="14"/>
     </row>
     <row r="18">
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C18" s="7" t="s">
@@ -1526,233 +1588,228 @@
       <c r="H18" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I18" s="21" t="s">
+      <c r="I18" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="K18" s="11" t="s">
+      <c r="K18" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="L18" s="12"/>
-      <c r="M18" s="13"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="17"/>
     </row>
     <row r="19">
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="9" t="str">
+      <c r="C19" s="29" t="str">
         <f>=IF(B19="","",MATCH(B19,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B19,B19))</f>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="10"/>
-      <c r="K19" s="14" t="s">
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="29" t="str">
+        <f>=IF(B20="","",MATCH(B20,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L19" s="15"/>
-      <c r="M19" s="16"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="12" t="str">
-        <f>=IF(B20="","",MATCH(B20,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
-      </c>
-      <c r="D20" s="12" t="s">
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="14"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="29" t="str">
+        <f>=IF(B21="","",MATCH(B21,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="13"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="12" t="str">
-        <f>=IF(B21="","",MATCH(B21,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
-      </c>
-      <c r="D21" s="12" t="s">
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="14"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="29" t="str">
+        <f>=IF(B22="","",MATCH(B22,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="13"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C22" s="12" t="str">
-        <f>=IF(B22="","",MATCH(B22,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
-      </c>
-      <c r="D22" s="12" t="s">
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="14"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="29" t="str">
+        <f>=IF(B23="","",MATCH(B23,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="13"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" s="12" t="str">
-        <f>=IF(B23="","",MATCH(B23,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
-      </c>
-      <c r="D23" s="12" t="s">
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="29" t="str">
+        <f>=IF(B24="","",MATCH(B24,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="13"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" s="12" t="str">
-        <f>=IF(B24="","",MATCH(B24,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
-      </c>
-      <c r="D24" s="12" t="s">
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="14"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="29" t="str">
+        <f>=IF(B25="","",MATCH(B25,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="13"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C25" s="12" t="str">
-        <f>=IF(B25="","",MATCH(B25,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
-      </c>
-      <c r="D25" s="12" t="s">
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="14"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26" s="29" t="str">
+        <f>=IF(B26="","",MATCH(B26,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B26,B26))</f>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="13"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="15" t="str">
-        <f>=IF(B26="","",MATCH(B26,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B26,B26))</f>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="16"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="14"/>
     </row>
     <row r="27" ht="20" customHeight="true">
-      <c r="B27" s="50" t="s">
+      <c r="B27" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51" t="str">
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (LC)])</f>
       </c>
-      <c r="F27" s="51" t="str">
+      <c r="F27" s="43" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Jahr 1])</f>
       </c>
-      <c r="G27" s="51" t="str">
+      <c r="G27" s="43" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Jahr 2])</f>
       </c>
-      <c r="H27" s="51" t="str">
+      <c r="H27" s="43" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])</f>
       </c>
-      <c r="I27" s="52" t="str">
+      <c r="I27" s="44" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (EUR)])</f>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="10"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="63"/>
     </row>
     <row r="30">
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="13" t="str">
+      <c r="C30" s="59"/>
+      <c r="D30" s="59"/>
+      <c r="E30" s="65" t="str">
         <f>=IF(ROUND($E$15-$O$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="13" t="str">
+      <c r="C31" s="59"/>
+      <c r="D31" s="59"/>
+      <c r="E31" s="65" t="str">
         <f>=IF(ROUND($I$15-$P$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="13" t="str">
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="65" t="str">
         <f>=IF(ROUND($H$4,4)=ROUND(IFERROR($O$12/$P$12,0),4),"OK","Abweichung")</f>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="13" t="str">
+      <c r="C33" s="59"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="65" t="str">
         <f>=IF(ROUND(($F$15+$G$15+$H$15)-$E$15,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="16" t="str">
+      <c r="C34" s="67"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="68" t="str">
         <f>=IF(ROUND(($F$27+$G$27+$H$27)-$O$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="K9:M9"/>
-    <mergeCell ref="K10:M13"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="K9:M12"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B31:D31"/>

</xml_diff>

<commit_message>
feat: add dropdown selection for approval status in budget generator
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -1817,9 +1817,12 @@
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B34:D34"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation allowBlank="true" sqref="B19:B26" type="list">
       <formula1>"Bauausgaben,Investitionen,Personalkosten,Projektaktivitaeten,Projektverwaltung,Evaluierung,Audit,Reserve"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="K5" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <tableParts count="2">

</xml_diff>

<commit_message>
refactor: implement conditional style cache and update formatting
Introduced `condStyleCache` in the `Generator` struct to manage conditional
formatting styles efficiently. Updated `addConditionalFormat` to handle
style creation internally via `getOrCreateConditionalStyle` and standardized
formula evaluation to improve Excel compatibility. Updated dependent calls in
`budget.go` to use the refactored conditional formatting logic.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>I. KERNDATEN BUDGET</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>Reserve freigeben:</t>
+  </si>
+  <si>
+    <t>Nein</t>
   </si>
   <si>
     <t>Begruendung</t>
@@ -183,7 +186,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -279,14 +282,7 @@
       <name val="Segoe UI"/>
       <family val="2"/>
       <b val="1"/>
-      <color rgb="FF006100"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF7F7F7F"/>
       <sz val="9"/>
     </font>
     <font>
@@ -295,15 +291,8 @@
       <color rgb="FF595959"/>
       <sz val="9"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF9C0006"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -330,16 +319,6 @@
         <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="36">
     <border>
@@ -747,7 +726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
@@ -893,9 +872,6 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -911,24 +887,15 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="33" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -938,16 +905,16 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="35" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="13" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -957,7 +924,122 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF3C3C3C"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFAE5"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
 </styleSheet>
 </file>
@@ -1288,14 +1370,14 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="31"/>
-      <c r="K2" s="50" t="s">
+      <c r="K2" s="49" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32"/>
       <c r="I3" s="33"/>
-      <c r="K3" s="51" t="str">
+      <c r="K3" s="50" t="str">
         <f>=$P$11</f>
       </c>
     </row>
@@ -1314,7 +1396,7 @@
         <f>=IFERROR($E$15/$I$15,0)</f>
       </c>
       <c r="I4" s="35"/>
-      <c r="K4" s="52" t="s">
+      <c r="K4" s="51" t="s">
         <v>34</v>
       </c>
       <c r="O4" s="3" t="str">
@@ -1345,8 +1427,8 @@
       <c r="I5" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="53" t="b">
-        <v>0</v>
+      <c r="K5" s="52" t="s">
+        <v>35</v>
       </c>
       <c r="O5" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Investitionen")</f>
@@ -1366,8 +1448,8 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
       <c r="I6" s="37"/>
-      <c r="K6" s="54" t="str">
-        <f>=IF($K$5=TRUE,"FREIGEGEBEN","NICHT FREIGEGEBEN")</f>
+      <c r="K6" s="53" t="str">
+        <f>=IF($K$5="Ja","FREIGEGEBEN","NICHT FREIGEGEBEN")</f>
       </c>
       <c r="O6" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Personalkosten")</f>
@@ -1395,11 +1477,11 @@
     <row r="8">
       <c r="B8" s="32"/>
       <c r="I8" s="33"/>
-      <c r="K8" s="55" t="s">
-        <v>35</v>
-      </c>
-      <c r="L8" s="55"/>
-      <c r="M8" s="55"/>
+      <c r="K8" s="54" t="s">
+        <v>36</v>
+      </c>
+      <c r="L8" s="54"/>
+      <c r="M8" s="54"/>
       <c r="O8" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Projektverwaltung")</f>
       </c>
@@ -1418,11 +1500,11 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
       <c r="I9" s="37"/>
-      <c r="K9" s="56" t="s">
+      <c r="K9" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="56"/>
-      <c r="M9" s="56"/>
+      <c r="L9" s="55"/>
+      <c r="M9" s="55"/>
       <c r="O9" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Evaluierung")</f>
       </c>
@@ -1446,9 +1528,9 @@
       <c r="I10" s="39" t="str">
         <f>=SUM(TblDrittmittel[Betrag (EUR)])</f>
       </c>
-      <c r="K10" s="56"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="56"/>
+      <c r="K10" s="55"/>
+      <c r="L10" s="55"/>
+      <c r="M10" s="55"/>
       <c r="O10" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Audit")</f>
       </c>
@@ -1459,9 +1541,9 @@
     <row r="11">
       <c r="B11" s="32"/>
       <c r="I11" s="33"/>
-      <c r="K11" s="56"/>
-      <c r="L11" s="56"/>
-      <c r="M11" s="56"/>
+      <c r="K11" s="55"/>
+      <c r="L11" s="55"/>
+      <c r="M11" s="55"/>
       <c r="O11" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Reserve")</f>
       </c>
@@ -1480,9 +1562,9 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
       <c r="I12" s="37"/>
-      <c r="K12" s="56"/>
-      <c r="L12" s="56"/>
-      <c r="M12" s="56"/>
+      <c r="K12" s="55"/>
+      <c r="L12" s="55"/>
+      <c r="M12" s="55"/>
       <c r="O12" s="3" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (LC)])</f>
       </c>
@@ -1748,60 +1830,60 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="61" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="62"/>
-      <c r="D29" s="62"/>
-      <c r="E29" s="63"/>
+      <c r="B29" s="57" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="59"/>
     </row>
     <row r="30">
-      <c r="B30" s="64" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="65" t="str">
+      <c r="B30" s="60" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="61" t="str">
         <f>=IF(ROUND($E$15-$O$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="64" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" s="59"/>
-      <c r="D31" s="59"/>
-      <c r="E31" s="65" t="str">
+      <c r="B31" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="61" t="str">
         <f>=IF(ROUND($I$15-$P$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="64" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-      <c r="E32" s="65" t="str">
+      <c r="B32" s="60" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="56"/>
+      <c r="D32" s="56"/>
+      <c r="E32" s="61" t="str">
         <f>=IF(ROUND($H$4,4)=ROUND(IFERROR($O$12/$P$12,0),4),"OK","Abweichung")</f>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="64" t="s">
-        <v>40</v>
-      </c>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="65" t="str">
+      <c r="B33" s="60" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="56"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="61" t="str">
         <f>=IF(ROUND(($F$15+$G$15+$H$15)-$E$15,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="66" t="s">
-        <v>41</v>
-      </c>
-      <c r="C34" s="67"/>
-      <c r="D34" s="67"/>
-      <c r="E34" s="68" t="str">
+      <c r="B34" s="62" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="63"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="64" t="str">
         <f>=IF(ROUND(($F$27+$G$27+$H$27)-$O$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
@@ -1817,12 +1899,77 @@
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B34:D34"/>
   </mergeCells>
+  <conditionalFormatting sqref="K6">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$K$5="Ja"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K8:M8">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$K$5="Ja"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9:M12">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>$K$5="Ja"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E30">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>$E$30="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E30">
+    <cfRule type="expression" dxfId="3" priority="5">
+      <formula>$E$30&lt;&gt;"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E31">
+    <cfRule type="expression" dxfId="0" priority="6">
+      <formula>$E$31="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E31">
+    <cfRule type="expression" dxfId="3" priority="7">
+      <formula>$E$31&lt;&gt;"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E32">
+    <cfRule type="expression" dxfId="0" priority="8">
+      <formula>$E$32="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E32">
+    <cfRule type="expression" dxfId="3" priority="9">
+      <formula>$E$32&lt;&gt;"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E33">
+    <cfRule type="expression" dxfId="0" priority="10">
+      <formula>$E$33="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E33">
+    <cfRule type="expression" dxfId="3" priority="11">
+      <formula>$E$33&lt;&gt;"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E34">
+    <cfRule type="expression" dxfId="0" priority="12">
+      <formula>$E$34="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E34">
+    <cfRule type="expression" dxfId="3" priority="13">
+      <formula>$E$34&lt;&gt;"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation allowBlank="true" sqref="B19:B26" type="list">
       <formula1>"Bauausgaben,Investitionen,Personalkosten,Projektaktivitaeten,Projektverwaltung,Evaluierung,Audit,Reserve"</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="K5" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+      <formula1>"Ja,Nein"</formula1>
     </dataValidation>
   </dataValidations>
   <tableParts count="2">

</xml_diff>

<commit_message>
style: update budget excel cell styles and borders
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -320,7 +320,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -477,6 +477,14 @@
       <right style="thin">
         <color rgb="FF808080"/>
       </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
       <top style="thin">
         <color rgb="FF808080"/>
       </top>
@@ -485,6 +493,12 @@
       </bottom>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
       <top style="thin">
         <color rgb="FF808080"/>
       </top>
@@ -782,7 +796,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -809,44 +823,41 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
@@ -860,6 +871,9 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -872,19 +886,19 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="33" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -896,13 +910,13 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="33" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="35" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="36" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -924,7 +938,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <font>
         <name val="Segoe UI"/>
@@ -940,17 +954,17 @@
       </fill>
       <alignment/>
       <border>
-        <left style="thin">
-          <color rgb="FFD3D3D3"/>
+        <left style="medium">
+          <color rgb="FF808080"/>
         </left>
-        <right style="thin">
-          <color rgb="FFD3D3D3"/>
+        <right style="medium">
+          <color rgb="FF808080"/>
         </right>
         <top style="thin">
-          <color rgb="FFD3D3D3"/>
+          <color rgb="FF808080"/>
         </top>
-        <bottom style="thin">
-          <color rgb="FFD3D3D3"/>
+        <bottom style="medium">
+          <color rgb="FF808080"/>
         </bottom>
       </border>
     </dxf>
@@ -1007,6 +1021,35 @@
         </top>
         <bottom style="thin">
           <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
         </bottom>
       </border>
     </dxf>
@@ -1915,52 +1958,52 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30">
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$E$30="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30">
-    <cfRule type="expression" dxfId="3" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>$E$30&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E31">
-    <cfRule type="expression" dxfId="0" priority="6">
+    <cfRule type="expression" dxfId="3" priority="6">
       <formula>$E$31="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E31">
-    <cfRule type="expression" dxfId="3" priority="7">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula>$E$31&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="3" priority="8">
       <formula>$E$32="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32">
-    <cfRule type="expression" dxfId="3" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>$E$32&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E33">
-    <cfRule type="expression" dxfId="0" priority="10">
+    <cfRule type="expression" dxfId="3" priority="10">
       <formula>$E$33="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E33">
-    <cfRule type="expression" dxfId="3" priority="11">
+    <cfRule type="expression" dxfId="4" priority="11">
       <formula>$E$33&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="0" priority="12">
+    <cfRule type="expression" dxfId="3" priority="12">
       <formula>$E$34="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="3" priority="13">
+    <cfRule type="expression" dxfId="4" priority="13">
       <formula>$E$34&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
refactor: make drittmittel table position dynamic
Update `bgDrawDrittmittelTable` to accept a row parameter instead of using
hardcoded values. Adjust styling logic to handle dynamic table borders.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -51,100 +51,100 @@
     <t>I. KERNDATEN BUDGET</t>
   </si>
   <si>
+    <t>1. GEPLANTE EINNAHMEN / FINANZIERUNG</t>
+  </si>
+  <si>
+    <t>€ Budget-Kurs:</t>
+  </si>
+  <si>
+    <t>Finanzierungsquelle</t>
+  </si>
+  <si>
+    <t>Betrag (LC)</t>
+  </si>
+  <si>
+    <t>Jahr 1</t>
+  </si>
+  <si>
+    <t>Jahr 2</t>
+  </si>
+  <si>
+    <t>Jahr 3</t>
+  </si>
+  <si>
+    <t>Betrag (EUR)</t>
+  </si>
+  <si>
+    <t>1.1 Eigenmittel</t>
+  </si>
+  <si>
+    <t>Eigenmittel</t>
+  </si>
+  <si>
+    <t>1.2 Drittmittel</t>
+  </si>
+  <si>
+    <t>Drittmittel (Summe):</t>
+  </si>
+  <si>
+    <t>Aufstellung je Geber → Tabelle rechts</t>
+  </si>
+  <si>
+    <t>1.3 KMW-Mittel</t>
+  </si>
+  <si>
+    <t>KMW-Mittel</t>
+  </si>
+  <si>
+    <t>GESAMTPROJEKTMITTEL</t>
+  </si>
+  <si>
+    <t>2. GEPLANTE AUSGABEN</t>
+  </si>
+  <si>
+    <t>Kostenkategorie</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Kostenposition</t>
+  </si>
+  <si>
+    <t>Bauausgaben</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Investitionen</t>
+  </si>
+  <si>
+    <t>Personalkosten</t>
+  </si>
+  <si>
+    <t>Projektaktivitaeten</t>
+  </si>
+  <si>
+    <t>Projektverwaltung</t>
+  </si>
+  <si>
+    <t>Evaluierung</t>
+  </si>
+  <si>
+    <t>Audit</t>
+  </si>
+  <si>
+    <t>Reserve</t>
+  </si>
+  <si>
+    <t>Geplante Gesamtausgaben</t>
+  </si>
+  <si>
     <t>Drittmittel – Aufstellung je Geber</t>
   </si>
   <si>
     <t>Name des Gebers</t>
-  </si>
-  <si>
-    <t>Betrag (LC)</t>
-  </si>
-  <si>
-    <t>Betrag (EUR)</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>1. GEPLANTE EINNAHMEN / FINANZIERUNG</t>
-  </si>
-  <si>
-    <t>€ Budget-Kurs:</t>
-  </si>
-  <si>
-    <t>Finanzierungsquelle</t>
-  </si>
-  <si>
-    <t>Jahr 1</t>
-  </si>
-  <si>
-    <t>Jahr 2</t>
-  </si>
-  <si>
-    <t>Jahr 3</t>
-  </si>
-  <si>
-    <t>1.1 Eigenmittel</t>
-  </si>
-  <si>
-    <t>Eigenmittel</t>
-  </si>
-  <si>
-    <t>1.2 Drittmittel</t>
-  </si>
-  <si>
-    <t>Drittmittel (Summe):</t>
-  </si>
-  <si>
-    <t>Aufstellung je Geber → Tabelle rechts</t>
-  </si>
-  <si>
-    <t>1.3 KMW-Mittel</t>
-  </si>
-  <si>
-    <t>KMW-Mittel</t>
-  </si>
-  <si>
-    <t>GESAMTPROJEKTMITTEL</t>
-  </si>
-  <si>
-    <t>2. GEPLANTE AUSGABEN</t>
-  </si>
-  <si>
-    <t>Kostenkategorie</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Kostenposition</t>
-  </si>
-  <si>
-    <t>Bauausgaben</t>
-  </si>
-  <si>
-    <t>Investitionen</t>
-  </si>
-  <si>
-    <t>Personalkosten</t>
-  </si>
-  <si>
-    <t>Projektaktivitaeten</t>
-  </si>
-  <si>
-    <t>Projektverwaltung</t>
-  </si>
-  <si>
-    <t>Evaluierung</t>
-  </si>
-  <si>
-    <t>Audit</t>
-  </si>
-  <si>
-    <t>Reserve</t>
-  </si>
-  <si>
-    <t>Geplante Gesamtausgaben</t>
   </si>
   <si>
     <t>Reserve Freigabe</t>
@@ -182,9 +182,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -199,24 +199,6 @@
       <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <color rgb="FF000000"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF3C3C3C"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -240,6 +222,18 @@
     <font>
       <name val="Segoe UI"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF3C3C3C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="10"/>
@@ -256,6 +250,12 @@
       <i val="1"/>
       <color rgb="FF595959"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -306,12 +306,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFAE5"/>
+        <fgColor rgb="FFF0F0F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0F0F0"/>
+        <fgColor rgb="FFFFFAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -337,172 +337,172 @@
       </bottom>
     </border>
     <border>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="FFD3D3D3"/>
+        <color rgb="FF808080"/>
       </left>
       <right style="thin">
-        <color rgb="FFD3D3D3"/>
-      </right>
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
       <top style="thin">
-        <color rgb="FFD3D3D3"/>
+        <color rgb="FF808080"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD3D3D3"/>
-      </bottom>
-    </border>
-    <border>
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
       <bottom style="medium">
         <color rgb="FF808080"/>
       </bottom>
     </border>
     <border>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FF808080"/>
       </left>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-    </border>
-    <border>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-    </border>
-    <border>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
       <right style="medium">
         <color rgb="FF808080"/>
       </right>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
     </border>
     <border>
       <left style="medium">
         <color rgb="FF808080"/>
       </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
       <bottom style="medium">
         <color rgb="FF808080"/>
       </bottom>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
       <right style="medium">
         <color rgb="FF808080"/>
       </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
       <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD3D3D3"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD3D3D3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD3D3D3"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD3D3D3"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD3D3D3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD3D3D3"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD3D3D3"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD3D3D3"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD3D3D3"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD3D3D3"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD3D3D3"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD3D3D3"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD3D3D3"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
         <color rgb="FF808080"/>
       </bottom>
     </border>
@@ -745,89 +745,89 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="13" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="14" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="16" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="17" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
@@ -841,73 +841,73 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="25" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="26" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="26" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="28" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="29" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="32" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="33" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -919,26 +919,26 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="36" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="13" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="7">
     <dxf>
       <font>
         <name val="Segoe UI"/>
@@ -1040,16 +1040,16 @@
       <alignment/>
       <border>
         <left style="thin">
-          <color rgb="FFD3D3D3"/>
+          <color rgb="FF808080"/>
         </left>
-        <right style="thin">
-          <color rgb="FFD3D3D3"/>
+        <right style="medium">
+          <color rgb="FF808080"/>
         </right>
         <top style="thin">
-          <color rgb="FFD3D3D3"/>
+          <color rgb="FF808080"/>
         </top>
         <bottom style="thin">
-          <color rgb="FFD3D3D3"/>
+          <color rgb="FF808080"/>
         </bottom>
       </border>
     </dxf>
@@ -1069,16 +1069,74 @@
       <alignment/>
       <border>
         <left style="thin">
-          <color rgb="FFD3D3D3"/>
+          <color rgb="FF808080"/>
         </left>
-        <right style="thin">
-          <color rgb="FFD3D3D3"/>
+        <right style="medium">
+          <color rgb="FF808080"/>
         </right>
         <top style="thin">
-          <color rgb="FFD3D3D3"/>
+          <color rgb="FF808080"/>
         </top>
         <bottom style="thin">
-          <color rgb="FFD3D3D3"/>
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF808080"/>
         </bottom>
       </border>
     </dxf>
@@ -1088,19 +1146,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TblDrittmittel" displayName="TblDrittmittel" ref="K15:M18">
-  <autoFilter ref="K15:M18"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Name des Gebers"/>
-    <tableColumn id="2" name="Betrag (LC)"/>
-    <tableColumn id="3" name="Betrag (EUR)"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TblBudgetAusgaben" displayName="TblBudgetAusgaben" ref="B18:I27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TblBudgetAusgaben" displayName="TblBudgetAusgaben" ref="B18:I27">
   <autoFilter ref="B18:I27"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Kostenkategorie"/>
@@ -1111,6 +1157,18 @@
     <tableColumn id="6" name="Jahr 2"/>
     <tableColumn id="7" name="Jahr 3"/>
     <tableColumn id="8" name="Betrag (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TblDrittmittel" displayName="TblDrittmittel" ref="K18:M21">
+  <autoFilter ref="K18:M21"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Name des Gebers"/>
+    <tableColumn id="2" name="Betrag (LC)"/>
+    <tableColumn id="3" name="Betrag (EUR)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
@@ -1395,10 +1453,10 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="R1" s="3" t="str">
+      <c r="R1" s="5" t="str">
         <f>=VSTACK({"Projektpartner";"Bank"},IFERROR(FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
       </c>
-      <c r="S1" s="3" t="str">
+      <c r="S1" s="5" t="str">
         <f>=IFERROR(FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
       </c>
     </row>
@@ -1426,94 +1484,94 @@
     </row>
     <row r="4" ht="24" customHeight="true">
       <c r="B4" s="34" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="20" t="str">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="4" t="str">
         <f>=IFERROR($E$15/$I$15,0)</f>
       </c>
       <c r="I4" s="35"/>
       <c r="K4" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="O4" s="3" t="str">
+      <c r="O4" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Bauausgaben")</f>
       </c>
-      <c r="P4" s="3" t="str">
+      <c r="P4" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Bauausgaben")</f>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="24" t="s">
         <v>8</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>4</v>
       </c>
       <c r="K5" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="O5" s="3" t="str">
+      <c r="O5" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Investitionen")</f>
       </c>
-      <c r="P5" s="3" t="str">
+      <c r="P5" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Investitionen")</f>
       </c>
     </row>
     <row r="6" ht="20" customHeight="true">
       <c r="B6" s="36" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
+        <v>9</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
       <c r="I6" s="37"/>
       <c r="K6" s="53" t="str">
         <f>=IF($K$5="Ja","FREIGEGEBEN","NICHT FREIGEGEBEN")</f>
       </c>
-      <c r="O6" s="3" t="str">
+      <c r="O6" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Personalkosten")</f>
       </c>
-      <c r="P6" s="3" t="str">
+      <c r="P6" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Personalkosten")</f>
       </c>
     </row>
     <row r="7" ht="22" customHeight="true">
       <c r="B7" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="14"/>
-      <c r="O7" s="3" t="str">
+        <v>10</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="26"/>
+      <c r="O7" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Projektaktivitaeten")</f>
       </c>
-      <c r="P7" s="3" t="str">
+      <c r="P7" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Projektaktivitaeten")</f>
       </c>
     </row>
@@ -1525,59 +1583,59 @@
       </c>
       <c r="L8" s="54"/>
       <c r="M8" s="54"/>
-      <c r="O8" s="3" t="str">
+      <c r="O8" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Projektverwaltung")</f>
       </c>
-      <c r="P8" s="3" t="str">
+      <c r="P8" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Projektverwaltung")</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="true">
       <c r="B9" s="36" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
+        <v>11</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="37"/>
       <c r="K9" s="55" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="L9" s="55"/>
       <c r="M9" s="55"/>
-      <c r="O9" s="3" t="str">
+      <c r="O9" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Evaluierung")</f>
       </c>
-      <c r="P9" s="3" t="str">
+      <c r="P9" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Evaluierung")</f>
       </c>
     </row>
     <row r="10" ht="22" customHeight="true">
       <c r="B10" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="24" t="str">
+        <v>12</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="12" t="str">
         <f>=SUM(TblDrittmittel[Betrag (LC)])</f>
       </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
       <c r="I10" s="39" t="str">
         <f>=SUM(TblDrittmittel[Betrag (EUR)])</f>
       </c>
       <c r="K10" s="55"/>
       <c r="L10" s="55"/>
       <c r="M10" s="55"/>
-      <c r="O10" s="3" t="str">
+      <c r="O10" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Audit")</f>
       </c>
-      <c r="P10" s="3" t="str">
+      <c r="P10" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Audit")</f>
       </c>
     </row>
@@ -1587,272 +1645,272 @@
       <c r="K11" s="55"/>
       <c r="L11" s="55"/>
       <c r="M11" s="55"/>
-      <c r="O11" s="3" t="str">
+      <c r="O11" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Reserve")</f>
       </c>
-      <c r="P11" s="3" t="str">
+      <c r="P11" s="5" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Reserve")</f>
       </c>
     </row>
     <row r="12" ht="20" customHeight="true">
       <c r="B12" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
+        <v>14</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
       <c r="I12" s="37"/>
       <c r="K12" s="55"/>
       <c r="L12" s="55"/>
       <c r="M12" s="55"/>
-      <c r="O12" s="3" t="str">
+      <c r="O12" s="5" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (LC)])</f>
       </c>
-      <c r="P12" s="3" t="str">
+      <c r="P12" s="5" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (EUR)])</f>
       </c>
     </row>
     <row r="13" ht="22" customHeight="true">
       <c r="B13" s="38" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="14"/>
+        <v>15</v>
+      </c>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14">
       <c r="B14" s="32"/>
       <c r="I14" s="33"/>
-      <c r="K14" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="L14" s="9"/>
-      <c r="M14" s="10"/>
     </row>
     <row r="15" ht="20" customHeight="true">
       <c r="B15" s="40" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28" t="str">
+        <v>16</v>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16" t="str">
         <f>=E7+E10+E13</f>
       </c>
-      <c r="F15" s="28" t="str">
+      <c r="F15" s="16" t="str">
         <f>=F7+F10+F13</f>
       </c>
-      <c r="G15" s="28" t="str">
+      <c r="G15" s="16" t="str">
         <f>=G7+G10+G13</f>
       </c>
-      <c r="H15" s="28" t="str">
+      <c r="H15" s="16" t="str">
         <f>=H7+H10+H13</f>
       </c>
       <c r="I15" s="41" t="str">
         <f>=I7+I10+I13</f>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="L15" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M15" s="12" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="32"/>
       <c r="I16" s="33"/>
-      <c r="K16" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="L16" s="5"/>
-      <c r="M16" s="14"/>
     </row>
     <row r="17" ht="24" customHeight="true">
       <c r="B17" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="35"/>
+      <c r="K17" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L17" s="21"/>
+      <c r="M17" s="22"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="35"/>
-      <c r="K17" s="13" t="s">
+      <c r="E18" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L17" s="5"/>
-      <c r="M17" s="14"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="11" t="s">
+      <c r="G18" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I18" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="K18" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M18" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C19" s="18" t="str">
+        <f>=IF(B19="","",MATCH(B19,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B19,B19))</f>
+      </c>
+      <c r="D19" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="26"/>
+      <c r="K19" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="L19" s="9"/>
+      <c r="M19" s="26"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I18" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="K18" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="L18" s="16"/>
-      <c r="M18" s="17"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="13" t="s">
+      <c r="C20" s="18" t="str">
+        <f>=IF(B20="","",MATCH(B20,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="26"/>
+      <c r="K20" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="L20" s="9"/>
+      <c r="M20" s="26"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="29" t="str">
-        <f>=IF(B19="","",MATCH(B19,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B19,B19))</f>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="14"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="13" t="s">
+      <c r="C21" s="18" t="str">
+        <f>=IF(B21="","",MATCH(B21,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="26"/>
+      <c r="K21" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="L21" s="28"/>
+      <c r="M21" s="29"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="29" t="str">
-        <f>=IF(B20="","",MATCH(B20,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="14"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="13" t="s">
+      <c r="C22" s="18" t="str">
+        <f>=IF(B22="","",MATCH(B22,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="26"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="29" t="str">
-        <f>=IF(B21="","",MATCH(B21,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="14"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="13" t="s">
+      <c r="C23" s="18" t="str">
+        <f>=IF(B23="","",MATCH(B23,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="26"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="29" t="str">
-        <f>=IF(B22="","",MATCH(B22,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="14"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="13" t="s">
+      <c r="C24" s="18" t="str">
+        <f>=IF(B24="","",MATCH(B24,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="26"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="29" t="str">
-        <f>=IF(B23="","",MATCH(B23,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="14"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="13" t="s">
+      <c r="C25" s="18" t="str">
+        <f>=IF(B25="","",MATCH(B25,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="26"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="29" t="str">
-        <f>=IF(B24="","",MATCH(B24,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="14"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C25" s="29" t="str">
-        <f>=IF(B25="","",MATCH(B25,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="14"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="29" t="str">
+      <c r="C26" s="18" t="str">
         <f>=IF(B26="","",MATCH(B26,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B26,B26))</f>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="14"/>
+      <c r="D26" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="26"/>
     </row>
     <row r="27" ht="20" customHeight="true">
       <c r="B27" s="42" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C27" s="43"/>
       <c r="D27" s="43"/>
@@ -1932,7 +1990,7 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="K17:M17"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="K9:M12"/>
     <mergeCell ref="B29:E29"/>
@@ -1998,12 +2056,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="3" priority="12">
+    <cfRule type="expression" dxfId="5" priority="12">
       <formula>$E$34="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="4" priority="13">
+    <cfRule type="expression" dxfId="6" priority="13">
       <formula>$E$34&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat: add dashboard sheet generation
Implement the dashboard sheet with project information fields, a
document checklist, conditional formatting for input fields, and support
for strike-through text styles.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -7,9 +7,12 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="I. Budget" sheetId="2" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="2" r:id="rId4"/>
+    <sheet name="I. Budget" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames>
+    <definedName name="Saldovortrag_LW">'Dashboard'!$C$13</definedName>
+    <definedName name="Saldovortrag_EUR">'Dashboard'!$E$13</definedName>
     <definedName name="Budget_Kurs">'I. Budget'!$H$4</definedName>
     <definedName name="Eigenmittel_LW">'I. Budget'!$E$7</definedName>
     <definedName name="Eigenmittel_EUR">'I. Budget'!$I$7</definedName>
@@ -46,7 +49,553 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
+  <si>
+    <t xml:space="preserve">  DASHBOARD (v1.0)</t>
+  </si>
+  <si>
+    <t>Statische Projektinformationen</t>
+  </si>
+  <si>
+    <t>AED</t>
+  </si>
+  <si>
+    <t>AFN</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>AMD</t>
+  </si>
+  <si>
+    <t>AOA</t>
+  </si>
+  <si>
+    <t>ARS</t>
+  </si>
+  <si>
+    <t>AUD</t>
+  </si>
+  <si>
+    <t>AWG</t>
+  </si>
+  <si>
+    <t>AZN</t>
+  </si>
+  <si>
+    <t>BAM</t>
+  </si>
+  <si>
+    <t>BBD</t>
+  </si>
+  <si>
+    <t>BDT</t>
+  </si>
+  <si>
+    <t>BHD</t>
+  </si>
+  <si>
+    <t>BIF</t>
+  </si>
+  <si>
+    <t>BMD</t>
+  </si>
+  <si>
+    <t>BND</t>
+  </si>
+  <si>
+    <t>BOB</t>
+  </si>
+  <si>
+    <t>BRL</t>
+  </si>
+  <si>
+    <t>BSD</t>
+  </si>
+  <si>
+    <t>BTN</t>
+  </si>
+  <si>
+    <t>BWP</t>
+  </si>
+  <si>
+    <t>BYN</t>
+  </si>
+  <si>
+    <t>BZD</t>
+  </si>
+  <si>
+    <t>CAD</t>
+  </si>
+  <si>
+    <t>CDF</t>
+  </si>
+  <si>
+    <t>CHF</t>
+  </si>
+  <si>
+    <t>CLP</t>
+  </si>
+  <si>
+    <t>CNY</t>
+  </si>
+  <si>
+    <t>COP</t>
+  </si>
+  <si>
+    <t>CRC</t>
+  </si>
+  <si>
+    <t>CUP</t>
+  </si>
+  <si>
+    <t>CVE</t>
+  </si>
+  <si>
+    <t>CZK</t>
+  </si>
+  <si>
+    <t>DJF</t>
+  </si>
+  <si>
+    <t>DKK</t>
+  </si>
+  <si>
+    <t>DOP</t>
+  </si>
+  <si>
+    <t>DZD</t>
+  </si>
+  <si>
+    <t>EGP</t>
+  </si>
+  <si>
+    <t>ERN</t>
+  </si>
+  <si>
+    <t>ETB</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>FJD</t>
+  </si>
+  <si>
+    <t>FKP</t>
+  </si>
+  <si>
+    <t>GBP</t>
+  </si>
+  <si>
+    <t>GEL</t>
+  </si>
+  <si>
+    <t>GHS</t>
+  </si>
+  <si>
+    <t>GIP</t>
+  </si>
+  <si>
+    <t>GMD</t>
+  </si>
+  <si>
+    <t>GNF</t>
+  </si>
+  <si>
+    <t>GTQ</t>
+  </si>
+  <si>
+    <t>GYD</t>
+  </si>
+  <si>
+    <t>HKD</t>
+  </si>
+  <si>
+    <t>HNL</t>
+  </si>
+  <si>
+    <t>HTG</t>
+  </si>
+  <si>
+    <t>HUF</t>
+  </si>
+  <si>
+    <t>IDR</t>
+  </si>
+  <si>
+    <t>ILS</t>
+  </si>
+  <si>
+    <t>INR</t>
+  </si>
+  <si>
+    <t>IQD</t>
+  </si>
+  <si>
+    <t>IRR</t>
+  </si>
+  <si>
+    <t>ISK</t>
+  </si>
+  <si>
+    <t>JMD</t>
+  </si>
+  <si>
+    <t>JOD</t>
+  </si>
+  <si>
+    <t>JPY</t>
+  </si>
+  <si>
+    <t>KES</t>
+  </si>
+  <si>
+    <t>KGS</t>
+  </si>
+  <si>
+    <t>KHR</t>
+  </si>
+  <si>
+    <t>KMF</t>
+  </si>
+  <si>
+    <t>KPW</t>
+  </si>
+  <si>
+    <t>KRW</t>
+  </si>
+  <si>
+    <t>KWD</t>
+  </si>
+  <si>
+    <t>KYD</t>
+  </si>
+  <si>
+    <t>KZT</t>
+  </si>
+  <si>
+    <t>LAK</t>
+  </si>
+  <si>
+    <t>LBP</t>
+  </si>
+  <si>
+    <t>LKR</t>
+  </si>
+  <si>
+    <t>LRD</t>
+  </si>
+  <si>
+    <t>LSL</t>
+  </si>
+  <si>
+    <t>LYD</t>
+  </si>
+  <si>
+    <t>MAD</t>
+  </si>
+  <si>
+    <t>MDL</t>
+  </si>
+  <si>
+    <t>MGA</t>
+  </si>
+  <si>
+    <t>MKD</t>
+  </si>
+  <si>
+    <t>MMK</t>
+  </si>
+  <si>
+    <t>MNT</t>
+  </si>
+  <si>
+    <t>MOP</t>
+  </si>
+  <si>
+    <t>MRU</t>
+  </si>
+  <si>
+    <t>MUR</t>
+  </si>
+  <si>
+    <t>MVR</t>
+  </si>
+  <si>
+    <t>MWK</t>
+  </si>
+  <si>
+    <t>MXN</t>
+  </si>
+  <si>
+    <t>MYR</t>
+  </si>
+  <si>
+    <t>MZN</t>
+  </si>
+  <si>
+    <t>NAD</t>
+  </si>
+  <si>
+    <t>NGN</t>
+  </si>
+  <si>
+    <t>NIO</t>
+  </si>
+  <si>
+    <t>NOK</t>
+  </si>
+  <si>
+    <t>NPR</t>
+  </si>
+  <si>
+    <t>NZD</t>
+  </si>
+  <si>
+    <t>OMR</t>
+  </si>
+  <si>
+    <t>PAB</t>
+  </si>
+  <si>
+    <t>PEN</t>
+  </si>
+  <si>
+    <t>PGK</t>
+  </si>
+  <si>
+    <t>PHP</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>PLN</t>
+  </si>
+  <si>
+    <t>PYG</t>
+  </si>
+  <si>
+    <t>QAR</t>
+  </si>
+  <si>
+    <t>RON</t>
+  </si>
+  <si>
+    <t>RSD</t>
+  </si>
+  <si>
+    <t>RUB</t>
+  </si>
+  <si>
+    <t>RWF</t>
+  </si>
+  <si>
+    <t>SAR</t>
+  </si>
+  <si>
+    <t>SBD</t>
+  </si>
+  <si>
+    <t>SCR</t>
+  </si>
+  <si>
+    <t>SDG</t>
+  </si>
+  <si>
+    <t>SEK</t>
+  </si>
+  <si>
+    <t>SGD</t>
+  </si>
+  <si>
+    <t>SHP</t>
+  </si>
+  <si>
+    <t>SLE</t>
+  </si>
+  <si>
+    <t>SOS</t>
+  </si>
+  <si>
+    <t>SRD</t>
+  </si>
+  <si>
+    <t>SSP</t>
+  </si>
+  <si>
+    <t>STN</t>
+  </si>
+  <si>
+    <t>SVC</t>
+  </si>
+  <si>
+    <t>SYP</t>
+  </si>
+  <si>
+    <t>SZL</t>
+  </si>
+  <si>
+    <t>THB</t>
+  </si>
+  <si>
+    <t>TJS</t>
+  </si>
+  <si>
+    <t>TMT</t>
+  </si>
+  <si>
+    <t>TND</t>
+  </si>
+  <si>
+    <t>TOP</t>
+  </si>
+  <si>
+    <t>TRY</t>
+  </si>
+  <si>
+    <t>TTD</t>
+  </si>
+  <si>
+    <t>TWD</t>
+  </si>
+  <si>
+    <t>TZS</t>
+  </si>
+  <si>
+    <t>UAH</t>
+  </si>
+  <si>
+    <t>UGX</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>UYU</t>
+  </si>
+  <si>
+    <t>UZS</t>
+  </si>
+  <si>
+    <t>VED</t>
+  </si>
+  <si>
+    <t>VES</t>
+  </si>
+  <si>
+    <t>VND</t>
+  </si>
+  <si>
+    <t>VUV</t>
+  </si>
+  <si>
+    <t>WST</t>
+  </si>
+  <si>
+    <t>XAF</t>
+  </si>
+  <si>
+    <t>XCD</t>
+  </si>
+  <si>
+    <t>XCG</t>
+  </si>
+  <si>
+    <t>XOF</t>
+  </si>
+  <si>
+    <t>XPF</t>
+  </si>
+  <si>
+    <t>YER</t>
+  </si>
+  <si>
+    <t>ZAR</t>
+  </si>
+  <si>
+    <t>ZMW</t>
+  </si>
+  <si>
+    <t>ZWG</t>
+  </si>
+  <si>
+    <t>Projektnummer</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Vorprojekt vorhanden</t>
+  </si>
+  <si>
+    <t>Projekttitel</t>
+  </si>
+  <si>
+    <t>Projekttraeger</t>
+  </si>
+  <si>
+    <t>Berichtswaehrung</t>
+  </si>
+  <si>
+    <t>Projektlaufzeit (geplant)</t>
+  </si>
+  <si>
+    <t>In Monate</t>
+  </si>
+  <si>
+    <t>Vorprojektnummer</t>
+  </si>
+  <si>
+    <t>VP-Berichtswaehrung</t>
+  </si>
+  <si>
+    <t>Vorprojektende</t>
+  </si>
+  <si>
+    <t>Wechselkurs</t>
+  </si>
+  <si>
+    <t>Saldo (LW)</t>
+  </si>
+  <si>
+    <t>Saldo (EUR)</t>
+  </si>
+  <si>
+    <t>Folgeprojektstart</t>
+  </si>
+  <si>
+    <t>Saldovortrag (LW)</t>
+  </si>
+  <si>
+    <t>Saldovortrag (EUR)</t>
+  </si>
+  <si>
+    <t>Folgende Dokumente liegen vor:</t>
+  </si>
+  <si>
+    <t>Vorprojektsaldo (Nachweis)</t>
+  </si>
+  <si>
+    <t>Vertrag</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>Bankbelege</t>
+  </si>
+  <si>
+    <t>Finanzbericht(e)</t>
+  </si>
+  <si>
+    <t>Einzelbelege und Beleglisten</t>
+  </si>
+  <si>
+    <t>Narrativer Bericht</t>
+  </si>
   <si>
     <t>I. KERNDATEN BUDGET</t>
   </si>
@@ -112,9 +661,6 @@
   </si>
   <si>
     <t>Bauausgaben</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Investitionen</t>
@@ -181,17 +727,44 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -222,21 +795,9 @@
     <font>
       <name val="Segoe UI"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
       <b val="1"/>
       <color rgb="FF3C3C3C"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -292,7 +853,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -301,7 +862,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD3D3D3"/>
+        <fgColor rgb="FF6C7A50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCDCDC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -311,7 +887,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFAE5"/>
+        <fgColor rgb="FFD3D3D3"/>
       </patternFill>
     </fill>
     <fill>
@@ -320,13 +896,51 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="41">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <bottom style="thick">
+        <color rgb="FF667022"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FF969696"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF969696"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF969696"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF969696"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF969696"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF969696"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF969696"/>
+      </right>
+      <top style="double">
+        <color rgb="FF969696"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF969696"/>
+      </bottom>
     </border>
     <border>
       <top style="medium">
@@ -740,205 +1354,272 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="12" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="13" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="16" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="19" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="22" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="23" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="26" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="27" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="28" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="29" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="25" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="33" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="34" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="35" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="36" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="36" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="36" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="37" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="38" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="39" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="14" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="16" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="17" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="25" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="26" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="28" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="29" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="32" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="33" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="35" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="36" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="14" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="21" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <color rgb="FF646464"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF0F0F0"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <strike val="1"/>
+        <color rgb="FF646464"/>
+      </font>
+      <alignment/>
+    </dxf>
     <dxf>
       <font>
         <name val="Segoe UI"/>
@@ -1433,6 +2114,1004 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
+    <tabColor rgb="D3D3D3"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3"/>
+    <col customWidth="true" max="2" min="2" width="25"/>
+    <col customWidth="true" max="3" min="3" width="31"/>
+    <col customWidth="true" max="4" min="4" width="22.5"/>
+    <col customWidth="true" max="5" min="5" width="25"/>
+    <col customWidth="true" hidden="true" max="27" min="27" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="AA1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="true">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="AA2" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="AA3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="true">
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="AA4" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="true">
+      <c r="B5" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E5" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="true">
+      <c r="B6" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="AA6" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="true">
+      <c r="B7" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA7" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="true">
+      <c r="B8" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" s="7" t="str">
+        <f>=IFERROR(LET(AllNums, TEXTJOIN("", TRUE, IFERROR(MID(C8, SEQUENCE(LEN(C8)), 1) * 1, "")), StartDate, DATE(MID(AllNums, 5, 4), MID(AllNums, 3, 2), LEFT(AllNums, 2)), EndDate, DATE(MID(AllNums, 13, 4), MID(AllNums, 11, 2), MID(AllNums, 9, 2)), DATEDIF(StartDate, EndDate + 1, "M")), "")</f>
+      </c>
+      <c r="AA8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="true">
+      <c r="B9" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA9" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="true">
+      <c r="B10" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA10" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="true">
+      <c r="B11" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA11" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="true">
+      <c r="B12" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA12" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="true">
+      <c r="B13" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="AA14" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="true">
+      <c r="B15" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" s="14"/>
+      <c r="D15" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="AA15" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="true">
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="AA16" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="true">
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA17" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="true">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="AA18" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="true">
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="AA19" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="true">
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="AA20" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="true">
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="AA21" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="AA22" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="AA23" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="AA24" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="AA25" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="AA26" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="AA27" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="AA28" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="AA29" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="AA30" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="AA31" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="AA32" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="AA33" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="AA34" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="AA35" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="AA36" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="AA37" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="AA38" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="AA39" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="AA40" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="AA41" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="AA42" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="AA43" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="AA44" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="AA45" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="AA46" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="AA47" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="AA48" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="AA49" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="AA50" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="AA51" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="AA52" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="AA53" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="AA54" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="AA55" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="AA56" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="AA57" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="AA58" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="AA59" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="AA60" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="AA61" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="AA62" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="AA63" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="AA64" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="AA65" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="AA66" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="AA67" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="AA68" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="AA69" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="AA70" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="AA71" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="AA72" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="AA73" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="AA74" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="AA75" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="AA76" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="AA77" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="AA78" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="AA79" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="AA80" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="AA81" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="AA82" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="AA83" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="AA84" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="AA85" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="AA86" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="AA87" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="AA88" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="AA89" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="AA90" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="AA91" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="AA92" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="AA93" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="AA94" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="AA95" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="AA96" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="AA97" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="AA98" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="AA99" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="AA100" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="AA101" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="AA102" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="AA103" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="AA104" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="AA105" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="AA106" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="AA107" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="AA108" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="AA109" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="AA110" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="AA111" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="AA112" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="AA113" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="AA114" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="AA115" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="AA116" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="AA117" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="AA118" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="AA119" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="AA120" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="AA121" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="AA122" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="AA123" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="AA124" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="AA125" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="AA126" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="AA127" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="AA128" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="AA129" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="AA130" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="AA131" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="AA132" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="AA133" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="AA134" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="AA135" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="AA136" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="AA137" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="AA138" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="AA139" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="AA140" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="AA141" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="AA142" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="AA143" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="AA144" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="AA145" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="AA146" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="AA147" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="AA148" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="AA149" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="AA150" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="AA151" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="AA152" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="AA153" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="AA154" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="AA155" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="B15:C21"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9:E13">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$E$5=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15:E21">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$D15=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D15:E15">
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>$E$5=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" sqref="E7" type="list">
+      <formula1>'Dashboard'!$AA$1:$AA$155</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="E9" type="list">
+      <formula1>'Dashboard'!$AA$1:$AA$155</formula1>
+    </dataValidation>
+  </dataValidations>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr>
     <tabColor rgb="5B9BD5"/>
   </sheetPr>
   <dimension ref="A1"/>
@@ -1453,538 +3132,538 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="R1" s="5" t="str">
+      <c r="R1" s="3" t="str">
         <f>=VSTACK({"Projektpartner";"Bank"},IFERROR(FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
       </c>
-      <c r="S1" s="5" t="str">
+      <c r="S1" s="3" t="str">
         <f>=IFERROR(FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
       </c>
     </row>
     <row r="2" ht="24" customHeight="true">
-      <c r="B2" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="31"/>
-      <c r="K2" s="49" t="s">
-        <v>33</v>
+      <c r="B2" s="45" t="s">
+        <v>182</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="46"/>
+      <c r="K2" s="64" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="32"/>
-      <c r="I3" s="33"/>
-      <c r="K3" s="50" t="str">
+      <c r="B3" s="47"/>
+      <c r="I3" s="48"/>
+      <c r="K3" s="65" t="str">
         <f>=$P$11</f>
       </c>
     </row>
     <row r="4" ht="24" customHeight="true">
-      <c r="B4" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="H4" s="4" t="str">
+      <c r="B4" s="49" t="s">
+        <v>183</v>
+      </c>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="H4" s="20" t="str">
         <f>=IFERROR($E$15/$I$15,0)</f>
       </c>
-      <c r="I4" s="35"/>
-      <c r="K4" s="51" t="s">
-        <v>34</v>
-      </c>
-      <c r="O4" s="5" t="str">
+      <c r="I4" s="50"/>
+      <c r="K4" s="66" t="s">
+        <v>215</v>
+      </c>
+      <c r="O4" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Bauausgaben")</f>
       </c>
-      <c r="P4" s="5" t="str">
+      <c r="P4" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Bauausgaben")</f>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="K5" s="52" t="s">
-        <v>35</v>
-      </c>
-      <c r="O5" s="5" t="str">
+      <c r="B5" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="I5" s="39" t="s">
+        <v>190</v>
+      </c>
+      <c r="K5" s="67" t="s">
+        <v>216</v>
+      </c>
+      <c r="O5" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Investitionen")</f>
       </c>
-      <c r="P5" s="5" t="str">
+      <c r="P5" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Investitionen")</f>
       </c>
     </row>
     <row r="6" ht="20" customHeight="true">
-      <c r="B6" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="37"/>
-      <c r="K6" s="53" t="str">
+      <c r="B6" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="52"/>
+      <c r="K6" s="68" t="str">
         <f>=IF($K$5="Ja","FREIGEGEBEN","NICHT FREIGEGEBEN")</f>
       </c>
-      <c r="O6" s="5" t="str">
+      <c r="O6" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Personalkosten")</f>
       </c>
-      <c r="P6" s="5" t="str">
+      <c r="P6" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Personalkosten")</f>
       </c>
     </row>
     <row r="7" ht="22" customHeight="true">
-      <c r="B7" s="38" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="26"/>
-      <c r="O7" s="5" t="str">
+      <c r="B7" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="41"/>
+      <c r="O7" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Projektaktivitaeten")</f>
       </c>
-      <c r="P7" s="5" t="str">
+      <c r="P7" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Projektaktivitaeten")</f>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="32"/>
-      <c r="I8" s="33"/>
-      <c r="K8" s="54" t="s">
-        <v>36</v>
-      </c>
-      <c r="L8" s="54"/>
-      <c r="M8" s="54"/>
-      <c r="O8" s="5" t="str">
+      <c r="B8" s="47"/>
+      <c r="I8" s="48"/>
+      <c r="K8" s="69" t="s">
+        <v>217</v>
+      </c>
+      <c r="L8" s="69"/>
+      <c r="M8" s="69"/>
+      <c r="O8" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Projektverwaltung")</f>
       </c>
-      <c r="P8" s="5" t="str">
+      <c r="P8" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Projektverwaltung")</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="true">
-      <c r="B9" s="36" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="37"/>
-      <c r="K9" s="55" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" s="55"/>
-      <c r="M9" s="55"/>
-      <c r="O9" s="5" t="str">
+      <c r="B9" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="52"/>
+      <c r="K9" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="L9" s="70"/>
+      <c r="M9" s="70"/>
+      <c r="O9" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Evaluierung")</f>
       </c>
-      <c r="P9" s="5" t="str">
+      <c r="P9" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Evaluierung")</f>
       </c>
     </row>
     <row r="10" ht="22" customHeight="true">
-      <c r="B10" s="38" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="12" t="str">
+      <c r="B10" s="53" t="s">
+        <v>194</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="E10" s="27" t="str">
         <f>=SUM(TblDrittmittel[Betrag (LC)])</f>
       </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="39" t="str">
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="54" t="str">
         <f>=SUM(TblDrittmittel[Betrag (EUR)])</f>
       </c>
-      <c r="K10" s="55"/>
-      <c r="L10" s="55"/>
-      <c r="M10" s="55"/>
-      <c r="O10" s="5" t="str">
+      <c r="K10" s="70"/>
+      <c r="L10" s="70"/>
+      <c r="M10" s="70"/>
+      <c r="O10" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Audit")</f>
       </c>
-      <c r="P10" s="5" t="str">
+      <c r="P10" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Audit")</f>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="32"/>
-      <c r="I11" s="33"/>
-      <c r="K11" s="55"/>
-      <c r="L11" s="55"/>
-      <c r="M11" s="55"/>
-      <c r="O11" s="5" t="str">
+      <c r="B11" s="47"/>
+      <c r="I11" s="48"/>
+      <c r="K11" s="70"/>
+      <c r="L11" s="70"/>
+      <c r="M11" s="70"/>
+      <c r="O11" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Reserve")</f>
       </c>
-      <c r="P11" s="5" t="str">
+      <c r="P11" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (EUR)],TblBudgetAusgaben[Kostenkategorie],"Reserve")</f>
       </c>
     </row>
     <row r="12" ht="20" customHeight="true">
-      <c r="B12" s="36" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="37"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="55"/>
-      <c r="M12" s="55"/>
-      <c r="O12" s="5" t="str">
+      <c r="B12" s="51" t="s">
+        <v>196</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="52"/>
+      <c r="K12" s="70"/>
+      <c r="L12" s="70"/>
+      <c r="M12" s="70"/>
+      <c r="O12" s="3" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (LC)])</f>
       </c>
-      <c r="P12" s="5" t="str">
+      <c r="P12" s="3" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (EUR)])</f>
       </c>
     </row>
     <row r="13" ht="22" customHeight="true">
-      <c r="B13" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="26"/>
+      <c r="B13" s="53" t="s">
+        <v>197</v>
+      </c>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="41"/>
     </row>
     <row r="14">
-      <c r="B14" s="32"/>
-      <c r="I14" s="33"/>
+      <c r="B14" s="47"/>
+      <c r="I14" s="48"/>
     </row>
     <row r="15" ht="20" customHeight="true">
-      <c r="B15" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16" t="str">
+      <c r="B15" s="55" t="s">
+        <v>198</v>
+      </c>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31" t="str">
         <f>=E7+E10+E13</f>
       </c>
-      <c r="F15" s="16" t="str">
+      <c r="F15" s="31" t="str">
         <f>=F7+F10+F13</f>
       </c>
-      <c r="G15" s="16" t="str">
+      <c r="G15" s="31" t="str">
         <f>=G7+G10+G13</f>
       </c>
-      <c r="H15" s="16" t="str">
+      <c r="H15" s="31" t="str">
         <f>=H7+H10+H13</f>
       </c>
-      <c r="I15" s="41" t="str">
+      <c r="I15" s="56" t="str">
         <f>=I7+I10+I13</f>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="32"/>
-      <c r="I16" s="33"/>
+      <c r="B16" s="47"/>
+      <c r="I16" s="48"/>
     </row>
     <row r="17" ht="24" customHeight="true">
-      <c r="B17" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="35"/>
-      <c r="K17" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="L17" s="21"/>
-      <c r="M17" s="22"/>
+      <c r="B17" s="49" t="s">
+        <v>199</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="50"/>
+      <c r="K17" s="35" t="s">
+        <v>212</v>
+      </c>
+      <c r="L17" s="36"/>
+      <c r="M17" s="37"/>
     </row>
     <row r="18">
-      <c r="B18" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I18" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="K18" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="L18" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="M18" s="24" t="s">
-        <v>8</v>
+      <c r="B18" s="38" t="s">
+        <v>200</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>201</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="I18" s="39" t="s">
+        <v>190</v>
+      </c>
+      <c r="K18" s="38" t="s">
+        <v>213</v>
+      </c>
+      <c r="L18" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="M18" s="39" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" s="18" t="str">
+      <c r="B19" s="40" t="s">
+        <v>203</v>
+      </c>
+      <c r="C19" s="33" t="str">
         <f>=IF(B19="","",MATCH(B19,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B19,B19))</f>
       </c>
-      <c r="D19" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="26"/>
-      <c r="K19" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="L19" s="9"/>
-      <c r="M19" s="26"/>
+      <c r="D19" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="41"/>
+      <c r="K19" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="L19" s="24"/>
+      <c r="M19" s="41"/>
     </row>
     <row r="20">
-      <c r="B20" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="18" t="str">
+      <c r="B20" s="40" t="s">
+        <v>204</v>
+      </c>
+      <c r="C20" s="33" t="str">
         <f>=IF(B20="","",MATCH(B20,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="26"/>
-      <c r="K20" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="L20" s="9"/>
-      <c r="M20" s="26"/>
+      <c r="D20" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="41"/>
+      <c r="K20" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="L20" s="24"/>
+      <c r="M20" s="41"/>
     </row>
     <row r="21">
-      <c r="B21" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" s="18" t="str">
+      <c r="B21" s="40" t="s">
+        <v>205</v>
+      </c>
+      <c r="C21" s="33" t="str">
         <f>=IF(B21="","",MATCH(B21,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
       </c>
-      <c r="D21" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="26"/>
-      <c r="K21" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="L21" s="28"/>
-      <c r="M21" s="29"/>
+      <c r="D21" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="41"/>
+      <c r="K21" s="42" t="s">
+        <v>158</v>
+      </c>
+      <c r="L21" s="43"/>
+      <c r="M21" s="44"/>
     </row>
     <row r="22">
-      <c r="B22" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="18" t="str">
+      <c r="B22" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="C22" s="33" t="str">
         <f>=IF(B22="","",MATCH(B22,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="26"/>
+      <c r="D22" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="41"/>
     </row>
     <row r="23">
-      <c r="B23" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" s="18" t="str">
+      <c r="B23" s="40" t="s">
+        <v>207</v>
+      </c>
+      <c r="C23" s="33" t="str">
         <f>=IF(B23="","",MATCH(B23,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="26"/>
+      <c r="D23" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="41"/>
     </row>
     <row r="24">
-      <c r="B24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="18" t="str">
+      <c r="B24" s="40" t="s">
+        <v>208</v>
+      </c>
+      <c r="C24" s="33" t="str">
         <f>=IF(B24="","",MATCH(B24,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
       </c>
-      <c r="D24" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="26"/>
+      <c r="D24" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="41"/>
     </row>
     <row r="25">
-      <c r="B25" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="18" t="str">
+      <c r="B25" s="40" t="s">
+        <v>209</v>
+      </c>
+      <c r="C25" s="33" t="str">
         <f>=IF(B25="","",MATCH(B25,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
       </c>
-      <c r="D25" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="26"/>
+      <c r="D25" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="41"/>
     </row>
     <row r="26">
-      <c r="B26" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="18" t="str">
+      <c r="B26" s="40" t="s">
+        <v>210</v>
+      </c>
+      <c r="C26" s="33" t="str">
         <f>=IF(B26="","",MATCH(B26,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B26,B26))</f>
       </c>
-      <c r="D26" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="26"/>
+      <c r="D26" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="41"/>
     </row>
     <row r="27" ht="20" customHeight="true">
-      <c r="B27" s="42" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43" t="str">
+      <c r="B27" s="57" t="s">
+        <v>211</v>
+      </c>
+      <c r="C27" s="58"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="58" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (LC)])</f>
       </c>
-      <c r="F27" s="43" t="str">
+      <c r="F27" s="58" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Jahr 1])</f>
       </c>
-      <c r="G27" s="43" t="str">
+      <c r="G27" s="58" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Jahr 2])</f>
       </c>
-      <c r="H27" s="43" t="str">
+      <c r="H27" s="58" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])</f>
       </c>
-      <c r="I27" s="44" t="str">
+      <c r="I27" s="59" t="str">
         <f>=SUBTOTAL(109,TblBudgetAusgaben[Betrag (EUR)])</f>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="57" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" s="58"/>
-      <c r="D29" s="58"/>
-      <c r="E29" s="59"/>
+      <c r="B29" s="72" t="s">
+        <v>218</v>
+      </c>
+      <c r="C29" s="73"/>
+      <c r="D29" s="73"/>
+      <c r="E29" s="74"/>
     </row>
     <row r="30">
-      <c r="B30" s="60" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="61" t="str">
+      <c r="B30" s="75" t="s">
+        <v>219</v>
+      </c>
+      <c r="C30" s="71"/>
+      <c r="D30" s="71"/>
+      <c r="E30" s="76" t="str">
         <f>=IF(ROUND($E$15-$O$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="60" t="s">
-        <v>39</v>
-      </c>
-      <c r="C31" s="56"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="61" t="str">
+      <c r="B31" s="75" t="s">
+        <v>220</v>
+      </c>
+      <c r="C31" s="71"/>
+      <c r="D31" s="71"/>
+      <c r="E31" s="76" t="str">
         <f>=IF(ROUND($I$15-$P$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="60" t="s">
-        <v>40</v>
-      </c>
-      <c r="C32" s="56"/>
-      <c r="D32" s="56"/>
-      <c r="E32" s="61" t="str">
+      <c r="B32" s="75" t="s">
+        <v>221</v>
+      </c>
+      <c r="C32" s="71"/>
+      <c r="D32" s="71"/>
+      <c r="E32" s="76" t="str">
         <f>=IF(ROUND($H$4,4)=ROUND(IFERROR($O$12/$P$12,0),4),"OK","Abweichung")</f>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="60" t="s">
-        <v>41</v>
-      </c>
-      <c r="C33" s="56"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="61" t="str">
+      <c r="B33" s="75" t="s">
+        <v>222</v>
+      </c>
+      <c r="C33" s="71"/>
+      <c r="D33" s="71"/>
+      <c r="E33" s="76" t="str">
         <f>=IF(ROUND(($F$15+$G$15+$H$15)-$E$15,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="62" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="63"/>
-      <c r="D34" s="63"/>
-      <c r="E34" s="64" t="str">
+      <c r="B34" s="77" t="s">
+        <v>223</v>
+      </c>
+      <c r="C34" s="78"/>
+      <c r="D34" s="78"/>
+      <c r="E34" s="79" t="str">
         <f>=IF(ROUND(($F$27+$G$27+$H$27)-$O$12,2)=0,"OK","Abweichung")</f>
       </c>
     </row>
@@ -2001,67 +3680,67 @@
     <mergeCell ref="B34:D34"/>
   </mergeCells>
   <conditionalFormatting sqref="K6">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$K$5="Ja"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K8:M8">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$K$5="Ja"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K9:M12">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>$K$5="Ja"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>$E$30="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>$E$30&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E31">
-    <cfRule type="expression" dxfId="3" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>$E$31="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E31">
-    <cfRule type="expression" dxfId="4" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>$E$31&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32">
-    <cfRule type="expression" dxfId="3" priority="8">
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>$E$32="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32">
-    <cfRule type="expression" dxfId="4" priority="9">
+    <cfRule type="expression" dxfId="6" priority="9">
       <formula>$E$32&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E33">
-    <cfRule type="expression" dxfId="3" priority="10">
+    <cfRule type="expression" dxfId="5" priority="10">
       <formula>$E$33="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E33">
-    <cfRule type="expression" dxfId="4" priority="11">
+    <cfRule type="expression" dxfId="6" priority="11">
       <formula>$E$33&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="5" priority="12">
+    <cfRule type="expression" dxfId="7" priority="12">
       <formula>$E$34="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="6" priority="13">
+    <cfRule type="expression" dxfId="8" priority="13">
       <formula>$E$34&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat: replace checkboxes with Yes/No dropdowns
Refactor dashboard input fields to use Ja/Nein dropdowns instead of
checkboxes. This includes updating conditional formatting logic,
column widths, and removing the legacy `dbCheckbox` helper in favor of
`dbDropdownJaNein`.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -531,6 +531,9 @@
     <t>Vorprojekt vorhanden</t>
   </si>
   <si>
+    <t>Ja</t>
+  </si>
+  <si>
     <t>Projekttitel</t>
   </si>
   <si>
@@ -576,6 +579,9 @@
     <t>Folgende Dokumente liegen vor:</t>
   </si>
   <si>
+    <t>Nein</t>
+  </si>
+  <si>
     <t>Vorprojektsaldo (Nachweis)</t>
   </si>
   <si>
@@ -697,9 +703,6 @@
   </si>
   <si>
     <t>Reserve freigeben:</t>
-  </si>
-  <si>
-    <t>Nein</t>
   </si>
   <si>
     <t>Begruendung</t>
@@ -2120,10 +2123,10 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="true" max="1" min="1" width="3"/>
-    <col customWidth="true" max="2" min="2" width="25"/>
-    <col customWidth="true" max="3" min="3" width="31"/>
-    <col customWidth="true" max="4" min="4" width="22.5"/>
-    <col customWidth="true" max="5" min="5" width="25"/>
+    <col customWidth="true" max="2" min="2" width="32"/>
+    <col customWidth="true" max="3" min="3" width="25"/>
+    <col customWidth="true" max="4" min="4" width="24"/>
+    <col customWidth="true" max="5" min="5" width="35"/>
     <col customWidth="true" hidden="true" max="27" min="27" width="9.140625"/>
   </cols>
   <sheetData>
@@ -2169,8 +2172,8 @@
       <c r="D5" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="E5" s="6" t="b">
-        <v>1</v>
+      <c r="E5" s="6" t="s">
+        <v>160</v>
       </c>
       <c r="AA5" s="3" t="s">
         <v>6</v>
@@ -2178,7 +2181,7 @@
     </row>
     <row r="6" ht="22" customHeight="true">
       <c r="B6" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>158</v>
@@ -2191,13 +2194,13 @@
     </row>
     <row r="7" ht="22" customHeight="true">
       <c r="B7" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>158</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>158</v>
@@ -2208,13 +2211,13 @@
     </row>
     <row r="8" ht="22" customHeight="true">
       <c r="B8" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>158</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E8" s="7" t="str">
         <f>=IFERROR(LET(AllNums, TEXTJOIN("", TRUE, IFERROR(MID(C8, SEQUENCE(LEN(C8)), 1) * 1, "")), StartDate, DATE(MID(AllNums, 5, 4), MID(AllNums, 3, 2), LEFT(AllNums, 2)), EndDate, DATE(MID(AllNums, 13, 4), MID(AllNums, 11, 2), MID(AllNums, 9, 2)), DATEDIF(StartDate, EndDate + 1, "M")), "")</f>
@@ -2225,13 +2228,13 @@
     </row>
     <row r="9" ht="22" customHeight="true">
       <c r="B9" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>158</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>158</v>
@@ -2242,13 +2245,13 @@
     </row>
     <row r="10" ht="22" customHeight="true">
       <c r="B10" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>158</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>158</v>
@@ -2259,13 +2262,13 @@
     </row>
     <row r="11" ht="22" customHeight="true">
       <c r="B11" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>158</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E11" s="13" t="s">
         <v>158</v>
@@ -2276,13 +2279,13 @@
     </row>
     <row r="12" ht="22" customHeight="true">
       <c r="B12" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>158</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>158</v>
@@ -2293,13 +2296,13 @@
     </row>
     <row r="13" ht="22" customHeight="true">
       <c r="B13" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>158</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>158</v>
@@ -2315,14 +2318,14 @@
     </row>
     <row r="15" ht="22" customHeight="true">
       <c r="B15" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C15" s="14"/>
-      <c r="D15" s="15" t="b">
-        <v>0</v>
+      <c r="D15" s="15" t="s">
+        <v>176</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AA15" s="3" t="s">
         <v>16</v>
@@ -2331,11 +2334,11 @@
     <row r="16" ht="22" customHeight="true">
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
-      <c r="D16" s="15" t="b">
-        <v>0</v>
+      <c r="D16" s="15" t="s">
+        <v>176</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AA16" s="3" t="s">
         <v>17</v>
@@ -2344,11 +2347,11 @@
     <row r="17" ht="22" customHeight="true">
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
-      <c r="D17" s="15" t="b">
-        <v>0</v>
+      <c r="D17" s="15" t="s">
+        <v>176</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AA17" s="3" t="s">
         <v>18</v>
@@ -2357,11 +2360,11 @@
     <row r="18" ht="22" customHeight="true">
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
-      <c r="D18" s="15" t="b">
-        <v>0</v>
+      <c r="D18" s="15" t="s">
+        <v>176</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AA18" s="3" t="s">
         <v>19</v>
@@ -2370,11 +2373,11 @@
     <row r="19" ht="22" customHeight="true">
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
-      <c r="D19" s="15" t="b">
-        <v>0</v>
+      <c r="D19" s="15" t="s">
+        <v>176</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AA19" s="3" t="s">
         <v>20</v>
@@ -2383,11 +2386,11 @@
     <row r="20" ht="22" customHeight="true">
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
-      <c r="D20" s="15" t="b">
-        <v>0</v>
+      <c r="D20" s="15" t="s">
+        <v>176</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="AA20" s="3" t="s">
         <v>21</v>
@@ -2396,11 +2399,11 @@
     <row r="21" ht="22" customHeight="true">
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
-      <c r="D21" s="15" t="b">
-        <v>0</v>
+      <c r="D21" s="15" t="s">
+        <v>176</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AA21" s="3" t="s">
         <v>22</v>
@@ -3085,25 +3088,49 @@
   </mergeCells>
   <conditionalFormatting sqref="B9:E13">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$E$5=FALSE</formula>
+      <formula>$E$5="Nein"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E15:E21">
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$D15=FALSE</formula>
+      <formula>$D15="Nein"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15:E15">
     <cfRule type="expression" dxfId="0" priority="3">
-      <formula>$E$5=FALSE</formula>
+      <formula>$E$5="Nein"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="10">
+    <dataValidation allowBlank="true" sqref="E5" type="list">
+      <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
     <dataValidation allowBlank="true" sqref="E7" type="list">
       <formula1>'Dashboard'!$AA$1:$AA$155</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="E9" type="list">
       <formula1>'Dashboard'!$AA$1:$AA$155</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D15" type="list">
+      <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D16" type="list">
+      <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D17" type="list">
+      <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D18" type="list">
+      <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D19" type="list">
+      <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D20" type="list">
+      <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D21" type="list">
+      <formula1>"Ja,Nein"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -3141,7 +3168,7 @@
     </row>
     <row r="2" ht="24" customHeight="true">
       <c r="B2" s="45" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -3151,7 +3178,7 @@
       <c r="H2" s="17"/>
       <c r="I2" s="46"/>
       <c r="K2" s="64" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
@@ -3163,21 +3190,21 @@
     </row>
     <row r="4" ht="24" customHeight="true">
       <c r="B4" s="49" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C4" s="18"/>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
       <c r="F4" s="18"/>
       <c r="G4" s="19" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H4" s="20" t="str">
         <f>=IFERROR($E$15/$I$15,0)</f>
       </c>
       <c r="I4" s="50"/>
       <c r="K4" s="66" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="O4" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Bauausgaben")</f>
@@ -3188,27 +3215,27 @@
     </row>
     <row r="5">
       <c r="B5" s="38" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C5" s="21"/>
       <c r="D5" s="21"/>
       <c r="E5" s="21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I5" s="39" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="K5" s="67" t="s">
-        <v>216</v>
+        <v>176</v>
       </c>
       <c r="O5" s="3" t="str">
         <f>=SUMIFS(TblBudgetAusgaben[Betrag (LC)],TblBudgetAusgaben[Kostenkategorie],"Investitionen")</f>
@@ -3219,7 +3246,7 @@
     </row>
     <row r="6" ht="20" customHeight="true">
       <c r="B6" s="51" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
@@ -3240,7 +3267,7 @@
     </row>
     <row r="7" ht="22" customHeight="true">
       <c r="B7" s="53" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E7" s="24"/>
       <c r="F7" s="24"/>
@@ -3258,7 +3285,7 @@
       <c r="B8" s="47"/>
       <c r="I8" s="48"/>
       <c r="K8" s="69" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="L8" s="69"/>
       <c r="M8" s="69"/>
@@ -3271,7 +3298,7 @@
     </row>
     <row r="9" ht="20" customHeight="true">
       <c r="B9" s="51" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
@@ -3294,10 +3321,10 @@
     </row>
     <row r="10" ht="22" customHeight="true">
       <c r="B10" s="53" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E10" s="27" t="str">
         <f>=SUM(TblDrittmittel[Betrag (LC)])</f>
@@ -3333,7 +3360,7 @@
     </row>
     <row r="12" ht="20" customHeight="true">
       <c r="B12" s="51" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C12" s="22"/>
       <c r="D12" s="22"/>
@@ -3354,7 +3381,7 @@
     </row>
     <row r="13" ht="22" customHeight="true">
       <c r="B13" s="53" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E13" s="24"/>
       <c r="F13" s="24"/>
@@ -3368,7 +3395,7 @@
     </row>
     <row r="15" ht="20" customHeight="true">
       <c r="B15" s="55" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
@@ -3394,7 +3421,7 @@
     </row>
     <row r="17" ht="24" customHeight="true">
       <c r="B17" s="49" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C17" s="18"/>
       <c r="D17" s="18"/>
@@ -3404,49 +3431,49 @@
       <c r="H17" s="18"/>
       <c r="I17" s="50"/>
       <c r="K17" s="35" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="L17" s="36"/>
       <c r="M17" s="37"/>
     </row>
     <row r="18">
       <c r="B18" s="38" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G18" s="21" t="s">
+        <v>190</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>191</v>
+      </c>
+      <c r="I18" s="39" t="s">
+        <v>192</v>
+      </c>
+      <c r="K18" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="L18" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="H18" s="21" t="s">
-        <v>189</v>
-      </c>
-      <c r="I18" s="39" t="s">
-        <v>190</v>
-      </c>
-      <c r="K18" s="38" t="s">
-        <v>213</v>
-      </c>
-      <c r="L18" s="21" t="s">
-        <v>186</v>
-      </c>
       <c r="M18" s="39" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="40" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C19" s="33" t="str">
         <f>=IF(B19="","",MATCH(B19,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B19,B19))</f>
@@ -3467,7 +3494,7 @@
     </row>
     <row r="20">
       <c r="B20" s="40" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C20" s="33" t="str">
         <f>=IF(B20="","",MATCH(B20,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
@@ -3488,7 +3515,7 @@
     </row>
     <row r="21">
       <c r="B21" s="40" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C21" s="33" t="str">
         <f>=IF(B21="","",MATCH(B21,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
@@ -3509,7 +3536,7 @@
     </row>
     <row r="22">
       <c r="B22" s="40" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C22" s="33" t="str">
         <f>=IF(B22="","",MATCH(B22,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
@@ -3525,7 +3552,7 @@
     </row>
     <row r="23">
       <c r="B23" s="40" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C23" s="33" t="str">
         <f>=IF(B23="","",MATCH(B23,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
@@ -3541,7 +3568,7 @@
     </row>
     <row r="24">
       <c r="B24" s="40" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C24" s="33" t="str">
         <f>=IF(B24="","",MATCH(B24,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
@@ -3557,7 +3584,7 @@
     </row>
     <row r="25">
       <c r="B25" s="40" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C25" s="33" t="str">
         <f>=IF(B25="","",MATCH(B25,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
@@ -3573,7 +3600,7 @@
     </row>
     <row r="26">
       <c r="B26" s="40" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C26" s="33" t="str">
         <f>=IF(B26="","",MATCH(B26,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B26,B26))</f>
@@ -3589,7 +3616,7 @@
     </row>
     <row r="27" ht="20" customHeight="true">
       <c r="B27" s="57" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C27" s="58"/>
       <c r="D27" s="58"/>
@@ -3611,7 +3638,7 @@
     </row>
     <row r="29">
       <c r="B29" s="72" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C29" s="73"/>
       <c r="D29" s="73"/>
@@ -3619,7 +3646,7 @@
     </row>
     <row r="30">
       <c r="B30" s="75" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C30" s="71"/>
       <c r="D30" s="71"/>
@@ -3629,7 +3656,7 @@
     </row>
     <row r="31">
       <c r="B31" s="75" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C31" s="71"/>
       <c r="D31" s="71"/>
@@ -3639,7 +3666,7 @@
     </row>
     <row r="32">
       <c r="B32" s="75" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C32" s="71"/>
       <c r="D32" s="71"/>
@@ -3649,7 +3676,7 @@
     </row>
     <row r="33">
       <c r="B33" s="75" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C33" s="71"/>
       <c r="D33" s="71"/>
@@ -3659,7 +3686,7 @@
     </row>
     <row r="34">
       <c r="B34" s="77" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C34" s="78"/>
       <c r="D34" s="78"/>

</xml_diff>

<commit_message>
feat: add KMW-Mittel sheet generation
Implement CreateKMWMittelSheet to generate the 'II. KMW-Mittel' worksheet
with layout, input validation, and formula-based summation. Update main
to include the new sheet in the generation process.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Dashboard" sheetId="2" r:id="rId4"/>
     <sheet name="I. Budget" sheetId="3" r:id="rId6"/>
+    <sheet name="II. KMW-Mittel" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="Saldovortrag_LW">'Dashboard'!$C$13</definedName>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="267">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -724,6 +725,132 @@
   </si>
   <si>
     <t>Ausgaben: Jahre = Gesamt (LC)</t>
+  </si>
+  <si>
+    <t>II. KMW-MITTEL BEREITGESTELLT</t>
+  </si>
+  <si>
+    <t>Periode 1</t>
+  </si>
+  <si>
+    <t>Periode 2</t>
+  </si>
+  <si>
+    <t>Periode 3</t>
+  </si>
+  <si>
+    <t>Periode 4</t>
+  </si>
+  <si>
+    <t>Periode 5</t>
+  </si>
+  <si>
+    <t>Periode 6</t>
+  </si>
+  <si>
+    <t>Periode 7</t>
+  </si>
+  <si>
+    <t>Periode 8</t>
+  </si>
+  <si>
+    <t>Periode 9</t>
+  </si>
+  <si>
+    <t>Periode 10</t>
+  </si>
+  <si>
+    <t>Periode 11</t>
+  </si>
+  <si>
+    <t>Periode 12</t>
+  </si>
+  <si>
+    <t>Periode 13</t>
+  </si>
+  <si>
+    <t>Periode 14</t>
+  </si>
+  <si>
+    <t>Periode 15</t>
+  </si>
+  <si>
+    <t>Periode 16</t>
+  </si>
+  <si>
+    <t>Periode 17</t>
+  </si>
+  <si>
+    <t>Periode 18</t>
+  </si>
+  <si>
+    <t>Periode 19</t>
+  </si>
+  <si>
+    <t>Periode 20</t>
+  </si>
+  <si>
+    <t>Periode 21</t>
+  </si>
+  <si>
+    <t>Periode 22</t>
+  </si>
+  <si>
+    <t>Periode 23</t>
+  </si>
+  <si>
+    <t>Periode 24</t>
+  </si>
+  <si>
+    <t>Periode 25</t>
+  </si>
+  <si>
+    <t>Periode 26</t>
+  </si>
+  <si>
+    <t>Periode 27</t>
+  </si>
+  <si>
+    <t>Periode 28</t>
+  </si>
+  <si>
+    <t>Periode 29</t>
+  </si>
+  <si>
+    <t>Periode 30</t>
+  </si>
+  <si>
+    <t>Periode 31</t>
+  </si>
+  <si>
+    <t>Periode 32</t>
+  </si>
+  <si>
+    <t>Periode 33</t>
+  </si>
+  <si>
+    <t>Periode 34</t>
+  </si>
+  <si>
+    <t>Periode 35</t>
+  </si>
+  <si>
+    <t>Periode 36</t>
+  </si>
+  <si>
+    <t>Periode</t>
+  </si>
+  <si>
+    <t>Waehrung</t>
+  </si>
+  <si>
+    <t>Betrag</t>
+  </si>
+  <si>
+    <t>Datum</t>
+  </si>
+  <si>
+    <t>GESAMT</t>
   </si>
 </sst>
 </file>
@@ -899,7 +1026,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="44">
     <border>
       <left/>
       <right/>
@@ -1353,11 +1480,53 @@
         <color rgb="FFD3D3D3"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
@@ -1595,6 +1764,78 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="21" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="7" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="41" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="42" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="43" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="38" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="39" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="39" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="19" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="41" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="42" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="7" borderId="42" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="43" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1855,6 +2096,19 @@
     <tableColumn id="3" name="Betrag (EUR)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TblKMWMittel" displayName="TblKMWMittel" ref="B4:E22">
+  <autoFilter ref="B4:E22"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Periode"/>
+    <tableColumn id="2" name="Waehrung"/>
+    <tableColumn id="3" name="Betrag"/>
+    <tableColumn id="4" name="Datum"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3784,4 +4038,315 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr>
+    <tabColor rgb="FFFF00"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="2" min="2" width="15"/>
+    <col customWidth="true" max="3" min="3" width="10"/>
+    <col customWidth="true" max="4" min="4" width="20"/>
+    <col customWidth="true" max="5" min="5" width="15"/>
+    <col customWidth="true" hidden="true" max="26" min="26" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="Z1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="true">
+      <c r="B2" s="80" t="s">
+        <v>225</v>
+      </c>
+      <c r="C2" s="80"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="Z2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="Z3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="true">
+      <c r="B4" s="87" t="s">
+        <v>262</v>
+      </c>
+      <c r="C4" s="88" t="s">
+        <v>263</v>
+      </c>
+      <c r="D4" s="88" t="s">
+        <v>264</v>
+      </c>
+      <c r="E4" s="89" t="s">
+        <v>265</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="90"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="93"/>
+      <c r="Z5" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="94"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="95"/>
+      <c r="Z6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="94"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="95"/>
+      <c r="Z7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="94"/>
+      <c r="C8" s="81"/>
+      <c r="D8" s="82"/>
+      <c r="E8" s="95"/>
+      <c r="Z8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="94"/>
+      <c r="C9" s="81"/>
+      <c r="D9" s="82"/>
+      <c r="E9" s="95"/>
+      <c r="Z9" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="94"/>
+      <c r="C10" s="81"/>
+      <c r="D10" s="82"/>
+      <c r="E10" s="95"/>
+      <c r="Z10" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="94"/>
+      <c r="C11" s="81"/>
+      <c r="D11" s="82"/>
+      <c r="E11" s="95"/>
+      <c r="Z11" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="94"/>
+      <c r="C12" s="81"/>
+      <c r="D12" s="82"/>
+      <c r="E12" s="95"/>
+      <c r="Z12" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="94"/>
+      <c r="C13" s="81"/>
+      <c r="D13" s="82"/>
+      <c r="E13" s="95"/>
+      <c r="Z13" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="94"/>
+      <c r="C14" s="81"/>
+      <c r="D14" s="82"/>
+      <c r="E14" s="95"/>
+      <c r="Z14" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="94"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="82"/>
+      <c r="E15" s="95"/>
+      <c r="Z15" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="94"/>
+      <c r="C16" s="81"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="95"/>
+      <c r="Z16" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="94"/>
+      <c r="C17" s="81"/>
+      <c r="D17" s="82"/>
+      <c r="E17" s="95"/>
+      <c r="Z17" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="94"/>
+      <c r="C18" s="81"/>
+      <c r="D18" s="82"/>
+      <c r="E18" s="95"/>
+      <c r="Z18" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="94"/>
+      <c r="C19" s="81"/>
+      <c r="D19" s="82"/>
+      <c r="E19" s="95"/>
+      <c r="Z19" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="94"/>
+      <c r="C20" s="81"/>
+      <c r="D20" s="82"/>
+      <c r="E20" s="95"/>
+      <c r="Z20" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="94"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="82"/>
+      <c r="E21" s="95"/>
+      <c r="Z21" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="96"/>
+      <c r="C22" s="97"/>
+      <c r="D22" s="98"/>
+      <c r="E22" s="99"/>
+      <c r="Z22" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="100" t="s">
+        <v>266</v>
+      </c>
+      <c r="C23" s="101"/>
+      <c r="D23" s="102" t="str">
+        <f>=SUBTOTAL(109,TblKMWMittel[Betrag])</f>
+      </c>
+      <c r="E23" s="103"/>
+      <c r="Z23" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="Z24" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="Z25" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="Z26" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="Z27" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="Z28" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="Z29" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="Z30" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="Z31" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="Z32" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="Z33" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="Z34" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="Z35" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="Z36" t="s">
+        <v>261</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" sqref="B5:B22" type="list">
+      <formula1>'II. KMW-Mittel'!$Z$1:$Z$36</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="C5:C22" type="list">
+      <formula1>"EUR,USD"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(vorpruefung): remove structured table references to prevent formula corruption in Finanzberichte
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -45,60 +45,60 @@
     <definedName name="Geber_Liste">='I. Budget'!$R$2#</definedName>
     <definedName name="Budget_ID_Liste">='I. Budget'!$S$2#</definedName>
     <definedName name="Reserve_Freigabe">'I. Budget'!$K$5</definedName>
-    <definedName name="FB_Kurs_1">'I. Budget'!$C$7</definedName>
-    <definedName name="FB_SaldoLC_1">'I. Budget'!$C$29</definedName>
-    <definedName name="FB_SaldoEUR_1">'I. Budget'!$D$29</definedName>
-    <definedName name="FB_Kurs_2">'I. Budget'!$J$7</definedName>
-    <definedName name="FB_SaldoLC_2">'I. Budget'!$J$29</definedName>
-    <definedName name="FB_SaldoEUR_2">'I. Budget'!$K$29</definedName>
-    <definedName name="FB_Kurs_3">'I. Budget'!$Q$7</definedName>
-    <definedName name="FB_SaldoLC_3">'I. Budget'!$Q$29</definedName>
-    <definedName name="FB_SaldoEUR_3">'I. Budget'!$R$29</definedName>
-    <definedName name="FB_Kurs_4">'I. Budget'!$X$7</definedName>
-    <definedName name="FB_SaldoLC_4">'I. Budget'!$X$29</definedName>
-    <definedName name="FB_SaldoEUR_4">'I. Budget'!$Y$29</definedName>
-    <definedName name="FB_Kurs_5">'I. Budget'!$AE$7</definedName>
-    <definedName name="FB_SaldoLC_5">'I. Budget'!$AE$29</definedName>
-    <definedName name="FB_SaldoEUR_5">'I. Budget'!$AF$29</definedName>
-    <definedName name="FB_Kurs_6">'I. Budget'!$AL$7</definedName>
-    <definedName name="FB_SaldoLC_6">'I. Budget'!$AL$29</definedName>
-    <definedName name="FB_SaldoEUR_6">'I. Budget'!$AM$29</definedName>
-    <definedName name="FB_Kurs_7">'I. Budget'!$AS$7</definedName>
-    <definedName name="FB_SaldoLC_7">'I. Budget'!$AS$29</definedName>
-    <definedName name="FB_SaldoEUR_7">'I. Budget'!$AT$29</definedName>
-    <definedName name="FB_Kurs_8">'I. Budget'!$AZ$7</definedName>
-    <definedName name="FB_SaldoLC_8">'I. Budget'!$AZ$29</definedName>
-    <definedName name="FB_SaldoEUR_8">'I. Budget'!$BA$29</definedName>
-    <definedName name="FB_Kurs_9">'I. Budget'!$BG$7</definedName>
-    <definedName name="FB_SaldoLC_9">'I. Budget'!$BG$29</definedName>
-    <definedName name="FB_SaldoEUR_9">'I. Budget'!$BH$29</definedName>
-    <definedName name="FB_Kurs_10">'I. Budget'!$BN$7</definedName>
-    <definedName name="FB_SaldoLC_10">'I. Budget'!$BN$29</definedName>
-    <definedName name="FB_SaldoEUR_10">'I. Budget'!$BO$29</definedName>
-    <definedName name="FB_Kurs_11">'I. Budget'!$BU$7</definedName>
-    <definedName name="FB_SaldoLC_11">'I. Budget'!$BU$29</definedName>
-    <definedName name="FB_SaldoEUR_11">'I. Budget'!$BV$29</definedName>
-    <definedName name="FB_Kurs_12">'I. Budget'!$CB$7</definedName>
-    <definedName name="FB_SaldoLC_12">'I. Budget'!$CB$29</definedName>
-    <definedName name="FB_SaldoEUR_12">'I. Budget'!$CC$29</definedName>
-    <definedName name="FB_Kurs_13">'I. Budget'!$CI$7</definedName>
-    <definedName name="FB_SaldoLC_13">'I. Budget'!$CI$29</definedName>
-    <definedName name="FB_SaldoEUR_13">'I. Budget'!$CJ$29</definedName>
-    <definedName name="FB_Kurs_14">'I. Budget'!$CP$7</definedName>
-    <definedName name="FB_SaldoLC_14">'I. Budget'!$CP$29</definedName>
-    <definedName name="FB_SaldoEUR_14">'I. Budget'!$CQ$29</definedName>
-    <definedName name="FB_Kurs_15">'I. Budget'!$CW$7</definedName>
-    <definedName name="FB_SaldoLC_15">'I. Budget'!$CW$29</definedName>
-    <definedName name="FB_SaldoEUR_15">'I. Budget'!$CX$29</definedName>
-    <definedName name="FB_Kurs_16">'I. Budget'!$DD$7</definedName>
-    <definedName name="FB_SaldoLC_16">'I. Budget'!$DD$29</definedName>
-    <definedName name="FB_SaldoEUR_16">'I. Budget'!$DE$29</definedName>
-    <definedName name="FB_Kurs_17">'I. Budget'!$DK$7</definedName>
-    <definedName name="FB_SaldoLC_17">'I. Budget'!$DK$29</definedName>
-    <definedName name="FB_SaldoEUR_17">'I. Budget'!$DL$29</definedName>
-    <definedName name="FB_Kurs_18">'I. Budget'!$DR$7</definedName>
-    <definedName name="FB_SaldoLC_18">'I. Budget'!$DR$29</definedName>
-    <definedName name="FB_SaldoEUR_18">'I. Budget'!$DS$29</definedName>
+    <definedName name="FB_Kurs_1">'III. Finanzberichte'!$C$7</definedName>
+    <definedName name="FB_SaldoLC_1">'III. Finanzberichte'!$C$29</definedName>
+    <definedName name="FB_SaldoEUR_1">'III. Finanzberichte'!$D$29</definedName>
+    <definedName name="FB_Kurs_2">'III. Finanzberichte'!$J$7</definedName>
+    <definedName name="FB_SaldoLC_2">'III. Finanzberichte'!$J$29</definedName>
+    <definedName name="FB_SaldoEUR_2">'III. Finanzberichte'!$K$29</definedName>
+    <definedName name="FB_Kurs_3">'III. Finanzberichte'!$Q$7</definedName>
+    <definedName name="FB_SaldoLC_3">'III. Finanzberichte'!$Q$29</definedName>
+    <definedName name="FB_SaldoEUR_3">'III. Finanzberichte'!$R$29</definedName>
+    <definedName name="FB_Kurs_4">'III. Finanzberichte'!$X$7</definedName>
+    <definedName name="FB_SaldoLC_4">'III. Finanzberichte'!$X$29</definedName>
+    <definedName name="FB_SaldoEUR_4">'III. Finanzberichte'!$Y$29</definedName>
+    <definedName name="FB_Kurs_5">'III. Finanzberichte'!$AE$7</definedName>
+    <definedName name="FB_SaldoLC_5">'III. Finanzberichte'!$AE$29</definedName>
+    <definedName name="FB_SaldoEUR_5">'III. Finanzberichte'!$AF$29</definedName>
+    <definedName name="FB_Kurs_6">'III. Finanzberichte'!$AL$7</definedName>
+    <definedName name="FB_SaldoLC_6">'III. Finanzberichte'!$AL$29</definedName>
+    <definedName name="FB_SaldoEUR_6">'III. Finanzberichte'!$AM$29</definedName>
+    <definedName name="FB_Kurs_7">'III. Finanzberichte'!$AS$7</definedName>
+    <definedName name="FB_SaldoLC_7">'III. Finanzberichte'!$AS$29</definedName>
+    <definedName name="FB_SaldoEUR_7">'III. Finanzberichte'!$AT$29</definedName>
+    <definedName name="FB_Kurs_8">'III. Finanzberichte'!$AZ$7</definedName>
+    <definedName name="FB_SaldoLC_8">'III. Finanzberichte'!$AZ$29</definedName>
+    <definedName name="FB_SaldoEUR_8">'III. Finanzberichte'!$BA$29</definedName>
+    <definedName name="FB_Kurs_9">'III. Finanzberichte'!$BG$7</definedName>
+    <definedName name="FB_SaldoLC_9">'III. Finanzberichte'!$BG$29</definedName>
+    <definedName name="FB_SaldoEUR_9">'III. Finanzberichte'!$BH$29</definedName>
+    <definedName name="FB_Kurs_10">'III. Finanzberichte'!$BN$7</definedName>
+    <definedName name="FB_SaldoLC_10">'III. Finanzberichte'!$BN$29</definedName>
+    <definedName name="FB_SaldoEUR_10">'III. Finanzberichte'!$BO$29</definedName>
+    <definedName name="FB_Kurs_11">'III. Finanzberichte'!$BU$7</definedName>
+    <definedName name="FB_SaldoLC_11">'III. Finanzberichte'!$BU$29</definedName>
+    <definedName name="FB_SaldoEUR_11">'III. Finanzberichte'!$BV$29</definedName>
+    <definedName name="FB_Kurs_12">'III. Finanzberichte'!$CB$7</definedName>
+    <definedName name="FB_SaldoLC_12">'III. Finanzberichte'!$CB$29</definedName>
+    <definedName name="FB_SaldoEUR_12">'III. Finanzberichte'!$CC$29</definedName>
+    <definedName name="FB_Kurs_13">'III. Finanzberichte'!$CI$7</definedName>
+    <definedName name="FB_SaldoLC_13">'III. Finanzberichte'!$CI$29</definedName>
+    <definedName name="FB_SaldoEUR_13">'III. Finanzberichte'!$CJ$29</definedName>
+    <definedName name="FB_Kurs_14">'III. Finanzberichte'!$CP$7</definedName>
+    <definedName name="FB_SaldoLC_14">'III. Finanzberichte'!$CP$29</definedName>
+    <definedName name="FB_SaldoEUR_14">'III. Finanzberichte'!$CQ$29</definedName>
+    <definedName name="FB_Kurs_15">'III. Finanzberichte'!$CW$7</definedName>
+    <definedName name="FB_SaldoLC_15">'III. Finanzberichte'!$CW$29</definedName>
+    <definedName name="FB_SaldoEUR_15">'III. Finanzberichte'!$CX$29</definedName>
+    <definedName name="FB_Kurs_16">'III. Finanzberichte'!$DD$7</definedName>
+    <definedName name="FB_SaldoLC_16">'III. Finanzberichte'!$DD$29</definedName>
+    <definedName name="FB_SaldoEUR_16">'III. Finanzberichte'!$DE$29</definedName>
+    <definedName name="FB_Kurs_17">'III. Finanzberichte'!$DK$7</definedName>
+    <definedName name="FB_SaldoLC_17">'III. Finanzberichte'!$DK$29</definedName>
+    <definedName name="FB_SaldoEUR_17">'III. Finanzberichte'!$DL$29</definedName>
+    <definedName name="FB_Kurs_18">'III. Finanzberichte'!$DR$7</definedName>
+    <definedName name="FB_SaldoLC_18">'III. Finanzberichte'!$DR$29</definedName>
+    <definedName name="FB_SaldoEUR_18">'III. Finanzberichte'!$DS$29</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
@@ -5966,7 +5966,7 @@
         <v>269</v>
       </c>
       <c r="C7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_1[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(F46,0),6)</f>
         <v>158</v>
       </c>
       <c r="D7" s="110"/>
@@ -5975,7 +5975,7 @@
         <v>269</v>
       </c>
       <c r="J7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_2[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(M46,0),6)</f>
         <v>158</v>
       </c>
       <c r="K7" s="110"/>
@@ -5984,7 +5984,7 @@
         <v>269</v>
       </c>
       <c r="Q7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_3[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(T46,0),6)</f>
         <v>158</v>
       </c>
       <c r="R7" s="110"/>
@@ -5993,7 +5993,7 @@
         <v>269</v>
       </c>
       <c r="X7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_4[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(AA46,0),6)</f>
         <v>158</v>
       </c>
       <c r="Y7" s="110"/>
@@ -6002,7 +6002,7 @@
         <v>269</v>
       </c>
       <c r="AE7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_5[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(AH46,0),6)</f>
         <v>158</v>
       </c>
       <c r="AF7" s="110"/>
@@ -6011,7 +6011,7 @@
         <v>269</v>
       </c>
       <c r="AL7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_6[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(AO46,0),6)</f>
         <v>158</v>
       </c>
       <c r="AM7" s="110"/>
@@ -6020,7 +6020,7 @@
         <v>269</v>
       </c>
       <c r="AS7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_7[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(AV46,0),6)</f>
         <v>158</v>
       </c>
       <c r="AT7" s="110"/>
@@ -6029,7 +6029,7 @@
         <v>269</v>
       </c>
       <c r="AZ7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_8[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(BC46,0),6)</f>
         <v>158</v>
       </c>
       <c r="BA7" s="110"/>
@@ -6038,7 +6038,7 @@
         <v>269</v>
       </c>
       <c r="BG7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_9[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(BJ46,0),6)</f>
         <v>158</v>
       </c>
       <c r="BH7" s="110"/>
@@ -6047,7 +6047,7 @@
         <v>269</v>
       </c>
       <c r="BN7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_10[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(BQ46,0),6)</f>
         <v>158</v>
       </c>
       <c r="BO7" s="110"/>
@@ -6056,7 +6056,7 @@
         <v>269</v>
       </c>
       <c r="BU7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_11[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(BX46,0),6)</f>
         <v>158</v>
       </c>
       <c r="BV7" s="110"/>
@@ -6065,7 +6065,7 @@
         <v>269</v>
       </c>
       <c r="CB7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_12[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(CE46,0),6)</f>
         <v>158</v>
       </c>
       <c r="CC7" s="110"/>
@@ -6074,7 +6074,7 @@
         <v>269</v>
       </c>
       <c r="CI7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_13[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(CL46,0),6)</f>
         <v>158</v>
       </c>
       <c r="CJ7" s="110"/>
@@ -6083,7 +6083,7 @@
         <v>269</v>
       </c>
       <c r="CP7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_14[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(CS46,0),6)</f>
         <v>158</v>
       </c>
       <c r="CQ7" s="110"/>
@@ -6092,7 +6092,7 @@
         <v>269</v>
       </c>
       <c r="CW7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_15[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(CZ46,0),6)</f>
         <v>158</v>
       </c>
       <c r="CX7" s="110"/>
@@ -6101,7 +6101,7 @@
         <v>269</v>
       </c>
       <c r="DD7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_16[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(DG46,0),6)</f>
         <v>158</v>
       </c>
       <c r="DE7" s="110"/>
@@ -6110,7 +6110,7 @@
         <v>269</v>
       </c>
       <c r="DK7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_17[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(DN46,0),6)</f>
         <v>158</v>
       </c>
       <c r="DL7" s="110"/>
@@ -6119,7 +6119,7 @@
         <v>269</v>
       </c>
       <c r="DR7" s="110" t="str">
-        <f>=ROUND(IFERROR(Einnahmen_18[[#Totals],[Kurs]],0),6)</f>
+        <f>=ROUND(IFERROR(DU46,0),6)</f>
         <v>158</v>
       </c>
       <c r="DS7" s="110"/>
@@ -8597,1890 +8597,1890 @@
     </row>
     <row r="19">
       <c r="B19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C19" s="24"/>
       <c r="D19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C19/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C19, 0)</f>
       </c>
       <c r="F19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D19, 0)</f>
       </c>
       <c r="I19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J19" s="24"/>
       <c r="K19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J19/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J19 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I19), J19)</f>
       </c>
       <c r="M19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K19 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I19), K19)</f>
       </c>
       <c r="P19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q19" s="24"/>
       <c r="R19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q19/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q19 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P19), Q19)</f>
       </c>
       <c r="T19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R19 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P19), R19)</f>
       </c>
       <c r="W19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X19" s="24"/>
       <c r="Y19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X19/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X19 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W19), X19)</f>
       </c>
       <c r="AA19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y19 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W19), Y19)</f>
       </c>
       <c r="AD19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE19" s="24"/>
       <c r="AF19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE19/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE19 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD19), AE19)</f>
       </c>
       <c r="AH19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF19 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD19), AF19)</f>
       </c>
       <c r="AK19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL19" s="24"/>
       <c r="AM19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL19/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL19 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK19), AL19)</f>
       </c>
       <c r="AO19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM19 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK19), AM19)</f>
       </c>
       <c r="AR19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS19" s="24"/>
       <c r="AT19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS19/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS19 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR19), AS19)</f>
       </c>
       <c r="AV19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT19 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR19), AT19)</f>
       </c>
       <c r="AY19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ19" s="24"/>
       <c r="BA19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ19/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ19 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY19), AZ19)</f>
       </c>
       <c r="BC19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA19 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY19), BA19)</f>
       </c>
       <c r="BF19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG19" s="24"/>
       <c r="BH19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG19/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG19 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF19), BG19)</f>
       </c>
       <c r="BJ19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH19 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF19), BH19)</f>
       </c>
       <c r="BM19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN19" s="24"/>
       <c r="BO19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN19/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN19 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM19), BN19)</f>
       </c>
       <c r="BQ19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO19 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM19), BO19)</f>
       </c>
       <c r="BT19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU19" s="24"/>
       <c r="BV19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU19/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU19 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT19), BU19)</f>
       </c>
       <c r="BX19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV19 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT19), BV19)</f>
       </c>
       <c r="CA19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB19" s="24"/>
       <c r="CC19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB19/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB19 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA19), CB19)</f>
       </c>
       <c r="CE19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC19 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA19), CC19)</f>
       </c>
       <c r="CH19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI19" s="24"/>
       <c r="CJ19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI19/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI19 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH19), CI19)</f>
       </c>
       <c r="CL19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ19 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH19), CJ19)</f>
       </c>
       <c r="CO19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP19" s="24"/>
       <c r="CQ19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP19/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP19 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO19), CP19)</f>
       </c>
       <c r="CS19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ19 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO19), CQ19)</f>
       </c>
       <c r="CV19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW19" s="24"/>
       <c r="CX19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW19/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW19 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV19), CW19)</f>
       </c>
       <c r="CZ19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX19 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV19), CX19)</f>
       </c>
       <c r="DC19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD19" s="24"/>
       <c r="DE19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD19/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD19 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC19), DD19)</f>
       </c>
       <c r="DG19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE19 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC19), DE19)</f>
       </c>
       <c r="DJ19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK19" s="24"/>
       <c r="DL19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK19/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK19 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ19), DK19)</f>
       </c>
       <c r="DN19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL19 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ19), DL19)</f>
       </c>
       <c r="DQ19" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR19" s="24"/>
       <c r="DS19" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR19/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT19" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR19 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ19), DR19)</f>
       </c>
       <c r="DU19" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS19 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ19), DS19)</f>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C20" s="24"/>
       <c r="D20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C20/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C20, 0)</f>
       </c>
       <c r="F20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D20, 0)</f>
       </c>
       <c r="I20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J20" s="24"/>
       <c r="K20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J20/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J20 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I20), J20)</f>
       </c>
       <c r="M20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K20 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I20), K20)</f>
       </c>
       <c r="P20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q20" s="24"/>
       <c r="R20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q20/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q20 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P20), Q20)</f>
       </c>
       <c r="T20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R20 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P20), R20)</f>
       </c>
       <c r="W20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X20" s="24"/>
       <c r="Y20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X20/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X20 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W20), X20)</f>
       </c>
       <c r="AA20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y20 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W20), Y20)</f>
       </c>
       <c r="AD20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE20" s="24"/>
       <c r="AF20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE20/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE20 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD20), AE20)</f>
       </c>
       <c r="AH20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF20 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD20), AF20)</f>
       </c>
       <c r="AK20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL20" s="24"/>
       <c r="AM20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL20/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL20 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK20), AL20)</f>
       </c>
       <c r="AO20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM20 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK20), AM20)</f>
       </c>
       <c r="AR20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS20" s="24"/>
       <c r="AT20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS20/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS20 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR20), AS20)</f>
       </c>
       <c r="AV20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT20 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR20), AT20)</f>
       </c>
       <c r="AY20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ20" s="24"/>
       <c r="BA20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ20/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ20 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY20), AZ20)</f>
       </c>
       <c r="BC20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA20 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY20), BA20)</f>
       </c>
       <c r="BF20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG20" s="24"/>
       <c r="BH20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG20/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG20 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF20), BG20)</f>
       </c>
       <c r="BJ20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH20 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF20), BH20)</f>
       </c>
       <c r="BM20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN20" s="24"/>
       <c r="BO20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN20/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN20 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM20), BN20)</f>
       </c>
       <c r="BQ20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO20 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM20), BO20)</f>
       </c>
       <c r="BT20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU20" s="24"/>
       <c r="BV20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU20/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU20 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT20), BU20)</f>
       </c>
       <c r="BX20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV20 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT20), BV20)</f>
       </c>
       <c r="CA20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB20" s="24"/>
       <c r="CC20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB20/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB20 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA20), CB20)</f>
       </c>
       <c r="CE20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC20 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA20), CC20)</f>
       </c>
       <c r="CH20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI20" s="24"/>
       <c r="CJ20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI20/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI20 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH20), CI20)</f>
       </c>
       <c r="CL20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ20 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH20), CJ20)</f>
       </c>
       <c r="CO20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP20" s="24"/>
       <c r="CQ20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP20/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP20 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO20), CP20)</f>
       </c>
       <c r="CS20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ20 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO20), CQ20)</f>
       </c>
       <c r="CV20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW20" s="24"/>
       <c r="CX20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW20/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW20 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV20), CW20)</f>
       </c>
       <c r="CZ20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX20 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV20), CX20)</f>
       </c>
       <c r="DC20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD20" s="24"/>
       <c r="DE20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD20/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD20 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC20), DD20)</f>
       </c>
       <c r="DG20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE20 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC20), DE20)</f>
       </c>
       <c r="DJ20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK20" s="24"/>
       <c r="DL20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK20/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK20 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ20), DK20)</f>
       </c>
       <c r="DN20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL20 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ20), DL20)</f>
       </c>
       <c r="DQ20" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR20" s="24"/>
       <c r="DS20" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR20/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT20" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR20 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ20), DR20)</f>
       </c>
       <c r="DU20" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS20 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ20), DS20)</f>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C21" s="24"/>
       <c r="D21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C21/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C21, 0)</f>
       </c>
       <c r="F21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D21, 0)</f>
       </c>
       <c r="I21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J21" s="24"/>
       <c r="K21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J21/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J21 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I21), J21)</f>
       </c>
       <c r="M21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K21 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I21), K21)</f>
       </c>
       <c r="P21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q21" s="24"/>
       <c r="R21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q21/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q21 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P21), Q21)</f>
       </c>
       <c r="T21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R21 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P21), R21)</f>
       </c>
       <c r="W21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X21" s="24"/>
       <c r="Y21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X21/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X21 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W21), X21)</f>
       </c>
       <c r="AA21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y21 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W21), Y21)</f>
       </c>
       <c r="AD21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE21" s="24"/>
       <c r="AF21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE21/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE21 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD21), AE21)</f>
       </c>
       <c r="AH21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF21 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD21), AF21)</f>
       </c>
       <c r="AK21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL21" s="24"/>
       <c r="AM21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL21/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL21 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK21), AL21)</f>
       </c>
       <c r="AO21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM21 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK21), AM21)</f>
       </c>
       <c r="AR21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS21" s="24"/>
       <c r="AT21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS21/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS21 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR21), AS21)</f>
       </c>
       <c r="AV21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT21 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR21), AT21)</f>
       </c>
       <c r="AY21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ21" s="24"/>
       <c r="BA21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ21/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ21 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY21), AZ21)</f>
       </c>
       <c r="BC21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA21 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY21), BA21)</f>
       </c>
       <c r="BF21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG21" s="24"/>
       <c r="BH21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG21/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG21 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF21), BG21)</f>
       </c>
       <c r="BJ21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH21 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF21), BH21)</f>
       </c>
       <c r="BM21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN21" s="24"/>
       <c r="BO21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN21/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN21 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM21), BN21)</f>
       </c>
       <c r="BQ21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO21 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM21), BO21)</f>
       </c>
       <c r="BT21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU21" s="24"/>
       <c r="BV21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU21/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU21 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT21), BU21)</f>
       </c>
       <c r="BX21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV21 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT21), BV21)</f>
       </c>
       <c r="CA21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB21" s="24"/>
       <c r="CC21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB21/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB21 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA21), CB21)</f>
       </c>
       <c r="CE21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC21 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA21), CC21)</f>
       </c>
       <c r="CH21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI21" s="24"/>
       <c r="CJ21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI21/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI21 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH21), CI21)</f>
       </c>
       <c r="CL21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ21 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH21), CJ21)</f>
       </c>
       <c r="CO21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP21" s="24"/>
       <c r="CQ21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP21/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP21 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO21), CP21)</f>
       </c>
       <c r="CS21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ21 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO21), CQ21)</f>
       </c>
       <c r="CV21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW21" s="24"/>
       <c r="CX21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW21/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW21 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV21), CW21)</f>
       </c>
       <c r="CZ21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX21 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV21), CX21)</f>
       </c>
       <c r="DC21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD21" s="24"/>
       <c r="DE21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD21/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD21 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC21), DD21)</f>
       </c>
       <c r="DG21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE21 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC21), DE21)</f>
       </c>
       <c r="DJ21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK21" s="24"/>
       <c r="DL21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK21/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK21 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ21), DK21)</f>
       </c>
       <c r="DN21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL21 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ21), DL21)</f>
       </c>
       <c r="DQ21" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR21" s="24"/>
       <c r="DS21" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR21/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT21" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR21 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ21), DR21)</f>
       </c>
       <c r="DU21" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS21 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ21), DS21)</f>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C22" s="24"/>
       <c r="D22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C22/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C22, 0)</f>
       </c>
       <c r="F22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D22, 0)</f>
       </c>
       <c r="I22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J22" s="24"/>
       <c r="K22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J22/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J22 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I22), J22)</f>
       </c>
       <c r="M22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K22 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I22), K22)</f>
       </c>
       <c r="P22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q22" s="24"/>
       <c r="R22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q22/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q22 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P22), Q22)</f>
       </c>
       <c r="T22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R22 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P22), R22)</f>
       </c>
       <c r="W22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X22" s="24"/>
       <c r="Y22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X22/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X22 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W22), X22)</f>
       </c>
       <c r="AA22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y22 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W22), Y22)</f>
       </c>
       <c r="AD22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE22" s="24"/>
       <c r="AF22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE22/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE22 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD22), AE22)</f>
       </c>
       <c r="AH22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF22 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD22), AF22)</f>
       </c>
       <c r="AK22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL22" s="24"/>
       <c r="AM22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL22/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL22 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK22), AL22)</f>
       </c>
       <c r="AO22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM22 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK22), AM22)</f>
       </c>
       <c r="AR22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS22" s="24"/>
       <c r="AT22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS22/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS22 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR22), AS22)</f>
       </c>
       <c r="AV22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT22 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR22), AT22)</f>
       </c>
       <c r="AY22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ22" s="24"/>
       <c r="BA22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ22/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ22 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY22), AZ22)</f>
       </c>
       <c r="BC22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA22 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY22), BA22)</f>
       </c>
       <c r="BF22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG22" s="24"/>
       <c r="BH22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG22/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG22 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF22), BG22)</f>
       </c>
       <c r="BJ22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH22 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF22), BH22)</f>
       </c>
       <c r="BM22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN22" s="24"/>
       <c r="BO22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN22/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN22 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM22), BN22)</f>
       </c>
       <c r="BQ22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO22 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM22), BO22)</f>
       </c>
       <c r="BT22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU22" s="24"/>
       <c r="BV22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU22/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU22 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT22), BU22)</f>
       </c>
       <c r="BX22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV22 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT22), BV22)</f>
       </c>
       <c r="CA22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB22" s="24"/>
       <c r="CC22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB22/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB22 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA22), CB22)</f>
       </c>
       <c r="CE22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC22 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA22), CC22)</f>
       </c>
       <c r="CH22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI22" s="24"/>
       <c r="CJ22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI22/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI22 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH22), CI22)</f>
       </c>
       <c r="CL22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ22 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH22), CJ22)</f>
       </c>
       <c r="CO22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP22" s="24"/>
       <c r="CQ22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP22/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP22 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO22), CP22)</f>
       </c>
       <c r="CS22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ22 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO22), CQ22)</f>
       </c>
       <c r="CV22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW22" s="24"/>
       <c r="CX22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW22/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW22 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV22), CW22)</f>
       </c>
       <c r="CZ22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX22 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV22), CX22)</f>
       </c>
       <c r="DC22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD22" s="24"/>
       <c r="DE22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD22/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD22 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC22), DD22)</f>
       </c>
       <c r="DG22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE22 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC22), DE22)</f>
       </c>
       <c r="DJ22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK22" s="24"/>
       <c r="DL22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK22/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK22 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ22), DK22)</f>
       </c>
       <c r="DN22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL22 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ22), DL22)</f>
       </c>
       <c r="DQ22" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR22" s="24"/>
       <c r="DS22" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR22/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT22" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR22 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ22), DR22)</f>
       </c>
       <c r="DU22" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS22 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ22), DS22)</f>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C23" s="24"/>
       <c r="D23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C23/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C23, 0)</f>
       </c>
       <c r="F23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D23, 0)</f>
       </c>
       <c r="I23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J23" s="24"/>
       <c r="K23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J23/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J23 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I23), J23)</f>
       </c>
       <c r="M23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K23 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I23), K23)</f>
       </c>
       <c r="P23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q23" s="24"/>
       <c r="R23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q23/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q23 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P23), Q23)</f>
       </c>
       <c r="T23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R23 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P23), R23)</f>
       </c>
       <c r="W23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X23" s="24"/>
       <c r="Y23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X23/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X23 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W23), X23)</f>
       </c>
       <c r="AA23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y23 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W23), Y23)</f>
       </c>
       <c r="AD23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE23" s="24"/>
       <c r="AF23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE23/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE23 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD23), AE23)</f>
       </c>
       <c r="AH23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF23 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD23), AF23)</f>
       </c>
       <c r="AK23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL23" s="24"/>
       <c r="AM23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL23/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL23 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK23), AL23)</f>
       </c>
       <c r="AO23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM23 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK23), AM23)</f>
       </c>
       <c r="AR23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS23" s="24"/>
       <c r="AT23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS23/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS23 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR23), AS23)</f>
       </c>
       <c r="AV23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT23 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR23), AT23)</f>
       </c>
       <c r="AY23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ23" s="24"/>
       <c r="BA23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ23/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ23 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY23), AZ23)</f>
       </c>
       <c r="BC23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA23 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY23), BA23)</f>
       </c>
       <c r="BF23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG23" s="24"/>
       <c r="BH23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG23/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG23 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF23), BG23)</f>
       </c>
       <c r="BJ23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH23 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF23), BH23)</f>
       </c>
       <c r="BM23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN23" s="24"/>
       <c r="BO23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN23/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN23 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM23), BN23)</f>
       </c>
       <c r="BQ23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO23 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM23), BO23)</f>
       </c>
       <c r="BT23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU23" s="24"/>
       <c r="BV23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU23/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU23 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT23), BU23)</f>
       </c>
       <c r="BX23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV23 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT23), BV23)</f>
       </c>
       <c r="CA23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB23" s="24"/>
       <c r="CC23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB23/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB23 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA23), CB23)</f>
       </c>
       <c r="CE23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC23 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA23), CC23)</f>
       </c>
       <c r="CH23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI23" s="24"/>
       <c r="CJ23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI23/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI23 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH23), CI23)</f>
       </c>
       <c r="CL23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ23 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH23), CJ23)</f>
       </c>
       <c r="CO23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP23" s="24"/>
       <c r="CQ23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP23/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP23 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO23), CP23)</f>
       </c>
       <c r="CS23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ23 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO23), CQ23)</f>
       </c>
       <c r="CV23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW23" s="24"/>
       <c r="CX23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW23/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW23 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV23), CW23)</f>
       </c>
       <c r="CZ23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX23 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV23), CX23)</f>
       </c>
       <c r="DC23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD23" s="24"/>
       <c r="DE23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD23/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD23 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC23), DD23)</f>
       </c>
       <c r="DG23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE23 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC23), DE23)</f>
       </c>
       <c r="DJ23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK23" s="24"/>
       <c r="DL23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK23/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK23 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ23), DK23)</f>
       </c>
       <c r="DN23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL23 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ23), DL23)</f>
       </c>
       <c r="DQ23" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR23" s="24"/>
       <c r="DS23" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR23/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT23" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR23 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ23), DR23)</f>
       </c>
       <c r="DU23" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS23 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ23), DS23)</f>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C24" s="24"/>
       <c r="D24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C24/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C24, 0)</f>
       </c>
       <c r="F24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D24, 0)</f>
       </c>
       <c r="I24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J24" s="24"/>
       <c r="K24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J24/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J24 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I24), J24)</f>
       </c>
       <c r="M24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K24 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I24), K24)</f>
       </c>
       <c r="P24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q24" s="24"/>
       <c r="R24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q24/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q24 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P24), Q24)</f>
       </c>
       <c r="T24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R24 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P24), R24)</f>
       </c>
       <c r="W24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X24" s="24"/>
       <c r="Y24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X24/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X24 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W24), X24)</f>
       </c>
       <c r="AA24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y24 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W24), Y24)</f>
       </c>
       <c r="AD24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE24" s="24"/>
       <c r="AF24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE24/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE24 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD24), AE24)</f>
       </c>
       <c r="AH24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF24 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD24), AF24)</f>
       </c>
       <c r="AK24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL24" s="24"/>
       <c r="AM24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL24/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL24 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK24), AL24)</f>
       </c>
       <c r="AO24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM24 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK24), AM24)</f>
       </c>
       <c r="AR24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS24" s="24"/>
       <c r="AT24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS24/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS24 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR24), AS24)</f>
       </c>
       <c r="AV24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT24 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR24), AT24)</f>
       </c>
       <c r="AY24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ24" s="24"/>
       <c r="BA24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ24/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ24 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY24), AZ24)</f>
       </c>
       <c r="BC24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA24 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY24), BA24)</f>
       </c>
       <c r="BF24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG24" s="24"/>
       <c r="BH24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG24/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG24 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF24), BG24)</f>
       </c>
       <c r="BJ24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH24 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF24), BH24)</f>
       </c>
       <c r="BM24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN24" s="24"/>
       <c r="BO24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN24/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN24 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM24), BN24)</f>
       </c>
       <c r="BQ24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO24 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM24), BO24)</f>
       </c>
       <c r="BT24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU24" s="24"/>
       <c r="BV24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU24/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU24 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT24), BU24)</f>
       </c>
       <c r="BX24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV24 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT24), BV24)</f>
       </c>
       <c r="CA24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB24" s="24"/>
       <c r="CC24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB24/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB24 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA24), CB24)</f>
       </c>
       <c r="CE24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC24 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA24), CC24)</f>
       </c>
       <c r="CH24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI24" s="24"/>
       <c r="CJ24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI24/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI24 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH24), CI24)</f>
       </c>
       <c r="CL24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ24 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH24), CJ24)</f>
       </c>
       <c r="CO24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP24" s="24"/>
       <c r="CQ24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP24/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP24 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO24), CP24)</f>
       </c>
       <c r="CS24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ24 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO24), CQ24)</f>
       </c>
       <c r="CV24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW24" s="24"/>
       <c r="CX24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW24/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW24 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV24), CW24)</f>
       </c>
       <c r="CZ24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX24 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV24), CX24)</f>
       </c>
       <c r="DC24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD24" s="24"/>
       <c r="DE24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD24/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD24 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC24), DD24)</f>
       </c>
       <c r="DG24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE24 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC24), DE24)</f>
       </c>
       <c r="DJ24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK24" s="24"/>
       <c r="DL24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK24/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK24 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ24), DK24)</f>
       </c>
       <c r="DN24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL24 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ24), DL24)</f>
       </c>
       <c r="DQ24" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR24" s="24"/>
       <c r="DS24" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR24/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT24" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR24 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ24), DR24)</f>
       </c>
       <c r="DU24" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS24 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ24), DS24)</f>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C25" s="24"/>
       <c r="D25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C25/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C25, 0)</f>
       </c>
       <c r="F25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D25, 0)</f>
       </c>
       <c r="I25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J25" s="24"/>
       <c r="K25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J25/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J25 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I25), J25)</f>
       </c>
       <c r="M25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K25 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I25), K25)</f>
       </c>
       <c r="P25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q25" s="24"/>
       <c r="R25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q25/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q25 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P25), Q25)</f>
       </c>
       <c r="T25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R25 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P25), R25)</f>
       </c>
       <c r="W25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X25" s="24"/>
       <c r="Y25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X25/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X25 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W25), X25)</f>
       </c>
       <c r="AA25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y25 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W25), Y25)</f>
       </c>
       <c r="AD25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE25" s="24"/>
       <c r="AF25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE25/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE25 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD25), AE25)</f>
       </c>
       <c r="AH25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF25 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD25), AF25)</f>
       </c>
       <c r="AK25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL25" s="24"/>
       <c r="AM25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL25/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL25 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK25), AL25)</f>
       </c>
       <c r="AO25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM25 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK25), AM25)</f>
       </c>
       <c r="AR25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS25" s="24"/>
       <c r="AT25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS25/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS25 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR25), AS25)</f>
       </c>
       <c r="AV25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT25 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR25), AT25)</f>
       </c>
       <c r="AY25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ25" s="24"/>
       <c r="BA25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ25/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ25 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY25), AZ25)</f>
       </c>
       <c r="BC25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA25 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY25), BA25)</f>
       </c>
       <c r="BF25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG25" s="24"/>
       <c r="BH25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG25/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG25 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF25), BG25)</f>
       </c>
       <c r="BJ25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH25 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF25), BH25)</f>
       </c>
       <c r="BM25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN25" s="24"/>
       <c r="BO25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN25/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN25 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM25), BN25)</f>
       </c>
       <c r="BQ25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO25 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM25), BO25)</f>
       </c>
       <c r="BT25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU25" s="24"/>
       <c r="BV25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU25/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU25 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT25), BU25)</f>
       </c>
       <c r="BX25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV25 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT25), BV25)</f>
       </c>
       <c r="CA25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB25" s="24"/>
       <c r="CC25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB25/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB25 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA25), CB25)</f>
       </c>
       <c r="CE25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC25 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA25), CC25)</f>
       </c>
       <c r="CH25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI25" s="24"/>
       <c r="CJ25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI25/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI25 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH25), CI25)</f>
       </c>
       <c r="CL25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ25 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH25), CJ25)</f>
       </c>
       <c r="CO25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP25" s="24"/>
       <c r="CQ25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP25/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP25 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO25), CP25)</f>
       </c>
       <c r="CS25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ25 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO25), CQ25)</f>
       </c>
       <c r="CV25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW25" s="24"/>
       <c r="CX25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW25/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW25 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV25), CW25)</f>
       </c>
       <c r="CZ25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX25 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV25), CX25)</f>
       </c>
       <c r="DC25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD25" s="24"/>
       <c r="DE25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD25/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD25 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC25), DD25)</f>
       </c>
       <c r="DG25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE25 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC25), DE25)</f>
       </c>
       <c r="DJ25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK25" s="24"/>
       <c r="DL25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK25/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK25 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ25), DK25)</f>
       </c>
       <c r="DN25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL25 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ25), DL25)</f>
       </c>
       <c r="DQ25" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR25" s="24"/>
       <c r="DS25" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR25/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT25" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR25 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ25), DR25)</f>
       </c>
       <c r="DU25" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS25 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ25), DS25)</f>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_1[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="C26" s="24"/>
       <c r="D26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_1,2),0)</f>
+        <f>=IFERROR(ROUND(C26/FB_Kurs_1,2),0)</f>
       </c>
       <c r="E26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]], 0)</f>
+        <f>=IFERROR(C26, 0)</f>
       </c>
       <c r="F26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]], 0)</f>
+        <f>=IFERROR(D26, 0)</f>
       </c>
       <c r="I26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_2[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="J26" s="24"/>
       <c r="K26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_2,2),0)</f>
+        <f>=IFERROR(ROUND(J26/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(J26 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I26), J26)</f>
       </c>
       <c r="M26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(K26 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I26), K26)</f>
       </c>
       <c r="P26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_3[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="Q26" s="24"/>
       <c r="R26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_3,2),0)</f>
+        <f>=IFERROR(ROUND(Q26/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(Q26 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P26), Q26)</f>
       </c>
       <c r="T26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(R26 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P26), R26)</f>
       </c>
       <c r="W26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_4[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="X26" s="24"/>
       <c r="Y26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_4,2),0)</f>
+        <f>=IFERROR(ROUND(X26/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(X26 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W26), X26)</f>
       </c>
       <c r="AA26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(Y26 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W26), Y26)</f>
       </c>
       <c r="AD26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_5[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AE26" s="24"/>
       <c r="AF26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_5,2),0)</f>
+        <f>=IFERROR(ROUND(AE26/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AE26 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD26), AE26)</f>
       </c>
       <c r="AH26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AF26 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD26), AF26)</f>
       </c>
       <c r="AK26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_6[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AL26" s="24"/>
       <c r="AM26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_6,2),0)</f>
+        <f>=IFERROR(ROUND(AL26/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AL26 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK26), AL26)</f>
       </c>
       <c r="AO26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AM26 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK26), AM26)</f>
       </c>
       <c r="AR26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_7[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AS26" s="24"/>
       <c r="AT26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_7,2),0)</f>
+        <f>=IFERROR(ROUND(AS26/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AS26 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR26), AS26)</f>
       </c>
       <c r="AV26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(AT26 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR26), AT26)</f>
       </c>
       <c r="AY26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_8[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="AZ26" s="24"/>
       <c r="BA26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_8,2),0)</f>
+        <f>=IFERROR(ROUND(AZ26/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(AZ26 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY26), AZ26)</f>
       </c>
       <c r="BC26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BA26 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY26), BA26)</f>
       </c>
       <c r="BF26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_9[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BG26" s="24"/>
       <c r="BH26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_9,2),0)</f>
+        <f>=IFERROR(ROUND(BG26/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BG26 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF26), BG26)</f>
       </c>
       <c r="BJ26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BH26 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF26), BH26)</f>
       </c>
       <c r="BM26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_10[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BN26" s="24"/>
       <c r="BO26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_10,2),0)</f>
+        <f>=IFERROR(ROUND(BN26/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BN26 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM26), BN26)</f>
       </c>
       <c r="BQ26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BO26 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM26), BO26)</f>
       </c>
       <c r="BT26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_11[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="BU26" s="24"/>
       <c r="BV26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_11,2),0)</f>
+        <f>=IFERROR(ROUND(BU26/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(BU26 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT26), BU26)</f>
       </c>
       <c r="BX26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(BV26 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT26), BV26)</f>
       </c>
       <c r="CA26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_12[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CB26" s="24"/>
       <c r="CC26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_12,2),0)</f>
+        <f>=IFERROR(ROUND(CB26/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CB26 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA26), CB26)</f>
       </c>
       <c r="CE26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CC26 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA26), CC26)</f>
       </c>
       <c r="CH26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_13[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CI26" s="24"/>
       <c r="CJ26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_13,2),0)</f>
+        <f>=IFERROR(ROUND(CI26/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CI26 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH26), CI26)</f>
       </c>
       <c r="CL26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CJ26 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH26), CJ26)</f>
       </c>
       <c r="CO26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_14[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CP26" s="24"/>
       <c r="CQ26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_14,2),0)</f>
+        <f>=IFERROR(ROUND(CP26/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CP26 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO26), CP26)</f>
       </c>
       <c r="CS26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CQ26 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO26), CQ26)</f>
       </c>
       <c r="CV26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_15[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="CW26" s="24"/>
       <c r="CX26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_15,2),0)</f>
+        <f>=IFERROR(ROUND(CW26/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(CW26 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV26), CW26)</f>
       </c>
       <c r="CZ26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(CX26 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV26), CX26)</f>
       </c>
       <c r="DC26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_16[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DD26" s="24"/>
       <c r="DE26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_16,2),0)</f>
+        <f>=IFERROR(ROUND(DD26/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DD26 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC26), DD26)</f>
       </c>
       <c r="DG26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DE26 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC26), DE26)</f>
       </c>
       <c r="DJ26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_17[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DK26" s="24"/>
       <c r="DL26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_17,2),0)</f>
+        <f>=IFERROR(ROUND(DK26/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DK26 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ26), DK26)</f>
       </c>
       <c r="DN26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DL26 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ26), DL26)</f>
       </c>
       <c r="DQ26" s="148" t="str">
-        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - ROW(Ausgaben_18[#Headers])), "")</f>
+        <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
       </c>
       <c r="DR26" s="24"/>
       <c r="DS26" s="116" t="str">
-        <f>=IFERROR(ROUND([@[Ausgaben (LC)]]/FB_Kurs_18,2),0)</f>
+        <f>=IFERROR(ROUND(DR26/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT26" s="115" t="str">
-        <f>=IFERROR([@[Ausgaben (LC)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (LC)]])</f>
+        <f>=IFERROR(DR26 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ26), DR26)</f>
       </c>
       <c r="DU26" s="143" t="str">
-        <f>=IFERROR([@[Ausgaben (EUR)]] + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], [@ID]), [@[Ausgaben (EUR)]])</f>
+        <f>=IFERROR(DS26 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ26), DS26)</f>
       </c>
     </row>
     <row r="27">
@@ -12195,7 +12195,7 @@
         <f>=ROUND(D11,2)</f>
       </c>
       <c r="F41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D41/E41,0),6)</f>
       </c>
       <c r="I41" s="159" t="s">
         <v>304</v>
@@ -12210,7 +12210,7 @@
         <f>=ROUND(K11,2)</f>
       </c>
       <c r="M41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K41/L41,0),6)</f>
       </c>
       <c r="P41" s="159" t="s">
         <v>304</v>
@@ -12225,7 +12225,7 @@
         <f>=ROUND(R11,2)</f>
       </c>
       <c r="T41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R41/S41,0),6)</f>
       </c>
       <c r="W41" s="159" t="s">
         <v>304</v>
@@ -12240,7 +12240,7 @@
         <f>=ROUND(Y11,2)</f>
       </c>
       <c r="AA41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y41/Z41,0),6)</f>
       </c>
       <c r="AD41" s="159" t="s">
         <v>304</v>
@@ -12255,7 +12255,7 @@
         <f>=ROUND(AF11,2)</f>
       </c>
       <c r="AH41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF41/AG41,0),6)</f>
       </c>
       <c r="AK41" s="159" t="s">
         <v>304</v>
@@ -12270,7 +12270,7 @@
         <f>=ROUND(AM11,2)</f>
       </c>
       <c r="AO41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM41/AN41,0),6)</f>
       </c>
       <c r="AR41" s="159" t="s">
         <v>304</v>
@@ -12285,7 +12285,7 @@
         <f>=ROUND(AT11,2)</f>
       </c>
       <c r="AV41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT41/AU41,0),6)</f>
       </c>
       <c r="AY41" s="159" t="s">
         <v>304</v>
@@ -12300,7 +12300,7 @@
         <f>=ROUND(BA11,2)</f>
       </c>
       <c r="BC41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA41/BB41,0),6)</f>
       </c>
       <c r="BF41" s="159" t="s">
         <v>304</v>
@@ -12315,7 +12315,7 @@
         <f>=ROUND(BH11,2)</f>
       </c>
       <c r="BJ41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH41/BI41,0),6)</f>
       </c>
       <c r="BM41" s="159" t="s">
         <v>304</v>
@@ -12330,7 +12330,7 @@
         <f>=ROUND(BO11,2)</f>
       </c>
       <c r="BQ41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO41/BP41,0),6)</f>
       </c>
       <c r="BT41" s="159" t="s">
         <v>304</v>
@@ -12345,7 +12345,7 @@
         <f>=ROUND(BV11,2)</f>
       </c>
       <c r="BX41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV41/BW41,0),6)</f>
       </c>
       <c r="CA41" s="159" t="s">
         <v>304</v>
@@ -12360,7 +12360,7 @@
         <f>=ROUND(CC11,2)</f>
       </c>
       <c r="CE41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC41/CD41,0),6)</f>
       </c>
       <c r="CH41" s="159" t="s">
         <v>304</v>
@@ -12375,7 +12375,7 @@
         <f>=ROUND(CJ11,2)</f>
       </c>
       <c r="CL41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ41/CK41,0),6)</f>
       </c>
       <c r="CO41" s="159" t="s">
         <v>304</v>
@@ -12390,7 +12390,7 @@
         <f>=ROUND(CQ11,2)</f>
       </c>
       <c r="CS41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ41/CR41,0),6)</f>
       </c>
       <c r="CV41" s="159" t="s">
         <v>304</v>
@@ -12405,7 +12405,7 @@
         <f>=ROUND(CX11,2)</f>
       </c>
       <c r="CZ41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX41/CY41,0),6)</f>
       </c>
       <c r="DC41" s="159" t="s">
         <v>304</v>
@@ -12420,7 +12420,7 @@
         <f>=ROUND(DE11,2)</f>
       </c>
       <c r="DG41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE41/DF41,0),6)</f>
       </c>
       <c r="DJ41" s="159" t="s">
         <v>304</v>
@@ -12435,7 +12435,7 @@
         <f>=ROUND(DL11,2)</f>
       </c>
       <c r="DN41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL41/DM41,0),6)</f>
       </c>
       <c r="DQ41" s="159" t="s">
         <v>304</v>
@@ -12450,7 +12450,7 @@
         <f>=ROUND(DS11,2)</f>
       </c>
       <c r="DU41" s="163" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS41/DT41,0),6)</f>
       </c>
     </row>
     <row r="42">
@@ -12463,7 +12463,7 @@
       <c r="D42" s="166"/>
       <c r="E42" s="167"/>
       <c r="F42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D42/E42,0),6)</f>
       </c>
       <c r="I42" s="164" t="s">
         <v>199</v>
@@ -12474,7 +12474,7 @@
       <c r="K42" s="166"/>
       <c r="L42" s="167"/>
       <c r="M42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K42/L42,0),6)</f>
       </c>
       <c r="P42" s="164" t="s">
         <v>199</v>
@@ -12485,7 +12485,7 @@
       <c r="R42" s="166"/>
       <c r="S42" s="167"/>
       <c r="T42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R42/S42,0),6)</f>
       </c>
       <c r="W42" s="164" t="s">
         <v>199</v>
@@ -12496,7 +12496,7 @@
       <c r="Y42" s="166"/>
       <c r="Z42" s="167"/>
       <c r="AA42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y42/Z42,0),6)</f>
       </c>
       <c r="AD42" s="164" t="s">
         <v>199</v>
@@ -12507,7 +12507,7 @@
       <c r="AF42" s="166"/>
       <c r="AG42" s="167"/>
       <c r="AH42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF42/AG42,0),6)</f>
       </c>
       <c r="AK42" s="164" t="s">
         <v>199</v>
@@ -12518,7 +12518,7 @@
       <c r="AM42" s="166"/>
       <c r="AN42" s="167"/>
       <c r="AO42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM42/AN42,0),6)</f>
       </c>
       <c r="AR42" s="164" t="s">
         <v>199</v>
@@ -12529,7 +12529,7 @@
       <c r="AT42" s="166"/>
       <c r="AU42" s="167"/>
       <c r="AV42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT42/AU42,0),6)</f>
       </c>
       <c r="AY42" s="164" t="s">
         <v>199</v>
@@ -12540,7 +12540,7 @@
       <c r="BA42" s="166"/>
       <c r="BB42" s="167"/>
       <c r="BC42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA42/BB42,0),6)</f>
       </c>
       <c r="BF42" s="164" t="s">
         <v>199</v>
@@ -12551,7 +12551,7 @@
       <c r="BH42" s="166"/>
       <c r="BI42" s="167"/>
       <c r="BJ42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH42/BI42,0),6)</f>
       </c>
       <c r="BM42" s="164" t="s">
         <v>199</v>
@@ -12562,7 +12562,7 @@
       <c r="BO42" s="166"/>
       <c r="BP42" s="167"/>
       <c r="BQ42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO42/BP42,0),6)</f>
       </c>
       <c r="BT42" s="164" t="s">
         <v>199</v>
@@ -12573,7 +12573,7 @@
       <c r="BV42" s="166"/>
       <c r="BW42" s="167"/>
       <c r="BX42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV42/BW42,0),6)</f>
       </c>
       <c r="CA42" s="164" t="s">
         <v>199</v>
@@ -12584,7 +12584,7 @@
       <c r="CC42" s="166"/>
       <c r="CD42" s="167"/>
       <c r="CE42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC42/CD42,0),6)</f>
       </c>
       <c r="CH42" s="164" t="s">
         <v>199</v>
@@ -12595,7 +12595,7 @@
       <c r="CJ42" s="166"/>
       <c r="CK42" s="167"/>
       <c r="CL42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ42/CK42,0),6)</f>
       </c>
       <c r="CO42" s="164" t="s">
         <v>199</v>
@@ -12606,7 +12606,7 @@
       <c r="CQ42" s="166"/>
       <c r="CR42" s="167"/>
       <c r="CS42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ42/CR42,0),6)</f>
       </c>
       <c r="CV42" s="164" t="s">
         <v>199</v>
@@ -12617,7 +12617,7 @@
       <c r="CX42" s="166"/>
       <c r="CY42" s="167"/>
       <c r="CZ42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX42/CY42,0),6)</f>
       </c>
       <c r="DC42" s="164" t="s">
         <v>199</v>
@@ -12628,7 +12628,7 @@
       <c r="DE42" s="166"/>
       <c r="DF42" s="167"/>
       <c r="DG42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE42/DF42,0),6)</f>
       </c>
       <c r="DJ42" s="164" t="s">
         <v>199</v>
@@ -12639,7 +12639,7 @@
       <c r="DL42" s="166"/>
       <c r="DM42" s="167"/>
       <c r="DN42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL42/DM42,0),6)</f>
       </c>
       <c r="DQ42" s="164" t="s">
         <v>199</v>
@@ -12650,7 +12650,7 @@
       <c r="DS42" s="166"/>
       <c r="DT42" s="167"/>
       <c r="DU42" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS42/DT42,0),6)</f>
       </c>
     </row>
     <row r="43">
@@ -12663,7 +12663,7 @@
       <c r="D43" s="166"/>
       <c r="E43" s="167"/>
       <c r="F43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D43/E43,0),6)</f>
       </c>
       <c r="I43" s="164" t="s">
         <v>158</v>
@@ -12674,7 +12674,7 @@
       <c r="K43" s="166"/>
       <c r="L43" s="167"/>
       <c r="M43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K43/L43,0),6)</f>
       </c>
       <c r="P43" s="164" t="s">
         <v>158</v>
@@ -12685,7 +12685,7 @@
       <c r="R43" s="166"/>
       <c r="S43" s="167"/>
       <c r="T43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R43/S43,0),6)</f>
       </c>
       <c r="W43" s="164" t="s">
         <v>158</v>
@@ -12696,7 +12696,7 @@
       <c r="Y43" s="166"/>
       <c r="Z43" s="167"/>
       <c r="AA43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y43/Z43,0),6)</f>
       </c>
       <c r="AD43" s="164" t="s">
         <v>158</v>
@@ -12707,7 +12707,7 @@
       <c r="AF43" s="166"/>
       <c r="AG43" s="167"/>
       <c r="AH43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF43/AG43,0),6)</f>
       </c>
       <c r="AK43" s="164" t="s">
         <v>158</v>
@@ -12718,7 +12718,7 @@
       <c r="AM43" s="166"/>
       <c r="AN43" s="167"/>
       <c r="AO43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM43/AN43,0),6)</f>
       </c>
       <c r="AR43" s="164" t="s">
         <v>158</v>
@@ -12729,7 +12729,7 @@
       <c r="AT43" s="166"/>
       <c r="AU43" s="167"/>
       <c r="AV43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT43/AU43,0),6)</f>
       </c>
       <c r="AY43" s="164" t="s">
         <v>158</v>
@@ -12740,7 +12740,7 @@
       <c r="BA43" s="166"/>
       <c r="BB43" s="167"/>
       <c r="BC43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA43/BB43,0),6)</f>
       </c>
       <c r="BF43" s="164" t="s">
         <v>158</v>
@@ -12751,7 +12751,7 @@
       <c r="BH43" s="166"/>
       <c r="BI43" s="167"/>
       <c r="BJ43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH43/BI43,0),6)</f>
       </c>
       <c r="BM43" s="164" t="s">
         <v>158</v>
@@ -12762,7 +12762,7 @@
       <c r="BO43" s="166"/>
       <c r="BP43" s="167"/>
       <c r="BQ43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO43/BP43,0),6)</f>
       </c>
       <c r="BT43" s="164" t="s">
         <v>158</v>
@@ -12773,7 +12773,7 @@
       <c r="BV43" s="166"/>
       <c r="BW43" s="167"/>
       <c r="BX43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV43/BW43,0),6)</f>
       </c>
       <c r="CA43" s="164" t="s">
         <v>158</v>
@@ -12784,7 +12784,7 @@
       <c r="CC43" s="166"/>
       <c r="CD43" s="167"/>
       <c r="CE43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC43/CD43,0),6)</f>
       </c>
       <c r="CH43" s="164" t="s">
         <v>158</v>
@@ -12795,7 +12795,7 @@
       <c r="CJ43" s="166"/>
       <c r="CK43" s="167"/>
       <c r="CL43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ43/CK43,0),6)</f>
       </c>
       <c r="CO43" s="164" t="s">
         <v>158</v>
@@ -12806,7 +12806,7 @@
       <c r="CQ43" s="166"/>
       <c r="CR43" s="167"/>
       <c r="CS43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ43/CR43,0),6)</f>
       </c>
       <c r="CV43" s="164" t="s">
         <v>158</v>
@@ -12817,7 +12817,7 @@
       <c r="CX43" s="166"/>
       <c r="CY43" s="167"/>
       <c r="CZ43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX43/CY43,0),6)</f>
       </c>
       <c r="DC43" s="164" t="s">
         <v>158</v>
@@ -12828,7 +12828,7 @@
       <c r="DE43" s="166"/>
       <c r="DF43" s="167"/>
       <c r="DG43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE43/DF43,0),6)</f>
       </c>
       <c r="DJ43" s="164" t="s">
         <v>158</v>
@@ -12839,7 +12839,7 @@
       <c r="DL43" s="166"/>
       <c r="DM43" s="167"/>
       <c r="DN43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL43/DM43,0),6)</f>
       </c>
       <c r="DQ43" s="164" t="s">
         <v>158</v>
@@ -12850,7 +12850,7 @@
       <c r="DS43" s="166"/>
       <c r="DT43" s="167"/>
       <c r="DU43" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS43/DT43,0),6)</f>
       </c>
     </row>
     <row r="44">
@@ -12863,7 +12863,7 @@
       <c r="D44" s="166"/>
       <c r="E44" s="167"/>
       <c r="F44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D44/E44,0),6)</f>
       </c>
       <c r="I44" s="164" t="s">
         <v>158</v>
@@ -12874,7 +12874,7 @@
       <c r="K44" s="166"/>
       <c r="L44" s="167"/>
       <c r="M44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K44/L44,0),6)</f>
       </c>
       <c r="P44" s="164" t="s">
         <v>158</v>
@@ -12885,7 +12885,7 @@
       <c r="R44" s="166"/>
       <c r="S44" s="167"/>
       <c r="T44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R44/S44,0),6)</f>
       </c>
       <c r="W44" s="164" t="s">
         <v>158</v>
@@ -12896,7 +12896,7 @@
       <c r="Y44" s="166"/>
       <c r="Z44" s="167"/>
       <c r="AA44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y44/Z44,0),6)</f>
       </c>
       <c r="AD44" s="164" t="s">
         <v>158</v>
@@ -12907,7 +12907,7 @@
       <c r="AF44" s="166"/>
       <c r="AG44" s="167"/>
       <c r="AH44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF44/AG44,0),6)</f>
       </c>
       <c r="AK44" s="164" t="s">
         <v>158</v>
@@ -12918,7 +12918,7 @@
       <c r="AM44" s="166"/>
       <c r="AN44" s="167"/>
       <c r="AO44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM44/AN44,0),6)</f>
       </c>
       <c r="AR44" s="164" t="s">
         <v>158</v>
@@ -12929,7 +12929,7 @@
       <c r="AT44" s="166"/>
       <c r="AU44" s="167"/>
       <c r="AV44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT44/AU44,0),6)</f>
       </c>
       <c r="AY44" s="164" t="s">
         <v>158</v>
@@ -12940,7 +12940,7 @@
       <c r="BA44" s="166"/>
       <c r="BB44" s="167"/>
       <c r="BC44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA44/BB44,0),6)</f>
       </c>
       <c r="BF44" s="164" t="s">
         <v>158</v>
@@ -12951,7 +12951,7 @@
       <c r="BH44" s="166"/>
       <c r="BI44" s="167"/>
       <c r="BJ44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH44/BI44,0),6)</f>
       </c>
       <c r="BM44" s="164" t="s">
         <v>158</v>
@@ -12962,7 +12962,7 @@
       <c r="BO44" s="166"/>
       <c r="BP44" s="167"/>
       <c r="BQ44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO44/BP44,0),6)</f>
       </c>
       <c r="BT44" s="164" t="s">
         <v>158</v>
@@ -12973,7 +12973,7 @@
       <c r="BV44" s="166"/>
       <c r="BW44" s="167"/>
       <c r="BX44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV44/BW44,0),6)</f>
       </c>
       <c r="CA44" s="164" t="s">
         <v>158</v>
@@ -12984,7 +12984,7 @@
       <c r="CC44" s="166"/>
       <c r="CD44" s="167"/>
       <c r="CE44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC44/CD44,0),6)</f>
       </c>
       <c r="CH44" s="164" t="s">
         <v>158</v>
@@ -12995,7 +12995,7 @@
       <c r="CJ44" s="166"/>
       <c r="CK44" s="167"/>
       <c r="CL44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ44/CK44,0),6)</f>
       </c>
       <c r="CO44" s="164" t="s">
         <v>158</v>
@@ -13006,7 +13006,7 @@
       <c r="CQ44" s="166"/>
       <c r="CR44" s="167"/>
       <c r="CS44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ44/CR44,0),6)</f>
       </c>
       <c r="CV44" s="164" t="s">
         <v>158</v>
@@ -13017,7 +13017,7 @@
       <c r="CX44" s="166"/>
       <c r="CY44" s="167"/>
       <c r="CZ44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX44/CY44,0),6)</f>
       </c>
       <c r="DC44" s="164" t="s">
         <v>158</v>
@@ -13028,7 +13028,7 @@
       <c r="DE44" s="166"/>
       <c r="DF44" s="167"/>
       <c r="DG44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE44/DF44,0),6)</f>
       </c>
       <c r="DJ44" s="164" t="s">
         <v>158</v>
@@ -13039,7 +13039,7 @@
       <c r="DL44" s="166"/>
       <c r="DM44" s="167"/>
       <c r="DN44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL44/DM44,0),6)</f>
       </c>
       <c r="DQ44" s="164" t="s">
         <v>158</v>
@@ -13050,7 +13050,7 @@
       <c r="DS44" s="166"/>
       <c r="DT44" s="167"/>
       <c r="DU44" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS44/DT44,0),6)</f>
       </c>
     </row>
     <row r="45">
@@ -13063,7 +13063,7 @@
       <c r="D45" s="166"/>
       <c r="E45" s="167"/>
       <c r="F45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D45/E45,0),6)</f>
       </c>
       <c r="I45" s="164" t="s">
         <v>158</v>
@@ -13074,7 +13074,7 @@
       <c r="K45" s="166"/>
       <c r="L45" s="167"/>
       <c r="M45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K45/L45,0),6)</f>
       </c>
       <c r="P45" s="164" t="s">
         <v>158</v>
@@ -13085,7 +13085,7 @@
       <c r="R45" s="166"/>
       <c r="S45" s="167"/>
       <c r="T45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R45/S45,0),6)</f>
       </c>
       <c r="W45" s="164" t="s">
         <v>158</v>
@@ -13096,7 +13096,7 @@
       <c r="Y45" s="166"/>
       <c r="Z45" s="167"/>
       <c r="AA45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y45/Z45,0),6)</f>
       </c>
       <c r="AD45" s="164" t="s">
         <v>158</v>
@@ -13107,7 +13107,7 @@
       <c r="AF45" s="166"/>
       <c r="AG45" s="167"/>
       <c r="AH45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF45/AG45,0),6)</f>
       </c>
       <c r="AK45" s="164" t="s">
         <v>158</v>
@@ -13118,7 +13118,7 @@
       <c r="AM45" s="166"/>
       <c r="AN45" s="167"/>
       <c r="AO45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM45/AN45,0),6)</f>
       </c>
       <c r="AR45" s="164" t="s">
         <v>158</v>
@@ -13129,7 +13129,7 @@
       <c r="AT45" s="166"/>
       <c r="AU45" s="167"/>
       <c r="AV45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT45/AU45,0),6)</f>
       </c>
       <c r="AY45" s="164" t="s">
         <v>158</v>
@@ -13140,7 +13140,7 @@
       <c r="BA45" s="166"/>
       <c r="BB45" s="167"/>
       <c r="BC45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA45/BB45,0),6)</f>
       </c>
       <c r="BF45" s="164" t="s">
         <v>158</v>
@@ -13151,7 +13151,7 @@
       <c r="BH45" s="166"/>
       <c r="BI45" s="167"/>
       <c r="BJ45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH45/BI45,0),6)</f>
       </c>
       <c r="BM45" s="164" t="s">
         <v>158</v>
@@ -13162,7 +13162,7 @@
       <c r="BO45" s="166"/>
       <c r="BP45" s="167"/>
       <c r="BQ45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO45/BP45,0),6)</f>
       </c>
       <c r="BT45" s="164" t="s">
         <v>158</v>
@@ -13173,7 +13173,7 @@
       <c r="BV45" s="166"/>
       <c r="BW45" s="167"/>
       <c r="BX45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV45/BW45,0),6)</f>
       </c>
       <c r="CA45" s="164" t="s">
         <v>158</v>
@@ -13184,7 +13184,7 @@
       <c r="CC45" s="166"/>
       <c r="CD45" s="167"/>
       <c r="CE45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC45/CD45,0),6)</f>
       </c>
       <c r="CH45" s="164" t="s">
         <v>158</v>
@@ -13195,7 +13195,7 @@
       <c r="CJ45" s="166"/>
       <c r="CK45" s="167"/>
       <c r="CL45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ45/CK45,0),6)</f>
       </c>
       <c r="CO45" s="164" t="s">
         <v>158</v>
@@ -13206,7 +13206,7 @@
       <c r="CQ45" s="166"/>
       <c r="CR45" s="167"/>
       <c r="CS45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ45/CR45,0),6)</f>
       </c>
       <c r="CV45" s="164" t="s">
         <v>158</v>
@@ -13217,7 +13217,7 @@
       <c r="CX45" s="166"/>
       <c r="CY45" s="167"/>
       <c r="CZ45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX45/CY45,0),6)</f>
       </c>
       <c r="DC45" s="164" t="s">
         <v>158</v>
@@ -13228,7 +13228,7 @@
       <c r="DE45" s="166"/>
       <c r="DF45" s="167"/>
       <c r="DG45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE45/DF45,0),6)</f>
       </c>
       <c r="DJ45" s="164" t="s">
         <v>158</v>
@@ -13239,7 +13239,7 @@
       <c r="DL45" s="166"/>
       <c r="DM45" s="167"/>
       <c r="DN45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL45/DM45,0),6)</f>
       </c>
       <c r="DQ45" s="164" t="s">
         <v>158</v>
@@ -13250,7 +13250,7 @@
       <c r="DS45" s="166"/>
       <c r="DT45" s="167"/>
       <c r="DU45" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS45/DT45,0),6)</f>
       </c>
     </row>
     <row r="46">
@@ -13862,10 +13862,10 @@
       </c>
       <c r="D50" s="166"/>
       <c r="E50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$C$7,2),0)</f>
+        <f>=IFERROR(ROUND(D50/$C$7,2),0)</f>
       </c>
       <c r="F50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D50/E50,0),6)</f>
       </c>
       <c r="I50" s="164" t="s">
         <v>194</v>
@@ -13875,10 +13875,10 @@
       </c>
       <c r="K50" s="166"/>
       <c r="L50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$J$7,2),0)</f>
+        <f>=IFERROR(ROUND(K50/$J$7,2),0)</f>
       </c>
       <c r="M50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K50/L50,0),6)</f>
       </c>
       <c r="P50" s="164" t="s">
         <v>194</v>
@@ -13888,10 +13888,10 @@
       </c>
       <c r="R50" s="166"/>
       <c r="S50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$Q$7,2),0)</f>
+        <f>=IFERROR(ROUND(R50/$Q$7,2),0)</f>
       </c>
       <c r="T50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R50/S50,0),6)</f>
       </c>
       <c r="W50" s="164" t="s">
         <v>194</v>
@@ -13901,10 +13901,10 @@
       </c>
       <c r="Y50" s="166"/>
       <c r="Z50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$X$7,2),0)</f>
+        <f>=IFERROR(ROUND(Y50/$X$7,2),0)</f>
       </c>
       <c r="AA50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y50/Z50,0),6)</f>
       </c>
       <c r="AD50" s="164" t="s">
         <v>194</v>
@@ -13914,10 +13914,10 @@
       </c>
       <c r="AF50" s="166"/>
       <c r="AG50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AE$7,2),0)</f>
+        <f>=IFERROR(ROUND(AF50/$AE$7,2),0)</f>
       </c>
       <c r="AH50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF50/AG50,0),6)</f>
       </c>
       <c r="AK50" s="164" t="s">
         <v>194</v>
@@ -13927,10 +13927,10 @@
       </c>
       <c r="AM50" s="166"/>
       <c r="AN50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AL$7,2),0)</f>
+        <f>=IFERROR(ROUND(AM50/$AL$7,2),0)</f>
       </c>
       <c r="AO50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM50/AN50,0),6)</f>
       </c>
       <c r="AR50" s="164" t="s">
         <v>194</v>
@@ -13940,10 +13940,10 @@
       </c>
       <c r="AT50" s="166"/>
       <c r="AU50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AS$7,2),0)</f>
+        <f>=IFERROR(ROUND(AT50/$AS$7,2),0)</f>
       </c>
       <c r="AV50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT50/AU50,0),6)</f>
       </c>
       <c r="AY50" s="164" t="s">
         <v>194</v>
@@ -13953,10 +13953,10 @@
       </c>
       <c r="BA50" s="166"/>
       <c r="BB50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AZ$7,2),0)</f>
+        <f>=IFERROR(ROUND(BA50/$AZ$7,2),0)</f>
       </c>
       <c r="BC50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA50/BB50,0),6)</f>
       </c>
       <c r="BF50" s="164" t="s">
         <v>194</v>
@@ -13966,10 +13966,10 @@
       </c>
       <c r="BH50" s="166"/>
       <c r="BI50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BG$7,2),0)</f>
+        <f>=IFERROR(ROUND(BH50/$BG$7,2),0)</f>
       </c>
       <c r="BJ50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH50/BI50,0),6)</f>
       </c>
       <c r="BM50" s="164" t="s">
         <v>194</v>
@@ -13979,10 +13979,10 @@
       </c>
       <c r="BO50" s="166"/>
       <c r="BP50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BN$7,2),0)</f>
+        <f>=IFERROR(ROUND(BO50/$BN$7,2),0)</f>
       </c>
       <c r="BQ50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO50/BP50,0),6)</f>
       </c>
       <c r="BT50" s="164" t="s">
         <v>194</v>
@@ -13992,10 +13992,10 @@
       </c>
       <c r="BV50" s="166"/>
       <c r="BW50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BU$7,2),0)</f>
+        <f>=IFERROR(ROUND(BV50/$BU$7,2),0)</f>
       </c>
       <c r="BX50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV50/BW50,0),6)</f>
       </c>
       <c r="CA50" s="164" t="s">
         <v>194</v>
@@ -14005,10 +14005,10 @@
       </c>
       <c r="CC50" s="166"/>
       <c r="CD50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CB$7,2),0)</f>
+        <f>=IFERROR(ROUND(CC50/$CB$7,2),0)</f>
       </c>
       <c r="CE50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC50/CD50,0),6)</f>
       </c>
       <c r="CH50" s="164" t="s">
         <v>194</v>
@@ -14018,10 +14018,10 @@
       </c>
       <c r="CJ50" s="166"/>
       <c r="CK50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CI$7,2),0)</f>
+        <f>=IFERROR(ROUND(CJ50/$CI$7,2),0)</f>
       </c>
       <c r="CL50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ50/CK50,0),6)</f>
       </c>
       <c r="CO50" s="164" t="s">
         <v>194</v>
@@ -14031,10 +14031,10 @@
       </c>
       <c r="CQ50" s="166"/>
       <c r="CR50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CP$7,2),0)</f>
+        <f>=IFERROR(ROUND(CQ50/$CP$7,2),0)</f>
       </c>
       <c r="CS50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ50/CR50,0),6)</f>
       </c>
       <c r="CV50" s="164" t="s">
         <v>194</v>
@@ -14044,10 +14044,10 @@
       </c>
       <c r="CX50" s="166"/>
       <c r="CY50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CW$7,2),0)</f>
+        <f>=IFERROR(ROUND(CX50/$CW$7,2),0)</f>
       </c>
       <c r="CZ50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX50/CY50,0),6)</f>
       </c>
       <c r="DC50" s="164" t="s">
         <v>194</v>
@@ -14057,10 +14057,10 @@
       </c>
       <c r="DE50" s="166"/>
       <c r="DF50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DD$7,2),0)</f>
+        <f>=IFERROR(ROUND(DE50/$DD$7,2),0)</f>
       </c>
       <c r="DG50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE50/DF50,0),6)</f>
       </c>
       <c r="DJ50" s="164" t="s">
         <v>194</v>
@@ -14070,10 +14070,10 @@
       </c>
       <c r="DL50" s="166"/>
       <c r="DM50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DK$7,2),0)</f>
+        <f>=IFERROR(ROUND(DL50/$DK$7,2),0)</f>
       </c>
       <c r="DN50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL50/DM50,0),6)</f>
       </c>
       <c r="DQ50" s="164" t="s">
         <v>194</v>
@@ -14083,10 +14083,10 @@
       </c>
       <c r="DS50" s="166"/>
       <c r="DT50" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DR$7,2),0)</f>
+        <f>=IFERROR(ROUND(DS50/$DR$7,2),0)</f>
       </c>
       <c r="DU50" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS50/DT50,0),6)</f>
       </c>
     </row>
     <row r="51">
@@ -14098,10 +14098,10 @@
       </c>
       <c r="D51" s="166"/>
       <c r="E51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$C$7,2),0)</f>
+        <f>=IFERROR(ROUND(D51/$C$7,2),0)</f>
       </c>
       <c r="F51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D51/E51,0),6)</f>
       </c>
       <c r="I51" s="164" t="s">
         <v>277</v>
@@ -14111,10 +14111,10 @@
       </c>
       <c r="K51" s="166"/>
       <c r="L51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$J$7,2),0)</f>
+        <f>=IFERROR(ROUND(K51/$J$7,2),0)</f>
       </c>
       <c r="M51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K51/L51,0),6)</f>
       </c>
       <c r="P51" s="164" t="s">
         <v>277</v>
@@ -14124,10 +14124,10 @@
       </c>
       <c r="R51" s="166"/>
       <c r="S51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$Q$7,2),0)</f>
+        <f>=IFERROR(ROUND(R51/$Q$7,2),0)</f>
       </c>
       <c r="T51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R51/S51,0),6)</f>
       </c>
       <c r="W51" s="164" t="s">
         <v>277</v>
@@ -14137,10 +14137,10 @@
       </c>
       <c r="Y51" s="166"/>
       <c r="Z51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$X$7,2),0)</f>
+        <f>=IFERROR(ROUND(Y51/$X$7,2),0)</f>
       </c>
       <c r="AA51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y51/Z51,0),6)</f>
       </c>
       <c r="AD51" s="164" t="s">
         <v>277</v>
@@ -14150,10 +14150,10 @@
       </c>
       <c r="AF51" s="166"/>
       <c r="AG51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AE$7,2),0)</f>
+        <f>=IFERROR(ROUND(AF51/$AE$7,2),0)</f>
       </c>
       <c r="AH51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF51/AG51,0),6)</f>
       </c>
       <c r="AK51" s="164" t="s">
         <v>277</v>
@@ -14163,10 +14163,10 @@
       </c>
       <c r="AM51" s="166"/>
       <c r="AN51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AL$7,2),0)</f>
+        <f>=IFERROR(ROUND(AM51/$AL$7,2),0)</f>
       </c>
       <c r="AO51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM51/AN51,0),6)</f>
       </c>
       <c r="AR51" s="164" t="s">
         <v>277</v>
@@ -14176,10 +14176,10 @@
       </c>
       <c r="AT51" s="166"/>
       <c r="AU51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AS$7,2),0)</f>
+        <f>=IFERROR(ROUND(AT51/$AS$7,2),0)</f>
       </c>
       <c r="AV51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT51/AU51,0),6)</f>
       </c>
       <c r="AY51" s="164" t="s">
         <v>277</v>
@@ -14189,10 +14189,10 @@
       </c>
       <c r="BA51" s="166"/>
       <c r="BB51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AZ$7,2),0)</f>
+        <f>=IFERROR(ROUND(BA51/$AZ$7,2),0)</f>
       </c>
       <c r="BC51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA51/BB51,0),6)</f>
       </c>
       <c r="BF51" s="164" t="s">
         <v>277</v>
@@ -14202,10 +14202,10 @@
       </c>
       <c r="BH51" s="166"/>
       <c r="BI51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BG$7,2),0)</f>
+        <f>=IFERROR(ROUND(BH51/$BG$7,2),0)</f>
       </c>
       <c r="BJ51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH51/BI51,0),6)</f>
       </c>
       <c r="BM51" s="164" t="s">
         <v>277</v>
@@ -14215,10 +14215,10 @@
       </c>
       <c r="BO51" s="166"/>
       <c r="BP51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BN$7,2),0)</f>
+        <f>=IFERROR(ROUND(BO51/$BN$7,2),0)</f>
       </c>
       <c r="BQ51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO51/BP51,0),6)</f>
       </c>
       <c r="BT51" s="164" t="s">
         <v>277</v>
@@ -14228,10 +14228,10 @@
       </c>
       <c r="BV51" s="166"/>
       <c r="BW51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BU$7,2),0)</f>
+        <f>=IFERROR(ROUND(BV51/$BU$7,2),0)</f>
       </c>
       <c r="BX51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV51/BW51,0),6)</f>
       </c>
       <c r="CA51" s="164" t="s">
         <v>277</v>
@@ -14241,10 +14241,10 @@
       </c>
       <c r="CC51" s="166"/>
       <c r="CD51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CB$7,2),0)</f>
+        <f>=IFERROR(ROUND(CC51/$CB$7,2),0)</f>
       </c>
       <c r="CE51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC51/CD51,0),6)</f>
       </c>
       <c r="CH51" s="164" t="s">
         <v>277</v>
@@ -14254,10 +14254,10 @@
       </c>
       <c r="CJ51" s="166"/>
       <c r="CK51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CI$7,2),0)</f>
+        <f>=IFERROR(ROUND(CJ51/$CI$7,2),0)</f>
       </c>
       <c r="CL51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ51/CK51,0),6)</f>
       </c>
       <c r="CO51" s="164" t="s">
         <v>277</v>
@@ -14267,10 +14267,10 @@
       </c>
       <c r="CQ51" s="166"/>
       <c r="CR51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CP$7,2),0)</f>
+        <f>=IFERROR(ROUND(CQ51/$CP$7,2),0)</f>
       </c>
       <c r="CS51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ51/CR51,0),6)</f>
       </c>
       <c r="CV51" s="164" t="s">
         <v>277</v>
@@ -14280,10 +14280,10 @@
       </c>
       <c r="CX51" s="166"/>
       <c r="CY51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CW$7,2),0)</f>
+        <f>=IFERROR(ROUND(CX51/$CW$7,2),0)</f>
       </c>
       <c r="CZ51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX51/CY51,0),6)</f>
       </c>
       <c r="DC51" s="164" t="s">
         <v>277</v>
@@ -14293,10 +14293,10 @@
       </c>
       <c r="DE51" s="166"/>
       <c r="DF51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DD$7,2),0)</f>
+        <f>=IFERROR(ROUND(DE51/$DD$7,2),0)</f>
       </c>
       <c r="DG51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE51/DF51,0),6)</f>
       </c>
       <c r="DJ51" s="164" t="s">
         <v>277</v>
@@ -14306,10 +14306,10 @@
       </c>
       <c r="DL51" s="166"/>
       <c r="DM51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DK$7,2),0)</f>
+        <f>=IFERROR(ROUND(DL51/$DK$7,2),0)</f>
       </c>
       <c r="DN51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL51/DM51,0),6)</f>
       </c>
       <c r="DQ51" s="164" t="s">
         <v>277</v>
@@ -14319,10 +14319,10 @@
       </c>
       <c r="DS51" s="166"/>
       <c r="DT51" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DR$7,2),0)</f>
+        <f>=IFERROR(ROUND(DS51/$DR$7,2),0)</f>
       </c>
       <c r="DU51" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS51/DT51,0),6)</f>
       </c>
     </row>
     <row r="52">
@@ -14334,10 +14334,10 @@
       </c>
       <c r="D52" s="166"/>
       <c r="E52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$C$7,2),0)</f>
+        <f>=IFERROR(ROUND(D52/$C$7,2),0)</f>
       </c>
       <c r="F52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D52/E52,0),6)</f>
       </c>
       <c r="I52" s="164" t="s">
         <v>278</v>
@@ -14347,10 +14347,10 @@
       </c>
       <c r="K52" s="166"/>
       <c r="L52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$J$7,2),0)</f>
+        <f>=IFERROR(ROUND(K52/$J$7,2),0)</f>
       </c>
       <c r="M52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K52/L52,0),6)</f>
       </c>
       <c r="P52" s="164" t="s">
         <v>278</v>
@@ -14360,10 +14360,10 @@
       </c>
       <c r="R52" s="166"/>
       <c r="S52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$Q$7,2),0)</f>
+        <f>=IFERROR(ROUND(R52/$Q$7,2),0)</f>
       </c>
       <c r="T52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R52/S52,0),6)</f>
       </c>
       <c r="W52" s="164" t="s">
         <v>278</v>
@@ -14373,10 +14373,10 @@
       </c>
       <c r="Y52" s="166"/>
       <c r="Z52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$X$7,2),0)</f>
+        <f>=IFERROR(ROUND(Y52/$X$7,2),0)</f>
       </c>
       <c r="AA52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y52/Z52,0),6)</f>
       </c>
       <c r="AD52" s="164" t="s">
         <v>278</v>
@@ -14386,10 +14386,10 @@
       </c>
       <c r="AF52" s="166"/>
       <c r="AG52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AE$7,2),0)</f>
+        <f>=IFERROR(ROUND(AF52/$AE$7,2),0)</f>
       </c>
       <c r="AH52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF52/AG52,0),6)</f>
       </c>
       <c r="AK52" s="164" t="s">
         <v>278</v>
@@ -14399,10 +14399,10 @@
       </c>
       <c r="AM52" s="166"/>
       <c r="AN52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AL$7,2),0)</f>
+        <f>=IFERROR(ROUND(AM52/$AL$7,2),0)</f>
       </c>
       <c r="AO52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM52/AN52,0),6)</f>
       </c>
       <c r="AR52" s="164" t="s">
         <v>278</v>
@@ -14412,10 +14412,10 @@
       </c>
       <c r="AT52" s="166"/>
       <c r="AU52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AS$7,2),0)</f>
+        <f>=IFERROR(ROUND(AT52/$AS$7,2),0)</f>
       </c>
       <c r="AV52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT52/AU52,0),6)</f>
       </c>
       <c r="AY52" s="164" t="s">
         <v>278</v>
@@ -14425,10 +14425,10 @@
       </c>
       <c r="BA52" s="166"/>
       <c r="BB52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AZ$7,2),0)</f>
+        <f>=IFERROR(ROUND(BA52/$AZ$7,2),0)</f>
       </c>
       <c r="BC52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA52/BB52,0),6)</f>
       </c>
       <c r="BF52" s="164" t="s">
         <v>278</v>
@@ -14438,10 +14438,10 @@
       </c>
       <c r="BH52" s="166"/>
       <c r="BI52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BG$7,2),0)</f>
+        <f>=IFERROR(ROUND(BH52/$BG$7,2),0)</f>
       </c>
       <c r="BJ52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH52/BI52,0),6)</f>
       </c>
       <c r="BM52" s="164" t="s">
         <v>278</v>
@@ -14451,10 +14451,10 @@
       </c>
       <c r="BO52" s="166"/>
       <c r="BP52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BN$7,2),0)</f>
+        <f>=IFERROR(ROUND(BO52/$BN$7,2),0)</f>
       </c>
       <c r="BQ52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO52/BP52,0),6)</f>
       </c>
       <c r="BT52" s="164" t="s">
         <v>278</v>
@@ -14464,10 +14464,10 @@
       </c>
       <c r="BV52" s="166"/>
       <c r="BW52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BU$7,2),0)</f>
+        <f>=IFERROR(ROUND(BV52/$BU$7,2),0)</f>
       </c>
       <c r="BX52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV52/BW52,0),6)</f>
       </c>
       <c r="CA52" s="164" t="s">
         <v>278</v>
@@ -14477,10 +14477,10 @@
       </c>
       <c r="CC52" s="166"/>
       <c r="CD52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CB$7,2),0)</f>
+        <f>=IFERROR(ROUND(CC52/$CB$7,2),0)</f>
       </c>
       <c r="CE52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC52/CD52,0),6)</f>
       </c>
       <c r="CH52" s="164" t="s">
         <v>278</v>
@@ -14490,10 +14490,10 @@
       </c>
       <c r="CJ52" s="166"/>
       <c r="CK52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CI$7,2),0)</f>
+        <f>=IFERROR(ROUND(CJ52/$CI$7,2),0)</f>
       </c>
       <c r="CL52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ52/CK52,0),6)</f>
       </c>
       <c r="CO52" s="164" t="s">
         <v>278</v>
@@ -14503,10 +14503,10 @@
       </c>
       <c r="CQ52" s="166"/>
       <c r="CR52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CP$7,2),0)</f>
+        <f>=IFERROR(ROUND(CQ52/$CP$7,2),0)</f>
       </c>
       <c r="CS52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ52/CR52,0),6)</f>
       </c>
       <c r="CV52" s="164" t="s">
         <v>278</v>
@@ -14516,10 +14516,10 @@
       </c>
       <c r="CX52" s="166"/>
       <c r="CY52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CW$7,2),0)</f>
+        <f>=IFERROR(ROUND(CX52/$CW$7,2),0)</f>
       </c>
       <c r="CZ52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX52/CY52,0),6)</f>
       </c>
       <c r="DC52" s="164" t="s">
         <v>278</v>
@@ -14529,10 +14529,10 @@
       </c>
       <c r="DE52" s="166"/>
       <c r="DF52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DD$7,2),0)</f>
+        <f>=IFERROR(ROUND(DE52/$DD$7,2),0)</f>
       </c>
       <c r="DG52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE52/DF52,0),6)</f>
       </c>
       <c r="DJ52" s="164" t="s">
         <v>278</v>
@@ -14542,10 +14542,10 @@
       </c>
       <c r="DL52" s="166"/>
       <c r="DM52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DK$7,2),0)</f>
+        <f>=IFERROR(ROUND(DL52/$DK$7,2),0)</f>
       </c>
       <c r="DN52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL52/DM52,0),6)</f>
       </c>
       <c r="DQ52" s="164" t="s">
         <v>278</v>
@@ -14555,10 +14555,10 @@
       </c>
       <c r="DS52" s="166"/>
       <c r="DT52" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DR$7,2),0)</f>
+        <f>=IFERROR(ROUND(DS52/$DR$7,2),0)</f>
       </c>
       <c r="DU52" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS52/DT52,0),6)</f>
       </c>
     </row>
     <row r="53">
@@ -14570,10 +14570,10 @@
       </c>
       <c r="D53" s="166"/>
       <c r="E53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$C$7,2),0)</f>
+        <f>=IFERROR(ROUND(D53/$C$7,2),0)</f>
       </c>
       <c r="F53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D53/E53,0),6)</f>
       </c>
       <c r="I53" s="164" t="s">
         <v>158</v>
@@ -14583,10 +14583,10 @@
       </c>
       <c r="K53" s="166"/>
       <c r="L53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$J$7,2),0)</f>
+        <f>=IFERROR(ROUND(K53/$J$7,2),0)</f>
       </c>
       <c r="M53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K53/L53,0),6)</f>
       </c>
       <c r="P53" s="164" t="s">
         <v>158</v>
@@ -14596,10 +14596,10 @@
       </c>
       <c r="R53" s="166"/>
       <c r="S53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$Q$7,2),0)</f>
+        <f>=IFERROR(ROUND(R53/$Q$7,2),0)</f>
       </c>
       <c r="T53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R53/S53,0),6)</f>
       </c>
       <c r="W53" s="164" t="s">
         <v>158</v>
@@ -14609,10 +14609,10 @@
       </c>
       <c r="Y53" s="166"/>
       <c r="Z53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$X$7,2),0)</f>
+        <f>=IFERROR(ROUND(Y53/$X$7,2),0)</f>
       </c>
       <c r="AA53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y53/Z53,0),6)</f>
       </c>
       <c r="AD53" s="164" t="s">
         <v>158</v>
@@ -14622,10 +14622,10 @@
       </c>
       <c r="AF53" s="166"/>
       <c r="AG53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AE$7,2),0)</f>
+        <f>=IFERROR(ROUND(AF53/$AE$7,2),0)</f>
       </c>
       <c r="AH53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF53/AG53,0),6)</f>
       </c>
       <c r="AK53" s="164" t="s">
         <v>158</v>
@@ -14635,10 +14635,10 @@
       </c>
       <c r="AM53" s="166"/>
       <c r="AN53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AL$7,2),0)</f>
+        <f>=IFERROR(ROUND(AM53/$AL$7,2),0)</f>
       </c>
       <c r="AO53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM53/AN53,0),6)</f>
       </c>
       <c r="AR53" s="164" t="s">
         <v>158</v>
@@ -14648,10 +14648,10 @@
       </c>
       <c r="AT53" s="166"/>
       <c r="AU53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AS$7,2),0)</f>
+        <f>=IFERROR(ROUND(AT53/$AS$7,2),0)</f>
       </c>
       <c r="AV53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT53/AU53,0),6)</f>
       </c>
       <c r="AY53" s="164" t="s">
         <v>158</v>
@@ -14661,10 +14661,10 @@
       </c>
       <c r="BA53" s="166"/>
       <c r="BB53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AZ$7,2),0)</f>
+        <f>=IFERROR(ROUND(BA53/$AZ$7,2),0)</f>
       </c>
       <c r="BC53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA53/BB53,0),6)</f>
       </c>
       <c r="BF53" s="164" t="s">
         <v>158</v>
@@ -14674,10 +14674,10 @@
       </c>
       <c r="BH53" s="166"/>
       <c r="BI53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BG$7,2),0)</f>
+        <f>=IFERROR(ROUND(BH53/$BG$7,2),0)</f>
       </c>
       <c r="BJ53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH53/BI53,0),6)</f>
       </c>
       <c r="BM53" s="164" t="s">
         <v>158</v>
@@ -14687,10 +14687,10 @@
       </c>
       <c r="BO53" s="166"/>
       <c r="BP53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BN$7,2),0)</f>
+        <f>=IFERROR(ROUND(BO53/$BN$7,2),0)</f>
       </c>
       <c r="BQ53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO53/BP53,0),6)</f>
       </c>
       <c r="BT53" s="164" t="s">
         <v>158</v>
@@ -14700,10 +14700,10 @@
       </c>
       <c r="BV53" s="166"/>
       <c r="BW53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BU$7,2),0)</f>
+        <f>=IFERROR(ROUND(BV53/$BU$7,2),0)</f>
       </c>
       <c r="BX53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV53/BW53,0),6)</f>
       </c>
       <c r="CA53" s="164" t="s">
         <v>158</v>
@@ -14713,10 +14713,10 @@
       </c>
       <c r="CC53" s="166"/>
       <c r="CD53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CB$7,2),0)</f>
+        <f>=IFERROR(ROUND(CC53/$CB$7,2),0)</f>
       </c>
       <c r="CE53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC53/CD53,0),6)</f>
       </c>
       <c r="CH53" s="164" t="s">
         <v>158</v>
@@ -14726,10 +14726,10 @@
       </c>
       <c r="CJ53" s="166"/>
       <c r="CK53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CI$7,2),0)</f>
+        <f>=IFERROR(ROUND(CJ53/$CI$7,2),0)</f>
       </c>
       <c r="CL53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ53/CK53,0),6)</f>
       </c>
       <c r="CO53" s="164" t="s">
         <v>158</v>
@@ -14739,10 +14739,10 @@
       </c>
       <c r="CQ53" s="166"/>
       <c r="CR53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CP$7,2),0)</f>
+        <f>=IFERROR(ROUND(CQ53/$CP$7,2),0)</f>
       </c>
       <c r="CS53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ53/CR53,0),6)</f>
       </c>
       <c r="CV53" s="164" t="s">
         <v>158</v>
@@ -14752,10 +14752,10 @@
       </c>
       <c r="CX53" s="166"/>
       <c r="CY53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CW$7,2),0)</f>
+        <f>=IFERROR(ROUND(CX53/$CW$7,2),0)</f>
       </c>
       <c r="CZ53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX53/CY53,0),6)</f>
       </c>
       <c r="DC53" s="164" t="s">
         <v>158</v>
@@ -14765,10 +14765,10 @@
       </c>
       <c r="DE53" s="166"/>
       <c r="DF53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DD$7,2),0)</f>
+        <f>=IFERROR(ROUND(DE53/$DD$7,2),0)</f>
       </c>
       <c r="DG53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE53/DF53,0),6)</f>
       </c>
       <c r="DJ53" s="164" t="s">
         <v>158</v>
@@ -14778,10 +14778,10 @@
       </c>
       <c r="DL53" s="166"/>
       <c r="DM53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DK$7,2),0)</f>
+        <f>=IFERROR(ROUND(DL53/$DK$7,2),0)</f>
       </c>
       <c r="DN53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL53/DM53,0),6)</f>
       </c>
       <c r="DQ53" s="164" t="s">
         <v>158</v>
@@ -14791,10 +14791,10 @@
       </c>
       <c r="DS53" s="166"/>
       <c r="DT53" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DR$7,2),0)</f>
+        <f>=IFERROR(ROUND(DS53/$DR$7,2),0)</f>
       </c>
       <c r="DU53" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS53/DT53,0),6)</f>
       </c>
     </row>
     <row r="54">
@@ -14806,10 +14806,10 @@
       </c>
       <c r="D54" s="166"/>
       <c r="E54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$C$7,2),0)</f>
+        <f>=IFERROR(ROUND(D54/$C$7,2),0)</f>
       </c>
       <c r="F54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D54/E54,0),6)</f>
       </c>
       <c r="I54" s="164" t="s">
         <v>158</v>
@@ -14819,10 +14819,10 @@
       </c>
       <c r="K54" s="166"/>
       <c r="L54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$J$7,2),0)</f>
+        <f>=IFERROR(ROUND(K54/$J$7,2),0)</f>
       </c>
       <c r="M54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K54/L54,0),6)</f>
       </c>
       <c r="P54" s="164" t="s">
         <v>158</v>
@@ -14832,10 +14832,10 @@
       </c>
       <c r="R54" s="166"/>
       <c r="S54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$Q$7,2),0)</f>
+        <f>=IFERROR(ROUND(R54/$Q$7,2),0)</f>
       </c>
       <c r="T54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R54/S54,0),6)</f>
       </c>
       <c r="W54" s="164" t="s">
         <v>158</v>
@@ -14845,10 +14845,10 @@
       </c>
       <c r="Y54" s="166"/>
       <c r="Z54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$X$7,2),0)</f>
+        <f>=IFERROR(ROUND(Y54/$X$7,2),0)</f>
       </c>
       <c r="AA54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y54/Z54,0),6)</f>
       </c>
       <c r="AD54" s="164" t="s">
         <v>158</v>
@@ -14858,10 +14858,10 @@
       </c>
       <c r="AF54" s="166"/>
       <c r="AG54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AE$7,2),0)</f>
+        <f>=IFERROR(ROUND(AF54/$AE$7,2),0)</f>
       </c>
       <c r="AH54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF54/AG54,0),6)</f>
       </c>
       <c r="AK54" s="164" t="s">
         <v>158</v>
@@ -14871,10 +14871,10 @@
       </c>
       <c r="AM54" s="166"/>
       <c r="AN54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AL$7,2),0)</f>
+        <f>=IFERROR(ROUND(AM54/$AL$7,2),0)</f>
       </c>
       <c r="AO54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM54/AN54,0),6)</f>
       </c>
       <c r="AR54" s="164" t="s">
         <v>158</v>
@@ -14884,10 +14884,10 @@
       </c>
       <c r="AT54" s="166"/>
       <c r="AU54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AS$7,2),0)</f>
+        <f>=IFERROR(ROUND(AT54/$AS$7,2),0)</f>
       </c>
       <c r="AV54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT54/AU54,0),6)</f>
       </c>
       <c r="AY54" s="164" t="s">
         <v>158</v>
@@ -14897,10 +14897,10 @@
       </c>
       <c r="BA54" s="166"/>
       <c r="BB54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AZ$7,2),0)</f>
+        <f>=IFERROR(ROUND(BA54/$AZ$7,2),0)</f>
       </c>
       <c r="BC54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA54/BB54,0),6)</f>
       </c>
       <c r="BF54" s="164" t="s">
         <v>158</v>
@@ -14910,10 +14910,10 @@
       </c>
       <c r="BH54" s="166"/>
       <c r="BI54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BG$7,2),0)</f>
+        <f>=IFERROR(ROUND(BH54/$BG$7,2),0)</f>
       </c>
       <c r="BJ54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH54/BI54,0),6)</f>
       </c>
       <c r="BM54" s="164" t="s">
         <v>158</v>
@@ -14923,10 +14923,10 @@
       </c>
       <c r="BO54" s="166"/>
       <c r="BP54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BN$7,2),0)</f>
+        <f>=IFERROR(ROUND(BO54/$BN$7,2),0)</f>
       </c>
       <c r="BQ54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO54/BP54,0),6)</f>
       </c>
       <c r="BT54" s="164" t="s">
         <v>158</v>
@@ -14936,10 +14936,10 @@
       </c>
       <c r="BV54" s="166"/>
       <c r="BW54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BU$7,2),0)</f>
+        <f>=IFERROR(ROUND(BV54/$BU$7,2),0)</f>
       </c>
       <c r="BX54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV54/BW54,0),6)</f>
       </c>
       <c r="CA54" s="164" t="s">
         <v>158</v>
@@ -14949,10 +14949,10 @@
       </c>
       <c r="CC54" s="166"/>
       <c r="CD54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CB$7,2),0)</f>
+        <f>=IFERROR(ROUND(CC54/$CB$7,2),0)</f>
       </c>
       <c r="CE54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC54/CD54,0),6)</f>
       </c>
       <c r="CH54" s="164" t="s">
         <v>158</v>
@@ -14962,10 +14962,10 @@
       </c>
       <c r="CJ54" s="166"/>
       <c r="CK54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CI$7,2),0)</f>
+        <f>=IFERROR(ROUND(CJ54/$CI$7,2),0)</f>
       </c>
       <c r="CL54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ54/CK54,0),6)</f>
       </c>
       <c r="CO54" s="164" t="s">
         <v>158</v>
@@ -14975,10 +14975,10 @@
       </c>
       <c r="CQ54" s="166"/>
       <c r="CR54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CP$7,2),0)</f>
+        <f>=IFERROR(ROUND(CQ54/$CP$7,2),0)</f>
       </c>
       <c r="CS54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ54/CR54,0),6)</f>
       </c>
       <c r="CV54" s="164" t="s">
         <v>158</v>
@@ -14988,10 +14988,10 @@
       </c>
       <c r="CX54" s="166"/>
       <c r="CY54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CW$7,2),0)</f>
+        <f>=IFERROR(ROUND(CX54/$CW$7,2),0)</f>
       </c>
       <c r="CZ54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX54/CY54,0),6)</f>
       </c>
       <c r="DC54" s="164" t="s">
         <v>158</v>
@@ -15001,10 +15001,10 @@
       </c>
       <c r="DE54" s="166"/>
       <c r="DF54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DD$7,2),0)</f>
+        <f>=IFERROR(ROUND(DE54/$DD$7,2),0)</f>
       </c>
       <c r="DG54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE54/DF54,0),6)</f>
       </c>
       <c r="DJ54" s="164" t="s">
         <v>158</v>
@@ -15014,10 +15014,10 @@
       </c>
       <c r="DL54" s="166"/>
       <c r="DM54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DK$7,2),0)</f>
+        <f>=IFERROR(ROUND(DL54/$DK$7,2),0)</f>
       </c>
       <c r="DN54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL54/DM54,0),6)</f>
       </c>
       <c r="DQ54" s="164" t="s">
         <v>158</v>
@@ -15027,10 +15027,10 @@
       </c>
       <c r="DS54" s="166"/>
       <c r="DT54" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DR$7,2),0)</f>
+        <f>=IFERROR(ROUND(DS54/$DR$7,2),0)</f>
       </c>
       <c r="DU54" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS54/DT54,0),6)</f>
       </c>
     </row>
     <row r="55">
@@ -15042,10 +15042,10 @@
       </c>
       <c r="D55" s="166"/>
       <c r="E55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$C$7,2),0)</f>
+        <f>=IFERROR(ROUND(D55/$C$7,2),0)</f>
       </c>
       <c r="F55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(D55/E55,0),6)</f>
       </c>
       <c r="I55" s="164" t="s">
         <v>158</v>
@@ -15055,10 +15055,10 @@
       </c>
       <c r="K55" s="166"/>
       <c r="L55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$J$7,2),0)</f>
+        <f>=IFERROR(ROUND(K55/$J$7,2),0)</f>
       </c>
       <c r="M55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(K55/L55,0),6)</f>
       </c>
       <c r="P55" s="164" t="s">
         <v>158</v>
@@ -15068,10 +15068,10 @@
       </c>
       <c r="R55" s="166"/>
       <c r="S55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$Q$7,2),0)</f>
+        <f>=IFERROR(ROUND(R55/$Q$7,2),0)</f>
       </c>
       <c r="T55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(R55/S55,0),6)</f>
       </c>
       <c r="W55" s="164" t="s">
         <v>158</v>
@@ -15081,10 +15081,10 @@
       </c>
       <c r="Y55" s="166"/>
       <c r="Z55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$X$7,2),0)</f>
+        <f>=IFERROR(ROUND(Y55/$X$7,2),0)</f>
       </c>
       <c r="AA55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(Y55/Z55,0),6)</f>
       </c>
       <c r="AD55" s="164" t="s">
         <v>158</v>
@@ -15094,10 +15094,10 @@
       </c>
       <c r="AF55" s="166"/>
       <c r="AG55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AE$7,2),0)</f>
+        <f>=IFERROR(ROUND(AF55/$AE$7,2),0)</f>
       </c>
       <c r="AH55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AF55/AG55,0),6)</f>
       </c>
       <c r="AK55" s="164" t="s">
         <v>158</v>
@@ -15107,10 +15107,10 @@
       </c>
       <c r="AM55" s="166"/>
       <c r="AN55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AL$7,2),0)</f>
+        <f>=IFERROR(ROUND(AM55/$AL$7,2),0)</f>
       </c>
       <c r="AO55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AM55/AN55,0),6)</f>
       </c>
       <c r="AR55" s="164" t="s">
         <v>158</v>
@@ -15120,10 +15120,10 @@
       </c>
       <c r="AT55" s="166"/>
       <c r="AU55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AS$7,2),0)</f>
+        <f>=IFERROR(ROUND(AT55/$AS$7,2),0)</f>
       </c>
       <c r="AV55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(AT55/AU55,0),6)</f>
       </c>
       <c r="AY55" s="164" t="s">
         <v>158</v>
@@ -15133,10 +15133,10 @@
       </c>
       <c r="BA55" s="166"/>
       <c r="BB55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$AZ$7,2),0)</f>
+        <f>=IFERROR(ROUND(BA55/$AZ$7,2),0)</f>
       </c>
       <c r="BC55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BA55/BB55,0),6)</f>
       </c>
       <c r="BF55" s="164" t="s">
         <v>158</v>
@@ -15146,10 +15146,10 @@
       </c>
       <c r="BH55" s="166"/>
       <c r="BI55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BG$7,2),0)</f>
+        <f>=IFERROR(ROUND(BH55/$BG$7,2),0)</f>
       </c>
       <c r="BJ55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BH55/BI55,0),6)</f>
       </c>
       <c r="BM55" s="164" t="s">
         <v>158</v>
@@ -15159,10 +15159,10 @@
       </c>
       <c r="BO55" s="166"/>
       <c r="BP55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BN$7,2),0)</f>
+        <f>=IFERROR(ROUND(BO55/$BN$7,2),0)</f>
       </c>
       <c r="BQ55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BO55/BP55,0),6)</f>
       </c>
       <c r="BT55" s="164" t="s">
         <v>158</v>
@@ -15172,10 +15172,10 @@
       </c>
       <c r="BV55" s="166"/>
       <c r="BW55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$BU$7,2),0)</f>
+        <f>=IFERROR(ROUND(BV55/$BU$7,2),0)</f>
       </c>
       <c r="BX55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(BV55/BW55,0),6)</f>
       </c>
       <c r="CA55" s="164" t="s">
         <v>158</v>
@@ -15185,10 +15185,10 @@
       </c>
       <c r="CC55" s="166"/>
       <c r="CD55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CB$7,2),0)</f>
+        <f>=IFERROR(ROUND(CC55/$CB$7,2),0)</f>
       </c>
       <c r="CE55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CC55/CD55,0),6)</f>
       </c>
       <c r="CH55" s="164" t="s">
         <v>158</v>
@@ -15198,10 +15198,10 @@
       </c>
       <c r="CJ55" s="166"/>
       <c r="CK55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CI$7,2),0)</f>
+        <f>=IFERROR(ROUND(CJ55/$CI$7,2),0)</f>
       </c>
       <c r="CL55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CJ55/CK55,0),6)</f>
       </c>
       <c r="CO55" s="164" t="s">
         <v>158</v>
@@ -15211,10 +15211,10 @@
       </c>
       <c r="CQ55" s="166"/>
       <c r="CR55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CP$7,2),0)</f>
+        <f>=IFERROR(ROUND(CQ55/$CP$7,2),0)</f>
       </c>
       <c r="CS55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CQ55/CR55,0),6)</f>
       </c>
       <c r="CV55" s="164" t="s">
         <v>158</v>
@@ -15224,10 +15224,10 @@
       </c>
       <c r="CX55" s="166"/>
       <c r="CY55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$CW$7,2),0)</f>
+        <f>=IFERROR(ROUND(CX55/$CW$7,2),0)</f>
       </c>
       <c r="CZ55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(CX55/CY55,0),6)</f>
       </c>
       <c r="DC55" s="164" t="s">
         <v>158</v>
@@ -15237,10 +15237,10 @@
       </c>
       <c r="DE55" s="166"/>
       <c r="DF55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DD$7,2),0)</f>
+        <f>=IFERROR(ROUND(DE55/$DD$7,2),0)</f>
       </c>
       <c r="DG55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DE55/DF55,0),6)</f>
       </c>
       <c r="DJ55" s="164" t="s">
         <v>158</v>
@@ -15250,10 +15250,10 @@
       </c>
       <c r="DL55" s="166"/>
       <c r="DM55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DK$7,2),0)</f>
+        <f>=IFERROR(ROUND(DL55/$DK$7,2),0)</f>
       </c>
       <c r="DN55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DL55/DM55,0),6)</f>
       </c>
       <c r="DQ55" s="164" t="s">
         <v>158</v>
@@ -15263,10 +15263,10 @@
       </c>
       <c r="DS55" s="166"/>
       <c r="DT55" s="174" t="str">
-        <f>=IFERROR(ROUND([@[Einnahmen (LC)]]/$DR$7,2),0)</f>
+        <f>=IFERROR(ROUND(DS55/$DR$7,2),0)</f>
       </c>
       <c r="DU55" s="168" t="str">
-        <f>=ROUND(IFERROR([@[Einnahmen (LC)]]/[@[Einnahmen (EUR)]],0),6)</f>
+        <f>=ROUND(IFERROR(DS55/DT55,0),6)</f>
       </c>
     </row>
     <row r="56">

</xml_diff>

<commit_message>
feat(vorpruefung): add Mittelanforderung implementation
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -11,6 +11,7 @@
     <sheet name="I. Budget" sheetId="3" r:id="rId6"/>
     <sheet name="II. KMW-Mittel" sheetId="4" r:id="rId7"/>
     <sheet name="III. Finanzberichte" sheetId="5" r:id="rId8"/>
+    <sheet name="IV. MA" sheetId="6" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="Saldovortrag_LW">'Dashboard'!$C$13</definedName>
@@ -99,13 +100,31 @@
     <definedName name="FB_Kurs_18">'III. Finanzberichte'!$DR$7</definedName>
     <definedName name="FB_SaldoLC_18">'III. Finanzberichte'!$DR$29</definedName>
     <definedName name="FB_SaldoEUR_18">'III. Finanzberichte'!$DS$29</definedName>
+    <definedName name="MA_Kurs_1">'IV. MA'!$C$7</definedName>
+    <definedName name="MA_Kurs_2">'IV. MA'!$G$7</definedName>
+    <definedName name="MA_Kurs_3">'IV. MA'!$K$7</definedName>
+    <definedName name="MA_Kurs_4">'IV. MA'!$O$7</definedName>
+    <definedName name="MA_Kurs_5">'IV. MA'!$S$7</definedName>
+    <definedName name="MA_Kurs_6">'IV. MA'!$W$7</definedName>
+    <definedName name="MA_Kurs_7">'IV. MA'!$AA$7</definedName>
+    <definedName name="MA_Kurs_8">'IV. MA'!$AE$7</definedName>
+    <definedName name="MA_Kurs_9">'IV. MA'!$AI$7</definedName>
+    <definedName name="MA_Kurs_10">'IV. MA'!$AM$7</definedName>
+    <definedName name="MA_Kurs_11">'IV. MA'!$AQ$7</definedName>
+    <definedName name="MA_Kurs_12">'IV. MA'!$AU$7</definedName>
+    <definedName name="MA_Kurs_13">'IV. MA'!$AY$7</definedName>
+    <definedName name="MA_Kurs_14">'IV. MA'!$BC$7</definedName>
+    <definedName name="MA_Kurs_15">'IV. MA'!$BG$7</definedName>
+    <definedName name="MA_Kurs_16">'IV. MA'!$BK$7</definedName>
+    <definedName name="MA_Kurs_17">'IV. MA'!$BO$7</definedName>
+    <definedName name="MA_Kurs_18">'IV. MA'!$BS$7</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="313">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1020,21 +1039,46 @@
   </si>
   <si>
     <t>Saldo der Vorperiode</t>
+  </si>
+  <si>
+    <t>OANDA-Kurs:</t>
+  </si>
+  <si>
+    <t>Angefordert (LC)</t>
+  </si>
+  <si>
+    <t>Angefordert (EUR)</t>
+  </si>
+  <si>
+    <t>SUMME</t>
+  </si>
+  <si>
+    <t>Gesamtbedarf an Mitteln:</t>
+  </si>
+  <si>
+    <t>abzueglich Eigenmittel:</t>
+  </si>
+  <si>
+    <t>abzueglich Drittmittel:</t>
+  </si>
+  <si>
+    <t>KMW-Mittel Anforderung:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="168" formatCode="0.000000"/>
     <numFmt numFmtId="169" formatCode="@"/>
+    <numFmt numFmtId="170" formatCode="DD.MM.YYYY"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1166,8 +1210,15 @@
       <color rgb="FF808080"/>
       <sz val="24"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1214,8 +1265,13 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="49">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -1751,11 +1807,30 @@
         <color rgb="FFD3D3D3"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="double">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="double">
+        <color rgb="FF808080"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="191">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
@@ -2281,6 +2356,51 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="44" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="3" fillId="5" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="49" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="8" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3257,6 +3377,30 @@
 </table>
 </file>
 
+<file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="MA_1" displayName="MA_1" ref="B9:D18">
+  <autoFilter ref="B9:D18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="MA_2" displayName="MA_2" ref="F9:H18">
+  <autoFilter ref="F9:H18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Einnahmen_WK_1" displayName="Einnahmen_WK_1" ref="B49:F56">
   <autoFilter ref="B49:F56"/>
@@ -3271,6 +3415,126 @@
 </table>
 </file>
 
+<file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="MA_3" displayName="MA_3" ref="J9:L18">
+  <autoFilter ref="J9:L18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="MA_4" displayName="MA_4" ref="N9:P18">
+  <autoFilter ref="N9:P18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="MA_5" displayName="MA_5" ref="R9:T18">
+  <autoFilter ref="R9:T18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="MA_6" displayName="MA_6" ref="V9:X18">
+  <autoFilter ref="V9:X18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="MA_7" displayName="MA_7" ref="Z9:AB18">
+  <autoFilter ref="Z9:AB18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="MA_8" displayName="MA_8" ref="AD9:AF18">
+  <autoFilter ref="AD9:AF18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="MA_9" displayName="MA_9" ref="AH9:AJ18">
+  <autoFilter ref="AH9:AJ18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="MA_10" displayName="MA_10" ref="AL9:AN18">
+  <autoFilter ref="AL9:AN18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="MA_11" displayName="MA_11" ref="AP9:AR18">
+  <autoFilter ref="AP9:AR18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="MA_12" displayName="MA_12" ref="AT9:AV18">
+  <autoFilter ref="AT9:AV18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Ausgaben_2" displayName="Ausgaben_2" ref="I18:M27">
   <autoFilter ref="I18:M27"/>
@@ -3280,6 +3544,78 @@
     <tableColumn id="3" name="Ausgaben (EUR)"/>
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="MA_13" displayName="MA_13" ref="AX9:AZ18">
+  <autoFilter ref="AX9:AZ18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="MA_14" displayName="MA_14" ref="BB9:BD18">
+  <autoFilter ref="BB9:BD18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table72.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="72" name="MA_15" displayName="MA_15" ref="BF9:BH18">
+  <autoFilter ref="BF9:BH18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table73.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="73" name="MA_16" displayName="MA_16" ref="BJ9:BL18">
+  <autoFilter ref="BJ9:BL18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table74.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="MA_17" displayName="MA_17" ref="BN9:BP18">
+  <autoFilter ref="BN9:BP18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+</table>
+</file>
+
+<file path=xl/tables/table75.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="MA_18" displayName="MA_18" ref="BR9:BT18">
+  <autoFilter ref="BR9:BT18"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Kostenkategorie"/>
+    <tableColumn id="2" name="Angefordert (LC)"/>
+    <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
@@ -16035,4 +16371,2714 @@
     <tablePart r:id="rId54"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr>
+    <tabColor rgb="FFFF00"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" hidden="true" max="1" min="1" width="9.140625"/>
+    <col customWidth="true" max="2" min="2" width="25"/>
+    <col customWidth="true" max="4" min="3" width="18"/>
+    <col customWidth="true" max="6" min="6" width="25"/>
+    <col customWidth="true" max="8" min="7" width="18"/>
+    <col customWidth="true" max="10" min="10" width="25"/>
+    <col customWidth="true" max="12" min="11" width="18"/>
+    <col customWidth="true" max="14" min="14" width="25"/>
+    <col customWidth="true" max="16" min="15" width="18"/>
+    <col customWidth="true" max="18" min="18" width="25"/>
+    <col customWidth="true" max="20" min="19" width="18"/>
+    <col customWidth="true" max="22" min="22" width="25"/>
+    <col customWidth="true" max="24" min="23" width="18"/>
+    <col customWidth="true" max="26" min="26" width="25"/>
+    <col customWidth="true" max="28" min="27" width="18"/>
+    <col customWidth="true" max="30" min="30" width="25"/>
+    <col customWidth="true" max="32" min="31" width="18"/>
+    <col customWidth="true" max="34" min="34" width="25"/>
+    <col customWidth="true" max="36" min="35" width="18"/>
+    <col customWidth="true" max="38" min="38" width="25"/>
+    <col customWidth="true" max="40" min="39" width="18"/>
+    <col customWidth="true" max="42" min="42" width="25"/>
+    <col customWidth="true" max="44" min="43" width="18"/>
+    <col customWidth="true" max="46" min="46" width="25"/>
+    <col customWidth="true" max="48" min="47" width="18"/>
+    <col customWidth="true" max="50" min="50" width="25"/>
+    <col customWidth="true" max="52" min="51" width="18"/>
+    <col customWidth="true" max="54" min="54" width="25"/>
+    <col customWidth="true" max="56" min="55" width="18"/>
+    <col customWidth="true" max="58" min="58" width="25"/>
+    <col customWidth="true" max="60" min="59" width="18"/>
+    <col customWidth="true" max="62" min="62" width="25"/>
+    <col customWidth="true" max="64" min="63" width="18"/>
+    <col customWidth="true" max="66" min="66" width="25"/>
+    <col customWidth="true" max="68" min="67" width="18"/>
+    <col customWidth="true" max="70" min="70" width="25"/>
+    <col customWidth="true" max="72" min="71" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="I3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="M3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="U3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="Y3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="AC3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="AG3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="AK3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="AO3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="AS3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="AW3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="BA3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="BE3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="BI3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="BM3" s="175" t="s">
+        <v>302</v>
+      </c>
+      <c r="BQ3" s="175" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="C5" s="176" t="s">
+        <v>226</v>
+      </c>
+      <c r="D5" s="176"/>
+      <c r="F5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="G5" s="176" t="s">
+        <v>227</v>
+      </c>
+      <c r="H5" s="176"/>
+      <c r="J5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="K5" s="176" t="s">
+        <v>228</v>
+      </c>
+      <c r="L5" s="176"/>
+      <c r="N5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="O5" s="176" t="s">
+        <v>229</v>
+      </c>
+      <c r="P5" s="176"/>
+      <c r="R5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="S5" s="176" t="s">
+        <v>230</v>
+      </c>
+      <c r="T5" s="176"/>
+      <c r="V5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="W5" s="176" t="s">
+        <v>231</v>
+      </c>
+      <c r="X5" s="176"/>
+      <c r="Z5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="AA5" s="176" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB5" s="176"/>
+      <c r="AD5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="AE5" s="176" t="s">
+        <v>233</v>
+      </c>
+      <c r="AF5" s="176"/>
+      <c r="AH5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI5" s="176" t="s">
+        <v>234</v>
+      </c>
+      <c r="AJ5" s="176"/>
+      <c r="AL5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="AM5" s="176" t="s">
+        <v>235</v>
+      </c>
+      <c r="AN5" s="176"/>
+      <c r="AP5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="AQ5" s="176" t="s">
+        <v>236</v>
+      </c>
+      <c r="AR5" s="176"/>
+      <c r="AT5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="AU5" s="176" t="s">
+        <v>237</v>
+      </c>
+      <c r="AV5" s="176"/>
+      <c r="AX5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="AY5" s="176" t="s">
+        <v>238</v>
+      </c>
+      <c r="AZ5" s="176"/>
+      <c r="BB5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="BC5" s="176" t="s">
+        <v>239</v>
+      </c>
+      <c r="BD5" s="176"/>
+      <c r="BF5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="BG5" s="176" t="s">
+        <v>240</v>
+      </c>
+      <c r="BH5" s="176"/>
+      <c r="BJ5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="BK5" s="176" t="s">
+        <v>241</v>
+      </c>
+      <c r="BL5" s="176"/>
+      <c r="BN5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="BO5" s="176" t="s">
+        <v>242</v>
+      </c>
+      <c r="BP5" s="176"/>
+      <c r="BR5" s="104" t="s">
+        <v>267</v>
+      </c>
+      <c r="BS5" s="176" t="s">
+        <v>243</v>
+      </c>
+      <c r="BT5" s="176"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>231</v>
+      </c>
+      <c r="B6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="C6" s="177"/>
+      <c r="D6" s="177"/>
+      <c r="F6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="G6" s="177"/>
+      <c r="H6" s="177"/>
+      <c r="J6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="K6" s="177"/>
+      <c r="L6" s="177"/>
+      <c r="N6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="O6" s="177"/>
+      <c r="P6" s="177"/>
+      <c r="R6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="S6" s="177"/>
+      <c r="T6" s="177"/>
+      <c r="V6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="W6" s="177"/>
+      <c r="X6" s="177"/>
+      <c r="Z6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="AA6" s="177"/>
+      <c r="AB6" s="177"/>
+      <c r="AD6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="AE6" s="177"/>
+      <c r="AF6" s="177"/>
+      <c r="AH6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="AI6" s="177"/>
+      <c r="AJ6" s="177"/>
+      <c r="AL6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="AM6" s="177"/>
+      <c r="AN6" s="177"/>
+      <c r="AP6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="AQ6" s="177"/>
+      <c r="AR6" s="177"/>
+      <c r="AT6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="AU6" s="177"/>
+      <c r="AV6" s="177"/>
+      <c r="AX6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="AY6" s="177"/>
+      <c r="AZ6" s="177"/>
+      <c r="BB6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="BC6" s="177"/>
+      <c r="BD6" s="177"/>
+      <c r="BF6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="BG6" s="177"/>
+      <c r="BH6" s="177"/>
+      <c r="BJ6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="BK6" s="177"/>
+      <c r="BL6" s="177"/>
+      <c r="BN6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="BO6" s="177"/>
+      <c r="BP6" s="177"/>
+      <c r="BR6" s="104" t="s">
+        <v>268</v>
+      </c>
+      <c r="BS6" s="177"/>
+      <c r="BT6" s="177"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>232</v>
+      </c>
+      <c r="B7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="C7" s="178"/>
+      <c r="D7" s="178"/>
+      <c r="F7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="G7" s="178"/>
+      <c r="H7" s="178"/>
+      <c r="J7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="K7" s="178"/>
+      <c r="L7" s="178"/>
+      <c r="N7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="O7" s="178"/>
+      <c r="P7" s="178"/>
+      <c r="R7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="S7" s="178"/>
+      <c r="T7" s="178"/>
+      <c r="V7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="W7" s="178"/>
+      <c r="X7" s="178"/>
+      <c r="Z7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="AA7" s="178"/>
+      <c r="AB7" s="178"/>
+      <c r="AD7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="AE7" s="178"/>
+      <c r="AF7" s="178"/>
+      <c r="AH7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="AI7" s="178"/>
+      <c r="AJ7" s="178"/>
+      <c r="AL7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="AM7" s="178"/>
+      <c r="AN7" s="178"/>
+      <c r="AP7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="AQ7" s="178"/>
+      <c r="AR7" s="178"/>
+      <c r="AT7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="AU7" s="178"/>
+      <c r="AV7" s="178"/>
+      <c r="AX7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="AY7" s="178"/>
+      <c r="AZ7" s="178"/>
+      <c r="BB7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="BC7" s="178"/>
+      <c r="BD7" s="178"/>
+      <c r="BF7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="BG7" s="178"/>
+      <c r="BH7" s="178"/>
+      <c r="BJ7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="BK7" s="178"/>
+      <c r="BL7" s="178"/>
+      <c r="BN7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="BO7" s="178"/>
+      <c r="BP7" s="178"/>
+      <c r="BR7" s="104" t="s">
+        <v>305</v>
+      </c>
+      <c r="BS7" s="178"/>
+      <c r="BT7" s="178"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="D9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="F9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="H9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="J9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="K9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="L9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="N9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="O9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="P9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="R9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="S9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="T9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="V9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="W9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="X9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="Z9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="AA9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="AB9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="AD9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="AE9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="AF9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="AH9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="AI9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="AJ9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="AL9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="AM9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="AN9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="AP9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="AQ9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="AR9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="AT9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="AU9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="AV9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="AX9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="AY9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="AZ9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="BB9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="BC9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="BD9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="BF9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="BG9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="BH9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="BJ9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="BK9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="BL9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="BN9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="BO9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="BP9" s="179" t="s">
+        <v>307</v>
+      </c>
+      <c r="BR9" s="179" t="s">
+        <v>202</v>
+      </c>
+      <c r="BS9" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="BT9" s="179" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="181" t="str">
+        <f>=IFERROR(ROUND(C10/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="G10" s="24"/>
+      <c r="H10" s="181" t="str">
+        <f>=IFERROR(ROUND(G10/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="K10" s="24"/>
+      <c r="L10" s="181" t="str">
+        <f>=IFERROR(ROUND(K10/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="O10" s="24"/>
+      <c r="P10" s="181" t="str">
+        <f>=IFERROR(ROUND(O10/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="S10" s="24"/>
+      <c r="T10" s="181" t="str">
+        <f>=IFERROR(ROUND(S10/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="W10" s="24"/>
+      <c r="X10" s="181" t="str">
+        <f>=IFERROR(ROUND(W10/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="AA10" s="24"/>
+      <c r="AB10" s="181" t="str">
+        <f>=IFERROR(ROUND(AA10/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="AE10" s="24"/>
+      <c r="AF10" s="181" t="str">
+        <f>=IFERROR(ROUND(AE10/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="AI10" s="24"/>
+      <c r="AJ10" s="181" t="str">
+        <f>=IFERROR(ROUND(AI10/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="AM10" s="24"/>
+      <c r="AN10" s="181" t="str">
+        <f>=IFERROR(ROUND(AM10/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="AQ10" s="24"/>
+      <c r="AR10" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ10/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="AU10" s="24"/>
+      <c r="AV10" s="181" t="str">
+        <f>=IFERROR(ROUND(AU10/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="AY10" s="24"/>
+      <c r="AZ10" s="181" t="str">
+        <f>=IFERROR(ROUND(AY10/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="BC10" s="24"/>
+      <c r="BD10" s="181" t="str">
+        <f>=IFERROR(ROUND(BC10/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="BG10" s="24"/>
+      <c r="BH10" s="181" t="str">
+        <f>=IFERROR(ROUND(BG10/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="BK10" s="24"/>
+      <c r="BL10" s="181" t="str">
+        <f>=IFERROR(ROUND(BK10/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="BO10" s="24"/>
+      <c r="BP10" s="181" t="str">
+        <f>=IFERROR(ROUND(BO10/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR10" s="180" t="s">
+        <v>205</v>
+      </c>
+      <c r="BS10" s="24"/>
+      <c r="BT10" s="181" t="str">
+        <f>=IFERROR(ROUND(BS10/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="C11" s="24"/>
+      <c r="D11" s="181" t="str">
+        <f>=IFERROR(ROUND(C11/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="G11" s="24"/>
+      <c r="H11" s="181" t="str">
+        <f>=IFERROR(ROUND(G11/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="K11" s="24"/>
+      <c r="L11" s="181" t="str">
+        <f>=IFERROR(ROUND(K11/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="O11" s="24"/>
+      <c r="P11" s="181" t="str">
+        <f>=IFERROR(ROUND(O11/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="S11" s="24"/>
+      <c r="T11" s="181" t="str">
+        <f>=IFERROR(ROUND(S11/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="W11" s="24"/>
+      <c r="X11" s="181" t="str">
+        <f>=IFERROR(ROUND(W11/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="AA11" s="24"/>
+      <c r="AB11" s="181" t="str">
+        <f>=IFERROR(ROUND(AA11/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="AE11" s="24"/>
+      <c r="AF11" s="181" t="str">
+        <f>=IFERROR(ROUND(AE11/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="AI11" s="24"/>
+      <c r="AJ11" s="181" t="str">
+        <f>=IFERROR(ROUND(AI11/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="AM11" s="24"/>
+      <c r="AN11" s="181" t="str">
+        <f>=IFERROR(ROUND(AM11/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ11" s="24"/>
+      <c r="AR11" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ11/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="AU11" s="24"/>
+      <c r="AV11" s="181" t="str">
+        <f>=IFERROR(ROUND(AU11/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="AY11" s="24"/>
+      <c r="AZ11" s="181" t="str">
+        <f>=IFERROR(ROUND(AY11/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="BC11" s="24"/>
+      <c r="BD11" s="181" t="str">
+        <f>=IFERROR(ROUND(BC11/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="BG11" s="24"/>
+      <c r="BH11" s="181" t="str">
+        <f>=IFERROR(ROUND(BG11/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="BK11" s="24"/>
+      <c r="BL11" s="181" t="str">
+        <f>=IFERROR(ROUND(BK11/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="BO11" s="24"/>
+      <c r="BP11" s="181" t="str">
+        <f>=IFERROR(ROUND(BO11/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR11" s="180" t="s">
+        <v>206</v>
+      </c>
+      <c r="BS11" s="24"/>
+      <c r="BT11" s="181" t="str">
+        <f>=IFERROR(ROUND(BS11/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>237</v>
+      </c>
+      <c r="B12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="C12" s="24"/>
+      <c r="D12" s="181" t="str">
+        <f>=IFERROR(ROUND(C12/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="G12" s="24"/>
+      <c r="H12" s="181" t="str">
+        <f>=IFERROR(ROUND(G12/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="K12" s="24"/>
+      <c r="L12" s="181" t="str">
+        <f>=IFERROR(ROUND(K12/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="O12" s="24"/>
+      <c r="P12" s="181" t="str">
+        <f>=IFERROR(ROUND(O12/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="S12" s="24"/>
+      <c r="T12" s="181" t="str">
+        <f>=IFERROR(ROUND(S12/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="W12" s="24"/>
+      <c r="X12" s="181" t="str">
+        <f>=IFERROR(ROUND(W12/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="AA12" s="24"/>
+      <c r="AB12" s="181" t="str">
+        <f>=IFERROR(ROUND(AA12/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="AE12" s="24"/>
+      <c r="AF12" s="181" t="str">
+        <f>=IFERROR(ROUND(AE12/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="AI12" s="24"/>
+      <c r="AJ12" s="181" t="str">
+        <f>=IFERROR(ROUND(AI12/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="AM12" s="24"/>
+      <c r="AN12" s="181" t="str">
+        <f>=IFERROR(ROUND(AM12/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="AQ12" s="24"/>
+      <c r="AR12" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ12/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="AU12" s="24"/>
+      <c r="AV12" s="181" t="str">
+        <f>=IFERROR(ROUND(AU12/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="AY12" s="24"/>
+      <c r="AZ12" s="181" t="str">
+        <f>=IFERROR(ROUND(AY12/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="BC12" s="24"/>
+      <c r="BD12" s="181" t="str">
+        <f>=IFERROR(ROUND(BC12/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="BG12" s="24"/>
+      <c r="BH12" s="181" t="str">
+        <f>=IFERROR(ROUND(BG12/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="BK12" s="24"/>
+      <c r="BL12" s="181" t="str">
+        <f>=IFERROR(ROUND(BK12/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="BO12" s="24"/>
+      <c r="BP12" s="181" t="str">
+        <f>=IFERROR(ROUND(BO12/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR12" s="180" t="s">
+        <v>207</v>
+      </c>
+      <c r="BS12" s="24"/>
+      <c r="BT12" s="181" t="str">
+        <f>=IFERROR(ROUND(BS12/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>238</v>
+      </c>
+      <c r="B13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="C13" s="24"/>
+      <c r="D13" s="181" t="str">
+        <f>=IFERROR(ROUND(C13/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="G13" s="24"/>
+      <c r="H13" s="181" t="str">
+        <f>=IFERROR(ROUND(G13/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="K13" s="24"/>
+      <c r="L13" s="181" t="str">
+        <f>=IFERROR(ROUND(K13/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="O13" s="24"/>
+      <c r="P13" s="181" t="str">
+        <f>=IFERROR(ROUND(O13/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="S13" s="24"/>
+      <c r="T13" s="181" t="str">
+        <f>=IFERROR(ROUND(S13/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="W13" s="24"/>
+      <c r="X13" s="181" t="str">
+        <f>=IFERROR(ROUND(W13/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="AA13" s="24"/>
+      <c r="AB13" s="181" t="str">
+        <f>=IFERROR(ROUND(AA13/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="AE13" s="24"/>
+      <c r="AF13" s="181" t="str">
+        <f>=IFERROR(ROUND(AE13/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="AI13" s="24"/>
+      <c r="AJ13" s="181" t="str">
+        <f>=IFERROR(ROUND(AI13/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="AM13" s="24"/>
+      <c r="AN13" s="181" t="str">
+        <f>=IFERROR(ROUND(AM13/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="AQ13" s="24"/>
+      <c r="AR13" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ13/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="AU13" s="24"/>
+      <c r="AV13" s="181" t="str">
+        <f>=IFERROR(ROUND(AU13/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="AY13" s="24"/>
+      <c r="AZ13" s="181" t="str">
+        <f>=IFERROR(ROUND(AY13/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="BC13" s="24"/>
+      <c r="BD13" s="181" t="str">
+        <f>=IFERROR(ROUND(BC13/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="BG13" s="24"/>
+      <c r="BH13" s="181" t="str">
+        <f>=IFERROR(ROUND(BG13/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="BK13" s="24"/>
+      <c r="BL13" s="181" t="str">
+        <f>=IFERROR(ROUND(BK13/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="BO13" s="24"/>
+      <c r="BP13" s="181" t="str">
+        <f>=IFERROR(ROUND(BO13/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR13" s="180" t="s">
+        <v>208</v>
+      </c>
+      <c r="BS13" s="24"/>
+      <c r="BT13" s="181" t="str">
+        <f>=IFERROR(ROUND(BS13/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>239</v>
+      </c>
+      <c r="B14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="C14" s="24"/>
+      <c r="D14" s="181" t="str">
+        <f>=IFERROR(ROUND(C14/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="G14" s="24"/>
+      <c r="H14" s="181" t="str">
+        <f>=IFERROR(ROUND(G14/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="K14" s="24"/>
+      <c r="L14" s="181" t="str">
+        <f>=IFERROR(ROUND(K14/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="O14" s="24"/>
+      <c r="P14" s="181" t="str">
+        <f>=IFERROR(ROUND(O14/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="S14" s="24"/>
+      <c r="T14" s="181" t="str">
+        <f>=IFERROR(ROUND(S14/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="W14" s="24"/>
+      <c r="X14" s="181" t="str">
+        <f>=IFERROR(ROUND(W14/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="AA14" s="24"/>
+      <c r="AB14" s="181" t="str">
+        <f>=IFERROR(ROUND(AA14/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="AE14" s="24"/>
+      <c r="AF14" s="181" t="str">
+        <f>=IFERROR(ROUND(AE14/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="AI14" s="24"/>
+      <c r="AJ14" s="181" t="str">
+        <f>=IFERROR(ROUND(AI14/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="AM14" s="24"/>
+      <c r="AN14" s="181" t="str">
+        <f>=IFERROR(ROUND(AM14/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="AQ14" s="24"/>
+      <c r="AR14" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ14/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="AU14" s="24"/>
+      <c r="AV14" s="181" t="str">
+        <f>=IFERROR(ROUND(AU14/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="AY14" s="24"/>
+      <c r="AZ14" s="181" t="str">
+        <f>=IFERROR(ROUND(AY14/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="BC14" s="24"/>
+      <c r="BD14" s="181" t="str">
+        <f>=IFERROR(ROUND(BC14/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="BG14" s="24"/>
+      <c r="BH14" s="181" t="str">
+        <f>=IFERROR(ROUND(BG14/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="BK14" s="24"/>
+      <c r="BL14" s="181" t="str">
+        <f>=IFERROR(ROUND(BK14/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="BO14" s="24"/>
+      <c r="BP14" s="181" t="str">
+        <f>=IFERROR(ROUND(BO14/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR14" s="180" t="s">
+        <v>209</v>
+      </c>
+      <c r="BS14" s="24"/>
+      <c r="BT14" s="181" t="str">
+        <f>=IFERROR(ROUND(BS14/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>240</v>
+      </c>
+      <c r="B15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="C15" s="24"/>
+      <c r="D15" s="181" t="str">
+        <f>=IFERROR(ROUND(C15/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="G15" s="24"/>
+      <c r="H15" s="181" t="str">
+        <f>=IFERROR(ROUND(G15/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="K15" s="24"/>
+      <c r="L15" s="181" t="str">
+        <f>=IFERROR(ROUND(K15/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="O15" s="24"/>
+      <c r="P15" s="181" t="str">
+        <f>=IFERROR(ROUND(O15/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="S15" s="24"/>
+      <c r="T15" s="181" t="str">
+        <f>=IFERROR(ROUND(S15/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="W15" s="24"/>
+      <c r="X15" s="181" t="str">
+        <f>=IFERROR(ROUND(W15/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="AA15" s="24"/>
+      <c r="AB15" s="181" t="str">
+        <f>=IFERROR(ROUND(AA15/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="AE15" s="24"/>
+      <c r="AF15" s="181" t="str">
+        <f>=IFERROR(ROUND(AE15/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="AI15" s="24"/>
+      <c r="AJ15" s="181" t="str">
+        <f>=IFERROR(ROUND(AI15/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="AM15" s="24"/>
+      <c r="AN15" s="181" t="str">
+        <f>=IFERROR(ROUND(AM15/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="AQ15" s="24"/>
+      <c r="AR15" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ15/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="AU15" s="24"/>
+      <c r="AV15" s="181" t="str">
+        <f>=IFERROR(ROUND(AU15/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="AY15" s="24"/>
+      <c r="AZ15" s="181" t="str">
+        <f>=IFERROR(ROUND(AY15/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="BC15" s="24"/>
+      <c r="BD15" s="181" t="str">
+        <f>=IFERROR(ROUND(BC15/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="BG15" s="24"/>
+      <c r="BH15" s="181" t="str">
+        <f>=IFERROR(ROUND(BG15/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="BK15" s="24"/>
+      <c r="BL15" s="181" t="str">
+        <f>=IFERROR(ROUND(BK15/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="BO15" s="24"/>
+      <c r="BP15" s="181" t="str">
+        <f>=IFERROR(ROUND(BO15/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR15" s="180" t="s">
+        <v>210</v>
+      </c>
+      <c r="BS15" s="24"/>
+      <c r="BT15" s="181" t="str">
+        <f>=IFERROR(ROUND(BS15/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>241</v>
+      </c>
+      <c r="B16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="C16" s="24"/>
+      <c r="D16" s="181" t="str">
+        <f>=IFERROR(ROUND(C16/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="G16" s="24"/>
+      <c r="H16" s="181" t="str">
+        <f>=IFERROR(ROUND(G16/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="K16" s="24"/>
+      <c r="L16" s="181" t="str">
+        <f>=IFERROR(ROUND(K16/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="O16" s="24"/>
+      <c r="P16" s="181" t="str">
+        <f>=IFERROR(ROUND(O16/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="S16" s="24"/>
+      <c r="T16" s="181" t="str">
+        <f>=IFERROR(ROUND(S16/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="W16" s="24"/>
+      <c r="X16" s="181" t="str">
+        <f>=IFERROR(ROUND(W16/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="AA16" s="24"/>
+      <c r="AB16" s="181" t="str">
+        <f>=IFERROR(ROUND(AA16/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="AE16" s="24"/>
+      <c r="AF16" s="181" t="str">
+        <f>=IFERROR(ROUND(AE16/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="AI16" s="24"/>
+      <c r="AJ16" s="181" t="str">
+        <f>=IFERROR(ROUND(AI16/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="AM16" s="24"/>
+      <c r="AN16" s="181" t="str">
+        <f>=IFERROR(ROUND(AM16/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="AQ16" s="24"/>
+      <c r="AR16" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ16/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="AU16" s="24"/>
+      <c r="AV16" s="181" t="str">
+        <f>=IFERROR(ROUND(AU16/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="AY16" s="24"/>
+      <c r="AZ16" s="181" t="str">
+        <f>=IFERROR(ROUND(AY16/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="BC16" s="24"/>
+      <c r="BD16" s="181" t="str">
+        <f>=IFERROR(ROUND(BC16/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="BG16" s="24"/>
+      <c r="BH16" s="181" t="str">
+        <f>=IFERROR(ROUND(BG16/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="BK16" s="24"/>
+      <c r="BL16" s="181" t="str">
+        <f>=IFERROR(ROUND(BK16/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="BO16" s="24"/>
+      <c r="BP16" s="181" t="str">
+        <f>=IFERROR(ROUND(BO16/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR16" s="180" t="s">
+        <v>211</v>
+      </c>
+      <c r="BS16" s="24"/>
+      <c r="BT16" s="181" t="str">
+        <f>=IFERROR(ROUND(BS16/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>242</v>
+      </c>
+      <c r="B17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="C17" s="24"/>
+      <c r="D17" s="181" t="str">
+        <f>=IFERROR(ROUND(C17/MA_Kurs_1,2),0)</f>
+      </c>
+      <c r="F17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="G17" s="24"/>
+      <c r="H17" s="181" t="str">
+        <f>=IFERROR(ROUND(G17/MA_Kurs_2,2),0)</f>
+      </c>
+      <c r="J17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="K17" s="24"/>
+      <c r="L17" s="181" t="str">
+        <f>=IFERROR(ROUND(K17/MA_Kurs_3,2),0)</f>
+      </c>
+      <c r="N17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="O17" s="24"/>
+      <c r="P17" s="181" t="str">
+        <f>=IFERROR(ROUND(O17/MA_Kurs_4,2),0)</f>
+      </c>
+      <c r="R17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="S17" s="24"/>
+      <c r="T17" s="181" t="str">
+        <f>=IFERROR(ROUND(S17/MA_Kurs_5,2),0)</f>
+      </c>
+      <c r="V17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="W17" s="24"/>
+      <c r="X17" s="181" t="str">
+        <f>=IFERROR(ROUND(W17/MA_Kurs_6,2),0)</f>
+      </c>
+      <c r="Z17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="AA17" s="24"/>
+      <c r="AB17" s="181" t="str">
+        <f>=IFERROR(ROUND(AA17/MA_Kurs_7,2),0)</f>
+      </c>
+      <c r="AD17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="AE17" s="24"/>
+      <c r="AF17" s="181" t="str">
+        <f>=IFERROR(ROUND(AE17/MA_Kurs_8,2),0)</f>
+      </c>
+      <c r="AH17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="AI17" s="24"/>
+      <c r="AJ17" s="181" t="str">
+        <f>=IFERROR(ROUND(AI17/MA_Kurs_9,2),0)</f>
+      </c>
+      <c r="AL17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="AM17" s="24"/>
+      <c r="AN17" s="181" t="str">
+        <f>=IFERROR(ROUND(AM17/MA_Kurs_10,2),0)</f>
+      </c>
+      <c r="AP17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="AQ17" s="24"/>
+      <c r="AR17" s="181" t="str">
+        <f>=IFERROR(ROUND(AQ17/MA_Kurs_11,2),0)</f>
+      </c>
+      <c r="AT17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="AU17" s="24"/>
+      <c r="AV17" s="181" t="str">
+        <f>=IFERROR(ROUND(AU17/MA_Kurs_12,2),0)</f>
+      </c>
+      <c r="AX17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="AY17" s="24"/>
+      <c r="AZ17" s="181" t="str">
+        <f>=IFERROR(ROUND(AY17/MA_Kurs_13,2),0)</f>
+      </c>
+      <c r="BB17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="BC17" s="24"/>
+      <c r="BD17" s="181" t="str">
+        <f>=IFERROR(ROUND(BC17/MA_Kurs_14,2),0)</f>
+      </c>
+      <c r="BF17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="BG17" s="24"/>
+      <c r="BH17" s="181" t="str">
+        <f>=IFERROR(ROUND(BG17/MA_Kurs_15,2),0)</f>
+      </c>
+      <c r="BJ17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="BK17" s="24"/>
+      <c r="BL17" s="181" t="str">
+        <f>=IFERROR(ROUND(BK17/MA_Kurs_16,2),0)</f>
+      </c>
+      <c r="BN17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="BO17" s="24"/>
+      <c r="BP17" s="181" t="str">
+        <f>=IFERROR(ROUND(BO17/MA_Kurs_17,2),0)</f>
+      </c>
+      <c r="BR17" s="180" t="s">
+        <v>212</v>
+      </c>
+      <c r="BS17" s="24"/>
+      <c r="BT17" s="181" t="str">
+        <f>=IFERROR(ROUND(BS17/MA_Kurs_18,2),0)</f>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>243</v>
+      </c>
+      <c r="B18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="C18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_1[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="D18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_1[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="F18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="G18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_2[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="H18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_2[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="J18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="K18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_3[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="L18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_3[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="N18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="O18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_4[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="P18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_4[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="R18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="S18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_5[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="T18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_5[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="V18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="W18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_6[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="X18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_6[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="Z18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="AA18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_7[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="AB18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_7[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="AD18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="AE18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_8[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="AF18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_8[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="AH18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="AI18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_9[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="AJ18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_9[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="AL18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="AM18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_10[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="AN18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_10[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="AP18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="AQ18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_11[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="AR18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_11[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="AT18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="AU18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_12[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="AV18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_12[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="AX18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="AY18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_13[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="AZ18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_13[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="BB18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="BC18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_14[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="BD18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_14[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="BF18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="BG18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_15[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="BH18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_15[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="BJ18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="BK18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_16[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="BL18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_16[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="BN18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="BO18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_17[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="BP18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_17[Angefordert (EUR)]),2)</f>
+      </c>
+      <c r="BR18" s="182" t="s">
+        <v>308</v>
+      </c>
+      <c r="BS18" s="183" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_18[Angefordert (LC)]),2)</f>
+      </c>
+      <c r="BT18" s="184" t="str">
+        <f>=ROUND(SUBTOTAL(109,MA_18[Angefordert (EUR)]),2)</f>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="s">
+        <v>309</v>
+      </c>
+      <c r="C20" s="185" t="str">
+        <f>=ROUND($C$18,2)</f>
+      </c>
+      <c r="D20" s="186" t="str">
+        <f>=ROUND($D$18,2)</f>
+      </c>
+      <c r="F20" t="s">
+        <v>309</v>
+      </c>
+      <c r="G20" s="185" t="str">
+        <f>=ROUND($G$18,2)</f>
+      </c>
+      <c r="H20" s="186" t="str">
+        <f>=ROUND($H$18,2)</f>
+      </c>
+      <c r="J20" t="s">
+        <v>309</v>
+      </c>
+      <c r="K20" s="185" t="str">
+        <f>=ROUND($K$18,2)</f>
+      </c>
+      <c r="L20" s="186" t="str">
+        <f>=ROUND($L$18,2)</f>
+      </c>
+      <c r="N20" t="s">
+        <v>309</v>
+      </c>
+      <c r="O20" s="185" t="str">
+        <f>=ROUND($O$18,2)</f>
+      </c>
+      <c r="P20" s="186" t="str">
+        <f>=ROUND($P$18,2)</f>
+      </c>
+      <c r="R20" t="s">
+        <v>309</v>
+      </c>
+      <c r="S20" s="185" t="str">
+        <f>=ROUND($S$18,2)</f>
+      </c>
+      <c r="T20" s="186" t="str">
+        <f>=ROUND($T$18,2)</f>
+      </c>
+      <c r="V20" t="s">
+        <v>309</v>
+      </c>
+      <c r="W20" s="185" t="str">
+        <f>=ROUND($W$18,2)</f>
+      </c>
+      <c r="X20" s="186" t="str">
+        <f>=ROUND($X$18,2)</f>
+      </c>
+      <c r="Z20" t="s">
+        <v>309</v>
+      </c>
+      <c r="AA20" s="185" t="str">
+        <f>=ROUND($AA$18,2)</f>
+      </c>
+      <c r="AB20" s="186" t="str">
+        <f>=ROUND($AB$18,2)</f>
+      </c>
+      <c r="AD20" t="s">
+        <v>309</v>
+      </c>
+      <c r="AE20" s="185" t="str">
+        <f>=ROUND($AE$18,2)</f>
+      </c>
+      <c r="AF20" s="186" t="str">
+        <f>=ROUND($AF$18,2)</f>
+      </c>
+      <c r="AH20" t="s">
+        <v>309</v>
+      </c>
+      <c r="AI20" s="185" t="str">
+        <f>=ROUND($AI$18,2)</f>
+      </c>
+      <c r="AJ20" s="186" t="str">
+        <f>=ROUND($AJ$18,2)</f>
+      </c>
+      <c r="AL20" t="s">
+        <v>309</v>
+      </c>
+      <c r="AM20" s="185" t="str">
+        <f>=ROUND($AM$18,2)</f>
+      </c>
+      <c r="AN20" s="186" t="str">
+        <f>=ROUND($AN$18,2)</f>
+      </c>
+      <c r="AP20" t="s">
+        <v>309</v>
+      </c>
+      <c r="AQ20" s="185" t="str">
+        <f>=ROUND($AQ$18,2)</f>
+      </c>
+      <c r="AR20" s="186" t="str">
+        <f>=ROUND($AR$18,2)</f>
+      </c>
+      <c r="AT20" t="s">
+        <v>309</v>
+      </c>
+      <c r="AU20" s="185" t="str">
+        <f>=ROUND($AU$18,2)</f>
+      </c>
+      <c r="AV20" s="186" t="str">
+        <f>=ROUND($AV$18,2)</f>
+      </c>
+      <c r="AX20" t="s">
+        <v>309</v>
+      </c>
+      <c r="AY20" s="185" t="str">
+        <f>=ROUND($AY$18,2)</f>
+      </c>
+      <c r="AZ20" s="186" t="str">
+        <f>=ROUND($AZ$18,2)</f>
+      </c>
+      <c r="BB20" t="s">
+        <v>309</v>
+      </c>
+      <c r="BC20" s="185" t="str">
+        <f>=ROUND($BC$18,2)</f>
+      </c>
+      <c r="BD20" s="186" t="str">
+        <f>=ROUND($BD$18,2)</f>
+      </c>
+      <c r="BF20" t="s">
+        <v>309</v>
+      </c>
+      <c r="BG20" s="185" t="str">
+        <f>=ROUND($BG$18,2)</f>
+      </c>
+      <c r="BH20" s="186" t="str">
+        <f>=ROUND($BH$18,2)</f>
+      </c>
+      <c r="BJ20" t="s">
+        <v>309</v>
+      </c>
+      <c r="BK20" s="185" t="str">
+        <f>=ROUND($BK$18,2)</f>
+      </c>
+      <c r="BL20" s="186" t="str">
+        <f>=ROUND($BL$18,2)</f>
+      </c>
+      <c r="BN20" t="s">
+        <v>309</v>
+      </c>
+      <c r="BO20" s="185" t="str">
+        <f>=ROUND($BO$18,2)</f>
+      </c>
+      <c r="BP20" s="186" t="str">
+        <f>=ROUND($BP$18,2)</f>
+      </c>
+      <c r="BR20" t="s">
+        <v>309</v>
+      </c>
+      <c r="BS20" s="185" t="str">
+        <f>=ROUND($BS$18,2)</f>
+      </c>
+      <c r="BT20" s="186" t="str">
+        <f>=ROUND($BT$18,2)</f>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="s">
+        <v>310</v>
+      </c>
+      <c r="C21" s="24"/>
+      <c r="D21" s="181" t="str">
+        <f>=IFERROR(ROUND($C$21/$C$7,2),0)</f>
+      </c>
+      <c r="F21" t="s">
+        <v>310</v>
+      </c>
+      <c r="G21" s="24"/>
+      <c r="H21" s="181" t="str">
+        <f>=IFERROR(ROUND($G$21/$G$7,2),0)</f>
+      </c>
+      <c r="J21" t="s">
+        <v>310</v>
+      </c>
+      <c r="K21" s="24"/>
+      <c r="L21" s="181" t="str">
+        <f>=IFERROR(ROUND($K$21/$K$7,2),0)</f>
+      </c>
+      <c r="N21" t="s">
+        <v>310</v>
+      </c>
+      <c r="O21" s="24"/>
+      <c r="P21" s="181" t="str">
+        <f>=IFERROR(ROUND($O$21/$O$7,2),0)</f>
+      </c>
+      <c r="R21" t="s">
+        <v>310</v>
+      </c>
+      <c r="S21" s="24"/>
+      <c r="T21" s="181" t="str">
+        <f>=IFERROR(ROUND($S$21/$S$7,2),0)</f>
+      </c>
+      <c r="V21" t="s">
+        <v>310</v>
+      </c>
+      <c r="W21" s="24"/>
+      <c r="X21" s="181" t="str">
+        <f>=IFERROR(ROUND($W$21/$W$7,2),0)</f>
+      </c>
+      <c r="Z21" t="s">
+        <v>310</v>
+      </c>
+      <c r="AA21" s="24"/>
+      <c r="AB21" s="181" t="str">
+        <f>=IFERROR(ROUND($AA$21/$AA$7,2),0)</f>
+      </c>
+      <c r="AD21" t="s">
+        <v>310</v>
+      </c>
+      <c r="AE21" s="24"/>
+      <c r="AF21" s="181" t="str">
+        <f>=IFERROR(ROUND($AE$21/$AE$7,2),0)</f>
+      </c>
+      <c r="AH21" t="s">
+        <v>310</v>
+      </c>
+      <c r="AI21" s="24"/>
+      <c r="AJ21" s="181" t="str">
+        <f>=IFERROR(ROUND($AI$21/$AI$7,2),0)</f>
+      </c>
+      <c r="AL21" t="s">
+        <v>310</v>
+      </c>
+      <c r="AM21" s="24"/>
+      <c r="AN21" s="181" t="str">
+        <f>=IFERROR(ROUND($AM$21/$AM$7,2),0)</f>
+      </c>
+      <c r="AP21" t="s">
+        <v>310</v>
+      </c>
+      <c r="AQ21" s="24"/>
+      <c r="AR21" s="181" t="str">
+        <f>=IFERROR(ROUND($AQ$21/$AQ$7,2),0)</f>
+      </c>
+      <c r="AT21" t="s">
+        <v>310</v>
+      </c>
+      <c r="AU21" s="24"/>
+      <c r="AV21" s="181" t="str">
+        <f>=IFERROR(ROUND($AU$21/$AU$7,2),0)</f>
+      </c>
+      <c r="AX21" t="s">
+        <v>310</v>
+      </c>
+      <c r="AY21" s="24"/>
+      <c r="AZ21" s="181" t="str">
+        <f>=IFERROR(ROUND($AY$21/$AY$7,2),0)</f>
+      </c>
+      <c r="BB21" t="s">
+        <v>310</v>
+      </c>
+      <c r="BC21" s="24"/>
+      <c r="BD21" s="181" t="str">
+        <f>=IFERROR(ROUND($BC$21/$BC$7,2),0)</f>
+      </c>
+      <c r="BF21" t="s">
+        <v>310</v>
+      </c>
+      <c r="BG21" s="24"/>
+      <c r="BH21" s="181" t="str">
+        <f>=IFERROR(ROUND($BG$21/$BG$7,2),0)</f>
+      </c>
+      <c r="BJ21" t="s">
+        <v>310</v>
+      </c>
+      <c r="BK21" s="24"/>
+      <c r="BL21" s="181" t="str">
+        <f>=IFERROR(ROUND($BK$21/$BK$7,2),0)</f>
+      </c>
+      <c r="BN21" t="s">
+        <v>310</v>
+      </c>
+      <c r="BO21" s="24"/>
+      <c r="BP21" s="181" t="str">
+        <f>=IFERROR(ROUND($BO$21/$BO$7,2),0)</f>
+      </c>
+      <c r="BR21" t="s">
+        <v>310</v>
+      </c>
+      <c r="BS21" s="24"/>
+      <c r="BT21" s="181" t="str">
+        <f>=IFERROR(ROUND($BS$21/$BS$7,2),0)</f>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="s">
+        <v>311</v>
+      </c>
+      <c r="C22" s="24"/>
+      <c r="D22" s="181" t="str">
+        <f>=IFERROR(ROUND($C$22/$C$7,2),0)</f>
+      </c>
+      <c r="F22" t="s">
+        <v>311</v>
+      </c>
+      <c r="G22" s="24"/>
+      <c r="H22" s="181" t="str">
+        <f>=IFERROR(ROUND($G$22/$G$7,2),0)</f>
+      </c>
+      <c r="J22" t="s">
+        <v>311</v>
+      </c>
+      <c r="K22" s="24"/>
+      <c r="L22" s="181" t="str">
+        <f>=IFERROR(ROUND($K$22/$K$7,2),0)</f>
+      </c>
+      <c r="N22" t="s">
+        <v>311</v>
+      </c>
+      <c r="O22" s="24"/>
+      <c r="P22" s="181" t="str">
+        <f>=IFERROR(ROUND($O$22/$O$7,2),0)</f>
+      </c>
+      <c r="R22" t="s">
+        <v>311</v>
+      </c>
+      <c r="S22" s="24"/>
+      <c r="T22" s="181" t="str">
+        <f>=IFERROR(ROUND($S$22/$S$7,2),0)</f>
+      </c>
+      <c r="V22" t="s">
+        <v>311</v>
+      </c>
+      <c r="W22" s="24"/>
+      <c r="X22" s="181" t="str">
+        <f>=IFERROR(ROUND($W$22/$W$7,2),0)</f>
+      </c>
+      <c r="Z22" t="s">
+        <v>311</v>
+      </c>
+      <c r="AA22" s="24"/>
+      <c r="AB22" s="181" t="str">
+        <f>=IFERROR(ROUND($AA$22/$AA$7,2),0)</f>
+      </c>
+      <c r="AD22" t="s">
+        <v>311</v>
+      </c>
+      <c r="AE22" s="24"/>
+      <c r="AF22" s="181" t="str">
+        <f>=IFERROR(ROUND($AE$22/$AE$7,2),0)</f>
+      </c>
+      <c r="AH22" t="s">
+        <v>311</v>
+      </c>
+      <c r="AI22" s="24"/>
+      <c r="AJ22" s="181" t="str">
+        <f>=IFERROR(ROUND($AI$22/$AI$7,2),0)</f>
+      </c>
+      <c r="AL22" t="s">
+        <v>311</v>
+      </c>
+      <c r="AM22" s="24"/>
+      <c r="AN22" s="181" t="str">
+        <f>=IFERROR(ROUND($AM$22/$AM$7,2),0)</f>
+      </c>
+      <c r="AP22" t="s">
+        <v>311</v>
+      </c>
+      <c r="AQ22" s="24"/>
+      <c r="AR22" s="181" t="str">
+        <f>=IFERROR(ROUND($AQ$22/$AQ$7,2),0)</f>
+      </c>
+      <c r="AT22" t="s">
+        <v>311</v>
+      </c>
+      <c r="AU22" s="24"/>
+      <c r="AV22" s="181" t="str">
+        <f>=IFERROR(ROUND($AU$22/$AU$7,2),0)</f>
+      </c>
+      <c r="AX22" t="s">
+        <v>311</v>
+      </c>
+      <c r="AY22" s="24"/>
+      <c r="AZ22" s="181" t="str">
+        <f>=IFERROR(ROUND($AY$22/$AY$7,2),0)</f>
+      </c>
+      <c r="BB22" t="s">
+        <v>311</v>
+      </c>
+      <c r="BC22" s="24"/>
+      <c r="BD22" s="181" t="str">
+        <f>=IFERROR(ROUND($BC$22/$BC$7,2),0)</f>
+      </c>
+      <c r="BF22" t="s">
+        <v>311</v>
+      </c>
+      <c r="BG22" s="24"/>
+      <c r="BH22" s="181" t="str">
+        <f>=IFERROR(ROUND($BG$22/$BG$7,2),0)</f>
+      </c>
+      <c r="BJ22" t="s">
+        <v>311</v>
+      </c>
+      <c r="BK22" s="24"/>
+      <c r="BL22" s="181" t="str">
+        <f>=IFERROR(ROUND($BK$22/$BK$7,2),0)</f>
+      </c>
+      <c r="BN22" t="s">
+        <v>311</v>
+      </c>
+      <c r="BO22" s="24"/>
+      <c r="BP22" s="181" t="str">
+        <f>=IFERROR(ROUND($BO$22/$BO$7,2),0)</f>
+      </c>
+      <c r="BR22" t="s">
+        <v>311</v>
+      </c>
+      <c r="BS22" s="24"/>
+      <c r="BT22" s="181" t="str">
+        <f>=IFERROR(ROUND($BS$22/$BS$7,2),0)</f>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="C23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="D23" s="181" t="str">
+        <f>=IFERROR(ROUND($C$23/$C$7,2),0)</f>
+      </c>
+      <c r="F23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="G23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="H23" s="181" t="str">
+        <f>=IFERROR(ROUND($G$23/$G$7,2),0)</f>
+      </c>
+      <c r="J23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="K23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="L23" s="181" t="str">
+        <f>=IFERROR(ROUND($K$23/$K$7,2),0)</f>
+      </c>
+      <c r="N23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="O23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="P23" s="181" t="str">
+        <f>=IFERROR(ROUND($O$23/$O$7,2),0)</f>
+      </c>
+      <c r="R23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="S23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="T23" s="181" t="str">
+        <f>=IFERROR(ROUND($S$23/$S$7,2),0)</f>
+      </c>
+      <c r="V23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="W23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="X23" s="181" t="str">
+        <f>=IFERROR(ROUND($W$23/$W$7,2),0)</f>
+      </c>
+      <c r="Z23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="AA23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="AB23" s="181" t="str">
+        <f>=IFERROR(ROUND($AA$23/$AA$7,2),0)</f>
+      </c>
+      <c r="AD23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="AE23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="AF23" s="181" t="str">
+        <f>=IFERROR(ROUND($AE$23/$AE$7,2),0)</f>
+      </c>
+      <c r="AH23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="AI23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="AJ23" s="181" t="str">
+        <f>=IFERROR(ROUND($AI$23/$AI$7,2),0)</f>
+      </c>
+      <c r="AL23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="AM23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="AN23" s="181" t="str">
+        <f>=IFERROR(ROUND($AM$23/$AM$7,2),0)</f>
+      </c>
+      <c r="AP23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="AQ23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="AR23" s="181" t="str">
+        <f>=IFERROR(ROUND($AQ$23/$AQ$7,2),0)</f>
+      </c>
+      <c r="AT23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="AU23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="AV23" s="181" t="str">
+        <f>=IFERROR(ROUND($AU$23/$AU$7,2),0)</f>
+      </c>
+      <c r="AX23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="AY23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="AZ23" s="181" t="str">
+        <f>=IFERROR(ROUND($AY$23/$AY$7,2),0)</f>
+      </c>
+      <c r="BB23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="BC23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="BD23" s="181" t="str">
+        <f>=IFERROR(ROUND($BC$23/$BC$7,2),0)</f>
+      </c>
+      <c r="BF23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="BG23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="BH23" s="181" t="str">
+        <f>=IFERROR(ROUND($BG$23/$BG$7,2),0)</f>
+      </c>
+      <c r="BJ23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="BK23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="BL23" s="181" t="str">
+        <f>=IFERROR(ROUND($BK$23/$BK$7,2),0)</f>
+      </c>
+      <c r="BN23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="BO23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="BP23" s="181" t="str">
+        <f>=IFERROR(ROUND($BO$23/$BO$7,2),0)</f>
+      </c>
+      <c r="BR23" t="str">
+        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      </c>
+      <c r="BS23" s="187" t="str">
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)-1)),0)),2)</f>
+      </c>
+      <c r="BT23" s="181" t="str">
+        <f>=IFERROR(ROUND($BS$23/$BS$7,2),0)</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="C25" s="189" t="str">
+        <f>=IFERROR(ROUND($C$18-$C$21-$C$22-$C$23,2),0)</f>
+      </c>
+      <c r="D25" s="190" t="str">
+        <f>=IFERROR(ROUND($D$18-$D$21-$D$22-$D$23,2),0)</f>
+      </c>
+      <c r="F25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="G25" s="189" t="str">
+        <f>=IFERROR(ROUND($G$18-$G$21-$G$22-$G$23,2),0)</f>
+      </c>
+      <c r="H25" s="190" t="str">
+        <f>=IFERROR(ROUND($H$18-$H$21-$H$22-$H$23,2),0)</f>
+      </c>
+      <c r="J25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="K25" s="189" t="str">
+        <f>=IFERROR(ROUND($K$18-$K$21-$K$22-$K$23,2),0)</f>
+      </c>
+      <c r="L25" s="190" t="str">
+        <f>=IFERROR(ROUND($L$18-$L$21-$L$22-$L$23,2),0)</f>
+      </c>
+      <c r="N25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="O25" s="189" t="str">
+        <f>=IFERROR(ROUND($O$18-$O$21-$O$22-$O$23,2),0)</f>
+      </c>
+      <c r="P25" s="190" t="str">
+        <f>=IFERROR(ROUND($P$18-$P$21-$P$22-$P$23,2),0)</f>
+      </c>
+      <c r="R25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="S25" s="189" t="str">
+        <f>=IFERROR(ROUND($S$18-$S$21-$S$22-$S$23,2),0)</f>
+      </c>
+      <c r="T25" s="190" t="str">
+        <f>=IFERROR(ROUND($T$18-$T$21-$T$22-$T$23,2),0)</f>
+      </c>
+      <c r="V25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="W25" s="189" t="str">
+        <f>=IFERROR(ROUND($W$18-$W$21-$W$22-$W$23,2),0)</f>
+      </c>
+      <c r="X25" s="190" t="str">
+        <f>=IFERROR(ROUND($X$18-$X$21-$X$22-$X$23,2),0)</f>
+      </c>
+      <c r="Z25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="AA25" s="189" t="str">
+        <f>=IFERROR(ROUND($AA$18-$AA$21-$AA$22-$AA$23,2),0)</f>
+      </c>
+      <c r="AB25" s="190" t="str">
+        <f>=IFERROR(ROUND($AB$18-$AB$21-$AB$22-$AB$23,2),0)</f>
+      </c>
+      <c r="AD25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="AE25" s="189" t="str">
+        <f>=IFERROR(ROUND($AE$18-$AE$21-$AE$22-$AE$23,2),0)</f>
+      </c>
+      <c r="AF25" s="190" t="str">
+        <f>=IFERROR(ROUND($AF$18-$AF$21-$AF$22-$AF$23,2),0)</f>
+      </c>
+      <c r="AH25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="AI25" s="189" t="str">
+        <f>=IFERROR(ROUND($AI$18-$AI$21-$AI$22-$AI$23,2),0)</f>
+      </c>
+      <c r="AJ25" s="190" t="str">
+        <f>=IFERROR(ROUND($AJ$18-$AJ$21-$AJ$22-$AJ$23,2),0)</f>
+      </c>
+      <c r="AL25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="AM25" s="189" t="str">
+        <f>=IFERROR(ROUND($AM$18-$AM$21-$AM$22-$AM$23,2),0)</f>
+      </c>
+      <c r="AN25" s="190" t="str">
+        <f>=IFERROR(ROUND($AN$18-$AN$21-$AN$22-$AN$23,2),0)</f>
+      </c>
+      <c r="AP25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="AQ25" s="189" t="str">
+        <f>=IFERROR(ROUND($AQ$18-$AQ$21-$AQ$22-$AQ$23,2),0)</f>
+      </c>
+      <c r="AR25" s="190" t="str">
+        <f>=IFERROR(ROUND($AR$18-$AR$21-$AR$22-$AR$23,2),0)</f>
+      </c>
+      <c r="AT25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="AU25" s="189" t="str">
+        <f>=IFERROR(ROUND($AU$18-$AU$21-$AU$22-$AU$23,2),0)</f>
+      </c>
+      <c r="AV25" s="190" t="str">
+        <f>=IFERROR(ROUND($AV$18-$AV$21-$AV$22-$AV$23,2),0)</f>
+      </c>
+      <c r="AX25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="AY25" s="189" t="str">
+        <f>=IFERROR(ROUND($AY$18-$AY$21-$AY$22-$AY$23,2),0)</f>
+      </c>
+      <c r="AZ25" s="190" t="str">
+        <f>=IFERROR(ROUND($AZ$18-$AZ$21-$AZ$22-$AZ$23,2),0)</f>
+      </c>
+      <c r="BB25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="BC25" s="189" t="str">
+        <f>=IFERROR(ROUND($BC$18-$BC$21-$BC$22-$BC$23,2),0)</f>
+      </c>
+      <c r="BD25" s="190" t="str">
+        <f>=IFERROR(ROUND($BD$18-$BD$21-$BD$22-$BD$23,2),0)</f>
+      </c>
+      <c r="BF25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="BG25" s="189" t="str">
+        <f>=IFERROR(ROUND($BG$18-$BG$21-$BG$22-$BG$23,2),0)</f>
+      </c>
+      <c r="BH25" s="190" t="str">
+        <f>=IFERROR(ROUND($BH$18-$BH$21-$BH$22-$BH$23,2),0)</f>
+      </c>
+      <c r="BJ25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="BK25" s="189" t="str">
+        <f>=IFERROR(ROUND($BK$18-$BK$21-$BK$22-$BK$23,2),0)</f>
+      </c>
+      <c r="BL25" s="190" t="str">
+        <f>=IFERROR(ROUND($BL$18-$BL$21-$BL$22-$BL$23,2),0)</f>
+      </c>
+      <c r="BN25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="BO25" s="189" t="str">
+        <f>=IFERROR(ROUND($BO$18-$BO$21-$BO$22-$BO$23,2),0)</f>
+      </c>
+      <c r="BP25" s="190" t="str">
+        <f>=IFERROR(ROUND($BP$18-$BP$21-$BP$22-$BP$23,2),0)</f>
+      </c>
+      <c r="BR25" s="188" t="s">
+        <v>312</v>
+      </c>
+      <c r="BS25" s="189" t="str">
+        <f>=IFERROR(ROUND($BS$18-$BS$21-$BS$22-$BS$23,2),0)</f>
+      </c>
+      <c r="BT25" s="190" t="str">
+        <f>=IFERROR(ROUND($BT$18-$BT$21-$BT$22-$BT$23,2),0)</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="54">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="W5:X5"/>
+    <mergeCell ref="W6:X6"/>
+    <mergeCell ref="W7:X7"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA6:AB6"/>
+    <mergeCell ref="AA7:AB7"/>
+    <mergeCell ref="AE5:AF5"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AE7:AF7"/>
+    <mergeCell ref="AI5:AJ5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="AI7:AJ7"/>
+    <mergeCell ref="AM5:AN5"/>
+    <mergeCell ref="AM6:AN6"/>
+    <mergeCell ref="AM7:AN7"/>
+    <mergeCell ref="AQ5:AR5"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="AQ7:AR7"/>
+    <mergeCell ref="AU5:AV5"/>
+    <mergeCell ref="AU6:AV6"/>
+    <mergeCell ref="AU7:AV7"/>
+    <mergeCell ref="AY5:AZ5"/>
+    <mergeCell ref="AY6:AZ6"/>
+    <mergeCell ref="AY7:AZ7"/>
+    <mergeCell ref="BC5:BD5"/>
+    <mergeCell ref="BC6:BD6"/>
+    <mergeCell ref="BC7:BD7"/>
+    <mergeCell ref="BG5:BH5"/>
+    <mergeCell ref="BG6:BH6"/>
+    <mergeCell ref="BG7:BH7"/>
+    <mergeCell ref="BK5:BL5"/>
+    <mergeCell ref="BK6:BL6"/>
+    <mergeCell ref="BK7:BL7"/>
+    <mergeCell ref="BO5:BP5"/>
+    <mergeCell ref="BO6:BP6"/>
+    <mergeCell ref="BO7:BP7"/>
+    <mergeCell ref="BS5:BT5"/>
+    <mergeCell ref="BS6:BT6"/>
+    <mergeCell ref="BS7:BT7"/>
+  </mergeCells>
+  <dataValidations count="18">
+    <dataValidation allowBlank="true" sqref="C5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="G5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="K5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="O5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="S5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="W5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="AA5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="AE5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="AI5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="AM5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="AQ5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="AU5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="AY5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="BC5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="BG5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="BK5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="BO5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="BS5" type="list">
+      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+    </dataValidation>
+  </dataValidations>
+  <tableParts count="18">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId12"/>
+    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
+    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId16"/>
+    <tablePart r:id="rId17"/>
+    <tablePart r:id="rId18"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(vorpruefung): prevent #VALUE! error on empty Saldovortrag in Mittelanforderung
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -18624,7 +18624,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="C23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="D23" s="181" t="str">
         <f>=IFERROR(ROUND($C$23/$C$7,2),0)</f>
@@ -18633,7 +18633,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="G23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="H23" s="181" t="str">
         <f>=IFERROR(ROUND($G$23/$G$7,2),0)</f>
@@ -18642,7 +18642,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="K23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="L23" s="181" t="str">
         <f>=IFERROR(ROUND($K$23/$K$7,2),0)</f>
@@ -18651,7 +18651,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="O23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="P23" s="181" t="str">
         <f>=IFERROR(ROUND($O$23/$O$7,2),0)</f>
@@ -18660,7 +18660,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="S23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="T23" s="181" t="str">
         <f>=IFERROR(ROUND($S$23/$S$7,2),0)</f>
@@ -18669,7 +18669,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="W23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="X23" s="181" t="str">
         <f>=IFERROR(ROUND($W$23/$W$7,2),0)</f>
@@ -18678,7 +18678,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="AA23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="AB23" s="181" t="str">
         <f>=IFERROR(ROUND($AA$23/$AA$7,2),0)</f>
@@ -18687,7 +18687,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="AE23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="AF23" s="181" t="str">
         <f>=IFERROR(ROUND($AE$23/$AE$7,2),0)</f>
@@ -18696,7 +18696,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="AI23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="AJ23" s="181" t="str">
         <f>=IFERROR(ROUND($AI$23/$AI$7,2),0)</f>
@@ -18705,7 +18705,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="AM23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="AN23" s="181" t="str">
         <f>=IFERROR(ROUND($AM$23/$AM$7,2),0)</f>
@@ -18714,7 +18714,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="AQ23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="AR23" s="181" t="str">
         <f>=IFERROR(ROUND($AQ$23/$AQ$7,2),0)</f>
@@ -18723,7 +18723,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="AU23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="AV23" s="181" t="str">
         <f>=IFERROR(ROUND($AU$23/$AU$7,2),0)</f>
@@ -18732,7 +18732,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="AY23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="AZ23" s="181" t="str">
         <f>=IFERROR(ROUND($AY$23/$AY$7,2),0)</f>
@@ -18741,7 +18741,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="BC23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="BD23" s="181" t="str">
         <f>=IFERROR(ROUND($BC$23/$BC$7,2),0)</f>
@@ -18750,7 +18750,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="BG23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="BH23" s="181" t="str">
         <f>=IFERROR(ROUND($BG$23/$BG$7,2),0)</f>
@@ -18759,7 +18759,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="BK23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="BL23" s="181" t="str">
         <f>=IFERROR(ROUND($BK$23/$BK$7,2),0)</f>
@@ -18768,7 +18768,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="BO23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="BP23" s="181" t="str">
         <f>=IFERROR(ROUND($BO$23/$BO$7,2),0)</f>
@@ -18777,7 +18777,7 @@
         <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
       </c>
       <c r="BS23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)&lt;=1,Saldovortrag_LW,IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)-1)),0)),2)</f>
       </c>
       <c r="BT23" s="181" t="str">
         <f>=IFERROR(ROUND($BS$23/$BS$7,2),0)</f>

</xml_diff>

<commit_message>
refactor(vorpruefung): remove dynamic INDIREKT formulas in MA for safer explicit references
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="315">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1062,7 +1062,13 @@
     <t>abzueglich Drittmittel:</t>
   </si>
   <si>
+    <t>abzueglich Saldo Vorprojekt:</t>
+  </si>
+  <si>
     <t>KMW-Mittel Anforderung:</t>
+  </si>
+  <si>
+    <t>abzueglich Saldo Vorperiode (FB):</t>
   </si>
 </sst>
 </file>
@@ -18620,164 +18626,164 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="B23" t="s">
+        <v>312</v>
       </c>
       <c r="C23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($C$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IF(Saldovortrag_LW="",0,Saldovortrag_LW),2)</f>
       </c>
       <c r="D23" s="181" t="str">
         <f>=IFERROR(ROUND($C$23/$C$7,2),0)</f>
       </c>
-      <c r="F23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="F23" t="s">
+        <v>314</v>
       </c>
       <c r="G23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($G$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_1,0),2)</f>
       </c>
       <c r="H23" s="181" t="str">
         <f>=IFERROR(ROUND($G$23/$G$7,2),0)</f>
       </c>
-      <c r="J23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="J23" t="s">
+        <v>314</v>
       </c>
       <c r="K23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($K$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_2,0),2)</f>
       </c>
       <c r="L23" s="181" t="str">
         <f>=IFERROR(ROUND($K$23/$K$7,2),0)</f>
       </c>
-      <c r="N23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="N23" t="s">
+        <v>314</v>
       </c>
       <c r="O23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($O$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_3,0),2)</f>
       </c>
       <c r="P23" s="181" t="str">
         <f>=IFERROR(ROUND($O$23/$O$7,2),0)</f>
       </c>
-      <c r="R23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="R23" t="s">
+        <v>314</v>
       </c>
       <c r="S23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($S$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_4,0),2)</f>
       </c>
       <c r="T23" s="181" t="str">
         <f>=IFERROR(ROUND($S$23/$S$7,2),0)</f>
       </c>
-      <c r="V23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="V23" t="s">
+        <v>314</v>
       </c>
       <c r="W23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($W$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_5,0),2)</f>
       </c>
       <c r="X23" s="181" t="str">
         <f>=IFERROR(ROUND($W$23/$W$7,2),0)</f>
       </c>
-      <c r="Z23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="Z23" t="s">
+        <v>314</v>
       </c>
       <c r="AA23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AA$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_6,0),2)</f>
       </c>
       <c r="AB23" s="181" t="str">
         <f>=IFERROR(ROUND($AA$23/$AA$7,2),0)</f>
       </c>
-      <c r="AD23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="AD23" t="s">
+        <v>314</v>
       </c>
       <c r="AE23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AE$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_7,0),2)</f>
       </c>
       <c r="AF23" s="181" t="str">
         <f>=IFERROR(ROUND($AE$23/$AE$7,2),0)</f>
       </c>
-      <c r="AH23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="AH23" t="s">
+        <v>314</v>
       </c>
       <c r="AI23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AI$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_8,0),2)</f>
       </c>
       <c r="AJ23" s="181" t="str">
         <f>=IFERROR(ROUND($AI$23/$AI$7,2),0)</f>
       </c>
-      <c r="AL23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="AL23" t="s">
+        <v>314</v>
       </c>
       <c r="AM23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AM$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_9,0),2)</f>
       </c>
       <c r="AN23" s="181" t="str">
         <f>=IFERROR(ROUND($AM$23/$AM$7,2),0)</f>
       </c>
-      <c r="AP23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="AP23" t="s">
+        <v>314</v>
       </c>
       <c r="AQ23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AQ$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_10,0),2)</f>
       </c>
       <c r="AR23" s="181" t="str">
         <f>=IFERROR(ROUND($AQ$23/$AQ$7,2),0)</f>
       </c>
-      <c r="AT23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="AT23" t="s">
+        <v>314</v>
       </c>
       <c r="AU23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AU$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_11,0),2)</f>
       </c>
       <c r="AV23" s="181" t="str">
         <f>=IFERROR(ROUND($AU$23/$AU$7,2),0)</f>
       </c>
-      <c r="AX23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="AX23" t="s">
+        <v>314</v>
       </c>
       <c r="AY23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($AY$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_12,0),2)</f>
       </c>
       <c r="AZ23" s="181" t="str">
         <f>=IFERROR(ROUND($AY$23/$AY$7,2),0)</f>
       </c>
-      <c r="BB23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="BB23" t="s">
+        <v>314</v>
       </c>
       <c r="BC23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BC$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_13,0),2)</f>
       </c>
       <c r="BD23" s="181" t="str">
         <f>=IFERROR(ROUND($BC$23/$BC$7,2),0)</f>
       </c>
-      <c r="BF23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="BF23" t="s">
+        <v>314</v>
       </c>
       <c r="BG23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BG$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_14,0),2)</f>
       </c>
       <c r="BH23" s="181" t="str">
         <f>=IFERROR(ROUND($BG$23/$BG$7,2),0)</f>
       </c>
-      <c r="BJ23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="BJ23" t="s">
+        <v>314</v>
       </c>
       <c r="BK23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BK$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_15,0),2)</f>
       </c>
       <c r="BL23" s="181" t="str">
         <f>=IFERROR(ROUND($BK$23/$BK$7,2),0)</f>
       </c>
-      <c r="BN23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="BN23" t="s">
+        <v>314</v>
       </c>
       <c r="BO23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BO$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_16,0),2)</f>
       </c>
       <c r="BP23" s="181" t="str">
         <f>=IFERROR(ROUND($BO$23/$BO$7,2),0)</f>
       </c>
-      <c r="BR23" t="str">
-        <f>=IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)&lt;=1,"abzueglich Saldo Vorprojekt:","abzueglich Saldo Vorperiode (FB):")</f>
+      <c r="BR23" t="s">
+        <v>314</v>
       </c>
       <c r="BS23" s="187" t="str">
-        <f>=ROUND(IF(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)&lt;=1,IF(Saldovortrag_LW="",0,Saldovortrag_LW),IFERROR(INDIRECT("FB_SaldoLC_"&amp;(IFERROR(VALUE(TRIM(SUBSTITUTE($BS$5,"Periode",""))),1)-1)),0)),2)</f>
+        <f>=ROUND(IFERROR(FB_SaldoLC_17,0),2)</f>
       </c>
       <c r="BT23" s="181" t="str">
         <f>=IFERROR(ROUND($BS$23/$BS$7,2),0)</f>
@@ -18785,7 +18791,7 @@
     </row>
     <row r="25">
       <c r="B25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C25" s="189" t="str">
         <f>=IFERROR(ROUND($C$18-$C$21-$C$22-$C$23,2),0)</f>
@@ -18794,7 +18800,7 @@
         <f>=IFERROR(ROUND($D$18-$D$21-$D$22-$D$23,2),0)</f>
       </c>
       <c r="F25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G25" s="189" t="str">
         <f>=IFERROR(ROUND($G$18-$G$21-$G$22-$G$23,2),0)</f>
@@ -18803,7 +18809,7 @@
         <f>=IFERROR(ROUND($H$18-$H$21-$H$22-$H$23,2),0)</f>
       </c>
       <c r="J25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="K25" s="189" t="str">
         <f>=IFERROR(ROUND($K$18-$K$21-$K$22-$K$23,2),0)</f>
@@ -18812,7 +18818,7 @@
         <f>=IFERROR(ROUND($L$18-$L$21-$L$22-$L$23,2),0)</f>
       </c>
       <c r="N25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="O25" s="189" t="str">
         <f>=IFERROR(ROUND($O$18-$O$21-$O$22-$O$23,2),0)</f>
@@ -18821,7 +18827,7 @@
         <f>=IFERROR(ROUND($P$18-$P$21-$P$22-$P$23,2),0)</f>
       </c>
       <c r="R25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="S25" s="189" t="str">
         <f>=IFERROR(ROUND($S$18-$S$21-$S$22-$S$23,2),0)</f>
@@ -18830,7 +18836,7 @@
         <f>=IFERROR(ROUND($T$18-$T$21-$T$22-$T$23,2),0)</f>
       </c>
       <c r="V25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="W25" s="189" t="str">
         <f>=IFERROR(ROUND($W$18-$W$21-$W$22-$W$23,2),0)</f>
@@ -18839,7 +18845,7 @@
         <f>=IFERROR(ROUND($X$18-$X$21-$X$22-$X$23,2),0)</f>
       </c>
       <c r="Z25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AA25" s="189" t="str">
         <f>=IFERROR(ROUND($AA$18-$AA$21-$AA$22-$AA$23,2),0)</f>
@@ -18848,7 +18854,7 @@
         <f>=IFERROR(ROUND($AB$18-$AB$21-$AB$22-$AB$23,2),0)</f>
       </c>
       <c r="AD25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AE25" s="189" t="str">
         <f>=IFERROR(ROUND($AE$18-$AE$21-$AE$22-$AE$23,2),0)</f>
@@ -18857,7 +18863,7 @@
         <f>=IFERROR(ROUND($AF$18-$AF$21-$AF$22-$AF$23,2),0)</f>
       </c>
       <c r="AH25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AI25" s="189" t="str">
         <f>=IFERROR(ROUND($AI$18-$AI$21-$AI$22-$AI$23,2),0)</f>
@@ -18866,7 +18872,7 @@
         <f>=IFERROR(ROUND($AJ$18-$AJ$21-$AJ$22-$AJ$23,2),0)</f>
       </c>
       <c r="AL25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AM25" s="189" t="str">
         <f>=IFERROR(ROUND($AM$18-$AM$21-$AM$22-$AM$23,2),0)</f>
@@ -18875,7 +18881,7 @@
         <f>=IFERROR(ROUND($AN$18-$AN$21-$AN$22-$AN$23,2),0)</f>
       </c>
       <c r="AP25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AQ25" s="189" t="str">
         <f>=IFERROR(ROUND($AQ$18-$AQ$21-$AQ$22-$AQ$23,2),0)</f>
@@ -18884,7 +18890,7 @@
         <f>=IFERROR(ROUND($AR$18-$AR$21-$AR$22-$AR$23,2),0)</f>
       </c>
       <c r="AT25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AU25" s="189" t="str">
         <f>=IFERROR(ROUND($AU$18-$AU$21-$AU$22-$AU$23,2),0)</f>
@@ -18893,7 +18899,7 @@
         <f>=IFERROR(ROUND($AV$18-$AV$21-$AV$22-$AV$23,2),0)</f>
       </c>
       <c r="AX25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AY25" s="189" t="str">
         <f>=IFERROR(ROUND($AY$18-$AY$21-$AY$22-$AY$23,2),0)</f>
@@ -18902,7 +18908,7 @@
         <f>=IFERROR(ROUND($AZ$18-$AZ$21-$AZ$22-$AZ$23,2),0)</f>
       </c>
       <c r="BB25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="BC25" s="189" t="str">
         <f>=IFERROR(ROUND($BC$18-$BC$21-$BC$22-$BC$23,2),0)</f>
@@ -18911,7 +18917,7 @@
         <f>=IFERROR(ROUND($BD$18-$BD$21-$BD$22-$BD$23,2),0)</f>
       </c>
       <c r="BF25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="BG25" s="189" t="str">
         <f>=IFERROR(ROUND($BG$18-$BG$21-$BG$22-$BG$23,2),0)</f>
@@ -18920,7 +18926,7 @@
         <f>=IFERROR(ROUND($BH$18-$BH$21-$BH$22-$BH$23,2),0)</f>
       </c>
       <c r="BJ25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="BK25" s="189" t="str">
         <f>=IFERROR(ROUND($BK$18-$BK$21-$BK$22-$BK$23,2),0)</f>
@@ -18929,7 +18935,7 @@
         <f>=IFERROR(ROUND($BL$18-$BL$21-$BL$22-$BL$23,2),0)</f>
       </c>
       <c r="BN25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="BO25" s="189" t="str">
         <f>=IFERROR(ROUND($BO$18-$BO$21-$BO$22-$BO$23,2),0)</f>
@@ -18938,7 +18944,7 @@
         <f>=IFERROR(ROUND($BP$18-$BP$21-$BP$22-$BP$23,2),0)</f>
       </c>
       <c r="BR25" s="188" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="BS25" s="189" t="str">
         <f>=IFERROR(ROUND($BS$18-$BS$21-$BS$22-$BS$23,2),0)</f>

</xml_diff>

<commit_message>
refactor(vorpruefung): remove all structural table references in Finanzberichte for robust calculation
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -7182,25 +7182,25 @@
         <v>194</v>
       </c>
       <c r="C12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Eigenmittel",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"Eigenmittel",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Eigenmittel",$D$41:$D$45)+SUMIF($B$50:$B$55,"Eigenmittel",$D$50:$D$55),2)</f>
       </c>
       <c r="D12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Eigenmittel",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"Eigenmittel",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Eigenmittel",$E$41:$E$45)+SUMIF($B$50:$B$55,"Eigenmittel",$E$50:$E$55),2)</f>
       </c>
       <c r="E12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Eigenmittel",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"Eigenmittel",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Eigenmittel",$D$41:$D$45)+SUMIF($B$50:$B$55,"Eigenmittel",$D$50:$D$55),2)</f>
       </c>
       <c r="F12" s="143" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Eigenmittel",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"Eigenmittel",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Eigenmittel",$E$41:$E$45)+SUMIF($B$50:$B$55,"Eigenmittel",$E$50:$E$55),2)</f>
       </c>
       <c r="I12" s="142" t="s">
         <v>194</v>
       </c>
       <c r="J12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"Eigenmittel",Einnahmen_2[Einnahmen (LC)])+SUMIF(Einnahmen_WK_2[Typ],"Eigenmittel",Einnahmen_WK_2[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"Eigenmittel",$K$41:$K$45)+SUMIF($I$50:$I$55,"Eigenmittel",$K$50:$K$55),2)</f>
       </c>
       <c r="K12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"Eigenmittel",Einnahmen_2[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_2[Typ],"Eigenmittel",Einnahmen_WK_2[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"Eigenmittel",$L$41:$L$45)+SUMIF($I$50:$I$55,"Eigenmittel",$L$50:$L$55),2)</f>
       </c>
       <c r="L12" s="115" t="str">
         <f>=IFERROR(ROUND(E12 + J12, 2), J12)</f>
@@ -7212,10 +7212,10 @@
         <v>194</v>
       </c>
       <c r="Q12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"Eigenmittel",Einnahmen_3[Einnahmen (LC)])+SUMIF(Einnahmen_WK_3[Typ],"Eigenmittel",Einnahmen_WK_3[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"Eigenmittel",$R$41:$R$45)+SUMIF($P$50:$P$55,"Eigenmittel",$R$50:$R$55),2)</f>
       </c>
       <c r="R12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"Eigenmittel",Einnahmen_3[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_3[Typ],"Eigenmittel",Einnahmen_WK_3[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"Eigenmittel",$S$41:$S$45)+SUMIF($P$50:$P$55,"Eigenmittel",$S$50:$S$55),2)</f>
       </c>
       <c r="S12" s="115" t="str">
         <f>=IFERROR(ROUND(L12 + Q12, 2), Q12)</f>
@@ -7227,10 +7227,10 @@
         <v>194</v>
       </c>
       <c r="X12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"Eigenmittel",Einnahmen_4[Einnahmen (LC)])+SUMIF(Einnahmen_WK_4[Typ],"Eigenmittel",Einnahmen_WK_4[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"Eigenmittel",$Y$41:$Y$45)+SUMIF($W$50:$W$55,"Eigenmittel",$Y$50:$Y$55),2)</f>
       </c>
       <c r="Y12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"Eigenmittel",Einnahmen_4[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_4[Typ],"Eigenmittel",Einnahmen_WK_4[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"Eigenmittel",$Z$41:$Z$45)+SUMIF($W$50:$W$55,"Eigenmittel",$Z$50:$Z$55),2)</f>
       </c>
       <c r="Z12" s="115" t="str">
         <f>=IFERROR(ROUND(S12 + X12, 2), X12)</f>
@@ -7242,10 +7242,10 @@
         <v>194</v>
       </c>
       <c r="AE12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"Eigenmittel",Einnahmen_5[Einnahmen (LC)])+SUMIF(Einnahmen_WK_5[Typ],"Eigenmittel",Einnahmen_WK_5[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"Eigenmittel",$AF$41:$AF$45)+SUMIF($AD$50:$AD$55,"Eigenmittel",$AF$50:$AF$55),2)</f>
       </c>
       <c r="AF12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"Eigenmittel",Einnahmen_5[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_5[Typ],"Eigenmittel",Einnahmen_WK_5[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"Eigenmittel",$AG$41:$AG$45)+SUMIF($AD$50:$AD$55,"Eigenmittel",$AG$50:$AG$55),2)</f>
       </c>
       <c r="AG12" s="115" t="str">
         <f>=IFERROR(ROUND(Z12 + AE12, 2), AE12)</f>
@@ -7257,10 +7257,10 @@
         <v>194</v>
       </c>
       <c r="AL12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"Eigenmittel",Einnahmen_6[Einnahmen (LC)])+SUMIF(Einnahmen_WK_6[Typ],"Eigenmittel",Einnahmen_WK_6[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"Eigenmittel",$AM$41:$AM$45)+SUMIF($AK$50:$AK$55,"Eigenmittel",$AM$50:$AM$55),2)</f>
       </c>
       <c r="AM12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"Eigenmittel",Einnahmen_6[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_6[Typ],"Eigenmittel",Einnahmen_WK_6[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"Eigenmittel",$AN$41:$AN$45)+SUMIF($AK$50:$AK$55,"Eigenmittel",$AN$50:$AN$55),2)</f>
       </c>
       <c r="AN12" s="115" t="str">
         <f>=IFERROR(ROUND(AG12 + AL12, 2), AL12)</f>
@@ -7272,10 +7272,10 @@
         <v>194</v>
       </c>
       <c r="AS12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"Eigenmittel",Einnahmen_7[Einnahmen (LC)])+SUMIF(Einnahmen_WK_7[Typ],"Eigenmittel",Einnahmen_WK_7[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"Eigenmittel",$AT$41:$AT$45)+SUMIF($AR$50:$AR$55,"Eigenmittel",$AT$50:$AT$55),2)</f>
       </c>
       <c r="AT12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"Eigenmittel",Einnahmen_7[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_7[Typ],"Eigenmittel",Einnahmen_WK_7[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"Eigenmittel",$AU$41:$AU$45)+SUMIF($AR$50:$AR$55,"Eigenmittel",$AU$50:$AU$55),2)</f>
       </c>
       <c r="AU12" s="115" t="str">
         <f>=IFERROR(ROUND(AN12 + AS12, 2), AS12)</f>
@@ -7287,10 +7287,10 @@
         <v>194</v>
       </c>
       <c r="AZ12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"Eigenmittel",Einnahmen_8[Einnahmen (LC)])+SUMIF(Einnahmen_WK_8[Typ],"Eigenmittel",Einnahmen_WK_8[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"Eigenmittel",$BA$41:$BA$45)+SUMIF($AY$50:$AY$55,"Eigenmittel",$BA$50:$BA$55),2)</f>
       </c>
       <c r="BA12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"Eigenmittel",Einnahmen_8[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_8[Typ],"Eigenmittel",Einnahmen_WK_8[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"Eigenmittel",$BB$41:$BB$45)+SUMIF($AY$50:$AY$55,"Eigenmittel",$BB$50:$BB$55),2)</f>
       </c>
       <c r="BB12" s="115" t="str">
         <f>=IFERROR(ROUND(AU12 + AZ12, 2), AZ12)</f>
@@ -7302,10 +7302,10 @@
         <v>194</v>
       </c>
       <c r="BG12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"Eigenmittel",Einnahmen_9[Einnahmen (LC)])+SUMIF(Einnahmen_WK_9[Typ],"Eigenmittel",Einnahmen_WK_9[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"Eigenmittel",$BH$41:$BH$45)+SUMIF($BF$50:$BF$55,"Eigenmittel",$BH$50:$BH$55),2)</f>
       </c>
       <c r="BH12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"Eigenmittel",Einnahmen_9[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_9[Typ],"Eigenmittel",Einnahmen_WK_9[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"Eigenmittel",$BI$41:$BI$45)+SUMIF($BF$50:$BF$55,"Eigenmittel",$BI$50:$BI$55),2)</f>
       </c>
       <c r="BI12" s="115" t="str">
         <f>=IFERROR(ROUND(BB12 + BG12, 2), BG12)</f>
@@ -7317,10 +7317,10 @@
         <v>194</v>
       </c>
       <c r="BN12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"Eigenmittel",Einnahmen_10[Einnahmen (LC)])+SUMIF(Einnahmen_WK_10[Typ],"Eigenmittel",Einnahmen_WK_10[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"Eigenmittel",$BO$41:$BO$45)+SUMIF($BM$50:$BM$55,"Eigenmittel",$BO$50:$BO$55),2)</f>
       </c>
       <c r="BO12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"Eigenmittel",Einnahmen_10[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_10[Typ],"Eigenmittel",Einnahmen_WK_10[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"Eigenmittel",$BP$41:$BP$45)+SUMIF($BM$50:$BM$55,"Eigenmittel",$BP$50:$BP$55),2)</f>
       </c>
       <c r="BP12" s="115" t="str">
         <f>=IFERROR(ROUND(BI12 + BN12, 2), BN12)</f>
@@ -7332,10 +7332,10 @@
         <v>194</v>
       </c>
       <c r="BU12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"Eigenmittel",Einnahmen_11[Einnahmen (LC)])+SUMIF(Einnahmen_WK_11[Typ],"Eigenmittel",Einnahmen_WK_11[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"Eigenmittel",$BV$41:$BV$45)+SUMIF($BT$50:$BT$55,"Eigenmittel",$BV$50:$BV$55),2)</f>
       </c>
       <c r="BV12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"Eigenmittel",Einnahmen_11[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_11[Typ],"Eigenmittel",Einnahmen_WK_11[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"Eigenmittel",$BW$41:$BW$45)+SUMIF($BT$50:$BT$55,"Eigenmittel",$BW$50:$BW$55),2)</f>
       </c>
       <c r="BW12" s="115" t="str">
         <f>=IFERROR(ROUND(BP12 + BU12, 2), BU12)</f>
@@ -7347,10 +7347,10 @@
         <v>194</v>
       </c>
       <c r="CB12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"Eigenmittel",Einnahmen_12[Einnahmen (LC)])+SUMIF(Einnahmen_WK_12[Typ],"Eigenmittel",Einnahmen_WK_12[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"Eigenmittel",$CC$41:$CC$45)+SUMIF($CA$50:$CA$55,"Eigenmittel",$CC$50:$CC$55),2)</f>
       </c>
       <c r="CC12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"Eigenmittel",Einnahmen_12[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_12[Typ],"Eigenmittel",Einnahmen_WK_12[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"Eigenmittel",$CD$41:$CD$45)+SUMIF($CA$50:$CA$55,"Eigenmittel",$CD$50:$CD$55),2)</f>
       </c>
       <c r="CD12" s="115" t="str">
         <f>=IFERROR(ROUND(BW12 + CB12, 2), CB12)</f>
@@ -7362,10 +7362,10 @@
         <v>194</v>
       </c>
       <c r="CI12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"Eigenmittel",Einnahmen_13[Einnahmen (LC)])+SUMIF(Einnahmen_WK_13[Typ],"Eigenmittel",Einnahmen_WK_13[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"Eigenmittel",$CJ$41:$CJ$45)+SUMIF($CH$50:$CH$55,"Eigenmittel",$CJ$50:$CJ$55),2)</f>
       </c>
       <c r="CJ12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"Eigenmittel",Einnahmen_13[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_13[Typ],"Eigenmittel",Einnahmen_WK_13[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"Eigenmittel",$CK$41:$CK$45)+SUMIF($CH$50:$CH$55,"Eigenmittel",$CK$50:$CK$55),2)</f>
       </c>
       <c r="CK12" s="115" t="str">
         <f>=IFERROR(ROUND(CD12 + CI12, 2), CI12)</f>
@@ -7377,10 +7377,10 @@
         <v>194</v>
       </c>
       <c r="CP12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"Eigenmittel",Einnahmen_14[Einnahmen (LC)])+SUMIF(Einnahmen_WK_14[Typ],"Eigenmittel",Einnahmen_WK_14[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"Eigenmittel",$CQ$41:$CQ$45)+SUMIF($CO$50:$CO$55,"Eigenmittel",$CQ$50:$CQ$55),2)</f>
       </c>
       <c r="CQ12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"Eigenmittel",Einnahmen_14[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_14[Typ],"Eigenmittel",Einnahmen_WK_14[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"Eigenmittel",$CR$41:$CR$45)+SUMIF($CO$50:$CO$55,"Eigenmittel",$CR$50:$CR$55),2)</f>
       </c>
       <c r="CR12" s="115" t="str">
         <f>=IFERROR(ROUND(CK12 + CP12, 2), CP12)</f>
@@ -7392,10 +7392,10 @@
         <v>194</v>
       </c>
       <c r="CW12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"Eigenmittel",Einnahmen_15[Einnahmen (LC)])+SUMIF(Einnahmen_WK_15[Typ],"Eigenmittel",Einnahmen_WK_15[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"Eigenmittel",$CX$41:$CX$45)+SUMIF($CV$50:$CV$55,"Eigenmittel",$CX$50:$CX$55),2)</f>
       </c>
       <c r="CX12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"Eigenmittel",Einnahmen_15[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_15[Typ],"Eigenmittel",Einnahmen_WK_15[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"Eigenmittel",$CY$41:$CY$45)+SUMIF($CV$50:$CV$55,"Eigenmittel",$CY$50:$CY$55),2)</f>
       </c>
       <c r="CY12" s="115" t="str">
         <f>=IFERROR(ROUND(CR12 + CW12, 2), CW12)</f>
@@ -7407,10 +7407,10 @@
         <v>194</v>
       </c>
       <c r="DD12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"Eigenmittel",Einnahmen_16[Einnahmen (LC)])+SUMIF(Einnahmen_WK_16[Typ],"Eigenmittel",Einnahmen_WK_16[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"Eigenmittel",$DE$41:$DE$45)+SUMIF($DC$50:$DC$55,"Eigenmittel",$DE$50:$DE$55),2)</f>
       </c>
       <c r="DE12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"Eigenmittel",Einnahmen_16[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_16[Typ],"Eigenmittel",Einnahmen_WK_16[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"Eigenmittel",$DF$41:$DF$45)+SUMIF($DC$50:$DC$55,"Eigenmittel",$DF$50:$DF$55),2)</f>
       </c>
       <c r="DF12" s="115" t="str">
         <f>=IFERROR(ROUND(CY12 + DD12, 2), DD12)</f>
@@ -7422,10 +7422,10 @@
         <v>194</v>
       </c>
       <c r="DK12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"Eigenmittel",Einnahmen_17[Einnahmen (LC)])+SUMIF(Einnahmen_WK_17[Typ],"Eigenmittel",Einnahmen_WK_17[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"Eigenmittel",$DL$41:$DL$45)+SUMIF($DJ$50:$DJ$55,"Eigenmittel",$DL$50:$DL$55),2)</f>
       </c>
       <c r="DL12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"Eigenmittel",Einnahmen_17[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_17[Typ],"Eigenmittel",Einnahmen_WK_17[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"Eigenmittel",$DM$41:$DM$45)+SUMIF($DJ$50:$DJ$55,"Eigenmittel",$DM$50:$DM$55),2)</f>
       </c>
       <c r="DM12" s="115" t="str">
         <f>=IFERROR(ROUND(DF12 + DK12, 2), DK12)</f>
@@ -7437,10 +7437,10 @@
         <v>194</v>
       </c>
       <c r="DR12" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"Eigenmittel",Einnahmen_18[Einnahmen (LC)])+SUMIF(Einnahmen_WK_18[Typ],"Eigenmittel",Einnahmen_WK_18[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"Eigenmittel",$DS$41:$DS$45)+SUMIF($DQ$50:$DQ$55,"Eigenmittel",$DS$50:$DS$55),2)</f>
       </c>
       <c r="DS12" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"Eigenmittel",Einnahmen_18[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_18[Typ],"Eigenmittel",Einnahmen_WK_18[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"Eigenmittel",$DT$41:$DT$45)+SUMIF($DQ$50:$DQ$55,"Eigenmittel",$DT$50:$DT$55),2)</f>
       </c>
       <c r="DT12" s="115" t="str">
         <f>=IFERROR(ROUND(DM12 + DR12, 2), DR12)</f>
@@ -7454,25 +7454,25 @@
         <v>277</v>
       </c>
       <c r="C13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Drittmittel",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"Drittmittel",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Drittmittel",$D$41:$D$45)+SUMIF($B$50:$B$55,"Drittmittel",$D$50:$D$55),2)</f>
       </c>
       <c r="D13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Drittmittel",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"Drittmittel",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Drittmittel",$E$41:$E$45)+SUMIF($B$50:$B$55,"Drittmittel",$E$50:$E$55),2)</f>
       </c>
       <c r="E13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Drittmittel",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"Drittmittel",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Drittmittel",$D$41:$D$45)+SUMIF($B$50:$B$55,"Drittmittel",$D$50:$D$55),2)</f>
       </c>
       <c r="F13" s="143" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Drittmittel",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"Drittmittel",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Drittmittel",$E$41:$E$45)+SUMIF($B$50:$B$55,"Drittmittel",$E$50:$E$55),2)</f>
       </c>
       <c r="I13" s="142" t="s">
         <v>277</v>
       </c>
       <c r="J13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"Drittmittel",Einnahmen_2[Einnahmen (LC)])+SUMIF(Einnahmen_WK_2[Typ],"Drittmittel",Einnahmen_WK_2[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"Drittmittel",$K$41:$K$45)+SUMIF($I$50:$I$55,"Drittmittel",$K$50:$K$55),2)</f>
       </c>
       <c r="K13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"Drittmittel",Einnahmen_2[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_2[Typ],"Drittmittel",Einnahmen_WK_2[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"Drittmittel",$L$41:$L$45)+SUMIF($I$50:$I$55,"Drittmittel",$L$50:$L$55),2)</f>
       </c>
       <c r="L13" s="115" t="str">
         <f>=IFERROR(ROUND(E13 + J13, 2), J13)</f>
@@ -7484,10 +7484,10 @@
         <v>277</v>
       </c>
       <c r="Q13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"Drittmittel",Einnahmen_3[Einnahmen (LC)])+SUMIF(Einnahmen_WK_3[Typ],"Drittmittel",Einnahmen_WK_3[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"Drittmittel",$R$41:$R$45)+SUMIF($P$50:$P$55,"Drittmittel",$R$50:$R$55),2)</f>
       </c>
       <c r="R13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"Drittmittel",Einnahmen_3[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_3[Typ],"Drittmittel",Einnahmen_WK_3[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"Drittmittel",$S$41:$S$45)+SUMIF($P$50:$P$55,"Drittmittel",$S$50:$S$55),2)</f>
       </c>
       <c r="S13" s="115" t="str">
         <f>=IFERROR(ROUND(L13 + Q13, 2), Q13)</f>
@@ -7499,10 +7499,10 @@
         <v>277</v>
       </c>
       <c r="X13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"Drittmittel",Einnahmen_4[Einnahmen (LC)])+SUMIF(Einnahmen_WK_4[Typ],"Drittmittel",Einnahmen_WK_4[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"Drittmittel",$Y$41:$Y$45)+SUMIF($W$50:$W$55,"Drittmittel",$Y$50:$Y$55),2)</f>
       </c>
       <c r="Y13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"Drittmittel",Einnahmen_4[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_4[Typ],"Drittmittel",Einnahmen_WK_4[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"Drittmittel",$Z$41:$Z$45)+SUMIF($W$50:$W$55,"Drittmittel",$Z$50:$Z$55),2)</f>
       </c>
       <c r="Z13" s="115" t="str">
         <f>=IFERROR(ROUND(S13 + X13, 2), X13)</f>
@@ -7514,10 +7514,10 @@
         <v>277</v>
       </c>
       <c r="AE13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"Drittmittel",Einnahmen_5[Einnahmen (LC)])+SUMIF(Einnahmen_WK_5[Typ],"Drittmittel",Einnahmen_WK_5[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"Drittmittel",$AF$41:$AF$45)+SUMIF($AD$50:$AD$55,"Drittmittel",$AF$50:$AF$55),2)</f>
       </c>
       <c r="AF13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"Drittmittel",Einnahmen_5[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_5[Typ],"Drittmittel",Einnahmen_WK_5[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"Drittmittel",$AG$41:$AG$45)+SUMIF($AD$50:$AD$55,"Drittmittel",$AG$50:$AG$55),2)</f>
       </c>
       <c r="AG13" s="115" t="str">
         <f>=IFERROR(ROUND(Z13 + AE13, 2), AE13)</f>
@@ -7529,10 +7529,10 @@
         <v>277</v>
       </c>
       <c r="AL13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"Drittmittel",Einnahmen_6[Einnahmen (LC)])+SUMIF(Einnahmen_WK_6[Typ],"Drittmittel",Einnahmen_WK_6[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"Drittmittel",$AM$41:$AM$45)+SUMIF($AK$50:$AK$55,"Drittmittel",$AM$50:$AM$55),2)</f>
       </c>
       <c r="AM13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"Drittmittel",Einnahmen_6[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_6[Typ],"Drittmittel",Einnahmen_WK_6[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"Drittmittel",$AN$41:$AN$45)+SUMIF($AK$50:$AK$55,"Drittmittel",$AN$50:$AN$55),2)</f>
       </c>
       <c r="AN13" s="115" t="str">
         <f>=IFERROR(ROUND(AG13 + AL13, 2), AL13)</f>
@@ -7544,10 +7544,10 @@
         <v>277</v>
       </c>
       <c r="AS13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"Drittmittel",Einnahmen_7[Einnahmen (LC)])+SUMIF(Einnahmen_WK_7[Typ],"Drittmittel",Einnahmen_WK_7[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"Drittmittel",$AT$41:$AT$45)+SUMIF($AR$50:$AR$55,"Drittmittel",$AT$50:$AT$55),2)</f>
       </c>
       <c r="AT13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"Drittmittel",Einnahmen_7[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_7[Typ],"Drittmittel",Einnahmen_WK_7[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"Drittmittel",$AU$41:$AU$45)+SUMIF($AR$50:$AR$55,"Drittmittel",$AU$50:$AU$55),2)</f>
       </c>
       <c r="AU13" s="115" t="str">
         <f>=IFERROR(ROUND(AN13 + AS13, 2), AS13)</f>
@@ -7559,10 +7559,10 @@
         <v>277</v>
       </c>
       <c r="AZ13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"Drittmittel",Einnahmen_8[Einnahmen (LC)])+SUMIF(Einnahmen_WK_8[Typ],"Drittmittel",Einnahmen_WK_8[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"Drittmittel",$BA$41:$BA$45)+SUMIF($AY$50:$AY$55,"Drittmittel",$BA$50:$BA$55),2)</f>
       </c>
       <c r="BA13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"Drittmittel",Einnahmen_8[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_8[Typ],"Drittmittel",Einnahmen_WK_8[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"Drittmittel",$BB$41:$BB$45)+SUMIF($AY$50:$AY$55,"Drittmittel",$BB$50:$BB$55),2)</f>
       </c>
       <c r="BB13" s="115" t="str">
         <f>=IFERROR(ROUND(AU13 + AZ13, 2), AZ13)</f>
@@ -7574,10 +7574,10 @@
         <v>277</v>
       </c>
       <c r="BG13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"Drittmittel",Einnahmen_9[Einnahmen (LC)])+SUMIF(Einnahmen_WK_9[Typ],"Drittmittel",Einnahmen_WK_9[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"Drittmittel",$BH$41:$BH$45)+SUMIF($BF$50:$BF$55,"Drittmittel",$BH$50:$BH$55),2)</f>
       </c>
       <c r="BH13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"Drittmittel",Einnahmen_9[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_9[Typ],"Drittmittel",Einnahmen_WK_9[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"Drittmittel",$BI$41:$BI$45)+SUMIF($BF$50:$BF$55,"Drittmittel",$BI$50:$BI$55),2)</f>
       </c>
       <c r="BI13" s="115" t="str">
         <f>=IFERROR(ROUND(BB13 + BG13, 2), BG13)</f>
@@ -7589,10 +7589,10 @@
         <v>277</v>
       </c>
       <c r="BN13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"Drittmittel",Einnahmen_10[Einnahmen (LC)])+SUMIF(Einnahmen_WK_10[Typ],"Drittmittel",Einnahmen_WK_10[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"Drittmittel",$BO$41:$BO$45)+SUMIF($BM$50:$BM$55,"Drittmittel",$BO$50:$BO$55),2)</f>
       </c>
       <c r="BO13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"Drittmittel",Einnahmen_10[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_10[Typ],"Drittmittel",Einnahmen_WK_10[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"Drittmittel",$BP$41:$BP$45)+SUMIF($BM$50:$BM$55,"Drittmittel",$BP$50:$BP$55),2)</f>
       </c>
       <c r="BP13" s="115" t="str">
         <f>=IFERROR(ROUND(BI13 + BN13, 2), BN13)</f>
@@ -7604,10 +7604,10 @@
         <v>277</v>
       </c>
       <c r="BU13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"Drittmittel",Einnahmen_11[Einnahmen (LC)])+SUMIF(Einnahmen_WK_11[Typ],"Drittmittel",Einnahmen_WK_11[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"Drittmittel",$BV$41:$BV$45)+SUMIF($BT$50:$BT$55,"Drittmittel",$BV$50:$BV$55),2)</f>
       </c>
       <c r="BV13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"Drittmittel",Einnahmen_11[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_11[Typ],"Drittmittel",Einnahmen_WK_11[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"Drittmittel",$BW$41:$BW$45)+SUMIF($BT$50:$BT$55,"Drittmittel",$BW$50:$BW$55),2)</f>
       </c>
       <c r="BW13" s="115" t="str">
         <f>=IFERROR(ROUND(BP13 + BU13, 2), BU13)</f>
@@ -7619,10 +7619,10 @@
         <v>277</v>
       </c>
       <c r="CB13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"Drittmittel",Einnahmen_12[Einnahmen (LC)])+SUMIF(Einnahmen_WK_12[Typ],"Drittmittel",Einnahmen_WK_12[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"Drittmittel",$CC$41:$CC$45)+SUMIF($CA$50:$CA$55,"Drittmittel",$CC$50:$CC$55),2)</f>
       </c>
       <c r="CC13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"Drittmittel",Einnahmen_12[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_12[Typ],"Drittmittel",Einnahmen_WK_12[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"Drittmittel",$CD$41:$CD$45)+SUMIF($CA$50:$CA$55,"Drittmittel",$CD$50:$CD$55),2)</f>
       </c>
       <c r="CD13" s="115" t="str">
         <f>=IFERROR(ROUND(BW13 + CB13, 2), CB13)</f>
@@ -7634,10 +7634,10 @@
         <v>277</v>
       </c>
       <c r="CI13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"Drittmittel",Einnahmen_13[Einnahmen (LC)])+SUMIF(Einnahmen_WK_13[Typ],"Drittmittel",Einnahmen_WK_13[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"Drittmittel",$CJ$41:$CJ$45)+SUMIF($CH$50:$CH$55,"Drittmittel",$CJ$50:$CJ$55),2)</f>
       </c>
       <c r="CJ13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"Drittmittel",Einnahmen_13[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_13[Typ],"Drittmittel",Einnahmen_WK_13[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"Drittmittel",$CK$41:$CK$45)+SUMIF($CH$50:$CH$55,"Drittmittel",$CK$50:$CK$55),2)</f>
       </c>
       <c r="CK13" s="115" t="str">
         <f>=IFERROR(ROUND(CD13 + CI13, 2), CI13)</f>
@@ -7649,10 +7649,10 @@
         <v>277</v>
       </c>
       <c r="CP13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"Drittmittel",Einnahmen_14[Einnahmen (LC)])+SUMIF(Einnahmen_WK_14[Typ],"Drittmittel",Einnahmen_WK_14[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"Drittmittel",$CQ$41:$CQ$45)+SUMIF($CO$50:$CO$55,"Drittmittel",$CQ$50:$CQ$55),2)</f>
       </c>
       <c r="CQ13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"Drittmittel",Einnahmen_14[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_14[Typ],"Drittmittel",Einnahmen_WK_14[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"Drittmittel",$CR$41:$CR$45)+SUMIF($CO$50:$CO$55,"Drittmittel",$CR$50:$CR$55),2)</f>
       </c>
       <c r="CR13" s="115" t="str">
         <f>=IFERROR(ROUND(CK13 + CP13, 2), CP13)</f>
@@ -7664,10 +7664,10 @@
         <v>277</v>
       </c>
       <c r="CW13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"Drittmittel",Einnahmen_15[Einnahmen (LC)])+SUMIF(Einnahmen_WK_15[Typ],"Drittmittel",Einnahmen_WK_15[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"Drittmittel",$CX$41:$CX$45)+SUMIF($CV$50:$CV$55,"Drittmittel",$CX$50:$CX$55),2)</f>
       </c>
       <c r="CX13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"Drittmittel",Einnahmen_15[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_15[Typ],"Drittmittel",Einnahmen_WK_15[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"Drittmittel",$CY$41:$CY$45)+SUMIF($CV$50:$CV$55,"Drittmittel",$CY$50:$CY$55),2)</f>
       </c>
       <c r="CY13" s="115" t="str">
         <f>=IFERROR(ROUND(CR13 + CW13, 2), CW13)</f>
@@ -7679,10 +7679,10 @@
         <v>277</v>
       </c>
       <c r="DD13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"Drittmittel",Einnahmen_16[Einnahmen (LC)])+SUMIF(Einnahmen_WK_16[Typ],"Drittmittel",Einnahmen_WK_16[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"Drittmittel",$DE$41:$DE$45)+SUMIF($DC$50:$DC$55,"Drittmittel",$DE$50:$DE$55),2)</f>
       </c>
       <c r="DE13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"Drittmittel",Einnahmen_16[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_16[Typ],"Drittmittel",Einnahmen_WK_16[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"Drittmittel",$DF$41:$DF$45)+SUMIF($DC$50:$DC$55,"Drittmittel",$DF$50:$DF$55),2)</f>
       </c>
       <c r="DF13" s="115" t="str">
         <f>=IFERROR(ROUND(CY13 + DD13, 2), DD13)</f>
@@ -7694,10 +7694,10 @@
         <v>277</v>
       </c>
       <c r="DK13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"Drittmittel",Einnahmen_17[Einnahmen (LC)])+SUMIF(Einnahmen_WK_17[Typ],"Drittmittel",Einnahmen_WK_17[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"Drittmittel",$DL$41:$DL$45)+SUMIF($DJ$50:$DJ$55,"Drittmittel",$DL$50:$DL$55),2)</f>
       </c>
       <c r="DL13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"Drittmittel",Einnahmen_17[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_17[Typ],"Drittmittel",Einnahmen_WK_17[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"Drittmittel",$DM$41:$DM$45)+SUMIF($DJ$50:$DJ$55,"Drittmittel",$DM$50:$DM$55),2)</f>
       </c>
       <c r="DM13" s="115" t="str">
         <f>=IFERROR(ROUND(DF13 + DK13, 2), DK13)</f>
@@ -7709,10 +7709,10 @@
         <v>277</v>
       </c>
       <c r="DR13" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"Drittmittel",Einnahmen_18[Einnahmen (LC)])+SUMIF(Einnahmen_WK_18[Typ],"Drittmittel",Einnahmen_WK_18[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"Drittmittel",$DS$41:$DS$45)+SUMIF($DQ$50:$DQ$55,"Drittmittel",$DS$50:$DS$55),2)</f>
       </c>
       <c r="DS13" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"Drittmittel",Einnahmen_18[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_18[Typ],"Drittmittel",Einnahmen_WK_18[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"Drittmittel",$DT$41:$DT$45)+SUMIF($DQ$50:$DQ$55,"Drittmittel",$DT$50:$DT$55),2)</f>
       </c>
       <c r="DT13" s="115" t="str">
         <f>=IFERROR(ROUND(DM13 + DR13, 2), DR13)</f>
@@ -7726,25 +7726,25 @@
         <v>199</v>
       </c>
       <c r="C14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"KMW-Mittel",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"KMW-Mittel",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"KMW-Mittel",$D$41:$D$45)+SUMIF($B$50:$B$55,"KMW-Mittel",$D$50:$D$55),2)</f>
       </c>
       <c r="D14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"KMW-Mittel",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"KMW-Mittel",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"KMW-Mittel",$E$41:$E$45)+SUMIF($B$50:$B$55,"KMW-Mittel",$E$50:$E$55),2)</f>
       </c>
       <c r="E14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"KMW-Mittel",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"KMW-Mittel",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"KMW-Mittel",$D$41:$D$45)+SUMIF($B$50:$B$55,"KMW-Mittel",$D$50:$D$55),2)</f>
       </c>
       <c r="F14" s="143" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"KMW-Mittel",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"KMW-Mittel",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"KMW-Mittel",$E$41:$E$45)+SUMIF($B$50:$B$55,"KMW-Mittel",$E$50:$E$55),2)</f>
       </c>
       <c r="I14" s="142" t="s">
         <v>199</v>
       </c>
       <c r="J14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"KMW-Mittel",Einnahmen_2[Einnahmen (LC)])+SUMIF(Einnahmen_WK_2[Typ],"KMW-Mittel",Einnahmen_WK_2[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"KMW-Mittel",$K$41:$K$45)+SUMIF($I$50:$I$55,"KMW-Mittel",$K$50:$K$55),2)</f>
       </c>
       <c r="K14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"KMW-Mittel",Einnahmen_2[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_2[Typ],"KMW-Mittel",Einnahmen_WK_2[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"KMW-Mittel",$L$41:$L$45)+SUMIF($I$50:$I$55,"KMW-Mittel",$L$50:$L$55),2)</f>
       </c>
       <c r="L14" s="115" t="str">
         <f>=IFERROR(ROUND(E14 + J14, 2), J14)</f>
@@ -7756,10 +7756,10 @@
         <v>199</v>
       </c>
       <c r="Q14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"KMW-Mittel",Einnahmen_3[Einnahmen (LC)])+SUMIF(Einnahmen_WK_3[Typ],"KMW-Mittel",Einnahmen_WK_3[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"KMW-Mittel",$R$41:$R$45)+SUMIF($P$50:$P$55,"KMW-Mittel",$R$50:$R$55),2)</f>
       </c>
       <c r="R14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"KMW-Mittel",Einnahmen_3[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_3[Typ],"KMW-Mittel",Einnahmen_WK_3[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"KMW-Mittel",$S$41:$S$45)+SUMIF($P$50:$P$55,"KMW-Mittel",$S$50:$S$55),2)</f>
       </c>
       <c r="S14" s="115" t="str">
         <f>=IFERROR(ROUND(L14 + Q14, 2), Q14)</f>
@@ -7771,10 +7771,10 @@
         <v>199</v>
       </c>
       <c r="X14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"KMW-Mittel",Einnahmen_4[Einnahmen (LC)])+SUMIF(Einnahmen_WK_4[Typ],"KMW-Mittel",Einnahmen_WK_4[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"KMW-Mittel",$Y$41:$Y$45)+SUMIF($W$50:$W$55,"KMW-Mittel",$Y$50:$Y$55),2)</f>
       </c>
       <c r="Y14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"KMW-Mittel",Einnahmen_4[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_4[Typ],"KMW-Mittel",Einnahmen_WK_4[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"KMW-Mittel",$Z$41:$Z$45)+SUMIF($W$50:$W$55,"KMW-Mittel",$Z$50:$Z$55),2)</f>
       </c>
       <c r="Z14" s="115" t="str">
         <f>=IFERROR(ROUND(S14 + X14, 2), X14)</f>
@@ -7786,10 +7786,10 @@
         <v>199</v>
       </c>
       <c r="AE14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"KMW-Mittel",Einnahmen_5[Einnahmen (LC)])+SUMIF(Einnahmen_WK_5[Typ],"KMW-Mittel",Einnahmen_WK_5[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"KMW-Mittel",$AF$41:$AF$45)+SUMIF($AD$50:$AD$55,"KMW-Mittel",$AF$50:$AF$55),2)</f>
       </c>
       <c r="AF14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"KMW-Mittel",Einnahmen_5[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_5[Typ],"KMW-Mittel",Einnahmen_WK_5[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"KMW-Mittel",$AG$41:$AG$45)+SUMIF($AD$50:$AD$55,"KMW-Mittel",$AG$50:$AG$55),2)</f>
       </c>
       <c r="AG14" s="115" t="str">
         <f>=IFERROR(ROUND(Z14 + AE14, 2), AE14)</f>
@@ -7801,10 +7801,10 @@
         <v>199</v>
       </c>
       <c r="AL14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"KMW-Mittel",Einnahmen_6[Einnahmen (LC)])+SUMIF(Einnahmen_WK_6[Typ],"KMW-Mittel",Einnahmen_WK_6[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"KMW-Mittel",$AM$41:$AM$45)+SUMIF($AK$50:$AK$55,"KMW-Mittel",$AM$50:$AM$55),2)</f>
       </c>
       <c r="AM14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"KMW-Mittel",Einnahmen_6[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_6[Typ],"KMW-Mittel",Einnahmen_WK_6[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"KMW-Mittel",$AN$41:$AN$45)+SUMIF($AK$50:$AK$55,"KMW-Mittel",$AN$50:$AN$55),2)</f>
       </c>
       <c r="AN14" s="115" t="str">
         <f>=IFERROR(ROUND(AG14 + AL14, 2), AL14)</f>
@@ -7816,10 +7816,10 @@
         <v>199</v>
       </c>
       <c r="AS14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"KMW-Mittel",Einnahmen_7[Einnahmen (LC)])+SUMIF(Einnahmen_WK_7[Typ],"KMW-Mittel",Einnahmen_WK_7[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"KMW-Mittel",$AT$41:$AT$45)+SUMIF($AR$50:$AR$55,"KMW-Mittel",$AT$50:$AT$55),2)</f>
       </c>
       <c r="AT14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"KMW-Mittel",Einnahmen_7[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_7[Typ],"KMW-Mittel",Einnahmen_WK_7[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"KMW-Mittel",$AU$41:$AU$45)+SUMIF($AR$50:$AR$55,"KMW-Mittel",$AU$50:$AU$55),2)</f>
       </c>
       <c r="AU14" s="115" t="str">
         <f>=IFERROR(ROUND(AN14 + AS14, 2), AS14)</f>
@@ -7831,10 +7831,10 @@
         <v>199</v>
       </c>
       <c r="AZ14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"KMW-Mittel",Einnahmen_8[Einnahmen (LC)])+SUMIF(Einnahmen_WK_8[Typ],"KMW-Mittel",Einnahmen_WK_8[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"KMW-Mittel",$BA$41:$BA$45)+SUMIF($AY$50:$AY$55,"KMW-Mittel",$BA$50:$BA$55),2)</f>
       </c>
       <c r="BA14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"KMW-Mittel",Einnahmen_8[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_8[Typ],"KMW-Mittel",Einnahmen_WK_8[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"KMW-Mittel",$BB$41:$BB$45)+SUMIF($AY$50:$AY$55,"KMW-Mittel",$BB$50:$BB$55),2)</f>
       </c>
       <c r="BB14" s="115" t="str">
         <f>=IFERROR(ROUND(AU14 + AZ14, 2), AZ14)</f>
@@ -7846,10 +7846,10 @@
         <v>199</v>
       </c>
       <c r="BG14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"KMW-Mittel",Einnahmen_9[Einnahmen (LC)])+SUMIF(Einnahmen_WK_9[Typ],"KMW-Mittel",Einnahmen_WK_9[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"KMW-Mittel",$BH$41:$BH$45)+SUMIF($BF$50:$BF$55,"KMW-Mittel",$BH$50:$BH$55),2)</f>
       </c>
       <c r="BH14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"KMW-Mittel",Einnahmen_9[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_9[Typ],"KMW-Mittel",Einnahmen_WK_9[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"KMW-Mittel",$BI$41:$BI$45)+SUMIF($BF$50:$BF$55,"KMW-Mittel",$BI$50:$BI$55),2)</f>
       </c>
       <c r="BI14" s="115" t="str">
         <f>=IFERROR(ROUND(BB14 + BG14, 2), BG14)</f>
@@ -7861,10 +7861,10 @@
         <v>199</v>
       </c>
       <c r="BN14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"KMW-Mittel",Einnahmen_10[Einnahmen (LC)])+SUMIF(Einnahmen_WK_10[Typ],"KMW-Mittel",Einnahmen_WK_10[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"KMW-Mittel",$BO$41:$BO$45)+SUMIF($BM$50:$BM$55,"KMW-Mittel",$BO$50:$BO$55),2)</f>
       </c>
       <c r="BO14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"KMW-Mittel",Einnahmen_10[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_10[Typ],"KMW-Mittel",Einnahmen_WK_10[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"KMW-Mittel",$BP$41:$BP$45)+SUMIF($BM$50:$BM$55,"KMW-Mittel",$BP$50:$BP$55),2)</f>
       </c>
       <c r="BP14" s="115" t="str">
         <f>=IFERROR(ROUND(BI14 + BN14, 2), BN14)</f>
@@ -7876,10 +7876,10 @@
         <v>199</v>
       </c>
       <c r="BU14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"KMW-Mittel",Einnahmen_11[Einnahmen (LC)])+SUMIF(Einnahmen_WK_11[Typ],"KMW-Mittel",Einnahmen_WK_11[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"KMW-Mittel",$BV$41:$BV$45)+SUMIF($BT$50:$BT$55,"KMW-Mittel",$BV$50:$BV$55),2)</f>
       </c>
       <c r="BV14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"KMW-Mittel",Einnahmen_11[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_11[Typ],"KMW-Mittel",Einnahmen_WK_11[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"KMW-Mittel",$BW$41:$BW$45)+SUMIF($BT$50:$BT$55,"KMW-Mittel",$BW$50:$BW$55),2)</f>
       </c>
       <c r="BW14" s="115" t="str">
         <f>=IFERROR(ROUND(BP14 + BU14, 2), BU14)</f>
@@ -7891,10 +7891,10 @@
         <v>199</v>
       </c>
       <c r="CB14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"KMW-Mittel",Einnahmen_12[Einnahmen (LC)])+SUMIF(Einnahmen_WK_12[Typ],"KMW-Mittel",Einnahmen_WK_12[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"KMW-Mittel",$CC$41:$CC$45)+SUMIF($CA$50:$CA$55,"KMW-Mittel",$CC$50:$CC$55),2)</f>
       </c>
       <c r="CC14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"KMW-Mittel",Einnahmen_12[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_12[Typ],"KMW-Mittel",Einnahmen_WK_12[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"KMW-Mittel",$CD$41:$CD$45)+SUMIF($CA$50:$CA$55,"KMW-Mittel",$CD$50:$CD$55),2)</f>
       </c>
       <c r="CD14" s="115" t="str">
         <f>=IFERROR(ROUND(BW14 + CB14, 2), CB14)</f>
@@ -7906,10 +7906,10 @@
         <v>199</v>
       </c>
       <c r="CI14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"KMW-Mittel",Einnahmen_13[Einnahmen (LC)])+SUMIF(Einnahmen_WK_13[Typ],"KMW-Mittel",Einnahmen_WK_13[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"KMW-Mittel",$CJ$41:$CJ$45)+SUMIF($CH$50:$CH$55,"KMW-Mittel",$CJ$50:$CJ$55),2)</f>
       </c>
       <c r="CJ14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"KMW-Mittel",Einnahmen_13[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_13[Typ],"KMW-Mittel",Einnahmen_WK_13[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"KMW-Mittel",$CK$41:$CK$45)+SUMIF($CH$50:$CH$55,"KMW-Mittel",$CK$50:$CK$55),2)</f>
       </c>
       <c r="CK14" s="115" t="str">
         <f>=IFERROR(ROUND(CD14 + CI14, 2), CI14)</f>
@@ -7921,10 +7921,10 @@
         <v>199</v>
       </c>
       <c r="CP14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"KMW-Mittel",Einnahmen_14[Einnahmen (LC)])+SUMIF(Einnahmen_WK_14[Typ],"KMW-Mittel",Einnahmen_WK_14[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"KMW-Mittel",$CQ$41:$CQ$45)+SUMIF($CO$50:$CO$55,"KMW-Mittel",$CQ$50:$CQ$55),2)</f>
       </c>
       <c r="CQ14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"KMW-Mittel",Einnahmen_14[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_14[Typ],"KMW-Mittel",Einnahmen_WK_14[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"KMW-Mittel",$CR$41:$CR$45)+SUMIF($CO$50:$CO$55,"KMW-Mittel",$CR$50:$CR$55),2)</f>
       </c>
       <c r="CR14" s="115" t="str">
         <f>=IFERROR(ROUND(CK14 + CP14, 2), CP14)</f>
@@ -7936,10 +7936,10 @@
         <v>199</v>
       </c>
       <c r="CW14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"KMW-Mittel",Einnahmen_15[Einnahmen (LC)])+SUMIF(Einnahmen_WK_15[Typ],"KMW-Mittel",Einnahmen_WK_15[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"KMW-Mittel",$CX$41:$CX$45)+SUMIF($CV$50:$CV$55,"KMW-Mittel",$CX$50:$CX$55),2)</f>
       </c>
       <c r="CX14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"KMW-Mittel",Einnahmen_15[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_15[Typ],"KMW-Mittel",Einnahmen_WK_15[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"KMW-Mittel",$CY$41:$CY$45)+SUMIF($CV$50:$CV$55,"KMW-Mittel",$CY$50:$CY$55),2)</f>
       </c>
       <c r="CY14" s="115" t="str">
         <f>=IFERROR(ROUND(CR14 + CW14, 2), CW14)</f>
@@ -7951,10 +7951,10 @@
         <v>199</v>
       </c>
       <c r="DD14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"KMW-Mittel",Einnahmen_16[Einnahmen (LC)])+SUMIF(Einnahmen_WK_16[Typ],"KMW-Mittel",Einnahmen_WK_16[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"KMW-Mittel",$DE$41:$DE$45)+SUMIF($DC$50:$DC$55,"KMW-Mittel",$DE$50:$DE$55),2)</f>
       </c>
       <c r="DE14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"KMW-Mittel",Einnahmen_16[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_16[Typ],"KMW-Mittel",Einnahmen_WK_16[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"KMW-Mittel",$DF$41:$DF$45)+SUMIF($DC$50:$DC$55,"KMW-Mittel",$DF$50:$DF$55),2)</f>
       </c>
       <c r="DF14" s="115" t="str">
         <f>=IFERROR(ROUND(CY14 + DD14, 2), DD14)</f>
@@ -7966,10 +7966,10 @@
         <v>199</v>
       </c>
       <c r="DK14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"KMW-Mittel",Einnahmen_17[Einnahmen (LC)])+SUMIF(Einnahmen_WK_17[Typ],"KMW-Mittel",Einnahmen_WK_17[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"KMW-Mittel",$DL$41:$DL$45)+SUMIF($DJ$50:$DJ$55,"KMW-Mittel",$DL$50:$DL$55),2)</f>
       </c>
       <c r="DL14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"KMW-Mittel",Einnahmen_17[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_17[Typ],"KMW-Mittel",Einnahmen_WK_17[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"KMW-Mittel",$DM$41:$DM$45)+SUMIF($DJ$50:$DJ$55,"KMW-Mittel",$DM$50:$DM$55),2)</f>
       </c>
       <c r="DM14" s="115" t="str">
         <f>=IFERROR(ROUND(DF14 + DK14, 2), DK14)</f>
@@ -7981,10 +7981,10 @@
         <v>199</v>
       </c>
       <c r="DR14" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"KMW-Mittel",Einnahmen_18[Einnahmen (LC)])+SUMIF(Einnahmen_WK_18[Typ],"KMW-Mittel",Einnahmen_WK_18[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"KMW-Mittel",$DS$41:$DS$45)+SUMIF($DQ$50:$DQ$55,"KMW-Mittel",$DS$50:$DS$55),2)</f>
       </c>
       <c r="DS14" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"KMW-Mittel",Einnahmen_18[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_18[Typ],"KMW-Mittel",Einnahmen_WK_18[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"KMW-Mittel",$DT$41:$DT$45)+SUMIF($DQ$50:$DQ$55,"KMW-Mittel",$DT$50:$DT$55),2)</f>
       </c>
       <c r="DT14" s="115" t="str">
         <f>=IFERROR(ROUND(DM14 + DR14, 2), DR14)</f>
@@ -7998,25 +7998,25 @@
         <v>278</v>
       </c>
       <c r="C15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Zinsertraege",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"Zinsertraege",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Zinsertraege",$D$41:$D$45)+SUMIF($B$50:$B$55,"Zinsertraege",$D$50:$D$55),2)</f>
       </c>
       <c r="D15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Zinsertraege",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"Zinsertraege",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Zinsertraege",$E$41:$E$45)+SUMIF($B$50:$B$55,"Zinsertraege",$E$50:$E$55),2)</f>
       </c>
       <c r="E15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Zinsertraege",Einnahmen_1[Einnahmen (LC)])+SUMIF(Einnahmen_WK_1[Typ],"Zinsertraege",Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Zinsertraege",$D$41:$D$45)+SUMIF($B$50:$B$55,"Zinsertraege",$D$50:$D$55),2)</f>
       </c>
       <c r="F15" s="143" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_1[Typ],"Zinsertraege",Einnahmen_1[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_1[Typ],"Zinsertraege",Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($B$41:$B$45,"Zinsertraege",$E$41:$E$45)+SUMIF($B$50:$B$55,"Zinsertraege",$E$50:$E$55),2)</f>
       </c>
       <c r="I15" s="142" t="s">
         <v>278</v>
       </c>
       <c r="J15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"Zinsertraege",Einnahmen_2[Einnahmen (LC)])+SUMIF(Einnahmen_WK_2[Typ],"Zinsertraege",Einnahmen_WK_2[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"Zinsertraege",$K$41:$K$45)+SUMIF($I$50:$I$55,"Zinsertraege",$K$50:$K$55),2)</f>
       </c>
       <c r="K15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_2[Typ],"Zinsertraege",Einnahmen_2[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_2[Typ],"Zinsertraege",Einnahmen_WK_2[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($I$41:$I$45,"Zinsertraege",$L$41:$L$45)+SUMIF($I$50:$I$55,"Zinsertraege",$L$50:$L$55),2)</f>
       </c>
       <c r="L15" s="115" t="str">
         <f>=IFERROR(ROUND(E15 + J15, 2), J15)</f>
@@ -8028,10 +8028,10 @@
         <v>278</v>
       </c>
       <c r="Q15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"Zinsertraege",Einnahmen_3[Einnahmen (LC)])+SUMIF(Einnahmen_WK_3[Typ],"Zinsertraege",Einnahmen_WK_3[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"Zinsertraege",$R$41:$R$45)+SUMIF($P$50:$P$55,"Zinsertraege",$R$50:$R$55),2)</f>
       </c>
       <c r="R15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_3[Typ],"Zinsertraege",Einnahmen_3[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_3[Typ],"Zinsertraege",Einnahmen_WK_3[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($P$41:$P$45,"Zinsertraege",$S$41:$S$45)+SUMIF($P$50:$P$55,"Zinsertraege",$S$50:$S$55),2)</f>
       </c>
       <c r="S15" s="115" t="str">
         <f>=IFERROR(ROUND(L15 + Q15, 2), Q15)</f>
@@ -8043,10 +8043,10 @@
         <v>278</v>
       </c>
       <c r="X15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"Zinsertraege",Einnahmen_4[Einnahmen (LC)])+SUMIF(Einnahmen_WK_4[Typ],"Zinsertraege",Einnahmen_WK_4[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"Zinsertraege",$Y$41:$Y$45)+SUMIF($W$50:$W$55,"Zinsertraege",$Y$50:$Y$55),2)</f>
       </c>
       <c r="Y15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_4[Typ],"Zinsertraege",Einnahmen_4[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_4[Typ],"Zinsertraege",Einnahmen_WK_4[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($W$41:$W$45,"Zinsertraege",$Z$41:$Z$45)+SUMIF($W$50:$W$55,"Zinsertraege",$Z$50:$Z$55),2)</f>
       </c>
       <c r="Z15" s="115" t="str">
         <f>=IFERROR(ROUND(S15 + X15, 2), X15)</f>
@@ -8058,10 +8058,10 @@
         <v>278</v>
       </c>
       <c r="AE15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"Zinsertraege",Einnahmen_5[Einnahmen (LC)])+SUMIF(Einnahmen_WK_5[Typ],"Zinsertraege",Einnahmen_WK_5[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"Zinsertraege",$AF$41:$AF$45)+SUMIF($AD$50:$AD$55,"Zinsertraege",$AF$50:$AF$55),2)</f>
       </c>
       <c r="AF15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_5[Typ],"Zinsertraege",Einnahmen_5[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_5[Typ],"Zinsertraege",Einnahmen_WK_5[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AD$41:$AD$45,"Zinsertraege",$AG$41:$AG$45)+SUMIF($AD$50:$AD$55,"Zinsertraege",$AG$50:$AG$55),2)</f>
       </c>
       <c r="AG15" s="115" t="str">
         <f>=IFERROR(ROUND(Z15 + AE15, 2), AE15)</f>
@@ -8073,10 +8073,10 @@
         <v>278</v>
       </c>
       <c r="AL15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"Zinsertraege",Einnahmen_6[Einnahmen (LC)])+SUMIF(Einnahmen_WK_6[Typ],"Zinsertraege",Einnahmen_WK_6[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"Zinsertraege",$AM$41:$AM$45)+SUMIF($AK$50:$AK$55,"Zinsertraege",$AM$50:$AM$55),2)</f>
       </c>
       <c r="AM15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_6[Typ],"Zinsertraege",Einnahmen_6[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_6[Typ],"Zinsertraege",Einnahmen_WK_6[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AK$41:$AK$45,"Zinsertraege",$AN$41:$AN$45)+SUMIF($AK$50:$AK$55,"Zinsertraege",$AN$50:$AN$55),2)</f>
       </c>
       <c r="AN15" s="115" t="str">
         <f>=IFERROR(ROUND(AG15 + AL15, 2), AL15)</f>
@@ -8088,10 +8088,10 @@
         <v>278</v>
       </c>
       <c r="AS15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"Zinsertraege",Einnahmen_7[Einnahmen (LC)])+SUMIF(Einnahmen_WK_7[Typ],"Zinsertraege",Einnahmen_WK_7[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"Zinsertraege",$AT$41:$AT$45)+SUMIF($AR$50:$AR$55,"Zinsertraege",$AT$50:$AT$55),2)</f>
       </c>
       <c r="AT15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_7[Typ],"Zinsertraege",Einnahmen_7[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_7[Typ],"Zinsertraege",Einnahmen_WK_7[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AR$41:$AR$45,"Zinsertraege",$AU$41:$AU$45)+SUMIF($AR$50:$AR$55,"Zinsertraege",$AU$50:$AU$55),2)</f>
       </c>
       <c r="AU15" s="115" t="str">
         <f>=IFERROR(ROUND(AN15 + AS15, 2), AS15)</f>
@@ -8103,10 +8103,10 @@
         <v>278</v>
       </c>
       <c r="AZ15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"Zinsertraege",Einnahmen_8[Einnahmen (LC)])+SUMIF(Einnahmen_WK_8[Typ],"Zinsertraege",Einnahmen_WK_8[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"Zinsertraege",$BA$41:$BA$45)+SUMIF($AY$50:$AY$55,"Zinsertraege",$BA$50:$BA$55),2)</f>
       </c>
       <c r="BA15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_8[Typ],"Zinsertraege",Einnahmen_8[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_8[Typ],"Zinsertraege",Einnahmen_WK_8[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($AY$41:$AY$45,"Zinsertraege",$BB$41:$BB$45)+SUMIF($AY$50:$AY$55,"Zinsertraege",$BB$50:$BB$55),2)</f>
       </c>
       <c r="BB15" s="115" t="str">
         <f>=IFERROR(ROUND(AU15 + AZ15, 2), AZ15)</f>
@@ -8118,10 +8118,10 @@
         <v>278</v>
       </c>
       <c r="BG15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"Zinsertraege",Einnahmen_9[Einnahmen (LC)])+SUMIF(Einnahmen_WK_9[Typ],"Zinsertraege",Einnahmen_WK_9[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"Zinsertraege",$BH$41:$BH$45)+SUMIF($BF$50:$BF$55,"Zinsertraege",$BH$50:$BH$55),2)</f>
       </c>
       <c r="BH15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_9[Typ],"Zinsertraege",Einnahmen_9[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_9[Typ],"Zinsertraege",Einnahmen_WK_9[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BF$41:$BF$45,"Zinsertraege",$BI$41:$BI$45)+SUMIF($BF$50:$BF$55,"Zinsertraege",$BI$50:$BI$55),2)</f>
       </c>
       <c r="BI15" s="115" t="str">
         <f>=IFERROR(ROUND(BB15 + BG15, 2), BG15)</f>
@@ -8133,10 +8133,10 @@
         <v>278</v>
       </c>
       <c r="BN15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"Zinsertraege",Einnahmen_10[Einnahmen (LC)])+SUMIF(Einnahmen_WK_10[Typ],"Zinsertraege",Einnahmen_WK_10[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"Zinsertraege",$BO$41:$BO$45)+SUMIF($BM$50:$BM$55,"Zinsertraege",$BO$50:$BO$55),2)</f>
       </c>
       <c r="BO15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_10[Typ],"Zinsertraege",Einnahmen_10[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_10[Typ],"Zinsertraege",Einnahmen_WK_10[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BM$41:$BM$45,"Zinsertraege",$BP$41:$BP$45)+SUMIF($BM$50:$BM$55,"Zinsertraege",$BP$50:$BP$55),2)</f>
       </c>
       <c r="BP15" s="115" t="str">
         <f>=IFERROR(ROUND(BI15 + BN15, 2), BN15)</f>
@@ -8148,10 +8148,10 @@
         <v>278</v>
       </c>
       <c r="BU15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"Zinsertraege",Einnahmen_11[Einnahmen (LC)])+SUMIF(Einnahmen_WK_11[Typ],"Zinsertraege",Einnahmen_WK_11[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"Zinsertraege",$BV$41:$BV$45)+SUMIF($BT$50:$BT$55,"Zinsertraege",$BV$50:$BV$55),2)</f>
       </c>
       <c r="BV15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_11[Typ],"Zinsertraege",Einnahmen_11[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_11[Typ],"Zinsertraege",Einnahmen_WK_11[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($BT$41:$BT$45,"Zinsertraege",$BW$41:$BW$45)+SUMIF($BT$50:$BT$55,"Zinsertraege",$BW$50:$BW$55),2)</f>
       </c>
       <c r="BW15" s="115" t="str">
         <f>=IFERROR(ROUND(BP15 + BU15, 2), BU15)</f>
@@ -8163,10 +8163,10 @@
         <v>278</v>
       </c>
       <c r="CB15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"Zinsertraege",Einnahmen_12[Einnahmen (LC)])+SUMIF(Einnahmen_WK_12[Typ],"Zinsertraege",Einnahmen_WK_12[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"Zinsertraege",$CC$41:$CC$45)+SUMIF($CA$50:$CA$55,"Zinsertraege",$CC$50:$CC$55),2)</f>
       </c>
       <c r="CC15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_12[Typ],"Zinsertraege",Einnahmen_12[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_12[Typ],"Zinsertraege",Einnahmen_WK_12[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CA$41:$CA$45,"Zinsertraege",$CD$41:$CD$45)+SUMIF($CA$50:$CA$55,"Zinsertraege",$CD$50:$CD$55),2)</f>
       </c>
       <c r="CD15" s="115" t="str">
         <f>=IFERROR(ROUND(BW15 + CB15, 2), CB15)</f>
@@ -8178,10 +8178,10 @@
         <v>278</v>
       </c>
       <c r="CI15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"Zinsertraege",Einnahmen_13[Einnahmen (LC)])+SUMIF(Einnahmen_WK_13[Typ],"Zinsertraege",Einnahmen_WK_13[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"Zinsertraege",$CJ$41:$CJ$45)+SUMIF($CH$50:$CH$55,"Zinsertraege",$CJ$50:$CJ$55),2)</f>
       </c>
       <c r="CJ15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_13[Typ],"Zinsertraege",Einnahmen_13[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_13[Typ],"Zinsertraege",Einnahmen_WK_13[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CH$41:$CH$45,"Zinsertraege",$CK$41:$CK$45)+SUMIF($CH$50:$CH$55,"Zinsertraege",$CK$50:$CK$55),2)</f>
       </c>
       <c r="CK15" s="115" t="str">
         <f>=IFERROR(ROUND(CD15 + CI15, 2), CI15)</f>
@@ -8193,10 +8193,10 @@
         <v>278</v>
       </c>
       <c r="CP15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"Zinsertraege",Einnahmen_14[Einnahmen (LC)])+SUMIF(Einnahmen_WK_14[Typ],"Zinsertraege",Einnahmen_WK_14[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"Zinsertraege",$CQ$41:$CQ$45)+SUMIF($CO$50:$CO$55,"Zinsertraege",$CQ$50:$CQ$55),2)</f>
       </c>
       <c r="CQ15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_14[Typ],"Zinsertraege",Einnahmen_14[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_14[Typ],"Zinsertraege",Einnahmen_WK_14[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CO$41:$CO$45,"Zinsertraege",$CR$41:$CR$45)+SUMIF($CO$50:$CO$55,"Zinsertraege",$CR$50:$CR$55),2)</f>
       </c>
       <c r="CR15" s="115" t="str">
         <f>=IFERROR(ROUND(CK15 + CP15, 2), CP15)</f>
@@ -8208,10 +8208,10 @@
         <v>278</v>
       </c>
       <c r="CW15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"Zinsertraege",Einnahmen_15[Einnahmen (LC)])+SUMIF(Einnahmen_WK_15[Typ],"Zinsertraege",Einnahmen_WK_15[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"Zinsertraege",$CX$41:$CX$45)+SUMIF($CV$50:$CV$55,"Zinsertraege",$CX$50:$CX$55),2)</f>
       </c>
       <c r="CX15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_15[Typ],"Zinsertraege",Einnahmen_15[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_15[Typ],"Zinsertraege",Einnahmen_WK_15[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($CV$41:$CV$45,"Zinsertraege",$CY$41:$CY$45)+SUMIF($CV$50:$CV$55,"Zinsertraege",$CY$50:$CY$55),2)</f>
       </c>
       <c r="CY15" s="115" t="str">
         <f>=IFERROR(ROUND(CR15 + CW15, 2), CW15)</f>
@@ -8223,10 +8223,10 @@
         <v>278</v>
       </c>
       <c r="DD15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"Zinsertraege",Einnahmen_16[Einnahmen (LC)])+SUMIF(Einnahmen_WK_16[Typ],"Zinsertraege",Einnahmen_WK_16[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"Zinsertraege",$DE$41:$DE$45)+SUMIF($DC$50:$DC$55,"Zinsertraege",$DE$50:$DE$55),2)</f>
       </c>
       <c r="DE15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_16[Typ],"Zinsertraege",Einnahmen_16[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_16[Typ],"Zinsertraege",Einnahmen_WK_16[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DC$41:$DC$45,"Zinsertraege",$DF$41:$DF$45)+SUMIF($DC$50:$DC$55,"Zinsertraege",$DF$50:$DF$55),2)</f>
       </c>
       <c r="DF15" s="115" t="str">
         <f>=IFERROR(ROUND(CY15 + DD15, 2), DD15)</f>
@@ -8238,10 +8238,10 @@
         <v>278</v>
       </c>
       <c r="DK15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"Zinsertraege",Einnahmen_17[Einnahmen (LC)])+SUMIF(Einnahmen_WK_17[Typ],"Zinsertraege",Einnahmen_WK_17[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"Zinsertraege",$DL$41:$DL$45)+SUMIF($DJ$50:$DJ$55,"Zinsertraege",$DL$50:$DL$55),2)</f>
       </c>
       <c r="DL15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_17[Typ],"Zinsertraege",Einnahmen_17[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_17[Typ],"Zinsertraege",Einnahmen_WK_17[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DJ$41:$DJ$45,"Zinsertraege",$DM$41:$DM$45)+SUMIF($DJ$50:$DJ$55,"Zinsertraege",$DM$50:$DM$55),2)</f>
       </c>
       <c r="DM15" s="115" t="str">
         <f>=IFERROR(ROUND(DF15 + DK15, 2), DK15)</f>
@@ -8253,10 +8253,10 @@
         <v>278</v>
       </c>
       <c r="DR15" s="115" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"Zinsertraege",Einnahmen_18[Einnahmen (LC)])+SUMIF(Einnahmen_WK_18[Typ],"Zinsertraege",Einnahmen_WK_18[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"Zinsertraege",$DS$41:$DS$45)+SUMIF($DQ$50:$DQ$55,"Zinsertraege",$DS$50:$DS$55),2)</f>
       </c>
       <c r="DS15" s="116" t="str">
-        <f>=ROUND(SUMIF(Einnahmen_18[Typ],"Zinsertraege",Einnahmen_18[Einnahmen (EUR)])+SUMIF(Einnahmen_WK_18[Typ],"Zinsertraege",Einnahmen_WK_18[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUMIF($DQ$41:$DQ$45,"Zinsertraege",$DT$41:$DT$45)+SUMIF($DQ$50:$DQ$55,"Zinsertraege",$DT$50:$DT$55),2)</f>
       </c>
       <c r="DT15" s="115" t="str">
         <f>=IFERROR(ROUND(DM15 + DR15, 2), DR15)</f>
@@ -8959,10 +8959,10 @@
         <f>=IFERROR(ROUND(J19/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L19" s="115" t="str">
-        <f>=IFERROR(J19 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I19), J19)</f>
+        <f>=IFERROR(J19 + SUMIFS($E$19:$E$26, $B$19:$B$26, I19), J19)</f>
       </c>
       <c r="M19" s="143" t="str">
-        <f>=IFERROR(K19 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I19), K19)</f>
+        <f>=IFERROR(K19 + SUMIFS($F$19:$F$26, $B$19:$B$26, I19), K19)</f>
       </c>
       <c r="P19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -8972,10 +8972,10 @@
         <f>=IFERROR(ROUND(Q19/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S19" s="115" t="str">
-        <f>=IFERROR(Q19 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P19), Q19)</f>
+        <f>=IFERROR(Q19 + SUMIFS($L$19:$L$26, $I$19:$I$26, P19), Q19)</f>
       </c>
       <c r="T19" s="143" t="str">
-        <f>=IFERROR(R19 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P19), R19)</f>
+        <f>=IFERROR(R19 + SUMIFS($M$19:$M$26, $I$19:$I$26, P19), R19)</f>
       </c>
       <c r="W19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -8985,10 +8985,10 @@
         <f>=IFERROR(ROUND(X19/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z19" s="115" t="str">
-        <f>=IFERROR(X19 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W19), X19)</f>
+        <f>=IFERROR(X19 + SUMIFS($S$19:$S$26, $P$19:$P$26, W19), X19)</f>
       </c>
       <c r="AA19" s="143" t="str">
-        <f>=IFERROR(Y19 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W19), Y19)</f>
+        <f>=IFERROR(Y19 + SUMIFS($T$19:$T$26, $P$19:$P$26, W19), Y19)</f>
       </c>
       <c r="AD19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -8998,10 +8998,10 @@
         <f>=IFERROR(ROUND(AE19/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG19" s="115" t="str">
-        <f>=IFERROR(AE19 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD19), AE19)</f>
+        <f>=IFERROR(AE19 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD19), AE19)</f>
       </c>
       <c r="AH19" s="143" t="str">
-        <f>=IFERROR(AF19 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD19), AF19)</f>
+        <f>=IFERROR(AF19 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD19), AF19)</f>
       </c>
       <c r="AK19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9011,10 +9011,10 @@
         <f>=IFERROR(ROUND(AL19/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN19" s="115" t="str">
-        <f>=IFERROR(AL19 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK19), AL19)</f>
+        <f>=IFERROR(AL19 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK19), AL19)</f>
       </c>
       <c r="AO19" s="143" t="str">
-        <f>=IFERROR(AM19 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK19), AM19)</f>
+        <f>=IFERROR(AM19 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK19), AM19)</f>
       </c>
       <c r="AR19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9024,10 +9024,10 @@
         <f>=IFERROR(ROUND(AS19/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU19" s="115" t="str">
-        <f>=IFERROR(AS19 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR19), AS19)</f>
+        <f>=IFERROR(AS19 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR19), AS19)</f>
       </c>
       <c r="AV19" s="143" t="str">
-        <f>=IFERROR(AT19 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR19), AT19)</f>
+        <f>=IFERROR(AT19 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR19), AT19)</f>
       </c>
       <c r="AY19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9037,10 +9037,10 @@
         <f>=IFERROR(ROUND(AZ19/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB19" s="115" t="str">
-        <f>=IFERROR(AZ19 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY19), AZ19)</f>
+        <f>=IFERROR(AZ19 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY19), AZ19)</f>
       </c>
       <c r="BC19" s="143" t="str">
-        <f>=IFERROR(BA19 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY19), BA19)</f>
+        <f>=IFERROR(BA19 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY19), BA19)</f>
       </c>
       <c r="BF19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9050,10 +9050,10 @@
         <f>=IFERROR(ROUND(BG19/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI19" s="115" t="str">
-        <f>=IFERROR(BG19 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF19), BG19)</f>
+        <f>=IFERROR(BG19 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF19), BG19)</f>
       </c>
       <c r="BJ19" s="143" t="str">
-        <f>=IFERROR(BH19 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF19), BH19)</f>
+        <f>=IFERROR(BH19 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF19), BH19)</f>
       </c>
       <c r="BM19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9063,10 +9063,10 @@
         <f>=IFERROR(ROUND(BN19/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP19" s="115" t="str">
-        <f>=IFERROR(BN19 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM19), BN19)</f>
+        <f>=IFERROR(BN19 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM19), BN19)</f>
       </c>
       <c r="BQ19" s="143" t="str">
-        <f>=IFERROR(BO19 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM19), BO19)</f>
+        <f>=IFERROR(BO19 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM19), BO19)</f>
       </c>
       <c r="BT19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9076,10 +9076,10 @@
         <f>=IFERROR(ROUND(BU19/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW19" s="115" t="str">
-        <f>=IFERROR(BU19 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT19), BU19)</f>
+        <f>=IFERROR(BU19 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT19), BU19)</f>
       </c>
       <c r="BX19" s="143" t="str">
-        <f>=IFERROR(BV19 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT19), BV19)</f>
+        <f>=IFERROR(BV19 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT19), BV19)</f>
       </c>
       <c r="CA19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9089,10 +9089,10 @@
         <f>=IFERROR(ROUND(CB19/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD19" s="115" t="str">
-        <f>=IFERROR(CB19 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA19), CB19)</f>
+        <f>=IFERROR(CB19 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA19), CB19)</f>
       </c>
       <c r="CE19" s="143" t="str">
-        <f>=IFERROR(CC19 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA19), CC19)</f>
+        <f>=IFERROR(CC19 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA19), CC19)</f>
       </c>
       <c r="CH19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9102,10 +9102,10 @@
         <f>=IFERROR(ROUND(CI19/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK19" s="115" t="str">
-        <f>=IFERROR(CI19 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH19), CI19)</f>
+        <f>=IFERROR(CI19 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH19), CI19)</f>
       </c>
       <c r="CL19" s="143" t="str">
-        <f>=IFERROR(CJ19 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH19), CJ19)</f>
+        <f>=IFERROR(CJ19 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH19), CJ19)</f>
       </c>
       <c r="CO19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9115,10 +9115,10 @@
         <f>=IFERROR(ROUND(CP19/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR19" s="115" t="str">
-        <f>=IFERROR(CP19 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO19), CP19)</f>
+        <f>=IFERROR(CP19 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO19), CP19)</f>
       </c>
       <c r="CS19" s="143" t="str">
-        <f>=IFERROR(CQ19 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO19), CQ19)</f>
+        <f>=IFERROR(CQ19 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO19), CQ19)</f>
       </c>
       <c r="CV19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9128,10 +9128,10 @@
         <f>=IFERROR(ROUND(CW19/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY19" s="115" t="str">
-        <f>=IFERROR(CW19 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV19), CW19)</f>
+        <f>=IFERROR(CW19 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV19), CW19)</f>
       </c>
       <c r="CZ19" s="143" t="str">
-        <f>=IFERROR(CX19 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV19), CX19)</f>
+        <f>=IFERROR(CX19 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV19), CX19)</f>
       </c>
       <c r="DC19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9141,10 +9141,10 @@
         <f>=IFERROR(ROUND(DD19/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF19" s="115" t="str">
-        <f>=IFERROR(DD19 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC19), DD19)</f>
+        <f>=IFERROR(DD19 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC19), DD19)</f>
       </c>
       <c r="DG19" s="143" t="str">
-        <f>=IFERROR(DE19 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC19), DE19)</f>
+        <f>=IFERROR(DE19 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC19), DE19)</f>
       </c>
       <c r="DJ19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9154,10 +9154,10 @@
         <f>=IFERROR(ROUND(DK19/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM19" s="115" t="str">
-        <f>=IFERROR(DK19 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ19), DK19)</f>
+        <f>=IFERROR(DK19 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ19), DK19)</f>
       </c>
       <c r="DN19" s="143" t="str">
-        <f>=IFERROR(DL19 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ19), DL19)</f>
+        <f>=IFERROR(DL19 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ19), DL19)</f>
       </c>
       <c r="DQ19" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9167,10 +9167,10 @@
         <f>=IFERROR(ROUND(DR19/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT19" s="115" t="str">
-        <f>=IFERROR(DR19 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ19), DR19)</f>
+        <f>=IFERROR(DR19 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ19), DR19)</f>
       </c>
       <c r="DU19" s="143" t="str">
-        <f>=IFERROR(DS19 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ19), DS19)</f>
+        <f>=IFERROR(DS19 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ19), DS19)</f>
       </c>
     </row>
     <row r="20">
@@ -9195,10 +9195,10 @@
         <f>=IFERROR(ROUND(J20/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L20" s="115" t="str">
-        <f>=IFERROR(J20 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I20), J20)</f>
+        <f>=IFERROR(J20 + SUMIFS($E$19:$E$26, $B$19:$B$26, I20), J20)</f>
       </c>
       <c r="M20" s="143" t="str">
-        <f>=IFERROR(K20 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I20), K20)</f>
+        <f>=IFERROR(K20 + SUMIFS($F$19:$F$26, $B$19:$B$26, I20), K20)</f>
       </c>
       <c r="P20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9208,10 +9208,10 @@
         <f>=IFERROR(ROUND(Q20/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S20" s="115" t="str">
-        <f>=IFERROR(Q20 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P20), Q20)</f>
+        <f>=IFERROR(Q20 + SUMIFS($L$19:$L$26, $I$19:$I$26, P20), Q20)</f>
       </c>
       <c r="T20" s="143" t="str">
-        <f>=IFERROR(R20 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P20), R20)</f>
+        <f>=IFERROR(R20 + SUMIFS($M$19:$M$26, $I$19:$I$26, P20), R20)</f>
       </c>
       <c r="W20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9221,10 +9221,10 @@
         <f>=IFERROR(ROUND(X20/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z20" s="115" t="str">
-        <f>=IFERROR(X20 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W20), X20)</f>
+        <f>=IFERROR(X20 + SUMIFS($S$19:$S$26, $P$19:$P$26, W20), X20)</f>
       </c>
       <c r="AA20" s="143" t="str">
-        <f>=IFERROR(Y20 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W20), Y20)</f>
+        <f>=IFERROR(Y20 + SUMIFS($T$19:$T$26, $P$19:$P$26, W20), Y20)</f>
       </c>
       <c r="AD20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9234,10 +9234,10 @@
         <f>=IFERROR(ROUND(AE20/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG20" s="115" t="str">
-        <f>=IFERROR(AE20 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD20), AE20)</f>
+        <f>=IFERROR(AE20 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD20), AE20)</f>
       </c>
       <c r="AH20" s="143" t="str">
-        <f>=IFERROR(AF20 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD20), AF20)</f>
+        <f>=IFERROR(AF20 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD20), AF20)</f>
       </c>
       <c r="AK20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9247,10 +9247,10 @@
         <f>=IFERROR(ROUND(AL20/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN20" s="115" t="str">
-        <f>=IFERROR(AL20 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK20), AL20)</f>
+        <f>=IFERROR(AL20 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK20), AL20)</f>
       </c>
       <c r="AO20" s="143" t="str">
-        <f>=IFERROR(AM20 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK20), AM20)</f>
+        <f>=IFERROR(AM20 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK20), AM20)</f>
       </c>
       <c r="AR20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9260,10 +9260,10 @@
         <f>=IFERROR(ROUND(AS20/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU20" s="115" t="str">
-        <f>=IFERROR(AS20 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR20), AS20)</f>
+        <f>=IFERROR(AS20 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR20), AS20)</f>
       </c>
       <c r="AV20" s="143" t="str">
-        <f>=IFERROR(AT20 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR20), AT20)</f>
+        <f>=IFERROR(AT20 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR20), AT20)</f>
       </c>
       <c r="AY20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9273,10 +9273,10 @@
         <f>=IFERROR(ROUND(AZ20/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB20" s="115" t="str">
-        <f>=IFERROR(AZ20 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY20), AZ20)</f>
+        <f>=IFERROR(AZ20 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY20), AZ20)</f>
       </c>
       <c r="BC20" s="143" t="str">
-        <f>=IFERROR(BA20 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY20), BA20)</f>
+        <f>=IFERROR(BA20 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY20), BA20)</f>
       </c>
       <c r="BF20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9286,10 +9286,10 @@
         <f>=IFERROR(ROUND(BG20/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI20" s="115" t="str">
-        <f>=IFERROR(BG20 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF20), BG20)</f>
+        <f>=IFERROR(BG20 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF20), BG20)</f>
       </c>
       <c r="BJ20" s="143" t="str">
-        <f>=IFERROR(BH20 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF20), BH20)</f>
+        <f>=IFERROR(BH20 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF20), BH20)</f>
       </c>
       <c r="BM20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9299,10 +9299,10 @@
         <f>=IFERROR(ROUND(BN20/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP20" s="115" t="str">
-        <f>=IFERROR(BN20 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM20), BN20)</f>
+        <f>=IFERROR(BN20 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM20), BN20)</f>
       </c>
       <c r="BQ20" s="143" t="str">
-        <f>=IFERROR(BO20 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM20), BO20)</f>
+        <f>=IFERROR(BO20 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM20), BO20)</f>
       </c>
       <c r="BT20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9312,10 +9312,10 @@
         <f>=IFERROR(ROUND(BU20/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW20" s="115" t="str">
-        <f>=IFERROR(BU20 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT20), BU20)</f>
+        <f>=IFERROR(BU20 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT20), BU20)</f>
       </c>
       <c r="BX20" s="143" t="str">
-        <f>=IFERROR(BV20 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT20), BV20)</f>
+        <f>=IFERROR(BV20 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT20), BV20)</f>
       </c>
       <c r="CA20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9325,10 +9325,10 @@
         <f>=IFERROR(ROUND(CB20/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD20" s="115" t="str">
-        <f>=IFERROR(CB20 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA20), CB20)</f>
+        <f>=IFERROR(CB20 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA20), CB20)</f>
       </c>
       <c r="CE20" s="143" t="str">
-        <f>=IFERROR(CC20 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA20), CC20)</f>
+        <f>=IFERROR(CC20 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA20), CC20)</f>
       </c>
       <c r="CH20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9338,10 +9338,10 @@
         <f>=IFERROR(ROUND(CI20/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK20" s="115" t="str">
-        <f>=IFERROR(CI20 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH20), CI20)</f>
+        <f>=IFERROR(CI20 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH20), CI20)</f>
       </c>
       <c r="CL20" s="143" t="str">
-        <f>=IFERROR(CJ20 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH20), CJ20)</f>
+        <f>=IFERROR(CJ20 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH20), CJ20)</f>
       </c>
       <c r="CO20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9351,10 +9351,10 @@
         <f>=IFERROR(ROUND(CP20/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR20" s="115" t="str">
-        <f>=IFERROR(CP20 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO20), CP20)</f>
+        <f>=IFERROR(CP20 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO20), CP20)</f>
       </c>
       <c r="CS20" s="143" t="str">
-        <f>=IFERROR(CQ20 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO20), CQ20)</f>
+        <f>=IFERROR(CQ20 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO20), CQ20)</f>
       </c>
       <c r="CV20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9364,10 +9364,10 @@
         <f>=IFERROR(ROUND(CW20/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY20" s="115" t="str">
-        <f>=IFERROR(CW20 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV20), CW20)</f>
+        <f>=IFERROR(CW20 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV20), CW20)</f>
       </c>
       <c r="CZ20" s="143" t="str">
-        <f>=IFERROR(CX20 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV20), CX20)</f>
+        <f>=IFERROR(CX20 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV20), CX20)</f>
       </c>
       <c r="DC20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9377,10 +9377,10 @@
         <f>=IFERROR(ROUND(DD20/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF20" s="115" t="str">
-        <f>=IFERROR(DD20 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC20), DD20)</f>
+        <f>=IFERROR(DD20 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC20), DD20)</f>
       </c>
       <c r="DG20" s="143" t="str">
-        <f>=IFERROR(DE20 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC20), DE20)</f>
+        <f>=IFERROR(DE20 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC20), DE20)</f>
       </c>
       <c r="DJ20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9390,10 +9390,10 @@
         <f>=IFERROR(ROUND(DK20/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM20" s="115" t="str">
-        <f>=IFERROR(DK20 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ20), DK20)</f>
+        <f>=IFERROR(DK20 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ20), DK20)</f>
       </c>
       <c r="DN20" s="143" t="str">
-        <f>=IFERROR(DL20 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ20), DL20)</f>
+        <f>=IFERROR(DL20 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ20), DL20)</f>
       </c>
       <c r="DQ20" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9403,10 +9403,10 @@
         <f>=IFERROR(ROUND(DR20/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT20" s="115" t="str">
-        <f>=IFERROR(DR20 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ20), DR20)</f>
+        <f>=IFERROR(DR20 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ20), DR20)</f>
       </c>
       <c r="DU20" s="143" t="str">
-        <f>=IFERROR(DS20 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ20), DS20)</f>
+        <f>=IFERROR(DS20 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ20), DS20)</f>
       </c>
     </row>
     <row r="21">
@@ -9431,10 +9431,10 @@
         <f>=IFERROR(ROUND(J21/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L21" s="115" t="str">
-        <f>=IFERROR(J21 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I21), J21)</f>
+        <f>=IFERROR(J21 + SUMIFS($E$19:$E$26, $B$19:$B$26, I21), J21)</f>
       </c>
       <c r="M21" s="143" t="str">
-        <f>=IFERROR(K21 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I21), K21)</f>
+        <f>=IFERROR(K21 + SUMIFS($F$19:$F$26, $B$19:$B$26, I21), K21)</f>
       </c>
       <c r="P21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9444,10 +9444,10 @@
         <f>=IFERROR(ROUND(Q21/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S21" s="115" t="str">
-        <f>=IFERROR(Q21 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P21), Q21)</f>
+        <f>=IFERROR(Q21 + SUMIFS($L$19:$L$26, $I$19:$I$26, P21), Q21)</f>
       </c>
       <c r="T21" s="143" t="str">
-        <f>=IFERROR(R21 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P21), R21)</f>
+        <f>=IFERROR(R21 + SUMIFS($M$19:$M$26, $I$19:$I$26, P21), R21)</f>
       </c>
       <c r="W21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9457,10 +9457,10 @@
         <f>=IFERROR(ROUND(X21/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z21" s="115" t="str">
-        <f>=IFERROR(X21 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W21), X21)</f>
+        <f>=IFERROR(X21 + SUMIFS($S$19:$S$26, $P$19:$P$26, W21), X21)</f>
       </c>
       <c r="AA21" s="143" t="str">
-        <f>=IFERROR(Y21 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W21), Y21)</f>
+        <f>=IFERROR(Y21 + SUMIFS($T$19:$T$26, $P$19:$P$26, W21), Y21)</f>
       </c>
       <c r="AD21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9470,10 +9470,10 @@
         <f>=IFERROR(ROUND(AE21/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG21" s="115" t="str">
-        <f>=IFERROR(AE21 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD21), AE21)</f>
+        <f>=IFERROR(AE21 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD21), AE21)</f>
       </c>
       <c r="AH21" s="143" t="str">
-        <f>=IFERROR(AF21 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD21), AF21)</f>
+        <f>=IFERROR(AF21 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD21), AF21)</f>
       </c>
       <c r="AK21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9483,10 +9483,10 @@
         <f>=IFERROR(ROUND(AL21/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN21" s="115" t="str">
-        <f>=IFERROR(AL21 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK21), AL21)</f>
+        <f>=IFERROR(AL21 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK21), AL21)</f>
       </c>
       <c r="AO21" s="143" t="str">
-        <f>=IFERROR(AM21 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK21), AM21)</f>
+        <f>=IFERROR(AM21 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK21), AM21)</f>
       </c>
       <c r="AR21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9496,10 +9496,10 @@
         <f>=IFERROR(ROUND(AS21/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU21" s="115" t="str">
-        <f>=IFERROR(AS21 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR21), AS21)</f>
+        <f>=IFERROR(AS21 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR21), AS21)</f>
       </c>
       <c r="AV21" s="143" t="str">
-        <f>=IFERROR(AT21 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR21), AT21)</f>
+        <f>=IFERROR(AT21 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR21), AT21)</f>
       </c>
       <c r="AY21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9509,10 +9509,10 @@
         <f>=IFERROR(ROUND(AZ21/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB21" s="115" t="str">
-        <f>=IFERROR(AZ21 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY21), AZ21)</f>
+        <f>=IFERROR(AZ21 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY21), AZ21)</f>
       </c>
       <c r="BC21" s="143" t="str">
-        <f>=IFERROR(BA21 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY21), BA21)</f>
+        <f>=IFERROR(BA21 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY21), BA21)</f>
       </c>
       <c r="BF21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9522,10 +9522,10 @@
         <f>=IFERROR(ROUND(BG21/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI21" s="115" t="str">
-        <f>=IFERROR(BG21 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF21), BG21)</f>
+        <f>=IFERROR(BG21 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF21), BG21)</f>
       </c>
       <c r="BJ21" s="143" t="str">
-        <f>=IFERROR(BH21 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF21), BH21)</f>
+        <f>=IFERROR(BH21 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF21), BH21)</f>
       </c>
       <c r="BM21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9535,10 +9535,10 @@
         <f>=IFERROR(ROUND(BN21/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP21" s="115" t="str">
-        <f>=IFERROR(BN21 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM21), BN21)</f>
+        <f>=IFERROR(BN21 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM21), BN21)</f>
       </c>
       <c r="BQ21" s="143" t="str">
-        <f>=IFERROR(BO21 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM21), BO21)</f>
+        <f>=IFERROR(BO21 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM21), BO21)</f>
       </c>
       <c r="BT21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9548,10 +9548,10 @@
         <f>=IFERROR(ROUND(BU21/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW21" s="115" t="str">
-        <f>=IFERROR(BU21 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT21), BU21)</f>
+        <f>=IFERROR(BU21 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT21), BU21)</f>
       </c>
       <c r="BX21" s="143" t="str">
-        <f>=IFERROR(BV21 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT21), BV21)</f>
+        <f>=IFERROR(BV21 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT21), BV21)</f>
       </c>
       <c r="CA21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9561,10 +9561,10 @@
         <f>=IFERROR(ROUND(CB21/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD21" s="115" t="str">
-        <f>=IFERROR(CB21 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA21), CB21)</f>
+        <f>=IFERROR(CB21 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA21), CB21)</f>
       </c>
       <c r="CE21" s="143" t="str">
-        <f>=IFERROR(CC21 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA21), CC21)</f>
+        <f>=IFERROR(CC21 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA21), CC21)</f>
       </c>
       <c r="CH21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9574,10 +9574,10 @@
         <f>=IFERROR(ROUND(CI21/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK21" s="115" t="str">
-        <f>=IFERROR(CI21 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH21), CI21)</f>
+        <f>=IFERROR(CI21 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH21), CI21)</f>
       </c>
       <c r="CL21" s="143" t="str">
-        <f>=IFERROR(CJ21 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH21), CJ21)</f>
+        <f>=IFERROR(CJ21 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH21), CJ21)</f>
       </c>
       <c r="CO21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9587,10 +9587,10 @@
         <f>=IFERROR(ROUND(CP21/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR21" s="115" t="str">
-        <f>=IFERROR(CP21 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO21), CP21)</f>
+        <f>=IFERROR(CP21 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO21), CP21)</f>
       </c>
       <c r="CS21" s="143" t="str">
-        <f>=IFERROR(CQ21 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO21), CQ21)</f>
+        <f>=IFERROR(CQ21 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO21), CQ21)</f>
       </c>
       <c r="CV21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9600,10 +9600,10 @@
         <f>=IFERROR(ROUND(CW21/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY21" s="115" t="str">
-        <f>=IFERROR(CW21 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV21), CW21)</f>
+        <f>=IFERROR(CW21 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV21), CW21)</f>
       </c>
       <c r="CZ21" s="143" t="str">
-        <f>=IFERROR(CX21 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV21), CX21)</f>
+        <f>=IFERROR(CX21 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV21), CX21)</f>
       </c>
       <c r="DC21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9613,10 +9613,10 @@
         <f>=IFERROR(ROUND(DD21/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF21" s="115" t="str">
-        <f>=IFERROR(DD21 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC21), DD21)</f>
+        <f>=IFERROR(DD21 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC21), DD21)</f>
       </c>
       <c r="DG21" s="143" t="str">
-        <f>=IFERROR(DE21 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC21), DE21)</f>
+        <f>=IFERROR(DE21 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC21), DE21)</f>
       </c>
       <c r="DJ21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9626,10 +9626,10 @@
         <f>=IFERROR(ROUND(DK21/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM21" s="115" t="str">
-        <f>=IFERROR(DK21 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ21), DK21)</f>
+        <f>=IFERROR(DK21 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ21), DK21)</f>
       </c>
       <c r="DN21" s="143" t="str">
-        <f>=IFERROR(DL21 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ21), DL21)</f>
+        <f>=IFERROR(DL21 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ21), DL21)</f>
       </c>
       <c r="DQ21" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9639,10 +9639,10 @@
         <f>=IFERROR(ROUND(DR21/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT21" s="115" t="str">
-        <f>=IFERROR(DR21 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ21), DR21)</f>
+        <f>=IFERROR(DR21 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ21), DR21)</f>
       </c>
       <c r="DU21" s="143" t="str">
-        <f>=IFERROR(DS21 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ21), DS21)</f>
+        <f>=IFERROR(DS21 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ21), DS21)</f>
       </c>
     </row>
     <row r="22">
@@ -9667,10 +9667,10 @@
         <f>=IFERROR(ROUND(J22/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L22" s="115" t="str">
-        <f>=IFERROR(J22 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I22), J22)</f>
+        <f>=IFERROR(J22 + SUMIFS($E$19:$E$26, $B$19:$B$26, I22), J22)</f>
       </c>
       <c r="M22" s="143" t="str">
-        <f>=IFERROR(K22 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I22), K22)</f>
+        <f>=IFERROR(K22 + SUMIFS($F$19:$F$26, $B$19:$B$26, I22), K22)</f>
       </c>
       <c r="P22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9680,10 +9680,10 @@
         <f>=IFERROR(ROUND(Q22/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S22" s="115" t="str">
-        <f>=IFERROR(Q22 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P22), Q22)</f>
+        <f>=IFERROR(Q22 + SUMIFS($L$19:$L$26, $I$19:$I$26, P22), Q22)</f>
       </c>
       <c r="T22" s="143" t="str">
-        <f>=IFERROR(R22 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P22), R22)</f>
+        <f>=IFERROR(R22 + SUMIFS($M$19:$M$26, $I$19:$I$26, P22), R22)</f>
       </c>
       <c r="W22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9693,10 +9693,10 @@
         <f>=IFERROR(ROUND(X22/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z22" s="115" t="str">
-        <f>=IFERROR(X22 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W22), X22)</f>
+        <f>=IFERROR(X22 + SUMIFS($S$19:$S$26, $P$19:$P$26, W22), X22)</f>
       </c>
       <c r="AA22" s="143" t="str">
-        <f>=IFERROR(Y22 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W22), Y22)</f>
+        <f>=IFERROR(Y22 + SUMIFS($T$19:$T$26, $P$19:$P$26, W22), Y22)</f>
       </c>
       <c r="AD22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9706,10 +9706,10 @@
         <f>=IFERROR(ROUND(AE22/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG22" s="115" t="str">
-        <f>=IFERROR(AE22 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD22), AE22)</f>
+        <f>=IFERROR(AE22 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD22), AE22)</f>
       </c>
       <c r="AH22" s="143" t="str">
-        <f>=IFERROR(AF22 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD22), AF22)</f>
+        <f>=IFERROR(AF22 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD22), AF22)</f>
       </c>
       <c r="AK22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9719,10 +9719,10 @@
         <f>=IFERROR(ROUND(AL22/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN22" s="115" t="str">
-        <f>=IFERROR(AL22 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK22), AL22)</f>
+        <f>=IFERROR(AL22 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK22), AL22)</f>
       </c>
       <c r="AO22" s="143" t="str">
-        <f>=IFERROR(AM22 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK22), AM22)</f>
+        <f>=IFERROR(AM22 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK22), AM22)</f>
       </c>
       <c r="AR22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9732,10 +9732,10 @@
         <f>=IFERROR(ROUND(AS22/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU22" s="115" t="str">
-        <f>=IFERROR(AS22 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR22), AS22)</f>
+        <f>=IFERROR(AS22 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR22), AS22)</f>
       </c>
       <c r="AV22" s="143" t="str">
-        <f>=IFERROR(AT22 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR22), AT22)</f>
+        <f>=IFERROR(AT22 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR22), AT22)</f>
       </c>
       <c r="AY22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9745,10 +9745,10 @@
         <f>=IFERROR(ROUND(AZ22/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB22" s="115" t="str">
-        <f>=IFERROR(AZ22 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY22), AZ22)</f>
+        <f>=IFERROR(AZ22 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY22), AZ22)</f>
       </c>
       <c r="BC22" s="143" t="str">
-        <f>=IFERROR(BA22 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY22), BA22)</f>
+        <f>=IFERROR(BA22 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY22), BA22)</f>
       </c>
       <c r="BF22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9758,10 +9758,10 @@
         <f>=IFERROR(ROUND(BG22/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI22" s="115" t="str">
-        <f>=IFERROR(BG22 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF22), BG22)</f>
+        <f>=IFERROR(BG22 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF22), BG22)</f>
       </c>
       <c r="BJ22" s="143" t="str">
-        <f>=IFERROR(BH22 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF22), BH22)</f>
+        <f>=IFERROR(BH22 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF22), BH22)</f>
       </c>
       <c r="BM22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9771,10 +9771,10 @@
         <f>=IFERROR(ROUND(BN22/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP22" s="115" t="str">
-        <f>=IFERROR(BN22 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM22), BN22)</f>
+        <f>=IFERROR(BN22 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM22), BN22)</f>
       </c>
       <c r="BQ22" s="143" t="str">
-        <f>=IFERROR(BO22 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM22), BO22)</f>
+        <f>=IFERROR(BO22 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM22), BO22)</f>
       </c>
       <c r="BT22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9784,10 +9784,10 @@
         <f>=IFERROR(ROUND(BU22/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW22" s="115" t="str">
-        <f>=IFERROR(BU22 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT22), BU22)</f>
+        <f>=IFERROR(BU22 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT22), BU22)</f>
       </c>
       <c r="BX22" s="143" t="str">
-        <f>=IFERROR(BV22 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT22), BV22)</f>
+        <f>=IFERROR(BV22 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT22), BV22)</f>
       </c>
       <c r="CA22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9797,10 +9797,10 @@
         <f>=IFERROR(ROUND(CB22/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD22" s="115" t="str">
-        <f>=IFERROR(CB22 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA22), CB22)</f>
+        <f>=IFERROR(CB22 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA22), CB22)</f>
       </c>
       <c r="CE22" s="143" t="str">
-        <f>=IFERROR(CC22 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA22), CC22)</f>
+        <f>=IFERROR(CC22 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA22), CC22)</f>
       </c>
       <c r="CH22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9810,10 +9810,10 @@
         <f>=IFERROR(ROUND(CI22/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK22" s="115" t="str">
-        <f>=IFERROR(CI22 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH22), CI22)</f>
+        <f>=IFERROR(CI22 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH22), CI22)</f>
       </c>
       <c r="CL22" s="143" t="str">
-        <f>=IFERROR(CJ22 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH22), CJ22)</f>
+        <f>=IFERROR(CJ22 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH22), CJ22)</f>
       </c>
       <c r="CO22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9823,10 +9823,10 @@
         <f>=IFERROR(ROUND(CP22/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR22" s="115" t="str">
-        <f>=IFERROR(CP22 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO22), CP22)</f>
+        <f>=IFERROR(CP22 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO22), CP22)</f>
       </c>
       <c r="CS22" s="143" t="str">
-        <f>=IFERROR(CQ22 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO22), CQ22)</f>
+        <f>=IFERROR(CQ22 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO22), CQ22)</f>
       </c>
       <c r="CV22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9836,10 +9836,10 @@
         <f>=IFERROR(ROUND(CW22/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY22" s="115" t="str">
-        <f>=IFERROR(CW22 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV22), CW22)</f>
+        <f>=IFERROR(CW22 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV22), CW22)</f>
       </c>
       <c r="CZ22" s="143" t="str">
-        <f>=IFERROR(CX22 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV22), CX22)</f>
+        <f>=IFERROR(CX22 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV22), CX22)</f>
       </c>
       <c r="DC22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9849,10 +9849,10 @@
         <f>=IFERROR(ROUND(DD22/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF22" s="115" t="str">
-        <f>=IFERROR(DD22 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC22), DD22)</f>
+        <f>=IFERROR(DD22 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC22), DD22)</f>
       </c>
       <c r="DG22" s="143" t="str">
-        <f>=IFERROR(DE22 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC22), DE22)</f>
+        <f>=IFERROR(DE22 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC22), DE22)</f>
       </c>
       <c r="DJ22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9862,10 +9862,10 @@
         <f>=IFERROR(ROUND(DK22/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM22" s="115" t="str">
-        <f>=IFERROR(DK22 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ22), DK22)</f>
+        <f>=IFERROR(DK22 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ22), DK22)</f>
       </c>
       <c r="DN22" s="143" t="str">
-        <f>=IFERROR(DL22 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ22), DL22)</f>
+        <f>=IFERROR(DL22 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ22), DL22)</f>
       </c>
       <c r="DQ22" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9875,10 +9875,10 @@
         <f>=IFERROR(ROUND(DR22/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT22" s="115" t="str">
-        <f>=IFERROR(DR22 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ22), DR22)</f>
+        <f>=IFERROR(DR22 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ22), DR22)</f>
       </c>
       <c r="DU22" s="143" t="str">
-        <f>=IFERROR(DS22 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ22), DS22)</f>
+        <f>=IFERROR(DS22 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ22), DS22)</f>
       </c>
     </row>
     <row r="23">
@@ -9903,10 +9903,10 @@
         <f>=IFERROR(ROUND(J23/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L23" s="115" t="str">
-        <f>=IFERROR(J23 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I23), J23)</f>
+        <f>=IFERROR(J23 + SUMIFS($E$19:$E$26, $B$19:$B$26, I23), J23)</f>
       </c>
       <c r="M23" s="143" t="str">
-        <f>=IFERROR(K23 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I23), K23)</f>
+        <f>=IFERROR(K23 + SUMIFS($F$19:$F$26, $B$19:$B$26, I23), K23)</f>
       </c>
       <c r="P23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9916,10 +9916,10 @@
         <f>=IFERROR(ROUND(Q23/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S23" s="115" t="str">
-        <f>=IFERROR(Q23 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P23), Q23)</f>
+        <f>=IFERROR(Q23 + SUMIFS($L$19:$L$26, $I$19:$I$26, P23), Q23)</f>
       </c>
       <c r="T23" s="143" t="str">
-        <f>=IFERROR(R23 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P23), R23)</f>
+        <f>=IFERROR(R23 + SUMIFS($M$19:$M$26, $I$19:$I$26, P23), R23)</f>
       </c>
       <c r="W23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9929,10 +9929,10 @@
         <f>=IFERROR(ROUND(X23/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z23" s="115" t="str">
-        <f>=IFERROR(X23 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W23), X23)</f>
+        <f>=IFERROR(X23 + SUMIFS($S$19:$S$26, $P$19:$P$26, W23), X23)</f>
       </c>
       <c r="AA23" s="143" t="str">
-        <f>=IFERROR(Y23 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W23), Y23)</f>
+        <f>=IFERROR(Y23 + SUMIFS($T$19:$T$26, $P$19:$P$26, W23), Y23)</f>
       </c>
       <c r="AD23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9942,10 +9942,10 @@
         <f>=IFERROR(ROUND(AE23/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG23" s="115" t="str">
-        <f>=IFERROR(AE23 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD23), AE23)</f>
+        <f>=IFERROR(AE23 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD23), AE23)</f>
       </c>
       <c r="AH23" s="143" t="str">
-        <f>=IFERROR(AF23 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD23), AF23)</f>
+        <f>=IFERROR(AF23 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD23), AF23)</f>
       </c>
       <c r="AK23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9955,10 +9955,10 @@
         <f>=IFERROR(ROUND(AL23/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN23" s="115" t="str">
-        <f>=IFERROR(AL23 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK23), AL23)</f>
+        <f>=IFERROR(AL23 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK23), AL23)</f>
       </c>
       <c r="AO23" s="143" t="str">
-        <f>=IFERROR(AM23 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK23), AM23)</f>
+        <f>=IFERROR(AM23 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK23), AM23)</f>
       </c>
       <c r="AR23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9968,10 +9968,10 @@
         <f>=IFERROR(ROUND(AS23/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU23" s="115" t="str">
-        <f>=IFERROR(AS23 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR23), AS23)</f>
+        <f>=IFERROR(AS23 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR23), AS23)</f>
       </c>
       <c r="AV23" s="143" t="str">
-        <f>=IFERROR(AT23 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR23), AT23)</f>
+        <f>=IFERROR(AT23 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR23), AT23)</f>
       </c>
       <c r="AY23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9981,10 +9981,10 @@
         <f>=IFERROR(ROUND(AZ23/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB23" s="115" t="str">
-        <f>=IFERROR(AZ23 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY23), AZ23)</f>
+        <f>=IFERROR(AZ23 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY23), AZ23)</f>
       </c>
       <c r="BC23" s="143" t="str">
-        <f>=IFERROR(BA23 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY23), BA23)</f>
+        <f>=IFERROR(BA23 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY23), BA23)</f>
       </c>
       <c r="BF23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -9994,10 +9994,10 @@
         <f>=IFERROR(ROUND(BG23/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI23" s="115" t="str">
-        <f>=IFERROR(BG23 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF23), BG23)</f>
+        <f>=IFERROR(BG23 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF23), BG23)</f>
       </c>
       <c r="BJ23" s="143" t="str">
-        <f>=IFERROR(BH23 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF23), BH23)</f>
+        <f>=IFERROR(BH23 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF23), BH23)</f>
       </c>
       <c r="BM23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10007,10 +10007,10 @@
         <f>=IFERROR(ROUND(BN23/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP23" s="115" t="str">
-        <f>=IFERROR(BN23 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM23), BN23)</f>
+        <f>=IFERROR(BN23 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM23), BN23)</f>
       </c>
       <c r="BQ23" s="143" t="str">
-        <f>=IFERROR(BO23 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM23), BO23)</f>
+        <f>=IFERROR(BO23 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM23), BO23)</f>
       </c>
       <c r="BT23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10020,10 +10020,10 @@
         <f>=IFERROR(ROUND(BU23/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW23" s="115" t="str">
-        <f>=IFERROR(BU23 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT23), BU23)</f>
+        <f>=IFERROR(BU23 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT23), BU23)</f>
       </c>
       <c r="BX23" s="143" t="str">
-        <f>=IFERROR(BV23 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT23), BV23)</f>
+        <f>=IFERROR(BV23 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT23), BV23)</f>
       </c>
       <c r="CA23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10033,10 +10033,10 @@
         <f>=IFERROR(ROUND(CB23/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD23" s="115" t="str">
-        <f>=IFERROR(CB23 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA23), CB23)</f>
+        <f>=IFERROR(CB23 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA23), CB23)</f>
       </c>
       <c r="CE23" s="143" t="str">
-        <f>=IFERROR(CC23 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA23), CC23)</f>
+        <f>=IFERROR(CC23 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA23), CC23)</f>
       </c>
       <c r="CH23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10046,10 +10046,10 @@
         <f>=IFERROR(ROUND(CI23/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK23" s="115" t="str">
-        <f>=IFERROR(CI23 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH23), CI23)</f>
+        <f>=IFERROR(CI23 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH23), CI23)</f>
       </c>
       <c r="CL23" s="143" t="str">
-        <f>=IFERROR(CJ23 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH23), CJ23)</f>
+        <f>=IFERROR(CJ23 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH23), CJ23)</f>
       </c>
       <c r="CO23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10059,10 +10059,10 @@
         <f>=IFERROR(ROUND(CP23/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR23" s="115" t="str">
-        <f>=IFERROR(CP23 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO23), CP23)</f>
+        <f>=IFERROR(CP23 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO23), CP23)</f>
       </c>
       <c r="CS23" s="143" t="str">
-        <f>=IFERROR(CQ23 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO23), CQ23)</f>
+        <f>=IFERROR(CQ23 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO23), CQ23)</f>
       </c>
       <c r="CV23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10072,10 +10072,10 @@
         <f>=IFERROR(ROUND(CW23/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY23" s="115" t="str">
-        <f>=IFERROR(CW23 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV23), CW23)</f>
+        <f>=IFERROR(CW23 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV23), CW23)</f>
       </c>
       <c r="CZ23" s="143" t="str">
-        <f>=IFERROR(CX23 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV23), CX23)</f>
+        <f>=IFERROR(CX23 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV23), CX23)</f>
       </c>
       <c r="DC23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10085,10 +10085,10 @@
         <f>=IFERROR(ROUND(DD23/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF23" s="115" t="str">
-        <f>=IFERROR(DD23 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC23), DD23)</f>
+        <f>=IFERROR(DD23 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC23), DD23)</f>
       </c>
       <c r="DG23" s="143" t="str">
-        <f>=IFERROR(DE23 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC23), DE23)</f>
+        <f>=IFERROR(DE23 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC23), DE23)</f>
       </c>
       <c r="DJ23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10098,10 +10098,10 @@
         <f>=IFERROR(ROUND(DK23/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM23" s="115" t="str">
-        <f>=IFERROR(DK23 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ23), DK23)</f>
+        <f>=IFERROR(DK23 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ23), DK23)</f>
       </c>
       <c r="DN23" s="143" t="str">
-        <f>=IFERROR(DL23 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ23), DL23)</f>
+        <f>=IFERROR(DL23 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ23), DL23)</f>
       </c>
       <c r="DQ23" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10111,10 +10111,10 @@
         <f>=IFERROR(ROUND(DR23/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT23" s="115" t="str">
-        <f>=IFERROR(DR23 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ23), DR23)</f>
+        <f>=IFERROR(DR23 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ23), DR23)</f>
       </c>
       <c r="DU23" s="143" t="str">
-        <f>=IFERROR(DS23 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ23), DS23)</f>
+        <f>=IFERROR(DS23 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ23), DS23)</f>
       </c>
     </row>
     <row r="24">
@@ -10139,10 +10139,10 @@
         <f>=IFERROR(ROUND(J24/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L24" s="115" t="str">
-        <f>=IFERROR(J24 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I24), J24)</f>
+        <f>=IFERROR(J24 + SUMIFS($E$19:$E$26, $B$19:$B$26, I24), J24)</f>
       </c>
       <c r="M24" s="143" t="str">
-        <f>=IFERROR(K24 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I24), K24)</f>
+        <f>=IFERROR(K24 + SUMIFS($F$19:$F$26, $B$19:$B$26, I24), K24)</f>
       </c>
       <c r="P24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10152,10 +10152,10 @@
         <f>=IFERROR(ROUND(Q24/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S24" s="115" t="str">
-        <f>=IFERROR(Q24 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P24), Q24)</f>
+        <f>=IFERROR(Q24 + SUMIFS($L$19:$L$26, $I$19:$I$26, P24), Q24)</f>
       </c>
       <c r="T24" s="143" t="str">
-        <f>=IFERROR(R24 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P24), R24)</f>
+        <f>=IFERROR(R24 + SUMIFS($M$19:$M$26, $I$19:$I$26, P24), R24)</f>
       </c>
       <c r="W24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10165,10 +10165,10 @@
         <f>=IFERROR(ROUND(X24/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z24" s="115" t="str">
-        <f>=IFERROR(X24 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W24), X24)</f>
+        <f>=IFERROR(X24 + SUMIFS($S$19:$S$26, $P$19:$P$26, W24), X24)</f>
       </c>
       <c r="AA24" s="143" t="str">
-        <f>=IFERROR(Y24 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W24), Y24)</f>
+        <f>=IFERROR(Y24 + SUMIFS($T$19:$T$26, $P$19:$P$26, W24), Y24)</f>
       </c>
       <c r="AD24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10178,10 +10178,10 @@
         <f>=IFERROR(ROUND(AE24/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG24" s="115" t="str">
-        <f>=IFERROR(AE24 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD24), AE24)</f>
+        <f>=IFERROR(AE24 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD24), AE24)</f>
       </c>
       <c r="AH24" s="143" t="str">
-        <f>=IFERROR(AF24 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD24), AF24)</f>
+        <f>=IFERROR(AF24 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD24), AF24)</f>
       </c>
       <c r="AK24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10191,10 +10191,10 @@
         <f>=IFERROR(ROUND(AL24/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN24" s="115" t="str">
-        <f>=IFERROR(AL24 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK24), AL24)</f>
+        <f>=IFERROR(AL24 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK24), AL24)</f>
       </c>
       <c r="AO24" s="143" t="str">
-        <f>=IFERROR(AM24 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK24), AM24)</f>
+        <f>=IFERROR(AM24 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK24), AM24)</f>
       </c>
       <c r="AR24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10204,10 +10204,10 @@
         <f>=IFERROR(ROUND(AS24/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU24" s="115" t="str">
-        <f>=IFERROR(AS24 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR24), AS24)</f>
+        <f>=IFERROR(AS24 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR24), AS24)</f>
       </c>
       <c r="AV24" s="143" t="str">
-        <f>=IFERROR(AT24 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR24), AT24)</f>
+        <f>=IFERROR(AT24 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR24), AT24)</f>
       </c>
       <c r="AY24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10217,10 +10217,10 @@
         <f>=IFERROR(ROUND(AZ24/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB24" s="115" t="str">
-        <f>=IFERROR(AZ24 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY24), AZ24)</f>
+        <f>=IFERROR(AZ24 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY24), AZ24)</f>
       </c>
       <c r="BC24" s="143" t="str">
-        <f>=IFERROR(BA24 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY24), BA24)</f>
+        <f>=IFERROR(BA24 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY24), BA24)</f>
       </c>
       <c r="BF24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10230,10 +10230,10 @@
         <f>=IFERROR(ROUND(BG24/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI24" s="115" t="str">
-        <f>=IFERROR(BG24 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF24), BG24)</f>
+        <f>=IFERROR(BG24 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF24), BG24)</f>
       </c>
       <c r="BJ24" s="143" t="str">
-        <f>=IFERROR(BH24 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF24), BH24)</f>
+        <f>=IFERROR(BH24 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF24), BH24)</f>
       </c>
       <c r="BM24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10243,10 +10243,10 @@
         <f>=IFERROR(ROUND(BN24/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP24" s="115" t="str">
-        <f>=IFERROR(BN24 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM24), BN24)</f>
+        <f>=IFERROR(BN24 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM24), BN24)</f>
       </c>
       <c r="BQ24" s="143" t="str">
-        <f>=IFERROR(BO24 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM24), BO24)</f>
+        <f>=IFERROR(BO24 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM24), BO24)</f>
       </c>
       <c r="BT24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10256,10 +10256,10 @@
         <f>=IFERROR(ROUND(BU24/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW24" s="115" t="str">
-        <f>=IFERROR(BU24 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT24), BU24)</f>
+        <f>=IFERROR(BU24 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT24), BU24)</f>
       </c>
       <c r="BX24" s="143" t="str">
-        <f>=IFERROR(BV24 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT24), BV24)</f>
+        <f>=IFERROR(BV24 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT24), BV24)</f>
       </c>
       <c r="CA24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10269,10 +10269,10 @@
         <f>=IFERROR(ROUND(CB24/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD24" s="115" t="str">
-        <f>=IFERROR(CB24 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA24), CB24)</f>
+        <f>=IFERROR(CB24 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA24), CB24)</f>
       </c>
       <c r="CE24" s="143" t="str">
-        <f>=IFERROR(CC24 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA24), CC24)</f>
+        <f>=IFERROR(CC24 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA24), CC24)</f>
       </c>
       <c r="CH24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10282,10 +10282,10 @@
         <f>=IFERROR(ROUND(CI24/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK24" s="115" t="str">
-        <f>=IFERROR(CI24 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH24), CI24)</f>
+        <f>=IFERROR(CI24 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH24), CI24)</f>
       </c>
       <c r="CL24" s="143" t="str">
-        <f>=IFERROR(CJ24 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH24), CJ24)</f>
+        <f>=IFERROR(CJ24 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH24), CJ24)</f>
       </c>
       <c r="CO24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10295,10 +10295,10 @@
         <f>=IFERROR(ROUND(CP24/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR24" s="115" t="str">
-        <f>=IFERROR(CP24 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO24), CP24)</f>
+        <f>=IFERROR(CP24 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO24), CP24)</f>
       </c>
       <c r="CS24" s="143" t="str">
-        <f>=IFERROR(CQ24 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO24), CQ24)</f>
+        <f>=IFERROR(CQ24 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO24), CQ24)</f>
       </c>
       <c r="CV24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10308,10 +10308,10 @@
         <f>=IFERROR(ROUND(CW24/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY24" s="115" t="str">
-        <f>=IFERROR(CW24 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV24), CW24)</f>
+        <f>=IFERROR(CW24 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV24), CW24)</f>
       </c>
       <c r="CZ24" s="143" t="str">
-        <f>=IFERROR(CX24 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV24), CX24)</f>
+        <f>=IFERROR(CX24 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV24), CX24)</f>
       </c>
       <c r="DC24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10321,10 +10321,10 @@
         <f>=IFERROR(ROUND(DD24/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF24" s="115" t="str">
-        <f>=IFERROR(DD24 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC24), DD24)</f>
+        <f>=IFERROR(DD24 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC24), DD24)</f>
       </c>
       <c r="DG24" s="143" t="str">
-        <f>=IFERROR(DE24 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC24), DE24)</f>
+        <f>=IFERROR(DE24 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC24), DE24)</f>
       </c>
       <c r="DJ24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10334,10 +10334,10 @@
         <f>=IFERROR(ROUND(DK24/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM24" s="115" t="str">
-        <f>=IFERROR(DK24 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ24), DK24)</f>
+        <f>=IFERROR(DK24 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ24), DK24)</f>
       </c>
       <c r="DN24" s="143" t="str">
-        <f>=IFERROR(DL24 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ24), DL24)</f>
+        <f>=IFERROR(DL24 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ24), DL24)</f>
       </c>
       <c r="DQ24" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10347,10 +10347,10 @@
         <f>=IFERROR(ROUND(DR24/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT24" s="115" t="str">
-        <f>=IFERROR(DR24 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ24), DR24)</f>
+        <f>=IFERROR(DR24 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ24), DR24)</f>
       </c>
       <c r="DU24" s="143" t="str">
-        <f>=IFERROR(DS24 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ24), DS24)</f>
+        <f>=IFERROR(DS24 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ24), DS24)</f>
       </c>
     </row>
     <row r="25">
@@ -10375,10 +10375,10 @@
         <f>=IFERROR(ROUND(J25/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L25" s="115" t="str">
-        <f>=IFERROR(J25 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I25), J25)</f>
+        <f>=IFERROR(J25 + SUMIFS($E$19:$E$26, $B$19:$B$26, I25), J25)</f>
       </c>
       <c r="M25" s="143" t="str">
-        <f>=IFERROR(K25 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I25), K25)</f>
+        <f>=IFERROR(K25 + SUMIFS($F$19:$F$26, $B$19:$B$26, I25), K25)</f>
       </c>
       <c r="P25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10388,10 +10388,10 @@
         <f>=IFERROR(ROUND(Q25/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S25" s="115" t="str">
-        <f>=IFERROR(Q25 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P25), Q25)</f>
+        <f>=IFERROR(Q25 + SUMIFS($L$19:$L$26, $I$19:$I$26, P25), Q25)</f>
       </c>
       <c r="T25" s="143" t="str">
-        <f>=IFERROR(R25 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P25), R25)</f>
+        <f>=IFERROR(R25 + SUMIFS($M$19:$M$26, $I$19:$I$26, P25), R25)</f>
       </c>
       <c r="W25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10401,10 +10401,10 @@
         <f>=IFERROR(ROUND(X25/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z25" s="115" t="str">
-        <f>=IFERROR(X25 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W25), X25)</f>
+        <f>=IFERROR(X25 + SUMIFS($S$19:$S$26, $P$19:$P$26, W25), X25)</f>
       </c>
       <c r="AA25" s="143" t="str">
-        <f>=IFERROR(Y25 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W25), Y25)</f>
+        <f>=IFERROR(Y25 + SUMIFS($T$19:$T$26, $P$19:$P$26, W25), Y25)</f>
       </c>
       <c r="AD25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10414,10 +10414,10 @@
         <f>=IFERROR(ROUND(AE25/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG25" s="115" t="str">
-        <f>=IFERROR(AE25 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD25), AE25)</f>
+        <f>=IFERROR(AE25 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD25), AE25)</f>
       </c>
       <c r="AH25" s="143" t="str">
-        <f>=IFERROR(AF25 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD25), AF25)</f>
+        <f>=IFERROR(AF25 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD25), AF25)</f>
       </c>
       <c r="AK25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10427,10 +10427,10 @@
         <f>=IFERROR(ROUND(AL25/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN25" s="115" t="str">
-        <f>=IFERROR(AL25 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK25), AL25)</f>
+        <f>=IFERROR(AL25 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK25), AL25)</f>
       </c>
       <c r="AO25" s="143" t="str">
-        <f>=IFERROR(AM25 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK25), AM25)</f>
+        <f>=IFERROR(AM25 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK25), AM25)</f>
       </c>
       <c r="AR25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10440,10 +10440,10 @@
         <f>=IFERROR(ROUND(AS25/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU25" s="115" t="str">
-        <f>=IFERROR(AS25 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR25), AS25)</f>
+        <f>=IFERROR(AS25 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR25), AS25)</f>
       </c>
       <c r="AV25" s="143" t="str">
-        <f>=IFERROR(AT25 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR25), AT25)</f>
+        <f>=IFERROR(AT25 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR25), AT25)</f>
       </c>
       <c r="AY25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10453,10 +10453,10 @@
         <f>=IFERROR(ROUND(AZ25/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB25" s="115" t="str">
-        <f>=IFERROR(AZ25 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY25), AZ25)</f>
+        <f>=IFERROR(AZ25 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY25), AZ25)</f>
       </c>
       <c r="BC25" s="143" t="str">
-        <f>=IFERROR(BA25 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY25), BA25)</f>
+        <f>=IFERROR(BA25 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY25), BA25)</f>
       </c>
       <c r="BF25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10466,10 +10466,10 @@
         <f>=IFERROR(ROUND(BG25/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI25" s="115" t="str">
-        <f>=IFERROR(BG25 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF25), BG25)</f>
+        <f>=IFERROR(BG25 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF25), BG25)</f>
       </c>
       <c r="BJ25" s="143" t="str">
-        <f>=IFERROR(BH25 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF25), BH25)</f>
+        <f>=IFERROR(BH25 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF25), BH25)</f>
       </c>
       <c r="BM25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10479,10 +10479,10 @@
         <f>=IFERROR(ROUND(BN25/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP25" s="115" t="str">
-        <f>=IFERROR(BN25 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM25), BN25)</f>
+        <f>=IFERROR(BN25 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM25), BN25)</f>
       </c>
       <c r="BQ25" s="143" t="str">
-        <f>=IFERROR(BO25 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM25), BO25)</f>
+        <f>=IFERROR(BO25 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM25), BO25)</f>
       </c>
       <c r="BT25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10492,10 +10492,10 @@
         <f>=IFERROR(ROUND(BU25/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW25" s="115" t="str">
-        <f>=IFERROR(BU25 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT25), BU25)</f>
+        <f>=IFERROR(BU25 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT25), BU25)</f>
       </c>
       <c r="BX25" s="143" t="str">
-        <f>=IFERROR(BV25 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT25), BV25)</f>
+        <f>=IFERROR(BV25 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT25), BV25)</f>
       </c>
       <c r="CA25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10505,10 +10505,10 @@
         <f>=IFERROR(ROUND(CB25/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD25" s="115" t="str">
-        <f>=IFERROR(CB25 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA25), CB25)</f>
+        <f>=IFERROR(CB25 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA25), CB25)</f>
       </c>
       <c r="CE25" s="143" t="str">
-        <f>=IFERROR(CC25 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA25), CC25)</f>
+        <f>=IFERROR(CC25 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA25), CC25)</f>
       </c>
       <c r="CH25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10518,10 +10518,10 @@
         <f>=IFERROR(ROUND(CI25/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK25" s="115" t="str">
-        <f>=IFERROR(CI25 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH25), CI25)</f>
+        <f>=IFERROR(CI25 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH25), CI25)</f>
       </c>
       <c r="CL25" s="143" t="str">
-        <f>=IFERROR(CJ25 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH25), CJ25)</f>
+        <f>=IFERROR(CJ25 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH25), CJ25)</f>
       </c>
       <c r="CO25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10531,10 +10531,10 @@
         <f>=IFERROR(ROUND(CP25/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR25" s="115" t="str">
-        <f>=IFERROR(CP25 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO25), CP25)</f>
+        <f>=IFERROR(CP25 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO25), CP25)</f>
       </c>
       <c r="CS25" s="143" t="str">
-        <f>=IFERROR(CQ25 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO25), CQ25)</f>
+        <f>=IFERROR(CQ25 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO25), CQ25)</f>
       </c>
       <c r="CV25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10544,10 +10544,10 @@
         <f>=IFERROR(ROUND(CW25/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY25" s="115" t="str">
-        <f>=IFERROR(CW25 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV25), CW25)</f>
+        <f>=IFERROR(CW25 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV25), CW25)</f>
       </c>
       <c r="CZ25" s="143" t="str">
-        <f>=IFERROR(CX25 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV25), CX25)</f>
+        <f>=IFERROR(CX25 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV25), CX25)</f>
       </c>
       <c r="DC25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10557,10 +10557,10 @@
         <f>=IFERROR(ROUND(DD25/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF25" s="115" t="str">
-        <f>=IFERROR(DD25 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC25), DD25)</f>
+        <f>=IFERROR(DD25 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC25), DD25)</f>
       </c>
       <c r="DG25" s="143" t="str">
-        <f>=IFERROR(DE25 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC25), DE25)</f>
+        <f>=IFERROR(DE25 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC25), DE25)</f>
       </c>
       <c r="DJ25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10570,10 +10570,10 @@
         <f>=IFERROR(ROUND(DK25/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM25" s="115" t="str">
-        <f>=IFERROR(DK25 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ25), DK25)</f>
+        <f>=IFERROR(DK25 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ25), DK25)</f>
       </c>
       <c r="DN25" s="143" t="str">
-        <f>=IFERROR(DL25 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ25), DL25)</f>
+        <f>=IFERROR(DL25 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ25), DL25)</f>
       </c>
       <c r="DQ25" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10583,10 +10583,10 @@
         <f>=IFERROR(ROUND(DR25/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT25" s="115" t="str">
-        <f>=IFERROR(DR25 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ25), DR25)</f>
+        <f>=IFERROR(DR25 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ25), DR25)</f>
       </c>
       <c r="DU25" s="143" t="str">
-        <f>=IFERROR(DS25 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ25), DS25)</f>
+        <f>=IFERROR(DS25 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ25), DS25)</f>
       </c>
     </row>
     <row r="26">
@@ -10611,10 +10611,10 @@
         <f>=IFERROR(ROUND(J26/FB_Kurs_2,2),0)</f>
       </c>
       <c r="L26" s="115" t="str">
-        <f>=IFERROR(J26 + SUMIFS(Ausgaben_1[Kum. Ausgaben (LC)], Ausgaben_1[ID], I26), J26)</f>
+        <f>=IFERROR(J26 + SUMIFS($E$19:$E$26, $B$19:$B$26, I26), J26)</f>
       </c>
       <c r="M26" s="143" t="str">
-        <f>=IFERROR(K26 + SUMIFS(Ausgaben_1[Kum. Ausgaben (EUR)], Ausgaben_1[ID], I26), K26)</f>
+        <f>=IFERROR(K26 + SUMIFS($F$19:$F$26, $B$19:$B$26, I26), K26)</f>
       </c>
       <c r="P26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10624,10 +10624,10 @@
         <f>=IFERROR(ROUND(Q26/FB_Kurs_3,2),0)</f>
       </c>
       <c r="S26" s="115" t="str">
-        <f>=IFERROR(Q26 + SUMIFS(Ausgaben_2[Kum. Ausgaben (LC)], Ausgaben_2[ID], P26), Q26)</f>
+        <f>=IFERROR(Q26 + SUMIFS($L$19:$L$26, $I$19:$I$26, P26), Q26)</f>
       </c>
       <c r="T26" s="143" t="str">
-        <f>=IFERROR(R26 + SUMIFS(Ausgaben_2[Kum. Ausgaben (EUR)], Ausgaben_2[ID], P26), R26)</f>
+        <f>=IFERROR(R26 + SUMIFS($M$19:$M$26, $I$19:$I$26, P26), R26)</f>
       </c>
       <c r="W26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10637,10 +10637,10 @@
         <f>=IFERROR(ROUND(X26/FB_Kurs_4,2),0)</f>
       </c>
       <c r="Z26" s="115" t="str">
-        <f>=IFERROR(X26 + SUMIFS(Ausgaben_3[Kum. Ausgaben (LC)], Ausgaben_3[ID], W26), X26)</f>
+        <f>=IFERROR(X26 + SUMIFS($S$19:$S$26, $P$19:$P$26, W26), X26)</f>
       </c>
       <c r="AA26" s="143" t="str">
-        <f>=IFERROR(Y26 + SUMIFS(Ausgaben_3[Kum. Ausgaben (EUR)], Ausgaben_3[ID], W26), Y26)</f>
+        <f>=IFERROR(Y26 + SUMIFS($T$19:$T$26, $P$19:$P$26, W26), Y26)</f>
       </c>
       <c r="AD26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10650,10 +10650,10 @@
         <f>=IFERROR(ROUND(AE26/FB_Kurs_5,2),0)</f>
       </c>
       <c r="AG26" s="115" t="str">
-        <f>=IFERROR(AE26 + SUMIFS(Ausgaben_4[Kum. Ausgaben (LC)], Ausgaben_4[ID], AD26), AE26)</f>
+        <f>=IFERROR(AE26 + SUMIFS($Z$19:$Z$26, $W$19:$W$26, AD26), AE26)</f>
       </c>
       <c r="AH26" s="143" t="str">
-        <f>=IFERROR(AF26 + SUMIFS(Ausgaben_4[Kum. Ausgaben (EUR)], Ausgaben_4[ID], AD26), AF26)</f>
+        <f>=IFERROR(AF26 + SUMIFS($AA$19:$AA$26, $W$19:$W$26, AD26), AF26)</f>
       </c>
       <c r="AK26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10663,10 +10663,10 @@
         <f>=IFERROR(ROUND(AL26/FB_Kurs_6,2),0)</f>
       </c>
       <c r="AN26" s="115" t="str">
-        <f>=IFERROR(AL26 + SUMIFS(Ausgaben_5[Kum. Ausgaben (LC)], Ausgaben_5[ID], AK26), AL26)</f>
+        <f>=IFERROR(AL26 + SUMIFS($AG$19:$AG$26, $AD$19:$AD$26, AK26), AL26)</f>
       </c>
       <c r="AO26" s="143" t="str">
-        <f>=IFERROR(AM26 + SUMIFS(Ausgaben_5[Kum. Ausgaben (EUR)], Ausgaben_5[ID], AK26), AM26)</f>
+        <f>=IFERROR(AM26 + SUMIFS($AH$19:$AH$26, $AD$19:$AD$26, AK26), AM26)</f>
       </c>
       <c r="AR26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10676,10 +10676,10 @@
         <f>=IFERROR(ROUND(AS26/FB_Kurs_7,2),0)</f>
       </c>
       <c r="AU26" s="115" t="str">
-        <f>=IFERROR(AS26 + SUMIFS(Ausgaben_6[Kum. Ausgaben (LC)], Ausgaben_6[ID], AR26), AS26)</f>
+        <f>=IFERROR(AS26 + SUMIFS($AN$19:$AN$26, $AK$19:$AK$26, AR26), AS26)</f>
       </c>
       <c r="AV26" s="143" t="str">
-        <f>=IFERROR(AT26 + SUMIFS(Ausgaben_6[Kum. Ausgaben (EUR)], Ausgaben_6[ID], AR26), AT26)</f>
+        <f>=IFERROR(AT26 + SUMIFS($AO$19:$AO$26, $AK$19:$AK$26, AR26), AT26)</f>
       </c>
       <c r="AY26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10689,10 +10689,10 @@
         <f>=IFERROR(ROUND(AZ26/FB_Kurs_8,2),0)</f>
       </c>
       <c r="BB26" s="115" t="str">
-        <f>=IFERROR(AZ26 + SUMIFS(Ausgaben_7[Kum. Ausgaben (LC)], Ausgaben_7[ID], AY26), AZ26)</f>
+        <f>=IFERROR(AZ26 + SUMIFS($AU$19:$AU$26, $AR$19:$AR$26, AY26), AZ26)</f>
       </c>
       <c r="BC26" s="143" t="str">
-        <f>=IFERROR(BA26 + SUMIFS(Ausgaben_7[Kum. Ausgaben (EUR)], Ausgaben_7[ID], AY26), BA26)</f>
+        <f>=IFERROR(BA26 + SUMIFS($AV$19:$AV$26, $AR$19:$AR$26, AY26), BA26)</f>
       </c>
       <c r="BF26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10702,10 +10702,10 @@
         <f>=IFERROR(ROUND(BG26/FB_Kurs_9,2),0)</f>
       </c>
       <c r="BI26" s="115" t="str">
-        <f>=IFERROR(BG26 + SUMIFS(Ausgaben_8[Kum. Ausgaben (LC)], Ausgaben_8[ID], BF26), BG26)</f>
+        <f>=IFERROR(BG26 + SUMIFS($BB$19:$BB$26, $AY$19:$AY$26, BF26), BG26)</f>
       </c>
       <c r="BJ26" s="143" t="str">
-        <f>=IFERROR(BH26 + SUMIFS(Ausgaben_8[Kum. Ausgaben (EUR)], Ausgaben_8[ID], BF26), BH26)</f>
+        <f>=IFERROR(BH26 + SUMIFS($BC$19:$BC$26, $AY$19:$AY$26, BF26), BH26)</f>
       </c>
       <c r="BM26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10715,10 +10715,10 @@
         <f>=IFERROR(ROUND(BN26/FB_Kurs_10,2),0)</f>
       </c>
       <c r="BP26" s="115" t="str">
-        <f>=IFERROR(BN26 + SUMIFS(Ausgaben_9[Kum. Ausgaben (LC)], Ausgaben_9[ID], BM26), BN26)</f>
+        <f>=IFERROR(BN26 + SUMIFS($BI$19:$BI$26, $BF$19:$BF$26, BM26), BN26)</f>
       </c>
       <c r="BQ26" s="143" t="str">
-        <f>=IFERROR(BO26 + SUMIFS(Ausgaben_9[Kum. Ausgaben (EUR)], Ausgaben_9[ID], BM26), BO26)</f>
+        <f>=IFERROR(BO26 + SUMIFS($BJ$19:$BJ$26, $BF$19:$BF$26, BM26), BO26)</f>
       </c>
       <c r="BT26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10728,10 +10728,10 @@
         <f>=IFERROR(ROUND(BU26/FB_Kurs_11,2),0)</f>
       </c>
       <c r="BW26" s="115" t="str">
-        <f>=IFERROR(BU26 + SUMIFS(Ausgaben_10[Kum. Ausgaben (LC)], Ausgaben_10[ID], BT26), BU26)</f>
+        <f>=IFERROR(BU26 + SUMIFS($BP$19:$BP$26, $BM$19:$BM$26, BT26), BU26)</f>
       </c>
       <c r="BX26" s="143" t="str">
-        <f>=IFERROR(BV26 + SUMIFS(Ausgaben_10[Kum. Ausgaben (EUR)], Ausgaben_10[ID], BT26), BV26)</f>
+        <f>=IFERROR(BV26 + SUMIFS($BQ$19:$BQ$26, $BM$19:$BM$26, BT26), BV26)</f>
       </c>
       <c r="CA26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10741,10 +10741,10 @@
         <f>=IFERROR(ROUND(CB26/FB_Kurs_12,2),0)</f>
       </c>
       <c r="CD26" s="115" t="str">
-        <f>=IFERROR(CB26 + SUMIFS(Ausgaben_11[Kum. Ausgaben (LC)], Ausgaben_11[ID], CA26), CB26)</f>
+        <f>=IFERROR(CB26 + SUMIFS($BW$19:$BW$26, $BT$19:$BT$26, CA26), CB26)</f>
       </c>
       <c r="CE26" s="143" t="str">
-        <f>=IFERROR(CC26 + SUMIFS(Ausgaben_11[Kum. Ausgaben (EUR)], Ausgaben_11[ID], CA26), CC26)</f>
+        <f>=IFERROR(CC26 + SUMIFS($BX$19:$BX$26, $BT$19:$BT$26, CA26), CC26)</f>
       </c>
       <c r="CH26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10754,10 +10754,10 @@
         <f>=IFERROR(ROUND(CI26/FB_Kurs_13,2),0)</f>
       </c>
       <c r="CK26" s="115" t="str">
-        <f>=IFERROR(CI26 + SUMIFS(Ausgaben_12[Kum. Ausgaben (LC)], Ausgaben_12[ID], CH26), CI26)</f>
+        <f>=IFERROR(CI26 + SUMIFS($CD$19:$CD$26, $CA$19:$CA$26, CH26), CI26)</f>
       </c>
       <c r="CL26" s="143" t="str">
-        <f>=IFERROR(CJ26 + SUMIFS(Ausgaben_12[Kum. Ausgaben (EUR)], Ausgaben_12[ID], CH26), CJ26)</f>
+        <f>=IFERROR(CJ26 + SUMIFS($CE$19:$CE$26, $CA$19:$CA$26, CH26), CJ26)</f>
       </c>
       <c r="CO26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10767,10 +10767,10 @@
         <f>=IFERROR(ROUND(CP26/FB_Kurs_14,2),0)</f>
       </c>
       <c r="CR26" s="115" t="str">
-        <f>=IFERROR(CP26 + SUMIFS(Ausgaben_13[Kum. Ausgaben (LC)], Ausgaben_13[ID], CO26), CP26)</f>
+        <f>=IFERROR(CP26 + SUMIFS($CK$19:$CK$26, $CH$19:$CH$26, CO26), CP26)</f>
       </c>
       <c r="CS26" s="143" t="str">
-        <f>=IFERROR(CQ26 + SUMIFS(Ausgaben_13[Kum. Ausgaben (EUR)], Ausgaben_13[ID], CO26), CQ26)</f>
+        <f>=IFERROR(CQ26 + SUMIFS($CL$19:$CL$26, $CH$19:$CH$26, CO26), CQ26)</f>
       </c>
       <c r="CV26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10780,10 +10780,10 @@
         <f>=IFERROR(ROUND(CW26/FB_Kurs_15,2),0)</f>
       </c>
       <c r="CY26" s="115" t="str">
-        <f>=IFERROR(CW26 + SUMIFS(Ausgaben_14[Kum. Ausgaben (LC)], Ausgaben_14[ID], CV26), CW26)</f>
+        <f>=IFERROR(CW26 + SUMIFS($CR$19:$CR$26, $CO$19:$CO$26, CV26), CW26)</f>
       </c>
       <c r="CZ26" s="143" t="str">
-        <f>=IFERROR(CX26 + SUMIFS(Ausgaben_14[Kum. Ausgaben (EUR)], Ausgaben_14[ID], CV26), CX26)</f>
+        <f>=IFERROR(CX26 + SUMIFS($CS$19:$CS$26, $CO$19:$CO$26, CV26), CX26)</f>
       </c>
       <c r="DC26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10793,10 +10793,10 @@
         <f>=IFERROR(ROUND(DD26/FB_Kurs_16,2),0)</f>
       </c>
       <c r="DF26" s="115" t="str">
-        <f>=IFERROR(DD26 + SUMIFS(Ausgaben_15[Kum. Ausgaben (LC)], Ausgaben_15[ID], DC26), DD26)</f>
+        <f>=IFERROR(DD26 + SUMIFS($CY$19:$CY$26, $CV$19:$CV$26, DC26), DD26)</f>
       </c>
       <c r="DG26" s="143" t="str">
-        <f>=IFERROR(DE26 + SUMIFS(Ausgaben_15[Kum. Ausgaben (EUR)], Ausgaben_15[ID], DC26), DE26)</f>
+        <f>=IFERROR(DE26 + SUMIFS($CZ$19:$CZ$26, $CV$19:$CV$26, DC26), DE26)</f>
       </c>
       <c r="DJ26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10806,10 +10806,10 @@
         <f>=IFERROR(ROUND(DK26/FB_Kurs_17,2),0)</f>
       </c>
       <c r="DM26" s="115" t="str">
-        <f>=IFERROR(DK26 + SUMIFS(Ausgaben_16[Kum. Ausgaben (LC)], Ausgaben_16[ID], DJ26), DK26)</f>
+        <f>=IFERROR(DK26 + SUMIFS($DF$19:$DF$26, $DC$19:$DC$26, DJ26), DK26)</f>
       </c>
       <c r="DN26" s="143" t="str">
-        <f>=IFERROR(DL26 + SUMIFS(Ausgaben_16[Kum. Ausgaben (EUR)], Ausgaben_16[ID], DJ26), DL26)</f>
+        <f>=IFERROR(DL26 + SUMIFS($DG$19:$DG$26, $DC$19:$DC$26, DJ26), DL26)</f>
       </c>
       <c r="DQ26" s="148" t="str">
         <f>=IFERROR(INDEX(Budget_ID_Liste, ROW() - 18), "")</f>
@@ -10819,10 +10819,10 @@
         <f>=IFERROR(ROUND(DR26/FB_Kurs_18,2),0)</f>
       </c>
       <c r="DT26" s="115" t="str">
-        <f>=IFERROR(DR26 + SUMIFS(Ausgaben_17[Kum. Ausgaben (LC)], Ausgaben_17[ID], DQ26), DR26)</f>
+        <f>=IFERROR(DR26 + SUMIFS($DM$19:$DM$26, $DJ$19:$DJ$26, DQ26), DR26)</f>
       </c>
       <c r="DU26" s="143" t="str">
-        <f>=IFERROR(DS26 + SUMIFS(Ausgaben_17[Kum. Ausgaben (EUR)], Ausgaben_17[ID], DQ26), DS26)</f>
+        <f>=IFERROR(DS26 + SUMIFS($DN$19:$DN$26, $DJ$19:$DJ$26, DQ26), DS26)</f>
       </c>
     </row>
     <row r="27">
@@ -10830,271 +10830,271 @@
         <v>285</v>
       </c>
       <c r="C27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_1[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$C$19:$C$26),2)</f>
       </c>
       <c r="D27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_1[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$D$19:$D$26),2)</f>
       </c>
       <c r="E27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_1[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$E$19:$E$26),2)</f>
       </c>
       <c r="F27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_1[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$F$19:$F$26),2)</f>
       </c>
       <c r="I27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="J27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_2[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$J$19:$J$26),2)</f>
       </c>
       <c r="K27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_2[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$K$19:$K$26),2)</f>
       </c>
       <c r="L27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_2[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$L$19:$L$26),2)</f>
       </c>
       <c r="M27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_2[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$M$19:$M$26),2)</f>
       </c>
       <c r="P27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="Q27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_3[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$Q$19:$Q$26),2)</f>
       </c>
       <c r="R27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_3[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$R$19:$R$26),2)</f>
       </c>
       <c r="S27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_3[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$S$19:$S$26),2)</f>
       </c>
       <c r="T27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_3[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$T$19:$T$26),2)</f>
       </c>
       <c r="W27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="X27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_4[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$X$19:$X$26),2)</f>
       </c>
       <c r="Y27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_4[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$Y$19:$Y$26),2)</f>
       </c>
       <c r="Z27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_4[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$Z$19:$Z$26),2)</f>
       </c>
       <c r="AA27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_4[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AA$19:$AA$26),2)</f>
       </c>
       <c r="AD27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="AE27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_5[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AE$19:$AE$26),2)</f>
       </c>
       <c r="AF27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_5[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AF$19:$AF$26),2)</f>
       </c>
       <c r="AG27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_5[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AG$19:$AG$26),2)</f>
       </c>
       <c r="AH27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_5[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AH$19:$AH$26),2)</f>
       </c>
       <c r="AK27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="AL27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_6[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AL$19:$AL$26),2)</f>
       </c>
       <c r="AM27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_6[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AM$19:$AM$26),2)</f>
       </c>
       <c r="AN27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_6[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AN$19:$AN$26),2)</f>
       </c>
       <c r="AO27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_6[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AO$19:$AO$26),2)</f>
       </c>
       <c r="AR27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="AS27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_7[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AS$19:$AS$26),2)</f>
       </c>
       <c r="AT27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_7[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AT$19:$AT$26),2)</f>
       </c>
       <c r="AU27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_7[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AU$19:$AU$26),2)</f>
       </c>
       <c r="AV27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_7[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AV$19:$AV$26),2)</f>
       </c>
       <c r="AY27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="AZ27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_8[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AZ$19:$AZ$26),2)</f>
       </c>
       <c r="BA27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_8[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BA$19:$BA$26),2)</f>
       </c>
       <c r="BB27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_8[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BB$19:$BB$26),2)</f>
       </c>
       <c r="BC27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_8[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BC$19:$BC$26),2)</f>
       </c>
       <c r="BF27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="BG27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_9[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BG$19:$BG$26),2)</f>
       </c>
       <c r="BH27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_9[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BH$19:$BH$26),2)</f>
       </c>
       <c r="BI27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_9[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BI$19:$BI$26),2)</f>
       </c>
       <c r="BJ27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_9[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BJ$19:$BJ$26),2)</f>
       </c>
       <c r="BM27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="BN27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_10[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BN$19:$BN$26),2)</f>
       </c>
       <c r="BO27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_10[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BO$19:$BO$26),2)</f>
       </c>
       <c r="BP27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_10[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BP$19:$BP$26),2)</f>
       </c>
       <c r="BQ27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_10[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BQ$19:$BQ$26),2)</f>
       </c>
       <c r="BT27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="BU27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_11[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BU$19:$BU$26),2)</f>
       </c>
       <c r="BV27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_11[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BV$19:$BV$26),2)</f>
       </c>
       <c r="BW27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_11[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BW$19:$BW$26),2)</f>
       </c>
       <c r="BX27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_11[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BX$19:$BX$26),2)</f>
       </c>
       <c r="CA27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="CB27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_12[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CB$19:$CB$26),2)</f>
       </c>
       <c r="CC27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_12[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CC$19:$CC$26),2)</f>
       </c>
       <c r="CD27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_12[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CD$19:$CD$26),2)</f>
       </c>
       <c r="CE27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_12[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CE$19:$CE$26),2)</f>
       </c>
       <c r="CH27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="CI27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_13[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CI$19:$CI$26),2)</f>
       </c>
       <c r="CJ27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_13[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CJ$19:$CJ$26),2)</f>
       </c>
       <c r="CK27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_13[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CK$19:$CK$26),2)</f>
       </c>
       <c r="CL27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_13[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CL$19:$CL$26),2)</f>
       </c>
       <c r="CO27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="CP27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_14[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CP$19:$CP$26),2)</f>
       </c>
       <c r="CQ27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_14[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CQ$19:$CQ$26),2)</f>
       </c>
       <c r="CR27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_14[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CR$19:$CR$26),2)</f>
       </c>
       <c r="CS27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_14[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CS$19:$CS$26),2)</f>
       </c>
       <c r="CV27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="CW27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_15[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CW$19:$CW$26),2)</f>
       </c>
       <c r="CX27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_15[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CX$19:$CX$26),2)</f>
       </c>
       <c r="CY27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_15[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CY$19:$CY$26),2)</f>
       </c>
       <c r="CZ27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_15[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CZ$19:$CZ$26),2)</f>
       </c>
       <c r="DC27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="DD27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_16[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DD$19:$DD$26),2)</f>
       </c>
       <c r="DE27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_16[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DE$19:$DE$26),2)</f>
       </c>
       <c r="DF27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_16[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DF$19:$DF$26),2)</f>
       </c>
       <c r="DG27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_16[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DG$19:$DG$26),2)</f>
       </c>
       <c r="DJ27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="DK27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_17[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DK$19:$DK$26),2)</f>
       </c>
       <c r="DL27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_17[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DL$19:$DL$26),2)</f>
       </c>
       <c r="DM27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_17[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DM$19:$DM$26),2)</f>
       </c>
       <c r="DN27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_17[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DN$19:$DN$26),2)</f>
       </c>
       <c r="DQ27" s="149" t="s">
         <v>285</v>
       </c>
       <c r="DR27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_18[Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DR$19:$DR$26),2)</f>
       </c>
       <c r="DS27" s="124" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_18[Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DS$19:$DS$26),2)</f>
       </c>
       <c r="DT27" s="123" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_18[Kum. Ausgaben (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DT$19:$DT$26),2)</f>
       </c>
       <c r="DU27" s="150" t="str">
-        <f>=ROUND(SUBTOTAL(109,Ausgaben_18[Kum. Ausgaben (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DU$19:$DU$26),2)</f>
       </c>
     </row>
     <row r="28">
@@ -13603,10 +13603,10 @@
         <v>269</v>
       </c>
       <c r="D46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$D$41:$D$45),2)</f>
       </c>
       <c r="E46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$E$41:$E$45),2)</f>
       </c>
       <c r="F46" s="173" t="str">
         <f>=ROUND(IFERROR(D46/E46,0),6)</f>
@@ -13618,10 +13618,10 @@
         <v>269</v>
       </c>
       <c r="K46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_2[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$K$41:$K$45),2)</f>
       </c>
       <c r="L46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_2[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$L$41:$L$45),2)</f>
       </c>
       <c r="M46" s="173" t="str">
         <f>=ROUND(IFERROR(K46/L46,0),6)</f>
@@ -13633,10 +13633,10 @@
         <v>269</v>
       </c>
       <c r="R46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_3[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$R$41:$R$45),2)</f>
       </c>
       <c r="S46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_3[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$S$41:$S$45),2)</f>
       </c>
       <c r="T46" s="173" t="str">
         <f>=ROUND(IFERROR(R46/S46,0),6)</f>
@@ -13648,10 +13648,10 @@
         <v>269</v>
       </c>
       <c r="Y46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_4[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$Y$41:$Y$45),2)</f>
       </c>
       <c r="Z46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_4[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$Z$41:$Z$45),2)</f>
       </c>
       <c r="AA46" s="173" t="str">
         <f>=ROUND(IFERROR(Y46/Z46,0),6)</f>
@@ -13663,10 +13663,10 @@
         <v>269</v>
       </c>
       <c r="AF46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_5[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AF$41:$AF$45),2)</f>
       </c>
       <c r="AG46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_5[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AG$41:$AG$45),2)</f>
       </c>
       <c r="AH46" s="173" t="str">
         <f>=ROUND(IFERROR(AF46/AG46,0),6)</f>
@@ -13678,10 +13678,10 @@
         <v>269</v>
       </c>
       <c r="AM46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_6[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AM$41:$AM$45),2)</f>
       </c>
       <c r="AN46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_6[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AN$41:$AN$45),2)</f>
       </c>
       <c r="AO46" s="173" t="str">
         <f>=ROUND(IFERROR(AM46/AN46,0),6)</f>
@@ -13693,10 +13693,10 @@
         <v>269</v>
       </c>
       <c r="AT46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_7[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AT$41:$AT$45),2)</f>
       </c>
       <c r="AU46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_7[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AU$41:$AU$45),2)</f>
       </c>
       <c r="AV46" s="173" t="str">
         <f>=ROUND(IFERROR(AT46/AU46,0),6)</f>
@@ -13708,10 +13708,10 @@
         <v>269</v>
       </c>
       <c r="BA46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_8[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BA$41:$BA$45),2)</f>
       </c>
       <c r="BB46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_8[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BB$41:$BB$45),2)</f>
       </c>
       <c r="BC46" s="173" t="str">
         <f>=ROUND(IFERROR(BA46/BB46,0),6)</f>
@@ -13723,10 +13723,10 @@
         <v>269</v>
       </c>
       <c r="BH46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_9[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BH$41:$BH$45),2)</f>
       </c>
       <c r="BI46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_9[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BI$41:$BI$45),2)</f>
       </c>
       <c r="BJ46" s="173" t="str">
         <f>=ROUND(IFERROR(BH46/BI46,0),6)</f>
@@ -13738,10 +13738,10 @@
         <v>269</v>
       </c>
       <c r="BO46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_10[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BO$41:$BO$45),2)</f>
       </c>
       <c r="BP46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_10[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BP$41:$BP$45),2)</f>
       </c>
       <c r="BQ46" s="173" t="str">
         <f>=ROUND(IFERROR(BO46/BP46,0),6)</f>
@@ -13753,10 +13753,10 @@
         <v>269</v>
       </c>
       <c r="BV46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_11[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BV$41:$BV$45),2)</f>
       </c>
       <c r="BW46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_11[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BW$41:$BW$45),2)</f>
       </c>
       <c r="BX46" s="173" t="str">
         <f>=ROUND(IFERROR(BV46/BW46,0),6)</f>
@@ -13768,10 +13768,10 @@
         <v>269</v>
       </c>
       <c r="CC46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_12[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CC$41:$CC$45),2)</f>
       </c>
       <c r="CD46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_12[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CD$41:$CD$45),2)</f>
       </c>
       <c r="CE46" s="173" t="str">
         <f>=ROUND(IFERROR(CC46/CD46,0),6)</f>
@@ -13783,10 +13783,10 @@
         <v>269</v>
       </c>
       <c r="CJ46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_13[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CJ$41:$CJ$45),2)</f>
       </c>
       <c r="CK46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_13[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CK$41:$CK$45),2)</f>
       </c>
       <c r="CL46" s="173" t="str">
         <f>=ROUND(IFERROR(CJ46/CK46,0),6)</f>
@@ -13798,10 +13798,10 @@
         <v>269</v>
       </c>
       <c r="CQ46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_14[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CQ$41:$CQ$45),2)</f>
       </c>
       <c r="CR46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_14[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CR$41:$CR$45),2)</f>
       </c>
       <c r="CS46" s="173" t="str">
         <f>=ROUND(IFERROR(CQ46/CR46,0),6)</f>
@@ -13813,10 +13813,10 @@
         <v>269</v>
       </c>
       <c r="CX46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_15[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CX$41:$CX$45),2)</f>
       </c>
       <c r="CY46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_15[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CY$41:$CY$45),2)</f>
       </c>
       <c r="CZ46" s="173" t="str">
         <f>=ROUND(IFERROR(CX46/CY46,0),6)</f>
@@ -13828,10 +13828,10 @@
         <v>269</v>
       </c>
       <c r="DE46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_16[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DE$41:$DE$45),2)</f>
       </c>
       <c r="DF46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_16[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DF$41:$DF$45),2)</f>
       </c>
       <c r="DG46" s="173" t="str">
         <f>=ROUND(IFERROR(DE46/DF46,0),6)</f>
@@ -13843,10 +13843,10 @@
         <v>269</v>
       </c>
       <c r="DL46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_17[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DL$41:$DL$45),2)</f>
       </c>
       <c r="DM46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_17[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DM$41:$DM$45),2)</f>
       </c>
       <c r="DN46" s="173" t="str">
         <f>=ROUND(IFERROR(DL46/DM46,0),6)</f>
@@ -13858,10 +13858,10 @@
         <v>269</v>
       </c>
       <c r="DS46" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_18[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DS$41:$DS$45),2)</f>
       </c>
       <c r="DT46" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_18[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DT$41:$DT$45),2)</f>
       </c>
       <c r="DU46" s="173" t="str">
         <f>=ROUND(IFERROR(DS46/DT46,0),6)</f>
@@ -15619,10 +15619,10 @@
         <v>269</v>
       </c>
       <c r="D56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_1[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$D$50:$D$55),2)</f>
       </c>
       <c r="E56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_1[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$E$50:$E$55),2)</f>
       </c>
       <c r="F56" s="173" t="str">
         <f>=ROUND(IFERROR(D56/E56,0),6)</f>
@@ -15634,10 +15634,10 @@
         <v>269</v>
       </c>
       <c r="K56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_2[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$K$50:$K$55),2)</f>
       </c>
       <c r="L56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_2[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$L$50:$L$55),2)</f>
       </c>
       <c r="M56" s="173" t="str">
         <f>=ROUND(IFERROR(K56/L56,0),6)</f>
@@ -15649,10 +15649,10 @@
         <v>269</v>
       </c>
       <c r="R56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_3[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$R$50:$R$55),2)</f>
       </c>
       <c r="S56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_3[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$S$50:$S$55),2)</f>
       </c>
       <c r="T56" s="173" t="str">
         <f>=ROUND(IFERROR(R56/S56,0),6)</f>
@@ -15664,10 +15664,10 @@
         <v>269</v>
       </c>
       <c r="Y56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_4[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$Y$50:$Y$55),2)</f>
       </c>
       <c r="Z56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_4[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$Z$50:$Z$55),2)</f>
       </c>
       <c r="AA56" s="173" t="str">
         <f>=ROUND(IFERROR(Y56/Z56,0),6)</f>
@@ -15679,10 +15679,10 @@
         <v>269</v>
       </c>
       <c r="AF56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_5[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AF$50:$AF$55),2)</f>
       </c>
       <c r="AG56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_5[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AG$50:$AG$55),2)</f>
       </c>
       <c r="AH56" s="173" t="str">
         <f>=ROUND(IFERROR(AF56/AG56,0),6)</f>
@@ -15694,10 +15694,10 @@
         <v>269</v>
       </c>
       <c r="AM56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_6[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AM$50:$AM$55),2)</f>
       </c>
       <c r="AN56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_6[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AN$50:$AN$55),2)</f>
       </c>
       <c r="AO56" s="173" t="str">
         <f>=ROUND(IFERROR(AM56/AN56,0),6)</f>
@@ -15709,10 +15709,10 @@
         <v>269</v>
       </c>
       <c r="AT56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_7[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AT$50:$AT$55),2)</f>
       </c>
       <c r="AU56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_7[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$AU$50:$AU$55),2)</f>
       </c>
       <c r="AV56" s="173" t="str">
         <f>=ROUND(IFERROR(AT56/AU56,0),6)</f>
@@ -15724,10 +15724,10 @@
         <v>269</v>
       </c>
       <c r="BA56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_8[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BA$50:$BA$55),2)</f>
       </c>
       <c r="BB56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_8[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BB$50:$BB$55),2)</f>
       </c>
       <c r="BC56" s="173" t="str">
         <f>=ROUND(IFERROR(BA56/BB56,0),6)</f>
@@ -15739,10 +15739,10 @@
         <v>269</v>
       </c>
       <c r="BH56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_9[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BH$50:$BH$55),2)</f>
       </c>
       <c r="BI56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_9[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BI$50:$BI$55),2)</f>
       </c>
       <c r="BJ56" s="173" t="str">
         <f>=ROUND(IFERROR(BH56/BI56,0),6)</f>
@@ -15754,10 +15754,10 @@
         <v>269</v>
       </c>
       <c r="BO56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_10[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BO$50:$BO$55),2)</f>
       </c>
       <c r="BP56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_10[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BP$50:$BP$55),2)</f>
       </c>
       <c r="BQ56" s="173" t="str">
         <f>=ROUND(IFERROR(BO56/BP56,0),6)</f>
@@ -15769,10 +15769,10 @@
         <v>269</v>
       </c>
       <c r="BV56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_11[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BV$50:$BV$55),2)</f>
       </c>
       <c r="BW56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_11[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$BW$50:$BW$55),2)</f>
       </c>
       <c r="BX56" s="173" t="str">
         <f>=ROUND(IFERROR(BV56/BW56,0),6)</f>
@@ -15784,10 +15784,10 @@
         <v>269</v>
       </c>
       <c r="CC56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_12[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CC$50:$CC$55),2)</f>
       </c>
       <c r="CD56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_12[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CD$50:$CD$55),2)</f>
       </c>
       <c r="CE56" s="173" t="str">
         <f>=ROUND(IFERROR(CC56/CD56,0),6)</f>
@@ -15799,10 +15799,10 @@
         <v>269</v>
       </c>
       <c r="CJ56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_13[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CJ$50:$CJ$55),2)</f>
       </c>
       <c r="CK56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_13[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CK$50:$CK$55),2)</f>
       </c>
       <c r="CL56" s="173" t="str">
         <f>=ROUND(IFERROR(CJ56/CK56,0),6)</f>
@@ -15814,10 +15814,10 @@
         <v>269</v>
       </c>
       <c r="CQ56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_14[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CQ$50:$CQ$55),2)</f>
       </c>
       <c r="CR56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_14[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CR$50:$CR$55),2)</f>
       </c>
       <c r="CS56" s="173" t="str">
         <f>=ROUND(IFERROR(CQ56/CR56,0),6)</f>
@@ -15829,10 +15829,10 @@
         <v>269</v>
       </c>
       <c r="CX56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_15[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CX$50:$CX$55),2)</f>
       </c>
       <c r="CY56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_15[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$CY$50:$CY$55),2)</f>
       </c>
       <c r="CZ56" s="173" t="str">
         <f>=ROUND(IFERROR(CX56/CY56,0),6)</f>
@@ -15844,10 +15844,10 @@
         <v>269</v>
       </c>
       <c r="DE56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_16[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DE$50:$DE$55),2)</f>
       </c>
       <c r="DF56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_16[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DF$50:$DF$55),2)</f>
       </c>
       <c r="DG56" s="173" t="str">
         <f>=ROUND(IFERROR(DE56/DF56,0),6)</f>
@@ -15859,10 +15859,10 @@
         <v>269</v>
       </c>
       <c r="DL56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_17[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DL$50:$DL$55),2)</f>
       </c>
       <c r="DM56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_17[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DM$50:$DM$55),2)</f>
       </c>
       <c r="DN56" s="173" t="str">
         <f>=ROUND(IFERROR(DL56/DM56,0),6)</f>
@@ -15874,10 +15874,10 @@
         <v>269</v>
       </c>
       <c r="DS56" s="171" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_18[Einnahmen (LC)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DS$50:$DS$55),2)</f>
       </c>
       <c r="DT56" s="172" t="str">
-        <f>=ROUND(SUBTOTAL(109,Einnahmen_WK_18[Einnahmen (EUR)]),2)</f>
+        <f>=ROUND(SUBTOTAL(109,$DT$50:$DT$55),2)</f>
       </c>
       <c r="DU56" s="173" t="str">
         <f>=ROUND(IFERROR(DS56/DT56,0),6)</f>

</xml_diff>

<commit_message>
feat: add hidden Daten sheet for VSTACK consolidations
Implemented a new hidden sheet to centralize range references for VSTACK
formulas and period dropdowns. Updated Einnahmen, Ausgaben, and
Mittelanforderung generation to track their data ranges for use in
this centralized sheet.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -12,6 +12,7 @@
     <sheet name="II. KMW-Mittel" sheetId="4" r:id="rId7"/>
     <sheet name="III. Finanzberichte" sheetId="5" r:id="rId8"/>
     <sheet name="IV. MA" sheetId="6" r:id="rId9"/>
+    <sheet name="Daten" sheetId="7" r:id="rId10" state="hidden"/>
   </sheets>
   <definedNames>
     <definedName name="Saldovortrag_LW">'Dashboard'!$C$13</definedName>
@@ -124,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="319">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1069,6 +1070,18 @@
   </si>
   <si>
     <t>abzueglich Saldo Vorperiode (FB):</t>
+  </si>
+  <si>
+    <t>Einnahmen_Explizit_Stack</t>
+  </si>
+  <si>
+    <t>Einnahmen_Durchschnittskurs_Stack</t>
+  </si>
+  <si>
+    <t>Ausgaben_Finanzbericht_Stack</t>
+  </si>
+  <si>
+    <t>Mittelanforderung_Stack</t>
   </si>
 </sst>
 </file>
@@ -1836,7 +1849,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="191">
+  <cellXfs count="192">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
@@ -2407,6 +2420,9 @@
     </xf>
     <xf numFmtId="167" fontId="20" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -16387,7 +16403,6 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" hidden="true" max="1" min="1" width="9.140625"/>
     <col customWidth="true" max="2" min="2" width="25"/>
     <col customWidth="true" max="4" min="3" width="18"/>
     <col customWidth="true" max="6" min="6" width="25"/>
@@ -16426,20 +16441,7 @@
     <col customWidth="true" max="72" min="71" width="18"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>227</v>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" t="s">
-        <v>228</v>
-      </c>
       <c r="E3" s="175" t="s">
         <v>302</v>
       </c>
@@ -16492,15 +16494,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>229</v>
-      </c>
-    </row>
     <row r="5">
-      <c r="A5" t="s">
-        <v>230</v>
-      </c>
       <c r="B5" s="104" t="s">
         <v>267</v>
       </c>
@@ -16629,9 +16623,6 @@
       <c r="BT5" s="176"/>
     </row>
     <row r="6">
-      <c r="A6" t="s">
-        <v>231</v>
-      </c>
       <c r="B6" s="104" t="s">
         <v>268</v>
       </c>
@@ -16724,9 +16715,6 @@
       <c r="BT6" s="177"/>
     </row>
     <row r="7">
-      <c r="A7" t="s">
-        <v>232</v>
-      </c>
       <c r="B7" s="104" t="s">
         <v>305</v>
       </c>
@@ -16818,15 +16806,7 @@
       <c r="BS7" s="178"/>
       <c r="BT7" s="178"/>
     </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>233</v>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" t="s">
-        <v>234</v>
-      </c>
       <c r="B9" s="179" t="s">
         <v>202</v>
       </c>
@@ -16991,9 +16971,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s">
-        <v>235</v>
-      </c>
       <c r="B10" s="180" t="s">
         <v>205</v>
       </c>
@@ -17122,9 +17099,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s">
-        <v>236</v>
-      </c>
       <c r="B11" s="180" t="s">
         <v>206</v>
       </c>
@@ -17253,9 +17227,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s">
-        <v>237</v>
-      </c>
       <c r="B12" s="180" t="s">
         <v>207</v>
       </c>
@@ -17384,9 +17355,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s">
-        <v>238</v>
-      </c>
       <c r="B13" s="180" t="s">
         <v>208</v>
       </c>
@@ -17515,9 +17483,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s">
-        <v>239</v>
-      </c>
       <c r="B14" s="180" t="s">
         <v>209</v>
       </c>
@@ -17646,9 +17611,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="s">
-        <v>240</v>
-      </c>
       <c r="B15" s="180" t="s">
         <v>210</v>
       </c>
@@ -17777,9 +17739,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="s">
-        <v>241</v>
-      </c>
       <c r="B16" s="180" t="s">
         <v>211</v>
       </c>
@@ -17908,9 +17867,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="s">
-        <v>242</v>
-      </c>
       <c r="B17" s="180" t="s">
         <v>212</v>
       </c>
@@ -18039,9 +17995,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="s">
-        <v>243</v>
-      </c>
       <c r="B18" s="182" t="s">
         <v>308</v>
       </c>
@@ -19012,58 +18965,58 @@
   </mergeCells>
   <dataValidations count="18">
     <dataValidation allowBlank="true" sqref="C5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="G5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="K5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="O5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="S5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="W5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="AA5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="AE5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="AI5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="AM5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="AQ5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="AU5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="AY5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="BC5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="BG5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="BK5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="BO5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" sqref="BS5" type="list">
-      <formula1>'IV. MA'!$A$1:$A$18</formula1>
+      <formula1>'Daten'!$A$1:$A$18</formula1>
     </dataValidation>
   </dataValidations>
   <tableParts count="18">
@@ -19087,4 +19040,126 @@
     <tablePart r:id="rId18"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="191" t="s">
+        <v>315</v>
+      </c>
+      <c r="I1" s="191" t="s">
+        <v>316</v>
+      </c>
+      <c r="O1" s="191" t="s">
+        <v>317</v>
+      </c>
+      <c r="U1" s="191" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C2" t="str">
+        <f>=VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
+      </c>
+      <c r="I2" t="str">
+        <f>=VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
+      </c>
+      <c r="O2" t="str">
+        <f>=VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
+      </c>
+      <c r="U2" t="str">
+        <f>=VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>243</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: ensure Excel compatibility for functions and tables
- Prefix Excel functions with `_xlfn.` for forward compatibility.
- Adjust table ranges to exclude total rows.
- Update data validation methods to use `SetSqrefDropList`.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -44,8 +44,8 @@
     <definedName name="Kosten_Reserve_EUR">'I. Budget'!$P$11</definedName>
     <definedName name="Gesamtausgaben_LW">'I. Budget'!$O$12</definedName>
     <definedName name="Gesamtausgaben_EUR">'I. Budget'!$P$12</definedName>
-    <definedName name="Geber_Liste">='I. Budget'!$R$2#</definedName>
-    <definedName name="Budget_ID_Liste">='I. Budget'!$S$2#</definedName>
+    <definedName name="Geber_Liste">'I. Budget'!$R$1#</definedName>
+    <definedName name="Budget_ID_Liste">'I. Budget'!$S$1#</definedName>
     <definedName name="Reserve_Freigabe">'I. Budget'!$K$5</definedName>
     <definedName name="FB_Kurs_1">'III. Finanzberichte'!$C$7</definedName>
     <definedName name="FB_SaldoLC_1">'III. Finanzberichte'!$C$29</definedName>
@@ -2658,8 +2658,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TblBudgetAusgaben" displayName="TblBudgetAusgaben" ref="B18:I27">
-  <autoFilter ref="B18:I27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TblBudgetAusgaben" displayName="TblBudgetAusgaben" ref="B18:I26">
+  <autoFilter ref="B18:I26"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="ID"/>
@@ -2675,8 +2675,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Ausgaben_3" displayName="Ausgaben_3" ref="P18:T27">
-  <autoFilter ref="P18:T27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Ausgaben_3" displayName="Ausgaben_3" ref="P18:T26">
+  <autoFilter ref="P18:T26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -2689,8 +2689,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Einnahmen_3" displayName="Einnahmen_3" ref="P40:T46">
-  <autoFilter ref="P40:T46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Einnahmen_3" displayName="Einnahmen_3" ref="P40:T45">
+  <autoFilter ref="P40:T45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2703,8 +2703,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Einnahmen_WK_3" displayName="Einnahmen_WK_3" ref="P49:T56">
-  <autoFilter ref="P49:T56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Einnahmen_WK_3" displayName="Einnahmen_WK_3" ref="P49:T55">
+  <autoFilter ref="P49:T55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2717,8 +2717,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Ausgaben_4" displayName="Ausgaben_4" ref="W18:AA27">
-  <autoFilter ref="W18:AA27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Ausgaben_4" displayName="Ausgaben_4" ref="W18:AA26">
+  <autoFilter ref="W18:AA26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -2731,8 +2731,8 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Einnahmen_4" displayName="Einnahmen_4" ref="W40:AA46">
-  <autoFilter ref="W40:AA46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Einnahmen_4" displayName="Einnahmen_4" ref="W40:AA45">
+  <autoFilter ref="W40:AA45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2745,8 +2745,8 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Einnahmen_WK_4" displayName="Einnahmen_WK_4" ref="W49:AA56">
-  <autoFilter ref="W49:AA56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Einnahmen_WK_4" displayName="Einnahmen_WK_4" ref="W49:AA55">
+  <autoFilter ref="W49:AA55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2759,8 +2759,8 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Ausgaben_5" displayName="Ausgaben_5" ref="AD18:AH27">
-  <autoFilter ref="AD18:AH27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Ausgaben_5" displayName="Ausgaben_5" ref="AD18:AH26">
+  <autoFilter ref="AD18:AH26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -2773,8 +2773,8 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Einnahmen_5" displayName="Einnahmen_5" ref="AD40:AH46">
-  <autoFilter ref="AD40:AH46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="Einnahmen_5" displayName="Einnahmen_5" ref="AD40:AH45">
+  <autoFilter ref="AD40:AH45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2787,8 +2787,8 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Einnahmen_WK_5" displayName="Einnahmen_WK_5" ref="AD49:AH56">
-  <autoFilter ref="AD49:AH56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Einnahmen_WK_5" displayName="Einnahmen_WK_5" ref="AD49:AH55">
+  <autoFilter ref="AD49:AH55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2801,8 +2801,8 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Ausgaben_6" displayName="Ausgaben_6" ref="AK18:AO27">
-  <autoFilter ref="AK18:AO27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="Ausgaben_6" displayName="Ausgaben_6" ref="AK18:AO26">
+  <autoFilter ref="AK18:AO26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -2827,8 +2827,8 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Einnahmen_6" displayName="Einnahmen_6" ref="AK40:AO46">
-  <autoFilter ref="AK40:AO46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="Einnahmen_6" displayName="Einnahmen_6" ref="AK40:AO45">
+  <autoFilter ref="AK40:AO45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2841,8 +2841,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Einnahmen_WK_6" displayName="Einnahmen_WK_6" ref="AK49:AO56">
-  <autoFilter ref="AK49:AO56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Einnahmen_WK_6" displayName="Einnahmen_WK_6" ref="AK49:AO55">
+  <autoFilter ref="AK49:AO55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2855,8 +2855,8 @@
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Ausgaben_7" displayName="Ausgaben_7" ref="AR18:AV27">
-  <autoFilter ref="AR18:AV27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="Ausgaben_7" displayName="Ausgaben_7" ref="AR18:AV26">
+  <autoFilter ref="AR18:AV26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -2869,8 +2869,8 @@
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Einnahmen_7" displayName="Einnahmen_7" ref="AR40:AV46">
-  <autoFilter ref="AR40:AV46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Einnahmen_7" displayName="Einnahmen_7" ref="AR40:AV45">
+  <autoFilter ref="AR40:AV45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2883,8 +2883,8 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Einnahmen_WK_7" displayName="Einnahmen_WK_7" ref="AR49:AV56">
-  <autoFilter ref="AR49:AV56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="Einnahmen_WK_7" displayName="Einnahmen_WK_7" ref="AR49:AV55">
+  <autoFilter ref="AR49:AV55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2897,8 +2897,8 @@
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Ausgaben_8" displayName="Ausgaben_8" ref="AY18:BC27">
-  <autoFilter ref="AY18:BC27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Ausgaben_8" displayName="Ausgaben_8" ref="AY18:BC26">
+  <autoFilter ref="AY18:BC26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -2911,8 +2911,8 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Einnahmen_8" displayName="Einnahmen_8" ref="AY40:BC46">
-  <autoFilter ref="AY40:BC46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="Einnahmen_8" displayName="Einnahmen_8" ref="AY40:BC45">
+  <autoFilter ref="AY40:BC45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2925,8 +2925,8 @@
 </file>
 
 <file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Einnahmen_WK_8" displayName="Einnahmen_WK_8" ref="AY49:BC56">
-  <autoFilter ref="AY49:BC56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="Einnahmen_WK_8" displayName="Einnahmen_WK_8" ref="AY49:BC55">
+  <autoFilter ref="AY49:BC55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2939,8 +2939,8 @@
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Ausgaben_9" displayName="Ausgaben_9" ref="BF18:BJ27">
-  <autoFilter ref="BF18:BJ27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="Ausgaben_9" displayName="Ausgaben_9" ref="BF18:BJ26">
+  <autoFilter ref="BF18:BJ26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -2953,8 +2953,8 @@
 </file>
 
 <file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Einnahmen_9" displayName="Einnahmen_9" ref="BF40:BJ46">
-  <autoFilter ref="BF40:BJ46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="Einnahmen_9" displayName="Einnahmen_9" ref="BF40:BJ45">
+  <autoFilter ref="BF40:BJ45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2980,8 +2980,8 @@
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Einnahmen_WK_9" displayName="Einnahmen_WK_9" ref="BF49:BJ56">
-  <autoFilter ref="BF49:BJ56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="Einnahmen_WK_9" displayName="Einnahmen_WK_9" ref="BF49:BJ55">
+  <autoFilter ref="BF49:BJ55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -2994,8 +2994,8 @@
 </file>
 
 <file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Ausgaben_10" displayName="Ausgaben_10" ref="BM18:BQ27">
-  <autoFilter ref="BM18:BQ27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="Ausgaben_10" displayName="Ausgaben_10" ref="BM18:BQ26">
+  <autoFilter ref="BM18:BQ26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3008,8 +3008,8 @@
 </file>
 
 <file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Einnahmen_10" displayName="Einnahmen_10" ref="BM40:BQ46">
-  <autoFilter ref="BM40:BQ46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="Einnahmen_10" displayName="Einnahmen_10" ref="BM40:BQ45">
+  <autoFilter ref="BM40:BQ45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3022,8 +3022,8 @@
 </file>
 
 <file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Einnahmen_WK_10" displayName="Einnahmen_WK_10" ref="BM49:BQ56">
-  <autoFilter ref="BM49:BQ56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="Einnahmen_WK_10" displayName="Einnahmen_WK_10" ref="BM49:BQ55">
+  <autoFilter ref="BM49:BQ55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3036,8 +3036,8 @@
 </file>
 
 <file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Ausgaben_11" displayName="Ausgaben_11" ref="BT18:BX27">
-  <autoFilter ref="BT18:BX27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="Ausgaben_11" displayName="Ausgaben_11" ref="BT18:BX26">
+  <autoFilter ref="BT18:BX26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3050,8 +3050,8 @@
 </file>
 
 <file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Einnahmen_11" displayName="Einnahmen_11" ref="BT40:BX46">
-  <autoFilter ref="BT40:BX46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="Einnahmen_11" displayName="Einnahmen_11" ref="BT40:BX45">
+  <autoFilter ref="BT40:BX45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3064,8 +3064,8 @@
 </file>
 
 <file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Einnahmen_WK_11" displayName="Einnahmen_WK_11" ref="BT49:BX56">
-  <autoFilter ref="BT49:BX56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="Einnahmen_WK_11" displayName="Einnahmen_WK_11" ref="BT49:BX55">
+  <autoFilter ref="BT49:BX55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3078,8 +3078,8 @@
 </file>
 
 <file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Ausgaben_12" displayName="Ausgaben_12" ref="CA18:CE27">
-  <autoFilter ref="CA18:CE27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="Ausgaben_12" displayName="Ausgaben_12" ref="CA18:CE26">
+  <autoFilter ref="CA18:CE26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3092,8 +3092,8 @@
 </file>
 
 <file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Einnahmen_12" displayName="Einnahmen_12" ref="CA40:CE46">
-  <autoFilter ref="CA40:CE46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="Einnahmen_12" displayName="Einnahmen_12" ref="CA40:CE45">
+  <autoFilter ref="CA40:CE45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3106,8 +3106,8 @@
 </file>
 
 <file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Einnahmen_WK_12" displayName="Einnahmen_WK_12" ref="CA49:CE56">
-  <autoFilter ref="CA49:CE56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="Einnahmen_WK_12" displayName="Einnahmen_WK_12" ref="CA49:CE55">
+  <autoFilter ref="CA49:CE55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3120,8 +3120,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Ausgaben_1" displayName="Ausgaben_1" ref="B18:F27">
-  <autoFilter ref="B18:F27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Ausgaben_1" displayName="Ausgaben_1" ref="B18:F26">
+  <autoFilter ref="B18:F26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3134,8 +3134,8 @@
 </file>
 
 <file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Ausgaben_13" displayName="Ausgaben_13" ref="CH18:CL27">
-  <autoFilter ref="CH18:CL27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="Ausgaben_13" displayName="Ausgaben_13" ref="CH18:CL26">
+  <autoFilter ref="CH18:CL26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3148,8 +3148,8 @@
 </file>
 
 <file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Einnahmen_13" displayName="Einnahmen_13" ref="CH40:CL46">
-  <autoFilter ref="CH40:CL46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="Einnahmen_13" displayName="Einnahmen_13" ref="CH40:CL45">
+  <autoFilter ref="CH40:CL45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3162,8 +3162,8 @@
 </file>
 
 <file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Einnahmen_WK_13" displayName="Einnahmen_WK_13" ref="CH49:CL56">
-  <autoFilter ref="CH49:CL56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="Einnahmen_WK_13" displayName="Einnahmen_WK_13" ref="CH49:CL55">
+  <autoFilter ref="CH49:CL55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3176,8 +3176,8 @@
 </file>
 
 <file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Ausgaben_14" displayName="Ausgaben_14" ref="CO18:CS27">
-  <autoFilter ref="CO18:CS27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="Ausgaben_14" displayName="Ausgaben_14" ref="CO18:CS26">
+  <autoFilter ref="CO18:CS26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3190,8 +3190,8 @@
 </file>
 
 <file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Einnahmen_14" displayName="Einnahmen_14" ref="CO40:CS46">
-  <autoFilter ref="CO40:CS46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="Einnahmen_14" displayName="Einnahmen_14" ref="CO40:CS45">
+  <autoFilter ref="CO40:CS45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3204,8 +3204,8 @@
 </file>
 
 <file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Einnahmen_WK_14" displayName="Einnahmen_WK_14" ref="CO49:CS56">
-  <autoFilter ref="CO49:CS56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="Einnahmen_WK_14" displayName="Einnahmen_WK_14" ref="CO49:CS55">
+  <autoFilter ref="CO49:CS55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3218,8 +3218,8 @@
 </file>
 
 <file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Ausgaben_15" displayName="Ausgaben_15" ref="CV18:CZ27">
-  <autoFilter ref="CV18:CZ27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="Ausgaben_15" displayName="Ausgaben_15" ref="CV18:CZ26">
+  <autoFilter ref="CV18:CZ26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3232,8 +3232,8 @@
 </file>
 
 <file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Einnahmen_15" displayName="Einnahmen_15" ref="CV40:CZ46">
-  <autoFilter ref="CV40:CZ46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="Einnahmen_15" displayName="Einnahmen_15" ref="CV40:CZ45">
+  <autoFilter ref="CV40:CZ45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3246,8 +3246,8 @@
 </file>
 
 <file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Einnahmen_WK_15" displayName="Einnahmen_WK_15" ref="CV49:CZ56">
-  <autoFilter ref="CV49:CZ56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="Einnahmen_WK_15" displayName="Einnahmen_WK_15" ref="CV49:CZ55">
+  <autoFilter ref="CV49:CZ55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3260,8 +3260,8 @@
 </file>
 
 <file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Ausgaben_16" displayName="Ausgaben_16" ref="DC18:DG27">
-  <autoFilter ref="DC18:DG27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="Ausgaben_16" displayName="Ausgaben_16" ref="DC18:DG26">
+  <autoFilter ref="DC18:DG26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3274,8 +3274,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Einnahmen_1" displayName="Einnahmen_1" ref="B40:F46">
-  <autoFilter ref="B40:F46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Einnahmen_1" displayName="Einnahmen_1" ref="B40:F45">
+  <autoFilter ref="B40:F45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3288,8 +3288,8 @@
 </file>
 
 <file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Einnahmen_16" displayName="Einnahmen_16" ref="DC40:DG46">
-  <autoFilter ref="DC40:DG46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="Einnahmen_16" displayName="Einnahmen_16" ref="DC40:DG45">
+  <autoFilter ref="DC40:DG45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3302,8 +3302,8 @@
 </file>
 
 <file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Einnahmen_WK_16" displayName="Einnahmen_WK_16" ref="DC49:DG56">
-  <autoFilter ref="DC49:DG56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="Einnahmen_WK_16" displayName="Einnahmen_WK_16" ref="DC49:DG55">
+  <autoFilter ref="DC49:DG55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3316,8 +3316,8 @@
 </file>
 
 <file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Ausgaben_17" displayName="Ausgaben_17" ref="DJ18:DN27">
-  <autoFilter ref="DJ18:DN27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="Ausgaben_17" displayName="Ausgaben_17" ref="DJ18:DN26">
+  <autoFilter ref="DJ18:DN26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3330,8 +3330,8 @@
 </file>
 
 <file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Einnahmen_17" displayName="Einnahmen_17" ref="DJ40:DN46">
-  <autoFilter ref="DJ40:DN46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="Einnahmen_17" displayName="Einnahmen_17" ref="DJ40:DN45">
+  <autoFilter ref="DJ40:DN45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3344,8 +3344,8 @@
 </file>
 
 <file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Einnahmen_WK_17" displayName="Einnahmen_WK_17" ref="DJ49:DN56">
-  <autoFilter ref="DJ49:DN56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="Einnahmen_WK_17" displayName="Einnahmen_WK_17" ref="DJ49:DN55">
+  <autoFilter ref="DJ49:DN55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3358,8 +3358,8 @@
 </file>
 
 <file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Ausgaben_18" displayName="Ausgaben_18" ref="DQ18:DU27">
-  <autoFilter ref="DQ18:DU27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="Ausgaben_18" displayName="Ausgaben_18" ref="DQ18:DU26">
+  <autoFilter ref="DQ18:DU26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3372,8 +3372,8 @@
 </file>
 
 <file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Einnahmen_18" displayName="Einnahmen_18" ref="DQ40:DU46">
-  <autoFilter ref="DQ40:DU46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="Einnahmen_18" displayName="Einnahmen_18" ref="DQ40:DU45">
+  <autoFilter ref="DQ40:DU45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3386,8 +3386,8 @@
 </file>
 
 <file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Einnahmen_WK_18" displayName="Einnahmen_WK_18" ref="DQ49:DU56">
-  <autoFilter ref="DQ49:DU56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="Einnahmen_WK_18" displayName="Einnahmen_WK_18" ref="DQ49:DU55">
+  <autoFilter ref="DQ49:DU55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3400,8 +3400,8 @@
 </file>
 
 <file path=xl/tables/table58.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="MA_1" displayName="MA_1" ref="B9:D18">
-  <autoFilter ref="B9:D18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="MA_1" displayName="MA_1" ref="B9:D17">
+  <autoFilter ref="B9:D17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3412,8 +3412,8 @@
 </file>
 
 <file path=xl/tables/table59.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="MA_2" displayName="MA_2" ref="F9:H18">
-  <autoFilter ref="F9:H18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="MA_2" displayName="MA_2" ref="F9:H17">
+  <autoFilter ref="F9:H17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3424,8 +3424,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Einnahmen_WK_1" displayName="Einnahmen_WK_1" ref="B49:F56">
-  <autoFilter ref="B49:F56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Einnahmen_WK_1" displayName="Einnahmen_WK_1" ref="B49:F55">
+  <autoFilter ref="B49:F55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3438,8 +3438,8 @@
 </file>
 
 <file path=xl/tables/table60.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="MA_3" displayName="MA_3" ref="J9:L18">
-  <autoFilter ref="J9:L18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="MA_3" displayName="MA_3" ref="J9:L17">
+  <autoFilter ref="J9:L17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3450,8 +3450,8 @@
 </file>
 
 <file path=xl/tables/table61.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="MA_4" displayName="MA_4" ref="N9:P18">
-  <autoFilter ref="N9:P18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="MA_4" displayName="MA_4" ref="N9:P17">
+  <autoFilter ref="N9:P17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3462,8 +3462,8 @@
 </file>
 
 <file path=xl/tables/table62.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="MA_5" displayName="MA_5" ref="R9:T18">
-  <autoFilter ref="R9:T18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="MA_5" displayName="MA_5" ref="R9:T17">
+  <autoFilter ref="R9:T17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3474,8 +3474,8 @@
 </file>
 
 <file path=xl/tables/table63.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="MA_6" displayName="MA_6" ref="V9:X18">
-  <autoFilter ref="V9:X18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="MA_6" displayName="MA_6" ref="V9:X17">
+  <autoFilter ref="V9:X17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3486,8 +3486,8 @@
 </file>
 
 <file path=xl/tables/table64.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="MA_7" displayName="MA_7" ref="Z9:AB18">
-  <autoFilter ref="Z9:AB18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="MA_7" displayName="MA_7" ref="Z9:AB17">
+  <autoFilter ref="Z9:AB17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3498,8 +3498,8 @@
 </file>
 
 <file path=xl/tables/table65.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="MA_8" displayName="MA_8" ref="AD9:AF18">
-  <autoFilter ref="AD9:AF18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="MA_8" displayName="MA_8" ref="AD9:AF17">
+  <autoFilter ref="AD9:AF17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3510,8 +3510,8 @@
 </file>
 
 <file path=xl/tables/table66.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="MA_9" displayName="MA_9" ref="AH9:AJ18">
-  <autoFilter ref="AH9:AJ18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="MA_9" displayName="MA_9" ref="AH9:AJ17">
+  <autoFilter ref="AH9:AJ17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3522,8 +3522,8 @@
 </file>
 
 <file path=xl/tables/table67.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="MA_10" displayName="MA_10" ref="AL9:AN18">
-  <autoFilter ref="AL9:AN18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="MA_10" displayName="MA_10" ref="AL9:AN17">
+  <autoFilter ref="AL9:AN17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3534,8 +3534,8 @@
 </file>
 
 <file path=xl/tables/table68.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="MA_11" displayName="MA_11" ref="AP9:AR18">
-  <autoFilter ref="AP9:AR18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="MA_11" displayName="MA_11" ref="AP9:AR17">
+  <autoFilter ref="AP9:AR17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3546,8 +3546,8 @@
 </file>
 
 <file path=xl/tables/table69.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="MA_12" displayName="MA_12" ref="AT9:AV18">
-  <autoFilter ref="AT9:AV18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="MA_12" displayName="MA_12" ref="AT9:AV17">
+  <autoFilter ref="AT9:AV17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3558,8 +3558,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Ausgaben_2" displayName="Ausgaben_2" ref="I18:M27">
-  <autoFilter ref="I18:M27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Ausgaben_2" displayName="Ausgaben_2" ref="I18:M26">
+  <autoFilter ref="I18:M26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ausgaben (LC)"/>
@@ -3572,8 +3572,8 @@
 </file>
 
 <file path=xl/tables/table70.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="MA_13" displayName="MA_13" ref="AX9:AZ18">
-  <autoFilter ref="AX9:AZ18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="MA_13" displayName="MA_13" ref="AX9:AZ17">
+  <autoFilter ref="AX9:AZ17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3584,8 +3584,8 @@
 </file>
 
 <file path=xl/tables/table71.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="MA_14" displayName="MA_14" ref="BB9:BD18">
-  <autoFilter ref="BB9:BD18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="MA_14" displayName="MA_14" ref="BB9:BD17">
+  <autoFilter ref="BB9:BD17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3596,8 +3596,8 @@
 </file>
 
 <file path=xl/tables/table72.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="72" name="MA_15" displayName="MA_15" ref="BF9:BH18">
-  <autoFilter ref="BF9:BH18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="72" name="MA_15" displayName="MA_15" ref="BF9:BH17">
+  <autoFilter ref="BF9:BH17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3608,8 +3608,8 @@
 </file>
 
 <file path=xl/tables/table73.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="73" name="MA_16" displayName="MA_16" ref="BJ9:BL18">
-  <autoFilter ref="BJ9:BL18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="73" name="MA_16" displayName="MA_16" ref="BJ9:BL17">
+  <autoFilter ref="BJ9:BL17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3620,8 +3620,8 @@
 </file>
 
 <file path=xl/tables/table74.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="MA_17" displayName="MA_17" ref="BN9:BP18">
-  <autoFilter ref="BN9:BP18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="MA_17" displayName="MA_17" ref="BN9:BP17">
+  <autoFilter ref="BN9:BP17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3632,8 +3632,8 @@
 </file>
 
 <file path=xl/tables/table75.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="MA_18" displayName="MA_18" ref="BR9:BT18">
-  <autoFilter ref="BR9:BT18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="MA_18" displayName="MA_18" ref="BR9:BT17">
+  <autoFilter ref="BR9:BT17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Kostenkategorie"/>
     <tableColumn id="2" name="Angefordert (LC)"/>
@@ -3644,8 +3644,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Einnahmen_2" displayName="Einnahmen_2" ref="I40:M46">
-  <autoFilter ref="I40:M46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Einnahmen_2" displayName="Einnahmen_2" ref="I40:M45">
+  <autoFilter ref="I40:M45"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -3658,8 +3658,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Einnahmen_WK_2" displayName="Einnahmen_WK_2" ref="I49:M56">
-  <autoFilter ref="I49:M56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Einnahmen_WK_2" displayName="Einnahmen_WK_2" ref="I49:M55">
+  <autoFilter ref="I49:M55"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Typ"/>
     <tableColumn id="2" name="Geber"/>
@@ -4973,10 +4973,10 @@
   <sheetData>
     <row r="1">
       <c r="R1" s="3" t="str">
-        <f>=VSTACK({"Projektpartner";"Bank"},IFERROR(FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
+        <f>=_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
       </c>
       <c r="S1" s="3" t="str">
-        <f>=IFERROR(FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
+        <f>=IFERROR(_xlfn.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
       </c>
     </row>
     <row r="2" ht="24" customHeight="true">
@@ -5289,7 +5289,7 @@
         <v>205</v>
       </c>
       <c r="C19" s="33" t="str">
-        <f>=IF(B19="","",MATCH(B19,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B19,B19))</f>
+        <f>=IF(B19="","",MATCH(B19,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B19,B19))</f>
       </c>
       <c r="D19" s="32" t="s">
         <v>158</v>
@@ -5310,7 +5310,7 @@
         <v>206</v>
       </c>
       <c r="C20" s="33" t="str">
-        <f>=IF(B20="","",MATCH(B20,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
+        <f>=IF(B20="","",MATCH(B20,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B20,B20))</f>
       </c>
       <c r="D20" s="32" t="s">
         <v>158</v>
@@ -5331,7 +5331,7 @@
         <v>207</v>
       </c>
       <c r="C21" s="33" t="str">
-        <f>=IF(B21="","",MATCH(B21,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
+        <f>=IF(B21="","",MATCH(B21,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B21,B21))</f>
       </c>
       <c r="D21" s="32" t="s">
         <v>158</v>
@@ -5352,7 +5352,7 @@
         <v>208</v>
       </c>
       <c r="C22" s="33" t="str">
-        <f>=IF(B22="","",MATCH(B22,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
+        <f>=IF(B22="","",MATCH(B22,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B22,B22))</f>
       </c>
       <c r="D22" s="32" t="s">
         <v>158</v>
@@ -5368,7 +5368,7 @@
         <v>209</v>
       </c>
       <c r="C23" s="33" t="str">
-        <f>=IF(B23="","",MATCH(B23,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
+        <f>=IF(B23="","",MATCH(B23,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B23,B23))</f>
       </c>
       <c r="D23" s="32" t="s">
         <v>158</v>
@@ -5384,7 +5384,7 @@
         <v>210</v>
       </c>
       <c r="C24" s="33" t="str">
-        <f>=IF(B24="","",MATCH(B24,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
+        <f>=IF(B24="","",MATCH(B24,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B24,B24))</f>
       </c>
       <c r="D24" s="32" t="s">
         <v>158</v>
@@ -5400,7 +5400,7 @@
         <v>211</v>
       </c>
       <c r="C25" s="33" t="str">
-        <f>=IF(B25="","",MATCH(B25,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
+        <f>=IF(B25="","",MATCH(B25,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B25,B25))</f>
       </c>
       <c r="D25" s="32" t="s">
         <v>158</v>
@@ -5416,7 +5416,7 @@
         <v>212</v>
       </c>
       <c r="C26" s="33" t="str">
-        <f>=IF(B26="","",MATCH(B26,{"Bauausgaben";"Investitionen";"Personalkosten";"Projektaktivitaeten";"Projektverwaltung";"Evaluierung";"Audit";"Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B26,B26))</f>
+        <f>=IF(B26="","",MATCH(B26,{"Bauausgaben","Investitionen","Personalkosten","Projektaktivitaeten","Projektverwaltung","Evaluierung","Audit","Reserve"},0)&amp;"."&amp;COUNTIF(B$19:B26,B26))</f>
       </c>
       <c r="D26" s="32" t="s">
         <v>158</v>
@@ -19068,16 +19068,16 @@
         <v>227</v>
       </c>
       <c r="C2" t="str">
-        <f>=VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
+        <f>=_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
       </c>
       <c r="I2" t="str">
-        <f>=VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
+        <f>=_xlfn.VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
       </c>
       <c r="O2" t="str">
-        <f>=VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
+        <f>=_xlfn.VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
       </c>
       <c r="U2" t="str">
-        <f>=VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
+        <f>=_xlfn.VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
refactor: remove table styles and replace dynamic arrays with OFFSET
- Set TableStyleName to empty string to ensure no default Excel table
  formatting is applied.
- Replace spilled range references (#) in named formulas with OFFSET
  functions to improve compatibility with older Excel versions.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -44,8 +44,8 @@
     <definedName name="Kosten_Reserve_EUR">'I. Budget'!$P$11</definedName>
     <definedName name="Gesamtausgaben_LW">'I. Budget'!$O$12</definedName>
     <definedName name="Gesamtausgaben_EUR">'I. Budget'!$P$12</definedName>
-    <definedName name="Geber_Liste">'I. Budget'!$R$1#</definedName>
-    <definedName name="Budget_ID_Liste">'I. Budget'!$S$1#</definedName>
+    <definedName name="Geber_Liste">OFFSET('I. Budget'!$R$1, 0, 0, COUNTA('I. Budget'!R:R), 1)</definedName>
+    <definedName name="Budget_ID_Liste">OFFSET('I. Budget'!$S$1, 0, 0, COUNTA('I. Budget'!S:S), 1)</definedName>
     <definedName name="Reserve_Freigabe">'I. Budget'!$K$5</definedName>
     <definedName name="FB_Kurs_1">'III. Finanzberichte'!$C$7</definedName>
     <definedName name="FB_SaldoLC_1">'III. Finanzberichte'!$C$29</definedName>
@@ -2670,7 +2670,7 @@
     <tableColumn id="7" name="Jahr 3"/>
     <tableColumn id="8" name="Betrag (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2684,7 +2684,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2698,7 +2698,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2712,7 +2712,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2726,7 +2726,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2740,7 +2740,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2754,7 +2754,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2768,7 +2768,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2782,7 +2782,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2796,7 +2796,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2810,7 +2810,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2822,7 +2822,7 @@
     <tableColumn id="2" name="Betrag (LC)"/>
     <tableColumn id="3" name="Betrag (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2836,7 +2836,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2850,7 +2850,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2864,7 +2864,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2878,7 +2878,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2892,7 +2892,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2906,7 +2906,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2920,7 +2920,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2934,7 +2934,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2948,7 +2948,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2962,7 +2962,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -2989,7 +2989,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3003,7 +3003,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3017,7 +3017,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3031,7 +3031,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3045,7 +3045,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3059,7 +3059,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3073,7 +3073,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3087,7 +3087,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3101,7 +3101,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3115,7 +3115,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3129,7 +3129,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3143,7 +3143,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3157,7 +3157,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3171,7 +3171,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3185,7 +3185,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3199,7 +3199,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3213,7 +3213,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3227,7 +3227,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3241,7 +3241,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3255,7 +3255,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3269,7 +3269,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3283,7 +3283,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3297,7 +3297,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3311,7 +3311,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3325,7 +3325,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3339,7 +3339,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3353,7 +3353,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3367,7 +3367,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3381,7 +3381,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3395,7 +3395,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3407,7 +3407,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3419,7 +3419,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3433,7 +3433,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3445,7 +3445,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3457,7 +3457,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3469,7 +3469,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3481,7 +3481,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3493,7 +3493,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3505,7 +3505,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3517,7 +3517,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3529,7 +3529,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3541,7 +3541,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3553,7 +3553,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3567,7 +3567,7 @@
     <tableColumn id="4" name="Kum. Ausgaben (LC)"/>
     <tableColumn id="5" name="Kum. Ausgaben (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3579,7 +3579,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3591,7 +3591,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3603,7 +3603,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3615,7 +3615,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3627,7 +3627,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3639,7 +3639,7 @@
     <tableColumn id="2" name="Angefordert (LC)"/>
     <tableColumn id="3" name="Angefordert (EUR)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3653,7 +3653,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 
@@ -3667,7 +3667,7 @@
     <tableColumn id="4" name="Einnahmen (EUR)"/>
     <tableColumn id="5" name="Kurs"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleNone" showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
+  <tableStyleInfo showFirstColumn="false" showLastColumn="false" showRowStripes="false" showColumnStripes="false"/>
 </table>
 </file>
 

</xml_diff>

<commit_message>
refactor: optimize spreadsheet formulas using dynamic arrays
Split VSTACK operations into intermediate helper columns to improve
formula performance and readability, enabling use of dynamic array
spilling for FILTER functions.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -19068,16 +19068,28 @@
         <v>227</v>
       </c>
       <c r="C2" t="str">
-        <f>_xlfn.LET(v, _xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45), _xlfn.FILTER(v, (_xlfn.CHOOSECOLS(v,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(v,4)&lt;&gt;0), ""))</f>
+        <f>_xlfn.FILTER(AA2#, (_xlfn.CHOOSECOLS(AA2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AA2#,4)&lt;&gt;0), "")</f>
       </c>
       <c r="I2" t="str">
-        <f>_xlfn.LET(v, _xlfn.VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55), _xlfn.FILTER(v, (_xlfn.CHOOSECOLS(v,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(v,4)&lt;&gt;0), ""))</f>
+        <f>_xlfn.FILTER(AG2#, (_xlfn.CHOOSECOLS(AG2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AG2#,4)&lt;&gt;0), "")</f>
       </c>
       <c r="O2" t="str">
-        <f>_xlfn.LET(v, _xlfn.VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26), _xlfn.FILTER(v, (_xlfn.CHOOSECOLS(v,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(v,3)&lt;&gt;0), ""))</f>
+        <f>_xlfn.FILTER(AM2#, (_xlfn.CHOOSECOLS(AM2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AM2#,3)&lt;&gt;0), "")</f>
       </c>
       <c r="U2" t="str">
-        <f>_xlfn.LET(v, _xlfn.VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17), _xlfn.FILTER(v, (_xlfn.CHOOSECOLS(v,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(v,3)&lt;&gt;0), ""))</f>
+        <f>_xlfn.FILTER(AS2#, (_xlfn.CHOOSECOLS(AS2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AS2#,3)&lt;&gt;0), "")</f>
+      </c>
+      <c r="AA2" t="str">
+        <f>_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
+      </c>
+      <c r="AG2" t="str">
+        <f>_xlfn.VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
+      </c>
+      <c r="AM2" t="str">
+        <f>_xlfn.VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
+      </c>
+      <c r="AS2" t="str">
+        <f>_xlfn.VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
fix: update FILTER function namespace to _xlws
Adjusted formula references from _xlfn.FILTER to _xlfn._xlws.FILTER to ensure compatibility with specific Excel versions.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -4973,10 +4973,10 @@
   <sheetData>
     <row r="1">
       <c r="R1" s="3" t="str">
-        <f>=_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
+        <f>=_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn._xlws.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
       </c>
       <c r="S1" s="3" t="str">
-        <f>=IFERROR(_xlfn.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
+        <f>=IFERROR(_xlfn._xlws.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
       </c>
     </row>
     <row r="2" ht="24" customHeight="true">
@@ -19068,16 +19068,16 @@
         <v>227</v>
       </c>
       <c r="C2" t="str">
-        <f>_xlfn.FILTER(AA2#, (_xlfn.CHOOSECOLS(AA2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AA2#,4)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(AA2#, (_xlfn.CHOOSECOLS(AA2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AA2#,4)&lt;&gt;0), "")</f>
       </c>
       <c r="I2" t="str">
-        <f>_xlfn.FILTER(AG2#, (_xlfn.CHOOSECOLS(AG2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AG2#,4)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(AG2#, (_xlfn.CHOOSECOLS(AG2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AG2#,4)&lt;&gt;0), "")</f>
       </c>
       <c r="O2" t="str">
-        <f>_xlfn.FILTER(AM2#, (_xlfn.CHOOSECOLS(AM2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AM2#,3)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(AM2#, (_xlfn.CHOOSECOLS(AM2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AM2#,3)&lt;&gt;0), "")</f>
       </c>
       <c r="U2" t="str">
-        <f>_xlfn.FILTER(AS2#, (_xlfn.CHOOSECOLS(AS2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AS2#,3)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(AS2#, (_xlfn.CHOOSECOLS(AS2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AS2#,3)&lt;&gt;0), "")</f>
       </c>
       <c r="AA2" t="str">
         <f>_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>

</xml_diff>

<commit_message>
refactor: replace spill range syntax with ANCHORARRAY in formulas
Replaced Excel spill range operators (#) with the _xlfn.ANCHORARRAY function
across budget and data generation logic to improve formula compatibility
and stability in generated output.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -4973,10 +4973,10 @@
   <sheetData>
     <row r="1">
       <c r="R1" s="3" t="str">
-        <f>=_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn._xlws.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
+        <f>_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn._xlws.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
       </c>
       <c r="S1" s="3" t="str">
-        <f>=IFERROR(_xlfn._xlws.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
+        <f>IFERROR(_xlfn._xlws.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
       </c>
     </row>
     <row r="2" ht="24" customHeight="true">
@@ -19068,16 +19068,16 @@
         <v>227</v>
       </c>
       <c r="C2" t="str">
-        <f>_xlfn._xlws.FILTER(AA2#, (_xlfn.CHOOSECOLS(AA2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AA2#,4)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AA2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),4)&lt;&gt;0), "")</f>
       </c>
       <c r="I2" t="str">
-        <f>_xlfn._xlws.FILTER(AG2#, (_xlfn.CHOOSECOLS(AG2#,3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AG2#,4)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AG2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),4)&lt;&gt;0), "")</f>
       </c>
       <c r="O2" t="str">
-        <f>_xlfn._xlws.FILTER(AM2#, (_xlfn.CHOOSECOLS(AM2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AM2#,3)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AM2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),3)&lt;&gt;0), "")</f>
       </c>
       <c r="U2" t="str">
-        <f>_xlfn._xlws.FILTER(AS2#, (_xlfn.CHOOSECOLS(AS2#,2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(AS2#,3)&lt;&gt;0), "")</f>
+        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AS2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),3)&lt;&gt;0), "")</f>
       </c>
       <c r="AA2" t="str">
         <f>_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>

</xml_diff>

<commit_message>
feat: implement dynamic array support for Excel formulas
Added support for dynamic array spill formulas (e.g., VSTACK, FILTER) by
injecting the required XLDAPR metadata into the .xlsx zip structure.
This prevents Excel from automatically inserting the implicit
intersection operator (@) in these formulas.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -122,6 +122,28 @@
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4972,11 +4994,11 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="R1" s="3" t="str">
-        <f>_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn._xlws.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
-      </c>
-      <c r="S1" s="3" t="str">
-        <f>IFERROR(_xlfn._xlws.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
+      <c r="R1" cm="1" s="3" t="str">
+        <f t="array" ref="R1" aca="1" ca="1">_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn._xlws.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
+      </c>
+      <c r="S1" cm="1" s="3" t="str">
+        <f t="array" ref="S1" aca="1" ca="1">IFERROR(_xlfn._xlws.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
       </c>
     </row>
     <row r="2" ht="24" customHeight="true">
@@ -19067,29 +19089,29 @@
       <c r="A2" t="s">
         <v>227</v>
       </c>
-      <c r="C2" t="str">
-        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AA2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),4)&lt;&gt;0), "")</f>
-      </c>
-      <c r="I2" t="str">
-        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AG2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),4)&lt;&gt;0), "")</f>
-      </c>
-      <c r="O2" t="str">
-        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AM2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),3)&lt;&gt;0), "")</f>
-      </c>
-      <c r="U2" t="str">
-        <f>_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AS2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),3)&lt;&gt;0), "")</f>
-      </c>
-      <c r="AA2" t="str">
-        <f>_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
-      </c>
-      <c r="AG2" t="str">
-        <f>_xlfn.VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
-      </c>
-      <c r="AM2" t="str">
-        <f>_xlfn.VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
-      </c>
-      <c r="AS2" t="str">
-        <f>_xlfn.VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
+      <c r="C2" cm="1" s="3" t="str">
+        <f t="array" ref="C2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AA2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),4)&lt;&gt;0), "")</f>
+      </c>
+      <c r="I2" cm="1" s="3" t="str">
+        <f t="array" ref="I2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AG2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),4)&lt;&gt;0), "")</f>
+      </c>
+      <c r="O2" cm="1" s="3" t="str">
+        <f t="array" ref="O2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AM2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),3)&lt;&gt;0), "")</f>
+      </c>
+      <c r="U2" cm="1" s="3" t="str">
+        <f t="array" ref="U2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AS2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),3)&lt;&gt;0), "")</f>
+      </c>
+      <c r="AA2" cm="1" s="3" t="str">
+        <f t="array" ref="AA2" aca="1" ca="1">_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
+      </c>
+      <c r="AG2" cm="1" s="3" t="str">
+        <f t="array" ref="AG2" aca="1" ca="1">_xlfn.VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
+      </c>
+      <c r="AM2" cm="1" s="3" t="str">
+        <f t="array" ref="AM2" aca="1" ca="1">_xlfn.VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
+      </c>
+      <c r="AS2" cm="1" s="3" t="str">
+        <f t="array" ref="AS2" aca="1" ca="1">_xlfn.VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
fix: adjust dynamic array formula marking
Update formula marking to match Excel's requirements for dynamic arrays
by removing legacy CSE attributes (aca/ca) and ensuring correct cm=1
usage to prevent accidental conversion to legacy array formulas. Also,
enable full calculation on load to ensure proper spilling.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -120,7 +120,7 @@
     <definedName name="MA_Kurs_17">'IV. MA'!$BO$7</definedName>
     <definedName name="MA_Kurs_18">'IV. MA'!$BS$7</definedName>
   </definedNames>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="122211" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
@@ -4994,11 +4994,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="R1" cm="1" s="3" t="str">
-        <f t="array" ref="R1" aca="1" ca="1">_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn._xlws.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
-      </c>
-      <c r="S1" cm="1" s="3" t="str">
-        <f t="array" ref="S1" aca="1" ca="1">IFERROR(_xlfn._xlws.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
+      <c r="R1" cm="1" s="3">
+        <f t="array" ref="R1">_xlfn.VSTACK({"Projektpartner";"Bank"},IFERROR(_xlfn._xlws.FILTER(TblDrittmittel[Name des Gebers],TblDrittmittel[Name des Gebers]&lt;&gt;""),""))</f>
+        <v>0</v>
+      </c>
+      <c r="S1" cm="1" s="3">
+        <f t="array" ref="S1">IFERROR(_xlfn._xlws.FILTER(TblBudgetAusgaben[ID],TblBudgetAusgaben[ID]&lt;&gt;""),"")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="true">
@@ -19089,29 +19091,37 @@
       <c r="A2" t="s">
         <v>227</v>
       </c>
-      <c r="C2" cm="1" s="3" t="str">
-        <f t="array" ref="C2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AA2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),4)&lt;&gt;0), "")</f>
-      </c>
-      <c r="I2" cm="1" s="3" t="str">
-        <f t="array" ref="I2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AG2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),4)&lt;&gt;0), "")</f>
-      </c>
-      <c r="O2" cm="1" s="3" t="str">
-        <f t="array" ref="O2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AM2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),3)&lt;&gt;0), "")</f>
-      </c>
-      <c r="U2" cm="1" s="3" t="str">
-        <f t="array" ref="U2" aca="1" ca="1">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AS2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),3)&lt;&gt;0), "")</f>
-      </c>
-      <c r="AA2" cm="1" s="3" t="str">
-        <f t="array" ref="AA2" aca="1" ca="1">_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
-      </c>
-      <c r="AG2" cm="1" s="3" t="str">
-        <f t="array" ref="AG2" aca="1" ca="1">_xlfn.VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
-      </c>
-      <c r="AM2" cm="1" s="3" t="str">
-        <f t="array" ref="AM2" aca="1" ca="1">_xlfn.VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
-      </c>
-      <c r="AS2" cm="1" s="3" t="str">
-        <f t="array" ref="AS2" aca="1" ca="1">_xlfn.VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
+      <c r="C2" cm="1" s="3">
+        <f t="array" ref="C2">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AA2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AA2),4)&lt;&gt;0), "")</f>
+        <v>0</v>
+      </c>
+      <c r="I2" cm="1" s="3">
+        <f t="array" ref="I2">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AG2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),3)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AG2),4)&lt;&gt;0), "")</f>
+        <v>0</v>
+      </c>
+      <c r="O2" cm="1" s="3">
+        <f t="array" ref="O2">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AM2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AM2),3)&lt;&gt;0), "")</f>
+        <v>0</v>
+      </c>
+      <c r="U2" cm="1" s="3">
+        <f t="array" ref="U2">_xlfn._xlws.FILTER(_xlfn.ANCHORARRAY(AS2), (_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),2)&lt;&gt;0)+(_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(AS2),3)&lt;&gt;0), "")</f>
+        <v>0</v>
+      </c>
+      <c r="AA2" cm="1" s="3">
+        <f t="array" ref="AA2">_xlfn.VSTACK('III. Finanzberichte'!$B$41:$F$45,'III. Finanzberichte'!$I$41:$M$45,'III. Finanzberichte'!$P$41:$T$45,'III. Finanzberichte'!$W$41:$AA$45,'III. Finanzberichte'!$AD$41:$AH$45,'III. Finanzberichte'!$AK$41:$AO$45,'III. Finanzberichte'!$AR$41:$AV$45,'III. Finanzberichte'!$AY$41:$BC$45,'III. Finanzberichte'!$BF$41:$BJ$45,'III. Finanzberichte'!$BM$41:$BQ$45,'III. Finanzberichte'!$BT$41:$BX$45,'III. Finanzberichte'!$CA$41:$CE$45,'III. Finanzberichte'!$CH$41:$CL$45,'III. Finanzberichte'!$CO$41:$CS$45,'III. Finanzberichte'!$CV$41:$CZ$45,'III. Finanzberichte'!$DC$41:$DG$45,'III. Finanzberichte'!$DJ$41:$DN$45,'III. Finanzberichte'!$DQ$41:$DU$45)</f>
+        <v>0</v>
+      </c>
+      <c r="AG2" cm="1" s="3">
+        <f t="array" ref="AG2">_xlfn.VSTACK('III. Finanzberichte'!$B$50:$F$55,'III. Finanzberichte'!$I$50:$M$55,'III. Finanzberichte'!$P$50:$T$55,'III. Finanzberichte'!$W$50:$AA$55,'III. Finanzberichte'!$AD$50:$AH$55,'III. Finanzberichte'!$AK$50:$AO$55,'III. Finanzberichte'!$AR$50:$AV$55,'III. Finanzberichte'!$AY$50:$BC$55,'III. Finanzberichte'!$BF$50:$BJ$55,'III. Finanzberichte'!$BM$50:$BQ$55,'III. Finanzberichte'!$BT$50:$BX$55,'III. Finanzberichte'!$CA$50:$CE$55,'III. Finanzberichte'!$CH$50:$CL$55,'III. Finanzberichte'!$CO$50:$CS$55,'III. Finanzberichte'!$CV$50:$CZ$55,'III. Finanzberichte'!$DC$50:$DG$55,'III. Finanzberichte'!$DJ$50:$DN$55,'III. Finanzberichte'!$DQ$50:$DU$55)</f>
+        <v>0</v>
+      </c>
+      <c r="AM2" cm="1" s="3">
+        <f t="array" ref="AM2">_xlfn.VSTACK('III. Finanzberichte'!$B$19:$F$26,'III. Finanzberichte'!$I$19:$M$26,'III. Finanzberichte'!$P$19:$T$26,'III. Finanzberichte'!$W$19:$AA$26,'III. Finanzberichte'!$AD$19:$AH$26,'III. Finanzberichte'!$AK$19:$AO$26,'III. Finanzberichte'!$AR$19:$AV$26,'III. Finanzberichte'!$AY$19:$BC$26,'III. Finanzberichte'!$BF$19:$BJ$26,'III. Finanzberichte'!$BM$19:$BQ$26,'III. Finanzberichte'!$BT$19:$BX$26,'III. Finanzberichte'!$CA$19:$CE$26,'III. Finanzberichte'!$CH$19:$CL$26,'III. Finanzberichte'!$CO$19:$CS$26,'III. Finanzberichte'!$CV$19:$CZ$26,'III. Finanzberichte'!$DC$19:$DG$26,'III. Finanzberichte'!$DJ$19:$DN$26,'III. Finanzberichte'!$DQ$19:$DU$26)</f>
+        <v>0</v>
+      </c>
+      <c r="AS2" cm="1" s="3">
+        <f t="array" ref="AS2">_xlfn.VSTACK('IV. MA'!$B$10:$D$17,'IV. MA'!$F$10:$H$17,'IV. MA'!$J$10:$L$17,'IV. MA'!$N$10:$P$17,'IV. MA'!$R$10:$T$17,'IV. MA'!$V$10:$X$17,'IV. MA'!$Z$10:$AB$17,'IV. MA'!$AD$10:$AF$17,'IV. MA'!$AH$10:$AJ$17,'IV. MA'!$AL$10:$AN$17,'IV. MA'!$AP$10:$AR$17,'IV. MA'!$AT$10:$AV$17,'IV. MA'!$AX$10:$AZ$17,'IV. MA'!$BB$10:$BD$17,'IV. MA'!$BF$10:$BH$17,'IV. MA'!$BJ$10:$BL$17,'IV. MA'!$BN$10:$BP$17,'IV. MA'!$BR$10:$BT$17)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
feat: add Auswertung sheet generation
Implement `CreateAuswertungSheet` to generate automated comparison tables
for funding requests and financial reports, utilizing structured spill
references instead of volatile ranges. Updated `main.go` to include this
sheet in the generator workflow.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -12,7 +12,8 @@
     <sheet name="II. KMW-Mittel" sheetId="4" r:id="rId7"/>
     <sheet name="III. Finanzberichte" sheetId="5" r:id="rId8"/>
     <sheet name="IV. MA" sheetId="6" r:id="rId9"/>
-    <sheet name="Daten" sheetId="7" r:id="rId10" state="hidden"/>
+    <sheet name="V. AUSWERTUNG" sheetId="7" r:id="rId10"/>
+    <sheet name="Daten" sheetId="8" r:id="rId11" state="hidden"/>
   </sheets>
   <definedNames>
     <definedName name="Saldovortrag_LW">'Dashboard'!$C$13</definedName>
@@ -147,7 +148,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="367">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1092,6 +1093,150 @@
   </si>
   <si>
     <t>abzueglich Saldo Vorperiode (FB):</t>
+  </si>
+  <si>
+    <t>V. AUSWERTUNG</t>
+  </si>
+  <si>
+    <t>Automatische Prüfung von Mittelanforderung und Finanzberichten</t>
+  </si>
+  <si>
+    <t>MITTELANFORDERUNGSPRÜFUNG</t>
+  </si>
+  <si>
+    <t>Basis: aktuelle Mittelanforderung</t>
+  </si>
+  <si>
+    <t>KMW-Mittelprüfung (Mittelanforderung)</t>
+  </si>
+  <si>
+    <t>Bewilligte KMW-Mittel</t>
+  </si>
+  <si>
+    <t>Davon Reserve</t>
+  </si>
+  <si>
+    <t>Operatives Budget (abzgl. Reserve)</t>
+  </si>
+  <si>
+    <t>Bereitgestellte KMW-Mittel</t>
+  </si>
+  <si>
+    <t>Verfügbare KMW-Mittel</t>
+  </si>
+  <si>
+    <t>Abzugsoptionen KMW-Mittel</t>
+  </si>
+  <si>
+    <t>− Saldovortrag</t>
+  </si>
+  <si>
+    <t>− Mehreinnahmen</t>
+  </si>
+  <si>
+    <t>Verfügbare KMW-Mittel (bereinigt)</t>
+  </si>
+  <si>
+    <t>Abzüglich aktuelle Anforderung</t>
+  </si>
+  <si>
+    <t>Verbleibende KMW-Mittel</t>
+  </si>
+  <si>
+    <t>Verbleibende KMW-Mittel (bereinigt)</t>
+  </si>
+  <si>
+    <t>Abzüglich manueller Betrag</t>
+  </si>
+  <si>
+    <t>Monatslimit-Prüfung (Lokalwährung)</t>
+  </si>
+  <si>
+    <t>Aktuelle Periode</t>
+  </si>
+  <si>
+    <t>Anforderungshöhe (LC)</t>
+  </si>
+  <si>
+    <t>Jahr</t>
+  </si>
+  <si>
+    <t>Jahresbudget (LC)</t>
+  </si>
+  <si>
+    <t>Limit-Monate</t>
+  </si>
+  <si>
+    <t>Bezugszeitraum (Monate)</t>
+  </si>
+  <si>
+    <t>Anforderung deckt (Monate)</t>
+  </si>
+  <si>
+    <t>8-Monats-Limit (LC)</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Überschreitung (LC)</t>
+  </si>
+  <si>
+    <t>Auslastung %</t>
+  </si>
+  <si>
+    <t>Prognostizierte Finanzierungsanteile</t>
+  </si>
+  <si>
+    <t>Kategorie</t>
+  </si>
+  <si>
+    <t>Prognose (LC)</t>
+  </si>
+  <si>
+    <t>Budget (LC)</t>
+  </si>
+  <si>
+    <t>Differenz (LC)</t>
+  </si>
+  <si>
+    <t>Abweichung (LC)</t>
+  </si>
+  <si>
+    <t>Prognose (EUR)</t>
+  </si>
+  <si>
+    <t>Budget (EUR)</t>
+  </si>
+  <si>
+    <t>Differenz (EUR)</t>
+  </si>
+  <si>
+    <t>Abweichung (EUR)</t>
+  </si>
+  <si>
+    <t>Prognoseprüfung (Ausgaben)</t>
+  </si>
+  <si>
+    <t>FINANZBERICHTSPRÜFUNG</t>
+  </si>
+  <si>
+    <t>Basis: aktuelle Finanzberichte</t>
+  </si>
+  <si>
+    <t>KMW-Mittelprüfung</t>
+  </si>
+  <si>
+    <t>Finanzierungsanteile</t>
+  </si>
+  <si>
+    <t>Kumulativ (LC)</t>
+  </si>
+  <si>
+    <t>Kumulativ (EUR)</t>
+  </si>
+  <si>
+    <t>Soll-Ist Abweichungsprüfung</t>
   </si>
   <si>
     <t>Einnahmen_Explizit_Stack</t>
@@ -1110,7 +1255,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <numFmts count="7">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
@@ -1118,8 +1263,10 @@
     <numFmt numFmtId="168" formatCode="0.000000"/>
     <numFmt numFmtId="169" formatCode="@"/>
     <numFmt numFmtId="170" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="171" formatCode="0"/>
+    <numFmt numFmtId="172" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1258,8 +1405,40 @@
       <color rgb="FF000000"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color rgb="FFB4BEC8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <color rgb="FF9C0006"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1311,8 +1490,13 @@
         <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF212F3D"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="51">
+  <borders count="53">
     <border>
       <left/>
       <right/>
@@ -1867,11 +2051,39 @@
         <color rgb="FF808080"/>
       </top>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="192">
+  <cellXfs count="276">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
@@ -2441,6 +2653,258 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="20" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="5" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="40" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
@@ -2450,7 +2914,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="14">
     <dxf>
       <font>
         <name val="Segoe UI"/>
@@ -2671,6 +3135,149 @@
         </top>
         <bottom style="medium">
           <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C640C"/>
+      </font>
+      <numFmt numFmtId="167" formatCode="0.0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCF3CF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD3D3D3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
         </bottom>
       </border>
     </dxf>
@@ -19067,6 +19674,1513 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr>
+    <tabColor rgb="FFFF00"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3"/>
+    <col customWidth="true" max="2" min="2" width="34"/>
+    <col customWidth="true" max="10" min="3" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="30" customHeight="true">
+      <c r="B2" s="191" t="s">
+        <v>315</v>
+      </c>
+      <c r="C2" s="191"/>
+      <c r="D2" s="191"/>
+      <c r="E2" s="191"/>
+      <c r="F2" s="191"/>
+      <c r="G2" s="191"/>
+      <c r="H2" s="191"/>
+      <c r="I2" s="191"/>
+      <c r="J2" s="191"/>
+    </row>
+    <row r="3" ht="18" customHeight="true">
+      <c r="B3" s="192" t="s">
+        <v>316</v>
+      </c>
+      <c r="C3" s="192"/>
+      <c r="D3" s="192"/>
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
+      <c r="H3" s="192"/>
+      <c r="I3" s="192"/>
+      <c r="J3" s="192"/>
+    </row>
+    <row r="5" ht="26" customHeight="true">
+      <c r="B5" s="193" t="s">
+        <v>317</v>
+      </c>
+      <c r="C5" s="193"/>
+      <c r="D5" s="193"/>
+      <c r="E5" s="193"/>
+      <c r="F5" s="193"/>
+      <c r="G5" s="193"/>
+      <c r="H5" s="193"/>
+      <c r="I5" s="193"/>
+      <c r="J5" s="193"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="194" t="s">
+        <v>318</v>
+      </c>
+      <c r="C6" s="194"/>
+      <c r="D6" s="194"/>
+      <c r="E6" s="194"/>
+      <c r="F6" s="194"/>
+      <c r="G6" s="194"/>
+      <c r="H6" s="194"/>
+      <c r="I6" s="194"/>
+      <c r="J6" s="194"/>
+    </row>
+    <row r="8" ht="22" customHeight="true">
+      <c r="B8" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="199" t="s">
+        <v>320</v>
+      </c>
+      <c r="C10" s="200"/>
+      <c r="D10" s="201" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
+      </c>
+      <c r="F10" s="207" t="s">
+        <v>325</v>
+      </c>
+      <c r="G10" s="208"/>
+      <c r="H10" s="209"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="202" t="s">
+        <v>321</v>
+      </c>
+      <c r="C11" s="195"/>
+      <c r="D11" s="203" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="F11" s="202" t="s">
+        <v>326</v>
+      </c>
+      <c r="G11" s="195"/>
+      <c r="H11" s="41" t="str">
+        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="202" t="s">
+        <v>322</v>
+      </c>
+      <c r="C12" s="195"/>
+      <c r="D12" s="203" t="str">
+        <f>=ROUND($D$10-$D$11,2)</f>
+      </c>
+      <c r="F12" s="202" t="s">
+        <v>327</v>
+      </c>
+      <c r="G12" s="195"/>
+      <c r="H12" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="202" t="s">
+        <v>323</v>
+      </c>
+      <c r="C13" s="195"/>
+      <c r="D13" s="203" t="str">
+        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
+      </c>
+      <c r="F13" s="47"/>
+      <c r="H13" s="48"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="204" t="s">
+        <v>324</v>
+      </c>
+      <c r="C14" s="205"/>
+      <c r="D14" s="206" t="str">
+        <f>=ROUND($D$12-$D$13,2)</f>
+      </c>
+      <c r="F14" s="204" t="s">
+        <v>328</v>
+      </c>
+      <c r="G14" s="205"/>
+      <c r="H14" s="206" t="str">
+        <f>=ROUND($D$14-MAX(0,$H$11)-MAX(0,$H$12),2)</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="199" t="s">
+        <v>329</v>
+      </c>
+      <c r="C16" s="200"/>
+      <c r="D16" s="211">
+        <v>0</v>
+      </c>
+      <c r="F16" s="199" t="s">
+        <v>329</v>
+      </c>
+      <c r="G16" s="200"/>
+      <c r="H16" s="211">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="204" t="s">
+        <v>330</v>
+      </c>
+      <c r="C17" s="205"/>
+      <c r="D17" s="206" t="str">
+        <f>=ROUND($D$14-MAX(0,$D$16),2)</f>
+      </c>
+      <c r="F17" s="204" t="s">
+        <v>331</v>
+      </c>
+      <c r="G17" s="205"/>
+      <c r="H17" s="206" t="str">
+        <f>=ROUND($H$14-MAX(0,$H$16),2)</f>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="199" t="s">
+        <v>332</v>
+      </c>
+      <c r="C19" s="200"/>
+      <c r="D19" s="211">
+        <v>0</v>
+      </c>
+      <c r="F19" s="199" t="s">
+        <v>332</v>
+      </c>
+      <c r="G19" s="200"/>
+      <c r="H19" s="211">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="204" t="s">
+        <v>330</v>
+      </c>
+      <c r="C20" s="205"/>
+      <c r="D20" s="206" t="str">
+        <f>=ROUND($D$14-MAX(0,$D$16)-MAX(0,$D$19),2)</f>
+      </c>
+      <c r="F20" s="204" t="s">
+        <v>331</v>
+      </c>
+      <c r="G20" s="205"/>
+      <c r="H20" s="206" t="str">
+        <f>=ROUND($H$14-MAX(0,$H$16)-MAX(0,$H$19),2)</f>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="true">
+      <c r="B23" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="199" t="s">
+        <v>334</v>
+      </c>
+      <c r="C25" s="200"/>
+      <c r="D25" s="217" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="202" t="s">
+        <v>335</v>
+      </c>
+      <c r="C26" s="195"/>
+      <c r="D26" s="218" t="str">
+        <f>=IFERROR(ROUND(SUBTOTAL(109,INDIRECT("MA_"&amp;VALUE(TRIM(MID($D$25,9,5)))&amp;"[Angefordert (LC)]")),2),0)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="202" t="s">
+        <v>336</v>
+      </c>
+      <c r="C27" s="195"/>
+      <c r="D27" s="219" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="202" t="s">
+        <v>337</v>
+      </c>
+      <c r="C28" s="195"/>
+      <c r="D28" s="218" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(MATCH($D$27,{"Jahr 1";"Jahr 2";"Jahr 3"},0),SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])),2),0)</f>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="202" t="s">
+        <v>338</v>
+      </c>
+      <c r="C29" s="195"/>
+      <c r="D29" s="220">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="202" t="s">
+        <v>339</v>
+      </c>
+      <c r="C30" s="195"/>
+      <c r="D30" s="221">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="202" t="s">
+        <v>340</v>
+      </c>
+      <c r="C31" s="195"/>
+      <c r="D31" s="222">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="223" t="s">
+        <v>341</v>
+      </c>
+      <c r="C32" s="197"/>
+      <c r="D32" s="224" t="str">
+        <f>=IFERROR(ROUND($D$28*$D$29/$D$30,2),0)</f>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="223" t="s">
+        <v>342</v>
+      </c>
+      <c r="C33" s="197"/>
+      <c r="D33" s="225" t="str">
+        <f>=IF($D$26&lt;=$D$32,"OK","ÜBERSCHRITTEN")</f>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="202" t="s">
+        <v>343</v>
+      </c>
+      <c r="C34" s="195"/>
+      <c r="D34" s="218" t="str">
+        <f>=ROUND(MAX(0,$D$26-$D$32),2)</f>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="226" t="s">
+        <v>344</v>
+      </c>
+      <c r="C35" s="227"/>
+      <c r="D35" s="228" t="str">
+        <f>=IFERROR($D$26/$D$32,0)</f>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="true">
+      <c r="B37" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
+      <c r="J37" s="18"/>
+    </row>
+    <row r="39" ht="28" customHeight="true">
+      <c r="B39" s="237" t="s">
+        <v>346</v>
+      </c>
+      <c r="C39" s="238" t="s">
+        <v>347</v>
+      </c>
+      <c r="D39" s="238" t="s">
+        <v>348</v>
+      </c>
+      <c r="E39" s="238" t="s">
+        <v>349</v>
+      </c>
+      <c r="F39" s="238" t="s">
+        <v>350</v>
+      </c>
+      <c r="G39" s="238" t="s">
+        <v>351</v>
+      </c>
+      <c r="H39" s="238" t="s">
+        <v>352</v>
+      </c>
+      <c r="I39" s="238" t="s">
+        <v>353</v>
+      </c>
+      <c r="J39" s="239" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="240" t="s">
+        <v>194</v>
+      </c>
+      <c r="C40" s="24">
+        <v>0</v>
+      </c>
+      <c r="D40" s="212" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
+      </c>
+      <c r="E40" s="230" t="str">
+        <f>=ROUND(IFERROR($C$40-$D$40,0),2)</f>
+      </c>
+      <c r="F40" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$40/$D$40)-1,0),4)</f>
+      </c>
+      <c r="G40" s="25">
+        <v>0</v>
+      </c>
+      <c r="H40" s="196" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
+      </c>
+      <c r="I40" s="181" t="str">
+        <f>=ROUND(IFERROR($G$40-$H$40,0),2)</f>
+      </c>
+      <c r="J40" s="241" t="str">
+        <f>=ROUND(IFERROR(($G$40/$H$40)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="240" t="s">
+        <v>277</v>
+      </c>
+      <c r="C41" s="24">
+        <v>0</v>
+      </c>
+      <c r="D41" s="212" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
+      </c>
+      <c r="E41" s="230" t="str">
+        <f>=ROUND(IFERROR($C$41-$D$41,0),2)</f>
+      </c>
+      <c r="F41" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$41/$D$41)-1,0),4)</f>
+      </c>
+      <c r="G41" s="25">
+        <v>0</v>
+      </c>
+      <c r="H41" s="196" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
+      </c>
+      <c r="I41" s="181" t="str">
+        <f>=ROUND(IFERROR($G$41-$H$41,0),2)</f>
+      </c>
+      <c r="J41" s="242" t="str">
+        <f>=ROUND(IFERROR(($G$41/$H$41)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="240" t="s">
+        <v>199</v>
+      </c>
+      <c r="C42" s="24">
+        <v>0</v>
+      </c>
+      <c r="D42" s="212" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
+      </c>
+      <c r="E42" s="230" t="str">
+        <f>=ROUND(IFERROR($C$42-$D$42,0),2)</f>
+      </c>
+      <c r="F42" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$42/$D$42)-1,0),4)</f>
+      </c>
+      <c r="G42" s="25">
+        <v>0</v>
+      </c>
+      <c r="H42" s="196" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
+      </c>
+      <c r="I42" s="181" t="str">
+        <f>=ROUND(IFERROR($G$42-$H$42,0),2)</f>
+      </c>
+      <c r="J42" s="243" t="str">
+        <f>=ROUND(IFERROR(($G$42/$H$42)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="240" t="s">
+        <v>278</v>
+      </c>
+      <c r="C43" s="232"/>
+      <c r="D43" s="232"/>
+      <c r="E43" s="232"/>
+      <c r="F43" s="232"/>
+      <c r="G43" s="232"/>
+      <c r="H43" s="232"/>
+      <c r="I43" s="232"/>
+      <c r="J43" s="244"/>
+    </row>
+    <row r="44" ht="20" customHeight="true">
+      <c r="B44" s="245" t="s">
+        <v>266</v>
+      </c>
+      <c r="C44" s="246" t="str">
+        <f>=ROUND(SUM($C$40:$C$43),2)</f>
+      </c>
+      <c r="D44" s="246" t="str">
+        <f>=ROUND(SUM($D$40:$D$43),2)</f>
+      </c>
+      <c r="E44" s="246" t="str">
+        <f>=ROUND(SUM($E$40:$E$43),2)</f>
+      </c>
+      <c r="F44" s="247" t="str">
+        <f>=ROUND(IFERROR(($C$44/$D$44)-1,0),4)</f>
+      </c>
+      <c r="G44" s="248" t="str">
+        <f>=ROUND(SUM($G$40:$G$43),2)</f>
+      </c>
+      <c r="H44" s="248" t="str">
+        <f>=ROUND(SUM($H$40:$H$43),2)</f>
+      </c>
+      <c r="I44" s="248" t="str">
+        <f>=ROUND(SUM($I$40:$I$43),2)</f>
+      </c>
+      <c r="J44" s="249" t="str">
+        <f>=ROUND(IFERROR(($G$44/$H$44)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="true">
+      <c r="B46" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="18"/>
+      <c r="J46" s="18"/>
+    </row>
+    <row r="48" ht="28" customHeight="true">
+      <c r="B48" s="237" t="s">
+        <v>346</v>
+      </c>
+      <c r="C48" s="238" t="s">
+        <v>347</v>
+      </c>
+      <c r="D48" s="238" t="s">
+        <v>348</v>
+      </c>
+      <c r="E48" s="238" t="s">
+        <v>349</v>
+      </c>
+      <c r="F48" s="238" t="s">
+        <v>350</v>
+      </c>
+      <c r="G48" s="238" t="s">
+        <v>351</v>
+      </c>
+      <c r="H48" s="238" t="s">
+        <v>352</v>
+      </c>
+      <c r="I48" s="238" t="s">
+        <v>353</v>
+      </c>
+      <c r="J48" s="239" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="240" t="s">
+        <v>205</v>
+      </c>
+      <c r="C49" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Bauausgaben",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D49" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
+      </c>
+      <c r="E49" s="230" t="str">
+        <f>=ROUND(IFERROR($C$49-$D$49,0),2)</f>
+      </c>
+      <c r="F49" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$49/$D$49)-1,0),4)</f>
+      </c>
+      <c r="G49" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Bauausgaben",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H49" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
+      </c>
+      <c r="I49" s="181" t="str">
+        <f>=ROUND(IFERROR($G$49-$H$49,0),2)</f>
+      </c>
+      <c r="J49" s="250" t="str">
+        <f>=ROUND(IFERROR(($G$49/$H$49)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="240" t="s">
+        <v>206</v>
+      </c>
+      <c r="C50" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Investitionen",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D50" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
+      </c>
+      <c r="E50" s="230" t="str">
+        <f>=ROUND(IFERROR($C$50-$D$50,0),2)</f>
+      </c>
+      <c r="F50" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$50/$D$50)-1,0),4)</f>
+      </c>
+      <c r="G50" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Investitionen",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H50" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
+      </c>
+      <c r="I50" s="181" t="str">
+        <f>=ROUND(IFERROR($G$50-$H$50,0),2)</f>
+      </c>
+      <c r="J50" s="251" t="str">
+        <f>=ROUND(IFERROR(($G$50/$H$50)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="240" t="s">
+        <v>207</v>
+      </c>
+      <c r="C51" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Personalkosten",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D51" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
+      </c>
+      <c r="E51" s="230" t="str">
+        <f>=ROUND(IFERROR($C$51-$D$51,0),2)</f>
+      </c>
+      <c r="F51" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$51/$D$51)-1,0),4)</f>
+      </c>
+      <c r="G51" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Personalkosten",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H51" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
+      </c>
+      <c r="I51" s="181" t="str">
+        <f>=ROUND(IFERROR($G$51-$H$51,0),2)</f>
+      </c>
+      <c r="J51" s="252" t="str">
+        <f>=ROUND(IFERROR(($G$51/$H$51)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="240" t="s">
+        <v>208</v>
+      </c>
+      <c r="C52" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Projektaktivitaeten",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D52" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
+      </c>
+      <c r="E52" s="230" t="str">
+        <f>=ROUND(IFERROR($C$52-$D$52,0),2)</f>
+      </c>
+      <c r="F52" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$52/$D$52)-1,0),4)</f>
+      </c>
+      <c r="G52" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Projektaktivitaeten",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H52" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
+      </c>
+      <c r="I52" s="181" t="str">
+        <f>=ROUND(IFERROR($G$52-$H$52,0),2)</f>
+      </c>
+      <c r="J52" s="253" t="str">
+        <f>=ROUND(IFERROR(($G$52/$H$52)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="240" t="s">
+        <v>209</v>
+      </c>
+      <c r="C53" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Projektverwaltung",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D53" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
+      </c>
+      <c r="E53" s="230" t="str">
+        <f>=ROUND(IFERROR($C$53-$D$53,0),2)</f>
+      </c>
+      <c r="F53" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$53/$D$53)-1,0),4)</f>
+      </c>
+      <c r="G53" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Projektverwaltung",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H53" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
+      </c>
+      <c r="I53" s="181" t="str">
+        <f>=ROUND(IFERROR($G$53-$H$53,0),2)</f>
+      </c>
+      <c r="J53" s="254" t="str">
+        <f>=ROUND(IFERROR(($G$53/$H$53)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="240" t="s">
+        <v>210</v>
+      </c>
+      <c r="C54" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Evaluierung",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D54" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
+      </c>
+      <c r="E54" s="230" t="str">
+        <f>=ROUND(IFERROR($C$54-$D$54,0),2)</f>
+      </c>
+      <c r="F54" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$54/$D$54)-1,0),4)</f>
+      </c>
+      <c r="G54" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Evaluierung",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H54" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+      </c>
+      <c r="I54" s="181" t="str">
+        <f>=ROUND(IFERROR($G$54-$H$54,0),2)</f>
+      </c>
+      <c r="J54" s="255" t="str">
+        <f>=ROUND(IFERROR(($G$54/$H$54)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="240" t="s">
+        <v>211</v>
+      </c>
+      <c r="C55" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Audit",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D55" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
+      </c>
+      <c r="E55" s="230" t="str">
+        <f>=ROUND(IFERROR($C$55-$D$55,0),2)</f>
+      </c>
+      <c r="F55" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$55/$D$55)-1,0),4)</f>
+      </c>
+      <c r="G55" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Audit",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H55" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+      </c>
+      <c r="I55" s="181" t="str">
+        <f>=ROUND(IFERROR($G$55-$H$55,0),2)</f>
+      </c>
+      <c r="J55" s="256" t="str">
+        <f>=ROUND(IFERROR(($G$55/$H$55)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="240" t="s">
+        <v>212</v>
+      </c>
+      <c r="C56" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Reserve",'Daten'!$V$2:$V$500),2)</f>
+      </c>
+      <c r="D56" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
+      </c>
+      <c r="E56" s="230" t="str">
+        <f>=ROUND(IFERROR($C$56-$D$56,0),2)</f>
+      </c>
+      <c r="F56" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$56/$D$56)-1,0),4)</f>
+      </c>
+      <c r="G56" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$U$2:$U$500,"Reserve",'Daten'!$W$2:$W$500),2)</f>
+      </c>
+      <c r="H56" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="I56" s="181" t="str">
+        <f>=ROUND(IFERROR($G$56-$H$56,0),2)</f>
+      </c>
+      <c r="J56" s="257" t="str">
+        <f>=ROUND(IFERROR(($G$56/$H$56)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="true">
+      <c r="B57" s="245" t="s">
+        <v>266</v>
+      </c>
+      <c r="C57" s="246" t="str">
+        <f>=ROUND(SUM($C$49:$C$56),2)</f>
+      </c>
+      <c r="D57" s="246" t="str">
+        <f>=ROUND(SUM($D$49:$D$56),2)</f>
+      </c>
+      <c r="E57" s="246" t="str">
+        <f>=ROUND(SUM($E$49:$E$56),2)</f>
+      </c>
+      <c r="F57" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$57/$D$57)-1,0),4)</f>
+      </c>
+      <c r="G57" s="248" t="str">
+        <f>=ROUND(SUM($G$49:$G$56),2)</f>
+      </c>
+      <c r="H57" s="248" t="str">
+        <f>=ROUND(SUM($H$49:$H$56),2)</f>
+      </c>
+      <c r="I57" s="248" t="str">
+        <f>=ROUND(SUM($I$49:$I$56),2)</f>
+      </c>
+      <c r="J57" s="259" t="str">
+        <f>=ROUND(IFERROR(($G$57/$H$57)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="59" ht="26" customHeight="true">
+      <c r="B59" s="193" t="s">
+        <v>356</v>
+      </c>
+      <c r="C59" s="193"/>
+      <c r="D59" s="193"/>
+      <c r="E59" s="193"/>
+      <c r="F59" s="193"/>
+      <c r="G59" s="193"/>
+      <c r="H59" s="193"/>
+      <c r="I59" s="193"/>
+      <c r="J59" s="193"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="194" t="s">
+        <v>357</v>
+      </c>
+      <c r="C60" s="194"/>
+      <c r="D60" s="194"/>
+      <c r="E60" s="194"/>
+      <c r="F60" s="194"/>
+      <c r="G60" s="194"/>
+      <c r="H60" s="194"/>
+      <c r="I60" s="194"/>
+      <c r="J60" s="194"/>
+    </row>
+    <row r="62" ht="22" customHeight="true">
+      <c r="B62" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="18"/>
+      <c r="I62" s="18"/>
+      <c r="J62" s="18"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="199" t="s">
+        <v>320</v>
+      </c>
+      <c r="C64" s="200"/>
+      <c r="D64" s="201" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
+      </c>
+      <c r="F64" s="207" t="s">
+        <v>325</v>
+      </c>
+      <c r="G64" s="208"/>
+      <c r="H64" s="209"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="202" t="s">
+        <v>321</v>
+      </c>
+      <c r="C65" s="195"/>
+      <c r="D65" s="203" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="F65" s="202" t="s">
+        <v>326</v>
+      </c>
+      <c r="G65" s="195"/>
+      <c r="H65" s="41" t="str">
+        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="202" t="s">
+        <v>322</v>
+      </c>
+      <c r="C66" s="195"/>
+      <c r="D66" s="203" t="str">
+        <f>=ROUND($D$64-$D$65,2)</f>
+      </c>
+      <c r="F66" s="202" t="s">
+        <v>327</v>
+      </c>
+      <c r="G66" s="195"/>
+      <c r="H66" s="196" t="str">
+        <f>=IFERROR(ROUND(MAX(0,(SUM($G$75:$G$78)-$G$77)-(SUM($H$75:$H$78)-$H$77)),2),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="202" t="s">
+        <v>323</v>
+      </c>
+      <c r="C67" s="195"/>
+      <c r="D67" s="203" t="str">
+        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
+      </c>
+      <c r="F67" s="47"/>
+      <c r="H67" s="48"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="204" t="s">
+        <v>324</v>
+      </c>
+      <c r="C68" s="205"/>
+      <c r="D68" s="206" t="str">
+        <f>=ROUND($D$66-$D$67,2)</f>
+      </c>
+      <c r="F68" s="204" t="s">
+        <v>328</v>
+      </c>
+      <c r="G68" s="205"/>
+      <c r="H68" s="206" t="str">
+        <f>=ROUND($D$68-MAX(0,$H$65)-MAX(0,$H$66),2)</f>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="true">
+      <c r="B72" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="C72" s="18"/>
+      <c r="D72" s="18"/>
+      <c r="E72" s="18"/>
+      <c r="F72" s="18"/>
+      <c r="G72" s="18"/>
+      <c r="H72" s="18"/>
+      <c r="I72" s="18"/>
+      <c r="J72" s="18"/>
+    </row>
+    <row r="74" ht="28" customHeight="true">
+      <c r="B74" s="237" t="s">
+        <v>346</v>
+      </c>
+      <c r="C74" s="238" t="s">
+        <v>360</v>
+      </c>
+      <c r="D74" s="238" t="s">
+        <v>348</v>
+      </c>
+      <c r="E74" s="238" t="s">
+        <v>349</v>
+      </c>
+      <c r="F74" s="238" t="s">
+        <v>350</v>
+      </c>
+      <c r="G74" s="238" t="s">
+        <v>361</v>
+      </c>
+      <c r="H74" s="238" t="s">
+        <v>352</v>
+      </c>
+      <c r="I74" s="238" t="s">
+        <v>353</v>
+      </c>
+      <c r="J74" s="239" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="240" t="s">
+        <v>194</v>
+      </c>
+      <c r="C75" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$C$2:$C$500,"Eigenmittel",'Daten'!$E$2:$E$500)+SUMIF('Daten'!$I$2:$I$500,"Eigenmittel",'Daten'!$K$2:$K$500),2)</f>
+      </c>
+      <c r="D75" s="212" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
+      </c>
+      <c r="E75" s="230" t="str">
+        <f>=ROUND(IFERROR($C$75-$D$75,0),2)</f>
+      </c>
+      <c r="F75" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$75/$D$75)-1,0),4)</f>
+      </c>
+      <c r="G75" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$C$2:$C$500,"Eigenmittel",'Daten'!$F$2:$F$500)+SUMIF('Daten'!$I$2:$I$500,"Eigenmittel",'Daten'!$L$2:$L$500),2)</f>
+      </c>
+      <c r="H75" s="196" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
+      </c>
+      <c r="I75" s="181" t="str">
+        <f>=ROUND(IFERROR($G$75-$H$75,0),2)</f>
+      </c>
+      <c r="J75" s="260" t="str">
+        <f>=ROUND(IFERROR(($G$75/$H$75)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="240" t="s">
+        <v>277</v>
+      </c>
+      <c r="C76" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$C$2:$C$500,"Drittmittel",'Daten'!$E$2:$E$500)+SUMIF('Daten'!$I$2:$I$500,"Drittmittel",'Daten'!$K$2:$K$500),2)</f>
+      </c>
+      <c r="D76" s="212" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
+      </c>
+      <c r="E76" s="230" t="str">
+        <f>=ROUND(IFERROR($C$76-$D$76,0),2)</f>
+      </c>
+      <c r="F76" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$76/$D$76)-1,0),4)</f>
+      </c>
+      <c r="G76" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$C$2:$C$500,"Drittmittel",'Daten'!$F$2:$F$500)+SUMIF('Daten'!$I$2:$I$500,"Drittmittel",'Daten'!$L$2:$L$500),2)</f>
+      </c>
+      <c r="H76" s="196" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
+      </c>
+      <c r="I76" s="181" t="str">
+        <f>=ROUND(IFERROR($G$76-$H$76,0),2)</f>
+      </c>
+      <c r="J76" s="261" t="str">
+        <f>=ROUND(IFERROR(($G$76/$H$76)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="240" t="s">
+        <v>199</v>
+      </c>
+      <c r="C77" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$C$2:$C$500,"KMW-Mittel",'Daten'!$E$2:$E$500)+SUMIF('Daten'!$I$2:$I$500,"KMW-Mittel",'Daten'!$K$2:$K$500),2)</f>
+      </c>
+      <c r="D77" s="212" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
+      </c>
+      <c r="E77" s="230" t="str">
+        <f>=ROUND(IFERROR($C$77-$D$77,0),2)</f>
+      </c>
+      <c r="F77" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$77/$D$77)-1,0),4)</f>
+      </c>
+      <c r="G77" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$C$2:$C$500,"KMW-Mittel",'Daten'!$F$2:$F$500)+SUMIF('Daten'!$I$2:$I$500,"KMW-Mittel",'Daten'!$L$2:$L$500),2)</f>
+      </c>
+      <c r="H77" s="196" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
+      </c>
+      <c r="I77" s="181" t="str">
+        <f>=ROUND(IFERROR($G$77-$H$77,0),2)</f>
+      </c>
+      <c r="J77" s="262" t="str">
+        <f>=ROUND(IFERROR(($G$77/$H$77)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="240" t="s">
+        <v>278</v>
+      </c>
+      <c r="C78" s="232"/>
+      <c r="D78" s="232"/>
+      <c r="E78" s="232"/>
+      <c r="F78" s="232"/>
+      <c r="G78" s="232"/>
+      <c r="H78" s="232"/>
+      <c r="I78" s="232"/>
+      <c r="J78" s="244"/>
+    </row>
+    <row r="79" ht="20" customHeight="true">
+      <c r="B79" s="245" t="s">
+        <v>266</v>
+      </c>
+      <c r="C79" s="246" t="str">
+        <f>=ROUND(SUM($C$75:$C$78),2)</f>
+      </c>
+      <c r="D79" s="246" t="str">
+        <f>=ROUND(SUM($D$75:$D$78),2)</f>
+      </c>
+      <c r="E79" s="246" t="str">
+        <f>=ROUND(SUM($E$75:$E$78),2)</f>
+      </c>
+      <c r="F79" s="263" t="str">
+        <f>=ROUND(IFERROR(($C$79/$D$79)-1,0),4)</f>
+      </c>
+      <c r="G79" s="248" t="str">
+        <f>=ROUND(SUM($G$75:$G$78),2)</f>
+      </c>
+      <c r="H79" s="248" t="str">
+        <f>=ROUND(SUM($H$75:$H$78),2)</f>
+      </c>
+      <c r="I79" s="248" t="str">
+        <f>=ROUND(SUM($I$75:$I$78),2)</f>
+      </c>
+      <c r="J79" s="264" t="str">
+        <f>=ROUND(IFERROR(($G$79/$H$79)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="true">
+      <c r="B81" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="C81" s="18"/>
+      <c r="D81" s="18"/>
+      <c r="E81" s="18"/>
+      <c r="F81" s="18"/>
+      <c r="G81" s="18"/>
+      <c r="H81" s="18"/>
+      <c r="I81" s="18"/>
+      <c r="J81" s="18"/>
+    </row>
+    <row r="83" ht="28" customHeight="true">
+      <c r="B83" s="237" t="s">
+        <v>346</v>
+      </c>
+      <c r="C83" s="238" t="s">
+        <v>360</v>
+      </c>
+      <c r="D83" s="238" t="s">
+        <v>348</v>
+      </c>
+      <c r="E83" s="238" t="s">
+        <v>349</v>
+      </c>
+      <c r="F83" s="238" t="s">
+        <v>350</v>
+      </c>
+      <c r="G83" s="238" t="s">
+        <v>361</v>
+      </c>
+      <c r="H83" s="238" t="s">
+        <v>352</v>
+      </c>
+      <c r="I83" s="238" t="s">
+        <v>353</v>
+      </c>
+      <c r="J83" s="239" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="240" t="s">
+        <v>205</v>
+      </c>
+      <c r="C84" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"1.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D84" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
+      </c>
+      <c r="E84" s="230" t="str">
+        <f>=ROUND(IFERROR($C$84-$D$84,0),2)</f>
+      </c>
+      <c r="F84" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$84/$D$84)-1,0),4)</f>
+      </c>
+      <c r="G84" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"1.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H84" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
+      </c>
+      <c r="I84" s="181" t="str">
+        <f>=ROUND(IFERROR($G$84-$H$84,0),2)</f>
+      </c>
+      <c r="J84" s="265" t="str">
+        <f>=ROUND(IFERROR(($G$84/$H$84)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="240" t="s">
+        <v>206</v>
+      </c>
+      <c r="C85" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"2.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D85" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
+      </c>
+      <c r="E85" s="230" t="str">
+        <f>=ROUND(IFERROR($C$85-$D$85,0),2)</f>
+      </c>
+      <c r="F85" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$85/$D$85)-1,0),4)</f>
+      </c>
+      <c r="G85" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"2.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H85" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
+      </c>
+      <c r="I85" s="181" t="str">
+        <f>=ROUND(IFERROR($G$85-$H$85,0),2)</f>
+      </c>
+      <c r="J85" s="266" t="str">
+        <f>=ROUND(IFERROR(($G$85/$H$85)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="240" t="s">
+        <v>207</v>
+      </c>
+      <c r="C86" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"3.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D86" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
+      </c>
+      <c r="E86" s="230" t="str">
+        <f>=ROUND(IFERROR($C$86-$D$86,0),2)</f>
+      </c>
+      <c r="F86" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$86/$D$86)-1,0),4)</f>
+      </c>
+      <c r="G86" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"3.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H86" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
+      </c>
+      <c r="I86" s="181" t="str">
+        <f>=ROUND(IFERROR($G$86-$H$86,0),2)</f>
+      </c>
+      <c r="J86" s="267" t="str">
+        <f>=ROUND(IFERROR(($G$86/$H$86)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="240" t="s">
+        <v>208</v>
+      </c>
+      <c r="C87" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"4.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D87" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
+      </c>
+      <c r="E87" s="230" t="str">
+        <f>=ROUND(IFERROR($C$87-$D$87,0),2)</f>
+      </c>
+      <c r="F87" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$87/$D$87)-1,0),4)</f>
+      </c>
+      <c r="G87" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"4.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H87" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
+      </c>
+      <c r="I87" s="181" t="str">
+        <f>=ROUND(IFERROR($G$87-$H$87,0),2)</f>
+      </c>
+      <c r="J87" s="268" t="str">
+        <f>=ROUND(IFERROR(($G$87/$H$87)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="240" t="s">
+        <v>209</v>
+      </c>
+      <c r="C88" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"5.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D88" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
+      </c>
+      <c r="E88" s="230" t="str">
+        <f>=ROUND(IFERROR($C$88-$D$88,0),2)</f>
+      </c>
+      <c r="F88" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$88/$D$88)-1,0),4)</f>
+      </c>
+      <c r="G88" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"5.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H88" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
+      </c>
+      <c r="I88" s="181" t="str">
+        <f>=ROUND(IFERROR($G$88-$H$88,0),2)</f>
+      </c>
+      <c r="J88" s="269" t="str">
+        <f>=ROUND(IFERROR(($G$88/$H$88)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="240" t="s">
+        <v>210</v>
+      </c>
+      <c r="C89" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"6.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D89" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
+      </c>
+      <c r="E89" s="230" t="str">
+        <f>=ROUND(IFERROR($C$89-$D$89,0),2)</f>
+      </c>
+      <c r="F89" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$89/$D$89)-1,0),4)</f>
+      </c>
+      <c r="G89" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"6.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H89" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+      </c>
+      <c r="I89" s="181" t="str">
+        <f>=ROUND(IFERROR($G$89-$H$89,0),2)</f>
+      </c>
+      <c r="J89" s="270" t="str">
+        <f>=ROUND(IFERROR(($G$89/$H$89)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="240" t="s">
+        <v>211</v>
+      </c>
+      <c r="C90" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"7.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D90" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
+      </c>
+      <c r="E90" s="230" t="str">
+        <f>=ROUND(IFERROR($C$90-$D$90,0),2)</f>
+      </c>
+      <c r="F90" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$90/$D$90)-1,0),4)</f>
+      </c>
+      <c r="G90" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"7.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H90" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+      </c>
+      <c r="I90" s="181" t="str">
+        <f>=ROUND(IFERROR($G$90-$H$90,0),2)</f>
+      </c>
+      <c r="J90" s="271" t="str">
+        <f>=ROUND(IFERROR(($G$90/$H$90)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="240" t="s">
+        <v>212</v>
+      </c>
+      <c r="C91" s="212" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"8.*",'Daten'!$P$2:$P$500),2)</f>
+      </c>
+      <c r="D91" s="212" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
+      </c>
+      <c r="E91" s="230" t="str">
+        <f>=ROUND(IFERROR($C$91-$D$91,0),2)</f>
+      </c>
+      <c r="F91" s="231" t="str">
+        <f>=ROUND(IFERROR(($C$91/$D$91)-1,0),4)</f>
+      </c>
+      <c r="G91" s="196" t="str">
+        <f>=ROUND(SUMIF('Daten'!$O$2:$O$500,"8.*",'Daten'!$Q$2:$Q$500),2)</f>
+      </c>
+      <c r="H91" s="196" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="I91" s="181" t="str">
+        <f>=ROUND(IFERROR($G$91-$H$91,0),2)</f>
+      </c>
+      <c r="J91" s="272" t="str">
+        <f>=ROUND(IFERROR(($G$91/$H$91)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="true">
+      <c r="B92" s="245" t="s">
+        <v>266</v>
+      </c>
+      <c r="C92" s="246" t="str">
+        <f>=ROUND(SUM($C$84:$C$91),2)</f>
+      </c>
+      <c r="D92" s="246" t="str">
+        <f>=ROUND(SUM($D$84:$D$91),2)</f>
+      </c>
+      <c r="E92" s="246" t="str">
+        <f>=ROUND(SUM($E$84:$E$91),2)</f>
+      </c>
+      <c r="F92" s="273" t="str">
+        <f>=ROUND(IFERROR(($C$92/$D$92)-1,0),4)</f>
+      </c>
+      <c r="G92" s="248" t="str">
+        <f>=ROUND(SUM($G$84:$G$91),2)</f>
+      </c>
+      <c r="H92" s="248" t="str">
+        <f>=ROUND(SUM($H$84:$H$91),2)</f>
+      </c>
+      <c r="I92" s="248" t="str">
+        <f>=ROUND(SUM($I$84:$I$91),2)</f>
+      </c>
+      <c r="J92" s="274" t="str">
+        <f>=ROUND(IFERROR(($G$92/$H$92)-1,0),4)</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="50">
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="B46:J46"/>
+    <mergeCell ref="B59:J59"/>
+    <mergeCell ref="B60:J60"/>
+    <mergeCell ref="B62:J62"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="F64:H64"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="B72:J72"/>
+    <mergeCell ref="B81:J81"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D33">
+    <cfRule type="expression" dxfId="9" priority="1">
+      <formula>$D$33="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D33">
+    <cfRule type="expression" dxfId="10" priority="2">
+      <formula>$D$33&lt;&gt;"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D34">
+    <cfRule type="expression" dxfId="11" priority="3">
+      <formula>$D$34&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F49:F56">
+    <cfRule type="expression" dxfId="12" priority="4">
+      <formula>F49&gt;0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F49:F56">
+    <cfRule type="expression" dxfId="13" priority="5">
+      <formula>AND(F49&gt;=0.1,F49&lt;=0.2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J49:J56">
+    <cfRule type="expression" dxfId="12" priority="6">
+      <formula>J49&gt;0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J49:J56">
+    <cfRule type="expression" dxfId="13" priority="7">
+      <formula>AND(J49&gt;=0.1,J49&lt;=0.2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F84:F91">
+    <cfRule type="expression" dxfId="12" priority="8">
+      <formula>F84&gt;0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F84:F91">
+    <cfRule type="expression" dxfId="13" priority="9">
+      <formula>AND(F84&gt;=0.1,F84&lt;=0.2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J84:J91">
+    <cfRule type="expression" dxfId="12" priority="10">
+      <formula>J84&gt;0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J84:J91">
+    <cfRule type="expression" dxfId="13" priority="11">
+      <formula>AND(J84&gt;=0.1,J84&lt;=0.2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" sqref="D25" type="list">
+      <formula1>'Daten'!$A$1:$A$18</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="true" sqref="D27" type="list">
+      <formula1>"Jahr 1,Jahr 2,Jahr 3"</formula1>
+    </dataValidation>
+  </dataValidations>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -19074,17 +21188,17 @@
       <c r="A1" t="s">
         <v>226</v>
       </c>
-      <c r="C1" s="191" t="s">
-        <v>315</v>
-      </c>
-      <c r="I1" s="191" t="s">
-        <v>316</v>
-      </c>
-      <c r="O1" s="191" t="s">
-        <v>317</v>
-      </c>
-      <c r="U1" s="191" t="s">
-        <v>318</v>
+      <c r="C1" s="275" t="s">
+        <v>363</v>
+      </c>
+      <c r="I1" s="275" t="s">
+        <v>364</v>
+      </c>
+      <c r="O1" s="275" t="s">
+        <v>365</v>
+      </c>
+      <c r="U1" s="275" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
refactor: redesign selection panels for MA and FB
Migrate selection panels to a centered layout (spanning columns C to I)
and consolidate helper methods for improved readability and maintenance.
Update the FB selection list to include a project start option.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="378">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1112,10 +1112,13 @@
     <t>Mittelanforderung auswählen</t>
   </si>
   <si>
-    <t>Periode (FB+1)</t>
-  </si>
-  <si>
-    <t>Ausgewählt (#)</t>
+    <t>Auswahl:</t>
+  </si>
+  <si>
+    <t>Geprüfte Periode (FB+1)</t>
+  </si>
+  <si>
+    <t>Ausgewählte Anforderung (#)</t>
   </si>
   <si>
     <t>Einbezogene Anforderungen</t>
@@ -1250,7 +1253,7 @@
     <t>Finanzbericht auswählen</t>
   </si>
   <si>
-    <t>Periode (N)</t>
+    <t>Geprüfte Periode (N)</t>
   </si>
   <si>
     <t>Saldo (LC)</t>
@@ -1298,7 +1301,7 @@
     <numFmt numFmtId="171" formatCode="0"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1450,6 +1453,13 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -2122,7 +2132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="296">
+  <cellXfs count="304">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
@@ -2709,14 +2719,20 @@
     <xf numFmtId="0" fontId="23" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -2727,81 +2743,105 @@
     <xf numFmtId="0" fontId="23" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="12" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="12" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="12" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="12" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="167" fontId="3" fillId="5" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2856,34 +2896,31 @@
     <xf numFmtId="172" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="172" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -2901,19 +2938,19 @@
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -2940,24 +2977,21 @@
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="3" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2970,10 +3004,10 @@
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3000,10 +3034,10 @@
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
@@ -3241,6 +3275,33 @@
       <font>
         <name val="Segoe UI"/>
         <family val="2"/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD6EAF8"/>
+        </patternFill>
+      </fill>
+      <alignment/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
         <b val="1"/>
         <color rgb="FF006100"/>
       </font>
@@ -3377,33 +3438,6 @@
         </top>
         <bottom style="thin">
           <color rgb="FFD3D3D3"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <color rgb="FF000000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFD6EAF8"/>
-        </patternFill>
-      </fill>
-      <alignment/>
-      <border>
-        <left style="thin">
-          <color rgb="FF808080"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF808080"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF808080"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF808080"/>
         </bottom>
       </border>
     </dxf>
@@ -19810,10 +19844,6 @@
     <col customWidth="true" max="1" min="1" width="3"/>
     <col customWidth="true" max="2" min="2" width="34"/>
     <col customWidth="true" max="10" min="3" width="16"/>
-    <col customWidth="true" max="11" min="11" width="3"/>
-    <col customWidth="true" max="12" min="12" width="20"/>
-    <col customWidth="true" max="13" min="13" width="10"/>
-    <col customWidth="true" max="15" min="14" width="16"/>
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="true">
@@ -19869,1711 +19899,1820 @@
       <c r="J6" s="194"/>
     </row>
     <row r="8" ht="22" customHeight="true">
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="201" t="s">
+        <v>319</v>
+      </c>
+      <c r="D8" s="202"/>
+      <c r="E8" s="202"/>
+      <c r="F8" s="202"/>
+      <c r="G8" s="202"/>
+      <c r="H8" s="202"/>
+      <c r="I8" s="203"/>
+    </row>
+    <row r="9">
+      <c r="C9" s="204" t="s">
+        <v>320</v>
+      </c>
+      <c r="D9" s="196"/>
+      <c r="E9" s="196"/>
+      <c r="F9" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="205"/>
+    </row>
+    <row r="10">
+      <c r="C10" s="204" t="s">
+        <v>321</v>
+      </c>
+      <c r="D10" s="196"/>
+      <c r="E10" s="196"/>
+      <c r="F10" s="197" t="str">
+        <f>=F77+1</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="197"/>
+      <c r="H10" s="197"/>
+      <c r="I10" s="206"/>
+    </row>
+    <row r="11">
+      <c r="C11" s="204" t="s">
+        <v>322</v>
+      </c>
+      <c r="D11" s="196"/>
+      <c r="E11" s="196"/>
+      <c r="F11" s="197" t="str">
+        <f>=IFERROR(VALUE(MID(F9,FIND("(#",F9)+2,FIND(")",F9)-FIND("(#",F9)-2)),0)</f>
+      </c>
+      <c r="G11" s="197"/>
+      <c r="H11" s="197"/>
+      <c r="I11" s="207"/>
+    </row>
+    <row r="12">
+      <c r="C12" s="208" t="s">
         <v>323</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="L8" s="199" t="s">
-        <v>319</v>
-      </c>
-      <c r="M8" s="200"/>
-      <c r="N8" s="200"/>
-      <c r="O8" s="201"/>
-    </row>
-    <row r="9">
-      <c r="L9" s="202" t="s">
-        <v>158</v>
-      </c>
-      <c r="M9" s="33"/>
-      <c r="N9" s="33"/>
-      <c r="O9" s="203"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="216" t="s">
+      <c r="D12" s="198"/>
+      <c r="E12" s="198"/>
+      <c r="F12" s="198"/>
+      <c r="G12" s="198"/>
+      <c r="H12" s="198"/>
+      <c r="I12" s="209"/>
+    </row>
+    <row r="13">
+      <c r="C13" s="210" t="str">
+        <f>=IF(1&lt;=F11,"Periode "&amp;F10&amp;" (#1)","")</f>
+      </c>
+      <c r="D13" s="199"/>
+      <c r="E13" s="199"/>
+      <c r="F13" s="200" t="str">
+        <f>=IF(1&lt;=F11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
+      </c>
+      <c r="G13" s="200"/>
+      <c r="H13" s="181" t="str">
+        <f>=IF(1&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
+      </c>
+      <c r="I13" s="211"/>
+    </row>
+    <row r="14">
+      <c r="C14" s="210" t="str">
+        <f>=IF(2&lt;=F11,"Periode "&amp;F10&amp;" (#2)","")</f>
+      </c>
+      <c r="D14" s="199"/>
+      <c r="E14" s="199"/>
+      <c r="F14" s="200" t="str">
+        <f>=IF(2&lt;=F11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
+      </c>
+      <c r="G14" s="200"/>
+      <c r="H14" s="181" t="str">
+        <f>=IF(2&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
+      </c>
+      <c r="I14" s="211"/>
+    </row>
+    <row r="15">
+      <c r="C15" s="210" t="str">
+        <f>=IF(3&lt;=F11,"Periode "&amp;F10&amp;" (#3)","")</f>
+      </c>
+      <c r="D15" s="199"/>
+      <c r="E15" s="199"/>
+      <c r="F15" s="200" t="str">
+        <f>=IF(3&lt;=F11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
+      </c>
+      <c r="G15" s="200"/>
+      <c r="H15" s="181" t="str">
+        <f>=IF(3&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
+      </c>
+      <c r="I15" s="211"/>
+    </row>
+    <row r="16">
+      <c r="C16" s="210" t="str">
+        <f>=IF(4&lt;=F11,"Periode "&amp;F10&amp;" (#4)","")</f>
+      </c>
+      <c r="D16" s="199"/>
+      <c r="E16" s="199"/>
+      <c r="F16" s="200" t="str">
+        <f>=IF(4&lt;=F11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
+      </c>
+      <c r="G16" s="200"/>
+      <c r="H16" s="181" t="str">
+        <f>=IF(4&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
+      </c>
+      <c r="I16" s="211"/>
+    </row>
+    <row r="17">
+      <c r="C17" s="210" t="str">
+        <f>=IF(5&lt;=F11,"Periode "&amp;F10&amp;" (#5)","")</f>
+      </c>
+      <c r="D17" s="199"/>
+      <c r="E17" s="199"/>
+      <c r="F17" s="200" t="str">
+        <f>=IF(5&lt;=F11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
+      </c>
+      <c r="G17" s="200"/>
+      <c r="H17" s="181" t="str">
+        <f>=IF(5&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
+      </c>
+      <c r="I17" s="211"/>
+    </row>
+    <row r="18">
+      <c r="C18" s="212" t="str">
+        <f>=IF(6&lt;=F11,"Periode "&amp;F10&amp;" (#6)","")</f>
+      </c>
+      <c r="D18" s="213"/>
+      <c r="E18" s="213"/>
+      <c r="F18" s="214" t="str">
+        <f>=IF(6&lt;=F11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
+      </c>
+      <c r="G18" s="214"/>
+      <c r="H18" s="215" t="str">
+        <f>=IF(6&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
+      </c>
+      <c r="I18" s="216"/>
+    </row>
+    <row r="20" ht="22" customHeight="true">
+      <c r="B20" s="18" t="s">
         <v>324</v>
       </c>
-      <c r="C10" s="217"/>
-      <c r="D10" s="218" t="str">
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="223" t="s">
+        <v>325</v>
+      </c>
+      <c r="C22" s="224"/>
+      <c r="D22" s="225" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
-      <c r="F10" s="199" t="s">
+      <c r="F22" s="230" t="s">
+        <v>330</v>
+      </c>
+      <c r="G22" s="231"/>
+      <c r="H22" s="231"/>
+      <c r="I22" s="232"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="204" t="s">
+        <v>326</v>
+      </c>
+      <c r="C23" s="196"/>
+      <c r="D23" s="226" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="F23" s="233" t="s">
+        <v>331</v>
+      </c>
+      <c r="G23" s="196" t="s">
+        <v>332</v>
+      </c>
+      <c r="H23" s="196"/>
+      <c r="I23" s="234" t="str">
+        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="204" t="s">
+        <v>327</v>
+      </c>
+      <c r="C24" s="196"/>
+      <c r="D24" s="226" t="str">
+        <f>=ROUND($D$22-$D$23,2)</f>
+      </c>
+      <c r="F24" s="233" t="s">
+        <v>331</v>
+      </c>
+      <c r="G24" s="196" t="s">
+        <v>333</v>
+      </c>
+      <c r="H24" s="196"/>
+      <c r="I24" s="222" t="str">
+        <f>=I85</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="204" t="s">
+        <v>328</v>
+      </c>
+      <c r="C25" s="196"/>
+      <c r="D25" s="226" t="str">
+        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
+      </c>
+      <c r="F25" s="233" t="s">
+        <v>331</v>
+      </c>
+      <c r="G25" s="196" t="s">
+        <v>334</v>
+      </c>
+      <c r="H25" s="196"/>
+      <c r="I25" s="222" t="str">
+        <f>=ROUND(MAX(0,MAX(0,(SUM($G$94:$G$97)-$G$96)+SUMIFS('Daten'!$BH$1:$BH$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;F11,'Daten'!$BD$1:$BD$18,"&gt;=1")-(SUM($H$94:$H$97)-$H$96))-I85),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="227" t="s">
         <v>329</v>
       </c>
-      <c r="G10" s="200"/>
-      <c r="H10" s="200"/>
-      <c r="I10" s="201"/>
-      <c r="L10" s="204" t="s">
-        <v>320</v>
-      </c>
-      <c r="M10" s="196"/>
-      <c r="N10" s="275" t="str">
-        <f>=N65+1</f>
+      <c r="C26" s="228"/>
+      <c r="D26" s="229" t="str">
+        <f>=ROUND($D$24-$D$25,2)</f>
+      </c>
+      <c r="F26" s="47"/>
+      <c r="G26" s="218" t="s">
+        <v>335</v>
+      </c>
+      <c r="H26" s="218"/>
+      <c r="I26" s="235" t="str">
+        <f>=ROUND(IF($F$23="Abzug",MAX(0,$I$23),0)+IF($F$24="Abzug",MAX(0,$I$24),0)+IF($F$25="Abzug",MAX(0,$I$25),0),2)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="F27" s="236"/>
+      <c r="G27" s="228" t="s">
+        <v>336</v>
+      </c>
+      <c r="H27" s="228"/>
+      <c r="I27" s="229" t="str">
+        <f>=ROUND($D$26-$I$26,2)</f>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="223" t="s">
+        <v>337</v>
+      </c>
+      <c r="C29" s="224"/>
+      <c r="D29" s="237">
         <v>0</v>
       </c>
-      <c r="O10" s="205"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="219" t="s">
-        <v>325</v>
-      </c>
-      <c r="C11" s="210"/>
-      <c r="D11" s="220" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
-      </c>
-      <c r="F11" s="224" t="s">
-        <v>330</v>
-      </c>
-      <c r="G11" s="210" t="s">
-        <v>331</v>
-      </c>
-      <c r="H11" s="210"/>
-      <c r="I11" s="225" t="str">
-        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
-      </c>
-      <c r="L11" s="204" t="s">
-        <v>321</v>
-      </c>
-      <c r="M11" s="196"/>
-      <c r="N11" s="197" t="str">
-        <f>=IFERROR(VALUE(MID(L9,FIND("(#",L9)+2,FIND(")",L9)-FIND("(#",L9)-2)),0)</f>
-      </c>
-      <c r="O11" s="206"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="219" t="s">
-        <v>326</v>
-      </c>
-      <c r="C12" s="210"/>
-      <c r="D12" s="220" t="str">
-        <f>=ROUND($D$10-$D$11,2)</f>
-      </c>
-      <c r="F12" s="224" t="s">
-        <v>330</v>
-      </c>
-      <c r="G12" s="210" t="s">
-        <v>332</v>
-      </c>
-      <c r="H12" s="210"/>
-      <c r="I12" s="215" t="str">
-        <f>=I67</f>
+      <c r="F29" s="223" t="s">
+        <v>337</v>
+      </c>
+      <c r="G29" s="224"/>
+      <c r="H29" s="224"/>
+      <c r="I29" s="237">
         <v>0</v>
       </c>
-      <c r="L12" s="207" t="s">
-        <v>322</v>
-      </c>
-      <c r="M12" s="198"/>
-      <c r="N12" s="198"/>
-      <c r="O12" s="208"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="219" t="s">
-        <v>327</v>
-      </c>
-      <c r="C13" s="210"/>
-      <c r="D13" s="220" t="str">
-        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
-      </c>
-      <c r="F13" s="224" t="s">
-        <v>330</v>
-      </c>
-      <c r="G13" s="210" t="s">
-        <v>333</v>
-      </c>
-      <c r="H13" s="210"/>
-      <c r="I13" s="215" t="str">
-        <f>=ROUND(MAX(0,MAX(0,(SUM($G$76:$G$79)-$G$78)+SUMIFS('Daten'!$BH$1:$BH$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;N11,'Daten'!$BD$1:$BD$18,"&gt;=1")-(SUM($H$76:$H$79)-$H$78))-I67),2)</f>
+    </row>
+    <row r="30">
+      <c r="B30" s="227" t="s">
+        <v>338</v>
+      </c>
+      <c r="C30" s="228"/>
+      <c r="D30" s="229" t="str">
+        <f>=ROUND($D$26-MAX(0,$D$29),2)</f>
+      </c>
+      <c r="F30" s="227" t="s">
+        <v>339</v>
+      </c>
+      <c r="G30" s="228"/>
+      <c r="H30" s="228"/>
+      <c r="I30" s="229" t="str">
+        <f>=ROUND($I$27-MAX(0,$I$29),2)</f>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="223" t="s">
+        <v>340</v>
+      </c>
+      <c r="C32" s="224"/>
+      <c r="D32" s="237">
         <v>0</v>
       </c>
-      <c r="L13" s="196" t="str">
-        <f>=IF(1&lt;=N11,"Periode "&amp;N10&amp;" (#1)","")</f>
-      </c>
-      <c r="N13" s="246" t="str">
-        <f>=IF(1&lt;=N11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
-      </c>
-      <c r="O13" s="48"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="221" t="s">
-        <v>328</v>
-      </c>
-      <c r="C14" s="222"/>
-      <c r="D14" s="223" t="str">
-        <f>=ROUND($D$12-$D$13,2)</f>
-      </c>
-      <c r="F14" s="47"/>
-      <c r="G14" s="212" t="s">
-        <v>334</v>
-      </c>
-      <c r="H14" s="212"/>
-      <c r="I14" s="226" t="str">
-        <f>=ROUND(IF($F$11="Abzug",MAX(0,$I$11),0)+IF($F$12="Abzug",MAX(0,$I$12),0)+IF($F$13="Abzug",MAX(0,$I$13),0),2)</f>
-      </c>
-      <c r="L14" s="196" t="str">
-        <f>=IF(2&lt;=N11,"Periode "&amp;N10&amp;" (#2)","")</f>
-      </c>
-      <c r="N14" s="246" t="str">
-        <f>=IF(2&lt;=N11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
-      </c>
-      <c r="O14" s="48"/>
-    </row>
-    <row r="15">
-      <c r="F15" s="209"/>
-      <c r="G15" s="222" t="s">
-        <v>335</v>
-      </c>
-      <c r="H15" s="222"/>
-      <c r="I15" s="223" t="str">
-        <f>=ROUND($D$14-$I$14,2)</f>
-      </c>
-      <c r="L15" s="196" t="str">
-        <f>=IF(3&lt;=N11,"Periode "&amp;N10&amp;" (#3)","")</f>
-      </c>
-      <c r="N15" s="246" t="str">
-        <f>=IF(3&lt;=N11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
-      </c>
-      <c r="O15" s="48"/>
-    </row>
-    <row r="16">
-      <c r="L16" s="196" t="str">
-        <f>=IF(4&lt;=N11,"Periode "&amp;N10&amp;" (#4)","")</f>
-      </c>
-      <c r="N16" s="246" t="str">
-        <f>=IF(4&lt;=N11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
-      </c>
-      <c r="O16" s="48"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="216" t="s">
-        <v>336</v>
-      </c>
-      <c r="C17" s="217"/>
-      <c r="D17" s="227">
+      <c r="F32" s="223" t="s">
+        <v>340</v>
+      </c>
+      <c r="G32" s="224"/>
+      <c r="H32" s="224"/>
+      <c r="I32" s="237">
         <v>0</v>
       </c>
-      <c r="G17" s="216" t="s">
-        <v>336</v>
-      </c>
-      <c r="H17" s="217"/>
-      <c r="I17" s="227">
+    </row>
+    <row r="33">
+      <c r="B33" s="227" t="s">
+        <v>338</v>
+      </c>
+      <c r="C33" s="228"/>
+      <c r="D33" s="229" t="str">
+        <f>=ROUND($D$26-MAX(0,$D$29)-MAX(0,$D$32),2)</f>
+      </c>
+      <c r="F33" s="227" t="s">
+        <v>339</v>
+      </c>
+      <c r="G33" s="228"/>
+      <c r="H33" s="228"/>
+      <c r="I33" s="229" t="str">
+        <f>=ROUND($I$27-MAX(0,$I$29)-MAX(0,$I$32),2)</f>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="true">
+      <c r="B36" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="18"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="223" t="s">
+        <v>342</v>
+      </c>
+      <c r="C38" s="224"/>
+      <c r="D38" s="244" t="str">
+        <f>=F10</f>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="204" t="s">
+        <v>343</v>
+      </c>
+      <c r="C39" s="196"/>
+      <c r="D39" s="245" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;F11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="204" t="s">
+        <v>344</v>
+      </c>
+      <c r="C40" s="196"/>
+      <c r="D40" s="205" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="204" t="s">
+        <v>345</v>
+      </c>
+      <c r="C41" s="196"/>
+      <c r="D41" s="245" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(MATCH($D$40,{"Jahr 1";"Jahr 2";"Jahr 3"},0),SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])),2),0)</f>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="204" t="s">
+        <v>346</v>
+      </c>
+      <c r="C42" s="196"/>
+      <c r="D42" s="246">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="204" t="s">
+        <v>347</v>
+      </c>
+      <c r="C43" s="196"/>
+      <c r="D43" s="247">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="204" t="s">
+        <v>348</v>
+      </c>
+      <c r="C44" s="196"/>
+      <c r="D44" s="248">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="249" t="s">
+        <v>349</v>
+      </c>
+      <c r="C45" s="218"/>
+      <c r="D45" s="250" t="str">
+        <f>=IFERROR(ROUND($D$41*$D$42/$D$43,2),0)</f>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="249" t="s">
+        <v>350</v>
+      </c>
+      <c r="C46" s="218"/>
+      <c r="D46" s="251" t="str">
+        <f>=IF($D$39&lt;=$D$45,"OK","ÜBERSCHRITTEN")</f>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="204" t="s">
+        <v>351</v>
+      </c>
+      <c r="C47" s="196"/>
+      <c r="D47" s="245" t="str">
+        <f>=ROUND(MAX(0,$D$39-$D$45),2)</f>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="252" t="s">
+        <v>352</v>
+      </c>
+      <c r="C48" s="253"/>
+      <c r="D48" s="254" t="str">
+        <f>=IFERROR($D$39/$D$45,0)</f>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="true">
+      <c r="B50" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
+    </row>
+    <row r="52" ht="28" customHeight="true">
+      <c r="B52" s="261" t="s">
+        <v>354</v>
+      </c>
+      <c r="C52" s="262" t="s">
+        <v>355</v>
+      </c>
+      <c r="D52" s="262" t="s">
+        <v>356</v>
+      </c>
+      <c r="E52" s="262" t="s">
+        <v>357</v>
+      </c>
+      <c r="F52" s="262" t="s">
+        <v>358</v>
+      </c>
+      <c r="G52" s="262" t="s">
+        <v>359</v>
+      </c>
+      <c r="H52" s="262" t="s">
+        <v>360</v>
+      </c>
+      <c r="I52" s="262" t="s">
+        <v>361</v>
+      </c>
+      <c r="J52" s="263" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="264" t="s">
+        <v>194</v>
+      </c>
+      <c r="C53" s="24">
         <v>0</v>
       </c>
-      <c r="L17" s="196" t="str">
-        <f>=IF(5&lt;=N11,"Periode "&amp;N10&amp;" (#5)","")</f>
-      </c>
-      <c r="N17" s="246" t="str">
-        <f>=IF(5&lt;=N11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
-      </c>
-      <c r="O17" s="48"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="221" t="s">
-        <v>337</v>
-      </c>
-      <c r="C18" s="222"/>
-      <c r="D18" s="223" t="str">
-        <f>=ROUND($D$14-MAX(0,$D$17),2)</f>
-      </c>
-      <c r="G18" s="221" t="s">
-        <v>338</v>
-      </c>
-      <c r="H18" s="222"/>
-      <c r="I18" s="223" t="str">
-        <f>=ROUND($I$15-MAX(0,$I$17),2)</f>
-      </c>
-      <c r="L18" s="196" t="str">
-        <f>=IF(6&lt;=N11,"Periode "&amp;N10&amp;" (#6)","")</f>
-      </c>
-      <c r="M18" s="157"/>
-      <c r="N18" s="246" t="str">
-        <f>=IF(6&lt;=N11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
-      </c>
-      <c r="O18" s="158"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="216" t="s">
-        <v>339</v>
-      </c>
-      <c r="C20" s="217"/>
-      <c r="D20" s="227">
+      <c r="D53" s="239" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
+      </c>
+      <c r="E53" s="200" t="str">
+        <f>=ROUND(IFERROR($C$53-$D$53,0),2)</f>
+      </c>
+      <c r="F53" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$53/$D$53)-1,0),4)</f>
+      </c>
+      <c r="G53" s="25">
         <v>0</v>
       </c>
-      <c r="G20" s="216" t="s">
-        <v>339</v>
-      </c>
-      <c r="H20" s="217"/>
-      <c r="I20" s="227">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="221" t="s">
-        <v>337</v>
-      </c>
-      <c r="C21" s="222"/>
-      <c r="D21" s="223" t="str">
-        <f>=ROUND($D$14-MAX(0,$D$17)-MAX(0,$D$20),2)</f>
-      </c>
-      <c r="G21" s="221" t="s">
-        <v>338</v>
-      </c>
-      <c r="H21" s="222"/>
-      <c r="I21" s="223" t="str">
-        <f>=ROUND($I$15-MAX(0,$I$17)-MAX(0,$I$20),2)</f>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="true">
-      <c r="B24" s="18" t="s">
-        <v>340</v>
-      </c>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="216" t="s">
-        <v>341</v>
-      </c>
-      <c r="C26" s="217"/>
-      <c r="D26" s="234" t="str">
-        <f>=N10</f>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="219" t="s">
-        <v>342</v>
-      </c>
-      <c r="C27" s="210"/>
-      <c r="D27" s="235" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,N10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;N11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="219" t="s">
-        <v>343</v>
-      </c>
-      <c r="C28" s="210"/>
-      <c r="D28" s="203" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="219" t="s">
-        <v>344</v>
-      </c>
-      <c r="C29" s="210"/>
-      <c r="D29" s="235" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(MATCH($D$28,{"Jahr 1";"Jahr 2";"Jahr 3"},0),SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])),2),0)</f>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="219" t="s">
-        <v>345</v>
-      </c>
-      <c r="C30" s="210"/>
-      <c r="D30" s="236">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="219" t="s">
-        <v>346</v>
-      </c>
-      <c r="C31" s="210"/>
-      <c r="D31" s="237">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="219" t="s">
-        <v>347</v>
-      </c>
-      <c r="C32" s="210"/>
-      <c r="D32" s="238">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="239" t="s">
-        <v>348</v>
-      </c>
-      <c r="C33" s="212"/>
-      <c r="D33" s="240" t="str">
-        <f>=IFERROR(ROUND($D$29*$D$30/$D$31,2),0)</f>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="239" t="s">
-        <v>349</v>
-      </c>
-      <c r="C34" s="212"/>
-      <c r="D34" s="241" t="str">
-        <f>=IF($D$27&lt;=$D$33,"OK","ÜBERSCHRITTEN")</f>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="219" t="s">
-        <v>350</v>
-      </c>
-      <c r="C35" s="210"/>
-      <c r="D35" s="235" t="str">
-        <f>=ROUND(MAX(0,$D$27-$D$33),2)</f>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="242" t="s">
-        <v>351</v>
-      </c>
-      <c r="C36" s="243"/>
-      <c r="D36" s="244" t="str">
-        <f>=IFERROR($D$27/$D$33,0)</f>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="true">
-      <c r="B38" s="18" t="s">
-        <v>352</v>
-      </c>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
-      <c r="J38" s="18"/>
-    </row>
-    <row r="40" ht="28" customHeight="true">
-      <c r="B40" s="252" t="s">
-        <v>353</v>
-      </c>
-      <c r="C40" s="253" t="s">
-        <v>354</v>
-      </c>
-      <c r="D40" s="253" t="s">
-        <v>355</v>
-      </c>
-      <c r="E40" s="253" t="s">
-        <v>356</v>
-      </c>
-      <c r="F40" s="253" t="s">
-        <v>357</v>
-      </c>
-      <c r="G40" s="253" t="s">
-        <v>358</v>
-      </c>
-      <c r="H40" s="253" t="s">
-        <v>359</v>
-      </c>
-      <c r="I40" s="253" t="s">
-        <v>360</v>
-      </c>
-      <c r="J40" s="254" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="255" t="s">
-        <v>194</v>
-      </c>
-      <c r="C41" s="24">
-        <v>0</v>
-      </c>
-      <c r="D41" s="229" t="str">
-        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
-      </c>
-      <c r="E41" s="246" t="str">
-        <f>=ROUND(IFERROR($C$41-$D$41,0),2)</f>
-      </c>
-      <c r="F41" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$41/$D$41)-1,0),4)</f>
-      </c>
-      <c r="G41" s="25">
-        <v>0</v>
-      </c>
-      <c r="H41" s="211" t="str">
+      <c r="H53" s="217" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
-      </c>
-      <c r="I41" s="181" t="str">
-        <f>=ROUND(IFERROR($G$41-$H$41,0),2)</f>
-      </c>
-      <c r="J41" s="256" t="str">
-        <f>=ROUND(IFERROR(($G$41/$H$41)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="255" t="s">
-        <v>277</v>
-      </c>
-      <c r="C42" s="24">
-        <v>0</v>
-      </c>
-      <c r="D42" s="229" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
-      </c>
-      <c r="E42" s="246" t="str">
-        <f>=ROUND(IFERROR($C$42-$D$42,0),2)</f>
-      </c>
-      <c r="F42" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$42/$D$42)-1,0),4)</f>
-      </c>
-      <c r="G42" s="25">
-        <v>0</v>
-      </c>
-      <c r="H42" s="211" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
-      </c>
-      <c r="I42" s="181" t="str">
-        <f>=ROUND(IFERROR($G$42-$H$42,0),2)</f>
-      </c>
-      <c r="J42" s="257" t="str">
-        <f>=ROUND(IFERROR(($G$42/$H$42)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="255" t="s">
-        <v>199</v>
-      </c>
-      <c r="C43" s="24">
-        <v>0</v>
-      </c>
-      <c r="D43" s="229" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
-      </c>
-      <c r="E43" s="246" t="str">
-        <f>=ROUND(IFERROR($C$43-$D$43,0),2)</f>
-      </c>
-      <c r="F43" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$43/$D$43)-1,0),4)</f>
-      </c>
-      <c r="G43" s="25">
-        <v>0</v>
-      </c>
-      <c r="H43" s="211" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
-      </c>
-      <c r="I43" s="181" t="str">
-        <f>=ROUND(IFERROR($G$43-$H$43,0),2)</f>
-      </c>
-      <c r="J43" s="258" t="str">
-        <f>=ROUND(IFERROR(($G$43/$H$43)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="255" t="s">
-        <v>278</v>
-      </c>
-      <c r="C44" s="24">
-        <v>0</v>
-      </c>
-      <c r="D44" s="229" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
-      </c>
-      <c r="E44" s="246" t="str">
-        <f>=ROUND(IFERROR($C$44-$D$44,0),2)</f>
-      </c>
-      <c r="F44" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$44/$D$44)-1,0),4)</f>
-      </c>
-      <c r="G44" s="25">
-        <v>0</v>
-      </c>
-      <c r="H44" s="211" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
-      </c>
-      <c r="I44" s="181" t="str">
-        <f>=ROUND(IFERROR($G$44-$H$44,0),2)</f>
-      </c>
-      <c r="J44" s="259" t="str">
-        <f>=ROUND(IFERROR(($G$44/$H$44)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="true">
-      <c r="B45" s="260" t="s">
-        <v>266</v>
-      </c>
-      <c r="C45" s="261" t="str">
-        <f>=ROUND(SUM($C$41:$C$44),2)</f>
-      </c>
-      <c r="D45" s="261" t="str">
-        <f>=ROUND(SUM($D$41:$D$44),2)</f>
-      </c>
-      <c r="E45" s="261" t="str">
-        <f>=ROUND(SUM($E$41:$E$44),2)</f>
-      </c>
-      <c r="F45" s="262" t="str">
-        <f>=ROUND(IFERROR(($C$45/$D$45)-1,0),4)</f>
-      </c>
-      <c r="G45" s="263" t="str">
-        <f>=ROUND(SUM($G$41:$G$44),2)</f>
-      </c>
-      <c r="H45" s="263" t="str">
-        <f>=ROUND(SUM($H$41:$H$44),2)</f>
-      </c>
-      <c r="I45" s="263" t="str">
-        <f>=ROUND(SUM($I$41:$I$44),2)</f>
-      </c>
-      <c r="J45" s="264" t="str">
-        <f>=ROUND(IFERROR(($G$45/$H$45)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="true">
-      <c r="B47" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="C47" s="18"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
-      <c r="F47" s="18"/>
-      <c r="G47" s="18"/>
-      <c r="H47" s="18"/>
-      <c r="I47" s="18"/>
-      <c r="J47" s="18"/>
-    </row>
-    <row r="49" ht="28" customHeight="true">
-      <c r="B49" s="252" t="s">
-        <v>353</v>
-      </c>
-      <c r="C49" s="253" t="s">
-        <v>354</v>
-      </c>
-      <c r="D49" s="253" t="s">
-        <v>355</v>
-      </c>
-      <c r="E49" s="253" t="s">
-        <v>356</v>
-      </c>
-      <c r="F49" s="253" t="s">
-        <v>357</v>
-      </c>
-      <c r="G49" s="253" t="s">
-        <v>358</v>
-      </c>
-      <c r="H49" s="253" t="s">
-        <v>359</v>
-      </c>
-      <c r="I49" s="253" t="s">
-        <v>360</v>
-      </c>
-      <c r="J49" s="254" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="255" t="s">
-        <v>205</v>
-      </c>
-      <c r="C50" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D50" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
-      </c>
-      <c r="E50" s="246" t="str">
-        <f>=ROUND(IFERROR($C$50-$D$50,0),2)</f>
-      </c>
-      <c r="F50" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$50/$D$50)-1,0),4)</f>
-      </c>
-      <c r="G50" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H50" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
-      </c>
-      <c r="I50" s="181" t="str">
-        <f>=ROUND(IFERROR($G$50-$H$50,0),2)</f>
-      </c>
-      <c r="J50" s="265" t="str">
-        <f>=ROUND(IFERROR(($G$50/$H$50)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="255" t="s">
-        <v>206</v>
-      </c>
-      <c r="C51" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D51" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
-      </c>
-      <c r="E51" s="246" t="str">
-        <f>=ROUND(IFERROR($C$51-$D$51,0),2)</f>
-      </c>
-      <c r="F51" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$51/$D$51)-1,0),4)</f>
-      </c>
-      <c r="G51" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H51" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
-      </c>
-      <c r="I51" s="181" t="str">
-        <f>=ROUND(IFERROR($G$51-$H$51,0),2)</f>
-      </c>
-      <c r="J51" s="266" t="str">
-        <f>=ROUND(IFERROR(($G$51/$H$51)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="255" t="s">
-        <v>207</v>
-      </c>
-      <c r="C52" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D52" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
-      </c>
-      <c r="E52" s="246" t="str">
-        <f>=ROUND(IFERROR($C$52-$D$52,0),2)</f>
-      </c>
-      <c r="F52" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$52/$D$52)-1,0),4)</f>
-      </c>
-      <c r="G52" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H52" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
-      </c>
-      <c r="I52" s="181" t="str">
-        <f>=ROUND(IFERROR($G$52-$H$52,0),2)</f>
-      </c>
-      <c r="J52" s="267" t="str">
-        <f>=ROUND(IFERROR(($G$52/$H$52)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="255" t="s">
-        <v>208</v>
-      </c>
-      <c r="C53" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D53" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
-      </c>
-      <c r="E53" s="246" t="str">
-        <f>=ROUND(IFERROR($C$53-$D$53,0),2)</f>
-      </c>
-      <c r="F53" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$53/$D$53)-1,0),4)</f>
-      </c>
-      <c r="G53" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H53" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
       </c>
       <c r="I53" s="181" t="str">
         <f>=ROUND(IFERROR($G$53-$H$53,0),2)</f>
       </c>
-      <c r="J53" s="268" t="str">
+      <c r="J53" s="265" t="str">
         <f>=ROUND(IFERROR(($G$53/$H$53)-1,0),4)</f>
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="255" t="s">
-        <v>209</v>
-      </c>
-      <c r="C54" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D54" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
-      </c>
-      <c r="E54" s="246" t="str">
+      <c r="B54" s="264" t="s">
+        <v>277</v>
+      </c>
+      <c r="C54" s="24">
+        <v>0</v>
+      </c>
+      <c r="D54" s="239" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
+      </c>
+      <c r="E54" s="200" t="str">
         <f>=ROUND(IFERROR($C$54-$D$54,0),2)</f>
       </c>
-      <c r="F54" s="247" t="str">
+      <c r="F54" s="256" t="str">
         <f>=ROUND(IFERROR(($C$54/$D$54)-1,0),4)</f>
       </c>
-      <c r="G54" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H54" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
+      <c r="G54" s="25">
+        <v>0</v>
+      </c>
+      <c r="H54" s="217" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
       </c>
       <c r="I54" s="181" t="str">
         <f>=ROUND(IFERROR($G$54-$H$54,0),2)</f>
       </c>
-      <c r="J54" s="269" t="str">
+      <c r="J54" s="266" t="str">
         <f>=ROUND(IFERROR(($G$54/$H$54)-1,0),4)</f>
       </c>
     </row>
     <row r="55">
-      <c r="B55" s="255" t="s">
-        <v>210</v>
-      </c>
-      <c r="C55" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D55" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
-      </c>
-      <c r="E55" s="246" t="str">
+      <c r="B55" s="264" t="s">
+        <v>199</v>
+      </c>
+      <c r="C55" s="24">
+        <v>0</v>
+      </c>
+      <c r="D55" s="239" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
+      </c>
+      <c r="E55" s="200" t="str">
         <f>=ROUND(IFERROR($C$55-$D$55,0),2)</f>
       </c>
-      <c r="F55" s="247" t="str">
+      <c r="F55" s="256" t="str">
         <f>=ROUND(IFERROR(($C$55/$D$55)-1,0),4)</f>
       </c>
-      <c r="G55" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H55" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+      <c r="G55" s="25">
+        <v>0</v>
+      </c>
+      <c r="H55" s="217" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="I55" s="181" t="str">
         <f>=ROUND(IFERROR($G$55-$H$55,0),2)</f>
       </c>
-      <c r="J55" s="270" t="str">
+      <c r="J55" s="267" t="str">
         <f>=ROUND(IFERROR(($G$55/$H$55)-1,0),4)</f>
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="255" t="s">
-        <v>211</v>
-      </c>
-      <c r="C56" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D56" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
-      </c>
-      <c r="E56" s="246" t="str">
+      <c r="B56" s="264" t="s">
+        <v>278</v>
+      </c>
+      <c r="C56" s="24">
+        <v>0</v>
+      </c>
+      <c r="D56" s="239" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
+      </c>
+      <c r="E56" s="200" t="str">
         <f>=ROUND(IFERROR($C$56-$D$56,0),2)</f>
       </c>
-      <c r="F56" s="247" t="str">
+      <c r="F56" s="256" t="str">
         <f>=ROUND(IFERROR(($C$56/$D$56)-1,0),4)</f>
       </c>
-      <c r="G56" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H56" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+      <c r="G56" s="25">
+        <v>0</v>
+      </c>
+      <c r="H56" s="217" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
       <c r="I56" s="181" t="str">
         <f>=ROUND(IFERROR($G$56-$H$56,0),2)</f>
       </c>
-      <c r="J56" s="271" t="str">
+      <c r="J56" s="268" t="str">
         <f>=ROUND(IFERROR(($G$56/$H$56)-1,0),4)</f>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="255" t="s">
+    <row r="57" ht="20" customHeight="true">
+      <c r="B57" s="269" t="s">
+        <v>266</v>
+      </c>
+      <c r="C57" s="270" t="str">
+        <f>=ROUND(SUM($C$53:$C$56),2)</f>
+      </c>
+      <c r="D57" s="270" t="str">
+        <f>=ROUND(SUM($D$53:$D$56),2)</f>
+      </c>
+      <c r="E57" s="270" t="str">
+        <f>=ROUND(SUM($E$53:$E$56),2)</f>
+      </c>
+      <c r="F57" s="271" t="str">
+        <f>=ROUND(IFERROR(($C$57/$D$57)-1,0),4)</f>
+      </c>
+      <c r="G57" s="272" t="str">
+        <f>=ROUND(SUM($G$53:$G$56),2)</f>
+      </c>
+      <c r="H57" s="272" t="str">
+        <f>=ROUND(SUM($H$53:$H$56),2)</f>
+      </c>
+      <c r="I57" s="272" t="str">
+        <f>=ROUND(SUM($I$53:$I$56),2)</f>
+      </c>
+      <c r="J57" s="273" t="str">
+        <f>=ROUND(IFERROR(($G$57/$H$57)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="true">
+      <c r="B59" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+      <c r="I59" s="18"/>
+      <c r="J59" s="18"/>
+    </row>
+    <row r="61" ht="28" customHeight="true">
+      <c r="B61" s="261" t="s">
+        <v>354</v>
+      </c>
+      <c r="C61" s="262" t="s">
+        <v>355</v>
+      </c>
+      <c r="D61" s="262" t="s">
+        <v>356</v>
+      </c>
+      <c r="E61" s="262" t="s">
+        <v>357</v>
+      </c>
+      <c r="F61" s="262" t="s">
+        <v>358</v>
+      </c>
+      <c r="G61" s="262" t="s">
+        <v>359</v>
+      </c>
+      <c r="H61" s="262" t="s">
+        <v>360</v>
+      </c>
+      <c r="I61" s="262" t="s">
+        <v>361</v>
+      </c>
+      <c r="J61" s="263" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="264" t="s">
+        <v>205</v>
+      </c>
+      <c r="C62" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D62" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
+      </c>
+      <c r="E62" s="200" t="str">
+        <f>=ROUND(IFERROR($C$62-$D$62,0),2)</f>
+      </c>
+      <c r="F62" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$62/$D$62)-1,0),4)</f>
+      </c>
+      <c r="G62" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H62" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
+      </c>
+      <c r="I62" s="181" t="str">
+        <f>=ROUND(IFERROR($G$62-$H$62,0),2)</f>
+      </c>
+      <c r="J62" s="274" t="str">
+        <f>=ROUND(IFERROR(($G$62/$H$62)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="264" t="s">
+        <v>206</v>
+      </c>
+      <c r="C63" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D63" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
+      </c>
+      <c r="E63" s="200" t="str">
+        <f>=ROUND(IFERROR($C$63-$D$63,0),2)</f>
+      </c>
+      <c r="F63" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$63/$D$63)-1,0),4)</f>
+      </c>
+      <c r="G63" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H63" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
+      </c>
+      <c r="I63" s="181" t="str">
+        <f>=ROUND(IFERROR($G$63-$H$63,0),2)</f>
+      </c>
+      <c r="J63" s="275" t="str">
+        <f>=ROUND(IFERROR(($G$63/$H$63)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="264" t="s">
+        <v>207</v>
+      </c>
+      <c r="C64" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D64" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
+      </c>
+      <c r="E64" s="200" t="str">
+        <f>=ROUND(IFERROR($C$64-$D$64,0),2)</f>
+      </c>
+      <c r="F64" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$64/$D$64)-1,0),4)</f>
+      </c>
+      <c r="G64" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H64" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
+      </c>
+      <c r="I64" s="181" t="str">
+        <f>=ROUND(IFERROR($G$64-$H$64,0),2)</f>
+      </c>
+      <c r="J64" s="276" t="str">
+        <f>=ROUND(IFERROR(($G$64/$H$64)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="264" t="s">
+        <v>208</v>
+      </c>
+      <c r="C65" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D65" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
+      </c>
+      <c r="E65" s="200" t="str">
+        <f>=ROUND(IFERROR($C$65-$D$65,0),2)</f>
+      </c>
+      <c r="F65" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$65/$D$65)-1,0),4)</f>
+      </c>
+      <c r="G65" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H65" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
+      </c>
+      <c r="I65" s="181" t="str">
+        <f>=ROUND(IFERROR($G$65-$H$65,0),2)</f>
+      </c>
+      <c r="J65" s="277" t="str">
+        <f>=ROUND(IFERROR(($G$65/$H$65)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="264" t="s">
+        <v>209</v>
+      </c>
+      <c r="C66" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D66" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
+      </c>
+      <c r="E66" s="200" t="str">
+        <f>=ROUND(IFERROR($C$66-$D$66,0),2)</f>
+      </c>
+      <c r="F66" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$66/$D$66)-1,0),4)</f>
+      </c>
+      <c r="G66" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H66" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
+      </c>
+      <c r="I66" s="181" t="str">
+        <f>=ROUND(IFERROR($G$66-$H$66,0),2)</f>
+      </c>
+      <c r="J66" s="278" t="str">
+        <f>=ROUND(IFERROR(($G$66/$H$66)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="264" t="s">
+        <v>210</v>
+      </c>
+      <c r="C67" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D67" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
+      </c>
+      <c r="E67" s="200" t="str">
+        <f>=ROUND(IFERROR($C$67-$D$67,0),2)</f>
+      </c>
+      <c r="F67" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$67/$D$67)-1,0),4)</f>
+      </c>
+      <c r="G67" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H67" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+      </c>
+      <c r="I67" s="181" t="str">
+        <f>=ROUND(IFERROR($G$67-$H$67,0),2)</f>
+      </c>
+      <c r="J67" s="279" t="str">
+        <f>=ROUND(IFERROR(($G$67/$H$67)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="264" t="s">
+        <v>211</v>
+      </c>
+      <c r="C68" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D68" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
+      </c>
+      <c r="E68" s="200" t="str">
+        <f>=ROUND(IFERROR($C$68-$D$68,0),2)</f>
+      </c>
+      <c r="F68" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$68/$D$68)-1,0),4)</f>
+      </c>
+      <c r="G68" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H68" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+      </c>
+      <c r="I68" s="181" t="str">
+        <f>=ROUND(IFERROR($G$68-$H$68,0),2)</f>
+      </c>
+      <c r="J68" s="280" t="str">
+        <f>=ROUND(IFERROR(($G$68/$H$68)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="264" t="s">
         <v>212</v>
       </c>
-      <c r="C57" s="229" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D57" s="229" t="str">
+      <c r="C69" s="239" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D69" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
       </c>
-      <c r="E57" s="246" t="str">
-        <f>=ROUND(IFERROR($C$57-$D$57,0),2)</f>
-      </c>
-      <c r="F57" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$57/$D$57)-1,0),4)</f>
-      </c>
-      <c r="G57" s="211" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,N10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;N11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H57" s="211" t="str">
+      <c r="E69" s="200" t="str">
+        <f>=ROUND(IFERROR($C$69-$D$69,0),2)</f>
+      </c>
+      <c r="F69" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$69/$D$69)-1,0),4)</f>
+      </c>
+      <c r="G69" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H69" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
-      <c r="I57" s="181" t="str">
-        <f>=ROUND(IFERROR($G$57-$H$57,0),2)</f>
-      </c>
-      <c r="J57" s="272" t="str">
-        <f>=ROUND(IFERROR(($G$57/$H$57)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="true">
-      <c r="B58" s="260" t="s">
+      <c r="I69" s="181" t="str">
+        <f>=ROUND(IFERROR($G$69-$H$69,0),2)</f>
+      </c>
+      <c r="J69" s="281" t="str">
+        <f>=ROUND(IFERROR(($G$69/$H$69)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="true">
+      <c r="B70" s="269" t="s">
         <v>266</v>
       </c>
-      <c r="C58" s="261" t="str">
-        <f>=ROUND(SUM($C$50:$C$57),2)</f>
-      </c>
-      <c r="D58" s="261" t="str">
-        <f>=ROUND(SUM($D$50:$D$57),2)</f>
-      </c>
-      <c r="E58" s="261" t="str">
-        <f>=ROUND(SUM($E$50:$E$57),2)</f>
-      </c>
-      <c r="F58" s="273" t="str">
-        <f>=ROUND(IFERROR(($C$58/$D$58)-1,0),4)</f>
-      </c>
-      <c r="G58" s="263" t="str">
-        <f>=ROUND(SUM($G$50:$G$57),2)</f>
-      </c>
-      <c r="H58" s="263" t="str">
-        <f>=ROUND(SUM($H$50:$H$57),2)</f>
-      </c>
-      <c r="I58" s="263" t="str">
-        <f>=ROUND(SUM($I$50:$I$57),2)</f>
-      </c>
-      <c r="J58" s="274" t="str">
-        <f>=ROUND(IFERROR(($G$58/$H$58)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="60" ht="26" customHeight="true">
-      <c r="B60" s="193" t="s">
-        <v>363</v>
-      </c>
-      <c r="C60" s="193"/>
-      <c r="D60" s="193"/>
-      <c r="E60" s="193"/>
-      <c r="F60" s="193"/>
-      <c r="G60" s="193"/>
-      <c r="H60" s="193"/>
-      <c r="I60" s="193"/>
-      <c r="J60" s="193"/>
-    </row>
-    <row r="61">
-      <c r="B61" s="194" t="s">
+      <c r="C70" s="270" t="str">
+        <f>=ROUND(SUM($C$62:$C$69),2)</f>
+      </c>
+      <c r="D70" s="270" t="str">
+        <f>=ROUND(SUM($D$62:$D$69),2)</f>
+      </c>
+      <c r="E70" s="270" t="str">
+        <f>=ROUND(SUM($E$62:$E$69),2)</f>
+      </c>
+      <c r="F70" s="282" t="str">
+        <f>=ROUND(IFERROR(($C$70/$D$70)-1,0),4)</f>
+      </c>
+      <c r="G70" s="272" t="str">
+        <f>=ROUND(SUM($G$62:$G$69),2)</f>
+      </c>
+      <c r="H70" s="272" t="str">
+        <f>=ROUND(SUM($H$62:$H$69),2)</f>
+      </c>
+      <c r="I70" s="272" t="str">
+        <f>=ROUND(SUM($I$62:$I$69),2)</f>
+      </c>
+      <c r="J70" s="283" t="str">
+        <f>=ROUND(IFERROR(($G$70/$H$70)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="72" ht="26" customHeight="true">
+      <c r="B72" s="193" t="s">
         <v>364</v>
       </c>
-      <c r="C61" s="194"/>
-      <c r="D61" s="194"/>
-      <c r="E61" s="194"/>
-      <c r="F61" s="194"/>
-      <c r="G61" s="194"/>
-      <c r="H61" s="194"/>
-      <c r="I61" s="194"/>
-      <c r="J61" s="194"/>
-    </row>
-    <row r="63" ht="22" customHeight="true">
-      <c r="B63" s="18" t="s">
+      <c r="C72" s="193"/>
+      <c r="D72" s="193"/>
+      <c r="E72" s="193"/>
+      <c r="F72" s="193"/>
+      <c r="G72" s="193"/>
+      <c r="H72" s="193"/>
+      <c r="I72" s="193"/>
+      <c r="J72" s="193"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="194" t="s">
+        <v>365</v>
+      </c>
+      <c r="C73" s="194"/>
+      <c r="D73" s="194"/>
+      <c r="E73" s="194"/>
+      <c r="F73" s="194"/>
+      <c r="G73" s="194"/>
+      <c r="H73" s="194"/>
+      <c r="I73" s="194"/>
+      <c r="J73" s="194"/>
+    </row>
+    <row r="75" ht="22" customHeight="true">
+      <c r="C75" s="201" t="s">
+        <v>366</v>
+      </c>
+      <c r="D75" s="202"/>
+      <c r="E75" s="202"/>
+      <c r="F75" s="202"/>
+      <c r="G75" s="202"/>
+      <c r="H75" s="202"/>
+      <c r="I75" s="203"/>
+    </row>
+    <row r="76">
+      <c r="C76" s="204" t="s">
+        <v>320</v>
+      </c>
+      <c r="D76" s="196"/>
+      <c r="E76" s="196"/>
+      <c r="F76" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="G76" s="33"/>
+      <c r="H76" s="33"/>
+      <c r="I76" s="205"/>
+    </row>
+    <row r="77">
+      <c r="C77" s="204" t="s">
+        <v>367</v>
+      </c>
+      <c r="D77" s="196"/>
+      <c r="E77" s="196"/>
+      <c r="F77" s="197" t="str">
+        <f>=IF(LEFT(F76,8)="Periode ",IFERROR(VALUE(TRIM(MID(F76,9,5))),0),0)</f>
+      </c>
+      <c r="G77" s="197"/>
+      <c r="H77" s="197"/>
+      <c r="I77" s="284"/>
+    </row>
+    <row r="78">
+      <c r="C78" s="204" t="s">
         <v>368</v>
       </c>
-      <c r="C63" s="18"/>
-      <c r="D63" s="18"/>
-      <c r="E63" s="18"/>
-      <c r="F63" s="18"/>
-      <c r="G63" s="18"/>
-      <c r="H63" s="18"/>
-      <c r="I63" s="18"/>
-      <c r="J63" s="18"/>
-      <c r="L63" s="199" t="s">
-        <v>365</v>
-      </c>
-      <c r="M63" s="200"/>
-      <c r="N63" s="200"/>
-      <c r="O63" s="201"/>
-    </row>
-    <row r="64">
-      <c r="L64" s="202" t="s">
-        <v>226</v>
-      </c>
-      <c r="O64" s="48"/>
-    </row>
-    <row r="65">
-      <c r="B65" s="216" t="s">
-        <v>324</v>
-      </c>
-      <c r="C65" s="217"/>
-      <c r="D65" s="218" t="str">
+      <c r="D78" s="196"/>
+      <c r="E78" s="196"/>
+      <c r="F78" s="239" t="str">
+        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoLC_"&amp;F77),2),0)</f>
+      </c>
+      <c r="G78" s="239"/>
+      <c r="H78" s="239"/>
+      <c r="I78" s="245"/>
+    </row>
+    <row r="79">
+      <c r="C79" s="252" t="s">
+        <v>171</v>
+      </c>
+      <c r="D79" s="253"/>
+      <c r="E79" s="253"/>
+      <c r="F79" s="285" t="str">
+        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoEUR_"&amp;F77),2),0)</f>
+      </c>
+      <c r="G79" s="285"/>
+      <c r="H79" s="285"/>
+      <c r="I79" s="286"/>
+    </row>
+    <row r="81" ht="22" customHeight="true">
+      <c r="B81" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="C81" s="18"/>
+      <c r="D81" s="18"/>
+      <c r="E81" s="18"/>
+      <c r="F81" s="18"/>
+      <c r="G81" s="18"/>
+      <c r="H81" s="18"/>
+      <c r="I81" s="18"/>
+      <c r="J81" s="18"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="223" t="s">
+        <v>325</v>
+      </c>
+      <c r="C83" s="224"/>
+      <c r="D83" s="225" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
-      <c r="F65" s="199" t="s">
+      <c r="F83" s="230" t="s">
+        <v>330</v>
+      </c>
+      <c r="G83" s="231"/>
+      <c r="H83" s="231"/>
+      <c r="I83" s="232"/>
+    </row>
+    <row r="84">
+      <c r="B84" s="204" t="s">
+        <v>326</v>
+      </c>
+      <c r="C84" s="196"/>
+      <c r="D84" s="226" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="F84" s="233" t="s">
+        <v>331</v>
+      </c>
+      <c r="G84" s="196" t="s">
+        <v>332</v>
+      </c>
+      <c r="H84" s="196"/>
+      <c r="I84" s="234" t="str">
+        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="204" t="s">
+        <v>327</v>
+      </c>
+      <c r="C85" s="196"/>
+      <c r="D85" s="226" t="str">
+        <f>=ROUND($D$83-$D$84,2)</f>
+      </c>
+      <c r="F85" s="233" t="s">
+        <v>331</v>
+      </c>
+      <c r="G85" s="196" t="s">
+        <v>333</v>
+      </c>
+      <c r="H85" s="196"/>
+      <c r="I85" s="222" t="str">
+        <f>=IFERROR(ROUND(MAX(0,(SUM($G$94:$G$97)-$G$96)-(SUM($H$94:$H$97)-$H$96)),2),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="204" t="s">
+        <v>328</v>
+      </c>
+      <c r="C86" s="196"/>
+      <c r="D86" s="226" t="str">
+        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
+      </c>
+      <c r="F86" s="47"/>
+      <c r="G86" s="218" t="s">
+        <v>335</v>
+      </c>
+      <c r="H86" s="218"/>
+      <c r="I86" s="235" t="str">
+        <f>=ROUND(IF($F$84="Abzug",MAX(0,$I$84),0)+IF($F$85="Abzug",MAX(0,$I$85),0),2)</f>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="227" t="s">
         <v>329</v>
       </c>
-      <c r="G65" s="200"/>
-      <c r="H65" s="200"/>
-      <c r="I65" s="201"/>
-      <c r="L65" s="204" t="s">
-        <v>366</v>
-      </c>
-      <c r="M65" s="196"/>
-      <c r="N65" s="275" t="str">
-        <f>=IFERROR(VALUE(TRIM(MID(L64,9,5))),0)</f>
-      </c>
-      <c r="O65" s="48"/>
-    </row>
-    <row r="66">
-      <c r="B66" s="219" t="s">
-        <v>325</v>
-      </c>
-      <c r="C66" s="210"/>
-      <c r="D66" s="220" t="str">
+      <c r="C87" s="228"/>
+      <c r="D87" s="229" t="str">
+        <f>=ROUND($D$85-$D$86,2)</f>
+      </c>
+      <c r="F87" s="236"/>
+      <c r="G87" s="228" t="s">
+        <v>336</v>
+      </c>
+      <c r="H87" s="228"/>
+      <c r="I87" s="229" t="str">
+        <f>=ROUND($D$87-$I$86,2)</f>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="true">
+      <c r="B91" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="C91" s="18"/>
+      <c r="D91" s="18"/>
+      <c r="E91" s="18"/>
+      <c r="F91" s="18"/>
+      <c r="G91" s="18"/>
+      <c r="H91" s="18"/>
+      <c r="I91" s="18"/>
+      <c r="J91" s="18"/>
+    </row>
+    <row r="93" ht="28" customHeight="true">
+      <c r="B93" s="261" t="s">
+        <v>354</v>
+      </c>
+      <c r="C93" s="262" t="s">
+        <v>371</v>
+      </c>
+      <c r="D93" s="262" t="s">
+        <v>356</v>
+      </c>
+      <c r="E93" s="262" t="s">
+        <v>357</v>
+      </c>
+      <c r="F93" s="262" t="s">
+        <v>358</v>
+      </c>
+      <c r="G93" s="262" t="s">
+        <v>372</v>
+      </c>
+      <c r="H93" s="262" t="s">
+        <v>360</v>
+      </c>
+      <c r="I93" s="262" t="s">
+        <v>361</v>
+      </c>
+      <c r="J93" s="263" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="264" t="s">
+        <v>194</v>
+      </c>
+      <c r="C94" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$12,'III. Finanzberichte'!$L$12,'III. Finanzberichte'!$S$12,'III. Finanzberichte'!$Z$12,'III. Finanzberichte'!$AG$12,'III. Finanzberichte'!$AN$12,'III. Finanzberichte'!$AU$12,'III. Finanzberichte'!$BB$12,'III. Finanzberichte'!$BI$12,'III. Finanzberichte'!$BP$12,'III. Finanzberichte'!$BW$12,'III. Finanzberichte'!$CD$12,'III. Finanzberichte'!$CK$12,'III. Finanzberichte'!$CR$12,'III. Finanzberichte'!$CY$12,'III. Finanzberichte'!$DF$12,'III. Finanzberichte'!$DM$12,'III. Finanzberichte'!$DT$12),2),0)</f>
+      </c>
+      <c r="D94" s="239" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
+      </c>
+      <c r="E94" s="200" t="str">
+        <f>=ROUND(IFERROR($C$94-$D$94,0),2)</f>
+      </c>
+      <c r="F94" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$94/$D$94)-1,0),4)</f>
+      </c>
+      <c r="G94" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$12,'III. Finanzberichte'!$M$12,'III. Finanzberichte'!$T$12,'III. Finanzberichte'!$AA$12,'III. Finanzberichte'!$AH$12,'III. Finanzberichte'!$AO$12,'III. Finanzberichte'!$AV$12,'III. Finanzberichte'!$BC$12,'III. Finanzberichte'!$BJ$12,'III. Finanzberichte'!$BQ$12,'III. Finanzberichte'!$BX$12,'III. Finanzberichte'!$CE$12,'III. Finanzberichte'!$CL$12,'III. Finanzberichte'!$CS$12,'III. Finanzberichte'!$CZ$12,'III. Finanzberichte'!$DG$12,'III. Finanzberichte'!$DN$12,'III. Finanzberichte'!$DU$12),2),0)</f>
+      </c>
+      <c r="H94" s="217" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
+      </c>
+      <c r="I94" s="181" t="str">
+        <f>=ROUND(IFERROR($G$94-$H$94,0),2)</f>
+      </c>
+      <c r="J94" s="287" t="str">
+        <f>=ROUND(IFERROR(($G$94/$H$94)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="264" t="s">
+        <v>277</v>
+      </c>
+      <c r="C95" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$13,'III. Finanzberichte'!$L$13,'III. Finanzberichte'!$S$13,'III. Finanzberichte'!$Z$13,'III. Finanzberichte'!$AG$13,'III. Finanzberichte'!$AN$13,'III. Finanzberichte'!$AU$13,'III. Finanzberichte'!$BB$13,'III. Finanzberichte'!$BI$13,'III. Finanzberichte'!$BP$13,'III. Finanzberichte'!$BW$13,'III. Finanzberichte'!$CD$13,'III. Finanzberichte'!$CK$13,'III. Finanzberichte'!$CR$13,'III. Finanzberichte'!$CY$13,'III. Finanzberichte'!$DF$13,'III. Finanzberichte'!$DM$13,'III. Finanzberichte'!$DT$13),2),0)</f>
+      </c>
+      <c r="D95" s="239" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
+      </c>
+      <c r="E95" s="200" t="str">
+        <f>=ROUND(IFERROR($C$95-$D$95,0),2)</f>
+      </c>
+      <c r="F95" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$95/$D$95)-1,0),4)</f>
+      </c>
+      <c r="G95" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$13,'III. Finanzberichte'!$M$13,'III. Finanzberichte'!$T$13,'III. Finanzberichte'!$AA$13,'III. Finanzberichte'!$AH$13,'III. Finanzberichte'!$AO$13,'III. Finanzberichte'!$AV$13,'III. Finanzberichte'!$BC$13,'III. Finanzberichte'!$BJ$13,'III. Finanzberichte'!$BQ$13,'III. Finanzberichte'!$BX$13,'III. Finanzberichte'!$CE$13,'III. Finanzberichte'!$CL$13,'III. Finanzberichte'!$CS$13,'III. Finanzberichte'!$CZ$13,'III. Finanzberichte'!$DG$13,'III. Finanzberichte'!$DN$13,'III. Finanzberichte'!$DU$13),2),0)</f>
+      </c>
+      <c r="H95" s="217" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
+      </c>
+      <c r="I95" s="181" t="str">
+        <f>=ROUND(IFERROR($G$95-$H$95,0),2)</f>
+      </c>
+      <c r="J95" s="288" t="str">
+        <f>=ROUND(IFERROR(($G$95/$H$95)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="264" t="s">
+        <v>199</v>
+      </c>
+      <c r="C96" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$14,'III. Finanzberichte'!$L$14,'III. Finanzberichte'!$S$14,'III. Finanzberichte'!$Z$14,'III. Finanzberichte'!$AG$14,'III. Finanzberichte'!$AN$14,'III. Finanzberichte'!$AU$14,'III. Finanzberichte'!$BB$14,'III. Finanzberichte'!$BI$14,'III. Finanzberichte'!$BP$14,'III. Finanzberichte'!$BW$14,'III. Finanzberichte'!$CD$14,'III. Finanzberichte'!$CK$14,'III. Finanzberichte'!$CR$14,'III. Finanzberichte'!$CY$14,'III. Finanzberichte'!$DF$14,'III. Finanzberichte'!$DM$14,'III. Finanzberichte'!$DT$14),2),0)</f>
+      </c>
+      <c r="D96" s="239" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
+      </c>
+      <c r="E96" s="200" t="str">
+        <f>=ROUND(IFERROR($C$96-$D$96,0),2)</f>
+      </c>
+      <c r="F96" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$96/$D$96)-1,0),4)</f>
+      </c>
+      <c r="G96" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$14,'III. Finanzberichte'!$M$14,'III. Finanzberichte'!$T$14,'III. Finanzberichte'!$AA$14,'III. Finanzberichte'!$AH$14,'III. Finanzberichte'!$AO$14,'III. Finanzberichte'!$AV$14,'III. Finanzberichte'!$BC$14,'III. Finanzberichte'!$BJ$14,'III. Finanzberichte'!$BQ$14,'III. Finanzberichte'!$BX$14,'III. Finanzberichte'!$CE$14,'III. Finanzberichte'!$CL$14,'III. Finanzberichte'!$CS$14,'III. Finanzberichte'!$CZ$14,'III. Finanzberichte'!$DG$14,'III. Finanzberichte'!$DN$14,'III. Finanzberichte'!$DU$14),2),0)</f>
+      </c>
+      <c r="H96" s="217" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
+      </c>
+      <c r="I96" s="181" t="str">
+        <f>=ROUND(IFERROR($G$96-$H$96,0),2)</f>
+      </c>
+      <c r="J96" s="289" t="str">
+        <f>=ROUND(IFERROR(($G$96/$H$96)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="264" t="s">
+        <v>278</v>
+      </c>
+      <c r="C97" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$15,'III. Finanzberichte'!$L$15,'III. Finanzberichte'!$S$15,'III. Finanzberichte'!$Z$15,'III. Finanzberichte'!$AG$15,'III. Finanzberichte'!$AN$15,'III. Finanzberichte'!$AU$15,'III. Finanzberichte'!$BB$15,'III. Finanzberichte'!$BI$15,'III. Finanzberichte'!$BP$15,'III. Finanzberichte'!$BW$15,'III. Finanzberichte'!$CD$15,'III. Finanzberichte'!$CK$15,'III. Finanzberichte'!$CR$15,'III. Finanzberichte'!$CY$15,'III. Finanzberichte'!$DF$15,'III. Finanzberichte'!$DM$15,'III. Finanzberichte'!$DT$15),2),0)</f>
+      </c>
+      <c r="D97" s="239" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
+      </c>
+      <c r="E97" s="200" t="str">
+        <f>=ROUND(IFERROR($C$97-$D$97,0),2)</f>
+      </c>
+      <c r="F97" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$97/$D$97)-1,0),4)</f>
+      </c>
+      <c r="G97" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$15,'III. Finanzberichte'!$M$15,'III. Finanzberichte'!$T$15,'III. Finanzberichte'!$AA$15,'III. Finanzberichte'!$AH$15,'III. Finanzberichte'!$AO$15,'III. Finanzberichte'!$AV$15,'III. Finanzberichte'!$BC$15,'III. Finanzberichte'!$BJ$15,'III. Finanzberichte'!$BQ$15,'III. Finanzberichte'!$BX$15,'III. Finanzberichte'!$CE$15,'III. Finanzberichte'!$CL$15,'III. Finanzberichte'!$CS$15,'III. Finanzberichte'!$CZ$15,'III. Finanzberichte'!$DG$15,'III. Finanzberichte'!$DN$15,'III. Finanzberichte'!$DU$15),2),0)</f>
+      </c>
+      <c r="H97" s="217" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
+      </c>
+      <c r="I97" s="181" t="str">
+        <f>=ROUND(IFERROR($G$97-$H$97,0),2)</f>
+      </c>
+      <c r="J97" s="290" t="str">
+        <f>=ROUND(IFERROR(($G$97/$H$97)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="98" ht="20" customHeight="true">
+      <c r="B98" s="269" t="s">
+        <v>266</v>
+      </c>
+      <c r="C98" s="270" t="str">
+        <f>=ROUND(SUM($C$94:$C$97),2)</f>
+      </c>
+      <c r="D98" s="270" t="str">
+        <f>=ROUND(SUM($D$94:$D$97),2)</f>
+      </c>
+      <c r="E98" s="270" t="str">
+        <f>=ROUND(SUM($E$94:$E$97),2)</f>
+      </c>
+      <c r="F98" s="291" t="str">
+        <f>=ROUND(IFERROR(($C$98/$D$98)-1,0),4)</f>
+      </c>
+      <c r="G98" s="272" t="str">
+        <f>=ROUND(SUM($G$94:$G$97),2)</f>
+      </c>
+      <c r="H98" s="272" t="str">
+        <f>=ROUND(SUM($H$94:$H$97),2)</f>
+      </c>
+      <c r="I98" s="272" t="str">
+        <f>=ROUND(SUM($I$94:$I$97),2)</f>
+      </c>
+      <c r="J98" s="292" t="str">
+        <f>=ROUND(IFERROR(($G$98/$H$98)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="true">
+      <c r="B100" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="C100" s="18"/>
+      <c r="D100" s="18"/>
+      <c r="E100" s="18"/>
+      <c r="F100" s="18"/>
+      <c r="G100" s="18"/>
+      <c r="H100" s="18"/>
+      <c r="I100" s="18"/>
+      <c r="J100" s="18"/>
+    </row>
+    <row r="102" ht="28" customHeight="true">
+      <c r="B102" s="261" t="s">
+        <v>354</v>
+      </c>
+      <c r="C102" s="262" t="s">
+        <v>371</v>
+      </c>
+      <c r="D102" s="262" t="s">
+        <v>356</v>
+      </c>
+      <c r="E102" s="262" t="s">
+        <v>357</v>
+      </c>
+      <c r="F102" s="262" t="s">
+        <v>358</v>
+      </c>
+      <c r="G102" s="262" t="s">
+        <v>372</v>
+      </c>
+      <c r="H102" s="262" t="s">
+        <v>360</v>
+      </c>
+      <c r="I102" s="262" t="s">
+        <v>361</v>
+      </c>
+      <c r="J102" s="263" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="264" t="s">
+        <v>205</v>
+      </c>
+      <c r="C103" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$19,'III. Finanzberichte'!$L$19,'III. Finanzberichte'!$S$19,'III. Finanzberichte'!$Z$19,'III. Finanzberichte'!$AG$19,'III. Finanzberichte'!$AN$19,'III. Finanzberichte'!$AU$19,'III. Finanzberichte'!$BB$19,'III. Finanzberichte'!$BI$19,'III. Finanzberichte'!$BP$19,'III. Finanzberichte'!$BW$19,'III. Finanzberichte'!$CD$19,'III. Finanzberichte'!$CK$19,'III. Finanzberichte'!$CR$19,'III. Finanzberichte'!$CY$19,'III. Finanzberichte'!$DF$19,'III. Finanzberichte'!$DM$19,'III. Finanzberichte'!$DT$19),2),0)</f>
+      </c>
+      <c r="D103" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
+      </c>
+      <c r="E103" s="200" t="str">
+        <f>=ROUND(IFERROR($C$103-$D$103,0),2)</f>
+      </c>
+      <c r="F103" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$103/$D$103)-1,0),4)</f>
+      </c>
+      <c r="G103" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$19,'III. Finanzberichte'!$M$19,'III. Finanzberichte'!$T$19,'III. Finanzberichte'!$AA$19,'III. Finanzberichte'!$AH$19,'III. Finanzberichte'!$AO$19,'III. Finanzberichte'!$AV$19,'III. Finanzberichte'!$BC$19,'III. Finanzberichte'!$BJ$19,'III. Finanzberichte'!$BQ$19,'III. Finanzberichte'!$BX$19,'III. Finanzberichte'!$CE$19,'III. Finanzberichte'!$CL$19,'III. Finanzberichte'!$CS$19,'III. Finanzberichte'!$CZ$19,'III. Finanzberichte'!$DG$19,'III. Finanzberichte'!$DN$19,'III. Finanzberichte'!$DU$19),2),0)</f>
+      </c>
+      <c r="H103" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
+      </c>
+      <c r="I103" s="181" t="str">
+        <f>=ROUND(IFERROR($G$103-$H$103,0),2)</f>
+      </c>
+      <c r="J103" s="293" t="str">
+        <f>=ROUND(IFERROR(($G$103/$H$103)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="264" t="s">
+        <v>206</v>
+      </c>
+      <c r="C104" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$20,'III. Finanzberichte'!$L$20,'III. Finanzberichte'!$S$20,'III. Finanzberichte'!$Z$20,'III. Finanzberichte'!$AG$20,'III. Finanzberichte'!$AN$20,'III. Finanzberichte'!$AU$20,'III. Finanzberichte'!$BB$20,'III. Finanzberichte'!$BI$20,'III. Finanzberichte'!$BP$20,'III. Finanzberichte'!$BW$20,'III. Finanzberichte'!$CD$20,'III. Finanzberichte'!$CK$20,'III. Finanzberichte'!$CR$20,'III. Finanzberichte'!$CY$20,'III. Finanzberichte'!$DF$20,'III. Finanzberichte'!$DM$20,'III. Finanzberichte'!$DT$20),2),0)</f>
+      </c>
+      <c r="D104" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
+      </c>
+      <c r="E104" s="200" t="str">
+        <f>=ROUND(IFERROR($C$104-$D$104,0),2)</f>
+      </c>
+      <c r="F104" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$104/$D$104)-1,0),4)</f>
+      </c>
+      <c r="G104" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$20,'III. Finanzberichte'!$M$20,'III. Finanzberichte'!$T$20,'III. Finanzberichte'!$AA$20,'III. Finanzberichte'!$AH$20,'III. Finanzberichte'!$AO$20,'III. Finanzberichte'!$AV$20,'III. Finanzberichte'!$BC$20,'III. Finanzberichte'!$BJ$20,'III. Finanzberichte'!$BQ$20,'III. Finanzberichte'!$BX$20,'III. Finanzberichte'!$CE$20,'III. Finanzberichte'!$CL$20,'III. Finanzberichte'!$CS$20,'III. Finanzberichte'!$CZ$20,'III. Finanzberichte'!$DG$20,'III. Finanzberichte'!$DN$20,'III. Finanzberichte'!$DU$20),2),0)</f>
+      </c>
+      <c r="H104" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
+      </c>
+      <c r="I104" s="181" t="str">
+        <f>=ROUND(IFERROR($G$104-$H$104,0),2)</f>
+      </c>
+      <c r="J104" s="294" t="str">
+        <f>=ROUND(IFERROR(($G$104/$H$104)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="264" t="s">
+        <v>207</v>
+      </c>
+      <c r="C105" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$21,'III. Finanzberichte'!$L$21,'III. Finanzberichte'!$S$21,'III. Finanzberichte'!$Z$21,'III. Finanzberichte'!$AG$21,'III. Finanzberichte'!$AN$21,'III. Finanzberichte'!$AU$21,'III. Finanzberichte'!$BB$21,'III. Finanzberichte'!$BI$21,'III. Finanzberichte'!$BP$21,'III. Finanzberichte'!$BW$21,'III. Finanzberichte'!$CD$21,'III. Finanzberichte'!$CK$21,'III. Finanzberichte'!$CR$21,'III. Finanzberichte'!$CY$21,'III. Finanzberichte'!$DF$21,'III. Finanzberichte'!$DM$21,'III. Finanzberichte'!$DT$21),2),0)</f>
+      </c>
+      <c r="D105" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
+      </c>
+      <c r="E105" s="200" t="str">
+        <f>=ROUND(IFERROR($C$105-$D$105,0),2)</f>
+      </c>
+      <c r="F105" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$105/$D$105)-1,0),4)</f>
+      </c>
+      <c r="G105" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$21,'III. Finanzberichte'!$M$21,'III. Finanzberichte'!$T$21,'III. Finanzberichte'!$AA$21,'III. Finanzberichte'!$AH$21,'III. Finanzberichte'!$AO$21,'III. Finanzberichte'!$AV$21,'III. Finanzberichte'!$BC$21,'III. Finanzberichte'!$BJ$21,'III. Finanzberichte'!$BQ$21,'III. Finanzberichte'!$BX$21,'III. Finanzberichte'!$CE$21,'III. Finanzberichte'!$CL$21,'III. Finanzberichte'!$CS$21,'III. Finanzberichte'!$CZ$21,'III. Finanzberichte'!$DG$21,'III. Finanzberichte'!$DN$21,'III. Finanzberichte'!$DU$21),2),0)</f>
+      </c>
+      <c r="H105" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
+      </c>
+      <c r="I105" s="181" t="str">
+        <f>=ROUND(IFERROR($G$105-$H$105,0),2)</f>
+      </c>
+      <c r="J105" s="295" t="str">
+        <f>=ROUND(IFERROR(($G$105/$H$105)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="264" t="s">
+        <v>208</v>
+      </c>
+      <c r="C106" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$22,'III. Finanzberichte'!$L$22,'III. Finanzberichte'!$S$22,'III. Finanzberichte'!$Z$22,'III. Finanzberichte'!$AG$22,'III. Finanzberichte'!$AN$22,'III. Finanzberichte'!$AU$22,'III. Finanzberichte'!$BB$22,'III. Finanzberichte'!$BI$22,'III. Finanzberichte'!$BP$22,'III. Finanzberichte'!$BW$22,'III. Finanzberichte'!$CD$22,'III. Finanzberichte'!$CK$22,'III. Finanzberichte'!$CR$22,'III. Finanzberichte'!$CY$22,'III. Finanzberichte'!$DF$22,'III. Finanzberichte'!$DM$22,'III. Finanzberichte'!$DT$22),2),0)</f>
+      </c>
+      <c r="D106" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
+      </c>
+      <c r="E106" s="200" t="str">
+        <f>=ROUND(IFERROR($C$106-$D$106,0),2)</f>
+      </c>
+      <c r="F106" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$106/$D$106)-1,0),4)</f>
+      </c>
+      <c r="G106" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$22,'III. Finanzberichte'!$M$22,'III. Finanzberichte'!$T$22,'III. Finanzberichte'!$AA$22,'III. Finanzberichte'!$AH$22,'III. Finanzberichte'!$AO$22,'III. Finanzberichte'!$AV$22,'III. Finanzberichte'!$BC$22,'III. Finanzberichte'!$BJ$22,'III. Finanzberichte'!$BQ$22,'III. Finanzberichte'!$BX$22,'III. Finanzberichte'!$CE$22,'III. Finanzberichte'!$CL$22,'III. Finanzberichte'!$CS$22,'III. Finanzberichte'!$CZ$22,'III. Finanzberichte'!$DG$22,'III. Finanzberichte'!$DN$22,'III. Finanzberichte'!$DU$22),2),0)</f>
+      </c>
+      <c r="H106" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
+      </c>
+      <c r="I106" s="181" t="str">
+        <f>=ROUND(IFERROR($G$106-$H$106,0),2)</f>
+      </c>
+      <c r="J106" s="296" t="str">
+        <f>=ROUND(IFERROR(($G$106/$H$106)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="264" t="s">
+        <v>209</v>
+      </c>
+      <c r="C107" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$23,'III. Finanzberichte'!$L$23,'III. Finanzberichte'!$S$23,'III. Finanzberichte'!$Z$23,'III. Finanzberichte'!$AG$23,'III. Finanzberichte'!$AN$23,'III. Finanzberichte'!$AU$23,'III. Finanzberichte'!$BB$23,'III. Finanzberichte'!$BI$23,'III. Finanzberichte'!$BP$23,'III. Finanzberichte'!$BW$23,'III. Finanzberichte'!$CD$23,'III. Finanzberichte'!$CK$23,'III. Finanzberichte'!$CR$23,'III. Finanzberichte'!$CY$23,'III. Finanzberichte'!$DF$23,'III. Finanzberichte'!$DM$23,'III. Finanzberichte'!$DT$23),2),0)</f>
+      </c>
+      <c r="D107" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
+      </c>
+      <c r="E107" s="200" t="str">
+        <f>=ROUND(IFERROR($C$107-$D$107,0),2)</f>
+      </c>
+      <c r="F107" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$107/$D$107)-1,0),4)</f>
+      </c>
+      <c r="G107" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$23,'III. Finanzberichte'!$M$23,'III. Finanzberichte'!$T$23,'III. Finanzberichte'!$AA$23,'III. Finanzberichte'!$AH$23,'III. Finanzberichte'!$AO$23,'III. Finanzberichte'!$AV$23,'III. Finanzberichte'!$BC$23,'III. Finanzberichte'!$BJ$23,'III. Finanzberichte'!$BQ$23,'III. Finanzberichte'!$BX$23,'III. Finanzberichte'!$CE$23,'III. Finanzberichte'!$CL$23,'III. Finanzberichte'!$CS$23,'III. Finanzberichte'!$CZ$23,'III. Finanzberichte'!$DG$23,'III. Finanzberichte'!$DN$23,'III. Finanzberichte'!$DU$23),2),0)</f>
+      </c>
+      <c r="H107" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
+      </c>
+      <c r="I107" s="181" t="str">
+        <f>=ROUND(IFERROR($G$107-$H$107,0),2)</f>
+      </c>
+      <c r="J107" s="297" t="str">
+        <f>=ROUND(IFERROR(($G$107/$H$107)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="264" t="s">
+        <v>210</v>
+      </c>
+      <c r="C108" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$24,'III. Finanzberichte'!$L$24,'III. Finanzberichte'!$S$24,'III. Finanzberichte'!$Z$24,'III. Finanzberichte'!$AG$24,'III. Finanzberichte'!$AN$24,'III. Finanzberichte'!$AU$24,'III. Finanzberichte'!$BB$24,'III. Finanzberichte'!$BI$24,'III. Finanzberichte'!$BP$24,'III. Finanzberichte'!$BW$24,'III. Finanzberichte'!$CD$24,'III. Finanzberichte'!$CK$24,'III. Finanzberichte'!$CR$24,'III. Finanzberichte'!$CY$24,'III. Finanzberichte'!$DF$24,'III. Finanzberichte'!$DM$24,'III. Finanzberichte'!$DT$24),2),0)</f>
+      </c>
+      <c r="D108" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
+      </c>
+      <c r="E108" s="200" t="str">
+        <f>=ROUND(IFERROR($C$108-$D$108,0),2)</f>
+      </c>
+      <c r="F108" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$108/$D$108)-1,0),4)</f>
+      </c>
+      <c r="G108" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$24,'III. Finanzberichte'!$M$24,'III. Finanzberichte'!$T$24,'III. Finanzberichte'!$AA$24,'III. Finanzberichte'!$AH$24,'III. Finanzberichte'!$AO$24,'III. Finanzberichte'!$AV$24,'III. Finanzberichte'!$BC$24,'III. Finanzberichte'!$BJ$24,'III. Finanzberichte'!$BQ$24,'III. Finanzberichte'!$BX$24,'III. Finanzberichte'!$CE$24,'III. Finanzberichte'!$CL$24,'III. Finanzberichte'!$CS$24,'III. Finanzberichte'!$CZ$24,'III. Finanzberichte'!$DG$24,'III. Finanzberichte'!$DN$24,'III. Finanzberichte'!$DU$24),2),0)</f>
+      </c>
+      <c r="H108" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+      </c>
+      <c r="I108" s="181" t="str">
+        <f>=ROUND(IFERROR($G$108-$H$108,0),2)</f>
+      </c>
+      <c r="J108" s="298" t="str">
+        <f>=ROUND(IFERROR(($G$108/$H$108)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="264" t="s">
+        <v>211</v>
+      </c>
+      <c r="C109" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$25,'III. Finanzberichte'!$L$25,'III. Finanzberichte'!$S$25,'III. Finanzberichte'!$Z$25,'III. Finanzberichte'!$AG$25,'III. Finanzberichte'!$AN$25,'III. Finanzberichte'!$AU$25,'III. Finanzberichte'!$BB$25,'III. Finanzberichte'!$BI$25,'III. Finanzberichte'!$BP$25,'III. Finanzberichte'!$BW$25,'III. Finanzberichte'!$CD$25,'III. Finanzberichte'!$CK$25,'III. Finanzberichte'!$CR$25,'III. Finanzberichte'!$CY$25,'III. Finanzberichte'!$DF$25,'III. Finanzberichte'!$DM$25,'III. Finanzberichte'!$DT$25),2),0)</f>
+      </c>
+      <c r="D109" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
+      </c>
+      <c r="E109" s="200" t="str">
+        <f>=ROUND(IFERROR($C$109-$D$109,0),2)</f>
+      </c>
+      <c r="F109" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$109/$D$109)-1,0),4)</f>
+      </c>
+      <c r="G109" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$25,'III. Finanzberichte'!$M$25,'III. Finanzberichte'!$T$25,'III. Finanzberichte'!$AA$25,'III. Finanzberichte'!$AH$25,'III. Finanzberichte'!$AO$25,'III. Finanzberichte'!$AV$25,'III. Finanzberichte'!$BC$25,'III. Finanzberichte'!$BJ$25,'III. Finanzberichte'!$BQ$25,'III. Finanzberichte'!$BX$25,'III. Finanzberichte'!$CE$25,'III. Finanzberichte'!$CL$25,'III. Finanzberichte'!$CS$25,'III. Finanzberichte'!$CZ$25,'III. Finanzberichte'!$DG$25,'III. Finanzberichte'!$DN$25,'III. Finanzberichte'!$DU$25),2),0)</f>
+      </c>
+      <c r="H109" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+      </c>
+      <c r="I109" s="181" t="str">
+        <f>=ROUND(IFERROR($G$109-$H$109,0),2)</f>
+      </c>
+      <c r="J109" s="299" t="str">
+        <f>=ROUND(IFERROR(($G$109/$H$109)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="264" t="s">
+        <v>212</v>
+      </c>
+      <c r="C110" s="239" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$26,'III. Finanzberichte'!$L$26,'III. Finanzberichte'!$S$26,'III. Finanzberichte'!$Z$26,'III. Finanzberichte'!$AG$26,'III. Finanzberichte'!$AN$26,'III. Finanzberichte'!$AU$26,'III. Finanzberichte'!$BB$26,'III. Finanzberichte'!$BI$26,'III. Finanzberichte'!$BP$26,'III. Finanzberichte'!$BW$26,'III. Finanzberichte'!$CD$26,'III. Finanzberichte'!$CK$26,'III. Finanzberichte'!$CR$26,'III. Finanzberichte'!$CY$26,'III. Finanzberichte'!$DF$26,'III. Finanzberichte'!$DM$26,'III. Finanzberichte'!$DT$26),2),0)</f>
+      </c>
+      <c r="D110" s="239" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
+      </c>
+      <c r="E110" s="200" t="str">
+        <f>=ROUND(IFERROR($C$110-$D$110,0),2)</f>
+      </c>
+      <c r="F110" s="256" t="str">
+        <f>=ROUND(IFERROR(($C$110/$D$110)-1,0),4)</f>
+      </c>
+      <c r="G110" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$26,'III. Finanzberichte'!$M$26,'III. Finanzberichte'!$T$26,'III. Finanzberichte'!$AA$26,'III. Finanzberichte'!$AH$26,'III. Finanzberichte'!$AO$26,'III. Finanzberichte'!$AV$26,'III. Finanzberichte'!$BC$26,'III. Finanzberichte'!$BJ$26,'III. Finanzberichte'!$BQ$26,'III. Finanzberichte'!$BX$26,'III. Finanzberichte'!$CE$26,'III. Finanzberichte'!$CL$26,'III. Finanzberichte'!$CS$26,'III. Finanzberichte'!$CZ$26,'III. Finanzberichte'!$DG$26,'III. Finanzberichte'!$DN$26,'III. Finanzberichte'!$DU$26),2),0)</f>
+      </c>
+      <c r="H110" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
-      <c r="F66" s="224" t="s">
-        <v>330</v>
-      </c>
-      <c r="G66" s="210" t="s">
-        <v>331</v>
-      </c>
-      <c r="H66" s="210"/>
-      <c r="I66" s="225" t="str">
-        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
-      </c>
-      <c r="L66" s="204" t="s">
-        <v>367</v>
-      </c>
-      <c r="M66" s="196"/>
-      <c r="N66" s="229" t="str">
-        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoLC_"&amp;N65),2),0)</f>
-      </c>
-      <c r="O66" s="48"/>
-    </row>
-    <row r="67">
-      <c r="B67" s="219" t="s">
-        <v>326</v>
-      </c>
-      <c r="C67" s="210"/>
-      <c r="D67" s="220" t="str">
-        <f>=ROUND($D$65-$D$66,2)</f>
-      </c>
-      <c r="F67" s="224" t="s">
-        <v>330</v>
-      </c>
-      <c r="G67" s="210" t="s">
-        <v>332</v>
-      </c>
-      <c r="H67" s="210"/>
-      <c r="I67" s="215" t="str">
-        <f>=IFERROR(ROUND(MAX(0,(SUM($G$76:$G$79)-$G$78)-(SUM($H$76:$H$79)-$H$78)),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L67" s="276" t="s">
-        <v>171</v>
-      </c>
-      <c r="M67" s="277"/>
-      <c r="N67" s="278" t="str">
-        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoEUR_"&amp;N65),2),0)</f>
-      </c>
-      <c r="O67" s="158"/>
-    </row>
-    <row r="68">
-      <c r="B68" s="219" t="s">
-        <v>327</v>
-      </c>
-      <c r="C68" s="210"/>
-      <c r="D68" s="220" t="str">
-        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
-      </c>
-      <c r="F68" s="47"/>
-      <c r="G68" s="212" t="s">
-        <v>334</v>
-      </c>
-      <c r="H68" s="212"/>
-      <c r="I68" s="226" t="str">
-        <f>=ROUND(IF($F$66="Abzug",MAX(0,$I$66),0)+IF($F$67="Abzug",MAX(0,$I$67),0),2)</f>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="221" t="s">
-        <v>328</v>
-      </c>
-      <c r="C69" s="222"/>
-      <c r="D69" s="223" t="str">
-        <f>=ROUND($D$67-$D$68,2)</f>
-      </c>
-      <c r="F69" s="209"/>
-      <c r="G69" s="222" t="s">
-        <v>335</v>
-      </c>
-      <c r="H69" s="222"/>
-      <c r="I69" s="223" t="str">
-        <f>=ROUND($D$69-$I$68,2)</f>
-      </c>
-    </row>
-    <row r="73" ht="22" customHeight="true">
-      <c r="B73" s="18" t="s">
-        <v>369</v>
-      </c>
-      <c r="C73" s="18"/>
-      <c r="D73" s="18"/>
-      <c r="E73" s="18"/>
-      <c r="F73" s="18"/>
-      <c r="G73" s="18"/>
-      <c r="H73" s="18"/>
-      <c r="I73" s="18"/>
-      <c r="J73" s="18"/>
-    </row>
-    <row r="75" ht="28" customHeight="true">
-      <c r="B75" s="252" t="s">
-        <v>353</v>
-      </c>
-      <c r="C75" s="253" t="s">
-        <v>370</v>
-      </c>
-      <c r="D75" s="253" t="s">
-        <v>355</v>
-      </c>
-      <c r="E75" s="253" t="s">
-        <v>356</v>
-      </c>
-      <c r="F75" s="253" t="s">
-        <v>357</v>
-      </c>
-      <c r="G75" s="253" t="s">
-        <v>371</v>
-      </c>
-      <c r="H75" s="253" t="s">
-        <v>359</v>
-      </c>
-      <c r="I75" s="253" t="s">
-        <v>360</v>
-      </c>
-      <c r="J75" s="254" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="255" t="s">
-        <v>194</v>
-      </c>
-      <c r="C76" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$12,'III. Finanzberichte'!$L$12,'III. Finanzberichte'!$S$12,'III. Finanzberichte'!$Z$12,'III. Finanzberichte'!$AG$12,'III. Finanzberichte'!$AN$12,'III. Finanzberichte'!$AU$12,'III. Finanzberichte'!$BB$12,'III. Finanzberichte'!$BI$12,'III. Finanzberichte'!$BP$12,'III. Finanzberichte'!$BW$12,'III. Finanzberichte'!$CD$12,'III. Finanzberichte'!$CK$12,'III. Finanzberichte'!$CR$12,'III. Finanzberichte'!$CY$12,'III. Finanzberichte'!$DF$12,'III. Finanzberichte'!$DM$12,'III. Finanzberichte'!$DT$12),2),0)</f>
-      </c>
-      <c r="D76" s="229" t="str">
-        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
-      </c>
-      <c r="E76" s="246" t="str">
-        <f>=ROUND(IFERROR($C$76-$D$76,0),2)</f>
-      </c>
-      <c r="F76" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$76/$D$76)-1,0),4)</f>
-      </c>
-      <c r="G76" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$12,'III. Finanzberichte'!$M$12,'III. Finanzberichte'!$T$12,'III. Finanzberichte'!$AA$12,'III. Finanzberichte'!$AH$12,'III. Finanzberichte'!$AO$12,'III. Finanzberichte'!$AV$12,'III. Finanzberichte'!$BC$12,'III. Finanzberichte'!$BJ$12,'III. Finanzberichte'!$BQ$12,'III. Finanzberichte'!$BX$12,'III. Finanzberichte'!$CE$12,'III. Finanzberichte'!$CL$12,'III. Finanzberichte'!$CS$12,'III. Finanzberichte'!$CZ$12,'III. Finanzberichte'!$DG$12,'III. Finanzberichte'!$DN$12,'III. Finanzberichte'!$DU$12),2),0)</f>
-      </c>
-      <c r="H76" s="211" t="str">
-        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
-      </c>
-      <c r="I76" s="181" t="str">
-        <f>=ROUND(IFERROR($G$76-$H$76,0),2)</f>
-      </c>
-      <c r="J76" s="279" t="str">
-        <f>=ROUND(IFERROR(($G$76/$H$76)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" s="255" t="s">
-        <v>277</v>
-      </c>
-      <c r="C77" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$13,'III. Finanzberichte'!$L$13,'III. Finanzberichte'!$S$13,'III. Finanzberichte'!$Z$13,'III. Finanzberichte'!$AG$13,'III. Finanzberichte'!$AN$13,'III. Finanzberichte'!$AU$13,'III. Finanzberichte'!$BB$13,'III. Finanzberichte'!$BI$13,'III. Finanzberichte'!$BP$13,'III. Finanzberichte'!$BW$13,'III. Finanzberichte'!$CD$13,'III. Finanzberichte'!$CK$13,'III. Finanzberichte'!$CR$13,'III. Finanzberichte'!$CY$13,'III. Finanzberichte'!$DF$13,'III. Finanzberichte'!$DM$13,'III. Finanzberichte'!$DT$13),2),0)</f>
-      </c>
-      <c r="D77" s="229" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
-      </c>
-      <c r="E77" s="246" t="str">
-        <f>=ROUND(IFERROR($C$77-$D$77,0),2)</f>
-      </c>
-      <c r="F77" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$77/$D$77)-1,0),4)</f>
-      </c>
-      <c r="G77" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$13,'III. Finanzberichte'!$M$13,'III. Finanzberichte'!$T$13,'III. Finanzberichte'!$AA$13,'III. Finanzberichte'!$AH$13,'III. Finanzberichte'!$AO$13,'III. Finanzberichte'!$AV$13,'III. Finanzberichte'!$BC$13,'III. Finanzberichte'!$BJ$13,'III. Finanzberichte'!$BQ$13,'III. Finanzberichte'!$BX$13,'III. Finanzberichte'!$CE$13,'III. Finanzberichte'!$CL$13,'III. Finanzberichte'!$CS$13,'III. Finanzberichte'!$CZ$13,'III. Finanzberichte'!$DG$13,'III. Finanzberichte'!$DN$13,'III. Finanzberichte'!$DU$13),2),0)</f>
-      </c>
-      <c r="H77" s="211" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
-      </c>
-      <c r="I77" s="181" t="str">
-        <f>=ROUND(IFERROR($G$77-$H$77,0),2)</f>
-      </c>
-      <c r="J77" s="280" t="str">
-        <f>=ROUND(IFERROR(($G$77/$H$77)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="255" t="s">
-        <v>199</v>
-      </c>
-      <c r="C78" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$14,'III. Finanzberichte'!$L$14,'III. Finanzberichte'!$S$14,'III. Finanzberichte'!$Z$14,'III. Finanzberichte'!$AG$14,'III. Finanzberichte'!$AN$14,'III. Finanzberichte'!$AU$14,'III. Finanzberichte'!$BB$14,'III. Finanzberichte'!$BI$14,'III. Finanzberichte'!$BP$14,'III. Finanzberichte'!$BW$14,'III. Finanzberichte'!$CD$14,'III. Finanzberichte'!$CK$14,'III. Finanzberichte'!$CR$14,'III. Finanzberichte'!$CY$14,'III. Finanzberichte'!$DF$14,'III. Finanzberichte'!$DM$14,'III. Finanzberichte'!$DT$14),2),0)</f>
-      </c>
-      <c r="D78" s="229" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
-      </c>
-      <c r="E78" s="246" t="str">
-        <f>=ROUND(IFERROR($C$78-$D$78,0),2)</f>
-      </c>
-      <c r="F78" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$78/$D$78)-1,0),4)</f>
-      </c>
-      <c r="G78" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$14,'III. Finanzberichte'!$M$14,'III. Finanzberichte'!$T$14,'III. Finanzberichte'!$AA$14,'III. Finanzberichte'!$AH$14,'III. Finanzberichte'!$AO$14,'III. Finanzberichte'!$AV$14,'III. Finanzberichte'!$BC$14,'III. Finanzberichte'!$BJ$14,'III. Finanzberichte'!$BQ$14,'III. Finanzberichte'!$BX$14,'III. Finanzberichte'!$CE$14,'III. Finanzberichte'!$CL$14,'III. Finanzberichte'!$CS$14,'III. Finanzberichte'!$CZ$14,'III. Finanzberichte'!$DG$14,'III. Finanzberichte'!$DN$14,'III. Finanzberichte'!$DU$14),2),0)</f>
-      </c>
-      <c r="H78" s="211" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
-      </c>
-      <c r="I78" s="181" t="str">
-        <f>=ROUND(IFERROR($G$78-$H$78,0),2)</f>
-      </c>
-      <c r="J78" s="281" t="str">
-        <f>=ROUND(IFERROR(($G$78/$H$78)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="255" t="s">
-        <v>278</v>
-      </c>
-      <c r="C79" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$15,'III. Finanzberichte'!$L$15,'III. Finanzberichte'!$S$15,'III. Finanzberichte'!$Z$15,'III. Finanzberichte'!$AG$15,'III. Finanzberichte'!$AN$15,'III. Finanzberichte'!$AU$15,'III. Finanzberichte'!$BB$15,'III. Finanzberichte'!$BI$15,'III. Finanzberichte'!$BP$15,'III. Finanzberichte'!$BW$15,'III. Finanzberichte'!$CD$15,'III. Finanzberichte'!$CK$15,'III. Finanzberichte'!$CR$15,'III. Finanzberichte'!$CY$15,'III. Finanzberichte'!$DF$15,'III. Finanzberichte'!$DM$15,'III. Finanzberichte'!$DT$15),2),0)</f>
-      </c>
-      <c r="D79" s="229" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
-      </c>
-      <c r="E79" s="246" t="str">
-        <f>=ROUND(IFERROR($C$79-$D$79,0),2)</f>
-      </c>
-      <c r="F79" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$79/$D$79)-1,0),4)</f>
-      </c>
-      <c r="G79" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$15,'III. Finanzberichte'!$M$15,'III. Finanzberichte'!$T$15,'III. Finanzberichte'!$AA$15,'III. Finanzberichte'!$AH$15,'III. Finanzberichte'!$AO$15,'III. Finanzberichte'!$AV$15,'III. Finanzberichte'!$BC$15,'III. Finanzberichte'!$BJ$15,'III. Finanzberichte'!$BQ$15,'III. Finanzberichte'!$BX$15,'III. Finanzberichte'!$CE$15,'III. Finanzberichte'!$CL$15,'III. Finanzberichte'!$CS$15,'III. Finanzberichte'!$CZ$15,'III. Finanzberichte'!$DG$15,'III. Finanzberichte'!$DN$15,'III. Finanzberichte'!$DU$15),2),0)</f>
-      </c>
-      <c r="H79" s="211" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
-      </c>
-      <c r="I79" s="181" t="str">
-        <f>=ROUND(IFERROR($G$79-$H$79,0),2)</f>
-      </c>
-      <c r="J79" s="282" t="str">
-        <f>=ROUND(IFERROR(($G$79/$H$79)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="80" ht="20" customHeight="true">
-      <c r="B80" s="260" t="s">
+      <c r="I110" s="181" t="str">
+        <f>=ROUND(IFERROR($G$110-$H$110,0),2)</f>
+      </c>
+      <c r="J110" s="300" t="str">
+        <f>=ROUND(IFERROR(($G$110/$H$110)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="true">
+      <c r="B111" s="269" t="s">
         <v>266</v>
       </c>
-      <c r="C80" s="261" t="str">
-        <f>=ROUND(SUM($C$76:$C$79),2)</f>
-      </c>
-      <c r="D80" s="261" t="str">
-        <f>=ROUND(SUM($D$76:$D$79),2)</f>
-      </c>
-      <c r="E80" s="261" t="str">
-        <f>=ROUND(SUM($E$76:$E$79),2)</f>
-      </c>
-      <c r="F80" s="283" t="str">
-        <f>=ROUND(IFERROR(($C$80/$D$80)-1,0),4)</f>
-      </c>
-      <c r="G80" s="263" t="str">
-        <f>=ROUND(SUM($G$76:$G$79),2)</f>
-      </c>
-      <c r="H80" s="263" t="str">
-        <f>=ROUND(SUM($H$76:$H$79),2)</f>
-      </c>
-      <c r="I80" s="263" t="str">
-        <f>=ROUND(SUM($I$76:$I$79),2)</f>
-      </c>
-      <c r="J80" s="284" t="str">
-        <f>=ROUND(IFERROR(($G$80/$H$80)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="82" ht="22" customHeight="true">
-      <c r="B82" s="18" t="s">
-        <v>372</v>
-      </c>
-      <c r="C82" s="18"/>
-      <c r="D82" s="18"/>
-      <c r="E82" s="18"/>
-      <c r="F82" s="18"/>
-      <c r="G82" s="18"/>
-      <c r="H82" s="18"/>
-      <c r="I82" s="18"/>
-      <c r="J82" s="18"/>
-    </row>
-    <row r="84" ht="28" customHeight="true">
-      <c r="B84" s="252" t="s">
-        <v>353</v>
-      </c>
-      <c r="C84" s="253" t="s">
-        <v>370</v>
-      </c>
-      <c r="D84" s="253" t="s">
-        <v>355</v>
-      </c>
-      <c r="E84" s="253" t="s">
-        <v>356</v>
-      </c>
-      <c r="F84" s="253" t="s">
-        <v>357</v>
-      </c>
-      <c r="G84" s="253" t="s">
-        <v>371</v>
-      </c>
-      <c r="H84" s="253" t="s">
-        <v>359</v>
-      </c>
-      <c r="I84" s="253" t="s">
-        <v>360</v>
-      </c>
-      <c r="J84" s="254" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" s="255" t="s">
-        <v>205</v>
-      </c>
-      <c r="C85" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$19,'III. Finanzberichte'!$L$19,'III. Finanzberichte'!$S$19,'III. Finanzberichte'!$Z$19,'III. Finanzberichte'!$AG$19,'III. Finanzberichte'!$AN$19,'III. Finanzberichte'!$AU$19,'III. Finanzberichte'!$BB$19,'III. Finanzberichte'!$BI$19,'III. Finanzberichte'!$BP$19,'III. Finanzberichte'!$BW$19,'III. Finanzberichte'!$CD$19,'III. Finanzberichte'!$CK$19,'III. Finanzberichte'!$CR$19,'III. Finanzberichte'!$CY$19,'III. Finanzberichte'!$DF$19,'III. Finanzberichte'!$DM$19,'III. Finanzberichte'!$DT$19),2),0)</f>
-      </c>
-      <c r="D85" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
-      </c>
-      <c r="E85" s="246" t="str">
-        <f>=ROUND(IFERROR($C$85-$D$85,0),2)</f>
-      </c>
-      <c r="F85" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$85/$D$85)-1,0),4)</f>
-      </c>
-      <c r="G85" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$19,'III. Finanzberichte'!$M$19,'III. Finanzberichte'!$T$19,'III. Finanzberichte'!$AA$19,'III. Finanzberichte'!$AH$19,'III. Finanzberichte'!$AO$19,'III. Finanzberichte'!$AV$19,'III. Finanzberichte'!$BC$19,'III. Finanzberichte'!$BJ$19,'III. Finanzberichte'!$BQ$19,'III. Finanzberichte'!$BX$19,'III. Finanzberichte'!$CE$19,'III. Finanzberichte'!$CL$19,'III. Finanzberichte'!$CS$19,'III. Finanzberichte'!$CZ$19,'III. Finanzberichte'!$DG$19,'III. Finanzberichte'!$DN$19,'III. Finanzberichte'!$DU$19),2),0)</f>
-      </c>
-      <c r="H85" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
-      </c>
-      <c r="I85" s="181" t="str">
-        <f>=ROUND(IFERROR($G$85-$H$85,0),2)</f>
-      </c>
-      <c r="J85" s="285" t="str">
-        <f>=ROUND(IFERROR(($G$85/$H$85)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="255" t="s">
-        <v>206</v>
-      </c>
-      <c r="C86" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$20,'III. Finanzberichte'!$L$20,'III. Finanzberichte'!$S$20,'III. Finanzberichte'!$Z$20,'III. Finanzberichte'!$AG$20,'III. Finanzberichte'!$AN$20,'III. Finanzberichte'!$AU$20,'III. Finanzberichte'!$BB$20,'III. Finanzberichte'!$BI$20,'III. Finanzberichte'!$BP$20,'III. Finanzberichte'!$BW$20,'III. Finanzberichte'!$CD$20,'III. Finanzberichte'!$CK$20,'III. Finanzberichte'!$CR$20,'III. Finanzberichte'!$CY$20,'III. Finanzberichte'!$DF$20,'III. Finanzberichte'!$DM$20,'III. Finanzberichte'!$DT$20),2),0)</f>
-      </c>
-      <c r="D86" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
-      </c>
-      <c r="E86" s="246" t="str">
-        <f>=ROUND(IFERROR($C$86-$D$86,0),2)</f>
-      </c>
-      <c r="F86" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$86/$D$86)-1,0),4)</f>
-      </c>
-      <c r="G86" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$20,'III. Finanzberichte'!$M$20,'III. Finanzberichte'!$T$20,'III. Finanzberichte'!$AA$20,'III. Finanzberichte'!$AH$20,'III. Finanzberichte'!$AO$20,'III. Finanzberichte'!$AV$20,'III. Finanzberichte'!$BC$20,'III. Finanzberichte'!$BJ$20,'III. Finanzberichte'!$BQ$20,'III. Finanzberichte'!$BX$20,'III. Finanzberichte'!$CE$20,'III. Finanzberichte'!$CL$20,'III. Finanzberichte'!$CS$20,'III. Finanzberichte'!$CZ$20,'III. Finanzberichte'!$DG$20,'III. Finanzberichte'!$DN$20,'III. Finanzberichte'!$DU$20),2),0)</f>
-      </c>
-      <c r="H86" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
-      </c>
-      <c r="I86" s="181" t="str">
-        <f>=ROUND(IFERROR($G$86-$H$86,0),2)</f>
-      </c>
-      <c r="J86" s="286" t="str">
-        <f>=ROUND(IFERROR(($G$86/$H$86)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="255" t="s">
-        <v>207</v>
-      </c>
-      <c r="C87" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$21,'III. Finanzberichte'!$L$21,'III. Finanzberichte'!$S$21,'III. Finanzberichte'!$Z$21,'III. Finanzberichte'!$AG$21,'III. Finanzberichte'!$AN$21,'III. Finanzberichte'!$AU$21,'III. Finanzberichte'!$BB$21,'III. Finanzberichte'!$BI$21,'III. Finanzberichte'!$BP$21,'III. Finanzberichte'!$BW$21,'III. Finanzberichte'!$CD$21,'III. Finanzberichte'!$CK$21,'III. Finanzberichte'!$CR$21,'III. Finanzberichte'!$CY$21,'III. Finanzberichte'!$DF$21,'III. Finanzberichte'!$DM$21,'III. Finanzberichte'!$DT$21),2),0)</f>
-      </c>
-      <c r="D87" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
-      </c>
-      <c r="E87" s="246" t="str">
-        <f>=ROUND(IFERROR($C$87-$D$87,0),2)</f>
-      </c>
-      <c r="F87" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$87/$D$87)-1,0),4)</f>
-      </c>
-      <c r="G87" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$21,'III. Finanzberichte'!$M$21,'III. Finanzberichte'!$T$21,'III. Finanzberichte'!$AA$21,'III. Finanzberichte'!$AH$21,'III. Finanzberichte'!$AO$21,'III. Finanzberichte'!$AV$21,'III. Finanzberichte'!$BC$21,'III. Finanzberichte'!$BJ$21,'III. Finanzberichte'!$BQ$21,'III. Finanzberichte'!$BX$21,'III. Finanzberichte'!$CE$21,'III. Finanzberichte'!$CL$21,'III. Finanzberichte'!$CS$21,'III. Finanzberichte'!$CZ$21,'III. Finanzberichte'!$DG$21,'III. Finanzberichte'!$DN$21,'III. Finanzberichte'!$DU$21),2),0)</f>
-      </c>
-      <c r="H87" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
-      </c>
-      <c r="I87" s="181" t="str">
-        <f>=ROUND(IFERROR($G$87-$H$87,0),2)</f>
-      </c>
-      <c r="J87" s="287" t="str">
-        <f>=ROUND(IFERROR(($G$87/$H$87)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="88">
-      <c r="B88" s="255" t="s">
-        <v>208</v>
-      </c>
-      <c r="C88" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$22,'III. Finanzberichte'!$L$22,'III. Finanzberichte'!$S$22,'III. Finanzberichte'!$Z$22,'III. Finanzberichte'!$AG$22,'III. Finanzberichte'!$AN$22,'III. Finanzberichte'!$AU$22,'III. Finanzberichte'!$BB$22,'III. Finanzberichte'!$BI$22,'III. Finanzberichte'!$BP$22,'III. Finanzberichte'!$BW$22,'III. Finanzberichte'!$CD$22,'III. Finanzberichte'!$CK$22,'III. Finanzberichte'!$CR$22,'III. Finanzberichte'!$CY$22,'III. Finanzberichte'!$DF$22,'III. Finanzberichte'!$DM$22,'III. Finanzberichte'!$DT$22),2),0)</f>
-      </c>
-      <c r="D88" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
-      </c>
-      <c r="E88" s="246" t="str">
-        <f>=ROUND(IFERROR($C$88-$D$88,0),2)</f>
-      </c>
-      <c r="F88" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$88/$D$88)-1,0),4)</f>
-      </c>
-      <c r="G88" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$22,'III. Finanzberichte'!$M$22,'III. Finanzberichte'!$T$22,'III. Finanzberichte'!$AA$22,'III. Finanzberichte'!$AH$22,'III. Finanzberichte'!$AO$22,'III. Finanzberichte'!$AV$22,'III. Finanzberichte'!$BC$22,'III. Finanzberichte'!$BJ$22,'III. Finanzberichte'!$BQ$22,'III. Finanzberichte'!$BX$22,'III. Finanzberichte'!$CE$22,'III. Finanzberichte'!$CL$22,'III. Finanzberichte'!$CS$22,'III. Finanzberichte'!$CZ$22,'III. Finanzberichte'!$DG$22,'III. Finanzberichte'!$DN$22,'III. Finanzberichte'!$DU$22),2),0)</f>
-      </c>
-      <c r="H88" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
-      </c>
-      <c r="I88" s="181" t="str">
-        <f>=ROUND(IFERROR($G$88-$H$88,0),2)</f>
-      </c>
-      <c r="J88" s="288" t="str">
-        <f>=ROUND(IFERROR(($G$88/$H$88)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="255" t="s">
-        <v>209</v>
-      </c>
-      <c r="C89" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$23,'III. Finanzberichte'!$L$23,'III. Finanzberichte'!$S$23,'III. Finanzberichte'!$Z$23,'III. Finanzberichte'!$AG$23,'III. Finanzberichte'!$AN$23,'III. Finanzberichte'!$AU$23,'III. Finanzberichte'!$BB$23,'III. Finanzberichte'!$BI$23,'III. Finanzberichte'!$BP$23,'III. Finanzberichte'!$BW$23,'III. Finanzberichte'!$CD$23,'III. Finanzberichte'!$CK$23,'III. Finanzberichte'!$CR$23,'III. Finanzberichte'!$CY$23,'III. Finanzberichte'!$DF$23,'III. Finanzberichte'!$DM$23,'III. Finanzberichte'!$DT$23),2),0)</f>
-      </c>
-      <c r="D89" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
-      </c>
-      <c r="E89" s="246" t="str">
-        <f>=ROUND(IFERROR($C$89-$D$89,0),2)</f>
-      </c>
-      <c r="F89" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$89/$D$89)-1,0),4)</f>
-      </c>
-      <c r="G89" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$23,'III. Finanzberichte'!$M$23,'III. Finanzberichte'!$T$23,'III. Finanzberichte'!$AA$23,'III. Finanzberichte'!$AH$23,'III. Finanzberichte'!$AO$23,'III. Finanzberichte'!$AV$23,'III. Finanzberichte'!$BC$23,'III. Finanzberichte'!$BJ$23,'III. Finanzberichte'!$BQ$23,'III. Finanzberichte'!$BX$23,'III. Finanzberichte'!$CE$23,'III. Finanzberichte'!$CL$23,'III. Finanzberichte'!$CS$23,'III. Finanzberichte'!$CZ$23,'III. Finanzberichte'!$DG$23,'III. Finanzberichte'!$DN$23,'III. Finanzberichte'!$DU$23),2),0)</f>
-      </c>
-      <c r="H89" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
-      </c>
-      <c r="I89" s="181" t="str">
-        <f>=ROUND(IFERROR($G$89-$H$89,0),2)</f>
-      </c>
-      <c r="J89" s="289" t="str">
-        <f>=ROUND(IFERROR(($G$89/$H$89)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="255" t="s">
-        <v>210</v>
-      </c>
-      <c r="C90" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$24,'III. Finanzberichte'!$L$24,'III. Finanzberichte'!$S$24,'III. Finanzberichte'!$Z$24,'III. Finanzberichte'!$AG$24,'III. Finanzberichte'!$AN$24,'III. Finanzberichte'!$AU$24,'III. Finanzberichte'!$BB$24,'III. Finanzberichte'!$BI$24,'III. Finanzberichte'!$BP$24,'III. Finanzberichte'!$BW$24,'III. Finanzberichte'!$CD$24,'III. Finanzberichte'!$CK$24,'III. Finanzberichte'!$CR$24,'III. Finanzberichte'!$CY$24,'III. Finanzberichte'!$DF$24,'III. Finanzberichte'!$DM$24,'III. Finanzberichte'!$DT$24),2),0)</f>
-      </c>
-      <c r="D90" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
-      </c>
-      <c r="E90" s="246" t="str">
-        <f>=ROUND(IFERROR($C$90-$D$90,0),2)</f>
-      </c>
-      <c r="F90" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$90/$D$90)-1,0),4)</f>
-      </c>
-      <c r="G90" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$24,'III. Finanzberichte'!$M$24,'III. Finanzberichte'!$T$24,'III. Finanzberichte'!$AA$24,'III. Finanzberichte'!$AH$24,'III. Finanzberichte'!$AO$24,'III. Finanzberichte'!$AV$24,'III. Finanzberichte'!$BC$24,'III. Finanzberichte'!$BJ$24,'III. Finanzberichte'!$BQ$24,'III. Finanzberichte'!$BX$24,'III. Finanzberichte'!$CE$24,'III. Finanzberichte'!$CL$24,'III. Finanzberichte'!$CS$24,'III. Finanzberichte'!$CZ$24,'III. Finanzberichte'!$DG$24,'III. Finanzberichte'!$DN$24,'III. Finanzberichte'!$DU$24),2),0)</f>
-      </c>
-      <c r="H90" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
-      </c>
-      <c r="I90" s="181" t="str">
-        <f>=ROUND(IFERROR($G$90-$H$90,0),2)</f>
-      </c>
-      <c r="J90" s="290" t="str">
-        <f>=ROUND(IFERROR(($G$90/$H$90)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="255" t="s">
-        <v>211</v>
-      </c>
-      <c r="C91" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$25,'III. Finanzberichte'!$L$25,'III. Finanzberichte'!$S$25,'III. Finanzberichte'!$Z$25,'III. Finanzberichte'!$AG$25,'III. Finanzberichte'!$AN$25,'III. Finanzberichte'!$AU$25,'III. Finanzberichte'!$BB$25,'III. Finanzberichte'!$BI$25,'III. Finanzberichte'!$BP$25,'III. Finanzberichte'!$BW$25,'III. Finanzberichte'!$CD$25,'III. Finanzberichte'!$CK$25,'III. Finanzberichte'!$CR$25,'III. Finanzberichte'!$CY$25,'III. Finanzberichte'!$DF$25,'III. Finanzberichte'!$DM$25,'III. Finanzberichte'!$DT$25),2),0)</f>
-      </c>
-      <c r="D91" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
-      </c>
-      <c r="E91" s="246" t="str">
-        <f>=ROUND(IFERROR($C$91-$D$91,0),2)</f>
-      </c>
-      <c r="F91" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$91/$D$91)-1,0),4)</f>
-      </c>
-      <c r="G91" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$25,'III. Finanzberichte'!$M$25,'III. Finanzberichte'!$T$25,'III. Finanzberichte'!$AA$25,'III. Finanzberichte'!$AH$25,'III. Finanzberichte'!$AO$25,'III. Finanzberichte'!$AV$25,'III. Finanzberichte'!$BC$25,'III. Finanzberichte'!$BJ$25,'III. Finanzberichte'!$BQ$25,'III. Finanzberichte'!$BX$25,'III. Finanzberichte'!$CE$25,'III. Finanzberichte'!$CL$25,'III. Finanzberichte'!$CS$25,'III. Finanzberichte'!$CZ$25,'III. Finanzberichte'!$DG$25,'III. Finanzberichte'!$DN$25,'III. Finanzberichte'!$DU$25),2),0)</f>
-      </c>
-      <c r="H91" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
-      </c>
-      <c r="I91" s="181" t="str">
-        <f>=ROUND(IFERROR($G$91-$H$91,0),2)</f>
-      </c>
-      <c r="J91" s="291" t="str">
-        <f>=ROUND(IFERROR(($G$91/$H$91)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" s="255" t="s">
-        <v>212</v>
-      </c>
-      <c r="C92" s="229" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$E$26,'III. Finanzberichte'!$L$26,'III. Finanzberichte'!$S$26,'III. Finanzberichte'!$Z$26,'III. Finanzberichte'!$AG$26,'III. Finanzberichte'!$AN$26,'III. Finanzberichte'!$AU$26,'III. Finanzberichte'!$BB$26,'III. Finanzberichte'!$BI$26,'III. Finanzberichte'!$BP$26,'III. Finanzberichte'!$BW$26,'III. Finanzberichte'!$CD$26,'III. Finanzberichte'!$CK$26,'III. Finanzberichte'!$CR$26,'III. Finanzberichte'!$CY$26,'III. Finanzberichte'!$DF$26,'III. Finanzberichte'!$DM$26,'III. Finanzberichte'!$DT$26),2),0)</f>
-      </c>
-      <c r="D92" s="229" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
-      </c>
-      <c r="E92" s="246" t="str">
-        <f>=ROUND(IFERROR($C$92-$D$92,0),2)</f>
-      </c>
-      <c r="F92" s="247" t="str">
-        <f>=ROUND(IFERROR(($C$92/$D$92)-1,0),4)</f>
-      </c>
-      <c r="G92" s="211" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(N65,'III. Finanzberichte'!$F$26,'III. Finanzberichte'!$M$26,'III. Finanzberichte'!$T$26,'III. Finanzberichte'!$AA$26,'III. Finanzberichte'!$AH$26,'III. Finanzberichte'!$AO$26,'III. Finanzberichte'!$AV$26,'III. Finanzberichte'!$BC$26,'III. Finanzberichte'!$BJ$26,'III. Finanzberichte'!$BQ$26,'III. Finanzberichte'!$BX$26,'III. Finanzberichte'!$CE$26,'III. Finanzberichte'!$CL$26,'III. Finanzberichte'!$CS$26,'III. Finanzberichte'!$CZ$26,'III. Finanzberichte'!$DG$26,'III. Finanzberichte'!$DN$26,'III. Finanzberichte'!$DU$26),2),0)</f>
-      </c>
-      <c r="H92" s="211" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
-      </c>
-      <c r="I92" s="181" t="str">
-        <f>=ROUND(IFERROR($G$92-$H$92,0),2)</f>
-      </c>
-      <c r="J92" s="292" t="str">
-        <f>=ROUND(IFERROR(($G$92/$H$92)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="93" ht="20" customHeight="true">
-      <c r="B93" s="260" t="s">
-        <v>266</v>
-      </c>
-      <c r="C93" s="261" t="str">
-        <f>=ROUND(SUM($C$85:$C$92),2)</f>
-      </c>
-      <c r="D93" s="261" t="str">
-        <f>=ROUND(SUM($D$85:$D$92),2)</f>
-      </c>
-      <c r="E93" s="261" t="str">
-        <f>=ROUND(SUM($E$85:$E$92),2)</f>
-      </c>
-      <c r="F93" s="293" t="str">
-        <f>=ROUND(IFERROR(($C$93/$D$93)-1,0),4)</f>
-      </c>
-      <c r="G93" s="263" t="str">
-        <f>=ROUND(SUM($G$85:$G$92),2)</f>
-      </c>
-      <c r="H93" s="263" t="str">
-        <f>=ROUND(SUM($H$85:$H$92),2)</f>
-      </c>
-      <c r="I93" s="263" t="str">
-        <f>=ROUND(SUM($I$85:$I$92),2)</f>
-      </c>
-      <c r="J93" s="294" t="str">
-        <f>=ROUND(IFERROR(($G$93/$H$93)-1,0),4)</f>
+      <c r="C111" s="270" t="str">
+        <f>=ROUND(SUM($C$103:$C$110),2)</f>
+      </c>
+      <c r="D111" s="270" t="str">
+        <f>=ROUND(SUM($D$103:$D$110),2)</f>
+      </c>
+      <c r="E111" s="270" t="str">
+        <f>=ROUND(SUM($E$103:$E$110),2)</f>
+      </c>
+      <c r="F111" s="301" t="str">
+        <f>=ROUND(IFERROR(($C$111/$D$111)-1,0),4)</f>
+      </c>
+      <c r="G111" s="272" t="str">
+        <f>=ROUND(SUM($G$103:$G$110),2)</f>
+      </c>
+      <c r="H111" s="272" t="str">
+        <f>=ROUND(SUM($H$103:$H$110),2)</f>
+      </c>
+      <c r="I111" s="272" t="str">
+        <f>=ROUND(SUM($I$103:$I$110),2)</f>
+      </c>
+      <c r="J111" s="302" t="str">
+        <f>=ROUND(IFERROR(($G$111/$H$111)-1,0),4)</f>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="80">
+  <mergeCells count="88">
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="B5:J5"/>
     <mergeCell ref="B6:J6"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="F10:I10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="F29:H29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="F30:H30"/>
     <mergeCell ref="B32:C32"/>
+    <mergeCell ref="F32:H32"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B38:J38"/>
-    <mergeCell ref="B47:J47"/>
-    <mergeCell ref="B60:J60"/>
-    <mergeCell ref="B61:J61"/>
-    <mergeCell ref="L63:O63"/>
-    <mergeCell ref="L64:O64"/>
-    <mergeCell ref="L65:M65"/>
-    <mergeCell ref="N65:O65"/>
-    <mergeCell ref="L66:M66"/>
-    <mergeCell ref="N66:O66"/>
-    <mergeCell ref="L67:M67"/>
-    <mergeCell ref="N67:O67"/>
-    <mergeCell ref="B63:J63"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="F65:I65"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B50:J50"/>
+    <mergeCell ref="B59:J59"/>
+    <mergeCell ref="B72:J72"/>
     <mergeCell ref="B73:J73"/>
-    <mergeCell ref="B82:J82"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="C75:I75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="F76:I76"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="F77:I77"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="F78:I78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="F79:I79"/>
+    <mergeCell ref="B81:J81"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="F83:I83"/>
+    <mergeCell ref="G84:H84"/>
+    <mergeCell ref="G85:H85"/>
+    <mergeCell ref="G86:H86"/>
+    <mergeCell ref="G87:H87"/>
+    <mergeCell ref="B91:J91"/>
+    <mergeCell ref="B100:J100"/>
   </mergeCells>
-  <conditionalFormatting sqref="D34">
+  <conditionalFormatting sqref="C13:I13">
     <cfRule type="expression" dxfId="9" priority="1">
-      <formula>$D$34="OK"</formula>
+      <formula>$C$13&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D34">
-    <cfRule type="expression" dxfId="10" priority="2">
-      <formula>$D$34&lt;&gt;"OK"</formula>
+  <conditionalFormatting sqref="C14:I14">
+    <cfRule type="expression" dxfId="9" priority="2">
+      <formula>$C$14&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D35">
-    <cfRule type="expression" dxfId="11" priority="3">
-      <formula>$D$35&gt;0</formula>
+  <conditionalFormatting sqref="C15:I15">
+    <cfRule type="expression" dxfId="9" priority="3">
+      <formula>$C$15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F50:F57">
-    <cfRule type="expression" dxfId="12" priority="4">
-      <formula>F50&gt;0.2</formula>
+  <conditionalFormatting sqref="C16:I16">
+    <cfRule type="expression" dxfId="9" priority="4">
+      <formula>$C$16&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F50:F57">
-    <cfRule type="expression" dxfId="13" priority="5">
-      <formula>AND(F50&gt;=0.1,F50&lt;=0.2)</formula>
+  <conditionalFormatting sqref="C17:I17">
+    <cfRule type="expression" dxfId="9" priority="5">
+      <formula>$C$17&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J50:J57">
-    <cfRule type="expression" dxfId="12" priority="6">
-      <formula>J50&gt;0.2</formula>
+  <conditionalFormatting sqref="C18:I18">
+    <cfRule type="expression" dxfId="9" priority="6">
+      <formula>$C$18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J50:J57">
-    <cfRule type="expression" dxfId="13" priority="7">
-      <formula>AND(J50&gt;=0.1,J50&lt;=0.2)</formula>
+  <conditionalFormatting sqref="D46">
+    <cfRule type="expression" dxfId="10" priority="7">
+      <formula>$D$46="OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F85:F92">
-    <cfRule type="expression" dxfId="12" priority="8">
-      <formula>F85&gt;0.2</formula>
+  <conditionalFormatting sqref="D46">
+    <cfRule type="expression" dxfId="11" priority="8">
+      <formula>$D$46&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F85:F92">
-    <cfRule type="expression" dxfId="13" priority="9">
-      <formula>AND(F85&gt;=0.1,F85&lt;=0.2)</formula>
+  <conditionalFormatting sqref="D47">
+    <cfRule type="expression" dxfId="12" priority="9">
+      <formula>$D$47&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J85:J92">
-    <cfRule type="expression" dxfId="12" priority="10">
-      <formula>J85&gt;0.2</formula>
+  <conditionalFormatting sqref="F62:F69">
+    <cfRule type="expression" dxfId="13" priority="10">
+      <formula>F62&gt;0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J85:J92">
-    <cfRule type="expression" dxfId="13" priority="11">
-      <formula>AND(J85&gt;=0.1,J85&lt;=0.2)</formula>
+  <conditionalFormatting sqref="F62:F69">
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>AND(F62&gt;=0.1,F62&lt;=0.2)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L13:O13">
-    <cfRule type="expression" dxfId="14" priority="12">
-      <formula>$L$13&lt;&gt;""</formula>
+  <conditionalFormatting sqref="J62:J69">
+    <cfRule type="expression" dxfId="13" priority="12">
+      <formula>J62&gt;0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L14:O14">
+  <conditionalFormatting sqref="J62:J69">
     <cfRule type="expression" dxfId="14" priority="13">
-      <formula>$L$14&lt;&gt;""</formula>
+      <formula>AND(J62&gt;=0.1,J62&lt;=0.2)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L15:O15">
-    <cfRule type="expression" dxfId="14" priority="14">
-      <formula>$L$15&lt;&gt;""</formula>
+  <conditionalFormatting sqref="F103:F110">
+    <cfRule type="expression" dxfId="13" priority="14">
+      <formula>F103&gt;0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L16:O16">
+  <conditionalFormatting sqref="F103:F110">
     <cfRule type="expression" dxfId="14" priority="15">
-      <formula>$L$16&lt;&gt;""</formula>
+      <formula>AND(F103&gt;=0.1,F103&lt;=0.2)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L17:O17">
-    <cfRule type="expression" dxfId="14" priority="16">
-      <formula>$L$17&lt;&gt;""</formula>
+  <conditionalFormatting sqref="J103:J110">
+    <cfRule type="expression" dxfId="13" priority="16">
+      <formula>J103&gt;0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L18:O18">
+  <conditionalFormatting sqref="J103:J110">
     <cfRule type="expression" dxfId="14" priority="17">
-      <formula>$L$18&lt;&gt;""</formula>
+      <formula>AND(J103&gt;=0.1,J103&lt;=0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="8">
-    <dataValidation allowBlank="true" sqref="L9" type="list">
+    <dataValidation allowBlank="true" sqref="F9" type="list">
       <formula1>=MA_Auswahl_Liste</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F11" type="list">
+    <dataValidation allowBlank="true" sqref="F23" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F12" type="list">
+    <dataValidation allowBlank="true" sqref="F24" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F13" type="list">
+    <dataValidation allowBlank="true" sqref="F25" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="D28" type="list">
+    <dataValidation allowBlank="true" sqref="D40" type="list">
       <formula1>"Jahr 1,Jahr 2,Jahr 3"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="L64" type="list">
+    <dataValidation allowBlank="true" sqref="F76" type="list">
       <formula1>=FB_Auswahl_Liste</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F66" type="list">
+    <dataValidation allowBlank="true" sqref="F84" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F67" type="list">
+    <dataValidation allowBlank="true" sqref="F85" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
   </dataValidations>
@@ -21591,17 +21730,17 @@
       <c r="A1" t="s">
         <v>226</v>
       </c>
-      <c r="C1" s="295" t="s">
-        <v>373</v>
-      </c>
-      <c r="I1" s="295" t="s">
+      <c r="C1" s="303" t="s">
         <v>374</v>
       </c>
-      <c r="O1" s="295" t="s">
+      <c r="I1" s="303" t="s">
         <v>375</v>
       </c>
-      <c r="U1" s="295" t="s">
+      <c r="O1" s="303" t="s">
         <v>376</v>
+      </c>
+      <c r="U1" s="303" t="s">
+        <v>377</v>
       </c>
       <c r="BA1">
         <v>1</v>
@@ -21637,11 +21776,11 @@
         <f>=IF(BK1=1,"Periode "&amp;BJ1,"")</f>
       </c>
       <c r="BN1" cm="1" s="3">
-        <f t="array" ref="BN1">_xlfn._xlws.FILTER($BE$1:$BE$18,($BB$1:$BB$18='V. AUSWERTUNG'!N65+1)*($BC$1:$BC$18=1),"")</f>
+        <f t="array" ref="BN1">_xlfn._xlws.FILTER($BE$1:$BE$18,($BB$1:$BB$18='V. AUSWERTUNG'!F77+1)*($BC$1:$BC$18=1),"")</f>
         <v>0</v>
       </c>
       <c r="BP1" cm="1" s="3">
-        <f t="array" ref="BP1">_xlfn._xlws.FILTER($BL$1:$BL$18,$BK$1:$BK$18=1,"")</f>
+        <f t="array" ref="BP1">_xlfn.VSTACK("Kein Finanzbericht (Projektbeginn)",_xlfn._xlws.FILTER($BL$1:$BL$18,$BK$1:$BK$18=1,""))</f>
         <v>0</v>
       </c>
       <c r="BR1" t="str">

</xml_diff>

<commit_message>
feat: add mirror panels and currency support to evaluation sheet
- Implement `evalDrawMAMirrorPanel` and `evalDrawFBMirrorPanel` to display dynamic, read-only mirrors of selected source documents.
- Support dual-currency (LC/EUR) display in the Monatslimit-Prüfung.
- Add `reapplyRightBorder` helper to maintain outer table borders after dynamic cell updates.
- Refactor Monatslimit-Prüfung logic to support dynamic currency conversion and consistent styling.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="384">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1175,19 +1175,25 @@
     <t>Abzüglich manueller Betrag</t>
   </si>
   <si>
-    <t>Monatslimit-Prüfung (Lokalwährung)</t>
+    <t>Monatslimit-Prüfung</t>
+  </si>
+  <si>
+    <t>Lokalwährung</t>
+  </si>
+  <si>
+    <t>Euro</t>
   </si>
   <si>
     <t>Geprüfte Periode (aus MA-Auswahl)</t>
   </si>
   <si>
-    <t>Anforderungshöhe (LC)</t>
+    <t>Anforderungshöhe</t>
   </si>
   <si>
     <t>Jahr</t>
   </si>
   <si>
-    <t>Jahresbudget (LC)</t>
+    <t>Jahresbudget</t>
   </si>
   <si>
     <t>Limit-Monate</t>
@@ -1199,13 +1205,13 @@
     <t>Anforderung deckt (Monate)</t>
   </si>
   <si>
-    <t>8-Monats-Limit (LC)</t>
+    <t>8-Monats-Limit</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Überschreitung (LC)</t>
+    <t>Überschreitung</t>
   </si>
   <si>
     <t>Auslastung %</t>
@@ -1272,6 +1278,18 @@
   </si>
   <si>
     <t>Soll-Ist Abweichungsprüfung</t>
+  </si>
+  <si>
+    <t>Aktuelle Mittelanforderung</t>
+  </si>
+  <si>
+    <t>abzüglich Eigenmittel:</t>
+  </si>
+  <si>
+    <t>abzüglich Drittmittel:</t>
+  </si>
+  <si>
+    <t>Aktueller Finanzbericht</t>
   </si>
   <si>
     <t>Einnahmen_Explizit_Stack</t>
@@ -1545,7 +1563,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="53">
+  <borders count="56">
     <border>
       <left/>
       <right/>
@@ -2128,11 +2146,53 @@
         <color rgb="FF808080"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="double">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="double">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="double">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="304">
+  <cellXfs count="346">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
@@ -2845,14 +2905,17 @@
     <xf numFmtId="167" fontId="3" fillId="5" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="171" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="171" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
@@ -2863,68 +2926,140 @@
     <xf numFmtId="172" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="39" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="40" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
@@ -2938,18 +3073,9 @@
     <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2983,61 +3109,121 @@
     <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="170" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="10" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="12" fillId="10" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="19" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="10" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="12" fillId="10" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="6" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="6" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="12" fillId="6" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="53" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="53" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="6" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="30" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="31" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="6" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="54" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="54" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="55" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
@@ -3047,7 +3233,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="18">
     <dxf>
       <font>
         <name val="Segoe UI"/>
@@ -3359,6 +3545,62 @@
         <name val="Segoe UI"/>
         <family val="2"/>
         <b val="1"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
         <color rgb="FF9C0006"/>
       </font>
       <numFmt numFmtId="165" formatCode="#,##0.00"/>
@@ -3390,7 +3632,36 @@
         <b val="1"/>
         <color rgb="FF9C0006"/>
       </font>
-      <numFmt numFmtId="166" formatCode="0.0%"/>
+      <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF808080"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF808080"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF808080"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <numFmt numFmtId="167" formatCode="0.0%"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
@@ -3419,7 +3690,7 @@
         <b val="1"/>
         <color rgb="FF9C640C"/>
       </font>
-      <numFmt numFmtId="167" formatCode="0.0%"/>
+      <numFmt numFmtId="168" formatCode="0.0%"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFCF3CF"/>
@@ -19844,6 +20115,10 @@
     <col customWidth="true" max="1" min="1" width="3"/>
     <col customWidth="true" max="2" min="2" width="34"/>
     <col customWidth="true" max="10" min="3" width="16"/>
+    <col customWidth="true" max="11" min="11" width="3"/>
+    <col customWidth="true" max="12" min="12" width="25"/>
+    <col customWidth="true" max="16" min="13" width="18"/>
+    <col customWidth="true" hidden="true" max="30" min="30" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="true">
@@ -19872,7 +20147,7 @@
       <c r="I3" s="192"/>
       <c r="J3" s="192"/>
     </row>
-    <row r="5" ht="26" customHeight="true">
+    <row r="5" ht="22" customHeight="true">
       <c r="B5" s="193" t="s">
         <v>317</v>
       </c>
@@ -19884,6 +20159,14 @@
       <c r="H5" s="193"/>
       <c r="I5" s="193"/>
       <c r="J5" s="193"/>
+      <c r="L5" s="201" t="s">
+        <v>376</v>
+      </c>
+      <c r="M5" s="202"/>
+      <c r="N5" s="203"/>
+      <c r="AD5" t="str">
+        <f>=IFERROR(SUMPRODUCT('Daten'!$BA$1:$BA$18,('Daten'!$BB$1:$BB$18=F10)*('Daten'!$BD$1:$BD$18=F11)),0)</f>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="194" t="s">
@@ -19897,6 +20180,22 @@
       <c r="H6" s="194"/>
       <c r="I6" s="194"/>
       <c r="J6" s="194"/>
+      <c r="L6" s="314" t="s">
+        <v>267</v>
+      </c>
+      <c r="M6" s="307" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$5,'IV. MA'!$G$5,'IV. MA'!$K$5,'IV. MA'!$O$5,'IV. MA'!$S$5,'IV. MA'!$W$5,'IV. MA'!$AA$5,'IV. MA'!$AE$5,'IV. MA'!$AI$5,'IV. MA'!$AM$5,'IV. MA'!$AQ$5,'IV. MA'!$AU$5,'IV. MA'!$AY$5,'IV. MA'!$BC$5,'IV. MA'!$BG$5,'IV. MA'!$BK$5,'IV. MA'!$BO$5,'IV. MA'!$BS$5),"")</f>
+      </c>
+      <c r="N6" s="315"/>
+    </row>
+    <row r="7">
+      <c r="L7" s="314" t="s">
+        <v>268</v>
+      </c>
+      <c r="M7" s="308" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$6,'IV. MA'!$G$6,'IV. MA'!$K$6,'IV. MA'!$O$6,'IV. MA'!$S$6,'IV. MA'!$W$6,'IV. MA'!$AA$6,'IV. MA'!$AE$6,'IV. MA'!$AI$6,'IV. MA'!$AM$6,'IV. MA'!$AQ$6,'IV. MA'!$AU$6,'IV. MA'!$AY$6,'IV. MA'!$BC$6,'IV. MA'!$BG$6,'IV. MA'!$BK$6,'IV. MA'!$BO$6,'IV. MA'!$BS$6),"")</f>
+      </c>
+      <c r="N7" s="316"/>
     </row>
     <row r="8" ht="22" customHeight="true">
       <c r="C8" s="201" t="s">
@@ -19908,6 +20207,13 @@
       <c r="G8" s="202"/>
       <c r="H8" s="202"/>
       <c r="I8" s="203"/>
+      <c r="L8" s="314" t="s">
+        <v>305</v>
+      </c>
+      <c r="M8" s="309" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$7,'IV. MA'!$G$7,'IV. MA'!$K$7,'IV. MA'!$O$7,'IV. MA'!$S$7,'IV. MA'!$W$7,'IV. MA'!$AA$7,'IV. MA'!$AE$7,'IV. MA'!$AI$7,'IV. MA'!$AM$7,'IV. MA'!$AQ$7,'IV. MA'!$AU$7,'IV. MA'!$AY$7,'IV. MA'!$BC$7,'IV. MA'!$BG$7,'IV. MA'!$BK$7,'IV. MA'!$BO$7,'IV. MA'!$BS$7),"")</f>
+      </c>
+      <c r="N8" s="317"/>
     </row>
     <row r="9">
       <c r="C9" s="204" t="s">
@@ -19921,6 +20227,8 @@
       <c r="G9" s="33"/>
       <c r="H9" s="33"/>
       <c r="I9" s="205"/>
+      <c r="L9" s="47"/>
+      <c r="N9" s="48"/>
     </row>
     <row r="10">
       <c r="C10" s="204" t="s">
@@ -19929,12 +20237,21 @@
       <c r="D10" s="196"/>
       <c r="E10" s="196"/>
       <c r="F10" s="197" t="str">
-        <f>=F77+1</f>
+        <f>=F82+1</f>
         <v>0</v>
       </c>
       <c r="G10" s="197"/>
       <c r="H10" s="197"/>
       <c r="I10" s="206"/>
+      <c r="L10" s="318" t="s">
+        <v>202</v>
+      </c>
+      <c r="M10" s="179" t="s">
+        <v>306</v>
+      </c>
+      <c r="N10" s="319" t="s">
+        <v>307</v>
+      </c>
     </row>
     <row r="11">
       <c r="C11" s="204" t="s">
@@ -19948,6 +20265,15 @@
       <c r="G11" s="197"/>
       <c r="H11" s="197"/>
       <c r="I11" s="207"/>
+      <c r="L11" s="142" t="s">
+        <v>205</v>
+      </c>
+      <c r="M11" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$10,'IV. MA'!$G$10,'IV. MA'!$K$10,'IV. MA'!$O$10,'IV. MA'!$S$10,'IV. MA'!$W$10,'IV. MA'!$AA$10,'IV. MA'!$AE$10,'IV. MA'!$AI$10,'IV. MA'!$AM$10,'IV. MA'!$AQ$10,'IV. MA'!$AU$10,'IV. MA'!$AY$10,'IV. MA'!$BC$10,'IV. MA'!$BG$10,'IV. MA'!$BK$10,'IV. MA'!$BO$10,'IV. MA'!$BS$10),"")</f>
+      </c>
+      <c r="N11" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$10,'IV. MA'!$H$10,'IV. MA'!$L$10,'IV. MA'!$P$10,'IV. MA'!$T$10,'IV. MA'!$X$10,'IV. MA'!$AB$10,'IV. MA'!$AF$10,'IV. MA'!$AJ$10,'IV. MA'!$AN$10,'IV. MA'!$AR$10,'IV. MA'!$AV$10,'IV. MA'!$AZ$10,'IV. MA'!$BD$10,'IV. MA'!$BH$10,'IV. MA'!$BL$10,'IV. MA'!$BP$10,'IV. MA'!$BT$10),"")</f>
+      </c>
     </row>
     <row r="12">
       <c r="C12" s="208" t="s">
@@ -19959,6 +20285,15 @@
       <c r="G12" s="198"/>
       <c r="H12" s="198"/>
       <c r="I12" s="209"/>
+      <c r="L12" s="142" t="s">
+        <v>206</v>
+      </c>
+      <c r="M12" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$11,'IV. MA'!$G$11,'IV. MA'!$K$11,'IV. MA'!$O$11,'IV. MA'!$S$11,'IV. MA'!$W$11,'IV. MA'!$AA$11,'IV. MA'!$AE$11,'IV. MA'!$AI$11,'IV. MA'!$AM$11,'IV. MA'!$AQ$11,'IV. MA'!$AU$11,'IV. MA'!$AY$11,'IV. MA'!$BC$11,'IV. MA'!$BG$11,'IV. MA'!$BK$11,'IV. MA'!$BO$11,'IV. MA'!$BS$11),"")</f>
+      </c>
+      <c r="N12" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$11,'IV. MA'!$H$11,'IV. MA'!$L$11,'IV. MA'!$P$11,'IV. MA'!$T$11,'IV. MA'!$X$11,'IV. MA'!$AB$11,'IV. MA'!$AF$11,'IV. MA'!$AJ$11,'IV. MA'!$AN$11,'IV. MA'!$AR$11,'IV. MA'!$AV$11,'IV. MA'!$AZ$11,'IV. MA'!$BD$11,'IV. MA'!$BH$11,'IV. MA'!$BL$11,'IV. MA'!$BP$11,'IV. MA'!$BT$11),"")</f>
+      </c>
     </row>
     <row r="13">
       <c r="C13" s="210" t="str">
@@ -19974,6 +20309,15 @@
         <f>=IF(1&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
       </c>
       <c r="I13" s="211"/>
+      <c r="L13" s="142" t="s">
+        <v>207</v>
+      </c>
+      <c r="M13" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$12,'IV. MA'!$G$12,'IV. MA'!$K$12,'IV. MA'!$O$12,'IV. MA'!$S$12,'IV. MA'!$W$12,'IV. MA'!$AA$12,'IV. MA'!$AE$12,'IV. MA'!$AI$12,'IV. MA'!$AM$12,'IV. MA'!$AQ$12,'IV. MA'!$AU$12,'IV. MA'!$AY$12,'IV. MA'!$BC$12,'IV. MA'!$BG$12,'IV. MA'!$BK$12,'IV. MA'!$BO$12,'IV. MA'!$BS$12),"")</f>
+      </c>
+      <c r="N13" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$12,'IV. MA'!$H$12,'IV. MA'!$L$12,'IV. MA'!$P$12,'IV. MA'!$T$12,'IV. MA'!$X$12,'IV. MA'!$AB$12,'IV. MA'!$AF$12,'IV. MA'!$AJ$12,'IV. MA'!$AN$12,'IV. MA'!$AR$12,'IV. MA'!$AV$12,'IV. MA'!$AZ$12,'IV. MA'!$BD$12,'IV. MA'!$BH$12,'IV. MA'!$BL$12,'IV. MA'!$BP$12,'IV. MA'!$BT$12),"")</f>
+      </c>
     </row>
     <row r="14">
       <c r="C14" s="210" t="str">
@@ -19989,6 +20333,15 @@
         <f>=IF(2&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
       </c>
       <c r="I14" s="211"/>
+      <c r="L14" s="142" t="s">
+        <v>208</v>
+      </c>
+      <c r="M14" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$13,'IV. MA'!$G$13,'IV. MA'!$K$13,'IV. MA'!$O$13,'IV. MA'!$S$13,'IV. MA'!$W$13,'IV. MA'!$AA$13,'IV. MA'!$AE$13,'IV. MA'!$AI$13,'IV. MA'!$AM$13,'IV. MA'!$AQ$13,'IV. MA'!$AU$13,'IV. MA'!$AY$13,'IV. MA'!$BC$13,'IV. MA'!$BG$13,'IV. MA'!$BK$13,'IV. MA'!$BO$13,'IV. MA'!$BS$13),"")</f>
+      </c>
+      <c r="N14" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$13,'IV. MA'!$H$13,'IV. MA'!$L$13,'IV. MA'!$P$13,'IV. MA'!$T$13,'IV. MA'!$X$13,'IV. MA'!$AB$13,'IV. MA'!$AF$13,'IV. MA'!$AJ$13,'IV. MA'!$AN$13,'IV. MA'!$AR$13,'IV. MA'!$AV$13,'IV. MA'!$AZ$13,'IV. MA'!$BD$13,'IV. MA'!$BH$13,'IV. MA'!$BL$13,'IV. MA'!$BP$13,'IV. MA'!$BT$13),"")</f>
+      </c>
     </row>
     <row r="15">
       <c r="C15" s="210" t="str">
@@ -20004,6 +20357,15 @@
         <f>=IF(3&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
       </c>
       <c r="I15" s="211"/>
+      <c r="L15" s="142" t="s">
+        <v>209</v>
+      </c>
+      <c r="M15" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$14,'IV. MA'!$G$14,'IV. MA'!$K$14,'IV. MA'!$O$14,'IV. MA'!$S$14,'IV. MA'!$W$14,'IV. MA'!$AA$14,'IV. MA'!$AE$14,'IV. MA'!$AI$14,'IV. MA'!$AM$14,'IV. MA'!$AQ$14,'IV. MA'!$AU$14,'IV. MA'!$AY$14,'IV. MA'!$BC$14,'IV. MA'!$BG$14,'IV. MA'!$BK$14,'IV. MA'!$BO$14,'IV. MA'!$BS$14),"")</f>
+      </c>
+      <c r="N15" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$14,'IV. MA'!$H$14,'IV. MA'!$L$14,'IV. MA'!$P$14,'IV. MA'!$T$14,'IV. MA'!$X$14,'IV. MA'!$AB$14,'IV. MA'!$AF$14,'IV. MA'!$AJ$14,'IV. MA'!$AN$14,'IV. MA'!$AR$14,'IV. MA'!$AV$14,'IV. MA'!$AZ$14,'IV. MA'!$BD$14,'IV. MA'!$BH$14,'IV. MA'!$BL$14,'IV. MA'!$BP$14,'IV. MA'!$BT$14),"")</f>
+      </c>
     </row>
     <row r="16">
       <c r="C16" s="210" t="str">
@@ -20019,6 +20381,15 @@
         <f>=IF(4&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
       </c>
       <c r="I16" s="211"/>
+      <c r="L16" s="142" t="s">
+        <v>210</v>
+      </c>
+      <c r="M16" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$15,'IV. MA'!$G$15,'IV. MA'!$K$15,'IV. MA'!$O$15,'IV. MA'!$S$15,'IV. MA'!$W$15,'IV. MA'!$AA$15,'IV. MA'!$AE$15,'IV. MA'!$AI$15,'IV. MA'!$AM$15,'IV. MA'!$AQ$15,'IV. MA'!$AU$15,'IV. MA'!$AY$15,'IV. MA'!$BC$15,'IV. MA'!$BG$15,'IV. MA'!$BK$15,'IV. MA'!$BO$15,'IV. MA'!$BS$15),"")</f>
+      </c>
+      <c r="N16" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$15,'IV. MA'!$H$15,'IV. MA'!$L$15,'IV. MA'!$P$15,'IV. MA'!$T$15,'IV. MA'!$X$15,'IV. MA'!$AB$15,'IV. MA'!$AF$15,'IV. MA'!$AJ$15,'IV. MA'!$AN$15,'IV. MA'!$AR$15,'IV. MA'!$AV$15,'IV. MA'!$AZ$15,'IV. MA'!$BD$15,'IV. MA'!$BH$15,'IV. MA'!$BL$15,'IV. MA'!$BP$15,'IV. MA'!$BT$15),"")</f>
+      </c>
     </row>
     <row r="17">
       <c r="C17" s="210" t="str">
@@ -20034,6 +20405,15 @@
         <f>=IF(5&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
       </c>
       <c r="I17" s="211"/>
+      <c r="L17" s="142" t="s">
+        <v>211</v>
+      </c>
+      <c r="M17" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$16,'IV. MA'!$G$16,'IV. MA'!$K$16,'IV. MA'!$O$16,'IV. MA'!$S$16,'IV. MA'!$W$16,'IV. MA'!$AA$16,'IV. MA'!$AE$16,'IV. MA'!$AI$16,'IV. MA'!$AM$16,'IV. MA'!$AQ$16,'IV. MA'!$AU$16,'IV. MA'!$AY$16,'IV. MA'!$BC$16,'IV. MA'!$BG$16,'IV. MA'!$BK$16,'IV. MA'!$BO$16,'IV. MA'!$BS$16),"")</f>
+      </c>
+      <c r="N17" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$16,'IV. MA'!$H$16,'IV. MA'!$L$16,'IV. MA'!$P$16,'IV. MA'!$T$16,'IV. MA'!$X$16,'IV. MA'!$AB$16,'IV. MA'!$AF$16,'IV. MA'!$AJ$16,'IV. MA'!$AN$16,'IV. MA'!$AR$16,'IV. MA'!$AV$16,'IV. MA'!$AZ$16,'IV. MA'!$BD$16,'IV. MA'!$BH$16,'IV. MA'!$BL$16,'IV. MA'!$BP$16,'IV. MA'!$BT$16),"")</f>
+      </c>
     </row>
     <row r="18">
       <c r="C18" s="212" t="str">
@@ -20049,6 +20429,26 @@
         <f>=IF(6&lt;=F11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
       </c>
       <c r="I18" s="216"/>
+      <c r="L18" s="142" t="s">
+        <v>212</v>
+      </c>
+      <c r="M18" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$17,'IV. MA'!$G$17,'IV. MA'!$K$17,'IV. MA'!$O$17,'IV. MA'!$S$17,'IV. MA'!$W$17,'IV. MA'!$AA$17,'IV. MA'!$AE$17,'IV. MA'!$AI$17,'IV. MA'!$AM$17,'IV. MA'!$AQ$17,'IV. MA'!$AU$17,'IV. MA'!$AY$17,'IV. MA'!$BC$17,'IV. MA'!$BG$17,'IV. MA'!$BK$17,'IV. MA'!$BO$17,'IV. MA'!$BS$17),"")</f>
+      </c>
+      <c r="N18" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$17,'IV. MA'!$H$17,'IV. MA'!$L$17,'IV. MA'!$P$17,'IV. MA'!$T$17,'IV. MA'!$X$17,'IV. MA'!$AB$17,'IV. MA'!$AF$17,'IV. MA'!$AJ$17,'IV. MA'!$AN$17,'IV. MA'!$AR$17,'IV. MA'!$AV$17,'IV. MA'!$AZ$17,'IV. MA'!$BD$17,'IV. MA'!$BH$17,'IV. MA'!$BL$17,'IV. MA'!$BP$17,'IV. MA'!$BT$17),"")</f>
+      </c>
+    </row>
+    <row r="19">
+      <c r="L19" s="320" t="s">
+        <v>308</v>
+      </c>
+      <c r="M19" s="242" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$18,'IV. MA'!$G$18,'IV. MA'!$K$18,'IV. MA'!$O$18,'IV. MA'!$S$18,'IV. MA'!$W$18,'IV. MA'!$AA$18,'IV. MA'!$AE$18,'IV. MA'!$AI$18,'IV. MA'!$AM$18,'IV. MA'!$AQ$18,'IV. MA'!$AU$18,'IV. MA'!$AY$18,'IV. MA'!$BC$18,'IV. MA'!$BG$18,'IV. MA'!$BK$18,'IV. MA'!$BO$18,'IV. MA'!$BS$18),"")</f>
+      </c>
+      <c r="N19" s="235" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$18,'IV. MA'!$H$18,'IV. MA'!$L$18,'IV. MA'!$P$18,'IV. MA'!$T$18,'IV. MA'!$X$18,'IV. MA'!$AB$18,'IV. MA'!$AF$18,'IV. MA'!$AJ$18,'IV. MA'!$AN$18,'IV. MA'!$AR$18,'IV. MA'!$AV$18,'IV. MA'!$AZ$18,'IV. MA'!$BD$18,'IV. MA'!$BH$18,'IV. MA'!$BL$18,'IV. MA'!$BP$18,'IV. MA'!$BT$18),"")</f>
+      </c>
     </row>
     <row r="20" ht="22" customHeight="true">
       <c r="B20" s="18" t="s">
@@ -20062,6 +20462,19 @@
       <c r="H20" s="18"/>
       <c r="I20" s="18"/>
       <c r="J20" s="18"/>
+      <c r="L20" s="47"/>
+      <c r="N20" s="48"/>
+    </row>
+    <row r="21">
+      <c r="L21" s="142" t="s">
+        <v>309</v>
+      </c>
+      <c r="M21" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$20,'IV. MA'!$G$20,'IV. MA'!$K$20,'IV. MA'!$O$20,'IV. MA'!$S$20,'IV. MA'!$W$20,'IV. MA'!$AA$20,'IV. MA'!$AE$20,'IV. MA'!$AI$20,'IV. MA'!$AM$20,'IV. MA'!$AQ$20,'IV. MA'!$AU$20,'IV. MA'!$AY$20,'IV. MA'!$BC$20,'IV. MA'!$BG$20,'IV. MA'!$BK$20,'IV. MA'!$BO$20,'IV. MA'!$BS$20),"")</f>
+      </c>
+      <c r="N21" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$20,'IV. MA'!$H$20,'IV. MA'!$L$20,'IV. MA'!$P$20,'IV. MA'!$T$20,'IV. MA'!$X$20,'IV. MA'!$AB$20,'IV. MA'!$AF$20,'IV. MA'!$AJ$20,'IV. MA'!$AN$20,'IV. MA'!$AR$20,'IV. MA'!$AV$20,'IV. MA'!$AZ$20,'IV. MA'!$BD$20,'IV. MA'!$BH$20,'IV. MA'!$BL$20,'IV. MA'!$BP$20,'IV. MA'!$BT$20),"")</f>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="223" t="s">
@@ -20077,6 +20490,15 @@
       <c r="G22" s="231"/>
       <c r="H22" s="231"/>
       <c r="I22" s="232"/>
+      <c r="L22" s="142" t="s">
+        <v>377</v>
+      </c>
+      <c r="M22" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$21,'IV. MA'!$G$21,'IV. MA'!$K$21,'IV. MA'!$O$21,'IV. MA'!$S$21,'IV. MA'!$W$21,'IV. MA'!$AA$21,'IV. MA'!$AE$21,'IV. MA'!$AI$21,'IV. MA'!$AM$21,'IV. MA'!$AQ$21,'IV. MA'!$AU$21,'IV. MA'!$AY$21,'IV. MA'!$BC$21,'IV. MA'!$BG$21,'IV. MA'!$BK$21,'IV. MA'!$BO$21,'IV. MA'!$BS$21),"")</f>
+      </c>
+      <c r="N22" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$21,'IV. MA'!$H$21,'IV. MA'!$L$21,'IV. MA'!$P$21,'IV. MA'!$T$21,'IV. MA'!$X$21,'IV. MA'!$AB$21,'IV. MA'!$AF$21,'IV. MA'!$AJ$21,'IV. MA'!$AN$21,'IV. MA'!$AR$21,'IV. MA'!$AV$21,'IV. MA'!$AZ$21,'IV. MA'!$BD$21,'IV. MA'!$BH$21,'IV. MA'!$BL$21,'IV. MA'!$BP$21,'IV. MA'!$BT$21),"")</f>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="204" t="s">
@@ -20096,6 +20518,15 @@
       <c r="I23" s="234" t="str">
         <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
       </c>
+      <c r="L23" s="142" t="s">
+        <v>378</v>
+      </c>
+      <c r="M23" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$22,'IV. MA'!$G$22,'IV. MA'!$K$22,'IV. MA'!$O$22,'IV. MA'!$S$22,'IV. MA'!$W$22,'IV. MA'!$AA$22,'IV. MA'!$AE$22,'IV. MA'!$AI$22,'IV. MA'!$AM$22,'IV. MA'!$AQ$22,'IV. MA'!$AU$22,'IV. MA'!$AY$22,'IV. MA'!$BC$22,'IV. MA'!$BG$22,'IV. MA'!$BK$22,'IV. MA'!$BO$22,'IV. MA'!$BS$22),"")</f>
+      </c>
+      <c r="N23" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$22,'IV. MA'!$H$22,'IV. MA'!$L$22,'IV. MA'!$P$22,'IV. MA'!$T$22,'IV. MA'!$X$22,'IV. MA'!$AB$22,'IV. MA'!$AF$22,'IV. MA'!$AJ$22,'IV. MA'!$AN$22,'IV. MA'!$AR$22,'IV. MA'!$AV$22,'IV. MA'!$AZ$22,'IV. MA'!$BD$22,'IV. MA'!$BH$22,'IV. MA'!$BL$22,'IV. MA'!$BP$22,'IV. MA'!$BT$22),"")</f>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="204" t="s">
@@ -20112,9 +20543,18 @@
         <v>333</v>
       </c>
       <c r="H24" s="196"/>
-      <c r="I24" s="222" t="str">
-        <f>=I85</f>
+      <c r="I24" s="234" t="str">
+        <f>=I90</f>
         <v>0</v>
+      </c>
+      <c r="L24" s="142" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$B$23,'IV. MA'!$F$23,'IV. MA'!$J$23,'IV. MA'!$N$23,'IV. MA'!$R$23,'IV. MA'!$V$23,'IV. MA'!$Z$23,'IV. MA'!$AD$23,'IV. MA'!$AH$23,'IV. MA'!$AL$23,'IV. MA'!$AP$23,'IV. MA'!$AT$23,'IV. MA'!$AX$23,'IV. MA'!$BB$23,'IV. MA'!$BF$23,'IV. MA'!$BJ$23,'IV. MA'!$BN$23,'IV. MA'!$BR$23),"")</f>
+      </c>
+      <c r="M24" s="115" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$23,'IV. MA'!$G$23,'IV. MA'!$K$23,'IV. MA'!$O$23,'IV. MA'!$S$23,'IV. MA'!$W$23,'IV. MA'!$AA$23,'IV. MA'!$AE$23,'IV. MA'!$AI$23,'IV. MA'!$AM$23,'IV. MA'!$AQ$23,'IV. MA'!$AU$23,'IV. MA'!$AY$23,'IV. MA'!$BC$23,'IV. MA'!$BG$23,'IV. MA'!$BK$23,'IV. MA'!$BO$23,'IV. MA'!$BS$23),"")</f>
+      </c>
+      <c r="N24" s="143" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$23,'IV. MA'!$H$23,'IV. MA'!$L$23,'IV. MA'!$P$23,'IV. MA'!$T$23,'IV. MA'!$X$23,'IV. MA'!$AB$23,'IV. MA'!$AF$23,'IV. MA'!$AJ$23,'IV. MA'!$AN$23,'IV. MA'!$AR$23,'IV. MA'!$AV$23,'IV. MA'!$AZ$23,'IV. MA'!$BD$23,'IV. MA'!$BH$23,'IV. MA'!$BL$23,'IV. MA'!$BP$23,'IV. MA'!$BT$23),"")</f>
       </c>
     </row>
     <row r="25">
@@ -20132,10 +20572,12 @@
         <v>334</v>
       </c>
       <c r="H25" s="196"/>
-      <c r="I25" s="222" t="str">
-        <f>=ROUND(MAX(0,MAX(0,(SUM($G$94:$G$97)-$G$96)+SUMIFS('Daten'!$BH$1:$BH$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;F11,'Daten'!$BD$1:$BD$18,"&gt;=1")-(SUM($H$94:$H$97)-$H$96))-I85),2)</f>
+      <c r="I25" s="234" t="str">
+        <f>=ROUND(MAX(0,MAX(0,(SUM($G$99:$G$102)-$G$101)+SUMIFS('Daten'!$BH$1:$BH$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;F11,'Daten'!$BD$1:$BD$18,"&gt;=1")-(SUM($H$99:$H$102)-$H$101))-I90),2)</f>
         <v>0</v>
       </c>
+      <c r="L25" s="47"/>
+      <c r="N25" s="48"/>
     </row>
     <row r="26">
       <c r="B26" s="227" t="s">
@@ -20152,6 +20594,15 @@
       <c r="H26" s="218"/>
       <c r="I26" s="235" t="str">
         <f>=ROUND(IF($F$23="Abzug",MAX(0,$I$23),0)+IF($F$24="Abzug",MAX(0,$I$24),0)+IF($F$25="Abzug",MAX(0,$I$25),0),2)</f>
+      </c>
+      <c r="L26" s="321" t="s">
+        <v>313</v>
+      </c>
+      <c r="M26" s="322" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$25,'IV. MA'!$G$25,'IV. MA'!$K$25,'IV. MA'!$O$25,'IV. MA'!$S$25,'IV. MA'!$W$25,'IV. MA'!$AA$25,'IV. MA'!$AE$25,'IV. MA'!$AI$25,'IV. MA'!$AM$25,'IV. MA'!$AQ$25,'IV. MA'!$AU$25,'IV. MA'!$AY$25,'IV. MA'!$BC$25,'IV. MA'!$BG$25,'IV. MA'!$BK$25,'IV. MA'!$BO$25,'IV. MA'!$BS$25),"")</f>
+      </c>
+      <c r="N26" s="323" t="str">
+        <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$25,'IV. MA'!$H$25,'IV. MA'!$L$25,'IV. MA'!$P$25,'IV. MA'!$T$25,'IV. MA'!$X$25,'IV. MA'!$AB$25,'IV. MA'!$AF$25,'IV. MA'!$AJ$25,'IV. MA'!$AN$25,'IV. MA'!$AR$25,'IV. MA'!$AV$25,'IV. MA'!$AZ$25,'IV. MA'!$BD$25,'IV. MA'!$BH$25,'IV. MA'!$BL$25,'IV. MA'!$BP$25,'IV. MA'!$BT$25),"")</f>
       </c>
     </row>
     <row r="27">
@@ -20247,1275 +20698,1646 @@
     </row>
     <row r="38">
       <c r="B38" s="223" t="s">
+        <v>158</v>
+      </c>
+      <c r="C38" s="224"/>
+      <c r="D38" s="245" t="s">
         <v>342</v>
       </c>
-      <c r="C38" s="224"/>
-      <c r="D38" s="244" t="str">
-        <f>=F10</f>
+      <c r="E38" s="246" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="204" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C39" s="196"/>
-      <c r="D39" s="245" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;F11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
-      </c>
+      <c r="D39" s="239" t="str">
+        <f>=F10</f>
+      </c>
+      <c r="E39" s="247"/>
     </row>
     <row r="40">
       <c r="B40" s="204" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C40" s="196"/>
-      <c r="D40" s="205" t="s">
-        <v>189</v>
+      <c r="D40" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;F11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="E40" s="226" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;F11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="204" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C41" s="196"/>
-      <c r="D41" s="245" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(MATCH($D$40,{"Jahr 1";"Jahr 2";"Jahr 3"},0),SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])),2),0)</f>
-      </c>
+      <c r="D41" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="E41" s="205"/>
     </row>
     <row r="42">
       <c r="B42" s="204" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C42" s="196"/>
-      <c r="D42" s="246">
-        <v>8</v>
+      <c r="D42" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(MATCH($D$41,{"Jahr 1";"Jahr 2";"Jahr 3"},0),SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])),2),0)</f>
+      </c>
+      <c r="E42" s="226" t="str">
+        <f>=IFERROR(ROUND($D$42/IFERROR(INDIRECT("MA_Kurs_"&amp;F10),0),2),0)</f>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="204" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C43" s="196"/>
-      <c r="D43" s="247">
-        <v>12</v>
-      </c>
+      <c r="D43" s="241">
+        <v>8</v>
+      </c>
+      <c r="E43" s="248"/>
     </row>
     <row r="44">
       <c r="B44" s="204" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C44" s="196"/>
-      <c r="D44" s="248">
+      <c r="D44" s="241">
+        <v>12</v>
+      </c>
+      <c r="E44" s="249"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="204" t="s">
+        <v>350</v>
+      </c>
+      <c r="C45" s="196"/>
+      <c r="D45" s="241">
         <v>6</v>
       </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="249" t="s">
-        <v>349</v>
-      </c>
-      <c r="C45" s="218"/>
-      <c r="D45" s="250" t="str">
-        <f>=IFERROR(ROUND($D$41*$D$42/$D$43,2),0)</f>
-      </c>
+      <c r="E45" s="250"/>
     </row>
     <row r="46">
-      <c r="B46" s="249" t="s">
-        <v>350</v>
+      <c r="B46" s="251" t="s">
+        <v>351</v>
       </c>
       <c r="C46" s="218"/>
-      <c r="D46" s="251" t="str">
-        <f>=IF($D$39&lt;=$D$45,"OK","ÜBERSCHRITTEN")</f>
+      <c r="D46" s="242" t="str">
+        <f>=IFERROR(ROUND($D$42*$D$43/$D$44,2),0)</f>
+      </c>
+      <c r="E46" s="235" t="str">
+        <f>=IFERROR(ROUND($E$42*$D$43/$D$44,2),0)</f>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="204" t="s">
-        <v>351</v>
-      </c>
-      <c r="C47" s="196"/>
-      <c r="D47" s="245" t="str">
-        <f>=ROUND(MAX(0,$D$39-$D$45),2)</f>
+      <c r="B47" s="251" t="s">
+        <v>352</v>
+      </c>
+      <c r="C47" s="218"/>
+      <c r="D47" s="243" t="str">
+        <f>=IF($D$40&lt;=$D$46,"OK","ÜBERSCHRITTEN")</f>
+      </c>
+      <c r="E47" s="252" t="str">
+        <f>=IF($E$40&lt;=$E$46,"OK","ÜBERSCHRITTEN")</f>
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="252" t="s">
-        <v>352</v>
-      </c>
-      <c r="C48" s="253"/>
-      <c r="D48" s="254" t="str">
-        <f>=IFERROR($D$39/$D$45,0)</f>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="true">
-      <c r="B50" s="18" t="s">
+      <c r="B48" s="204" t="s">
         <v>353</v>
       </c>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="18"/>
-      <c r="F50" s="18"/>
-      <c r="G50" s="18"/>
-      <c r="H50" s="18"/>
-      <c r="I50" s="18"/>
-      <c r="J50" s="18"/>
-    </row>
-    <row r="52" ht="28" customHeight="true">
-      <c r="B52" s="261" t="s">
+      <c r="C48" s="196"/>
+      <c r="D48" s="240" t="str">
+        <f>=ROUND(MAX(0,$D$40-$D$46),2)</f>
+      </c>
+      <c r="E48" s="226" t="str">
+        <f>=ROUND(MAX(0,$E$40-$E$46),2)</f>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="253" t="s">
         <v>354</v>
       </c>
-      <c r="C52" s="262" t="s">
+      <c r="C49" s="254"/>
+      <c r="D49" s="255" t="str">
+        <f>=IFERROR($D$40/$D$46,0)</f>
+      </c>
+      <c r="E49" s="256" t="str">
+        <f>=IFERROR($E$40/$E$46,0)</f>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="true">
+      <c r="B51" s="18" t="s">
         <v>355</v>
       </c>
-      <c r="D52" s="262" t="s">
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="18"/>
+      <c r="J51" s="18"/>
+    </row>
+    <row r="53" ht="28" customHeight="true">
+      <c r="B53" s="263" t="s">
         <v>356</v>
       </c>
-      <c r="E52" s="262" t="s">
+      <c r="C53" s="264" t="s">
         <v>357</v>
       </c>
-      <c r="F52" s="262" t="s">
+      <c r="D53" s="264" t="s">
         <v>358</v>
       </c>
-      <c r="G52" s="262" t="s">
+      <c r="E53" s="264" t="s">
         <v>359</v>
       </c>
-      <c r="H52" s="262" t="s">
+      <c r="F53" s="264" t="s">
         <v>360</v>
       </c>
-      <c r="I52" s="262" t="s">
+      <c r="G53" s="264" t="s">
         <v>361</v>
       </c>
-      <c r="J52" s="263" t="s">
+      <c r="H53" s="264" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="264" t="s">
+      <c r="I53" s="264" t="s">
+        <v>363</v>
+      </c>
+      <c r="J53" s="265" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="266" t="s">
         <v>194</v>
-      </c>
-      <c r="C53" s="24">
-        <v>0</v>
-      </c>
-      <c r="D53" s="239" t="str">
-        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
-      </c>
-      <c r="E53" s="200" t="str">
-        <f>=ROUND(IFERROR($C$53-$D$53,0),2)</f>
-      </c>
-      <c r="F53" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$53/$D$53)-1,0),4)</f>
-      </c>
-      <c r="G53" s="25">
-        <v>0</v>
-      </c>
-      <c r="H53" s="217" t="str">
-        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
-      </c>
-      <c r="I53" s="181" t="str">
-        <f>=ROUND(IFERROR($G$53-$H$53,0),2)</f>
-      </c>
-      <c r="J53" s="265" t="str">
-        <f>=ROUND(IFERROR(($G$53/$H$53)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="264" t="s">
-        <v>277</v>
       </c>
       <c r="C54" s="24">
         <v>0</v>
       </c>
-      <c r="D54" s="239" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
+      <c r="D54" s="240" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
       </c>
       <c r="E54" s="200" t="str">
         <f>=ROUND(IFERROR($C$54-$D$54,0),2)</f>
       </c>
-      <c r="F54" s="256" t="str">
+      <c r="F54" s="258" t="str">
         <f>=ROUND(IFERROR(($C$54/$D$54)-1,0),4)</f>
       </c>
       <c r="G54" s="25">
         <v>0</v>
       </c>
       <c r="H54" s="217" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
       </c>
       <c r="I54" s="181" t="str">
         <f>=ROUND(IFERROR($G$54-$H$54,0),2)</f>
       </c>
-      <c r="J54" s="266" t="str">
+      <c r="J54" s="267" t="str">
         <f>=ROUND(IFERROR(($G$54/$H$54)-1,0),4)</f>
       </c>
     </row>
     <row r="55">
-      <c r="B55" s="264" t="s">
-        <v>199</v>
+      <c r="B55" s="266" t="s">
+        <v>277</v>
       </c>
       <c r="C55" s="24">
         <v>0</v>
       </c>
-      <c r="D55" s="239" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
+      <c r="D55" s="240" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
       </c>
       <c r="E55" s="200" t="str">
         <f>=ROUND(IFERROR($C$55-$D$55,0),2)</f>
       </c>
-      <c r="F55" s="256" t="str">
+      <c r="F55" s="258" t="str">
         <f>=ROUND(IFERROR(($C$55/$D$55)-1,0),4)</f>
       </c>
       <c r="G55" s="25">
         <v>0</v>
       </c>
       <c r="H55" s="217" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
       </c>
       <c r="I55" s="181" t="str">
         <f>=ROUND(IFERROR($G$55-$H$55,0),2)</f>
       </c>
-      <c r="J55" s="267" t="str">
+      <c r="J55" s="268" t="str">
         <f>=ROUND(IFERROR(($G$55/$H$55)-1,0),4)</f>
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="264" t="s">
-        <v>278</v>
+      <c r="B56" s="266" t="s">
+        <v>199</v>
       </c>
       <c r="C56" s="24">
         <v>0</v>
       </c>
-      <c r="D56" s="239" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
+      <c r="D56" s="240" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
       </c>
       <c r="E56" s="200" t="str">
         <f>=ROUND(IFERROR($C$56-$D$56,0),2)</f>
       </c>
-      <c r="F56" s="256" t="str">
+      <c r="F56" s="258" t="str">
         <f>=ROUND(IFERROR(($C$56/$D$56)-1,0),4)</f>
       </c>
       <c r="G56" s="25">
         <v>0</v>
       </c>
       <c r="H56" s="217" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="I56" s="181" t="str">
         <f>=ROUND(IFERROR($G$56-$H$56,0),2)</f>
       </c>
-      <c r="J56" s="268" t="str">
+      <c r="J56" s="269" t="str">
         <f>=ROUND(IFERROR(($G$56/$H$56)-1,0),4)</f>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="true">
-      <c r="B57" s="269" t="s">
+    <row r="57">
+      <c r="B57" s="266" t="s">
+        <v>278</v>
+      </c>
+      <c r="C57" s="24">
+        <v>0</v>
+      </c>
+      <c r="D57" s="240" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
+      </c>
+      <c r="E57" s="200" t="str">
+        <f>=ROUND(IFERROR($C$57-$D$57,0),2)</f>
+      </c>
+      <c r="F57" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$57/$D$57)-1,0),4)</f>
+      </c>
+      <c r="G57" s="25">
+        <v>0</v>
+      </c>
+      <c r="H57" s="217" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
+      </c>
+      <c r="I57" s="181" t="str">
+        <f>=ROUND(IFERROR($G$57-$H$57,0),2)</f>
+      </c>
+      <c r="J57" s="270" t="str">
+        <f>=ROUND(IFERROR(($G$57/$H$57)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="true">
+      <c r="B58" s="271" t="s">
         <v>266</v>
       </c>
-      <c r="C57" s="270" t="str">
-        <f>=ROUND(SUM($C$53:$C$56),2)</f>
-      </c>
-      <c r="D57" s="270" t="str">
-        <f>=ROUND(SUM($D$53:$D$56),2)</f>
-      </c>
-      <c r="E57" s="270" t="str">
-        <f>=ROUND(SUM($E$53:$E$56),2)</f>
-      </c>
-      <c r="F57" s="271" t="str">
-        <f>=ROUND(IFERROR(($C$57/$D$57)-1,0),4)</f>
-      </c>
-      <c r="G57" s="272" t="str">
-        <f>=ROUND(SUM($G$53:$G$56),2)</f>
-      </c>
-      <c r="H57" s="272" t="str">
-        <f>=ROUND(SUM($H$53:$H$56),2)</f>
-      </c>
-      <c r="I57" s="272" t="str">
-        <f>=ROUND(SUM($I$53:$I$56),2)</f>
-      </c>
-      <c r="J57" s="273" t="str">
-        <f>=ROUND(IFERROR(($G$57/$H$57)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="59" ht="22" customHeight="true">
-      <c r="B59" s="18" t="s">
+      <c r="C58" s="272" t="str">
+        <f>=ROUND(SUM($C$54:$C$57),2)</f>
+      </c>
+      <c r="D58" s="272" t="str">
+        <f>=ROUND(SUM($D$54:$D$57),2)</f>
+      </c>
+      <c r="E58" s="272" t="str">
+        <f>=ROUND(SUM($E$54:$E$57),2)</f>
+      </c>
+      <c r="F58" s="273" t="str">
+        <f>=ROUND(IFERROR(($C$58/$D$58)-1,0),4)</f>
+      </c>
+      <c r="G58" s="274" t="str">
+        <f>=ROUND(SUM($G$54:$G$57),2)</f>
+      </c>
+      <c r="H58" s="274" t="str">
+        <f>=ROUND(SUM($H$54:$H$57),2)</f>
+      </c>
+      <c r="I58" s="274" t="str">
+        <f>=ROUND(SUM($I$54:$I$57),2)</f>
+      </c>
+      <c r="J58" s="275" t="str">
+        <f>=ROUND(IFERROR(($G$58/$H$58)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="true">
+      <c r="B60" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+      <c r="I60" s="18"/>
+      <c r="J60" s="18"/>
+    </row>
+    <row r="62" ht="28" customHeight="true">
+      <c r="B62" s="263" t="s">
+        <v>356</v>
+      </c>
+      <c r="C62" s="264" t="s">
+        <v>357</v>
+      </c>
+      <c r="D62" s="264" t="s">
+        <v>358</v>
+      </c>
+      <c r="E62" s="264" t="s">
+        <v>359</v>
+      </c>
+      <c r="F62" s="264" t="s">
+        <v>360</v>
+      </c>
+      <c r="G62" s="264" t="s">
+        <v>361</v>
+      </c>
+      <c r="H62" s="264" t="s">
+        <v>362</v>
+      </c>
+      <c r="I62" s="264" t="s">
         <v>363</v>
       </c>
-      <c r="C59" s="18"/>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="18"/>
-      <c r="G59" s="18"/>
-      <c r="H59" s="18"/>
-      <c r="I59" s="18"/>
-      <c r="J59" s="18"/>
-    </row>
-    <row r="61" ht="28" customHeight="true">
-      <c r="B61" s="261" t="s">
-        <v>354</v>
-      </c>
-      <c r="C61" s="262" t="s">
-        <v>355</v>
-      </c>
-      <c r="D61" s="262" t="s">
-        <v>356</v>
-      </c>
-      <c r="E61" s="262" t="s">
-        <v>357</v>
-      </c>
-      <c r="F61" s="262" t="s">
-        <v>358</v>
-      </c>
-      <c r="G61" s="262" t="s">
-        <v>359</v>
-      </c>
-      <c r="H61" s="262" t="s">
-        <v>360</v>
-      </c>
-      <c r="I61" s="262" t="s">
-        <v>361</v>
-      </c>
-      <c r="J61" s="263" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="264" t="s">
+      <c r="J62" s="265" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="266" t="s">
         <v>205</v>
       </c>
-      <c r="C62" s="239" t="str">
+      <c r="C63" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D62" s="239" t="str">
+      <c r="D63" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
-      </c>
-      <c r="E62" s="200" t="str">
-        <f>=ROUND(IFERROR($C$62-$D$62,0),2)</f>
-      </c>
-      <c r="F62" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$62/$D$62)-1,0),4)</f>
-      </c>
-      <c r="G62" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="H62" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
-      </c>
-      <c r="I62" s="181" t="str">
-        <f>=ROUND(IFERROR($G$62-$H$62,0),2)</f>
-      </c>
-      <c r="J62" s="274" t="str">
-        <f>=ROUND(IFERROR(($G$62/$H$62)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="264" t="s">
-        <v>206</v>
-      </c>
-      <c r="C63" s="239" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D63" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
       </c>
       <c r="E63" s="200" t="str">
         <f>=ROUND(IFERROR($C$63-$D$63,0),2)</f>
       </c>
-      <c r="F63" s="256" t="str">
+      <c r="F63" s="258" t="str">
         <f>=ROUND(IFERROR(($C$63/$D$63)-1,0),4)</f>
       </c>
       <c r="G63" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
       <c r="H63" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
       </c>
       <c r="I63" s="181" t="str">
         <f>=ROUND(IFERROR($G$63-$H$63,0),2)</f>
       </c>
-      <c r="J63" s="275" t="str">
+      <c r="J63" s="276" t="str">
         <f>=ROUND(IFERROR(($G$63/$H$63)-1,0),4)</f>
       </c>
     </row>
     <row r="64">
-      <c r="B64" s="264" t="s">
-        <v>207</v>
-      </c>
-      <c r="C64" s="239" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D64" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
+      <c r="B64" s="266" t="s">
+        <v>206</v>
+      </c>
+      <c r="C64" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D64" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
       </c>
       <c r="E64" s="200" t="str">
         <f>=ROUND(IFERROR($C$64-$D$64,0),2)</f>
       </c>
-      <c r="F64" s="256" t="str">
+      <c r="F64" s="258" t="str">
         <f>=ROUND(IFERROR(($C$64/$D$64)-1,0),4)</f>
       </c>
       <c r="G64" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
       <c r="H64" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
       </c>
       <c r="I64" s="181" t="str">
         <f>=ROUND(IFERROR($G$64-$H$64,0),2)</f>
       </c>
-      <c r="J64" s="276" t="str">
+      <c r="J64" s="277" t="str">
         <f>=ROUND(IFERROR(($G$64/$H$64)-1,0),4)</f>
       </c>
     </row>
     <row r="65">
-      <c r="B65" s="264" t="s">
-        <v>208</v>
-      </c>
-      <c r="C65" s="239" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D65" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
+      <c r="B65" s="266" t="s">
+        <v>207</v>
+      </c>
+      <c r="C65" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D65" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
       </c>
       <c r="E65" s="200" t="str">
         <f>=ROUND(IFERROR($C$65-$D$65,0),2)</f>
       </c>
-      <c r="F65" s="256" t="str">
+      <c r="F65" s="258" t="str">
         <f>=ROUND(IFERROR(($C$65/$D$65)-1,0),4)</f>
       </c>
       <c r="G65" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
       <c r="H65" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
       </c>
       <c r="I65" s="181" t="str">
         <f>=ROUND(IFERROR($G$65-$H$65,0),2)</f>
       </c>
-      <c r="J65" s="277" t="str">
+      <c r="J65" s="278" t="str">
         <f>=ROUND(IFERROR(($G$65/$H$65)-1,0),4)</f>
       </c>
     </row>
     <row r="66">
-      <c r="B66" s="264" t="s">
-        <v>209</v>
-      </c>
-      <c r="C66" s="239" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D66" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
+      <c r="B66" s="266" t="s">
+        <v>208</v>
+      </c>
+      <c r="C66" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D66" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
       </c>
       <c r="E66" s="200" t="str">
         <f>=ROUND(IFERROR($C$66-$D$66,0),2)</f>
       </c>
-      <c r="F66" s="256" t="str">
+      <c r="F66" s="258" t="str">
         <f>=ROUND(IFERROR(($C$66/$D$66)-1,0),4)</f>
       </c>
       <c r="G66" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
       <c r="H66" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
       </c>
       <c r="I66" s="181" t="str">
         <f>=ROUND(IFERROR($G$66-$H$66,0),2)</f>
       </c>
-      <c r="J66" s="278" t="str">
+      <c r="J66" s="279" t="str">
         <f>=ROUND(IFERROR(($G$66/$H$66)-1,0),4)</f>
       </c>
     </row>
     <row r="67">
-      <c r="B67" s="264" t="s">
-        <v>210</v>
-      </c>
-      <c r="C67" s="239" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D67" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
+      <c r="B67" s="266" t="s">
+        <v>209</v>
+      </c>
+      <c r="C67" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D67" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
       </c>
       <c r="E67" s="200" t="str">
         <f>=ROUND(IFERROR($C$67-$D$67,0),2)</f>
       </c>
-      <c r="F67" s="256" t="str">
+      <c r="F67" s="258" t="str">
         <f>=ROUND(IFERROR(($C$67/$D$67)-1,0),4)</f>
       </c>
       <c r="G67" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
       <c r="H67" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
       </c>
       <c r="I67" s="181" t="str">
         <f>=ROUND(IFERROR($G$67-$H$67,0),2)</f>
       </c>
-      <c r="J67" s="279" t="str">
+      <c r="J67" s="280" t="str">
         <f>=ROUND(IFERROR(($G$67/$H$67)-1,0),4)</f>
       </c>
     </row>
     <row r="68">
-      <c r="B68" s="264" t="s">
-        <v>211</v>
-      </c>
-      <c r="C68" s="239" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D68" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
+      <c r="B68" s="266" t="s">
+        <v>210</v>
+      </c>
+      <c r="C68" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D68" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
       </c>
       <c r="E68" s="200" t="str">
         <f>=ROUND(IFERROR($C$68-$D$68,0),2)</f>
       </c>
-      <c r="F68" s="256" t="str">
+      <c r="F68" s="258" t="str">
         <f>=ROUND(IFERROR(($C$68/$D$68)-1,0),4)</f>
       </c>
       <c r="G68" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
       <c r="H68" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
       </c>
       <c r="I68" s="181" t="str">
         <f>=ROUND(IFERROR($G$68-$H$68,0),2)</f>
       </c>
-      <c r="J68" s="280" t="str">
+      <c r="J68" s="281" t="str">
         <f>=ROUND(IFERROR(($G$68/$H$68)-1,0),4)</f>
       </c>
     </row>
     <row r="69">
-      <c r="B69" s="264" t="s">
-        <v>212</v>
-      </c>
-      <c r="C69" s="239" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
-      </c>
-      <c r="D69" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
+      <c r="B69" s="266" t="s">
+        <v>211</v>
+      </c>
+      <c r="C69" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D69" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
       </c>
       <c r="E69" s="200" t="str">
         <f>=ROUND(IFERROR($C$69-$D$69,0),2)</f>
       </c>
-      <c r="F69" s="256" t="str">
+      <c r="F69" s="258" t="str">
         <f>=ROUND(IFERROR(($C$69/$D$69)-1,0),4)</f>
       </c>
       <c r="G69" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
       </c>
       <c r="H69" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
       </c>
       <c r="I69" s="181" t="str">
         <f>=ROUND(IFERROR($G$69-$H$69,0),2)</f>
       </c>
-      <c r="J69" s="281" t="str">
+      <c r="J69" s="282" t="str">
         <f>=ROUND(IFERROR(($G$69/$H$69)-1,0),4)</f>
       </c>
     </row>
-    <row r="70" ht="20" customHeight="true">
-      <c r="B70" s="269" t="s">
-        <v>266</v>
-      </c>
-      <c r="C70" s="270" t="str">
-        <f>=ROUND(SUM($C$62:$C$69),2)</f>
-      </c>
-      <c r="D70" s="270" t="str">
-        <f>=ROUND(SUM($D$62:$D$69),2)</f>
-      </c>
-      <c r="E70" s="270" t="str">
-        <f>=ROUND(SUM($E$62:$E$69),2)</f>
-      </c>
-      <c r="F70" s="282" t="str">
+    <row r="70">
+      <c r="B70" s="266" t="s">
+        <v>212</v>
+      </c>
+      <c r="C70" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="D70" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
+      </c>
+      <c r="E70" s="200" t="str">
+        <f>=ROUND(IFERROR($C$70-$D$70,0),2)</f>
+      </c>
+      <c r="F70" s="258" t="str">
         <f>=ROUND(IFERROR(($C$70/$D$70)-1,0),4)</f>
       </c>
-      <c r="G70" s="272" t="str">
-        <f>=ROUND(SUM($G$62:$G$69),2)</f>
-      </c>
-      <c r="H70" s="272" t="str">
-        <f>=ROUND(SUM($H$62:$H$69),2)</f>
-      </c>
-      <c r="I70" s="272" t="str">
-        <f>=ROUND(SUM($I$62:$I$69),2)</f>
+      <c r="G70" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+      </c>
+      <c r="H70" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="I70" s="181" t="str">
+        <f>=ROUND(IFERROR($G$70-$H$70,0),2)</f>
       </c>
       <c r="J70" s="283" t="str">
         <f>=ROUND(IFERROR(($G$70/$H$70)-1,0),4)</f>
       </c>
     </row>
-    <row r="72" ht="26" customHeight="true">
-      <c r="B72" s="193" t="s">
+    <row r="71" ht="20" customHeight="true">
+      <c r="B71" s="271" t="s">
+        <v>266</v>
+      </c>
+      <c r="C71" s="272" t="str">
+        <f>=ROUND(SUM($C$63:$C$70),2)</f>
+      </c>
+      <c r="D71" s="272" t="str">
+        <f>=ROUND(SUM($D$63:$D$70),2)</f>
+      </c>
+      <c r="E71" s="272" t="str">
+        <f>=ROUND(SUM($E$63:$E$70),2)</f>
+      </c>
+      <c r="F71" s="284" t="str">
+        <f>=ROUND(IFERROR(($C$71/$D$71)-1,0),4)</f>
+      </c>
+      <c r="G71" s="274" t="str">
+        <f>=ROUND(SUM($G$63:$G$70),2)</f>
+      </c>
+      <c r="H71" s="274" t="str">
+        <f>=ROUND(SUM($H$63:$H$70),2)</f>
+      </c>
+      <c r="I71" s="274" t="str">
+        <f>=ROUND(SUM($I$63:$I$70),2)</f>
+      </c>
+      <c r="J71" s="285" t="str">
+        <f>=ROUND(IFERROR(($G$71/$H$71)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="true">
+      <c r="B77" s="193" t="s">
+        <v>366</v>
+      </c>
+      <c r="C77" s="193"/>
+      <c r="D77" s="193"/>
+      <c r="E77" s="193"/>
+      <c r="F77" s="193"/>
+      <c r="G77" s="193"/>
+      <c r="H77" s="193"/>
+      <c r="I77" s="193"/>
+      <c r="J77" s="193"/>
+      <c r="L77" s="201" t="s">
+        <v>379</v>
+      </c>
+      <c r="M77" s="202"/>
+      <c r="N77" s="202"/>
+      <c r="O77" s="202"/>
+      <c r="P77" s="203"/>
+    </row>
+    <row r="78">
+      <c r="B78" s="194" t="s">
+        <v>367</v>
+      </c>
+      <c r="C78" s="194"/>
+      <c r="D78" s="194"/>
+      <c r="E78" s="194"/>
+      <c r="F78" s="194"/>
+      <c r="G78" s="194"/>
+      <c r="H78" s="194"/>
+      <c r="I78" s="194"/>
+      <c r="J78" s="194"/>
+      <c r="L78" s="314" t="s">
+        <v>267</v>
+      </c>
+      <c r="M78" s="324" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$5,'III. Finanzberichte'!$J$5,'III. Finanzberichte'!$Q$5,'III. Finanzberichte'!$X$5,'III. Finanzberichte'!$AE$5,'III. Finanzberichte'!$AL$5,'III. Finanzberichte'!$AS$5,'III. Finanzberichte'!$AZ$5,'III. Finanzberichte'!$BG$5,'III. Finanzberichte'!$BN$5,'III. Finanzberichte'!$BU$5,'III. Finanzberichte'!$CB$5,'III. Finanzberichte'!$CI$5,'III. Finanzberichte'!$CP$5,'III. Finanzberichte'!$CW$5,'III. Finanzberichte'!$DD$5,'III. Finanzberichte'!$DK$5,'III. Finanzberichte'!$DR$5),"")</f>
+      </c>
+      <c r="N78" s="324"/>
+      <c r="O78" s="324"/>
+      <c r="P78" s="333"/>
+    </row>
+    <row r="79">
+      <c r="L79" s="314" t="s">
+        <v>268</v>
+      </c>
+      <c r="M79" s="324" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$6,'III. Finanzberichte'!$J$6,'III. Finanzberichte'!$Q$6,'III. Finanzberichte'!$X$6,'III. Finanzberichte'!$AE$6,'III. Finanzberichte'!$AL$6,'III. Finanzberichte'!$AS$6,'III. Finanzberichte'!$AZ$6,'III. Finanzberichte'!$BG$6,'III. Finanzberichte'!$BN$6,'III. Finanzberichte'!$BU$6,'III. Finanzberichte'!$CB$6,'III. Finanzberichte'!$CI$6,'III. Finanzberichte'!$CP$6,'III. Finanzberichte'!$CW$6,'III. Finanzberichte'!$DD$6,'III. Finanzberichte'!$DK$6,'III. Finanzberichte'!$DR$6),"")</f>
+      </c>
+      <c r="N79" s="324"/>
+      <c r="O79" s="324"/>
+      <c r="P79" s="333"/>
+    </row>
+    <row r="80" ht="22" customHeight="true">
+      <c r="C80" s="201" t="s">
+        <v>368</v>
+      </c>
+      <c r="D80" s="202"/>
+      <c r="E80" s="202"/>
+      <c r="F80" s="202"/>
+      <c r="G80" s="202"/>
+      <c r="H80" s="202"/>
+      <c r="I80" s="203"/>
+      <c r="L80" s="314" t="s">
+        <v>269</v>
+      </c>
+      <c r="M80" s="325" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$7,'III. Finanzberichte'!$J$7,'III. Finanzberichte'!$Q$7,'III. Finanzberichte'!$X$7,'III. Finanzberichte'!$AE$7,'III. Finanzberichte'!$AL$7,'III. Finanzberichte'!$AS$7,'III. Finanzberichte'!$AZ$7,'III. Finanzberichte'!$BG$7,'III. Finanzberichte'!$BN$7,'III. Finanzberichte'!$BU$7,'III. Finanzberichte'!$CB$7,'III. Finanzberichte'!$CI$7,'III. Finanzberichte'!$CP$7,'III. Finanzberichte'!$CW$7,'III. Finanzberichte'!$DD$7,'III. Finanzberichte'!$DK$7,'III. Finanzberichte'!$DR$7),"")</f>
+      </c>
+      <c r="N80" s="325"/>
+      <c r="O80" s="325"/>
+      <c r="P80" s="334"/>
+    </row>
+    <row r="81">
+      <c r="C81" s="204" t="s">
+        <v>320</v>
+      </c>
+      <c r="D81" s="196"/>
+      <c r="E81" s="196"/>
+      <c r="F81" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="G81" s="33"/>
+      <c r="H81" s="33"/>
+      <c r="I81" s="205"/>
+      <c r="L81" s="47"/>
+      <c r="P81" s="48"/>
+    </row>
+    <row r="82">
+      <c r="C82" s="204" t="s">
+        <v>369</v>
+      </c>
+      <c r="D82" s="196"/>
+      <c r="E82" s="196"/>
+      <c r="F82" s="197" t="str">
+        <f>=IF(LEFT(F81,8)="Periode ",IFERROR(VALUE(TRIM(MID(F81,9,5))),0),0)</f>
+      </c>
+      <c r="G82" s="197"/>
+      <c r="H82" s="197"/>
+      <c r="I82" s="286"/>
+      <c r="L82" s="335" t="s">
+        <v>270</v>
+      </c>
+      <c r="M82" s="326"/>
+      <c r="N82" s="326"/>
+      <c r="O82" s="326"/>
+      <c r="P82" s="336"/>
+    </row>
+    <row r="83" ht="26" customHeight="true">
+      <c r="C83" s="204" t="s">
+        <v>370</v>
+      </c>
+      <c r="D83" s="196"/>
+      <c r="E83" s="196"/>
+      <c r="F83" s="240" t="str">
+        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoLC_"&amp;F82),2),0)</f>
+      </c>
+      <c r="G83" s="240"/>
+      <c r="H83" s="240"/>
+      <c r="I83" s="287"/>
+      <c r="L83" s="337" t="s">
+        <v>271</v>
+      </c>
+      <c r="M83" s="327" t="s">
+        <v>272</v>
+      </c>
+      <c r="N83" s="327" t="s">
+        <v>273</v>
+      </c>
+      <c r="O83" s="327" t="s">
+        <v>274</v>
+      </c>
+      <c r="P83" s="338" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="C84" s="253" t="s">
+        <v>171</v>
+      </c>
+      <c r="D84" s="254"/>
+      <c r="E84" s="254"/>
+      <c r="F84" s="288" t="str">
+        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoEUR_"&amp;F82),2),0)</f>
+      </c>
+      <c r="G84" s="288"/>
+      <c r="H84" s="288"/>
+      <c r="I84" s="289"/>
+      <c r="L84" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$11,'III. Finanzberichte'!$I$11,'III. Finanzberichte'!$P$11,'III. Finanzberichte'!$W$11,'III. Finanzberichte'!$AD$11,'III. Finanzberichte'!$AK$11,'III. Finanzberichte'!$AR$11,'III. Finanzberichte'!$AY$11,'III. Finanzberichte'!$BF$11,'III. Finanzberichte'!$BM$11,'III. Finanzberichte'!$BT$11,'III. Finanzberichte'!$CA$11,'III. Finanzberichte'!$CH$11,'III. Finanzberichte'!$CO$11,'III. Finanzberichte'!$CV$11,'III. Finanzberichte'!$DC$11,'III. Finanzberichte'!$DJ$11,'III. Finanzberichte'!$DQ$11),"")</f>
+      </c>
+      <c r="M84" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$11,'III. Finanzberichte'!$J$11,'III. Finanzberichte'!$Q$11,'III. Finanzberichte'!$X$11,'III. Finanzberichte'!$AE$11,'III. Finanzberichte'!$AL$11,'III. Finanzberichte'!$AS$11,'III. Finanzberichte'!$AZ$11,'III. Finanzberichte'!$BG$11,'III. Finanzberichte'!$BN$11,'III. Finanzberichte'!$BU$11,'III. Finanzberichte'!$CB$11,'III. Finanzberichte'!$CI$11,'III. Finanzberichte'!$CP$11,'III. Finanzberichte'!$CW$11,'III. Finanzberichte'!$DD$11,'III. Finanzberichte'!$DK$11,'III. Finanzberichte'!$DR$11),"")</f>
+      </c>
+      <c r="N84" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$11,'III. Finanzberichte'!$K$11,'III. Finanzberichte'!$R$11,'III. Finanzberichte'!$Y$11,'III. Finanzberichte'!$AF$11,'III. Finanzberichte'!$AM$11,'III. Finanzberichte'!$AT$11,'III. Finanzberichte'!$BA$11,'III. Finanzberichte'!$BH$11,'III. Finanzberichte'!$BO$11,'III. Finanzberichte'!$BV$11,'III. Finanzberichte'!$CC$11,'III. Finanzberichte'!$CJ$11,'III. Finanzberichte'!$CQ$11,'III. Finanzberichte'!$CX$11,'III. Finanzberichte'!$DE$11,'III. Finanzberichte'!$DL$11,'III. Finanzberichte'!$DS$11),"")</f>
+      </c>
+      <c r="O84" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$11,'III. Finanzberichte'!$L$11,'III. Finanzberichte'!$S$11,'III. Finanzberichte'!$Z$11,'III. Finanzberichte'!$AG$11,'III. Finanzberichte'!$AN$11,'III. Finanzberichte'!$AU$11,'III. Finanzberichte'!$BB$11,'III. Finanzberichte'!$BI$11,'III. Finanzberichte'!$BP$11,'III. Finanzberichte'!$BW$11,'III. Finanzberichte'!$CD$11,'III. Finanzberichte'!$CK$11,'III. Finanzberichte'!$CR$11,'III. Finanzberichte'!$CY$11,'III. Finanzberichte'!$DF$11,'III. Finanzberichte'!$DM$11,'III. Finanzberichte'!$DT$11),"")</f>
+      </c>
+      <c r="P84" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$11,'III. Finanzberichte'!$M$11,'III. Finanzberichte'!$T$11,'III. Finanzberichte'!$AA$11,'III. Finanzberichte'!$AH$11,'III. Finanzberichte'!$AO$11,'III. Finanzberichte'!$AV$11,'III. Finanzberichte'!$BC$11,'III. Finanzberichte'!$BJ$11,'III. Finanzberichte'!$BQ$11,'III. Finanzberichte'!$BX$11,'III. Finanzberichte'!$CE$11,'III. Finanzberichte'!$CL$11,'III. Finanzberichte'!$CS$11,'III. Finanzberichte'!$CZ$11,'III. Finanzberichte'!$DG$11,'III. Finanzberichte'!$DN$11,'III. Finanzberichte'!$DU$11),"")</f>
+      </c>
+    </row>
+    <row r="85">
+      <c r="L85" s="142" t="s">
+        <v>194</v>
+      </c>
+      <c r="M85" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$12,'III. Finanzberichte'!$J$12,'III. Finanzberichte'!$Q$12,'III. Finanzberichte'!$X$12,'III. Finanzberichte'!$AE$12,'III. Finanzberichte'!$AL$12,'III. Finanzberichte'!$AS$12,'III. Finanzberichte'!$AZ$12,'III. Finanzberichte'!$BG$12,'III. Finanzberichte'!$BN$12,'III. Finanzberichte'!$BU$12,'III. Finanzberichte'!$CB$12,'III. Finanzberichte'!$CI$12,'III. Finanzberichte'!$CP$12,'III. Finanzberichte'!$CW$12,'III. Finanzberichte'!$DD$12,'III. Finanzberichte'!$DK$12,'III. Finanzberichte'!$DR$12),"")</f>
+      </c>
+      <c r="N85" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$12,'III. Finanzberichte'!$K$12,'III. Finanzberichte'!$R$12,'III. Finanzberichte'!$Y$12,'III. Finanzberichte'!$AF$12,'III. Finanzberichte'!$AM$12,'III. Finanzberichte'!$AT$12,'III. Finanzberichte'!$BA$12,'III. Finanzberichte'!$BH$12,'III. Finanzberichte'!$BO$12,'III. Finanzberichte'!$BV$12,'III. Finanzberichte'!$CC$12,'III. Finanzberichte'!$CJ$12,'III. Finanzberichte'!$CQ$12,'III. Finanzberichte'!$CX$12,'III. Finanzberichte'!$DE$12,'III. Finanzberichte'!$DL$12,'III. Finanzberichte'!$DS$12),"")</f>
+      </c>
+      <c r="O85" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$12,'III. Finanzberichte'!$L$12,'III. Finanzberichte'!$S$12,'III. Finanzberichte'!$Z$12,'III. Finanzberichte'!$AG$12,'III. Finanzberichte'!$AN$12,'III. Finanzberichte'!$AU$12,'III. Finanzberichte'!$BB$12,'III. Finanzberichte'!$BI$12,'III. Finanzberichte'!$BP$12,'III. Finanzberichte'!$BW$12,'III. Finanzberichte'!$CD$12,'III. Finanzberichte'!$CK$12,'III. Finanzberichte'!$CR$12,'III. Finanzberichte'!$CY$12,'III. Finanzberichte'!$DF$12,'III. Finanzberichte'!$DM$12,'III. Finanzberichte'!$DT$12),"")</f>
+      </c>
+      <c r="P85" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$12,'III. Finanzberichte'!$M$12,'III. Finanzberichte'!$T$12,'III. Finanzberichte'!$AA$12,'III. Finanzberichte'!$AH$12,'III. Finanzberichte'!$AO$12,'III. Finanzberichte'!$AV$12,'III. Finanzberichte'!$BC$12,'III. Finanzberichte'!$BJ$12,'III. Finanzberichte'!$BQ$12,'III. Finanzberichte'!$BX$12,'III. Finanzberichte'!$CE$12,'III. Finanzberichte'!$CL$12,'III. Finanzberichte'!$CS$12,'III. Finanzberichte'!$CZ$12,'III. Finanzberichte'!$DG$12,'III. Finanzberichte'!$DN$12,'III. Finanzberichte'!$DU$12),"")</f>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="true">
+      <c r="B86" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="C86" s="18"/>
+      <c r="D86" s="18"/>
+      <c r="E86" s="18"/>
+      <c r="F86" s="18"/>
+      <c r="G86" s="18"/>
+      <c r="H86" s="18"/>
+      <c r="I86" s="18"/>
+      <c r="J86" s="18"/>
+      <c r="L86" s="142" t="s">
+        <v>277</v>
+      </c>
+      <c r="M86" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$13,'III. Finanzberichte'!$J$13,'III. Finanzberichte'!$Q$13,'III. Finanzberichte'!$X$13,'III. Finanzberichte'!$AE$13,'III. Finanzberichte'!$AL$13,'III. Finanzberichte'!$AS$13,'III. Finanzberichte'!$AZ$13,'III. Finanzberichte'!$BG$13,'III. Finanzberichte'!$BN$13,'III. Finanzberichte'!$BU$13,'III. Finanzberichte'!$CB$13,'III. Finanzberichte'!$CI$13,'III. Finanzberichte'!$CP$13,'III. Finanzberichte'!$CW$13,'III. Finanzberichte'!$DD$13,'III. Finanzberichte'!$DK$13,'III. Finanzberichte'!$DR$13),"")</f>
+      </c>
+      <c r="N86" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$13,'III. Finanzberichte'!$K$13,'III. Finanzberichte'!$R$13,'III. Finanzberichte'!$Y$13,'III. Finanzberichte'!$AF$13,'III. Finanzberichte'!$AM$13,'III. Finanzberichte'!$AT$13,'III. Finanzberichte'!$BA$13,'III. Finanzberichte'!$BH$13,'III. Finanzberichte'!$BO$13,'III. Finanzberichte'!$BV$13,'III. Finanzberichte'!$CC$13,'III. Finanzberichte'!$CJ$13,'III. Finanzberichte'!$CQ$13,'III. Finanzberichte'!$CX$13,'III. Finanzberichte'!$DE$13,'III. Finanzberichte'!$DL$13,'III. Finanzberichte'!$DS$13),"")</f>
+      </c>
+      <c r="O86" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$13,'III. Finanzberichte'!$L$13,'III. Finanzberichte'!$S$13,'III. Finanzberichte'!$Z$13,'III. Finanzberichte'!$AG$13,'III. Finanzberichte'!$AN$13,'III. Finanzberichte'!$AU$13,'III. Finanzberichte'!$BB$13,'III. Finanzberichte'!$BI$13,'III. Finanzberichte'!$BP$13,'III. Finanzberichte'!$BW$13,'III. Finanzberichte'!$CD$13,'III. Finanzberichte'!$CK$13,'III. Finanzberichte'!$CR$13,'III. Finanzberichte'!$CY$13,'III. Finanzberichte'!$DF$13,'III. Finanzberichte'!$DM$13,'III. Finanzberichte'!$DT$13),"")</f>
+      </c>
+      <c r="P86" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$13,'III. Finanzberichte'!$M$13,'III. Finanzberichte'!$T$13,'III. Finanzberichte'!$AA$13,'III. Finanzberichte'!$AH$13,'III. Finanzberichte'!$AO$13,'III. Finanzberichte'!$AV$13,'III. Finanzberichte'!$BC$13,'III. Finanzberichte'!$BJ$13,'III. Finanzberichte'!$BQ$13,'III. Finanzberichte'!$BX$13,'III. Finanzberichte'!$CE$13,'III. Finanzberichte'!$CL$13,'III. Finanzberichte'!$CS$13,'III. Finanzberichte'!$CZ$13,'III. Finanzberichte'!$DG$13,'III. Finanzberichte'!$DN$13,'III. Finanzberichte'!$DU$13),"")</f>
+      </c>
+    </row>
+    <row r="87">
+      <c r="L87" s="142" t="s">
+        <v>199</v>
+      </c>
+      <c r="M87" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$14,'III. Finanzberichte'!$J$14,'III. Finanzberichte'!$Q$14,'III. Finanzberichte'!$X$14,'III. Finanzberichte'!$AE$14,'III. Finanzberichte'!$AL$14,'III. Finanzberichte'!$AS$14,'III. Finanzberichte'!$AZ$14,'III. Finanzberichte'!$BG$14,'III. Finanzberichte'!$BN$14,'III. Finanzberichte'!$BU$14,'III. Finanzberichte'!$CB$14,'III. Finanzberichte'!$CI$14,'III. Finanzberichte'!$CP$14,'III. Finanzberichte'!$CW$14,'III. Finanzberichte'!$DD$14,'III. Finanzberichte'!$DK$14,'III. Finanzberichte'!$DR$14),"")</f>
+      </c>
+      <c r="N87" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$14,'III. Finanzberichte'!$K$14,'III. Finanzberichte'!$R$14,'III. Finanzberichte'!$Y$14,'III. Finanzberichte'!$AF$14,'III. Finanzberichte'!$AM$14,'III. Finanzberichte'!$AT$14,'III. Finanzberichte'!$BA$14,'III. Finanzberichte'!$BH$14,'III. Finanzberichte'!$BO$14,'III. Finanzberichte'!$BV$14,'III. Finanzberichte'!$CC$14,'III. Finanzberichte'!$CJ$14,'III. Finanzberichte'!$CQ$14,'III. Finanzberichte'!$CX$14,'III. Finanzberichte'!$DE$14,'III. Finanzberichte'!$DL$14,'III. Finanzberichte'!$DS$14),"")</f>
+      </c>
+      <c r="O87" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$14,'III. Finanzberichte'!$L$14,'III. Finanzberichte'!$S$14,'III. Finanzberichte'!$Z$14,'III. Finanzberichte'!$AG$14,'III. Finanzberichte'!$AN$14,'III. Finanzberichte'!$AU$14,'III. Finanzberichte'!$BB$14,'III. Finanzberichte'!$BI$14,'III. Finanzberichte'!$BP$14,'III. Finanzberichte'!$BW$14,'III. Finanzberichte'!$CD$14,'III. Finanzberichte'!$CK$14,'III. Finanzberichte'!$CR$14,'III. Finanzberichte'!$CY$14,'III. Finanzberichte'!$DF$14,'III. Finanzberichte'!$DM$14,'III. Finanzberichte'!$DT$14),"")</f>
+      </c>
+      <c r="P87" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$14,'III. Finanzberichte'!$M$14,'III. Finanzberichte'!$T$14,'III. Finanzberichte'!$AA$14,'III. Finanzberichte'!$AH$14,'III. Finanzberichte'!$AO$14,'III. Finanzberichte'!$AV$14,'III. Finanzberichte'!$BC$14,'III. Finanzberichte'!$BJ$14,'III. Finanzberichte'!$BQ$14,'III. Finanzberichte'!$BX$14,'III. Finanzberichte'!$CE$14,'III. Finanzberichte'!$CL$14,'III. Finanzberichte'!$CS$14,'III. Finanzberichte'!$CZ$14,'III. Finanzberichte'!$DG$14,'III. Finanzberichte'!$DN$14,'III. Finanzberichte'!$DU$14),"")</f>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="223" t="s">
+        <v>325</v>
+      </c>
+      <c r="C88" s="224"/>
+      <c r="D88" s="225" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
+      </c>
+      <c r="F88" s="230" t="s">
+        <v>330</v>
+      </c>
+      <c r="G88" s="231"/>
+      <c r="H88" s="231"/>
+      <c r="I88" s="232"/>
+      <c r="L88" s="142" t="s">
+        <v>278</v>
+      </c>
+      <c r="M88" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$15,'III. Finanzberichte'!$J$15,'III. Finanzberichte'!$Q$15,'III. Finanzberichte'!$X$15,'III. Finanzberichte'!$AE$15,'III. Finanzberichte'!$AL$15,'III. Finanzberichte'!$AS$15,'III. Finanzberichte'!$AZ$15,'III. Finanzberichte'!$BG$15,'III. Finanzberichte'!$BN$15,'III. Finanzberichte'!$BU$15,'III. Finanzberichte'!$CB$15,'III. Finanzberichte'!$CI$15,'III. Finanzberichte'!$CP$15,'III. Finanzberichte'!$CW$15,'III. Finanzberichte'!$DD$15,'III. Finanzberichte'!$DK$15,'III. Finanzberichte'!$DR$15),"")</f>
+      </c>
+      <c r="N88" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$15,'III. Finanzberichte'!$K$15,'III. Finanzberichte'!$R$15,'III. Finanzberichte'!$Y$15,'III. Finanzberichte'!$AF$15,'III. Finanzberichte'!$AM$15,'III. Finanzberichte'!$AT$15,'III. Finanzberichte'!$BA$15,'III. Finanzberichte'!$BH$15,'III. Finanzberichte'!$BO$15,'III. Finanzberichte'!$BV$15,'III. Finanzberichte'!$CC$15,'III. Finanzberichte'!$CJ$15,'III. Finanzberichte'!$CQ$15,'III. Finanzberichte'!$CX$15,'III. Finanzberichte'!$DE$15,'III. Finanzberichte'!$DL$15,'III. Finanzberichte'!$DS$15),"")</f>
+      </c>
+      <c r="O88" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$15,'III. Finanzberichte'!$L$15,'III. Finanzberichte'!$S$15,'III. Finanzberichte'!$Z$15,'III. Finanzberichte'!$AG$15,'III. Finanzberichte'!$AN$15,'III. Finanzberichte'!$AU$15,'III. Finanzberichte'!$BB$15,'III. Finanzberichte'!$BI$15,'III. Finanzberichte'!$BP$15,'III. Finanzberichte'!$BW$15,'III. Finanzberichte'!$CD$15,'III. Finanzberichte'!$CK$15,'III. Finanzberichte'!$CR$15,'III. Finanzberichte'!$CY$15,'III. Finanzberichte'!$DF$15,'III. Finanzberichte'!$DM$15,'III. Finanzberichte'!$DT$15),"")</f>
+      </c>
+      <c r="P88" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$15,'III. Finanzberichte'!$M$15,'III. Finanzberichte'!$T$15,'III. Finanzberichte'!$AA$15,'III. Finanzberichte'!$AH$15,'III. Finanzberichte'!$AO$15,'III. Finanzberichte'!$AV$15,'III. Finanzberichte'!$BC$15,'III. Finanzberichte'!$BJ$15,'III. Finanzberichte'!$BQ$15,'III. Finanzberichte'!$BX$15,'III. Finanzberichte'!$CE$15,'III. Finanzberichte'!$CL$15,'III. Finanzberichte'!$CS$15,'III. Finanzberichte'!$CZ$15,'III. Finanzberichte'!$DG$15,'III. Finanzberichte'!$DN$15,'III. Finanzberichte'!$DU$15),"")</f>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="204" t="s">
+        <v>326</v>
+      </c>
+      <c r="C89" s="196"/>
+      <c r="D89" s="226" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="F89" s="233" t="s">
+        <v>331</v>
+      </c>
+      <c r="G89" s="196" t="s">
+        <v>332</v>
+      </c>
+      <c r="H89" s="196"/>
+      <c r="I89" s="234" t="str">
+        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
+      </c>
+      <c r="L89" s="339" t="s">
+        <v>279</v>
+      </c>
+      <c r="M89" s="329" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$16,'III. Finanzberichte'!$J$16,'III. Finanzberichte'!$Q$16,'III. Finanzberichte'!$X$16,'III. Finanzberichte'!$AE$16,'III. Finanzberichte'!$AL$16,'III. Finanzberichte'!$AS$16,'III. Finanzberichte'!$AZ$16,'III. Finanzberichte'!$BG$16,'III. Finanzberichte'!$BN$16,'III. Finanzberichte'!$BU$16,'III. Finanzberichte'!$CB$16,'III. Finanzberichte'!$CI$16,'III. Finanzberichte'!$CP$16,'III. Finanzberichte'!$CW$16,'III. Finanzberichte'!$DD$16,'III. Finanzberichte'!$DK$16,'III. Finanzberichte'!$DR$16),"")</f>
+      </c>
+      <c r="N89" s="330" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$16,'III. Finanzberichte'!$K$16,'III. Finanzberichte'!$R$16,'III. Finanzberichte'!$Y$16,'III. Finanzberichte'!$AF$16,'III. Finanzberichte'!$AM$16,'III. Finanzberichte'!$AT$16,'III. Finanzberichte'!$BA$16,'III. Finanzberichte'!$BH$16,'III. Finanzberichte'!$BO$16,'III. Finanzberichte'!$BV$16,'III. Finanzberichte'!$CC$16,'III. Finanzberichte'!$CJ$16,'III. Finanzberichte'!$CQ$16,'III. Finanzberichte'!$CX$16,'III. Finanzberichte'!$DE$16,'III. Finanzberichte'!$DL$16,'III. Finanzberichte'!$DS$16),"")</f>
+      </c>
+      <c r="O89" s="329" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$16,'III. Finanzberichte'!$L$16,'III. Finanzberichte'!$S$16,'III. Finanzberichte'!$Z$16,'III. Finanzberichte'!$AG$16,'III. Finanzberichte'!$AN$16,'III. Finanzberichte'!$AU$16,'III. Finanzberichte'!$BB$16,'III. Finanzberichte'!$BI$16,'III. Finanzberichte'!$BP$16,'III. Finanzberichte'!$BW$16,'III. Finanzberichte'!$CD$16,'III. Finanzberichte'!$CK$16,'III. Finanzberichte'!$CR$16,'III. Finanzberichte'!$CY$16,'III. Finanzberichte'!$DF$16,'III. Finanzberichte'!$DM$16,'III. Finanzberichte'!$DT$16),"")</f>
+      </c>
+      <c r="P89" s="340" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$16,'III. Finanzberichte'!$M$16,'III. Finanzberichte'!$T$16,'III. Finanzberichte'!$AA$16,'III. Finanzberichte'!$AH$16,'III. Finanzberichte'!$AO$16,'III. Finanzberichte'!$AV$16,'III. Finanzberichte'!$BC$16,'III. Finanzberichte'!$BJ$16,'III. Finanzberichte'!$BQ$16,'III. Finanzberichte'!$BX$16,'III. Finanzberichte'!$CE$16,'III. Finanzberichte'!$CL$16,'III. Finanzberichte'!$CS$16,'III. Finanzberichte'!$CZ$16,'III. Finanzberichte'!$DG$16,'III. Finanzberichte'!$DN$16,'III. Finanzberichte'!$DU$16),"")</f>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="204" t="s">
+        <v>327</v>
+      </c>
+      <c r="C90" s="196"/>
+      <c r="D90" s="226" t="str">
+        <f>=ROUND($D$88-$D$89,2)</f>
+      </c>
+      <c r="F90" s="233" t="s">
+        <v>331</v>
+      </c>
+      <c r="G90" s="196" t="s">
+        <v>333</v>
+      </c>
+      <c r="H90" s="196"/>
+      <c r="I90" s="234" t="str">
+        <f>=IFERROR(ROUND(MAX(0,(SUM($G$99:$G$102)-$G$101)-(SUM($H$99:$H$102)-$H$101)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L90" s="335" t="s">
+        <v>280</v>
+      </c>
+      <c r="M90" s="326"/>
+      <c r="N90" s="326"/>
+      <c r="O90" s="326"/>
+      <c r="P90" s="336"/>
+    </row>
+    <row r="91" ht="26" customHeight="true">
+      <c r="B91" s="204" t="s">
+        <v>328</v>
+      </c>
+      <c r="C91" s="196"/>
+      <c r="D91" s="226" t="str">
+        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
+      </c>
+      <c r="F91" s="47"/>
+      <c r="G91" s="218" t="s">
+        <v>335</v>
+      </c>
+      <c r="H91" s="218"/>
+      <c r="I91" s="235" t="str">
+        <f>=ROUND(IF($F$89="Abzug",MAX(0,$I$89),0)+IF($F$90="Abzug",MAX(0,$I$90),0),2)</f>
+      </c>
+      <c r="L91" s="337" t="s">
+        <v>203</v>
+      </c>
+      <c r="M91" s="327" t="s">
+        <v>281</v>
+      </c>
+      <c r="N91" s="327" t="s">
+        <v>282</v>
+      </c>
+      <c r="O91" s="327" t="s">
+        <v>283</v>
+      </c>
+      <c r="P91" s="338" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="227" t="s">
+        <v>329</v>
+      </c>
+      <c r="C92" s="228"/>
+      <c r="D92" s="229" t="str">
+        <f>=ROUND($D$90-$D$91,2)</f>
+      </c>
+      <c r="F92" s="236"/>
+      <c r="G92" s="228" t="s">
+        <v>336</v>
+      </c>
+      <c r="H92" s="228"/>
+      <c r="I92" s="229" t="str">
+        <f>=ROUND($D$92-$I$91,2)</f>
+      </c>
+      <c r="L92" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$19,'III. Finanzberichte'!$I$19,'III. Finanzberichte'!$P$19,'III. Finanzberichte'!$W$19,'III. Finanzberichte'!$AD$19,'III. Finanzberichte'!$AK$19,'III. Finanzberichte'!$AR$19,'III. Finanzberichte'!$AY$19,'III. Finanzberichte'!$BF$19,'III. Finanzberichte'!$BM$19,'III. Finanzberichte'!$BT$19,'III. Finanzberichte'!$CA$19,'III. Finanzberichte'!$CH$19,'III. Finanzberichte'!$CO$19,'III. Finanzberichte'!$CV$19,'III. Finanzberichte'!$DC$19,'III. Finanzberichte'!$DJ$19,'III. Finanzberichte'!$DQ$19),"")</f>
+      </c>
+      <c r="M92" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$19,'III. Finanzberichte'!$J$19,'III. Finanzberichte'!$Q$19,'III. Finanzberichte'!$X$19,'III. Finanzberichte'!$AE$19,'III. Finanzberichte'!$AL$19,'III. Finanzberichte'!$AS$19,'III. Finanzberichte'!$AZ$19,'III. Finanzberichte'!$BG$19,'III. Finanzberichte'!$BN$19,'III. Finanzberichte'!$BU$19,'III. Finanzberichte'!$CB$19,'III. Finanzberichte'!$CI$19,'III. Finanzberichte'!$CP$19,'III. Finanzberichte'!$CW$19,'III. Finanzberichte'!$DD$19,'III. Finanzberichte'!$DK$19,'III. Finanzberichte'!$DR$19),"")</f>
+      </c>
+      <c r="N92" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$19,'III. Finanzberichte'!$K$19,'III. Finanzberichte'!$R$19,'III. Finanzberichte'!$Y$19,'III. Finanzberichte'!$AF$19,'III. Finanzberichte'!$AM$19,'III. Finanzberichte'!$AT$19,'III. Finanzberichte'!$BA$19,'III. Finanzberichte'!$BH$19,'III. Finanzberichte'!$BO$19,'III. Finanzberichte'!$BV$19,'III. Finanzberichte'!$CC$19,'III. Finanzberichte'!$CJ$19,'III. Finanzberichte'!$CQ$19,'III. Finanzberichte'!$CX$19,'III. Finanzberichte'!$DE$19,'III. Finanzberichte'!$DL$19,'III. Finanzberichte'!$DS$19),"")</f>
+      </c>
+      <c r="O92" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$19,'III. Finanzberichte'!$L$19,'III. Finanzberichte'!$S$19,'III. Finanzberichte'!$Z$19,'III. Finanzberichte'!$AG$19,'III. Finanzberichte'!$AN$19,'III. Finanzberichte'!$AU$19,'III. Finanzberichte'!$BB$19,'III. Finanzberichte'!$BI$19,'III. Finanzberichte'!$BP$19,'III. Finanzberichte'!$BW$19,'III. Finanzberichte'!$CD$19,'III. Finanzberichte'!$CK$19,'III. Finanzberichte'!$CR$19,'III. Finanzberichte'!$CY$19,'III. Finanzberichte'!$DF$19,'III. Finanzberichte'!$DM$19,'III. Finanzberichte'!$DT$19),"")</f>
+      </c>
+      <c r="P92" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$19,'III. Finanzberichte'!$M$19,'III. Finanzberichte'!$T$19,'III. Finanzberichte'!$AA$19,'III. Finanzberichte'!$AH$19,'III. Finanzberichte'!$AO$19,'III. Finanzberichte'!$AV$19,'III. Finanzberichte'!$BC$19,'III. Finanzberichte'!$BJ$19,'III. Finanzberichte'!$BQ$19,'III. Finanzberichte'!$BX$19,'III. Finanzberichte'!$CE$19,'III. Finanzberichte'!$CL$19,'III. Finanzberichte'!$CS$19,'III. Finanzberichte'!$CZ$19,'III. Finanzberichte'!$DG$19,'III. Finanzberichte'!$DN$19,'III. Finanzberichte'!$DU$19),"")</f>
+      </c>
+    </row>
+    <row r="93">
+      <c r="L93" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$20,'III. Finanzberichte'!$I$20,'III. Finanzberichte'!$P$20,'III. Finanzberichte'!$W$20,'III. Finanzberichte'!$AD$20,'III. Finanzberichte'!$AK$20,'III. Finanzberichte'!$AR$20,'III. Finanzberichte'!$AY$20,'III. Finanzberichte'!$BF$20,'III. Finanzberichte'!$BM$20,'III. Finanzberichte'!$BT$20,'III. Finanzberichte'!$CA$20,'III. Finanzberichte'!$CH$20,'III. Finanzberichte'!$CO$20,'III. Finanzberichte'!$CV$20,'III. Finanzberichte'!$DC$20,'III. Finanzberichte'!$DJ$20,'III. Finanzberichte'!$DQ$20),"")</f>
+      </c>
+      <c r="M93" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$20,'III. Finanzberichte'!$J$20,'III. Finanzberichte'!$Q$20,'III. Finanzberichte'!$X$20,'III. Finanzberichte'!$AE$20,'III. Finanzberichte'!$AL$20,'III. Finanzberichte'!$AS$20,'III. Finanzberichte'!$AZ$20,'III. Finanzberichte'!$BG$20,'III. Finanzberichte'!$BN$20,'III. Finanzberichte'!$BU$20,'III. Finanzberichte'!$CB$20,'III. Finanzberichte'!$CI$20,'III. Finanzberichte'!$CP$20,'III. Finanzberichte'!$CW$20,'III. Finanzberichte'!$DD$20,'III. Finanzberichte'!$DK$20,'III. Finanzberichte'!$DR$20),"")</f>
+      </c>
+      <c r="N93" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$20,'III. Finanzberichte'!$K$20,'III. Finanzberichte'!$R$20,'III. Finanzberichte'!$Y$20,'III. Finanzberichte'!$AF$20,'III. Finanzberichte'!$AM$20,'III. Finanzberichte'!$AT$20,'III. Finanzberichte'!$BA$20,'III. Finanzberichte'!$BH$20,'III. Finanzberichte'!$BO$20,'III. Finanzberichte'!$BV$20,'III. Finanzberichte'!$CC$20,'III. Finanzberichte'!$CJ$20,'III. Finanzberichte'!$CQ$20,'III. Finanzberichte'!$CX$20,'III. Finanzberichte'!$DE$20,'III. Finanzberichte'!$DL$20,'III. Finanzberichte'!$DS$20),"")</f>
+      </c>
+      <c r="O93" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$20,'III. Finanzberichte'!$L$20,'III. Finanzberichte'!$S$20,'III. Finanzberichte'!$Z$20,'III. Finanzberichte'!$AG$20,'III. Finanzberichte'!$AN$20,'III. Finanzberichte'!$AU$20,'III. Finanzberichte'!$BB$20,'III. Finanzberichte'!$BI$20,'III. Finanzberichte'!$BP$20,'III. Finanzberichte'!$BW$20,'III. Finanzberichte'!$CD$20,'III. Finanzberichte'!$CK$20,'III. Finanzberichte'!$CR$20,'III. Finanzberichte'!$CY$20,'III. Finanzberichte'!$DF$20,'III. Finanzberichte'!$DM$20,'III. Finanzberichte'!$DT$20),"")</f>
+      </c>
+      <c r="P93" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$20,'III. Finanzberichte'!$M$20,'III. Finanzberichte'!$T$20,'III. Finanzberichte'!$AA$20,'III. Finanzberichte'!$AH$20,'III. Finanzberichte'!$AO$20,'III. Finanzberichte'!$AV$20,'III. Finanzberichte'!$BC$20,'III. Finanzberichte'!$BJ$20,'III. Finanzberichte'!$BQ$20,'III. Finanzberichte'!$BX$20,'III. Finanzberichte'!$CE$20,'III. Finanzberichte'!$CL$20,'III. Finanzberichte'!$CS$20,'III. Finanzberichte'!$CZ$20,'III. Finanzberichte'!$DG$20,'III. Finanzberichte'!$DN$20,'III. Finanzberichte'!$DU$20),"")</f>
+      </c>
+    </row>
+    <row r="94">
+      <c r="L94" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$21,'III. Finanzberichte'!$I$21,'III. Finanzberichte'!$P$21,'III. Finanzberichte'!$W$21,'III. Finanzberichte'!$AD$21,'III. Finanzberichte'!$AK$21,'III. Finanzberichte'!$AR$21,'III. Finanzberichte'!$AY$21,'III. Finanzberichte'!$BF$21,'III. Finanzberichte'!$BM$21,'III. Finanzberichte'!$BT$21,'III. Finanzberichte'!$CA$21,'III. Finanzberichte'!$CH$21,'III. Finanzberichte'!$CO$21,'III. Finanzberichte'!$CV$21,'III. Finanzberichte'!$DC$21,'III. Finanzberichte'!$DJ$21,'III. Finanzberichte'!$DQ$21),"")</f>
+      </c>
+      <c r="M94" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$21,'III. Finanzberichte'!$J$21,'III. Finanzberichte'!$Q$21,'III. Finanzberichte'!$X$21,'III. Finanzberichte'!$AE$21,'III. Finanzberichte'!$AL$21,'III. Finanzberichte'!$AS$21,'III. Finanzberichte'!$AZ$21,'III. Finanzberichte'!$BG$21,'III. Finanzberichte'!$BN$21,'III. Finanzberichte'!$BU$21,'III. Finanzberichte'!$CB$21,'III. Finanzberichte'!$CI$21,'III. Finanzberichte'!$CP$21,'III. Finanzberichte'!$CW$21,'III. Finanzberichte'!$DD$21,'III. Finanzberichte'!$DK$21,'III. Finanzberichte'!$DR$21),"")</f>
+      </c>
+      <c r="N94" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$21,'III. Finanzberichte'!$K$21,'III. Finanzberichte'!$R$21,'III. Finanzberichte'!$Y$21,'III. Finanzberichte'!$AF$21,'III. Finanzberichte'!$AM$21,'III. Finanzberichte'!$AT$21,'III. Finanzberichte'!$BA$21,'III. Finanzberichte'!$BH$21,'III. Finanzberichte'!$BO$21,'III. Finanzberichte'!$BV$21,'III. Finanzberichte'!$CC$21,'III. Finanzberichte'!$CJ$21,'III. Finanzberichte'!$CQ$21,'III. Finanzberichte'!$CX$21,'III. Finanzberichte'!$DE$21,'III. Finanzberichte'!$DL$21,'III. Finanzberichte'!$DS$21),"")</f>
+      </c>
+      <c r="O94" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$21,'III. Finanzberichte'!$L$21,'III. Finanzberichte'!$S$21,'III. Finanzberichte'!$Z$21,'III. Finanzberichte'!$AG$21,'III. Finanzberichte'!$AN$21,'III. Finanzberichte'!$AU$21,'III. Finanzberichte'!$BB$21,'III. Finanzberichte'!$BI$21,'III. Finanzberichte'!$BP$21,'III. Finanzberichte'!$BW$21,'III. Finanzberichte'!$CD$21,'III. Finanzberichte'!$CK$21,'III. Finanzberichte'!$CR$21,'III. Finanzberichte'!$CY$21,'III. Finanzberichte'!$DF$21,'III. Finanzberichte'!$DM$21,'III. Finanzberichte'!$DT$21),"")</f>
+      </c>
+      <c r="P94" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$21,'III. Finanzberichte'!$M$21,'III. Finanzberichte'!$T$21,'III. Finanzberichte'!$AA$21,'III. Finanzberichte'!$AH$21,'III. Finanzberichte'!$AO$21,'III. Finanzberichte'!$AV$21,'III. Finanzberichte'!$BC$21,'III. Finanzberichte'!$BJ$21,'III. Finanzberichte'!$BQ$21,'III. Finanzberichte'!$BX$21,'III. Finanzberichte'!$CE$21,'III. Finanzberichte'!$CL$21,'III. Finanzberichte'!$CS$21,'III. Finanzberichte'!$CZ$21,'III. Finanzberichte'!$DG$21,'III. Finanzberichte'!$DN$21,'III. Finanzberichte'!$DU$21),"")</f>
+      </c>
+    </row>
+    <row r="95">
+      <c r="L95" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$22,'III. Finanzberichte'!$I$22,'III. Finanzberichte'!$P$22,'III. Finanzberichte'!$W$22,'III. Finanzberichte'!$AD$22,'III. Finanzberichte'!$AK$22,'III. Finanzberichte'!$AR$22,'III. Finanzberichte'!$AY$22,'III. Finanzberichte'!$BF$22,'III. Finanzberichte'!$BM$22,'III. Finanzberichte'!$BT$22,'III. Finanzberichte'!$CA$22,'III. Finanzberichte'!$CH$22,'III. Finanzberichte'!$CO$22,'III. Finanzberichte'!$CV$22,'III. Finanzberichte'!$DC$22,'III. Finanzberichte'!$DJ$22,'III. Finanzberichte'!$DQ$22),"")</f>
+      </c>
+      <c r="M95" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$22,'III. Finanzberichte'!$J$22,'III. Finanzberichte'!$Q$22,'III. Finanzberichte'!$X$22,'III. Finanzberichte'!$AE$22,'III. Finanzberichte'!$AL$22,'III. Finanzberichte'!$AS$22,'III. Finanzberichte'!$AZ$22,'III. Finanzberichte'!$BG$22,'III. Finanzberichte'!$BN$22,'III. Finanzberichte'!$BU$22,'III. Finanzberichte'!$CB$22,'III. Finanzberichte'!$CI$22,'III. Finanzberichte'!$CP$22,'III. Finanzberichte'!$CW$22,'III. Finanzberichte'!$DD$22,'III. Finanzberichte'!$DK$22,'III. Finanzberichte'!$DR$22),"")</f>
+      </c>
+      <c r="N95" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$22,'III. Finanzberichte'!$K$22,'III. Finanzberichte'!$R$22,'III. Finanzberichte'!$Y$22,'III. Finanzberichte'!$AF$22,'III. Finanzberichte'!$AM$22,'III. Finanzberichte'!$AT$22,'III. Finanzberichte'!$BA$22,'III. Finanzberichte'!$BH$22,'III. Finanzberichte'!$BO$22,'III. Finanzberichte'!$BV$22,'III. Finanzberichte'!$CC$22,'III. Finanzberichte'!$CJ$22,'III. Finanzberichte'!$CQ$22,'III. Finanzberichte'!$CX$22,'III. Finanzberichte'!$DE$22,'III. Finanzberichte'!$DL$22,'III. Finanzberichte'!$DS$22),"")</f>
+      </c>
+      <c r="O95" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$22,'III. Finanzberichte'!$L$22,'III. Finanzberichte'!$S$22,'III. Finanzberichte'!$Z$22,'III. Finanzberichte'!$AG$22,'III. Finanzberichte'!$AN$22,'III. Finanzberichte'!$AU$22,'III. Finanzberichte'!$BB$22,'III. Finanzberichte'!$BI$22,'III. Finanzberichte'!$BP$22,'III. Finanzberichte'!$BW$22,'III. Finanzberichte'!$CD$22,'III. Finanzberichte'!$CK$22,'III. Finanzberichte'!$CR$22,'III. Finanzberichte'!$CY$22,'III. Finanzberichte'!$DF$22,'III. Finanzberichte'!$DM$22,'III. Finanzberichte'!$DT$22),"")</f>
+      </c>
+      <c r="P95" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$22,'III. Finanzberichte'!$M$22,'III. Finanzberichte'!$T$22,'III. Finanzberichte'!$AA$22,'III. Finanzberichte'!$AH$22,'III. Finanzberichte'!$AO$22,'III. Finanzberichte'!$AV$22,'III. Finanzberichte'!$BC$22,'III. Finanzberichte'!$BJ$22,'III. Finanzberichte'!$BQ$22,'III. Finanzberichte'!$BX$22,'III. Finanzberichte'!$CE$22,'III. Finanzberichte'!$CL$22,'III. Finanzberichte'!$CS$22,'III. Finanzberichte'!$CZ$22,'III. Finanzberichte'!$DG$22,'III. Finanzberichte'!$DN$22,'III. Finanzberichte'!$DU$22),"")</f>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="true">
+      <c r="B96" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="C96" s="18"/>
+      <c r="D96" s="18"/>
+      <c r="E96" s="18"/>
+      <c r="F96" s="18"/>
+      <c r="G96" s="18"/>
+      <c r="H96" s="18"/>
+      <c r="I96" s="18"/>
+      <c r="J96" s="18"/>
+      <c r="L96" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$23,'III. Finanzberichte'!$I$23,'III. Finanzberichte'!$P$23,'III. Finanzberichte'!$W$23,'III. Finanzberichte'!$AD$23,'III. Finanzberichte'!$AK$23,'III. Finanzberichte'!$AR$23,'III. Finanzberichte'!$AY$23,'III. Finanzberichte'!$BF$23,'III. Finanzberichte'!$BM$23,'III. Finanzberichte'!$BT$23,'III. Finanzberichte'!$CA$23,'III. Finanzberichte'!$CH$23,'III. Finanzberichte'!$CO$23,'III. Finanzberichte'!$CV$23,'III. Finanzberichte'!$DC$23,'III. Finanzberichte'!$DJ$23,'III. Finanzberichte'!$DQ$23),"")</f>
+      </c>
+      <c r="M96" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$23,'III. Finanzberichte'!$J$23,'III. Finanzberichte'!$Q$23,'III. Finanzberichte'!$X$23,'III. Finanzberichte'!$AE$23,'III. Finanzberichte'!$AL$23,'III. Finanzberichte'!$AS$23,'III. Finanzberichte'!$AZ$23,'III. Finanzberichte'!$BG$23,'III. Finanzberichte'!$BN$23,'III. Finanzberichte'!$BU$23,'III. Finanzberichte'!$CB$23,'III. Finanzberichte'!$CI$23,'III. Finanzberichte'!$CP$23,'III. Finanzberichte'!$CW$23,'III. Finanzberichte'!$DD$23,'III. Finanzberichte'!$DK$23,'III. Finanzberichte'!$DR$23),"")</f>
+      </c>
+      <c r="N96" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$23,'III. Finanzberichte'!$K$23,'III. Finanzberichte'!$R$23,'III. Finanzberichte'!$Y$23,'III. Finanzberichte'!$AF$23,'III. Finanzberichte'!$AM$23,'III. Finanzberichte'!$AT$23,'III. Finanzberichte'!$BA$23,'III. Finanzberichte'!$BH$23,'III. Finanzberichte'!$BO$23,'III. Finanzberichte'!$BV$23,'III. Finanzberichte'!$CC$23,'III. Finanzberichte'!$CJ$23,'III. Finanzberichte'!$CQ$23,'III. Finanzberichte'!$CX$23,'III. Finanzberichte'!$DE$23,'III. Finanzberichte'!$DL$23,'III. Finanzberichte'!$DS$23),"")</f>
+      </c>
+      <c r="O96" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$23,'III. Finanzberichte'!$L$23,'III. Finanzberichte'!$S$23,'III. Finanzberichte'!$Z$23,'III. Finanzberichte'!$AG$23,'III. Finanzberichte'!$AN$23,'III. Finanzberichte'!$AU$23,'III. Finanzberichte'!$BB$23,'III. Finanzberichte'!$BI$23,'III. Finanzberichte'!$BP$23,'III. Finanzberichte'!$BW$23,'III. Finanzberichte'!$CD$23,'III. Finanzberichte'!$CK$23,'III. Finanzberichte'!$CR$23,'III. Finanzberichte'!$CY$23,'III. Finanzberichte'!$DF$23,'III. Finanzberichte'!$DM$23,'III. Finanzberichte'!$DT$23),"")</f>
+      </c>
+      <c r="P96" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$23,'III. Finanzberichte'!$M$23,'III. Finanzberichte'!$T$23,'III. Finanzberichte'!$AA$23,'III. Finanzberichte'!$AH$23,'III. Finanzberichte'!$AO$23,'III. Finanzberichte'!$AV$23,'III. Finanzberichte'!$BC$23,'III. Finanzberichte'!$BJ$23,'III. Finanzberichte'!$BQ$23,'III. Finanzberichte'!$BX$23,'III. Finanzberichte'!$CE$23,'III. Finanzberichte'!$CL$23,'III. Finanzberichte'!$CS$23,'III. Finanzberichte'!$CZ$23,'III. Finanzberichte'!$DG$23,'III. Finanzberichte'!$DN$23,'III. Finanzberichte'!$DU$23),"")</f>
+      </c>
+    </row>
+    <row r="97">
+      <c r="L97" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$24,'III. Finanzberichte'!$I$24,'III. Finanzberichte'!$P$24,'III. Finanzberichte'!$W$24,'III. Finanzberichte'!$AD$24,'III. Finanzberichte'!$AK$24,'III. Finanzberichte'!$AR$24,'III. Finanzberichte'!$AY$24,'III. Finanzberichte'!$BF$24,'III. Finanzberichte'!$BM$24,'III. Finanzberichte'!$BT$24,'III. Finanzberichte'!$CA$24,'III. Finanzberichte'!$CH$24,'III. Finanzberichte'!$CO$24,'III. Finanzberichte'!$CV$24,'III. Finanzberichte'!$DC$24,'III. Finanzberichte'!$DJ$24,'III. Finanzberichte'!$DQ$24),"")</f>
+      </c>
+      <c r="M97" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$24,'III. Finanzberichte'!$J$24,'III. Finanzberichte'!$Q$24,'III. Finanzberichte'!$X$24,'III. Finanzberichte'!$AE$24,'III. Finanzberichte'!$AL$24,'III. Finanzberichte'!$AS$24,'III. Finanzberichte'!$AZ$24,'III. Finanzberichte'!$BG$24,'III. Finanzberichte'!$BN$24,'III. Finanzberichte'!$BU$24,'III. Finanzberichte'!$CB$24,'III. Finanzberichte'!$CI$24,'III. Finanzberichte'!$CP$24,'III. Finanzberichte'!$CW$24,'III. Finanzberichte'!$DD$24,'III. Finanzberichte'!$DK$24,'III. Finanzberichte'!$DR$24),"")</f>
+      </c>
+      <c r="N97" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$24,'III. Finanzberichte'!$K$24,'III. Finanzberichte'!$R$24,'III. Finanzberichte'!$Y$24,'III. Finanzberichte'!$AF$24,'III. Finanzberichte'!$AM$24,'III. Finanzberichte'!$AT$24,'III. Finanzberichte'!$BA$24,'III. Finanzberichte'!$BH$24,'III. Finanzberichte'!$BO$24,'III. Finanzberichte'!$BV$24,'III. Finanzberichte'!$CC$24,'III. Finanzberichte'!$CJ$24,'III. Finanzberichte'!$CQ$24,'III. Finanzberichte'!$CX$24,'III. Finanzberichte'!$DE$24,'III. Finanzberichte'!$DL$24,'III. Finanzberichte'!$DS$24),"")</f>
+      </c>
+      <c r="O97" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$24,'III. Finanzberichte'!$L$24,'III. Finanzberichte'!$S$24,'III. Finanzberichte'!$Z$24,'III. Finanzberichte'!$AG$24,'III. Finanzberichte'!$AN$24,'III. Finanzberichte'!$AU$24,'III. Finanzberichte'!$BB$24,'III. Finanzberichte'!$BI$24,'III. Finanzberichte'!$BP$24,'III. Finanzberichte'!$BW$24,'III. Finanzberichte'!$CD$24,'III. Finanzberichte'!$CK$24,'III. Finanzberichte'!$CR$24,'III. Finanzberichte'!$CY$24,'III. Finanzberichte'!$DF$24,'III. Finanzberichte'!$DM$24,'III. Finanzberichte'!$DT$24),"")</f>
+      </c>
+      <c r="P97" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$24,'III. Finanzberichte'!$M$24,'III. Finanzberichte'!$T$24,'III. Finanzberichte'!$AA$24,'III. Finanzberichte'!$AH$24,'III. Finanzberichte'!$AO$24,'III. Finanzberichte'!$AV$24,'III. Finanzberichte'!$BC$24,'III. Finanzberichte'!$BJ$24,'III. Finanzberichte'!$BQ$24,'III. Finanzberichte'!$BX$24,'III. Finanzberichte'!$CE$24,'III. Finanzberichte'!$CL$24,'III. Finanzberichte'!$CS$24,'III. Finanzberichte'!$CZ$24,'III. Finanzberichte'!$DG$24,'III. Finanzberichte'!$DN$24,'III. Finanzberichte'!$DU$24),"")</f>
+      </c>
+    </row>
+    <row r="98" ht="28" customHeight="true">
+      <c r="B98" s="263" t="s">
+        <v>356</v>
+      </c>
+      <c r="C98" s="264" t="s">
+        <v>373</v>
+      </c>
+      <c r="D98" s="264" t="s">
+        <v>358</v>
+      </c>
+      <c r="E98" s="264" t="s">
+        <v>359</v>
+      </c>
+      <c r="F98" s="264" t="s">
+        <v>360</v>
+      </c>
+      <c r="G98" s="264" t="s">
+        <v>374</v>
+      </c>
+      <c r="H98" s="264" t="s">
+        <v>362</v>
+      </c>
+      <c r="I98" s="264" t="s">
+        <v>363</v>
+      </c>
+      <c r="J98" s="265" t="s">
         <v>364</v>
       </c>
-      <c r="C72" s="193"/>
-      <c r="D72" s="193"/>
-      <c r="E72" s="193"/>
-      <c r="F72" s="193"/>
-      <c r="G72" s="193"/>
-      <c r="H72" s="193"/>
-      <c r="I72" s="193"/>
-      <c r="J72" s="193"/>
-    </row>
-    <row r="73">
-      <c r="B73" s="194" t="s">
-        <v>365</v>
-      </c>
-      <c r="C73" s="194"/>
-      <c r="D73" s="194"/>
-      <c r="E73" s="194"/>
-      <c r="F73" s="194"/>
-      <c r="G73" s="194"/>
-      <c r="H73" s="194"/>
-      <c r="I73" s="194"/>
-      <c r="J73" s="194"/>
-    </row>
-    <row r="75" ht="22" customHeight="true">
-      <c r="C75" s="201" t="s">
-        <v>366</v>
-      </c>
-      <c r="D75" s="202"/>
-      <c r="E75" s="202"/>
-      <c r="F75" s="202"/>
-      <c r="G75" s="202"/>
-      <c r="H75" s="202"/>
-      <c r="I75" s="203"/>
-    </row>
-    <row r="76">
-      <c r="C76" s="204" t="s">
-        <v>320</v>
-      </c>
-      <c r="D76" s="196"/>
-      <c r="E76" s="196"/>
-      <c r="F76" s="33" t="s">
-        <v>158</v>
-      </c>
-      <c r="G76" s="33"/>
-      <c r="H76" s="33"/>
-      <c r="I76" s="205"/>
-    </row>
-    <row r="77">
-      <c r="C77" s="204" t="s">
-        <v>367</v>
-      </c>
-      <c r="D77" s="196"/>
-      <c r="E77" s="196"/>
-      <c r="F77" s="197" t="str">
-        <f>=IF(LEFT(F76,8)="Periode ",IFERROR(VALUE(TRIM(MID(F76,9,5))),0),0)</f>
-      </c>
-      <c r="G77" s="197"/>
-      <c r="H77" s="197"/>
-      <c r="I77" s="284"/>
-    </row>
-    <row r="78">
-      <c r="C78" s="204" t="s">
-        <v>368</v>
-      </c>
-      <c r="D78" s="196"/>
-      <c r="E78" s="196"/>
-      <c r="F78" s="239" t="str">
-        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoLC_"&amp;F77),2),0)</f>
-      </c>
-      <c r="G78" s="239"/>
-      <c r="H78" s="239"/>
-      <c r="I78" s="245"/>
-    </row>
-    <row r="79">
-      <c r="C79" s="252" t="s">
-        <v>171</v>
-      </c>
-      <c r="D79" s="253"/>
-      <c r="E79" s="253"/>
-      <c r="F79" s="285" t="str">
-        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoEUR_"&amp;F77),2),0)</f>
-      </c>
-      <c r="G79" s="285"/>
-      <c r="H79" s="285"/>
-      <c r="I79" s="286"/>
-    </row>
-    <row r="81" ht="22" customHeight="true">
-      <c r="B81" s="18" t="s">
-        <v>369</v>
-      </c>
-      <c r="C81" s="18"/>
-      <c r="D81" s="18"/>
-      <c r="E81" s="18"/>
-      <c r="F81" s="18"/>
-      <c r="G81" s="18"/>
-      <c r="H81" s="18"/>
-      <c r="I81" s="18"/>
-      <c r="J81" s="18"/>
-    </row>
-    <row r="83">
-      <c r="B83" s="223" t="s">
-        <v>325</v>
-      </c>
-      <c r="C83" s="224"/>
-      <c r="D83" s="225" t="str">
+      <c r="L98" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$25,'III. Finanzberichte'!$I$25,'III. Finanzberichte'!$P$25,'III. Finanzberichte'!$W$25,'III. Finanzberichte'!$AD$25,'III. Finanzberichte'!$AK$25,'III. Finanzberichte'!$AR$25,'III. Finanzberichte'!$AY$25,'III. Finanzberichte'!$BF$25,'III. Finanzberichte'!$BM$25,'III. Finanzberichte'!$BT$25,'III. Finanzberichte'!$CA$25,'III. Finanzberichte'!$CH$25,'III. Finanzberichte'!$CO$25,'III. Finanzberichte'!$CV$25,'III. Finanzberichte'!$DC$25,'III. Finanzberichte'!$DJ$25,'III. Finanzberichte'!$DQ$25),"")</f>
+      </c>
+      <c r="M98" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$25,'III. Finanzberichte'!$J$25,'III. Finanzberichte'!$Q$25,'III. Finanzberichte'!$X$25,'III. Finanzberichte'!$AE$25,'III. Finanzberichte'!$AL$25,'III. Finanzberichte'!$AS$25,'III. Finanzberichte'!$AZ$25,'III. Finanzberichte'!$BG$25,'III. Finanzberichte'!$BN$25,'III. Finanzberichte'!$BU$25,'III. Finanzberichte'!$CB$25,'III. Finanzberichte'!$CI$25,'III. Finanzberichte'!$CP$25,'III. Finanzberichte'!$CW$25,'III. Finanzberichte'!$DD$25,'III. Finanzberichte'!$DK$25,'III. Finanzberichte'!$DR$25),"")</f>
+      </c>
+      <c r="N98" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$25,'III. Finanzberichte'!$K$25,'III. Finanzberichte'!$R$25,'III. Finanzberichte'!$Y$25,'III. Finanzberichte'!$AF$25,'III. Finanzberichte'!$AM$25,'III. Finanzberichte'!$AT$25,'III. Finanzberichte'!$BA$25,'III. Finanzberichte'!$BH$25,'III. Finanzberichte'!$BO$25,'III. Finanzberichte'!$BV$25,'III. Finanzberichte'!$CC$25,'III. Finanzberichte'!$CJ$25,'III. Finanzberichte'!$CQ$25,'III. Finanzberichte'!$CX$25,'III. Finanzberichte'!$DE$25,'III. Finanzberichte'!$DL$25,'III. Finanzberichte'!$DS$25),"")</f>
+      </c>
+      <c r="O98" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$25,'III. Finanzberichte'!$L$25,'III. Finanzberichte'!$S$25,'III. Finanzberichte'!$Z$25,'III. Finanzberichte'!$AG$25,'III. Finanzberichte'!$AN$25,'III. Finanzberichte'!$AU$25,'III. Finanzberichte'!$BB$25,'III. Finanzberichte'!$BI$25,'III. Finanzberichte'!$BP$25,'III. Finanzberichte'!$BW$25,'III. Finanzberichte'!$CD$25,'III. Finanzberichte'!$CK$25,'III. Finanzberichte'!$CR$25,'III. Finanzberichte'!$CY$25,'III. Finanzberichte'!$DF$25,'III. Finanzberichte'!$DM$25,'III. Finanzberichte'!$DT$25),"")</f>
+      </c>
+      <c r="P98" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$25,'III. Finanzberichte'!$M$25,'III. Finanzberichte'!$T$25,'III. Finanzberichte'!$AA$25,'III. Finanzberichte'!$AH$25,'III. Finanzberichte'!$AO$25,'III. Finanzberichte'!$AV$25,'III. Finanzberichte'!$BC$25,'III. Finanzberichte'!$BJ$25,'III. Finanzberichte'!$BQ$25,'III. Finanzberichte'!$BX$25,'III. Finanzberichte'!$CE$25,'III. Finanzberichte'!$CL$25,'III. Finanzberichte'!$CS$25,'III. Finanzberichte'!$CZ$25,'III. Finanzberichte'!$DG$25,'III. Finanzberichte'!$DN$25,'III. Finanzberichte'!$DU$25),"")</f>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="266" t="s">
+        <v>194</v>
+      </c>
+      <c r="C99" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$12,'III. Finanzberichte'!$L$12,'III. Finanzberichte'!$S$12,'III. Finanzberichte'!$Z$12,'III. Finanzberichte'!$AG$12,'III. Finanzberichte'!$AN$12,'III. Finanzberichte'!$AU$12,'III. Finanzberichte'!$BB$12,'III. Finanzberichte'!$BI$12,'III. Finanzberichte'!$BP$12,'III. Finanzberichte'!$BW$12,'III. Finanzberichte'!$CD$12,'III. Finanzberichte'!$CK$12,'III. Finanzberichte'!$CR$12,'III. Finanzberichte'!$CY$12,'III. Finanzberichte'!$DF$12,'III. Finanzberichte'!$DM$12,'III. Finanzberichte'!$DT$12),2),0)</f>
+      </c>
+      <c r="D99" s="240" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
+      </c>
+      <c r="E99" s="200" t="str">
+        <f>=ROUND(IFERROR($C$99-$D$99,0),2)</f>
+      </c>
+      <c r="F99" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$99/$D$99)-1,0),4)</f>
+      </c>
+      <c r="G99" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$12,'III. Finanzberichte'!$M$12,'III. Finanzberichte'!$T$12,'III. Finanzberichte'!$AA$12,'III. Finanzberichte'!$AH$12,'III. Finanzberichte'!$AO$12,'III. Finanzberichte'!$AV$12,'III. Finanzberichte'!$BC$12,'III. Finanzberichte'!$BJ$12,'III. Finanzberichte'!$BQ$12,'III. Finanzberichte'!$BX$12,'III. Finanzberichte'!$CE$12,'III. Finanzberichte'!$CL$12,'III. Finanzberichte'!$CS$12,'III. Finanzberichte'!$CZ$12,'III. Finanzberichte'!$DG$12,'III. Finanzberichte'!$DN$12,'III. Finanzberichte'!$DU$12),2),0)</f>
+      </c>
+      <c r="H99" s="217" t="str">
+        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
+      </c>
+      <c r="I99" s="181" t="str">
+        <f>=ROUND(IFERROR($G$99-$H$99,0),2)</f>
+      </c>
+      <c r="J99" s="290" t="str">
+        <f>=ROUND(IFERROR(($G$99/$H$99)-1,0),4)</f>
+      </c>
+      <c r="L99" s="142" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$B$26,'III. Finanzberichte'!$I$26,'III. Finanzberichte'!$P$26,'III. Finanzberichte'!$W$26,'III. Finanzberichte'!$AD$26,'III. Finanzberichte'!$AK$26,'III. Finanzberichte'!$AR$26,'III. Finanzberichte'!$AY$26,'III. Finanzberichte'!$BF$26,'III. Finanzberichte'!$BM$26,'III. Finanzberichte'!$BT$26,'III. Finanzberichte'!$CA$26,'III. Finanzberichte'!$CH$26,'III. Finanzberichte'!$CO$26,'III. Finanzberichte'!$CV$26,'III. Finanzberichte'!$DC$26,'III. Finanzberichte'!$DJ$26,'III. Finanzberichte'!$DQ$26),"")</f>
+      </c>
+      <c r="M99" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$26,'III. Finanzberichte'!$J$26,'III. Finanzberichte'!$Q$26,'III. Finanzberichte'!$X$26,'III. Finanzberichte'!$AE$26,'III. Finanzberichte'!$AL$26,'III. Finanzberichte'!$AS$26,'III. Finanzberichte'!$AZ$26,'III. Finanzberichte'!$BG$26,'III. Finanzberichte'!$BN$26,'III. Finanzberichte'!$BU$26,'III. Finanzberichte'!$CB$26,'III. Finanzberichte'!$CI$26,'III. Finanzberichte'!$CP$26,'III. Finanzberichte'!$CW$26,'III. Finanzberichte'!$DD$26,'III. Finanzberichte'!$DK$26,'III. Finanzberichte'!$DR$26),"")</f>
+      </c>
+      <c r="N99" s="116" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$26,'III. Finanzberichte'!$K$26,'III. Finanzberichte'!$R$26,'III. Finanzberichte'!$Y$26,'III. Finanzberichte'!$AF$26,'III. Finanzberichte'!$AM$26,'III. Finanzberichte'!$AT$26,'III. Finanzberichte'!$BA$26,'III. Finanzberichte'!$BH$26,'III. Finanzberichte'!$BO$26,'III. Finanzberichte'!$BV$26,'III. Finanzberichte'!$CC$26,'III. Finanzberichte'!$CJ$26,'III. Finanzberichte'!$CQ$26,'III. Finanzberichte'!$CX$26,'III. Finanzberichte'!$DE$26,'III. Finanzberichte'!$DL$26,'III. Finanzberichte'!$DS$26),"")</f>
+      </c>
+      <c r="O99" s="115" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$26,'III. Finanzberichte'!$L$26,'III. Finanzberichte'!$S$26,'III. Finanzberichte'!$Z$26,'III. Finanzberichte'!$AG$26,'III. Finanzberichte'!$AN$26,'III. Finanzberichte'!$AU$26,'III. Finanzberichte'!$BB$26,'III. Finanzberichte'!$BI$26,'III. Finanzberichte'!$BP$26,'III. Finanzberichte'!$BW$26,'III. Finanzberichte'!$CD$26,'III. Finanzberichte'!$CK$26,'III. Finanzberichte'!$CR$26,'III. Finanzberichte'!$CY$26,'III. Finanzberichte'!$DF$26,'III. Finanzberichte'!$DM$26,'III. Finanzberichte'!$DT$26),"")</f>
+      </c>
+      <c r="P99" s="143" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$26,'III. Finanzberichte'!$M$26,'III. Finanzberichte'!$T$26,'III. Finanzberichte'!$AA$26,'III. Finanzberichte'!$AH$26,'III. Finanzberichte'!$AO$26,'III. Finanzberichte'!$AV$26,'III. Finanzberichte'!$BC$26,'III. Finanzberichte'!$BJ$26,'III. Finanzberichte'!$BQ$26,'III. Finanzberichte'!$BX$26,'III. Finanzberichte'!$CE$26,'III. Finanzberichte'!$CL$26,'III. Finanzberichte'!$CS$26,'III. Finanzberichte'!$CZ$26,'III. Finanzberichte'!$DG$26,'III. Finanzberichte'!$DN$26,'III. Finanzberichte'!$DU$26),"")</f>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="266" t="s">
+        <v>277</v>
+      </c>
+      <c r="C100" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$13,'III. Finanzberichte'!$L$13,'III. Finanzberichte'!$S$13,'III. Finanzberichte'!$Z$13,'III. Finanzberichte'!$AG$13,'III. Finanzberichte'!$AN$13,'III. Finanzberichte'!$AU$13,'III. Finanzberichte'!$BB$13,'III. Finanzberichte'!$BI$13,'III. Finanzberichte'!$BP$13,'III. Finanzberichte'!$BW$13,'III. Finanzberichte'!$CD$13,'III. Finanzberichte'!$CK$13,'III. Finanzberichte'!$CR$13,'III. Finanzberichte'!$CY$13,'III. Finanzberichte'!$DF$13,'III. Finanzberichte'!$DM$13,'III. Finanzberichte'!$DT$13),2),0)</f>
+      </c>
+      <c r="D100" s="240" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
+      </c>
+      <c r="E100" s="200" t="str">
+        <f>=ROUND(IFERROR($C$100-$D$100,0),2)</f>
+      </c>
+      <c r="F100" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$100/$D$100)-1,0),4)</f>
+      </c>
+      <c r="G100" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$13,'III. Finanzberichte'!$M$13,'III. Finanzberichte'!$T$13,'III. Finanzberichte'!$AA$13,'III. Finanzberichte'!$AH$13,'III. Finanzberichte'!$AO$13,'III. Finanzberichte'!$AV$13,'III. Finanzberichte'!$BC$13,'III. Finanzberichte'!$BJ$13,'III. Finanzberichte'!$BQ$13,'III. Finanzberichte'!$BX$13,'III. Finanzberichte'!$CE$13,'III. Finanzberichte'!$CL$13,'III. Finanzberichte'!$CS$13,'III. Finanzberichte'!$CZ$13,'III. Finanzberichte'!$DG$13,'III. Finanzberichte'!$DN$13,'III. Finanzberichte'!$DU$13),2),0)</f>
+      </c>
+      <c r="H100" s="217" t="str">
+        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
+      </c>
+      <c r="I100" s="181" t="str">
+        <f>=ROUND(IFERROR($G$100-$H$100,0),2)</f>
+      </c>
+      <c r="J100" s="291" t="str">
+        <f>=ROUND(IFERROR(($G$100/$H$100)-1,0),4)</f>
+      </c>
+      <c r="L100" s="339" t="s">
+        <v>285</v>
+      </c>
+      <c r="M100" s="329" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$27,'III. Finanzberichte'!$J$27,'III. Finanzberichte'!$Q$27,'III. Finanzberichte'!$X$27,'III. Finanzberichte'!$AE$27,'III. Finanzberichte'!$AL$27,'III. Finanzberichte'!$AS$27,'III. Finanzberichte'!$AZ$27,'III. Finanzberichte'!$BG$27,'III. Finanzberichte'!$BN$27,'III. Finanzberichte'!$BU$27,'III. Finanzberichte'!$CB$27,'III. Finanzberichte'!$CI$27,'III. Finanzberichte'!$CP$27,'III. Finanzberichte'!$CW$27,'III. Finanzberichte'!$DD$27,'III. Finanzberichte'!$DK$27,'III. Finanzberichte'!$DR$27),"")</f>
+      </c>
+      <c r="N100" s="330" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$27,'III. Finanzberichte'!$K$27,'III. Finanzberichte'!$R$27,'III. Finanzberichte'!$Y$27,'III. Finanzberichte'!$AF$27,'III. Finanzberichte'!$AM$27,'III. Finanzberichte'!$AT$27,'III. Finanzberichte'!$BA$27,'III. Finanzberichte'!$BH$27,'III. Finanzberichte'!$BO$27,'III. Finanzberichte'!$BV$27,'III. Finanzberichte'!$CC$27,'III. Finanzberichte'!$CJ$27,'III. Finanzberichte'!$CQ$27,'III. Finanzberichte'!$CX$27,'III. Finanzberichte'!$DE$27,'III. Finanzberichte'!$DL$27,'III. Finanzberichte'!$DS$27),"")</f>
+      </c>
+      <c r="O100" s="329" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$27,'III. Finanzberichte'!$L$27,'III. Finanzberichte'!$S$27,'III. Finanzberichte'!$Z$27,'III. Finanzberichte'!$AG$27,'III. Finanzberichte'!$AN$27,'III. Finanzberichte'!$AU$27,'III. Finanzberichte'!$BB$27,'III. Finanzberichte'!$BI$27,'III. Finanzberichte'!$BP$27,'III. Finanzberichte'!$BW$27,'III. Finanzberichte'!$CD$27,'III. Finanzberichte'!$CK$27,'III. Finanzberichte'!$CR$27,'III. Finanzberichte'!$CY$27,'III. Finanzberichte'!$DF$27,'III. Finanzberichte'!$DM$27,'III. Finanzberichte'!$DT$27),"")</f>
+      </c>
+      <c r="P100" s="340" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$27,'III. Finanzberichte'!$M$27,'III. Finanzberichte'!$T$27,'III. Finanzberichte'!$AA$27,'III. Finanzberichte'!$AH$27,'III. Finanzberichte'!$AO$27,'III. Finanzberichte'!$AV$27,'III. Finanzberichte'!$BC$27,'III. Finanzberichte'!$BJ$27,'III. Finanzberichte'!$BQ$27,'III. Finanzberichte'!$BX$27,'III. Finanzberichte'!$CE$27,'III. Finanzberichte'!$CL$27,'III. Finanzberichte'!$CS$27,'III. Finanzberichte'!$CZ$27,'III. Finanzberichte'!$DG$27,'III. Finanzberichte'!$DN$27,'III. Finanzberichte'!$DU$27),"")</f>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="266" t="s">
+        <v>199</v>
+      </c>
+      <c r="C101" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$14,'III. Finanzberichte'!$L$14,'III. Finanzberichte'!$S$14,'III. Finanzberichte'!$Z$14,'III. Finanzberichte'!$AG$14,'III. Finanzberichte'!$AN$14,'III. Finanzberichte'!$AU$14,'III. Finanzberichte'!$BB$14,'III. Finanzberichte'!$BI$14,'III. Finanzberichte'!$BP$14,'III. Finanzberichte'!$BW$14,'III. Finanzberichte'!$CD$14,'III. Finanzberichte'!$CK$14,'III. Finanzberichte'!$CR$14,'III. Finanzberichte'!$CY$14,'III. Finanzberichte'!$DF$14,'III. Finanzberichte'!$DM$14,'III. Finanzberichte'!$DT$14),2),0)</f>
+      </c>
+      <c r="D101" s="240" t="str">
+        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
+      </c>
+      <c r="E101" s="200" t="str">
+        <f>=ROUND(IFERROR($C$101-$D$101,0),2)</f>
+      </c>
+      <c r="F101" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$101/$D$101)-1,0),4)</f>
+      </c>
+      <c r="G101" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$14,'III. Finanzberichte'!$M$14,'III. Finanzberichte'!$T$14,'III. Finanzberichte'!$AA$14,'III. Finanzberichte'!$AH$14,'III. Finanzberichte'!$AO$14,'III. Finanzberichte'!$AV$14,'III. Finanzberichte'!$BC$14,'III. Finanzberichte'!$BJ$14,'III. Finanzberichte'!$BQ$14,'III. Finanzberichte'!$BX$14,'III. Finanzberichte'!$CE$14,'III. Finanzberichte'!$CL$14,'III. Finanzberichte'!$CS$14,'III. Finanzberichte'!$CZ$14,'III. Finanzberichte'!$DG$14,'III. Finanzberichte'!$DN$14,'III. Finanzberichte'!$DU$14),2),0)</f>
+      </c>
+      <c r="H101" s="217" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
-      <c r="F83" s="230" t="s">
-        <v>330</v>
-      </c>
-      <c r="G83" s="231"/>
-      <c r="H83" s="231"/>
-      <c r="I83" s="232"/>
-    </row>
-    <row r="84">
-      <c r="B84" s="204" t="s">
-        <v>326</v>
-      </c>
-      <c r="C84" s="196"/>
-      <c r="D84" s="226" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
-      </c>
-      <c r="F84" s="233" t="s">
-        <v>331</v>
-      </c>
-      <c r="G84" s="196" t="s">
-        <v>332</v>
-      </c>
-      <c r="H84" s="196"/>
-      <c r="I84" s="234" t="str">
-        <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" s="204" t="s">
-        <v>327</v>
-      </c>
-      <c r="C85" s="196"/>
-      <c r="D85" s="226" t="str">
-        <f>=ROUND($D$83-$D$84,2)</f>
-      </c>
-      <c r="F85" s="233" t="s">
-        <v>331</v>
-      </c>
-      <c r="G85" s="196" t="s">
-        <v>333</v>
-      </c>
-      <c r="H85" s="196"/>
-      <c r="I85" s="222" t="str">
-        <f>=IFERROR(ROUND(MAX(0,(SUM($G$94:$G$97)-$G$96)-(SUM($H$94:$H$97)-$H$96)),2),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="204" t="s">
-        <v>328</v>
-      </c>
-      <c r="C86" s="196"/>
-      <c r="D86" s="226" t="str">
-        <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
-      </c>
-      <c r="F86" s="47"/>
-      <c r="G86" s="218" t="s">
-        <v>335</v>
-      </c>
-      <c r="H86" s="218"/>
-      <c r="I86" s="235" t="str">
-        <f>=ROUND(IF($F$84="Abzug",MAX(0,$I$84),0)+IF($F$85="Abzug",MAX(0,$I$85),0),2)</f>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="227" t="s">
-        <v>329</v>
-      </c>
-      <c r="C87" s="228"/>
-      <c r="D87" s="229" t="str">
-        <f>=ROUND($D$85-$D$86,2)</f>
-      </c>
-      <c r="F87" s="236"/>
-      <c r="G87" s="228" t="s">
-        <v>336</v>
-      </c>
-      <c r="H87" s="228"/>
-      <c r="I87" s="229" t="str">
-        <f>=ROUND($D$87-$I$86,2)</f>
-      </c>
-    </row>
-    <row r="91" ht="22" customHeight="true">
-      <c r="B91" s="18" t="s">
-        <v>370</v>
-      </c>
-      <c r="C91" s="18"/>
-      <c r="D91" s="18"/>
-      <c r="E91" s="18"/>
-      <c r="F91" s="18"/>
-      <c r="G91" s="18"/>
-      <c r="H91" s="18"/>
-      <c r="I91" s="18"/>
-      <c r="J91" s="18"/>
-    </row>
-    <row r="93" ht="28" customHeight="true">
-      <c r="B93" s="261" t="s">
-        <v>354</v>
-      </c>
-      <c r="C93" s="262" t="s">
-        <v>371</v>
-      </c>
-      <c r="D93" s="262" t="s">
+      <c r="I101" s="181" t="str">
+        <f>=ROUND(IFERROR($G$101-$H$101,0),2)</f>
+      </c>
+      <c r="J101" s="292" t="str">
+        <f>=ROUND(IFERROR(($G$101/$H$101)-1,0),4)</f>
+      </c>
+      <c r="L101" s="47"/>
+      <c r="P101" s="48"/>
+    </row>
+    <row r="102">
+      <c r="B102" s="266" t="s">
+        <v>278</v>
+      </c>
+      <c r="C102" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$15,'III. Finanzberichte'!$L$15,'III. Finanzberichte'!$S$15,'III. Finanzberichte'!$Z$15,'III. Finanzberichte'!$AG$15,'III. Finanzberichte'!$AN$15,'III. Finanzberichte'!$AU$15,'III. Finanzberichte'!$BB$15,'III. Finanzberichte'!$BI$15,'III. Finanzberichte'!$BP$15,'III. Finanzberichte'!$BW$15,'III. Finanzberichte'!$CD$15,'III. Finanzberichte'!$CK$15,'III. Finanzberichte'!$CR$15,'III. Finanzberichte'!$CY$15,'III. Finanzberichte'!$DF$15,'III. Finanzberichte'!$DM$15,'III. Finanzberichte'!$DT$15),2),0)</f>
+      </c>
+      <c r="D102" s="240" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
+      </c>
+      <c r="E102" s="200" t="str">
+        <f>=ROUND(IFERROR($C$102-$D$102,0),2)</f>
+      </c>
+      <c r="F102" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$102/$D$102)-1,0),4)</f>
+      </c>
+      <c r="G102" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$15,'III. Finanzberichte'!$M$15,'III. Finanzberichte'!$T$15,'III. Finanzberichte'!$AA$15,'III. Finanzberichte'!$AH$15,'III. Finanzberichte'!$AO$15,'III. Finanzberichte'!$AV$15,'III. Finanzberichte'!$BC$15,'III. Finanzberichte'!$BJ$15,'III. Finanzberichte'!$BQ$15,'III. Finanzberichte'!$BX$15,'III. Finanzberichte'!$CE$15,'III. Finanzberichte'!$CL$15,'III. Finanzberichte'!$CS$15,'III. Finanzberichte'!$CZ$15,'III. Finanzberichte'!$DG$15,'III. Finanzberichte'!$DN$15,'III. Finanzberichte'!$DU$15),2),0)</f>
+      </c>
+      <c r="H102" s="217" t="str">
+        <f>=IFERROR(ROUND(0,2),0)</f>
+      </c>
+      <c r="I102" s="181" t="str">
+        <f>=ROUND(IFERROR($G$102-$H$102,0),2)</f>
+      </c>
+      <c r="J102" s="293" t="str">
+        <f>=ROUND(IFERROR(($G$102/$H$102)-1,0),4)</f>
+      </c>
+      <c r="L102" s="341" t="s">
+        <v>286</v>
+      </c>
+      <c r="M102" s="342" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$C$29,'III. Finanzberichte'!$J$29,'III. Finanzberichte'!$Q$29,'III. Finanzberichte'!$X$29,'III. Finanzberichte'!$AE$29,'III. Finanzberichte'!$AL$29,'III. Finanzberichte'!$AS$29,'III. Finanzberichte'!$AZ$29,'III. Finanzberichte'!$BG$29,'III. Finanzberichte'!$BN$29,'III. Finanzberichte'!$BU$29,'III. Finanzberichte'!$CB$29,'III. Finanzberichte'!$CI$29,'III. Finanzberichte'!$CP$29,'III. Finanzberichte'!$CW$29,'III. Finanzberichte'!$DD$29,'III. Finanzberichte'!$DK$29,'III. Finanzberichte'!$DR$29),"")</f>
+      </c>
+      <c r="N102" s="343" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$D$29,'III. Finanzberichte'!$K$29,'III. Finanzberichte'!$R$29,'III. Finanzberichte'!$Y$29,'III. Finanzberichte'!$AF$29,'III. Finanzberichte'!$AM$29,'III. Finanzberichte'!$AT$29,'III. Finanzberichte'!$BA$29,'III. Finanzberichte'!$BH$29,'III. Finanzberichte'!$BO$29,'III. Finanzberichte'!$BV$29,'III. Finanzberichte'!$CC$29,'III. Finanzberichte'!$CJ$29,'III. Finanzberichte'!$CQ$29,'III. Finanzberichte'!$CX$29,'III. Finanzberichte'!$DE$29,'III. Finanzberichte'!$DL$29,'III. Finanzberichte'!$DS$29),"")</f>
+      </c>
+      <c r="O102" s="342" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$E$29,'III. Finanzberichte'!$L$29,'III. Finanzberichte'!$S$29,'III. Finanzberichte'!$Z$29,'III. Finanzberichte'!$AG$29,'III. Finanzberichte'!$AN$29,'III. Finanzberichte'!$AU$29,'III. Finanzberichte'!$BB$29,'III. Finanzberichte'!$BI$29,'III. Finanzberichte'!$BP$29,'III. Finanzberichte'!$BW$29,'III. Finanzberichte'!$CD$29,'III. Finanzberichte'!$CK$29,'III. Finanzberichte'!$CR$29,'III. Finanzberichte'!$CY$29,'III. Finanzberichte'!$DF$29,'III. Finanzberichte'!$DM$29,'III. Finanzberichte'!$DT$29),"")</f>
+      </c>
+      <c r="P102" s="344" t="str">
+        <f>=IFERROR(CHOOSE(F82,'III. Finanzberichte'!$F$29,'III. Finanzberichte'!$M$29,'III. Finanzberichte'!$T$29,'III. Finanzberichte'!$AA$29,'III. Finanzberichte'!$AH$29,'III. Finanzberichte'!$AO$29,'III. Finanzberichte'!$AV$29,'III. Finanzberichte'!$BC$29,'III. Finanzberichte'!$BJ$29,'III. Finanzberichte'!$BQ$29,'III. Finanzberichte'!$BX$29,'III. Finanzberichte'!$CE$29,'III. Finanzberichte'!$CL$29,'III. Finanzberichte'!$CS$29,'III. Finanzberichte'!$CZ$29,'III. Finanzberichte'!$DG$29,'III. Finanzberichte'!$DN$29,'III. Finanzberichte'!$DU$29),"")</f>
+      </c>
+    </row>
+    <row r="103" ht="20" customHeight="true">
+      <c r="B103" s="271" t="s">
+        <v>266</v>
+      </c>
+      <c r="C103" s="272" t="str">
+        <f>=ROUND(SUM($C$99:$C$102),2)</f>
+      </c>
+      <c r="D103" s="272" t="str">
+        <f>=ROUND(SUM($D$99:$D$102),2)</f>
+      </c>
+      <c r="E103" s="272" t="str">
+        <f>=ROUND(SUM($E$99:$E$102),2)</f>
+      </c>
+      <c r="F103" s="294" t="str">
+        <f>=ROUND(IFERROR(($C$103/$D$103)-1,0),4)</f>
+      </c>
+      <c r="G103" s="274" t="str">
+        <f>=ROUND(SUM($G$99:$G$102),2)</f>
+      </c>
+      <c r="H103" s="274" t="str">
+        <f>=ROUND(SUM($H$99:$H$102),2)</f>
+      </c>
+      <c r="I103" s="274" t="str">
+        <f>=ROUND(SUM($I$99:$I$102),2)</f>
+      </c>
+      <c r="J103" s="295" t="str">
+        <f>=ROUND(IFERROR(($G$103/$H$103)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="true">
+      <c r="B105" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="C105" s="18"/>
+      <c r="D105" s="18"/>
+      <c r="E105" s="18"/>
+      <c r="F105" s="18"/>
+      <c r="G105" s="18"/>
+      <c r="H105" s="18"/>
+      <c r="I105" s="18"/>
+      <c r="J105" s="18"/>
+    </row>
+    <row r="107" ht="28" customHeight="true">
+      <c r="B107" s="263" t="s">
         <v>356</v>
       </c>
-      <c r="E93" s="262" t="s">
-        <v>357</v>
-      </c>
-      <c r="F93" s="262" t="s">
+      <c r="C107" s="264" t="s">
+        <v>373</v>
+      </c>
+      <c r="D107" s="264" t="s">
         <v>358</v>
       </c>
-      <c r="G93" s="262" t="s">
-        <v>372</v>
-      </c>
-      <c r="H93" s="262" t="s">
+      <c r="E107" s="264" t="s">
+        <v>359</v>
+      </c>
+      <c r="F107" s="264" t="s">
         <v>360</v>
       </c>
-      <c r="I93" s="262" t="s">
-        <v>361</v>
-      </c>
-      <c r="J93" s="263" t="s">
+      <c r="G107" s="264" t="s">
+        <v>374</v>
+      </c>
+      <c r="H107" s="264" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="94">
-      <c r="B94" s="264" t="s">
-        <v>194</v>
-      </c>
-      <c r="C94" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$12,'III. Finanzberichte'!$L$12,'III. Finanzberichte'!$S$12,'III. Finanzberichte'!$Z$12,'III. Finanzberichte'!$AG$12,'III. Finanzberichte'!$AN$12,'III. Finanzberichte'!$AU$12,'III. Finanzberichte'!$BB$12,'III. Finanzberichte'!$BI$12,'III. Finanzberichte'!$BP$12,'III. Finanzberichte'!$BW$12,'III. Finanzberichte'!$CD$12,'III. Finanzberichte'!$CK$12,'III. Finanzberichte'!$CR$12,'III. Finanzberichte'!$CY$12,'III. Finanzberichte'!$DF$12,'III. Finanzberichte'!$DM$12,'III. Finanzberichte'!$DT$12),2),0)</f>
-      </c>
-      <c r="D94" s="239" t="str">
-        <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
-      </c>
-      <c r="E94" s="200" t="str">
-        <f>=ROUND(IFERROR($C$94-$D$94,0),2)</f>
-      </c>
-      <c r="F94" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$94/$D$94)-1,0),4)</f>
-      </c>
-      <c r="G94" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$12,'III. Finanzberichte'!$M$12,'III. Finanzberichte'!$T$12,'III. Finanzberichte'!$AA$12,'III. Finanzberichte'!$AH$12,'III. Finanzberichte'!$AO$12,'III. Finanzberichte'!$AV$12,'III. Finanzberichte'!$BC$12,'III. Finanzberichte'!$BJ$12,'III. Finanzberichte'!$BQ$12,'III. Finanzberichte'!$BX$12,'III. Finanzberichte'!$CE$12,'III. Finanzberichte'!$CL$12,'III. Finanzberichte'!$CS$12,'III. Finanzberichte'!$CZ$12,'III. Finanzberichte'!$DG$12,'III. Finanzberichte'!$DN$12,'III. Finanzberichte'!$DU$12),2),0)</f>
-      </c>
-      <c r="H94" s="217" t="str">
-        <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
-      </c>
-      <c r="I94" s="181" t="str">
-        <f>=ROUND(IFERROR($G$94-$H$94,0),2)</f>
-      </c>
-      <c r="J94" s="287" t="str">
-        <f>=ROUND(IFERROR(($G$94/$H$94)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="95">
-      <c r="B95" s="264" t="s">
-        <v>277</v>
-      </c>
-      <c r="C95" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$13,'III. Finanzberichte'!$L$13,'III. Finanzberichte'!$S$13,'III. Finanzberichte'!$Z$13,'III. Finanzberichte'!$AG$13,'III. Finanzberichte'!$AN$13,'III. Finanzberichte'!$AU$13,'III. Finanzberichte'!$BB$13,'III. Finanzberichte'!$BI$13,'III. Finanzberichte'!$BP$13,'III. Finanzberichte'!$BW$13,'III. Finanzberichte'!$CD$13,'III. Finanzberichte'!$CK$13,'III. Finanzberichte'!$CR$13,'III. Finanzberichte'!$CY$13,'III. Finanzberichte'!$DF$13,'III. Finanzberichte'!$DM$13,'III. Finanzberichte'!$DT$13),2),0)</f>
-      </c>
-      <c r="D95" s="239" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
-      </c>
-      <c r="E95" s="200" t="str">
-        <f>=ROUND(IFERROR($C$95-$D$95,0),2)</f>
-      </c>
-      <c r="F95" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$95/$D$95)-1,0),4)</f>
-      </c>
-      <c r="G95" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$13,'III. Finanzberichte'!$M$13,'III. Finanzberichte'!$T$13,'III. Finanzberichte'!$AA$13,'III. Finanzberichte'!$AH$13,'III. Finanzberichte'!$AO$13,'III. Finanzberichte'!$AV$13,'III. Finanzberichte'!$BC$13,'III. Finanzberichte'!$BJ$13,'III. Finanzberichte'!$BQ$13,'III. Finanzberichte'!$BX$13,'III. Finanzberichte'!$CE$13,'III. Finanzberichte'!$CL$13,'III. Finanzberichte'!$CS$13,'III. Finanzberichte'!$CZ$13,'III. Finanzberichte'!$DG$13,'III. Finanzberichte'!$DN$13,'III. Finanzberichte'!$DU$13),2),0)</f>
-      </c>
-      <c r="H95" s="217" t="str">
-        <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
-      </c>
-      <c r="I95" s="181" t="str">
-        <f>=ROUND(IFERROR($G$95-$H$95,0),2)</f>
-      </c>
-      <c r="J95" s="288" t="str">
-        <f>=ROUND(IFERROR(($G$95/$H$95)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="96">
-      <c r="B96" s="264" t="s">
-        <v>199</v>
-      </c>
-      <c r="C96" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$14,'III. Finanzberichte'!$L$14,'III. Finanzberichte'!$S$14,'III. Finanzberichte'!$Z$14,'III. Finanzberichte'!$AG$14,'III. Finanzberichte'!$AN$14,'III. Finanzberichte'!$AU$14,'III. Finanzberichte'!$BB$14,'III. Finanzberichte'!$BI$14,'III. Finanzberichte'!$BP$14,'III. Finanzberichte'!$BW$14,'III. Finanzberichte'!$CD$14,'III. Finanzberichte'!$CK$14,'III. Finanzberichte'!$CR$14,'III. Finanzberichte'!$CY$14,'III. Finanzberichte'!$DF$14,'III. Finanzberichte'!$DM$14,'III. Finanzberichte'!$DT$14),2),0)</f>
-      </c>
-      <c r="D96" s="239" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
-      </c>
-      <c r="E96" s="200" t="str">
-        <f>=ROUND(IFERROR($C$96-$D$96,0),2)</f>
-      </c>
-      <c r="F96" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$96/$D$96)-1,0),4)</f>
-      </c>
-      <c r="G96" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$14,'III. Finanzberichte'!$M$14,'III. Finanzberichte'!$T$14,'III. Finanzberichte'!$AA$14,'III. Finanzberichte'!$AH$14,'III. Finanzberichte'!$AO$14,'III. Finanzberichte'!$AV$14,'III. Finanzberichte'!$BC$14,'III. Finanzberichte'!$BJ$14,'III. Finanzberichte'!$BQ$14,'III. Finanzberichte'!$BX$14,'III. Finanzberichte'!$CE$14,'III. Finanzberichte'!$CL$14,'III. Finanzberichte'!$CS$14,'III. Finanzberichte'!$CZ$14,'III. Finanzberichte'!$DG$14,'III. Finanzberichte'!$DN$14,'III. Finanzberichte'!$DU$14),2),0)</f>
-      </c>
-      <c r="H96" s="217" t="str">
-        <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
-      </c>
-      <c r="I96" s="181" t="str">
-        <f>=ROUND(IFERROR($G$96-$H$96,0),2)</f>
-      </c>
-      <c r="J96" s="289" t="str">
-        <f>=ROUND(IFERROR(($G$96/$H$96)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="97">
-      <c r="B97" s="264" t="s">
-        <v>278</v>
-      </c>
-      <c r="C97" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$15,'III. Finanzberichte'!$L$15,'III. Finanzberichte'!$S$15,'III. Finanzberichte'!$Z$15,'III. Finanzberichte'!$AG$15,'III. Finanzberichte'!$AN$15,'III. Finanzberichte'!$AU$15,'III. Finanzberichte'!$BB$15,'III. Finanzberichte'!$BI$15,'III. Finanzberichte'!$BP$15,'III. Finanzberichte'!$BW$15,'III. Finanzberichte'!$CD$15,'III. Finanzberichte'!$CK$15,'III. Finanzberichte'!$CR$15,'III. Finanzberichte'!$CY$15,'III. Finanzberichte'!$DF$15,'III. Finanzberichte'!$DM$15,'III. Finanzberichte'!$DT$15),2),0)</f>
-      </c>
-      <c r="D97" s="239" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
-      </c>
-      <c r="E97" s="200" t="str">
-        <f>=ROUND(IFERROR($C$97-$D$97,0),2)</f>
-      </c>
-      <c r="F97" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$97/$D$97)-1,0),4)</f>
-      </c>
-      <c r="G97" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$15,'III. Finanzberichte'!$M$15,'III. Finanzberichte'!$T$15,'III. Finanzberichte'!$AA$15,'III. Finanzberichte'!$AH$15,'III. Finanzberichte'!$AO$15,'III. Finanzberichte'!$AV$15,'III. Finanzberichte'!$BC$15,'III. Finanzberichte'!$BJ$15,'III. Finanzberichte'!$BQ$15,'III. Finanzberichte'!$BX$15,'III. Finanzberichte'!$CE$15,'III. Finanzberichte'!$CL$15,'III. Finanzberichte'!$CS$15,'III. Finanzberichte'!$CZ$15,'III. Finanzberichte'!$DG$15,'III. Finanzberichte'!$DN$15,'III. Finanzberichte'!$DU$15),2),0)</f>
-      </c>
-      <c r="H97" s="217" t="str">
-        <f>=IFERROR(ROUND(0,2),0)</f>
-      </c>
-      <c r="I97" s="181" t="str">
-        <f>=ROUND(IFERROR($G$97-$H$97,0),2)</f>
-      </c>
-      <c r="J97" s="290" t="str">
-        <f>=ROUND(IFERROR(($G$97/$H$97)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="98" ht="20" customHeight="true">
-      <c r="B98" s="269" t="s">
-        <v>266</v>
-      </c>
-      <c r="C98" s="270" t="str">
-        <f>=ROUND(SUM($C$94:$C$97),2)</f>
-      </c>
-      <c r="D98" s="270" t="str">
-        <f>=ROUND(SUM($D$94:$D$97),2)</f>
-      </c>
-      <c r="E98" s="270" t="str">
-        <f>=ROUND(SUM($E$94:$E$97),2)</f>
-      </c>
-      <c r="F98" s="291" t="str">
-        <f>=ROUND(IFERROR(($C$98/$D$98)-1,0),4)</f>
-      </c>
-      <c r="G98" s="272" t="str">
-        <f>=ROUND(SUM($G$94:$G$97),2)</f>
-      </c>
-      <c r="H98" s="272" t="str">
-        <f>=ROUND(SUM($H$94:$H$97),2)</f>
-      </c>
-      <c r="I98" s="272" t="str">
-        <f>=ROUND(SUM($I$94:$I$97),2)</f>
-      </c>
-      <c r="J98" s="292" t="str">
-        <f>=ROUND(IFERROR(($G$98/$H$98)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="100" ht="22" customHeight="true">
-      <c r="B100" s="18" t="s">
-        <v>373</v>
-      </c>
-      <c r="C100" s="18"/>
-      <c r="D100" s="18"/>
-      <c r="E100" s="18"/>
-      <c r="F100" s="18"/>
-      <c r="G100" s="18"/>
-      <c r="H100" s="18"/>
-      <c r="I100" s="18"/>
-      <c r="J100" s="18"/>
-    </row>
-    <row r="102" ht="28" customHeight="true">
-      <c r="B102" s="261" t="s">
-        <v>354</v>
-      </c>
-      <c r="C102" s="262" t="s">
-        <v>371</v>
-      </c>
-      <c r="D102" s="262" t="s">
-        <v>356</v>
-      </c>
-      <c r="E102" s="262" t="s">
-        <v>357</v>
-      </c>
-      <c r="F102" s="262" t="s">
-        <v>358</v>
-      </c>
-      <c r="G102" s="262" t="s">
-        <v>372</v>
-      </c>
-      <c r="H102" s="262" t="s">
-        <v>360</v>
-      </c>
-      <c r="I102" s="262" t="s">
-        <v>361</v>
-      </c>
-      <c r="J102" s="263" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="B103" s="264" t="s">
+      <c r="I107" s="264" t="s">
+        <v>363</v>
+      </c>
+      <c r="J107" s="265" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="266" t="s">
         <v>205</v>
       </c>
-      <c r="C103" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$19,'III. Finanzberichte'!$L$19,'III. Finanzberichte'!$S$19,'III. Finanzberichte'!$Z$19,'III. Finanzberichte'!$AG$19,'III. Finanzberichte'!$AN$19,'III. Finanzberichte'!$AU$19,'III. Finanzberichte'!$BB$19,'III. Finanzberichte'!$BI$19,'III. Finanzberichte'!$BP$19,'III. Finanzberichte'!$BW$19,'III. Finanzberichte'!$CD$19,'III. Finanzberichte'!$CK$19,'III. Finanzberichte'!$CR$19,'III. Finanzberichte'!$CY$19,'III. Finanzberichte'!$DF$19,'III. Finanzberichte'!$DM$19,'III. Finanzberichte'!$DT$19),2),0)</f>
-      </c>
-      <c r="D103" s="239" t="str">
+      <c r="C108" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$19,'III. Finanzberichte'!$L$19,'III. Finanzberichte'!$S$19,'III. Finanzberichte'!$Z$19,'III. Finanzberichte'!$AG$19,'III. Finanzberichte'!$AN$19,'III. Finanzberichte'!$AU$19,'III. Finanzberichte'!$BB$19,'III. Finanzberichte'!$BI$19,'III. Finanzberichte'!$BP$19,'III. Finanzberichte'!$BW$19,'III. Finanzberichte'!$CD$19,'III. Finanzberichte'!$CK$19,'III. Finanzberichte'!$CR$19,'III. Finanzberichte'!$CY$19,'III. Finanzberichte'!$DF$19,'III. Finanzberichte'!$DM$19,'III. Finanzberichte'!$DT$19),2),0)</f>
+      </c>
+      <c r="D108" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
-      </c>
-      <c r="E103" s="200" t="str">
-        <f>=ROUND(IFERROR($C$103-$D$103,0),2)</f>
-      </c>
-      <c r="F103" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$103/$D$103)-1,0),4)</f>
-      </c>
-      <c r="G103" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$19,'III. Finanzberichte'!$M$19,'III. Finanzberichte'!$T$19,'III. Finanzberichte'!$AA$19,'III. Finanzberichte'!$AH$19,'III. Finanzberichte'!$AO$19,'III. Finanzberichte'!$AV$19,'III. Finanzberichte'!$BC$19,'III. Finanzberichte'!$BJ$19,'III. Finanzberichte'!$BQ$19,'III. Finanzberichte'!$BX$19,'III. Finanzberichte'!$CE$19,'III. Finanzberichte'!$CL$19,'III. Finanzberichte'!$CS$19,'III. Finanzberichte'!$CZ$19,'III. Finanzberichte'!$DG$19,'III. Finanzberichte'!$DN$19,'III. Finanzberichte'!$DU$19),2),0)</f>
-      </c>
-      <c r="H103" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
-      </c>
-      <c r="I103" s="181" t="str">
-        <f>=ROUND(IFERROR($G$103-$H$103,0),2)</f>
-      </c>
-      <c r="J103" s="293" t="str">
-        <f>=ROUND(IFERROR(($G$103/$H$103)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="104">
-      <c r="B104" s="264" t="s">
-        <v>206</v>
-      </c>
-      <c r="C104" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$20,'III. Finanzberichte'!$L$20,'III. Finanzberichte'!$S$20,'III. Finanzberichte'!$Z$20,'III. Finanzberichte'!$AG$20,'III. Finanzberichte'!$AN$20,'III. Finanzberichte'!$AU$20,'III. Finanzberichte'!$BB$20,'III. Finanzberichte'!$BI$20,'III. Finanzberichte'!$BP$20,'III. Finanzberichte'!$BW$20,'III. Finanzberichte'!$CD$20,'III. Finanzberichte'!$CK$20,'III. Finanzberichte'!$CR$20,'III. Finanzberichte'!$CY$20,'III. Finanzberichte'!$DF$20,'III. Finanzberichte'!$DM$20,'III. Finanzberichte'!$DT$20),2),0)</f>
-      </c>
-      <c r="D104" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
-      </c>
-      <c r="E104" s="200" t="str">
-        <f>=ROUND(IFERROR($C$104-$D$104,0),2)</f>
-      </c>
-      <c r="F104" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$104/$D$104)-1,0),4)</f>
-      </c>
-      <c r="G104" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$20,'III. Finanzberichte'!$M$20,'III. Finanzberichte'!$T$20,'III. Finanzberichte'!$AA$20,'III. Finanzberichte'!$AH$20,'III. Finanzberichte'!$AO$20,'III. Finanzberichte'!$AV$20,'III. Finanzberichte'!$BC$20,'III. Finanzberichte'!$BJ$20,'III. Finanzberichte'!$BQ$20,'III. Finanzberichte'!$BX$20,'III. Finanzberichte'!$CE$20,'III. Finanzberichte'!$CL$20,'III. Finanzberichte'!$CS$20,'III. Finanzberichte'!$CZ$20,'III. Finanzberichte'!$DG$20,'III. Finanzberichte'!$DN$20,'III. Finanzberichte'!$DU$20),2),0)</f>
-      </c>
-      <c r="H104" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
-      </c>
-      <c r="I104" s="181" t="str">
-        <f>=ROUND(IFERROR($G$104-$H$104,0),2)</f>
-      </c>
-      <c r="J104" s="294" t="str">
-        <f>=ROUND(IFERROR(($G$104/$H$104)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="105">
-      <c r="B105" s="264" t="s">
-        <v>207</v>
-      </c>
-      <c r="C105" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$21,'III. Finanzberichte'!$L$21,'III. Finanzberichte'!$S$21,'III. Finanzberichte'!$Z$21,'III. Finanzberichte'!$AG$21,'III. Finanzberichte'!$AN$21,'III. Finanzberichte'!$AU$21,'III. Finanzberichte'!$BB$21,'III. Finanzberichte'!$BI$21,'III. Finanzberichte'!$BP$21,'III. Finanzberichte'!$BW$21,'III. Finanzberichte'!$CD$21,'III. Finanzberichte'!$CK$21,'III. Finanzberichte'!$CR$21,'III. Finanzberichte'!$CY$21,'III. Finanzberichte'!$DF$21,'III. Finanzberichte'!$DM$21,'III. Finanzberichte'!$DT$21),2),0)</f>
-      </c>
-      <c r="D105" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
-      </c>
-      <c r="E105" s="200" t="str">
-        <f>=ROUND(IFERROR($C$105-$D$105,0),2)</f>
-      </c>
-      <c r="F105" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$105/$D$105)-1,0),4)</f>
-      </c>
-      <c r="G105" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$21,'III. Finanzberichte'!$M$21,'III. Finanzberichte'!$T$21,'III. Finanzberichte'!$AA$21,'III. Finanzberichte'!$AH$21,'III. Finanzberichte'!$AO$21,'III. Finanzberichte'!$AV$21,'III. Finanzberichte'!$BC$21,'III. Finanzberichte'!$BJ$21,'III. Finanzberichte'!$BQ$21,'III. Finanzberichte'!$BX$21,'III. Finanzberichte'!$CE$21,'III. Finanzberichte'!$CL$21,'III. Finanzberichte'!$CS$21,'III. Finanzberichte'!$CZ$21,'III. Finanzberichte'!$DG$21,'III. Finanzberichte'!$DN$21,'III. Finanzberichte'!$DU$21),2),0)</f>
-      </c>
-      <c r="H105" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
-      </c>
-      <c r="I105" s="181" t="str">
-        <f>=ROUND(IFERROR($G$105-$H$105,0),2)</f>
-      </c>
-      <c r="J105" s="295" t="str">
-        <f>=ROUND(IFERROR(($G$105/$H$105)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="106">
-      <c r="B106" s="264" t="s">
-        <v>208</v>
-      </c>
-      <c r="C106" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$22,'III. Finanzberichte'!$L$22,'III. Finanzberichte'!$S$22,'III. Finanzberichte'!$Z$22,'III. Finanzberichte'!$AG$22,'III. Finanzberichte'!$AN$22,'III. Finanzberichte'!$AU$22,'III. Finanzberichte'!$BB$22,'III. Finanzberichte'!$BI$22,'III. Finanzberichte'!$BP$22,'III. Finanzberichte'!$BW$22,'III. Finanzberichte'!$CD$22,'III. Finanzberichte'!$CK$22,'III. Finanzberichte'!$CR$22,'III. Finanzberichte'!$CY$22,'III. Finanzberichte'!$DF$22,'III. Finanzberichte'!$DM$22,'III. Finanzberichte'!$DT$22),2),0)</f>
-      </c>
-      <c r="D106" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
-      </c>
-      <c r="E106" s="200" t="str">
-        <f>=ROUND(IFERROR($C$106-$D$106,0),2)</f>
-      </c>
-      <c r="F106" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$106/$D$106)-1,0),4)</f>
-      </c>
-      <c r="G106" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$22,'III. Finanzberichte'!$M$22,'III. Finanzberichte'!$T$22,'III. Finanzberichte'!$AA$22,'III. Finanzberichte'!$AH$22,'III. Finanzberichte'!$AO$22,'III. Finanzberichte'!$AV$22,'III. Finanzberichte'!$BC$22,'III. Finanzberichte'!$BJ$22,'III. Finanzberichte'!$BQ$22,'III. Finanzberichte'!$BX$22,'III. Finanzberichte'!$CE$22,'III. Finanzberichte'!$CL$22,'III. Finanzberichte'!$CS$22,'III. Finanzberichte'!$CZ$22,'III. Finanzberichte'!$DG$22,'III. Finanzberichte'!$DN$22,'III. Finanzberichte'!$DU$22),2),0)</f>
-      </c>
-      <c r="H106" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
-      </c>
-      <c r="I106" s="181" t="str">
-        <f>=ROUND(IFERROR($G$106-$H$106,0),2)</f>
-      </c>
-      <c r="J106" s="296" t="str">
-        <f>=ROUND(IFERROR(($G$106/$H$106)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="107">
-      <c r="B107" s="264" t="s">
-        <v>209</v>
-      </c>
-      <c r="C107" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$23,'III. Finanzberichte'!$L$23,'III. Finanzberichte'!$S$23,'III. Finanzberichte'!$Z$23,'III. Finanzberichte'!$AG$23,'III. Finanzberichte'!$AN$23,'III. Finanzberichte'!$AU$23,'III. Finanzberichte'!$BB$23,'III. Finanzberichte'!$BI$23,'III. Finanzberichte'!$BP$23,'III. Finanzberichte'!$BW$23,'III. Finanzberichte'!$CD$23,'III. Finanzberichte'!$CK$23,'III. Finanzberichte'!$CR$23,'III. Finanzberichte'!$CY$23,'III. Finanzberichte'!$DF$23,'III. Finanzberichte'!$DM$23,'III. Finanzberichte'!$DT$23),2),0)</f>
-      </c>
-      <c r="D107" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
-      </c>
-      <c r="E107" s="200" t="str">
-        <f>=ROUND(IFERROR($C$107-$D$107,0),2)</f>
-      </c>
-      <c r="F107" s="256" t="str">
-        <f>=ROUND(IFERROR(($C$107/$D$107)-1,0),4)</f>
-      </c>
-      <c r="G107" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$23,'III. Finanzberichte'!$M$23,'III. Finanzberichte'!$T$23,'III. Finanzberichte'!$AA$23,'III. Finanzberichte'!$AH$23,'III. Finanzberichte'!$AO$23,'III. Finanzberichte'!$AV$23,'III. Finanzberichte'!$BC$23,'III. Finanzberichte'!$BJ$23,'III. Finanzberichte'!$BQ$23,'III. Finanzberichte'!$BX$23,'III. Finanzberichte'!$CE$23,'III. Finanzberichte'!$CL$23,'III. Finanzberichte'!$CS$23,'III. Finanzberichte'!$CZ$23,'III. Finanzberichte'!$DG$23,'III. Finanzberichte'!$DN$23,'III. Finanzberichte'!$DU$23),2),0)</f>
-      </c>
-      <c r="H107" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
-      </c>
-      <c r="I107" s="181" t="str">
-        <f>=ROUND(IFERROR($G$107-$H$107,0),2)</f>
-      </c>
-      <c r="J107" s="297" t="str">
-        <f>=ROUND(IFERROR(($G$107/$H$107)-1,0),4)</f>
-      </c>
-    </row>
-    <row r="108">
-      <c r="B108" s="264" t="s">
-        <v>210</v>
-      </c>
-      <c r="C108" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$24,'III. Finanzberichte'!$L$24,'III. Finanzberichte'!$S$24,'III. Finanzberichte'!$Z$24,'III. Finanzberichte'!$AG$24,'III. Finanzberichte'!$AN$24,'III. Finanzberichte'!$AU$24,'III. Finanzberichte'!$BB$24,'III. Finanzberichte'!$BI$24,'III. Finanzberichte'!$BP$24,'III. Finanzberichte'!$BW$24,'III. Finanzberichte'!$CD$24,'III. Finanzberichte'!$CK$24,'III. Finanzberichte'!$CR$24,'III. Finanzberichte'!$CY$24,'III. Finanzberichte'!$DF$24,'III. Finanzberichte'!$DM$24,'III. Finanzberichte'!$DT$24),2),0)</f>
-      </c>
-      <c r="D108" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
       </c>
       <c r="E108" s="200" t="str">
         <f>=ROUND(IFERROR($C$108-$D$108,0),2)</f>
       </c>
-      <c r="F108" s="256" t="str">
+      <c r="F108" s="258" t="str">
         <f>=ROUND(IFERROR(($C$108/$D$108)-1,0),4)</f>
       </c>
       <c r="G108" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$24,'III. Finanzberichte'!$M$24,'III. Finanzberichte'!$T$24,'III. Finanzberichte'!$AA$24,'III. Finanzberichte'!$AH$24,'III. Finanzberichte'!$AO$24,'III. Finanzberichte'!$AV$24,'III. Finanzberichte'!$BC$24,'III. Finanzberichte'!$BJ$24,'III. Finanzberichte'!$BQ$24,'III. Finanzberichte'!$BX$24,'III. Finanzberichte'!$CE$24,'III. Finanzberichte'!$CL$24,'III. Finanzberichte'!$CS$24,'III. Finanzberichte'!$CZ$24,'III. Finanzberichte'!$DG$24,'III. Finanzberichte'!$DN$24,'III. Finanzberichte'!$DU$24),2),0)</f>
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$19,'III. Finanzberichte'!$M$19,'III. Finanzberichte'!$T$19,'III. Finanzberichte'!$AA$19,'III. Finanzberichte'!$AH$19,'III. Finanzberichte'!$AO$19,'III. Finanzberichte'!$AV$19,'III. Finanzberichte'!$BC$19,'III. Finanzberichte'!$BJ$19,'III. Finanzberichte'!$BQ$19,'III. Finanzberichte'!$BX$19,'III. Finanzberichte'!$CE$19,'III. Finanzberichte'!$CL$19,'III. Finanzberichte'!$CS$19,'III. Finanzberichte'!$CZ$19,'III. Finanzberichte'!$DG$19,'III. Finanzberichte'!$DN$19,'III. Finanzberichte'!$DU$19),2),0)</f>
       </c>
       <c r="H108" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
       </c>
       <c r="I108" s="181" t="str">
         <f>=ROUND(IFERROR($G$108-$H$108,0),2)</f>
       </c>
-      <c r="J108" s="298" t="str">
+      <c r="J108" s="296" t="str">
         <f>=ROUND(IFERROR(($G$108/$H$108)-1,0),4)</f>
       </c>
     </row>
     <row r="109">
-      <c r="B109" s="264" t="s">
-        <v>211</v>
-      </c>
-      <c r="C109" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$25,'III. Finanzberichte'!$L$25,'III. Finanzberichte'!$S$25,'III. Finanzberichte'!$Z$25,'III. Finanzberichte'!$AG$25,'III. Finanzberichte'!$AN$25,'III. Finanzberichte'!$AU$25,'III. Finanzberichte'!$BB$25,'III. Finanzberichte'!$BI$25,'III. Finanzberichte'!$BP$25,'III. Finanzberichte'!$BW$25,'III. Finanzberichte'!$CD$25,'III. Finanzberichte'!$CK$25,'III. Finanzberichte'!$CR$25,'III. Finanzberichte'!$CY$25,'III. Finanzberichte'!$DF$25,'III. Finanzberichte'!$DM$25,'III. Finanzberichte'!$DT$25),2),0)</f>
-      </c>
-      <c r="D109" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
+      <c r="B109" s="266" t="s">
+        <v>206</v>
+      </c>
+      <c r="C109" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$20,'III. Finanzberichte'!$L$20,'III. Finanzberichte'!$S$20,'III. Finanzberichte'!$Z$20,'III. Finanzberichte'!$AG$20,'III. Finanzberichte'!$AN$20,'III. Finanzberichte'!$AU$20,'III. Finanzberichte'!$BB$20,'III. Finanzberichte'!$BI$20,'III. Finanzberichte'!$BP$20,'III. Finanzberichte'!$BW$20,'III. Finanzberichte'!$CD$20,'III. Finanzberichte'!$CK$20,'III. Finanzberichte'!$CR$20,'III. Finanzberichte'!$CY$20,'III. Finanzberichte'!$DF$20,'III. Finanzberichte'!$DM$20,'III. Finanzberichte'!$DT$20),2),0)</f>
+      </c>
+      <c r="D109" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
       </c>
       <c r="E109" s="200" t="str">
         <f>=ROUND(IFERROR($C$109-$D$109,0),2)</f>
       </c>
-      <c r="F109" s="256" t="str">
+      <c r="F109" s="258" t="str">
         <f>=ROUND(IFERROR(($C$109/$D$109)-1,0),4)</f>
       </c>
       <c r="G109" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$25,'III. Finanzberichte'!$M$25,'III. Finanzberichte'!$T$25,'III. Finanzberichte'!$AA$25,'III. Finanzberichte'!$AH$25,'III. Finanzberichte'!$AO$25,'III. Finanzberichte'!$AV$25,'III. Finanzberichte'!$BC$25,'III. Finanzberichte'!$BJ$25,'III. Finanzberichte'!$BQ$25,'III. Finanzberichte'!$BX$25,'III. Finanzberichte'!$CE$25,'III. Finanzberichte'!$CL$25,'III. Finanzberichte'!$CS$25,'III. Finanzberichte'!$CZ$25,'III. Finanzberichte'!$DG$25,'III. Finanzberichte'!$DN$25,'III. Finanzberichte'!$DU$25),2),0)</f>
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$20,'III. Finanzberichte'!$M$20,'III. Finanzberichte'!$T$20,'III. Finanzberichte'!$AA$20,'III. Finanzberichte'!$AH$20,'III. Finanzberichte'!$AO$20,'III. Finanzberichte'!$AV$20,'III. Finanzberichte'!$BC$20,'III. Finanzberichte'!$BJ$20,'III. Finanzberichte'!$BQ$20,'III. Finanzberichte'!$BX$20,'III. Finanzberichte'!$CE$20,'III. Finanzberichte'!$CL$20,'III. Finanzberichte'!$CS$20,'III. Finanzberichte'!$CZ$20,'III. Finanzberichte'!$DG$20,'III. Finanzberichte'!$DN$20,'III. Finanzberichte'!$DU$20),2),0)</f>
       </c>
       <c r="H109" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
       </c>
       <c r="I109" s="181" t="str">
         <f>=ROUND(IFERROR($G$109-$H$109,0),2)</f>
       </c>
-      <c r="J109" s="299" t="str">
+      <c r="J109" s="297" t="str">
         <f>=ROUND(IFERROR(($G$109/$H$109)-1,0),4)</f>
       </c>
     </row>
     <row r="110">
-      <c r="B110" s="264" t="s">
-        <v>212</v>
-      </c>
-      <c r="C110" s="239" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$E$26,'III. Finanzberichte'!$L$26,'III. Finanzberichte'!$S$26,'III. Finanzberichte'!$Z$26,'III. Finanzberichte'!$AG$26,'III. Finanzberichte'!$AN$26,'III. Finanzberichte'!$AU$26,'III. Finanzberichte'!$BB$26,'III. Finanzberichte'!$BI$26,'III. Finanzberichte'!$BP$26,'III. Finanzberichte'!$BW$26,'III. Finanzberichte'!$CD$26,'III. Finanzberichte'!$CK$26,'III. Finanzberichte'!$CR$26,'III. Finanzberichte'!$CY$26,'III. Finanzberichte'!$DF$26,'III. Finanzberichte'!$DM$26,'III. Finanzberichte'!$DT$26),2),0)</f>
-      </c>
-      <c r="D110" s="239" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
+      <c r="B110" s="266" t="s">
+        <v>207</v>
+      </c>
+      <c r="C110" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$21,'III. Finanzberichte'!$L$21,'III. Finanzberichte'!$S$21,'III. Finanzberichte'!$Z$21,'III. Finanzberichte'!$AG$21,'III. Finanzberichte'!$AN$21,'III. Finanzberichte'!$AU$21,'III. Finanzberichte'!$BB$21,'III. Finanzberichte'!$BI$21,'III. Finanzberichte'!$BP$21,'III. Finanzberichte'!$BW$21,'III. Finanzberichte'!$CD$21,'III. Finanzberichte'!$CK$21,'III. Finanzberichte'!$CR$21,'III. Finanzberichte'!$CY$21,'III. Finanzberichte'!$DF$21,'III. Finanzberichte'!$DM$21,'III. Finanzberichte'!$DT$21),2),0)</f>
+      </c>
+      <c r="D110" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
       </c>
       <c r="E110" s="200" t="str">
         <f>=ROUND(IFERROR($C$110-$D$110,0),2)</f>
       </c>
-      <c r="F110" s="256" t="str">
+      <c r="F110" s="258" t="str">
         <f>=ROUND(IFERROR(($C$110/$D$110)-1,0),4)</f>
       </c>
       <c r="G110" s="217" t="str">
-        <f>=IFERROR(ROUND(CHOOSE(F77,'III. Finanzberichte'!$F$26,'III. Finanzberichte'!$M$26,'III. Finanzberichte'!$T$26,'III. Finanzberichte'!$AA$26,'III. Finanzberichte'!$AH$26,'III. Finanzberichte'!$AO$26,'III. Finanzberichte'!$AV$26,'III. Finanzberichte'!$BC$26,'III. Finanzberichte'!$BJ$26,'III. Finanzberichte'!$BQ$26,'III. Finanzberichte'!$BX$26,'III. Finanzberichte'!$CE$26,'III. Finanzberichte'!$CL$26,'III. Finanzberichte'!$CS$26,'III. Finanzberichte'!$CZ$26,'III. Finanzberichte'!$DG$26,'III. Finanzberichte'!$DN$26,'III. Finanzberichte'!$DU$26),2),0)</f>
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$21,'III. Finanzberichte'!$M$21,'III. Finanzberichte'!$T$21,'III. Finanzberichte'!$AA$21,'III. Finanzberichte'!$AH$21,'III. Finanzberichte'!$AO$21,'III. Finanzberichte'!$AV$21,'III. Finanzberichte'!$BC$21,'III. Finanzberichte'!$BJ$21,'III. Finanzberichte'!$BQ$21,'III. Finanzberichte'!$BX$21,'III. Finanzberichte'!$CE$21,'III. Finanzberichte'!$CL$21,'III. Finanzberichte'!$CS$21,'III. Finanzberichte'!$CZ$21,'III. Finanzberichte'!$DG$21,'III. Finanzberichte'!$DN$21,'III. Finanzberichte'!$DU$21),2),0)</f>
       </c>
       <c r="H110" s="217" t="str">
-        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+        <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
       </c>
       <c r="I110" s="181" t="str">
         <f>=ROUND(IFERROR($G$110-$H$110,0),2)</f>
       </c>
-      <c r="J110" s="300" t="str">
+      <c r="J110" s="298" t="str">
         <f>=ROUND(IFERROR(($G$110/$H$110)-1,0),4)</f>
       </c>
     </row>
-    <row r="111" ht="20" customHeight="true">
-      <c r="B111" s="269" t="s">
+    <row r="111">
+      <c r="B111" s="266" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$22,'III. Finanzberichte'!$L$22,'III. Finanzberichte'!$S$22,'III. Finanzberichte'!$Z$22,'III. Finanzberichte'!$AG$22,'III. Finanzberichte'!$AN$22,'III. Finanzberichte'!$AU$22,'III. Finanzberichte'!$BB$22,'III. Finanzberichte'!$BI$22,'III. Finanzberichte'!$BP$22,'III. Finanzberichte'!$BW$22,'III. Finanzberichte'!$CD$22,'III. Finanzberichte'!$CK$22,'III. Finanzberichte'!$CR$22,'III. Finanzberichte'!$CY$22,'III. Finanzberichte'!$DF$22,'III. Finanzberichte'!$DM$22,'III. Finanzberichte'!$DT$22),2),0)</f>
+      </c>
+      <c r="D111" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
+      </c>
+      <c r="E111" s="200" t="str">
+        <f>=ROUND(IFERROR($C$111-$D$111,0),2)</f>
+      </c>
+      <c r="F111" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$111/$D$111)-1,0),4)</f>
+      </c>
+      <c r="G111" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$22,'III. Finanzberichte'!$M$22,'III. Finanzberichte'!$T$22,'III. Finanzberichte'!$AA$22,'III. Finanzberichte'!$AH$22,'III. Finanzberichte'!$AO$22,'III. Finanzberichte'!$AV$22,'III. Finanzberichte'!$BC$22,'III. Finanzberichte'!$BJ$22,'III. Finanzberichte'!$BQ$22,'III. Finanzberichte'!$BX$22,'III. Finanzberichte'!$CE$22,'III. Finanzberichte'!$CL$22,'III. Finanzberichte'!$CS$22,'III. Finanzberichte'!$CZ$22,'III. Finanzberichte'!$DG$22,'III. Finanzberichte'!$DN$22,'III. Finanzberichte'!$DU$22),2),0)</f>
+      </c>
+      <c r="H111" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
+      </c>
+      <c r="I111" s="181" t="str">
+        <f>=ROUND(IFERROR($G$111-$H$111,0),2)</f>
+      </c>
+      <c r="J111" s="299" t="str">
+        <f>=ROUND(IFERROR(($G$111/$H$111)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="266" t="s">
+        <v>209</v>
+      </c>
+      <c r="C112" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$23,'III. Finanzberichte'!$L$23,'III. Finanzberichte'!$S$23,'III. Finanzberichte'!$Z$23,'III. Finanzberichte'!$AG$23,'III. Finanzberichte'!$AN$23,'III. Finanzberichte'!$AU$23,'III. Finanzberichte'!$BB$23,'III. Finanzberichte'!$BI$23,'III. Finanzberichte'!$BP$23,'III. Finanzberichte'!$BW$23,'III. Finanzberichte'!$CD$23,'III. Finanzberichte'!$CK$23,'III. Finanzberichte'!$CR$23,'III. Finanzberichte'!$CY$23,'III. Finanzberichte'!$DF$23,'III. Finanzberichte'!$DM$23,'III. Finanzberichte'!$DT$23),2),0)</f>
+      </c>
+      <c r="D112" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
+      </c>
+      <c r="E112" s="200" t="str">
+        <f>=ROUND(IFERROR($C$112-$D$112,0),2)</f>
+      </c>
+      <c r="F112" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$112/$D$112)-1,0),4)</f>
+      </c>
+      <c r="G112" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$23,'III. Finanzberichte'!$M$23,'III. Finanzberichte'!$T$23,'III. Finanzberichte'!$AA$23,'III. Finanzberichte'!$AH$23,'III. Finanzberichte'!$AO$23,'III. Finanzberichte'!$AV$23,'III. Finanzberichte'!$BC$23,'III. Finanzberichte'!$BJ$23,'III. Finanzberichte'!$BQ$23,'III. Finanzberichte'!$BX$23,'III. Finanzberichte'!$CE$23,'III. Finanzberichte'!$CL$23,'III. Finanzberichte'!$CS$23,'III. Finanzberichte'!$CZ$23,'III. Finanzberichte'!$DG$23,'III. Finanzberichte'!$DN$23,'III. Finanzberichte'!$DU$23),2),0)</f>
+      </c>
+      <c r="H112" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
+      </c>
+      <c r="I112" s="181" t="str">
+        <f>=ROUND(IFERROR($G$112-$H$112,0),2)</f>
+      </c>
+      <c r="J112" s="300" t="str">
+        <f>=ROUND(IFERROR(($G$112/$H$112)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="266" t="s">
+        <v>210</v>
+      </c>
+      <c r="C113" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$24,'III. Finanzberichte'!$L$24,'III. Finanzberichte'!$S$24,'III. Finanzberichte'!$Z$24,'III. Finanzberichte'!$AG$24,'III. Finanzberichte'!$AN$24,'III. Finanzberichte'!$AU$24,'III. Finanzberichte'!$BB$24,'III. Finanzberichte'!$BI$24,'III. Finanzberichte'!$BP$24,'III. Finanzberichte'!$BW$24,'III. Finanzberichte'!$CD$24,'III. Finanzberichte'!$CK$24,'III. Finanzberichte'!$CR$24,'III. Finanzberichte'!$CY$24,'III. Finanzberichte'!$DF$24,'III. Finanzberichte'!$DM$24,'III. Finanzberichte'!$DT$24),2),0)</f>
+      </c>
+      <c r="D113" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
+      </c>
+      <c r="E113" s="200" t="str">
+        <f>=ROUND(IFERROR($C$113-$D$113,0),2)</f>
+      </c>
+      <c r="F113" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$113/$D$113)-1,0),4)</f>
+      </c>
+      <c r="G113" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$24,'III. Finanzberichte'!$M$24,'III. Finanzberichte'!$T$24,'III. Finanzberichte'!$AA$24,'III. Finanzberichte'!$AH$24,'III. Finanzberichte'!$AO$24,'III. Finanzberichte'!$AV$24,'III. Finanzberichte'!$BC$24,'III. Finanzberichte'!$BJ$24,'III. Finanzberichte'!$BQ$24,'III. Finanzberichte'!$BX$24,'III. Finanzberichte'!$CE$24,'III. Finanzberichte'!$CL$24,'III. Finanzberichte'!$CS$24,'III. Finanzberichte'!$CZ$24,'III. Finanzberichte'!$DG$24,'III. Finanzberichte'!$DN$24,'III. Finanzberichte'!$DU$24),2),0)</f>
+      </c>
+      <c r="H113" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
+      </c>
+      <c r="I113" s="181" t="str">
+        <f>=ROUND(IFERROR($G$113-$H$113,0),2)</f>
+      </c>
+      <c r="J113" s="301" t="str">
+        <f>=ROUND(IFERROR(($G$113/$H$113)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="266" t="s">
+        <v>211</v>
+      </c>
+      <c r="C114" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$25,'III. Finanzberichte'!$L$25,'III. Finanzberichte'!$S$25,'III. Finanzberichte'!$Z$25,'III. Finanzberichte'!$AG$25,'III. Finanzberichte'!$AN$25,'III. Finanzberichte'!$AU$25,'III. Finanzberichte'!$BB$25,'III. Finanzberichte'!$BI$25,'III. Finanzberichte'!$BP$25,'III. Finanzberichte'!$BW$25,'III. Finanzberichte'!$CD$25,'III. Finanzberichte'!$CK$25,'III. Finanzberichte'!$CR$25,'III. Finanzberichte'!$CY$25,'III. Finanzberichte'!$DF$25,'III. Finanzberichte'!$DM$25,'III. Finanzberichte'!$DT$25),2),0)</f>
+      </c>
+      <c r="D114" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
+      </c>
+      <c r="E114" s="200" t="str">
+        <f>=ROUND(IFERROR($C$114-$D$114,0),2)</f>
+      </c>
+      <c r="F114" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$114/$D$114)-1,0),4)</f>
+      </c>
+      <c r="G114" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$25,'III. Finanzberichte'!$M$25,'III. Finanzberichte'!$T$25,'III. Finanzberichte'!$AA$25,'III. Finanzberichte'!$AH$25,'III. Finanzberichte'!$AO$25,'III. Finanzberichte'!$AV$25,'III. Finanzberichte'!$BC$25,'III. Finanzberichte'!$BJ$25,'III. Finanzberichte'!$BQ$25,'III. Finanzberichte'!$BX$25,'III. Finanzberichte'!$CE$25,'III. Finanzberichte'!$CL$25,'III. Finanzberichte'!$CS$25,'III. Finanzberichte'!$CZ$25,'III. Finanzberichte'!$DG$25,'III. Finanzberichte'!$DN$25,'III. Finanzberichte'!$DU$25),2),0)</f>
+      </c>
+      <c r="H114" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
+      </c>
+      <c r="I114" s="181" t="str">
+        <f>=ROUND(IFERROR($G$114-$H$114,0),2)</f>
+      </c>
+      <c r="J114" s="302" t="str">
+        <f>=ROUND(IFERROR(($G$114/$H$114)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="266" t="s">
+        <v>212</v>
+      </c>
+      <c r="C115" s="240" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$E$26,'III. Finanzberichte'!$L$26,'III. Finanzberichte'!$S$26,'III. Finanzberichte'!$Z$26,'III. Finanzberichte'!$AG$26,'III. Finanzberichte'!$AN$26,'III. Finanzberichte'!$AU$26,'III. Finanzberichte'!$BB$26,'III. Finanzberichte'!$BI$26,'III. Finanzberichte'!$BP$26,'III. Finanzberichte'!$BW$26,'III. Finanzberichte'!$CD$26,'III. Finanzberichte'!$CK$26,'III. Finanzberichte'!$CR$26,'III. Finanzberichte'!$CY$26,'III. Finanzberichte'!$DF$26,'III. Finanzberichte'!$DM$26,'III. Finanzberichte'!$DT$26),2),0)</f>
+      </c>
+      <c r="D115" s="240" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
+      </c>
+      <c r="E115" s="200" t="str">
+        <f>=ROUND(IFERROR($C$115-$D$115,0),2)</f>
+      </c>
+      <c r="F115" s="258" t="str">
+        <f>=ROUND(IFERROR(($C$115/$D$115)-1,0),4)</f>
+      </c>
+      <c r="G115" s="217" t="str">
+        <f>=IFERROR(ROUND(CHOOSE(F82,'III. Finanzberichte'!$F$26,'III. Finanzberichte'!$M$26,'III. Finanzberichte'!$T$26,'III. Finanzberichte'!$AA$26,'III. Finanzberichte'!$AH$26,'III. Finanzberichte'!$AO$26,'III. Finanzberichte'!$AV$26,'III. Finanzberichte'!$BC$26,'III. Finanzberichte'!$BJ$26,'III. Finanzberichte'!$BQ$26,'III. Finanzberichte'!$BX$26,'III. Finanzberichte'!$CE$26,'III. Finanzberichte'!$CL$26,'III. Finanzberichte'!$CS$26,'III. Finanzberichte'!$CZ$26,'III. Finanzberichte'!$DG$26,'III. Finanzberichte'!$DN$26,'III. Finanzberichte'!$DU$26),2),0)</f>
+      </c>
+      <c r="H115" s="217" t="str">
+        <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
+      </c>
+      <c r="I115" s="181" t="str">
+        <f>=ROUND(IFERROR($G$115-$H$115,0),2)</f>
+      </c>
+      <c r="J115" s="303" t="str">
+        <f>=ROUND(IFERROR(($G$115/$H$115)-1,0),4)</f>
+      </c>
+    </row>
+    <row r="116" ht="20" customHeight="true">
+      <c r="B116" s="271" t="s">
         <v>266</v>
       </c>
-      <c r="C111" s="270" t="str">
-        <f>=ROUND(SUM($C$103:$C$110),2)</f>
-      </c>
-      <c r="D111" s="270" t="str">
-        <f>=ROUND(SUM($D$103:$D$110),2)</f>
-      </c>
-      <c r="E111" s="270" t="str">
-        <f>=ROUND(SUM($E$103:$E$110),2)</f>
-      </c>
-      <c r="F111" s="301" t="str">
-        <f>=ROUND(IFERROR(($C$111/$D$111)-1,0),4)</f>
-      </c>
-      <c r="G111" s="272" t="str">
-        <f>=ROUND(SUM($G$103:$G$110),2)</f>
-      </c>
-      <c r="H111" s="272" t="str">
-        <f>=ROUND(SUM($H$103:$H$110),2)</f>
-      </c>
-      <c r="I111" s="272" t="str">
-        <f>=ROUND(SUM($I$103:$I$110),2)</f>
-      </c>
-      <c r="J111" s="302" t="str">
-        <f>=ROUND(IFERROR(($G$111/$H$111)-1,0),4)</f>
+      <c r="C116" s="272" t="str">
+        <f>=ROUND(SUM($C$108:$C$115),2)</f>
+      </c>
+      <c r="D116" s="272" t="str">
+        <f>=ROUND(SUM($D$108:$D$115),2)</f>
+      </c>
+      <c r="E116" s="272" t="str">
+        <f>=ROUND(SUM($E$108:$E$115),2)</f>
+      </c>
+      <c r="F116" s="304" t="str">
+        <f>=ROUND(IFERROR(($C$116/$D$116)-1,0),4)</f>
+      </c>
+      <c r="G116" s="274" t="str">
+        <f>=ROUND(SUM($G$108:$G$115),2)</f>
+      </c>
+      <c r="H116" s="274" t="str">
+        <f>=ROUND(SUM($H$108:$H$115),2)</f>
+      </c>
+      <c r="I116" s="274" t="str">
+        <f>=ROUND(SUM($I$108:$I$115),2)</f>
+      </c>
+      <c r="J116" s="305" t="str">
+        <f>=ROUND(IFERROR(($G$116/$H$116)-1,0),4)</f>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="88">
+  <mergeCells count="104">
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="B5:J5"/>
@@ -21569,41 +22391,57 @@
     <mergeCell ref="B36:J36"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:E39"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D43:E43"/>
     <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D44:E44"/>
     <mergeCell ref="B45:C45"/>
+    <mergeCell ref="D45:E45"/>
     <mergeCell ref="B46:C46"/>
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B50:J50"/>
-    <mergeCell ref="B59:J59"/>
-    <mergeCell ref="B72:J72"/>
-    <mergeCell ref="B73:J73"/>
-    <mergeCell ref="C75:I75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="F76:I76"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="F77:I77"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="F78:I78"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="F79:I79"/>
-    <mergeCell ref="B81:J81"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B51:J51"/>
+    <mergeCell ref="B60:J60"/>
+    <mergeCell ref="B77:J77"/>
+    <mergeCell ref="B78:J78"/>
+    <mergeCell ref="C80:I80"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="F81:I81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="F82:I82"/>
+    <mergeCell ref="C83:E83"/>
     <mergeCell ref="F83:I83"/>
-    <mergeCell ref="G84:H84"/>
-    <mergeCell ref="G85:H85"/>
-    <mergeCell ref="G86:H86"/>
-    <mergeCell ref="G87:H87"/>
-    <mergeCell ref="B91:J91"/>
-    <mergeCell ref="B100:J100"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="F84:I84"/>
+    <mergeCell ref="B86:J86"/>
+    <mergeCell ref="B88:C88"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="F88:I88"/>
+    <mergeCell ref="G89:H89"/>
+    <mergeCell ref="G90:H90"/>
+    <mergeCell ref="G91:H91"/>
+    <mergeCell ref="G92:H92"/>
+    <mergeCell ref="B96:J96"/>
+    <mergeCell ref="B105:J105"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="L77:P77"/>
+    <mergeCell ref="M78:P78"/>
+    <mergeCell ref="M79:P79"/>
+    <mergeCell ref="M80:P80"/>
+    <mergeCell ref="L82:P82"/>
+    <mergeCell ref="L90:P90"/>
   </mergeCells>
   <conditionalFormatting sqref="C13:I13">
     <cfRule type="expression" dxfId="9" priority="1">
@@ -21635,59 +22473,74 @@
       <formula>$C$18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D46">
+  <conditionalFormatting sqref="D47">
     <cfRule type="expression" dxfId="10" priority="7">
-      <formula>$D$46="OK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D46">
-    <cfRule type="expression" dxfId="11" priority="8">
-      <formula>$D$46&lt;&gt;"OK"</formula>
+      <formula>$D$47="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D47">
-    <cfRule type="expression" dxfId="12" priority="9">
-      <formula>$D$47&gt;0</formula>
+    <cfRule type="expression" dxfId="11" priority="8">
+      <formula>$D$47&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F62:F69">
-    <cfRule type="expression" dxfId="13" priority="10">
-      <formula>F62&gt;0.2</formula>
+  <conditionalFormatting sqref="E47">
+    <cfRule type="expression" dxfId="12" priority="9">
+      <formula>$E$47="OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F62:F69">
-    <cfRule type="expression" dxfId="14" priority="11">
-      <formula>AND(F62&gt;=0.1,F62&lt;=0.2)</formula>
+  <conditionalFormatting sqref="E47">
+    <cfRule type="expression" dxfId="13" priority="10">
+      <formula>$E$47&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J62:J69">
-    <cfRule type="expression" dxfId="13" priority="12">
-      <formula>J62&gt;0.2</formula>
+  <conditionalFormatting sqref="D48">
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>$D$48&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J62:J69">
-    <cfRule type="expression" dxfId="14" priority="13">
-      <formula>AND(J62&gt;=0.1,J62&lt;=0.2)</formula>
+  <conditionalFormatting sqref="E48">
+    <cfRule type="expression" dxfId="15" priority="12">
+      <formula>$E$48&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F103:F110">
-    <cfRule type="expression" dxfId="13" priority="14">
-      <formula>F103&gt;0.2</formula>
+  <conditionalFormatting sqref="F63:F70">
+    <cfRule type="expression" dxfId="16" priority="13">
+      <formula>F63&gt;0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F103:F110">
-    <cfRule type="expression" dxfId="14" priority="15">
-      <formula>AND(F103&gt;=0.1,F103&lt;=0.2)</formula>
+  <conditionalFormatting sqref="F63:F70">
+    <cfRule type="expression" dxfId="17" priority="14">
+      <formula>AND(F63&gt;=0.1,F63&lt;=0.2)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J103:J110">
-    <cfRule type="expression" dxfId="13" priority="16">
-      <formula>J103&gt;0.2</formula>
+  <conditionalFormatting sqref="J63:J70">
+    <cfRule type="expression" dxfId="16" priority="15">
+      <formula>J63&gt;0.2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J103:J110">
-    <cfRule type="expression" dxfId="14" priority="17">
-      <formula>AND(J103&gt;=0.1,J103&lt;=0.2)</formula>
+  <conditionalFormatting sqref="J63:J70">
+    <cfRule type="expression" dxfId="17" priority="16">
+      <formula>AND(J63&gt;=0.1,J63&lt;=0.2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F108:F115">
+    <cfRule type="expression" dxfId="16" priority="17">
+      <formula>F108&gt;0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F108:F115">
+    <cfRule type="expression" dxfId="17" priority="18">
+      <formula>AND(F108&gt;=0.1,F108&lt;=0.2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J108:J115">
+    <cfRule type="expression" dxfId="16" priority="19">
+      <formula>J108&gt;0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J108:J115">
+    <cfRule type="expression" dxfId="17" priority="20">
+      <formula>AND(J108&gt;=0.1,J108&lt;=0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="8">
@@ -21703,16 +22556,16 @@
     <dataValidation allowBlank="true" sqref="F25" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="D40" type="list">
+    <dataValidation allowBlank="true" sqref="D41" type="list">
       <formula1>"Jahr 1,Jahr 2,Jahr 3"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F76" type="list">
+    <dataValidation allowBlank="true" sqref="F81" type="list">
       <formula1>=FB_Auswahl_Liste</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F84" type="list">
+    <dataValidation allowBlank="true" sqref="F89" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" sqref="F85" type="list">
+    <dataValidation allowBlank="true" sqref="F90" type="list">
       <formula1>"Abzug,Kein Abzug"</formula1>
     </dataValidation>
   </dataValidations>
@@ -21730,17 +22583,17 @@
       <c r="A1" t="s">
         <v>226</v>
       </c>
-      <c r="C1" s="303" t="s">
-        <v>374</v>
-      </c>
-      <c r="I1" s="303" t="s">
-        <v>375</v>
-      </c>
-      <c r="O1" s="303" t="s">
-        <v>376</v>
-      </c>
-      <c r="U1" s="303" t="s">
-        <v>377</v>
+      <c r="C1" s="345" t="s">
+        <v>380</v>
+      </c>
+      <c r="I1" s="345" t="s">
+        <v>381</v>
+      </c>
+      <c r="O1" s="345" t="s">
+        <v>382</v>
+      </c>
+      <c r="U1" s="345" t="s">
+        <v>383</v>
       </c>
       <c r="BA1">
         <v>1</v>
@@ -21776,7 +22629,7 @@
         <f>=IF(BK1=1,"Periode "&amp;BJ1,"")</f>
       </c>
       <c r="BN1" cm="1" s="3">
-        <f t="array" ref="BN1">_xlfn._xlws.FILTER($BE$1:$BE$18,($BB$1:$BB$18='V. AUSWERTUNG'!F77+1)*($BC$1:$BC$18=1),"")</f>
+        <f t="array" ref="BN1">_xlfn._xlws.FILTER($BE$1:$BE$18,($BB$1:$BB$18='V. AUSWERTUNG'!F82+1)*($BC$1:$BC$18=1),"")</f>
         <v>0</v>
       </c>
       <c r="BP1" cm="1" s="3">

</xml_diff>

<commit_message>
fix: prepend _xlfn prefix to MAXIFS formula
Updates Excel formula generation to use compatibility prefix for broader 
version support.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -20758,7 +20758,7 @@
       <c r="D11" s="196"/>
       <c r="E11" s="196"/>
       <c r="F11" s="197" t="str">
-        <f>=IF(F9="Neuste MA",IFERROR(MAXIFS('Daten'!$BD$1:$BD$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BC$1:$BC$18,1),0),IFERROR(VALUE(MID(F9,FIND("(#",F9)+2,FIND(")",F9)-FIND("(#",F9)-2)),0))</f>
+        <f>=IF(F9="Neuste MA",IFERROR(_xlfn.MAXIFS('Daten'!$BD$1:$BD$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BC$1:$BC$18,1),0),IFERROR(VALUE(MID(F9,FIND("(#",F9)+2,FIND(")",F9)-FIND("(#",F9)-2)),0))</f>
       </c>
       <c r="G11" s="197"/>
       <c r="H11" s="197"/>
@@ -21933,7 +21933,7 @@
       <c r="D82" s="196"/>
       <c r="E82" s="196"/>
       <c r="F82" s="197" t="str">
-        <f>=IF(F81="Neuester FB",IFERROR(MAXIFS('Daten'!$BJ$1:$BJ$18,'Daten'!$BK$1:$BK$18,1),0),IF(LEFT(F81,8)="Periode ",IFERROR(VALUE(TRIM(MID(F81,9,5))),0),0))</f>
+        <f>=IF(F81="Neuester FB",IFERROR(_xlfn.MAXIFS('Daten'!$BJ$1:$BJ$18,'Daten'!$BK$1:$BK$18,1),0),IF(LEFT(F81,8)="Periode ",IFERROR(VALUE(TRIM(MID(F81,9,5))),0),0))</f>
       </c>
       <c r="G82" s="197"/>
       <c r="H82" s="197"/>

</xml_diff>

<commit_message>
feat: integrate funding sources into MA-Grid
Extend the MA-Grid to include financing types (Eigenmittel, Drittmittel, KMW-Mittel) for improved forecast accuracy. Updated Excel formula generation to use robust SUMPRODUCT patterns and synchronized the grid structure across data generation and evaluation logic.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -20758,7 +20758,7 @@
       <c r="D11" s="196"/>
       <c r="E11" s="196"/>
       <c r="F11" s="197" t="str">
-        <f>=IF(F9="Neuste MA",IFERROR(_xlfn.MAXIFS('Daten'!$BD$1:$BD$18,'Daten'!$BB$1:$BB$18,F10,'Daten'!$BC$1:$BC$18,1),0),IFERROR(VALUE(MID(F9,FIND("(#",F9)+2,FIND(")",F9)-FIND("(#",F9)-2)),0))</f>
+        <f>=IF(F9="Neuste MA",IFERROR(SUMPRODUCT(MAX(('Daten'!$BB$1:$BB$18=F10)*('Daten'!$BC$1:$BC$18=1)*'Daten'!$BD$1:$BD$18)),0),IFERROR(VALUE(MID(F9,FIND("(#",F9)+2,FIND(")",F9)-FIND("(#",F9)-2)),0))</f>
       </c>
       <c r="G11" s="197"/>
       <c r="H11" s="197"/>
@@ -21387,8 +21387,8 @@
       <c r="B54" s="266" t="s">
         <v>194</v>
       </c>
-      <c r="C54" s="24">
-        <v>0</v>
+      <c r="C54" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Eigenmittel",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D54" s="240" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
@@ -21399,8 +21399,8 @@
       <c r="F54" s="258" t="str">
         <f>=ROUND(IFERROR(($C$54/$D$54)-1,0),4)</f>
       </c>
-      <c r="G54" s="25">
-        <v>0</v>
+      <c r="G54" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Eigenmittel",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H54" s="217" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
@@ -21416,8 +21416,8 @@
       <c r="B55" s="266" t="s">
         <v>279</v>
       </c>
-      <c r="C55" s="24">
-        <v>0</v>
+      <c r="C55" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Drittmittel",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D55" s="240" t="str">
         <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
@@ -21428,8 +21428,8 @@
       <c r="F55" s="258" t="str">
         <f>=ROUND(IFERROR(($C$55/$D$55)-1,0),4)</f>
       </c>
-      <c r="G55" s="25">
-        <v>0</v>
+      <c r="G55" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Drittmittel",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H55" s="217" t="str">
         <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
@@ -21445,8 +21445,8 @@
       <c r="B56" s="266" t="s">
         <v>199</v>
       </c>
-      <c r="C56" s="24">
-        <v>0</v>
+      <c r="C56" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D56" s="240" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
@@ -21457,8 +21457,8 @@
       <c r="F56" s="258" t="str">
         <f>=ROUND(IFERROR(($C$56/$D$56)-1,0),4)</f>
       </c>
-      <c r="G56" s="25">
-        <v>0</v>
+      <c r="G56" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H56" s="217" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
@@ -21474,8 +21474,8 @@
       <c r="B57" s="266" t="s">
         <v>280</v>
       </c>
-      <c r="C57" s="24">
-        <v>0</v>
+      <c r="C57" s="240" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Zinsertraege",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D57" s="240" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
@@ -21486,8 +21486,8 @@
       <c r="F57" s="258" t="str">
         <f>=ROUND(IFERROR(($C$57/$D$57)-1,0),4)</f>
       </c>
-      <c r="G57" s="25">
-        <v>0</v>
+      <c r="G57" s="217" t="str">
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Zinsertraege",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H57" s="217" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
@@ -21575,7 +21575,7 @@
         <v>205</v>
       </c>
       <c r="C63" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Bauausgaben",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D63" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
@@ -21587,7 +21587,7 @@
         <f>=ROUND(IFERROR(($C$63/$D$63)-1,0),4)</f>
       </c>
       <c r="G63" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Bauausgaben",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Bauausgaben",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H63" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
@@ -21604,7 +21604,7 @@
         <v>206</v>
       </c>
       <c r="C64" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Investitionen",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D64" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
@@ -21616,7 +21616,7 @@
         <f>=ROUND(IFERROR(($C$64/$D$64)-1,0),4)</f>
       </c>
       <c r="G64" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Investitionen",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Investitionen",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H64" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
@@ -21633,7 +21633,7 @@
         <v>207</v>
       </c>
       <c r="C65" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Personalkosten",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D65" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
@@ -21645,7 +21645,7 @@
         <f>=ROUND(IFERROR(($C$65/$D$65)-1,0),4)</f>
       </c>
       <c r="G65" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Personalkosten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Personalkosten",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H65" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
@@ -21662,7 +21662,7 @@
         <v>208</v>
       </c>
       <c r="C66" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Projektaktivitaeten",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D66" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
@@ -21674,7 +21674,7 @@
         <f>=ROUND(IFERROR(($C$66/$D$66)-1,0),4)</f>
       </c>
       <c r="G66" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektaktivitaeten",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Projektaktivitaeten",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H66" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
@@ -21691,7 +21691,7 @@
         <v>209</v>
       </c>
       <c r="C67" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Projektverwaltung",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D67" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
@@ -21703,7 +21703,7 @@
         <f>=ROUND(IFERROR(($C$67/$D$67)-1,0),4)</f>
       </c>
       <c r="G67" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Projektverwaltung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Projektverwaltung",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H67" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
@@ -21720,7 +21720,7 @@
         <v>210</v>
       </c>
       <c r="C68" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Evaluierung",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D68" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
@@ -21732,7 +21732,7 @@
         <f>=ROUND(IFERROR(($C$68/$D$68)-1,0),4)</f>
       </c>
       <c r="G68" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Evaluierung",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Evaluierung",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H68" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
@@ -21749,7 +21749,7 @@
         <v>211</v>
       </c>
       <c r="C69" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Audit",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D69" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
@@ -21761,7 +21761,7 @@
         <f>=ROUND(IFERROR(($C$69/$D$69)-1,0),4)</f>
       </c>
       <c r="G69" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Audit",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Audit",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H69" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
@@ -21778,7 +21778,7 @@
         <v>212</v>
       </c>
       <c r="C70" s="240" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Reserve",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="D70" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
@@ -21790,7 +21790,7 @@
         <f>=ROUND(IFERROR(($C$70/$D$70)-1,0),4)</f>
       </c>
       <c r="G70" s="217" t="str">
-        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$144,'Daten'!$BT$1:$BT$144,"Reserve",'Daten'!$BR$1:$BR$144,F10,'Daten'!$BS$1:$BS$144,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$144,"&gt;=1"),2),0)</f>
+        <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Reserve",'Daten'!$BR$1:$BR$198,F10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;F11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
       <c r="H70" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
@@ -21933,7 +21933,7 @@
       <c r="D82" s="196"/>
       <c r="E82" s="196"/>
       <c r="F82" s="197" t="str">
-        <f>=IF(F81="Neuester FB",IFERROR(_xlfn.MAXIFS('Daten'!$BJ$1:$BJ$18,'Daten'!$BK$1:$BK$18,1),0),IF(LEFT(F81,8)="Periode ",IFERROR(VALUE(TRIM(MID(F81,9,5))),0),0))</f>
+        <f>=IF(F81="Neuester FB",IFERROR(SUMPRODUCT(MAX(('Daten'!$BK$1:$BK$18=1)*'Daten'!$BJ$1:$BJ$18)),0),IF(LEFT(F81,8)="Periode ",IFERROR(VALUE(TRIM(MID(F81,9,5))),0),0))</f>
       </c>
       <c r="G82" s="197"/>
       <c r="H82" s="197"/>
@@ -23688,19 +23688,19 @@
         <f>=IF(BK9=1,"Periode "&amp;BJ9,"")</f>
       </c>
       <c r="BR9" t="str">
-        <f>=$BB$2</f>
+        <f>=$BB$1</f>
       </c>
       <c r="BS9" t="str">
-        <f>=$BD$2</f>
+        <f>=$BD$1</f>
       </c>
       <c r="BT9" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="BU9" t="str">
-        <f>=IFERROR('IV. MA'!G10,0)</f>
+        <f>=IFERROR('IV. MA'!C21,0)</f>
       </c>
       <c r="BV9" t="str">
-        <f>=IFERROR('IV. MA'!H10,0)</f>
+        <f>=IFERROR('IV. MA'!D21,0)</f>
       </c>
     </row>
     <row r="10">
@@ -23741,19 +23741,19 @@
         <f>=IF(BK10=1,"Periode "&amp;BJ10,"")</f>
       </c>
       <c r="BR10" t="str">
-        <f>=$BB$2</f>
+        <f>=$BB$1</f>
       </c>
       <c r="BS10" t="str">
-        <f>=$BD$2</f>
+        <f>=$BD$1</f>
       </c>
       <c r="BT10" t="s">
-        <v>206</v>
+        <v>279</v>
       </c>
       <c r="BU10" t="str">
-        <f>=IFERROR('IV. MA'!G11,0)</f>
+        <f>=IFERROR('IV. MA'!C22,0)</f>
       </c>
       <c r="BV10" t="str">
-        <f>=IFERROR('IV. MA'!H11,0)</f>
+        <f>=IFERROR('IV. MA'!D22,0)</f>
       </c>
     </row>
     <row r="11">
@@ -23794,19 +23794,19 @@
         <f>=IF(BK11=1,"Periode "&amp;BJ11,"")</f>
       </c>
       <c r="BR11" t="str">
-        <f>=$BB$2</f>
+        <f>=$BB$1</f>
       </c>
       <c r="BS11" t="str">
-        <f>=$BD$2</f>
+        <f>=$BD$1</f>
       </c>
       <c r="BT11" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="BU11" t="str">
-        <f>=IFERROR('IV. MA'!G12,0)</f>
+        <f>=IFERROR('IV. MA'!C25,0)</f>
       </c>
       <c r="BV11" t="str">
-        <f>=IFERROR('IV. MA'!H12,0)</f>
+        <f>=IFERROR('IV. MA'!D25,0)</f>
       </c>
     </row>
     <row r="12">
@@ -23853,13 +23853,13 @@
         <f>=$BD$2</f>
       </c>
       <c r="BT12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="BU12" t="str">
-        <f>=IFERROR('IV. MA'!G13,0)</f>
+        <f>=IFERROR('IV. MA'!G10,0)</f>
       </c>
       <c r="BV12" t="str">
-        <f>=IFERROR('IV. MA'!H13,0)</f>
+        <f>=IFERROR('IV. MA'!H10,0)</f>
       </c>
     </row>
     <row r="13">
@@ -23906,13 +23906,13 @@
         <f>=$BD$2</f>
       </c>
       <c r="BT13" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="BU13" t="str">
-        <f>=IFERROR('IV. MA'!G14,0)</f>
+        <f>=IFERROR('IV. MA'!G11,0)</f>
       </c>
       <c r="BV13" t="str">
-        <f>=IFERROR('IV. MA'!H14,0)</f>
+        <f>=IFERROR('IV. MA'!H11,0)</f>
       </c>
     </row>
     <row r="14">
@@ -23959,13 +23959,13 @@
         <f>=$BD$2</f>
       </c>
       <c r="BT14" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="BU14" t="str">
-        <f>=IFERROR('IV. MA'!G15,0)</f>
+        <f>=IFERROR('IV. MA'!G12,0)</f>
       </c>
       <c r="BV14" t="str">
-        <f>=IFERROR('IV. MA'!H15,0)</f>
+        <f>=IFERROR('IV. MA'!H12,0)</f>
       </c>
     </row>
     <row r="15">
@@ -24012,13 +24012,13 @@
         <f>=$BD$2</f>
       </c>
       <c r="BT15" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="BU15" t="str">
-        <f>=IFERROR('IV. MA'!G16,0)</f>
+        <f>=IFERROR('IV. MA'!G13,0)</f>
       </c>
       <c r="BV15" t="str">
-        <f>=IFERROR('IV. MA'!H16,0)</f>
+        <f>=IFERROR('IV. MA'!H13,0)</f>
       </c>
     </row>
     <row r="16">
@@ -24065,13 +24065,13 @@
         <f>=$BD$2</f>
       </c>
       <c r="BT16" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="BU16" t="str">
-        <f>=IFERROR('IV. MA'!G17,0)</f>
+        <f>=IFERROR('IV. MA'!G14,0)</f>
       </c>
       <c r="BV16" t="str">
-        <f>=IFERROR('IV. MA'!H17,0)</f>
+        <f>=IFERROR('IV. MA'!H14,0)</f>
       </c>
     </row>
     <row r="17">
@@ -24112,19 +24112,19 @@
         <f>=IF(BK17=1,"Periode "&amp;BJ17,"")</f>
       </c>
       <c r="BR17" t="str">
-        <f>=$BB$3</f>
+        <f>=$BB$2</f>
       </c>
       <c r="BS17" t="str">
-        <f>=$BD$3</f>
+        <f>=$BD$2</f>
       </c>
       <c r="BT17" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="BU17" t="str">
-        <f>=IFERROR('IV. MA'!K10,0)</f>
+        <f>=IFERROR('IV. MA'!G15,0)</f>
       </c>
       <c r="BV17" t="str">
-        <f>=IFERROR('IV. MA'!L10,0)</f>
+        <f>=IFERROR('IV. MA'!H15,0)</f>
       </c>
     </row>
     <row r="18">
@@ -24165,87 +24165,87 @@
         <f>=IF(BK18=1,"Periode "&amp;BJ18,"")</f>
       </c>
       <c r="BR18" t="str">
-        <f>=$BB$3</f>
+        <f>=$BB$2</f>
       </c>
       <c r="BS18" t="str">
-        <f>=$BD$3</f>
+        <f>=$BD$2</f>
       </c>
       <c r="BT18" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="BU18" t="str">
-        <f>=IFERROR('IV. MA'!K11,0)</f>
+        <f>=IFERROR('IV. MA'!G16,0)</f>
       </c>
       <c r="BV18" t="str">
-        <f>=IFERROR('IV. MA'!L11,0)</f>
+        <f>=IFERROR('IV. MA'!H16,0)</f>
       </c>
     </row>
     <row r="19">
       <c r="BR19" t="str">
-        <f>=$BB$3</f>
+        <f>=$BB$2</f>
       </c>
       <c r="BS19" t="str">
-        <f>=$BD$3</f>
+        <f>=$BD$2</f>
       </c>
       <c r="BT19" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="BU19" t="str">
-        <f>=IFERROR('IV. MA'!K12,0)</f>
+        <f>=IFERROR('IV. MA'!G17,0)</f>
       </c>
       <c r="BV19" t="str">
-        <f>=IFERROR('IV. MA'!L12,0)</f>
+        <f>=IFERROR('IV. MA'!H17,0)</f>
       </c>
     </row>
     <row r="20">
       <c r="BR20" t="str">
-        <f>=$BB$3</f>
+        <f>=$BB$2</f>
       </c>
       <c r="BS20" t="str">
-        <f>=$BD$3</f>
+        <f>=$BD$2</f>
       </c>
       <c r="BT20" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="BU20" t="str">
-        <f>=IFERROR('IV. MA'!K13,0)</f>
+        <f>=IFERROR('IV. MA'!G21,0)</f>
       </c>
       <c r="BV20" t="str">
-        <f>=IFERROR('IV. MA'!L13,0)</f>
+        <f>=IFERROR('IV. MA'!H21,0)</f>
       </c>
     </row>
     <row r="21">
       <c r="BR21" t="str">
-        <f>=$BB$3</f>
+        <f>=$BB$2</f>
       </c>
       <c r="BS21" t="str">
-        <f>=$BD$3</f>
+        <f>=$BD$2</f>
       </c>
       <c r="BT21" t="s">
-        <v>209</v>
+        <v>279</v>
       </c>
       <c r="BU21" t="str">
-        <f>=IFERROR('IV. MA'!K14,0)</f>
+        <f>=IFERROR('IV. MA'!G22,0)</f>
       </c>
       <c r="BV21" t="str">
-        <f>=IFERROR('IV. MA'!L14,0)</f>
+        <f>=IFERROR('IV. MA'!H22,0)</f>
       </c>
     </row>
     <row r="22">
       <c r="BR22" t="str">
-        <f>=$BB$3</f>
+        <f>=$BB$2</f>
       </c>
       <c r="BS22" t="str">
-        <f>=$BD$3</f>
+        <f>=$BD$2</f>
       </c>
       <c r="BT22" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="BU22" t="str">
-        <f>=IFERROR('IV. MA'!K15,0)</f>
+        <f>=IFERROR('IV. MA'!G25,0)</f>
       </c>
       <c r="BV22" t="str">
-        <f>=IFERROR('IV. MA'!L15,0)</f>
+        <f>=IFERROR('IV. MA'!H25,0)</f>
       </c>
     </row>
     <row r="23">
@@ -24256,13 +24256,13 @@
         <f>=$BD$3</f>
       </c>
       <c r="BT23" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="BU23" t="str">
-        <f>=IFERROR('IV. MA'!K16,0)</f>
+        <f>=IFERROR('IV. MA'!K10,0)</f>
       </c>
       <c r="BV23" t="str">
-        <f>=IFERROR('IV. MA'!L16,0)</f>
+        <f>=IFERROR('IV. MA'!L10,0)</f>
       </c>
     </row>
     <row r="24">
@@ -24273,2053 +24273,2971 @@
         <f>=$BD$3</f>
       </c>
       <c r="BT24" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="BU24" t="str">
-        <f>=IFERROR('IV. MA'!K17,0)</f>
+        <f>=IFERROR('IV. MA'!K11,0)</f>
       </c>
       <c r="BV24" t="str">
-        <f>=IFERROR('IV. MA'!L17,0)</f>
+        <f>=IFERROR('IV. MA'!L11,0)</f>
       </c>
     </row>
     <row r="25">
       <c r="BR25" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS25" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT25" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="BU25" t="str">
-        <f>=IFERROR('IV. MA'!O10,0)</f>
+        <f>=IFERROR('IV. MA'!K12,0)</f>
       </c>
       <c r="BV25" t="str">
-        <f>=IFERROR('IV. MA'!P10,0)</f>
+        <f>=IFERROR('IV. MA'!L12,0)</f>
       </c>
     </row>
     <row r="26">
       <c r="BR26" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS26" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT26" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="BU26" t="str">
-        <f>=IFERROR('IV. MA'!O11,0)</f>
+        <f>=IFERROR('IV. MA'!K13,0)</f>
       </c>
       <c r="BV26" t="str">
-        <f>=IFERROR('IV. MA'!P11,0)</f>
+        <f>=IFERROR('IV. MA'!L13,0)</f>
       </c>
     </row>
     <row r="27">
       <c r="BR27" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS27" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT27" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="BU27" t="str">
-        <f>=IFERROR('IV. MA'!O12,0)</f>
+        <f>=IFERROR('IV. MA'!K14,0)</f>
       </c>
       <c r="BV27" t="str">
-        <f>=IFERROR('IV. MA'!P12,0)</f>
+        <f>=IFERROR('IV. MA'!L14,0)</f>
       </c>
     </row>
     <row r="28">
       <c r="BR28" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS28" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT28" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="BU28" t="str">
-        <f>=IFERROR('IV. MA'!O13,0)</f>
+        <f>=IFERROR('IV. MA'!K15,0)</f>
       </c>
       <c r="BV28" t="str">
-        <f>=IFERROR('IV. MA'!P13,0)</f>
+        <f>=IFERROR('IV. MA'!L15,0)</f>
       </c>
     </row>
     <row r="29">
       <c r="BR29" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS29" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT29" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="BU29" t="str">
-        <f>=IFERROR('IV. MA'!O14,0)</f>
+        <f>=IFERROR('IV. MA'!K16,0)</f>
       </c>
       <c r="BV29" t="str">
-        <f>=IFERROR('IV. MA'!P14,0)</f>
+        <f>=IFERROR('IV. MA'!L16,0)</f>
       </c>
     </row>
     <row r="30">
       <c r="BR30" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS30" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT30" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="BU30" t="str">
-        <f>=IFERROR('IV. MA'!O15,0)</f>
+        <f>=IFERROR('IV. MA'!K17,0)</f>
       </c>
       <c r="BV30" t="str">
-        <f>=IFERROR('IV. MA'!P15,0)</f>
+        <f>=IFERROR('IV. MA'!L17,0)</f>
       </c>
     </row>
     <row r="31">
       <c r="BR31" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS31" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT31" t="s">
-        <v>211</v>
+        <v>194</v>
       </c>
       <c r="BU31" t="str">
-        <f>=IFERROR('IV. MA'!O16,0)</f>
+        <f>=IFERROR('IV. MA'!K21,0)</f>
       </c>
       <c r="BV31" t="str">
-        <f>=IFERROR('IV. MA'!P16,0)</f>
+        <f>=IFERROR('IV. MA'!L21,0)</f>
       </c>
     </row>
     <row r="32">
       <c r="BR32" t="str">
-        <f>=$BB$4</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS32" t="str">
-        <f>=$BD$4</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT32" t="s">
-        <v>212</v>
+        <v>279</v>
       </c>
       <c r="BU32" t="str">
-        <f>=IFERROR('IV. MA'!O17,0)</f>
+        <f>=IFERROR('IV. MA'!K22,0)</f>
       </c>
       <c r="BV32" t="str">
-        <f>=IFERROR('IV. MA'!P17,0)</f>
+        <f>=IFERROR('IV. MA'!L22,0)</f>
       </c>
     </row>
     <row r="33">
       <c r="BR33" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$3</f>
       </c>
       <c r="BS33" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$3</f>
       </c>
       <c r="BT33" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="BU33" t="str">
-        <f>=IFERROR('IV. MA'!S10,0)</f>
+        <f>=IFERROR('IV. MA'!K25,0)</f>
       </c>
       <c r="BV33" t="str">
-        <f>=IFERROR('IV. MA'!T10,0)</f>
+        <f>=IFERROR('IV. MA'!L25,0)</f>
       </c>
     </row>
     <row r="34">
       <c r="BR34" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS34" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT34" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="BU34" t="str">
-        <f>=IFERROR('IV. MA'!S11,0)</f>
+        <f>=IFERROR('IV. MA'!O10,0)</f>
       </c>
       <c r="BV34" t="str">
-        <f>=IFERROR('IV. MA'!T11,0)</f>
+        <f>=IFERROR('IV. MA'!P10,0)</f>
       </c>
     </row>
     <row r="35">
       <c r="BR35" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS35" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT35" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="BU35" t="str">
-        <f>=IFERROR('IV. MA'!S12,0)</f>
+        <f>=IFERROR('IV. MA'!O11,0)</f>
       </c>
       <c r="BV35" t="str">
-        <f>=IFERROR('IV. MA'!T12,0)</f>
+        <f>=IFERROR('IV. MA'!P11,0)</f>
       </c>
     </row>
     <row r="36">
       <c r="BR36" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS36" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT36" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BU36" t="str">
-        <f>=IFERROR('IV. MA'!S13,0)</f>
+        <f>=IFERROR('IV. MA'!O12,0)</f>
       </c>
       <c r="BV36" t="str">
-        <f>=IFERROR('IV. MA'!T13,0)</f>
+        <f>=IFERROR('IV. MA'!P12,0)</f>
       </c>
     </row>
     <row r="37">
       <c r="BR37" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS37" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT37" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="BU37" t="str">
-        <f>=IFERROR('IV. MA'!S14,0)</f>
+        <f>=IFERROR('IV. MA'!O13,0)</f>
       </c>
       <c r="BV37" t="str">
-        <f>=IFERROR('IV. MA'!T14,0)</f>
+        <f>=IFERROR('IV. MA'!P13,0)</f>
       </c>
     </row>
     <row r="38">
       <c r="BR38" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS38" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT38" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="BU38" t="str">
-        <f>=IFERROR('IV. MA'!S15,0)</f>
+        <f>=IFERROR('IV. MA'!O14,0)</f>
       </c>
       <c r="BV38" t="str">
-        <f>=IFERROR('IV. MA'!T15,0)</f>
+        <f>=IFERROR('IV. MA'!P14,0)</f>
       </c>
     </row>
     <row r="39">
       <c r="BR39" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS39" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT39" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="BU39" t="str">
-        <f>=IFERROR('IV. MA'!S16,0)</f>
+        <f>=IFERROR('IV. MA'!O15,0)</f>
       </c>
       <c r="BV39" t="str">
-        <f>=IFERROR('IV. MA'!T16,0)</f>
+        <f>=IFERROR('IV. MA'!P15,0)</f>
       </c>
     </row>
     <row r="40">
       <c r="BR40" t="str">
-        <f>=$BB$5</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS40" t="str">
-        <f>=$BD$5</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT40" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="BU40" t="str">
-        <f>=IFERROR('IV. MA'!S17,0)</f>
+        <f>=IFERROR('IV. MA'!O16,0)</f>
       </c>
       <c r="BV40" t="str">
-        <f>=IFERROR('IV. MA'!T17,0)</f>
+        <f>=IFERROR('IV. MA'!P16,0)</f>
       </c>
     </row>
     <row r="41">
       <c r="BR41" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS41" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT41" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="BU41" t="str">
-        <f>=IFERROR('IV. MA'!W10,0)</f>
+        <f>=IFERROR('IV. MA'!O17,0)</f>
       </c>
       <c r="BV41" t="str">
-        <f>=IFERROR('IV. MA'!X10,0)</f>
+        <f>=IFERROR('IV. MA'!P17,0)</f>
       </c>
     </row>
     <row r="42">
       <c r="BR42" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS42" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT42" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="BU42" t="str">
-        <f>=IFERROR('IV. MA'!W11,0)</f>
+        <f>=IFERROR('IV. MA'!O21,0)</f>
       </c>
       <c r="BV42" t="str">
-        <f>=IFERROR('IV. MA'!X11,0)</f>
+        <f>=IFERROR('IV. MA'!P21,0)</f>
       </c>
     </row>
     <row r="43">
       <c r="BR43" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS43" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT43" t="s">
-        <v>207</v>
+        <v>279</v>
       </c>
       <c r="BU43" t="str">
-        <f>=IFERROR('IV. MA'!W12,0)</f>
+        <f>=IFERROR('IV. MA'!O22,0)</f>
       </c>
       <c r="BV43" t="str">
-        <f>=IFERROR('IV. MA'!X12,0)</f>
+        <f>=IFERROR('IV. MA'!P22,0)</f>
       </c>
     </row>
     <row r="44">
       <c r="BR44" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$4</f>
       </c>
       <c r="BS44" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$4</f>
       </c>
       <c r="BT44" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="BU44" t="str">
-        <f>=IFERROR('IV. MA'!W13,0)</f>
+        <f>=IFERROR('IV. MA'!O25,0)</f>
       </c>
       <c r="BV44" t="str">
-        <f>=IFERROR('IV. MA'!X13,0)</f>
+        <f>=IFERROR('IV. MA'!P25,0)</f>
       </c>
     </row>
     <row r="45">
       <c r="BR45" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS45" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT45" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="BU45" t="str">
-        <f>=IFERROR('IV. MA'!W14,0)</f>
+        <f>=IFERROR('IV. MA'!S10,0)</f>
       </c>
       <c r="BV45" t="str">
-        <f>=IFERROR('IV. MA'!X14,0)</f>
+        <f>=IFERROR('IV. MA'!T10,0)</f>
       </c>
     </row>
     <row r="46">
       <c r="BR46" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS46" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT46" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="BU46" t="str">
-        <f>=IFERROR('IV. MA'!W15,0)</f>
+        <f>=IFERROR('IV. MA'!S11,0)</f>
       </c>
       <c r="BV46" t="str">
-        <f>=IFERROR('IV. MA'!X15,0)</f>
+        <f>=IFERROR('IV. MA'!T11,0)</f>
       </c>
     </row>
     <row r="47">
       <c r="BR47" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS47" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT47" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="BU47" t="str">
-        <f>=IFERROR('IV. MA'!W16,0)</f>
+        <f>=IFERROR('IV. MA'!S12,0)</f>
       </c>
       <c r="BV47" t="str">
-        <f>=IFERROR('IV. MA'!X16,0)</f>
+        <f>=IFERROR('IV. MA'!T12,0)</f>
       </c>
     </row>
     <row r="48">
       <c r="BR48" t="str">
-        <f>=$BB$6</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS48" t="str">
-        <f>=$BD$6</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT48" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="BU48" t="str">
-        <f>=IFERROR('IV. MA'!W17,0)</f>
+        <f>=IFERROR('IV. MA'!S13,0)</f>
       </c>
       <c r="BV48" t="str">
-        <f>=IFERROR('IV. MA'!X17,0)</f>
+        <f>=IFERROR('IV. MA'!T13,0)</f>
       </c>
     </row>
     <row r="49">
       <c r="BR49" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS49" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT49" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="BU49" t="str">
-        <f>=IFERROR('IV. MA'!AA10,0)</f>
+        <f>=IFERROR('IV. MA'!S14,0)</f>
       </c>
       <c r="BV49" t="str">
-        <f>=IFERROR('IV. MA'!AB10,0)</f>
+        <f>=IFERROR('IV. MA'!T14,0)</f>
       </c>
     </row>
     <row r="50">
       <c r="BR50" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS50" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT50" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="BU50" t="str">
-        <f>=IFERROR('IV. MA'!AA11,0)</f>
+        <f>=IFERROR('IV. MA'!S15,0)</f>
       </c>
       <c r="BV50" t="str">
-        <f>=IFERROR('IV. MA'!AB11,0)</f>
+        <f>=IFERROR('IV. MA'!T15,0)</f>
       </c>
     </row>
     <row r="51">
       <c r="BR51" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS51" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT51" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="BU51" t="str">
-        <f>=IFERROR('IV. MA'!AA12,0)</f>
+        <f>=IFERROR('IV. MA'!S16,0)</f>
       </c>
       <c r="BV51" t="str">
-        <f>=IFERROR('IV. MA'!AB12,0)</f>
+        <f>=IFERROR('IV. MA'!T16,0)</f>
       </c>
     </row>
     <row r="52">
       <c r="BR52" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS52" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT52" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="BU52" t="str">
-        <f>=IFERROR('IV. MA'!AA13,0)</f>
+        <f>=IFERROR('IV. MA'!S17,0)</f>
       </c>
       <c r="BV52" t="str">
-        <f>=IFERROR('IV. MA'!AB13,0)</f>
+        <f>=IFERROR('IV. MA'!T17,0)</f>
       </c>
     </row>
     <row r="53">
       <c r="BR53" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS53" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT53" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="BU53" t="str">
-        <f>=IFERROR('IV. MA'!AA14,0)</f>
+        <f>=IFERROR('IV. MA'!S21,0)</f>
       </c>
       <c r="BV53" t="str">
-        <f>=IFERROR('IV. MA'!AB14,0)</f>
+        <f>=IFERROR('IV. MA'!T21,0)</f>
       </c>
     </row>
     <row r="54">
       <c r="BR54" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS54" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT54" t="s">
-        <v>210</v>
+        <v>279</v>
       </c>
       <c r="BU54" t="str">
-        <f>=IFERROR('IV. MA'!AA15,0)</f>
+        <f>=IFERROR('IV. MA'!S22,0)</f>
       </c>
       <c r="BV54" t="str">
-        <f>=IFERROR('IV. MA'!AB15,0)</f>
+        <f>=IFERROR('IV. MA'!T22,0)</f>
       </c>
     </row>
     <row r="55">
       <c r="BR55" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$5</f>
       </c>
       <c r="BS55" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$5</f>
       </c>
       <c r="BT55" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="BU55" t="str">
-        <f>=IFERROR('IV. MA'!AA16,0)</f>
+        <f>=IFERROR('IV. MA'!S25,0)</f>
       </c>
       <c r="BV55" t="str">
-        <f>=IFERROR('IV. MA'!AB16,0)</f>
+        <f>=IFERROR('IV. MA'!T25,0)</f>
       </c>
     </row>
     <row r="56">
       <c r="BR56" t="str">
-        <f>=$BB$7</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS56" t="str">
-        <f>=$BD$7</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT56" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="BU56" t="str">
-        <f>=IFERROR('IV. MA'!AA17,0)</f>
+        <f>=IFERROR('IV. MA'!W10,0)</f>
       </c>
       <c r="BV56" t="str">
-        <f>=IFERROR('IV. MA'!AB17,0)</f>
+        <f>=IFERROR('IV. MA'!X10,0)</f>
       </c>
     </row>
     <row r="57">
       <c r="BR57" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS57" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT57" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="BU57" t="str">
-        <f>=IFERROR('IV. MA'!AE10,0)</f>
+        <f>=IFERROR('IV. MA'!W11,0)</f>
       </c>
       <c r="BV57" t="str">
-        <f>=IFERROR('IV. MA'!AF10,0)</f>
+        <f>=IFERROR('IV. MA'!X11,0)</f>
       </c>
     </row>
     <row r="58">
       <c r="BR58" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS58" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT58" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="BU58" t="str">
-        <f>=IFERROR('IV. MA'!AE11,0)</f>
+        <f>=IFERROR('IV. MA'!W12,0)</f>
       </c>
       <c r="BV58" t="str">
-        <f>=IFERROR('IV. MA'!AF11,0)</f>
+        <f>=IFERROR('IV. MA'!X12,0)</f>
       </c>
     </row>
     <row r="59">
       <c r="BR59" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS59" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT59" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="BU59" t="str">
-        <f>=IFERROR('IV. MA'!AE12,0)</f>
+        <f>=IFERROR('IV. MA'!W13,0)</f>
       </c>
       <c r="BV59" t="str">
-        <f>=IFERROR('IV. MA'!AF12,0)</f>
+        <f>=IFERROR('IV. MA'!X13,0)</f>
       </c>
     </row>
     <row r="60">
       <c r="BR60" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS60" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT60" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="BU60" t="str">
-        <f>=IFERROR('IV. MA'!AE13,0)</f>
+        <f>=IFERROR('IV. MA'!W14,0)</f>
       </c>
       <c r="BV60" t="str">
-        <f>=IFERROR('IV. MA'!AF13,0)</f>
+        <f>=IFERROR('IV. MA'!X14,0)</f>
       </c>
     </row>
     <row r="61">
       <c r="BR61" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS61" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT61" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="BU61" t="str">
-        <f>=IFERROR('IV. MA'!AE14,0)</f>
+        <f>=IFERROR('IV. MA'!W15,0)</f>
       </c>
       <c r="BV61" t="str">
-        <f>=IFERROR('IV. MA'!AF14,0)</f>
+        <f>=IFERROR('IV. MA'!X15,0)</f>
       </c>
     </row>
     <row r="62">
       <c r="BR62" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS62" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT62" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="BU62" t="str">
-        <f>=IFERROR('IV. MA'!AE15,0)</f>
+        <f>=IFERROR('IV. MA'!W16,0)</f>
       </c>
       <c r="BV62" t="str">
-        <f>=IFERROR('IV. MA'!AF15,0)</f>
+        <f>=IFERROR('IV. MA'!X16,0)</f>
       </c>
     </row>
     <row r="63">
       <c r="BR63" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS63" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT63" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="BU63" t="str">
-        <f>=IFERROR('IV. MA'!AE16,0)</f>
+        <f>=IFERROR('IV. MA'!W17,0)</f>
       </c>
       <c r="BV63" t="str">
-        <f>=IFERROR('IV. MA'!AF16,0)</f>
+        <f>=IFERROR('IV. MA'!X17,0)</f>
       </c>
     </row>
     <row r="64">
       <c r="BR64" t="str">
-        <f>=$BB$8</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS64" t="str">
-        <f>=$BD$8</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT64" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="BU64" t="str">
-        <f>=IFERROR('IV. MA'!AE17,0)</f>
+        <f>=IFERROR('IV. MA'!W21,0)</f>
       </c>
       <c r="BV64" t="str">
-        <f>=IFERROR('IV. MA'!AF17,0)</f>
+        <f>=IFERROR('IV. MA'!X21,0)</f>
       </c>
     </row>
     <row r="65">
       <c r="BR65" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS65" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT65" t="s">
-        <v>205</v>
+        <v>279</v>
       </c>
       <c r="BU65" t="str">
-        <f>=IFERROR('IV. MA'!AI10,0)</f>
+        <f>=IFERROR('IV. MA'!W22,0)</f>
       </c>
       <c r="BV65" t="str">
-        <f>=IFERROR('IV. MA'!AJ10,0)</f>
+        <f>=IFERROR('IV. MA'!X22,0)</f>
       </c>
     </row>
     <row r="66">
       <c r="BR66" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$6</f>
       </c>
       <c r="BS66" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$6</f>
       </c>
       <c r="BT66" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="BU66" t="str">
-        <f>=IFERROR('IV. MA'!AI11,0)</f>
+        <f>=IFERROR('IV. MA'!W25,0)</f>
       </c>
       <c r="BV66" t="str">
-        <f>=IFERROR('IV. MA'!AJ11,0)</f>
+        <f>=IFERROR('IV. MA'!X25,0)</f>
       </c>
     </row>
     <row r="67">
       <c r="BR67" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS67" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT67" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="BU67" t="str">
-        <f>=IFERROR('IV. MA'!AI12,0)</f>
+        <f>=IFERROR('IV. MA'!AA10,0)</f>
       </c>
       <c r="BV67" t="str">
-        <f>=IFERROR('IV. MA'!AJ12,0)</f>
+        <f>=IFERROR('IV. MA'!AB10,0)</f>
       </c>
     </row>
     <row r="68">
       <c r="BR68" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS68" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT68" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="BU68" t="str">
-        <f>=IFERROR('IV. MA'!AI13,0)</f>
+        <f>=IFERROR('IV. MA'!AA11,0)</f>
       </c>
       <c r="BV68" t="str">
-        <f>=IFERROR('IV. MA'!AJ13,0)</f>
+        <f>=IFERROR('IV. MA'!AB11,0)</f>
       </c>
     </row>
     <row r="69">
       <c r="BR69" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS69" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT69" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="BU69" t="str">
-        <f>=IFERROR('IV. MA'!AI14,0)</f>
+        <f>=IFERROR('IV. MA'!AA12,0)</f>
       </c>
       <c r="BV69" t="str">
-        <f>=IFERROR('IV. MA'!AJ14,0)</f>
+        <f>=IFERROR('IV. MA'!AB12,0)</f>
       </c>
     </row>
     <row r="70">
       <c r="BR70" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS70" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT70" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="BU70" t="str">
-        <f>=IFERROR('IV. MA'!AI15,0)</f>
+        <f>=IFERROR('IV. MA'!AA13,0)</f>
       </c>
       <c r="BV70" t="str">
-        <f>=IFERROR('IV. MA'!AJ15,0)</f>
+        <f>=IFERROR('IV. MA'!AB13,0)</f>
       </c>
     </row>
     <row r="71">
       <c r="BR71" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS71" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT71" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="BU71" t="str">
-        <f>=IFERROR('IV. MA'!AI16,0)</f>
+        <f>=IFERROR('IV. MA'!AA14,0)</f>
       </c>
       <c r="BV71" t="str">
-        <f>=IFERROR('IV. MA'!AJ16,0)</f>
+        <f>=IFERROR('IV. MA'!AB14,0)</f>
       </c>
     </row>
     <row r="72">
       <c r="BR72" t="str">
-        <f>=$BB$9</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS72" t="str">
-        <f>=$BD$9</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT72" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="BU72" t="str">
-        <f>=IFERROR('IV. MA'!AI17,0)</f>
+        <f>=IFERROR('IV. MA'!AA15,0)</f>
       </c>
       <c r="BV72" t="str">
-        <f>=IFERROR('IV. MA'!AJ17,0)</f>
+        <f>=IFERROR('IV. MA'!AB15,0)</f>
       </c>
     </row>
     <row r="73">
       <c r="BR73" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS73" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT73" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="BU73" t="str">
-        <f>=IFERROR('IV. MA'!AM10,0)</f>
+        <f>=IFERROR('IV. MA'!AA16,0)</f>
       </c>
       <c r="BV73" t="str">
-        <f>=IFERROR('IV. MA'!AN10,0)</f>
+        <f>=IFERROR('IV. MA'!AB16,0)</f>
       </c>
     </row>
     <row r="74">
       <c r="BR74" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS74" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT74" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="BU74" t="str">
-        <f>=IFERROR('IV. MA'!AM11,0)</f>
+        <f>=IFERROR('IV. MA'!AA17,0)</f>
       </c>
       <c r="BV74" t="str">
-        <f>=IFERROR('IV. MA'!AN11,0)</f>
+        <f>=IFERROR('IV. MA'!AB17,0)</f>
       </c>
     </row>
     <row r="75">
       <c r="BR75" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS75" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT75" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="BU75" t="str">
-        <f>=IFERROR('IV. MA'!AM12,0)</f>
+        <f>=IFERROR('IV. MA'!AA21,0)</f>
       </c>
       <c r="BV75" t="str">
-        <f>=IFERROR('IV. MA'!AN12,0)</f>
+        <f>=IFERROR('IV. MA'!AB21,0)</f>
       </c>
     </row>
     <row r="76">
       <c r="BR76" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS76" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT76" t="s">
-        <v>208</v>
+        <v>279</v>
       </c>
       <c r="BU76" t="str">
-        <f>=IFERROR('IV. MA'!AM13,0)</f>
+        <f>=IFERROR('IV. MA'!AA22,0)</f>
       </c>
       <c r="BV76" t="str">
-        <f>=IFERROR('IV. MA'!AN13,0)</f>
+        <f>=IFERROR('IV. MA'!AB22,0)</f>
       </c>
     </row>
     <row r="77">
       <c r="BR77" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$7</f>
       </c>
       <c r="BS77" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$7</f>
       </c>
       <c r="BT77" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="BU77" t="str">
-        <f>=IFERROR('IV. MA'!AM14,0)</f>
+        <f>=IFERROR('IV. MA'!AA25,0)</f>
       </c>
       <c r="BV77" t="str">
-        <f>=IFERROR('IV. MA'!AN14,0)</f>
+        <f>=IFERROR('IV. MA'!AB25,0)</f>
       </c>
     </row>
     <row r="78">
       <c r="BR78" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS78" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT78" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="BU78" t="str">
-        <f>=IFERROR('IV. MA'!AM15,0)</f>
+        <f>=IFERROR('IV. MA'!AE10,0)</f>
       </c>
       <c r="BV78" t="str">
-        <f>=IFERROR('IV. MA'!AN15,0)</f>
+        <f>=IFERROR('IV. MA'!AF10,0)</f>
       </c>
     </row>
     <row r="79">
       <c r="BR79" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS79" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT79" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="BU79" t="str">
-        <f>=IFERROR('IV. MA'!AM16,0)</f>
+        <f>=IFERROR('IV. MA'!AE11,0)</f>
       </c>
       <c r="BV79" t="str">
-        <f>=IFERROR('IV. MA'!AN16,0)</f>
+        <f>=IFERROR('IV. MA'!AF11,0)</f>
       </c>
     </row>
     <row r="80">
       <c r="BR80" t="str">
-        <f>=$BB$10</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS80" t="str">
-        <f>=$BD$10</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT80" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="BU80" t="str">
-        <f>=IFERROR('IV. MA'!AM17,0)</f>
+        <f>=IFERROR('IV. MA'!AE12,0)</f>
       </c>
       <c r="BV80" t="str">
-        <f>=IFERROR('IV. MA'!AN17,0)</f>
+        <f>=IFERROR('IV. MA'!AF12,0)</f>
       </c>
     </row>
     <row r="81">
       <c r="BR81" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS81" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT81" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="BU81" t="str">
-        <f>=IFERROR('IV. MA'!AQ10,0)</f>
+        <f>=IFERROR('IV. MA'!AE13,0)</f>
       </c>
       <c r="BV81" t="str">
-        <f>=IFERROR('IV. MA'!AR10,0)</f>
+        <f>=IFERROR('IV. MA'!AF13,0)</f>
       </c>
     </row>
     <row r="82">
       <c r="BR82" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS82" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT82" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="BU82" t="str">
-        <f>=IFERROR('IV. MA'!AQ11,0)</f>
+        <f>=IFERROR('IV. MA'!AE14,0)</f>
       </c>
       <c r="BV82" t="str">
-        <f>=IFERROR('IV. MA'!AR11,0)</f>
+        <f>=IFERROR('IV. MA'!AF14,0)</f>
       </c>
     </row>
     <row r="83">
       <c r="BR83" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS83" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT83" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="BU83" t="str">
-        <f>=IFERROR('IV. MA'!AQ12,0)</f>
+        <f>=IFERROR('IV. MA'!AE15,0)</f>
       </c>
       <c r="BV83" t="str">
-        <f>=IFERROR('IV. MA'!AR12,0)</f>
+        <f>=IFERROR('IV. MA'!AF15,0)</f>
       </c>
     </row>
     <row r="84">
       <c r="BR84" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS84" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT84" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="BU84" t="str">
-        <f>=IFERROR('IV. MA'!AQ13,0)</f>
+        <f>=IFERROR('IV. MA'!AE16,0)</f>
       </c>
       <c r="BV84" t="str">
-        <f>=IFERROR('IV. MA'!AR13,0)</f>
+        <f>=IFERROR('IV. MA'!AF16,0)</f>
       </c>
     </row>
     <row r="85">
       <c r="BR85" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS85" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT85" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="BU85" t="str">
-        <f>=IFERROR('IV. MA'!AQ14,0)</f>
+        <f>=IFERROR('IV. MA'!AE17,0)</f>
       </c>
       <c r="BV85" t="str">
-        <f>=IFERROR('IV. MA'!AR14,0)</f>
+        <f>=IFERROR('IV. MA'!AF17,0)</f>
       </c>
     </row>
     <row r="86">
       <c r="BR86" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS86" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT86" t="s">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="BU86" t="str">
-        <f>=IFERROR('IV. MA'!AQ15,0)</f>
+        <f>=IFERROR('IV. MA'!AE21,0)</f>
       </c>
       <c r="BV86" t="str">
-        <f>=IFERROR('IV. MA'!AR15,0)</f>
+        <f>=IFERROR('IV. MA'!AF21,0)</f>
       </c>
     </row>
     <row r="87">
       <c r="BR87" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS87" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT87" t="s">
-        <v>211</v>
+        <v>279</v>
       </c>
       <c r="BU87" t="str">
-        <f>=IFERROR('IV. MA'!AQ16,0)</f>
+        <f>=IFERROR('IV. MA'!AE22,0)</f>
       </c>
       <c r="BV87" t="str">
-        <f>=IFERROR('IV. MA'!AR16,0)</f>
+        <f>=IFERROR('IV. MA'!AF22,0)</f>
       </c>
     </row>
     <row r="88">
       <c r="BR88" t="str">
-        <f>=$BB$11</f>
+        <f>=$BB$8</f>
       </c>
       <c r="BS88" t="str">
-        <f>=$BD$11</f>
+        <f>=$BD$8</f>
       </c>
       <c r="BT88" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="BU88" t="str">
-        <f>=IFERROR('IV. MA'!AQ17,0)</f>
+        <f>=IFERROR('IV. MA'!AE25,0)</f>
       </c>
       <c r="BV88" t="str">
-        <f>=IFERROR('IV. MA'!AR17,0)</f>
+        <f>=IFERROR('IV. MA'!AF25,0)</f>
       </c>
     </row>
     <row r="89">
       <c r="BR89" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS89" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT89" t="s">
         <v>205</v>
       </c>
       <c r="BU89" t="str">
-        <f>=IFERROR('IV. MA'!AU10,0)</f>
+        <f>=IFERROR('IV. MA'!AI10,0)</f>
       </c>
       <c r="BV89" t="str">
-        <f>=IFERROR('IV. MA'!AV10,0)</f>
+        <f>=IFERROR('IV. MA'!AJ10,0)</f>
       </c>
     </row>
     <row r="90">
       <c r="BR90" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS90" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT90" t="s">
         <v>206</v>
       </c>
       <c r="BU90" t="str">
-        <f>=IFERROR('IV. MA'!AU11,0)</f>
+        <f>=IFERROR('IV. MA'!AI11,0)</f>
       </c>
       <c r="BV90" t="str">
-        <f>=IFERROR('IV. MA'!AV11,0)</f>
+        <f>=IFERROR('IV. MA'!AJ11,0)</f>
       </c>
     </row>
     <row r="91">
       <c r="BR91" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS91" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT91" t="s">
         <v>207</v>
       </c>
       <c r="BU91" t="str">
-        <f>=IFERROR('IV. MA'!AU12,0)</f>
+        <f>=IFERROR('IV. MA'!AI12,0)</f>
       </c>
       <c r="BV91" t="str">
-        <f>=IFERROR('IV. MA'!AV12,0)</f>
+        <f>=IFERROR('IV. MA'!AJ12,0)</f>
       </c>
     </row>
     <row r="92">
       <c r="BR92" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS92" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT92" t="s">
         <v>208</v>
       </c>
       <c r="BU92" t="str">
-        <f>=IFERROR('IV. MA'!AU13,0)</f>
+        <f>=IFERROR('IV. MA'!AI13,0)</f>
       </c>
       <c r="BV92" t="str">
-        <f>=IFERROR('IV. MA'!AV13,0)</f>
+        <f>=IFERROR('IV. MA'!AJ13,0)</f>
       </c>
     </row>
     <row r="93">
       <c r="BR93" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS93" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT93" t="s">
         <v>209</v>
       </c>
       <c r="BU93" t="str">
-        <f>=IFERROR('IV. MA'!AU14,0)</f>
+        <f>=IFERROR('IV. MA'!AI14,0)</f>
       </c>
       <c r="BV93" t="str">
-        <f>=IFERROR('IV. MA'!AV14,0)</f>
+        <f>=IFERROR('IV. MA'!AJ14,0)</f>
       </c>
     </row>
     <row r="94">
       <c r="BR94" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS94" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT94" t="s">
         <v>210</v>
       </c>
       <c r="BU94" t="str">
-        <f>=IFERROR('IV. MA'!AU15,0)</f>
+        <f>=IFERROR('IV. MA'!AI15,0)</f>
       </c>
       <c r="BV94" t="str">
-        <f>=IFERROR('IV. MA'!AV15,0)</f>
+        <f>=IFERROR('IV. MA'!AJ15,0)</f>
       </c>
     </row>
     <row r="95">
       <c r="BR95" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS95" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT95" t="s">
         <v>211</v>
       </c>
       <c r="BU95" t="str">
-        <f>=IFERROR('IV. MA'!AU16,0)</f>
+        <f>=IFERROR('IV. MA'!AI16,0)</f>
       </c>
       <c r="BV95" t="str">
-        <f>=IFERROR('IV. MA'!AV16,0)</f>
+        <f>=IFERROR('IV. MA'!AJ16,0)</f>
       </c>
     </row>
     <row r="96">
       <c r="BR96" t="str">
-        <f>=$BB$12</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS96" t="str">
-        <f>=$BD$12</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT96" t="s">
         <v>212</v>
       </c>
       <c r="BU96" t="str">
-        <f>=IFERROR('IV. MA'!AU17,0)</f>
+        <f>=IFERROR('IV. MA'!AI17,0)</f>
       </c>
       <c r="BV96" t="str">
-        <f>=IFERROR('IV. MA'!AV17,0)</f>
+        <f>=IFERROR('IV. MA'!AJ17,0)</f>
       </c>
     </row>
     <row r="97">
       <c r="BR97" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS97" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT97" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="BU97" t="str">
-        <f>=IFERROR('IV. MA'!AY10,0)</f>
+        <f>=IFERROR('IV. MA'!AI21,0)</f>
       </c>
       <c r="BV97" t="str">
-        <f>=IFERROR('IV. MA'!AZ10,0)</f>
+        <f>=IFERROR('IV. MA'!AJ21,0)</f>
       </c>
     </row>
     <row r="98">
       <c r="BR98" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS98" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT98" t="s">
-        <v>206</v>
+        <v>279</v>
       </c>
       <c r="BU98" t="str">
-        <f>=IFERROR('IV. MA'!AY11,0)</f>
+        <f>=IFERROR('IV. MA'!AI22,0)</f>
       </c>
       <c r="BV98" t="str">
-        <f>=IFERROR('IV. MA'!AZ11,0)</f>
+        <f>=IFERROR('IV. MA'!AJ22,0)</f>
       </c>
     </row>
     <row r="99">
       <c r="BR99" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$9</f>
       </c>
       <c r="BS99" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$9</f>
       </c>
       <c r="BT99" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="BU99" t="str">
-        <f>=IFERROR('IV. MA'!AY12,0)</f>
+        <f>=IFERROR('IV. MA'!AI25,0)</f>
       </c>
       <c r="BV99" t="str">
-        <f>=IFERROR('IV. MA'!AZ12,0)</f>
+        <f>=IFERROR('IV. MA'!AJ25,0)</f>
       </c>
     </row>
     <row r="100">
       <c r="BR100" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS100" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT100" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="BU100" t="str">
-        <f>=IFERROR('IV. MA'!AY13,0)</f>
+        <f>=IFERROR('IV. MA'!AM10,0)</f>
       </c>
       <c r="BV100" t="str">
-        <f>=IFERROR('IV. MA'!AZ13,0)</f>
+        <f>=IFERROR('IV. MA'!AN10,0)</f>
       </c>
     </row>
     <row r="101">
       <c r="BR101" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS101" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT101" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="BU101" t="str">
-        <f>=IFERROR('IV. MA'!AY14,0)</f>
+        <f>=IFERROR('IV. MA'!AM11,0)</f>
       </c>
       <c r="BV101" t="str">
-        <f>=IFERROR('IV. MA'!AZ14,0)</f>
+        <f>=IFERROR('IV. MA'!AN11,0)</f>
       </c>
     </row>
     <row r="102">
       <c r="BR102" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS102" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT102" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="BU102" t="str">
-        <f>=IFERROR('IV. MA'!AY15,0)</f>
+        <f>=IFERROR('IV. MA'!AM12,0)</f>
       </c>
       <c r="BV102" t="str">
-        <f>=IFERROR('IV. MA'!AZ15,0)</f>
+        <f>=IFERROR('IV. MA'!AN12,0)</f>
       </c>
     </row>
     <row r="103">
       <c r="BR103" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS103" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT103" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="BU103" t="str">
-        <f>=IFERROR('IV. MA'!AY16,0)</f>
+        <f>=IFERROR('IV. MA'!AM13,0)</f>
       </c>
       <c r="BV103" t="str">
-        <f>=IFERROR('IV. MA'!AZ16,0)</f>
+        <f>=IFERROR('IV. MA'!AN13,0)</f>
       </c>
     </row>
     <row r="104">
       <c r="BR104" t="str">
-        <f>=$BB$13</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS104" t="str">
-        <f>=$BD$13</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT104" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="BU104" t="str">
-        <f>=IFERROR('IV. MA'!AY17,0)</f>
+        <f>=IFERROR('IV. MA'!AM14,0)</f>
       </c>
       <c r="BV104" t="str">
-        <f>=IFERROR('IV. MA'!AZ17,0)</f>
+        <f>=IFERROR('IV. MA'!AN14,0)</f>
       </c>
     </row>
     <row r="105">
       <c r="BR105" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS105" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT105" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="BU105" t="str">
-        <f>=IFERROR('IV. MA'!BC10,0)</f>
+        <f>=IFERROR('IV. MA'!AM15,0)</f>
       </c>
       <c r="BV105" t="str">
-        <f>=IFERROR('IV. MA'!BD10,0)</f>
+        <f>=IFERROR('IV. MA'!AN15,0)</f>
       </c>
     </row>
     <row r="106">
       <c r="BR106" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS106" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT106" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="BU106" t="str">
-        <f>=IFERROR('IV. MA'!BC11,0)</f>
+        <f>=IFERROR('IV. MA'!AM16,0)</f>
       </c>
       <c r="BV106" t="str">
-        <f>=IFERROR('IV. MA'!BD11,0)</f>
+        <f>=IFERROR('IV. MA'!AN16,0)</f>
       </c>
     </row>
     <row r="107">
       <c r="BR107" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS107" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT107" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="BU107" t="str">
-        <f>=IFERROR('IV. MA'!BC12,0)</f>
+        <f>=IFERROR('IV. MA'!AM17,0)</f>
       </c>
       <c r="BV107" t="str">
-        <f>=IFERROR('IV. MA'!BD12,0)</f>
+        <f>=IFERROR('IV. MA'!AN17,0)</f>
       </c>
     </row>
     <row r="108">
       <c r="BR108" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS108" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT108" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="BU108" t="str">
-        <f>=IFERROR('IV. MA'!BC13,0)</f>
+        <f>=IFERROR('IV. MA'!AM21,0)</f>
       </c>
       <c r="BV108" t="str">
-        <f>=IFERROR('IV. MA'!BD13,0)</f>
+        <f>=IFERROR('IV. MA'!AN21,0)</f>
       </c>
     </row>
     <row r="109">
       <c r="BR109" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS109" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT109" t="s">
-        <v>209</v>
+        <v>279</v>
       </c>
       <c r="BU109" t="str">
-        <f>=IFERROR('IV. MA'!BC14,0)</f>
+        <f>=IFERROR('IV. MA'!AM22,0)</f>
       </c>
       <c r="BV109" t="str">
-        <f>=IFERROR('IV. MA'!BD14,0)</f>
+        <f>=IFERROR('IV. MA'!AN22,0)</f>
       </c>
     </row>
     <row r="110">
       <c r="BR110" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$10</f>
       </c>
       <c r="BS110" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$10</f>
       </c>
       <c r="BT110" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="BU110" t="str">
-        <f>=IFERROR('IV. MA'!BC15,0)</f>
+        <f>=IFERROR('IV. MA'!AM25,0)</f>
       </c>
       <c r="BV110" t="str">
-        <f>=IFERROR('IV. MA'!BD15,0)</f>
+        <f>=IFERROR('IV. MA'!AN25,0)</f>
       </c>
     </row>
     <row r="111">
       <c r="BR111" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS111" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT111" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="BU111" t="str">
-        <f>=IFERROR('IV. MA'!BC16,0)</f>
+        <f>=IFERROR('IV. MA'!AQ10,0)</f>
       </c>
       <c r="BV111" t="str">
-        <f>=IFERROR('IV. MA'!BD16,0)</f>
+        <f>=IFERROR('IV. MA'!AR10,0)</f>
       </c>
     </row>
     <row r="112">
       <c r="BR112" t="str">
-        <f>=$BB$14</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS112" t="str">
-        <f>=$BD$14</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT112" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="BU112" t="str">
-        <f>=IFERROR('IV. MA'!BC17,0)</f>
+        <f>=IFERROR('IV. MA'!AQ11,0)</f>
       </c>
       <c r="BV112" t="str">
-        <f>=IFERROR('IV. MA'!BD17,0)</f>
+        <f>=IFERROR('IV. MA'!AR11,0)</f>
       </c>
     </row>
     <row r="113">
       <c r="BR113" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS113" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT113" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="BU113" t="str">
-        <f>=IFERROR('IV. MA'!BG10,0)</f>
+        <f>=IFERROR('IV. MA'!AQ12,0)</f>
       </c>
       <c r="BV113" t="str">
-        <f>=IFERROR('IV. MA'!BH10,0)</f>
+        <f>=IFERROR('IV. MA'!AR12,0)</f>
       </c>
     </row>
     <row r="114">
       <c r="BR114" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS114" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT114" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="BU114" t="str">
-        <f>=IFERROR('IV. MA'!BG11,0)</f>
+        <f>=IFERROR('IV. MA'!AQ13,0)</f>
       </c>
       <c r="BV114" t="str">
-        <f>=IFERROR('IV. MA'!BH11,0)</f>
+        <f>=IFERROR('IV. MA'!AR13,0)</f>
       </c>
     </row>
     <row r="115">
       <c r="BR115" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS115" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT115" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="BU115" t="str">
-        <f>=IFERROR('IV. MA'!BG12,0)</f>
+        <f>=IFERROR('IV. MA'!AQ14,0)</f>
       </c>
       <c r="BV115" t="str">
-        <f>=IFERROR('IV. MA'!BH12,0)</f>
+        <f>=IFERROR('IV. MA'!AR14,0)</f>
       </c>
     </row>
     <row r="116">
       <c r="BR116" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS116" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT116" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="BU116" t="str">
-        <f>=IFERROR('IV. MA'!BG13,0)</f>
+        <f>=IFERROR('IV. MA'!AQ15,0)</f>
       </c>
       <c r="BV116" t="str">
-        <f>=IFERROR('IV. MA'!BH13,0)</f>
+        <f>=IFERROR('IV. MA'!AR15,0)</f>
       </c>
     </row>
     <row r="117">
       <c r="BR117" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS117" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT117" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="BU117" t="str">
-        <f>=IFERROR('IV. MA'!BG14,0)</f>
+        <f>=IFERROR('IV. MA'!AQ16,0)</f>
       </c>
       <c r="BV117" t="str">
-        <f>=IFERROR('IV. MA'!BH14,0)</f>
+        <f>=IFERROR('IV. MA'!AR16,0)</f>
       </c>
     </row>
     <row r="118">
       <c r="BR118" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS118" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT118" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="BU118" t="str">
-        <f>=IFERROR('IV. MA'!BG15,0)</f>
+        <f>=IFERROR('IV. MA'!AQ17,0)</f>
       </c>
       <c r="BV118" t="str">
-        <f>=IFERROR('IV. MA'!BH15,0)</f>
+        <f>=IFERROR('IV. MA'!AR17,0)</f>
       </c>
     </row>
     <row r="119">
       <c r="BR119" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS119" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT119" t="s">
-        <v>211</v>
+        <v>194</v>
       </c>
       <c r="BU119" t="str">
-        <f>=IFERROR('IV. MA'!BG16,0)</f>
+        <f>=IFERROR('IV. MA'!AQ21,0)</f>
       </c>
       <c r="BV119" t="str">
-        <f>=IFERROR('IV. MA'!BH16,0)</f>
+        <f>=IFERROR('IV. MA'!AR21,0)</f>
       </c>
     </row>
     <row r="120">
       <c r="BR120" t="str">
-        <f>=$BB$15</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS120" t="str">
-        <f>=$BD$15</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT120" t="s">
-        <v>212</v>
+        <v>279</v>
       </c>
       <c r="BU120" t="str">
-        <f>=IFERROR('IV. MA'!BG17,0)</f>
+        <f>=IFERROR('IV. MA'!AQ22,0)</f>
       </c>
       <c r="BV120" t="str">
-        <f>=IFERROR('IV. MA'!BH17,0)</f>
+        <f>=IFERROR('IV. MA'!AR22,0)</f>
       </c>
     </row>
     <row r="121">
       <c r="BR121" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$11</f>
       </c>
       <c r="BS121" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$11</f>
       </c>
       <c r="BT121" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="BU121" t="str">
-        <f>=IFERROR('IV. MA'!BK10,0)</f>
+        <f>=IFERROR('IV. MA'!AQ25,0)</f>
       </c>
       <c r="BV121" t="str">
-        <f>=IFERROR('IV. MA'!BL10,0)</f>
+        <f>=IFERROR('IV. MA'!AR25,0)</f>
       </c>
     </row>
     <row r="122">
       <c r="BR122" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS122" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT122" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="BU122" t="str">
-        <f>=IFERROR('IV. MA'!BK11,0)</f>
+        <f>=IFERROR('IV. MA'!AU10,0)</f>
       </c>
       <c r="BV122" t="str">
-        <f>=IFERROR('IV. MA'!BL11,0)</f>
+        <f>=IFERROR('IV. MA'!AV10,0)</f>
       </c>
     </row>
     <row r="123">
       <c r="BR123" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS123" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT123" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="BU123" t="str">
-        <f>=IFERROR('IV. MA'!BK12,0)</f>
+        <f>=IFERROR('IV. MA'!AU11,0)</f>
       </c>
       <c r="BV123" t="str">
-        <f>=IFERROR('IV. MA'!BL12,0)</f>
+        <f>=IFERROR('IV. MA'!AV11,0)</f>
       </c>
     </row>
     <row r="124">
       <c r="BR124" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS124" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT124" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BU124" t="str">
-        <f>=IFERROR('IV. MA'!BK13,0)</f>
+        <f>=IFERROR('IV. MA'!AU12,0)</f>
       </c>
       <c r="BV124" t="str">
-        <f>=IFERROR('IV. MA'!BL13,0)</f>
+        <f>=IFERROR('IV. MA'!AV12,0)</f>
       </c>
     </row>
     <row r="125">
       <c r="BR125" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS125" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT125" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="BU125" t="str">
-        <f>=IFERROR('IV. MA'!BK14,0)</f>
+        <f>=IFERROR('IV. MA'!AU13,0)</f>
       </c>
       <c r="BV125" t="str">
-        <f>=IFERROR('IV. MA'!BL14,0)</f>
+        <f>=IFERROR('IV. MA'!AV13,0)</f>
       </c>
     </row>
     <row r="126">
       <c r="BR126" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS126" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT126" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="BU126" t="str">
-        <f>=IFERROR('IV. MA'!BK15,0)</f>
+        <f>=IFERROR('IV. MA'!AU14,0)</f>
       </c>
       <c r="BV126" t="str">
-        <f>=IFERROR('IV. MA'!BL15,0)</f>
+        <f>=IFERROR('IV. MA'!AV14,0)</f>
       </c>
     </row>
     <row r="127">
       <c r="BR127" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS127" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT127" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="BU127" t="str">
-        <f>=IFERROR('IV. MA'!BK16,0)</f>
+        <f>=IFERROR('IV. MA'!AU15,0)</f>
       </c>
       <c r="BV127" t="str">
-        <f>=IFERROR('IV. MA'!BL16,0)</f>
+        <f>=IFERROR('IV. MA'!AV15,0)</f>
       </c>
     </row>
     <row r="128">
       <c r="BR128" t="str">
-        <f>=$BB$16</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS128" t="str">
-        <f>=$BD$16</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT128" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="BU128" t="str">
-        <f>=IFERROR('IV. MA'!BK17,0)</f>
+        <f>=IFERROR('IV. MA'!AU16,0)</f>
       </c>
       <c r="BV128" t="str">
-        <f>=IFERROR('IV. MA'!BL17,0)</f>
+        <f>=IFERROR('IV. MA'!AV16,0)</f>
       </c>
     </row>
     <row r="129">
       <c r="BR129" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS129" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT129" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="BU129" t="str">
-        <f>=IFERROR('IV. MA'!BO10,0)</f>
+        <f>=IFERROR('IV. MA'!AU17,0)</f>
       </c>
       <c r="BV129" t="str">
-        <f>=IFERROR('IV. MA'!BP10,0)</f>
+        <f>=IFERROR('IV. MA'!AV17,0)</f>
       </c>
     </row>
     <row r="130">
       <c r="BR130" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS130" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT130" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="BU130" t="str">
-        <f>=IFERROR('IV. MA'!BO11,0)</f>
+        <f>=IFERROR('IV. MA'!AU21,0)</f>
       </c>
       <c r="BV130" t="str">
-        <f>=IFERROR('IV. MA'!BP11,0)</f>
+        <f>=IFERROR('IV. MA'!AV21,0)</f>
       </c>
     </row>
     <row r="131">
       <c r="BR131" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS131" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT131" t="s">
-        <v>207</v>
+        <v>279</v>
       </c>
       <c r="BU131" t="str">
-        <f>=IFERROR('IV. MA'!BO12,0)</f>
+        <f>=IFERROR('IV. MA'!AU22,0)</f>
       </c>
       <c r="BV131" t="str">
-        <f>=IFERROR('IV. MA'!BP12,0)</f>
+        <f>=IFERROR('IV. MA'!AV22,0)</f>
       </c>
     </row>
     <row r="132">
       <c r="BR132" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$12</f>
       </c>
       <c r="BS132" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$12</f>
       </c>
       <c r="BT132" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="BU132" t="str">
-        <f>=IFERROR('IV. MA'!BO13,0)</f>
+        <f>=IFERROR('IV. MA'!AU25,0)</f>
       </c>
       <c r="BV132" t="str">
-        <f>=IFERROR('IV. MA'!BP13,0)</f>
+        <f>=IFERROR('IV. MA'!AV25,0)</f>
       </c>
     </row>
     <row r="133">
       <c r="BR133" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS133" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT133" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="BU133" t="str">
-        <f>=IFERROR('IV. MA'!BO14,0)</f>
+        <f>=IFERROR('IV. MA'!AY10,0)</f>
       </c>
       <c r="BV133" t="str">
-        <f>=IFERROR('IV. MA'!BP14,0)</f>
+        <f>=IFERROR('IV. MA'!AZ10,0)</f>
       </c>
     </row>
     <row r="134">
       <c r="BR134" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS134" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT134" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="BU134" t="str">
-        <f>=IFERROR('IV. MA'!BO15,0)</f>
+        <f>=IFERROR('IV. MA'!AY11,0)</f>
       </c>
       <c r="BV134" t="str">
-        <f>=IFERROR('IV. MA'!BP15,0)</f>
+        <f>=IFERROR('IV. MA'!AZ11,0)</f>
       </c>
     </row>
     <row r="135">
       <c r="BR135" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS135" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT135" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="BU135" t="str">
-        <f>=IFERROR('IV. MA'!BO16,0)</f>
+        <f>=IFERROR('IV. MA'!AY12,0)</f>
       </c>
       <c r="BV135" t="str">
-        <f>=IFERROR('IV. MA'!BP16,0)</f>
+        <f>=IFERROR('IV. MA'!AZ12,0)</f>
       </c>
     </row>
     <row r="136">
       <c r="BR136" t="str">
-        <f>=$BB$17</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS136" t="str">
-        <f>=$BD$17</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT136" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="BU136" t="str">
-        <f>=IFERROR('IV. MA'!BO17,0)</f>
+        <f>=IFERROR('IV. MA'!AY13,0)</f>
       </c>
       <c r="BV136" t="str">
-        <f>=IFERROR('IV. MA'!BP17,0)</f>
+        <f>=IFERROR('IV. MA'!AZ13,0)</f>
       </c>
     </row>
     <row r="137">
       <c r="BR137" t="str">
-        <f>=$BB$18</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS137" t="str">
-        <f>=$BD$18</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT137" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="BU137" t="str">
-        <f>=IFERROR('IV. MA'!BS10,0)</f>
+        <f>=IFERROR('IV. MA'!AY14,0)</f>
       </c>
       <c r="BV137" t="str">
-        <f>=IFERROR('IV. MA'!BT10,0)</f>
+        <f>=IFERROR('IV. MA'!AZ14,0)</f>
       </c>
     </row>
     <row r="138">
       <c r="BR138" t="str">
-        <f>=$BB$18</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS138" t="str">
-        <f>=$BD$18</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT138" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="BU138" t="str">
-        <f>=IFERROR('IV. MA'!BS11,0)</f>
+        <f>=IFERROR('IV. MA'!AY15,0)</f>
       </c>
       <c r="BV138" t="str">
-        <f>=IFERROR('IV. MA'!BT11,0)</f>
+        <f>=IFERROR('IV. MA'!AZ15,0)</f>
       </c>
     </row>
     <row r="139">
       <c r="BR139" t="str">
-        <f>=$BB$18</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS139" t="str">
-        <f>=$BD$18</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT139" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="BU139" t="str">
-        <f>=IFERROR('IV. MA'!BS12,0)</f>
+        <f>=IFERROR('IV. MA'!AY16,0)</f>
       </c>
       <c r="BV139" t="str">
-        <f>=IFERROR('IV. MA'!BT12,0)</f>
+        <f>=IFERROR('IV. MA'!AZ16,0)</f>
       </c>
     </row>
     <row r="140">
       <c r="BR140" t="str">
-        <f>=$BB$18</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS140" t="str">
-        <f>=$BD$18</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT140" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="BU140" t="str">
-        <f>=IFERROR('IV. MA'!BS13,0)</f>
+        <f>=IFERROR('IV. MA'!AY17,0)</f>
       </c>
       <c r="BV140" t="str">
-        <f>=IFERROR('IV. MA'!BT13,0)</f>
+        <f>=IFERROR('IV. MA'!AZ17,0)</f>
       </c>
     </row>
     <row r="141">
       <c r="BR141" t="str">
-        <f>=$BB$18</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS141" t="str">
-        <f>=$BD$18</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT141" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="BU141" t="str">
-        <f>=IFERROR('IV. MA'!BS14,0)</f>
+        <f>=IFERROR('IV. MA'!AY21,0)</f>
       </c>
       <c r="BV141" t="str">
-        <f>=IFERROR('IV. MA'!BT14,0)</f>
+        <f>=IFERROR('IV. MA'!AZ21,0)</f>
       </c>
     </row>
     <row r="142">
       <c r="BR142" t="str">
-        <f>=$BB$18</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS142" t="str">
-        <f>=$BD$18</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT142" t="s">
-        <v>210</v>
+        <v>279</v>
       </c>
       <c r="BU142" t="str">
-        <f>=IFERROR('IV. MA'!BS15,0)</f>
+        <f>=IFERROR('IV. MA'!AY22,0)</f>
       </c>
       <c r="BV142" t="str">
-        <f>=IFERROR('IV. MA'!BT15,0)</f>
+        <f>=IFERROR('IV. MA'!AZ22,0)</f>
       </c>
     </row>
     <row r="143">
       <c r="BR143" t="str">
-        <f>=$BB$18</f>
+        <f>=$BB$13</f>
       </c>
       <c r="BS143" t="str">
-        <f>=$BD$18</f>
+        <f>=$BD$13</f>
       </c>
       <c r="BT143" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="BU143" t="str">
-        <f>=IFERROR('IV. MA'!BS16,0)</f>
+        <f>=IFERROR('IV. MA'!AY25,0)</f>
       </c>
       <c r="BV143" t="str">
-        <f>=IFERROR('IV. MA'!BT16,0)</f>
+        <f>=IFERROR('IV. MA'!AZ25,0)</f>
       </c>
     </row>
     <row r="144">
       <c r="BR144" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS144" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT144" t="s">
+        <v>205</v>
+      </c>
+      <c r="BU144" t="str">
+        <f>=IFERROR('IV. MA'!BC10,0)</f>
+      </c>
+      <c r="BV144" t="str">
+        <f>=IFERROR('IV. MA'!BD10,0)</f>
+      </c>
+    </row>
+    <row r="145">
+      <c r="BR145" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS145" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT145" t="s">
+        <v>206</v>
+      </c>
+      <c r="BU145" t="str">
+        <f>=IFERROR('IV. MA'!BC11,0)</f>
+      </c>
+      <c r="BV145" t="str">
+        <f>=IFERROR('IV. MA'!BD11,0)</f>
+      </c>
+    </row>
+    <row r="146">
+      <c r="BR146" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS146" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT146" t="s">
+        <v>207</v>
+      </c>
+      <c r="BU146" t="str">
+        <f>=IFERROR('IV. MA'!BC12,0)</f>
+      </c>
+      <c r="BV146" t="str">
+        <f>=IFERROR('IV. MA'!BD12,0)</f>
+      </c>
+    </row>
+    <row r="147">
+      <c r="BR147" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS147" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT147" t="s">
+        <v>208</v>
+      </c>
+      <c r="BU147" t="str">
+        <f>=IFERROR('IV. MA'!BC13,0)</f>
+      </c>
+      <c r="BV147" t="str">
+        <f>=IFERROR('IV. MA'!BD13,0)</f>
+      </c>
+    </row>
+    <row r="148">
+      <c r="BR148" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS148" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT148" t="s">
+        <v>209</v>
+      </c>
+      <c r="BU148" t="str">
+        <f>=IFERROR('IV. MA'!BC14,0)</f>
+      </c>
+      <c r="BV148" t="str">
+        <f>=IFERROR('IV. MA'!BD14,0)</f>
+      </c>
+    </row>
+    <row r="149">
+      <c r="BR149" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS149" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT149" t="s">
+        <v>210</v>
+      </c>
+      <c r="BU149" t="str">
+        <f>=IFERROR('IV. MA'!BC15,0)</f>
+      </c>
+      <c r="BV149" t="str">
+        <f>=IFERROR('IV. MA'!BD15,0)</f>
+      </c>
+    </row>
+    <row r="150">
+      <c r="BR150" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS150" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT150" t="s">
+        <v>211</v>
+      </c>
+      <c r="BU150" t="str">
+        <f>=IFERROR('IV. MA'!BC16,0)</f>
+      </c>
+      <c r="BV150" t="str">
+        <f>=IFERROR('IV. MA'!BD16,0)</f>
+      </c>
+    </row>
+    <row r="151">
+      <c r="BR151" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS151" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT151" t="s">
+        <v>212</v>
+      </c>
+      <c r="BU151" t="str">
+        <f>=IFERROR('IV. MA'!BC17,0)</f>
+      </c>
+      <c r="BV151" t="str">
+        <f>=IFERROR('IV. MA'!BD17,0)</f>
+      </c>
+    </row>
+    <row r="152">
+      <c r="BR152" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS152" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT152" t="s">
+        <v>194</v>
+      </c>
+      <c r="BU152" t="str">
+        <f>=IFERROR('IV. MA'!BC21,0)</f>
+      </c>
+      <c r="BV152" t="str">
+        <f>=IFERROR('IV. MA'!BD21,0)</f>
+      </c>
+    </row>
+    <row r="153">
+      <c r="BR153" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS153" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT153" t="s">
+        <v>279</v>
+      </c>
+      <c r="BU153" t="str">
+        <f>=IFERROR('IV. MA'!BC22,0)</f>
+      </c>
+      <c r="BV153" t="str">
+        <f>=IFERROR('IV. MA'!BD22,0)</f>
+      </c>
+    </row>
+    <row r="154">
+      <c r="BR154" t="str">
+        <f>=$BB$14</f>
+      </c>
+      <c r="BS154" t="str">
+        <f>=$BD$14</f>
+      </c>
+      <c r="BT154" t="s">
+        <v>199</v>
+      </c>
+      <c r="BU154" t="str">
+        <f>=IFERROR('IV. MA'!BC25,0)</f>
+      </c>
+      <c r="BV154" t="str">
+        <f>=IFERROR('IV. MA'!BD25,0)</f>
+      </c>
+    </row>
+    <row r="155">
+      <c r="BR155" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS155" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT155" t="s">
+        <v>205</v>
+      </c>
+      <c r="BU155" t="str">
+        <f>=IFERROR('IV. MA'!BG10,0)</f>
+      </c>
+      <c r="BV155" t="str">
+        <f>=IFERROR('IV. MA'!BH10,0)</f>
+      </c>
+    </row>
+    <row r="156">
+      <c r="BR156" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS156" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT156" t="s">
+        <v>206</v>
+      </c>
+      <c r="BU156" t="str">
+        <f>=IFERROR('IV. MA'!BG11,0)</f>
+      </c>
+      <c r="BV156" t="str">
+        <f>=IFERROR('IV. MA'!BH11,0)</f>
+      </c>
+    </row>
+    <row r="157">
+      <c r="BR157" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS157" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT157" t="s">
+        <v>207</v>
+      </c>
+      <c r="BU157" t="str">
+        <f>=IFERROR('IV. MA'!BG12,0)</f>
+      </c>
+      <c r="BV157" t="str">
+        <f>=IFERROR('IV. MA'!BH12,0)</f>
+      </c>
+    </row>
+    <row r="158">
+      <c r="BR158" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS158" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT158" t="s">
+        <v>208</v>
+      </c>
+      <c r="BU158" t="str">
+        <f>=IFERROR('IV. MA'!BG13,0)</f>
+      </c>
+      <c r="BV158" t="str">
+        <f>=IFERROR('IV. MA'!BH13,0)</f>
+      </c>
+    </row>
+    <row r="159">
+      <c r="BR159" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS159" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT159" t="s">
+        <v>209</v>
+      </c>
+      <c r="BU159" t="str">
+        <f>=IFERROR('IV. MA'!BG14,0)</f>
+      </c>
+      <c r="BV159" t="str">
+        <f>=IFERROR('IV. MA'!BH14,0)</f>
+      </c>
+    </row>
+    <row r="160">
+      <c r="BR160" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS160" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT160" t="s">
+        <v>210</v>
+      </c>
+      <c r="BU160" t="str">
+        <f>=IFERROR('IV. MA'!BG15,0)</f>
+      </c>
+      <c r="BV160" t="str">
+        <f>=IFERROR('IV. MA'!BH15,0)</f>
+      </c>
+    </row>
+    <row r="161">
+      <c r="BR161" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS161" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT161" t="s">
+        <v>211</v>
+      </c>
+      <c r="BU161" t="str">
+        <f>=IFERROR('IV. MA'!BG16,0)</f>
+      </c>
+      <c r="BV161" t="str">
+        <f>=IFERROR('IV. MA'!BH16,0)</f>
+      </c>
+    </row>
+    <row r="162">
+      <c r="BR162" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS162" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT162" t="s">
+        <v>212</v>
+      </c>
+      <c r="BU162" t="str">
+        <f>=IFERROR('IV. MA'!BG17,0)</f>
+      </c>
+      <c r="BV162" t="str">
+        <f>=IFERROR('IV. MA'!BH17,0)</f>
+      </c>
+    </row>
+    <row r="163">
+      <c r="BR163" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS163" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT163" t="s">
+        <v>194</v>
+      </c>
+      <c r="BU163" t="str">
+        <f>=IFERROR('IV. MA'!BG21,0)</f>
+      </c>
+      <c r="BV163" t="str">
+        <f>=IFERROR('IV. MA'!BH21,0)</f>
+      </c>
+    </row>
+    <row r="164">
+      <c r="BR164" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS164" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT164" t="s">
+        <v>279</v>
+      </c>
+      <c r="BU164" t="str">
+        <f>=IFERROR('IV. MA'!BG22,0)</f>
+      </c>
+      <c r="BV164" t="str">
+        <f>=IFERROR('IV. MA'!BH22,0)</f>
+      </c>
+    </row>
+    <row r="165">
+      <c r="BR165" t="str">
+        <f>=$BB$15</f>
+      </c>
+      <c r="BS165" t="str">
+        <f>=$BD$15</f>
+      </c>
+      <c r="BT165" t="s">
+        <v>199</v>
+      </c>
+      <c r="BU165" t="str">
+        <f>=IFERROR('IV. MA'!BG25,0)</f>
+      </c>
+      <c r="BV165" t="str">
+        <f>=IFERROR('IV. MA'!BH25,0)</f>
+      </c>
+    </row>
+    <row r="166">
+      <c r="BR166" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS166" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT166" t="s">
+        <v>205</v>
+      </c>
+      <c r="BU166" t="str">
+        <f>=IFERROR('IV. MA'!BK10,0)</f>
+      </c>
+      <c r="BV166" t="str">
+        <f>=IFERROR('IV. MA'!BL10,0)</f>
+      </c>
+    </row>
+    <row r="167">
+      <c r="BR167" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS167" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT167" t="s">
+        <v>206</v>
+      </c>
+      <c r="BU167" t="str">
+        <f>=IFERROR('IV. MA'!BK11,0)</f>
+      </c>
+      <c r="BV167" t="str">
+        <f>=IFERROR('IV. MA'!BL11,0)</f>
+      </c>
+    </row>
+    <row r="168">
+      <c r="BR168" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS168" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT168" t="s">
+        <v>207</v>
+      </c>
+      <c r="BU168" t="str">
+        <f>=IFERROR('IV. MA'!BK12,0)</f>
+      </c>
+      <c r="BV168" t="str">
+        <f>=IFERROR('IV. MA'!BL12,0)</f>
+      </c>
+    </row>
+    <row r="169">
+      <c r="BR169" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS169" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT169" t="s">
+        <v>208</v>
+      </c>
+      <c r="BU169" t="str">
+        <f>=IFERROR('IV. MA'!BK13,0)</f>
+      </c>
+      <c r="BV169" t="str">
+        <f>=IFERROR('IV. MA'!BL13,0)</f>
+      </c>
+    </row>
+    <row r="170">
+      <c r="BR170" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS170" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT170" t="s">
+        <v>209</v>
+      </c>
+      <c r="BU170" t="str">
+        <f>=IFERROR('IV. MA'!BK14,0)</f>
+      </c>
+      <c r="BV170" t="str">
+        <f>=IFERROR('IV. MA'!BL14,0)</f>
+      </c>
+    </row>
+    <row r="171">
+      <c r="BR171" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS171" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT171" t="s">
+        <v>210</v>
+      </c>
+      <c r="BU171" t="str">
+        <f>=IFERROR('IV. MA'!BK15,0)</f>
+      </c>
+      <c r="BV171" t="str">
+        <f>=IFERROR('IV. MA'!BL15,0)</f>
+      </c>
+    </row>
+    <row r="172">
+      <c r="BR172" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS172" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT172" t="s">
+        <v>211</v>
+      </c>
+      <c r="BU172" t="str">
+        <f>=IFERROR('IV. MA'!BK16,0)</f>
+      </c>
+      <c r="BV172" t="str">
+        <f>=IFERROR('IV. MA'!BL16,0)</f>
+      </c>
+    </row>
+    <row r="173">
+      <c r="BR173" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS173" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT173" t="s">
+        <v>212</v>
+      </c>
+      <c r="BU173" t="str">
+        <f>=IFERROR('IV. MA'!BK17,0)</f>
+      </c>
+      <c r="BV173" t="str">
+        <f>=IFERROR('IV. MA'!BL17,0)</f>
+      </c>
+    </row>
+    <row r="174">
+      <c r="BR174" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS174" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT174" t="s">
+        <v>194</v>
+      </c>
+      <c r="BU174" t="str">
+        <f>=IFERROR('IV. MA'!BK21,0)</f>
+      </c>
+      <c r="BV174" t="str">
+        <f>=IFERROR('IV. MA'!BL21,0)</f>
+      </c>
+    </row>
+    <row r="175">
+      <c r="BR175" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS175" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT175" t="s">
+        <v>279</v>
+      </c>
+      <c r="BU175" t="str">
+        <f>=IFERROR('IV. MA'!BK22,0)</f>
+      </c>
+      <c r="BV175" t="str">
+        <f>=IFERROR('IV. MA'!BL22,0)</f>
+      </c>
+    </row>
+    <row r="176">
+      <c r="BR176" t="str">
+        <f>=$BB$16</f>
+      </c>
+      <c r="BS176" t="str">
+        <f>=$BD$16</f>
+      </c>
+      <c r="BT176" t="s">
+        <v>199</v>
+      </c>
+      <c r="BU176" t="str">
+        <f>=IFERROR('IV. MA'!BK25,0)</f>
+      </c>
+      <c r="BV176" t="str">
+        <f>=IFERROR('IV. MA'!BL25,0)</f>
+      </c>
+    </row>
+    <row r="177">
+      <c r="BR177" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS177" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT177" t="s">
+        <v>205</v>
+      </c>
+      <c r="BU177" t="str">
+        <f>=IFERROR('IV. MA'!BO10,0)</f>
+      </c>
+      <c r="BV177" t="str">
+        <f>=IFERROR('IV. MA'!BP10,0)</f>
+      </c>
+    </row>
+    <row r="178">
+      <c r="BR178" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS178" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT178" t="s">
+        <v>206</v>
+      </c>
+      <c r="BU178" t="str">
+        <f>=IFERROR('IV. MA'!BO11,0)</f>
+      </c>
+      <c r="BV178" t="str">
+        <f>=IFERROR('IV. MA'!BP11,0)</f>
+      </c>
+    </row>
+    <row r="179">
+      <c r="BR179" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS179" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT179" t="s">
+        <v>207</v>
+      </c>
+      <c r="BU179" t="str">
+        <f>=IFERROR('IV. MA'!BO12,0)</f>
+      </c>
+      <c r="BV179" t="str">
+        <f>=IFERROR('IV. MA'!BP12,0)</f>
+      </c>
+    </row>
+    <row r="180">
+      <c r="BR180" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS180" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT180" t="s">
+        <v>208</v>
+      </c>
+      <c r="BU180" t="str">
+        <f>=IFERROR('IV. MA'!BO13,0)</f>
+      </c>
+      <c r="BV180" t="str">
+        <f>=IFERROR('IV. MA'!BP13,0)</f>
+      </c>
+    </row>
+    <row r="181">
+      <c r="BR181" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS181" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT181" t="s">
+        <v>209</v>
+      </c>
+      <c r="BU181" t="str">
+        <f>=IFERROR('IV. MA'!BO14,0)</f>
+      </c>
+      <c r="BV181" t="str">
+        <f>=IFERROR('IV. MA'!BP14,0)</f>
+      </c>
+    </row>
+    <row r="182">
+      <c r="BR182" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS182" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT182" t="s">
+        <v>210</v>
+      </c>
+      <c r="BU182" t="str">
+        <f>=IFERROR('IV. MA'!BO15,0)</f>
+      </c>
+      <c r="BV182" t="str">
+        <f>=IFERROR('IV. MA'!BP15,0)</f>
+      </c>
+    </row>
+    <row r="183">
+      <c r="BR183" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS183" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT183" t="s">
+        <v>211</v>
+      </c>
+      <c r="BU183" t="str">
+        <f>=IFERROR('IV. MA'!BO16,0)</f>
+      </c>
+      <c r="BV183" t="str">
+        <f>=IFERROR('IV. MA'!BP16,0)</f>
+      </c>
+    </row>
+    <row r="184">
+      <c r="BR184" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS184" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT184" t="s">
+        <v>212</v>
+      </c>
+      <c r="BU184" t="str">
+        <f>=IFERROR('IV. MA'!BO17,0)</f>
+      </c>
+      <c r="BV184" t="str">
+        <f>=IFERROR('IV. MA'!BP17,0)</f>
+      </c>
+    </row>
+    <row r="185">
+      <c r="BR185" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS185" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT185" t="s">
+        <v>194</v>
+      </c>
+      <c r="BU185" t="str">
+        <f>=IFERROR('IV. MA'!BO21,0)</f>
+      </c>
+      <c r="BV185" t="str">
+        <f>=IFERROR('IV. MA'!BP21,0)</f>
+      </c>
+    </row>
+    <row r="186">
+      <c r="BR186" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS186" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT186" t="s">
+        <v>279</v>
+      </c>
+      <c r="BU186" t="str">
+        <f>=IFERROR('IV. MA'!BO22,0)</f>
+      </c>
+      <c r="BV186" t="str">
+        <f>=IFERROR('IV. MA'!BP22,0)</f>
+      </c>
+    </row>
+    <row r="187">
+      <c r="BR187" t="str">
+        <f>=$BB$17</f>
+      </c>
+      <c r="BS187" t="str">
+        <f>=$BD$17</f>
+      </c>
+      <c r="BT187" t="s">
+        <v>199</v>
+      </c>
+      <c r="BU187" t="str">
+        <f>=IFERROR('IV. MA'!BO25,0)</f>
+      </c>
+      <c r="BV187" t="str">
+        <f>=IFERROR('IV. MA'!BP25,0)</f>
+      </c>
+    </row>
+    <row r="188">
+      <c r="BR188" t="str">
         <f>=$BB$18</f>
       </c>
-      <c r="BS144" t="str">
+      <c r="BS188" t="str">
         <f>=$BD$18</f>
       </c>
-      <c r="BT144" t="s">
+      <c r="BT188" t="s">
+        <v>205</v>
+      </c>
+      <c r="BU188" t="str">
+        <f>=IFERROR('IV. MA'!BS10,0)</f>
+      </c>
+      <c r="BV188" t="str">
+        <f>=IFERROR('IV. MA'!BT10,0)</f>
+      </c>
+    </row>
+    <row r="189">
+      <c r="BR189" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS189" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT189" t="s">
+        <v>206</v>
+      </c>
+      <c r="BU189" t="str">
+        <f>=IFERROR('IV. MA'!BS11,0)</f>
+      </c>
+      <c r="BV189" t="str">
+        <f>=IFERROR('IV. MA'!BT11,0)</f>
+      </c>
+    </row>
+    <row r="190">
+      <c r="BR190" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS190" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT190" t="s">
+        <v>207</v>
+      </c>
+      <c r="BU190" t="str">
+        <f>=IFERROR('IV. MA'!BS12,0)</f>
+      </c>
+      <c r="BV190" t="str">
+        <f>=IFERROR('IV. MA'!BT12,0)</f>
+      </c>
+    </row>
+    <row r="191">
+      <c r="BR191" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS191" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT191" t="s">
+        <v>208</v>
+      </c>
+      <c r="BU191" t="str">
+        <f>=IFERROR('IV. MA'!BS13,0)</f>
+      </c>
+      <c r="BV191" t="str">
+        <f>=IFERROR('IV. MA'!BT13,0)</f>
+      </c>
+    </row>
+    <row r="192">
+      <c r="BR192" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS192" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT192" t="s">
+        <v>209</v>
+      </c>
+      <c r="BU192" t="str">
+        <f>=IFERROR('IV. MA'!BS14,0)</f>
+      </c>
+      <c r="BV192" t="str">
+        <f>=IFERROR('IV. MA'!BT14,0)</f>
+      </c>
+    </row>
+    <row r="193">
+      <c r="BR193" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS193" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT193" t="s">
+        <v>210</v>
+      </c>
+      <c r="BU193" t="str">
+        <f>=IFERROR('IV. MA'!BS15,0)</f>
+      </c>
+      <c r="BV193" t="str">
+        <f>=IFERROR('IV. MA'!BT15,0)</f>
+      </c>
+    </row>
+    <row r="194">
+      <c r="BR194" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS194" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT194" t="s">
+        <v>211</v>
+      </c>
+      <c r="BU194" t="str">
+        <f>=IFERROR('IV. MA'!BS16,0)</f>
+      </c>
+      <c r="BV194" t="str">
+        <f>=IFERROR('IV. MA'!BT16,0)</f>
+      </c>
+    </row>
+    <row r="195">
+      <c r="BR195" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS195" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT195" t="s">
         <v>212</v>
       </c>
-      <c r="BU144" t="str">
+      <c r="BU195" t="str">
         <f>=IFERROR('IV. MA'!BS17,0)</f>
       </c>
-      <c r="BV144" t="str">
+      <c r="BV195" t="str">
         <f>=IFERROR('IV. MA'!BT17,0)</f>
+      </c>
+    </row>
+    <row r="196">
+      <c r="BR196" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS196" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT196" t="s">
+        <v>194</v>
+      </c>
+      <c r="BU196" t="str">
+        <f>=IFERROR('IV. MA'!BS21,0)</f>
+      </c>
+      <c r="BV196" t="str">
+        <f>=IFERROR('IV. MA'!BT21,0)</f>
+      </c>
+    </row>
+    <row r="197">
+      <c r="BR197" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS197" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT197" t="s">
+        <v>279</v>
+      </c>
+      <c r="BU197" t="str">
+        <f>=IFERROR('IV. MA'!BS22,0)</f>
+      </c>
+      <c r="BV197" t="str">
+        <f>=IFERROR('IV. MA'!BT22,0)</f>
+      </c>
+    </row>
+    <row r="198">
+      <c r="BR198" t="str">
+        <f>=$BB$18</f>
+      </c>
+      <c r="BS198" t="str">
+        <f>=$BD$18</f>
+      </c>
+      <c r="BT198" t="s">
+        <v>199</v>
+      </c>
+      <c r="BU198" t="str">
+        <f>=IFERROR('IV. MA'!BS25,0)</f>
+      </c>
+      <c r="BV198" t="str">
+        <f>=IFERROR('IV. MA'!BT25,0)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: calculate EUR values for Saldo and Saldovortrag
Replace manual input with formulas that calculate EUR values by dividing the local currency (LW) amount by the respective exchange rate.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_output.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_output.xlsx
@@ -2285,7 +2285,7 @@
     <xf numFmtId="166" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="6" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -5130,8 +5130,8 @@
       <c r="D11" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>158</v>
+      <c r="E11" s="13" t="str">
+        <f>=IFERROR(ROUND($C$11/$E$10,2),0)</f>
       </c>
       <c r="AA11" s="3" t="s">
         <v>12</v>
@@ -5164,8 +5164,8 @@
       <c r="D13" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>158</v>
+      <c r="E13" s="13" t="str">
+        <f>=IFERROR(ROUND($C$13/$E$12,2),0)</f>
       </c>
       <c r="AA13" s="3" t="s">
         <v>14</v>

</xml_diff>